<commit_message>
release: V1.8.25 - Unified Speaking Practice Controller refactor & edge-case fixes
</commit_message>
<xml_diff>
--- a/public/database/Highlight Incorrect Words/HIW/HIW.xlsx
+++ b/public/database/Highlight Incorrect Words/HIW/HIW.xlsx
@@ -37,7 +37,7 @@
     <t>Happy New Year! And if you've been away from work for a few days, you deserve some time off. After all, you've traveled far. Even if you just stayed at home. According to NASA, just by being on the planet Earth in the last year, you've zipped about 584 million miles around the sun. At an average speed of about 67,000 miles per hour. Hey, I wasn't speeding—in my __initial/inertial__ reference frame. Of course, the trip was not a perfect circle. As Kepler showed, the Earth's orbit is an __eclipse/ellipse__ , with the sun at one of the two __vocal/focal__ points. He also figured out the planet goes faster when it's at perihelion, nearer the sun, than when it's at aphelion, its furthest distance. Which would explain why summer seems to zip by, except that the seasons are a function of the tilt of the Earth's __crust/axis__ , not its different distances from the sun. And the Earth rotated 365 and a quarter times during its sweep around the sun. The trip took 8,766 hours. Or 525,960 minutes. Or 31,557,600 seconds.</t>
   </si>
   <si>
-    <t>Happy New Year! And if you've been away from work for a few days, you deserve some time off. After all, you've traveled far. Even if you just stayed at home. According to NASA, just by being on the planet Earth in the last year, you've zipped about 584 million miles around the sun. At an average speed of about 67,000 miles per hour. Hey, I wasn't speeding—in my initial reference frame. Of course, the trip was not a perfect circle. As Kepler showed, the Earth's orbit is an eclipse , with the sun at one of the two vocal points. He also figured out the planet goes faster when it's at perihelion, nearer the sun, than when it's at aphelion, its furthest distance. Which would explain why summer seems to zip by, except that the seasons are a function of the tilt of the Earth's crust , not its different distances from the sun. And the Earth rotated 365 and a quarter times during its sweep around the sun. The trip took 8,766 hours. Or 525,960 minutes. Or 31,557,600 seconds.</t>
+    <t>Happy New Year! And if you've been away from work for a few days, you deserve some time off. After all, you've traveled far. Even if you just stayed at home. According to NASA, just by being on the planet Earth in the last year, you've zipped about 584 million miles around the sun. At an average speed of about 67,000 miles per hour. Hey, I wasn't speeding—in my inertial reference frame. Of course, the trip was not a perfect circle. As Kepler showed, the Earth's orbit is an ellipse , with the sun at one of the two focal points. He also figured out the planet goes faster when it's at perihelion, nearer the sun, than when it's at aphelion, its furthest distance. Which would explain why summer seems to zip by, except that the seasons are a function of the tilt of the Earth's axis , not its different distances from the sun. And the Earth rotated 365 and a quarter times during its sweep around the sun. The trip took 8,766 hours. Or 525,960 minutes. Or 31,557,600 seconds.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;Understanding the Listening Highlight - Incorrect Words&lt;/h3&gt;
@@ -88,7 +88,7 @@
     <t>Humans can recognize each other by voice alone. I sound different from other 60-Second Science reporters, for example. In fact, lots of nonhuman animals, of all types, use voices to distinguish familiar individuals, including frogs, fish, lemurs, and penguins. And that __universal/unique__ audio fingerprint extends to a sound you may have heard in the forest on occasion: the drumming of a woodpecker. Researchers recorded __motive/multiple__ drum rolls, from 41 great spotted woodpeckers—colorful red, white and black birds—living in Polish forests. They then used audio software to analyze them. And they found that the length of the drumrolls, and the spacing between beats varied enough from bird to bird to tell the woodpeckers apart by drumming alone. The study is in the journal PLOS ONE. The scientists say this fact might be useful to woodpeckers, in __intensifying/identifying__ each other. And to __conversation/conservation__ biologists, trying to tease one bird from another in a recording, for example, to count individuals in a given area. The birds' head-banging could thus do away with that research headache.</t>
   </si>
   <si>
-    <t>Humans can recognize each other by voice alone. I sound different from other 60-Second Science reporters, for example. In fact, lots of nonhuman animals, of all types, use voices to distinguish familiar individuals, including frogs, fish, lemurs, and penguins. And that universal audio fingerprint extends to a sound you may have heard in the forest on occasion: the drumming of a woodpecker. Researchers recorded motive drum rolls, from 41 great spotted woodpeckers—colorful red, white and black birds—living in Polish forests. They then used audio software to analyze them. And they found that the length of the drumrolls, and the spacing between beats varied enough from bird to bird to tell the woodpeckers apart by drumming alone. The study is in the journal PLOS ONE. The scientists say this fact might be useful to woodpeckers, in intensifying each other. And to conversation biologists, trying to tease one bird from another in a recording, for example, to count individuals in a given area. The birds' head-banging could thus do away with that research headache.</t>
+    <t>Humans can recognize each other by voice alone. I sound different from other 60-Second Science reporters, for example. In fact, lots of nonhuman animals, of all types, use voices to distinguish familiar individuals, including frogs, fish, lemurs, and penguins. And that unique audio fingerprint extends to a sound you may have heard in the forest on occasion: the drumming of a woodpecker. Researchers recorded multiple drum rolls, from 41 great spotted woodpeckers—colorful red, white and black birds—living in Polish forests. They then used audio software to analyze them. And they found that the length of the drumrolls, and the spacing between beats varied enough from bird to bird to tell the woodpeckers apart by drumming alone. The study is in the journal PLOS ONE. The scientists say this fact might be useful to woodpeckers, in identifying each other. And to conservation biologists, trying to tease one bird from another in a recording, for example, to count individuals in a given area. The birds' head-banging could thus do away with that research headache.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🎧 PTE Listening Strategy: Incorrect Word Identification&lt;/h3&gt;
@@ -128,7 +128,7 @@
     <t>Parts of the planet warm and cool during El Niño and La Niña. And infectious __acacias/diseases__ also wax and wane in step with the climate cycle. Take malaria—shown to spike in northern Venezuela during cool, La Niña conditions. Or flu pandemics, which often follow months after La Niña sets in. Now researchers have linked another public health risk to El Niño climate cycling: poisonous viper bites. Their study area was Costa Rica—where health centers keep rigorous records on snakebites. They compared nine years of those snakebite records—including some 6,500 bites—to climate data over the same period. And they found that __vaporise/snakebites__ were two to three times as prevalent in the hottest and coldest years of the El Niño climate cycle. Sounds counterintuitive, right —you might expect the climate extremes to have opposite effects. But the researchers say in hot, dry years, plant productivity peaks, driving an __retrieve/increase__ in the number of rodents—aka snake food, potentially increasing the number of snakes. And snakes tend to move around more in hot, dry weather—increasing chances they'll encounter—and attack—an unlucky farmer. In cold, wet years, on the other hand, prey numbers plummet—forcing snakes to travel beyond their usual slithering grounds to eat—again increasing chances of an unlucky meeting. The study is in the journal Science Advances. The researchers also found two more variables that __navigate/correlate__ strongly with Costa Ricans' odds of being bit: poverty and destitute housing. A reminder that, when it comes to dangers from environmental disruption, it's often the least __coordinate/fortunate__ who are at the greatest risk.</t>
   </si>
   <si>
-    <t>Parts of the planet warm and cool during El Niño and La Niña. And infectious acacias also wax and wane in step with the climate cycle. Take malaria—shown to spike in northern Venezuela during cool, La Niña conditions. Or flu pandemics, which often follow months after La Niña sets in. Now researchers have linked another public health risk to El Niño climate cycling: poisonous viper bites. Their study area was Costa Rica—where health centers keep rigorous records on snakebites. They compared nine years of those snakebite records—including some 6,500 bites—to climate data over the same period. And they found that vaporise were two to three times as prevalent in the hottest and coldest years of the El Niño climate cycle. Sounds counterintuitive, right —you might expect the climate extremes to have opposite effects. But the researchers say in hot, dry years, plant productivity peaks, driving an retrieve in the number of rodents—aka snake food, potentially increasing the number of snakes. And snakes tend to move around more in hot, dry weather—increasing chances they'll encounter—and attack—an unlucky farmer. In cold, wet years, on the other hand, prey numbers plummet—forcing snakes to travel beyond their usual slithering grounds to eat—again increasing chances of an unlucky meeting. The study is in the journal Science Advances. The researchers also found two more variables that navigate strongly with Costa Ricans' odds of being bit: poverty and destitute housing. A reminder that, when it comes to dangers from environmental disruption, it's often the least coordinate who are at the greatest risk.</t>
+    <t>Parts of the planet warm and cool during El Niño and La Niña. And infectious diseases also wax and wane in step with the climate cycle. Take malaria—shown to spike in northern Venezuela during cool, La Niña conditions. Or flu pandemics, which often follow months after La Niña sets in. Now researchers have linked another public health risk to El Niño climate cycling: poisonous viper bites. Their study area was Costa Rica—where health centers keep rigorous records on snakebites. They compared nine years of those snakebite records—including some 6,500 bites—to climate data over the same period. And they found that snakebites were two to three times as prevalent in the hottest and coldest years of the El Niño climate cycle. Sounds counterintuitive, right —you might expect the climate extremes to have opposite effects. But the researchers say in hot, dry years, plant productivity peaks, driving an increase in the number of rodents—aka snake food, potentially increasing the number of snakes. And snakes tend to move around more in hot, dry weather—increasing chances they'll encounter—and attack—an unlucky farmer. In cold, wet years, on the other hand, prey numbers plummet—forcing snakes to travel beyond their usual slithering grounds to eat—again increasing chances of an unlucky meeting. The study is in the journal Science Advances. The researchers also found two more variables that correlate strongly with Costa Ricans' odds of being bit: poverty and destitute housing. A reminder that, when it comes to dangers from environmental disruption, it's often the least fortunate who are at the greatest risk.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This is a common and often challenging question type in the PTE Listening section. The goal is to identify subtle phonetic changes, subject-matter vocabulary shifts, and structural mismatches between the visual transcript and the actual spoken audio.&lt;/p&gt;
@@ -182,7 +182,7 @@
     <t>In the __digestibility/celebrity__ vaccine wars, I'm siding with actress Amanda Peet. And comedian Bill Maher, well, I like your show, but when it comes to vaccines you don't know a punchline from a clothesline. Maher recently tweeted to his Twitter followers "if u get a swine flu shot ur an idiot." On his HBO program Real Time last week, Maher went head-to-head with former Senator Dr. Bill Frist, who patiently __grenade/explained__ why vaccines were in fact good. But Maher wasn't buying it. He advocates a healthy lifestyle over vaccines. But polio and smallpox outmatched many robust immune systems. Actress Amanda Peet, meanwhile, has used her celebrity to encourage vaccinations, specifically in response to the alleged vaccine-autism connection, for which there's no scientific evidence, but which has some parents afraid of __plywood/childhood__ vaccinations. In a letter to a parenting magazine, Peet wrote: (quote)"It's __reversible/irresponsible__ to suggest that virtually the entire medical community, and the CDC, and the American Academy of Pediatrics are behind a massive cover-up about vaccine safety."(end quote) See you in the line for the flu shot.</t>
   </si>
   <si>
-    <t>In the digestibility vaccine wars, I'm siding with actress Amanda Peet. And comedian Bill Maher, well, I like your show, but when it comes to vaccines you don't know a punchline from a clothesline. Maher recently tweeted to his Twitter followers "if u get a swine flu shot ur an idiot." On his HBO program Real Time last week, Maher went head-to-head with former Senator Dr. Bill Frist, who patiently grenade why vaccines were in fact good. But Maher wasn't buying it. He advocates a healthy lifestyle over vaccines. But polio and smallpox outmatched many robust immune systems. Actress Amanda Peet, meanwhile, has used her celebrity to encourage vaccinations, specifically in response to the alleged vaccine-autism connection, for which there's no scientific evidence, but which has some parents afraid of plywood vaccinations. In a letter to a parenting magazine, Peet wrote: (quote)"It's reversible to suggest that virtually the entire medical community, and the CDC, and the American Academy of Pediatrics are behind a massive cover-up about vaccine safety."(end quote) See you in the line for the flu shot.</t>
+    <t>In the celebrity vaccine wars, I'm siding with actress Amanda Peet. And comedian Bill Maher, well, I like your show, but when it comes to vaccines you don't know a punchline from a clothesline. Maher recently tweeted to his Twitter followers "if u get a swine flu shot ur an idiot." On his HBO program Real Time last week, Maher went head-to-head with former Senator Dr. Bill Frist, who patiently explained why vaccines were in fact good. But Maher wasn't buying it. He advocates a healthy lifestyle over vaccines. But polio and smallpox outmatched many robust immune systems. Actress Amanda Peet, meanwhile, has used her celebrity to encourage vaccinations, specifically in response to the alleged vaccine-autism connection, for which there's no scientific evidence, but which has some parents afraid of childhood vaccinations. In a letter to a parenting magazine, Peet wrote: (quote)"It's irresponsible to suggest that virtually the entire medical community, and the CDC, and the American Academy of Pediatrics are behind a massive cover-up about vaccine safety."(end quote) See you in the line for the flu shot.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your PTE Academic teacher, I can tell you that the 'Highlight Incorrect Words' task is not just about catching mishearings; it's about advanced listening comprehension, phonological awareness, and understanding context. The distractors are designed to sound very similar to the correct words, making deep focus essential.&lt;/p&gt;
@@ -238,7 +238,7 @@
     <t>Using less energy saves money and lowers greenhouse gas emissions. And various studies have looked at ways to get households to use less energy. Now there's evidence that people in such a study use less energy…because they're in a study. The general phenomenon is called the Hawthorne effect: study subjects change their __gratia/behavior__ because they're being observed. So __freelances/researchers__ collaborated with a utility to test for the Hawthorne effect in electricity use. They __domiciled/monitored__ almost 5,600 randomly __blended/selected__ households. Half received a postcard saying that their energy use would be monitored for a month for research purposes. They also got four follow-up reminder postcards over the month. They received no other information, instructions or incentives. The control group monitored for the study got no notifications. That group continued using the same amount of electricity. But the families being tracked reduced energy use 2.7 percent. And when the study period ended, their energy use shot back up. The report is in the Proceedings of the National Academy of Sciences. Clearly, mindful consumers can find ways to easily lower their energy consumption. Perhaps policy makers can find a way to use the Hawthorne effect to everyone's advantage.</t>
   </si>
   <si>
-    <t>Using less energy saves money and lowers greenhouse gas emissions. And various studies have looked at ways to get households to use less energy. Now there's evidence that people in such a study use less energy…because they're in a study. The general phenomenon is called the Hawthorne effect: study subjects change their gratia because they're being observed. So freelances collaborated with a utility to test for the Hawthorne effect in electricity use. They domiciled almost 5,600 randomly blended households. Half received a postcard saying that their energy use would be monitored for a month for research purposes. They also got four follow-up reminder postcards over the month. They received no other information, instructions or incentives. The control group monitored for the study got no notifications. That group continued using the same amount of electricity. But the families being tracked reduced energy use 2.7 percent. And when the study period ended, their energy use shot back up. The report is in the Proceedings of the National Academy of Sciences. Clearly, mindful consumers can find ways to easily lower their energy consumption. Perhaps policy makers can find a way to use the Hawthorne effect to everyone's advantage.</t>
+    <t>Using less energy saves money and lowers greenhouse gas emissions. And various studies have looked at ways to get households to use less energy. Now there's evidence that people in such a study use less energy…because they're in a study. The general phenomenon is called the Hawthorne effect: study subjects change their behavior because they're being observed. So researchers collaborated with a utility to test for the Hawthorne effect in electricity use. They monitored almost 5,600 randomly selected households. Half received a postcard saying that their energy use would be monitored for a month for research purposes. They also got four follow-up reminder postcards over the month. They received no other information, instructions or incentives. The control group monitored for the study got no notifications. That group continued using the same amount of electricity. But the families being tracked reduced energy use 2.7 percent. And when the study period ended, their energy use shot back up. The report is in the Proceedings of the National Academy of Sciences. Clearly, mindful consumers can find ways to easily lower their energy consumption. Perhaps policy makers can find a way to use the Hawthorne effect to everyone's advantage.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a premium PTE instructor, I can guide you through this specific type of Listening question. In the "Highlight Incorrect Words" task, you must listen carefully for subtle differences in pronunciation, word choice, or overall meaning compared to the written transcript. Below is a detailed analysis of the words you highlighted incorrectly, explaining the correction and the context behind it.&lt;/p&gt;
@@ -278,7 +278,7 @@
     <t>It's Friday the 13th. "You've gotta ask yourself a question: 'Do I feel lucky?'" If you don't, you could be suffering from triskaidekaphobia. That's a fear of the number 13. Napoleon, Herbert Hoover and FDR are __welcome/well-documented__ triskaidekaphobics. But why do folks think 13 is unlucky? Particularly when it falls on a Friday, as it will three times this year? The University of Delaware's Thomas __gobbler/Fernsler__ is known as Dr. 13. He's an expert on the number's bad reputation, which may date back to biblical times. After all, the 13th guest at the Last Supper was Judas. And you know how that worked out for Jesus, who was crucified on a Friday. Other factoids from Fernsler: The first person to die in a car __consummate/accident__ was killed in New York City on September the 13th in 1899, although that was a Wednesday. And the ill-fated flight of Apollo 13 launched at the 13th minute of the 13th hour Central Standard Time on April 11th, 1970. And the __newscasters/numerals__ in the date 4/11/70 add up to, guess, 13! As long as you don't include the 19 in 1970. Hey, sometimes superstition can be hard work. Today, some tall buildings lack a 13th floor. Well, they have a 13th floor, but they call it the 14th floor. Because the __destinations/purveyors__ of bad luck are apparently easily fooled. Meanwhile, over in France, panicky Parisian __doses/party-throwers__ can even hire a quatorziéme, a professional 14th guest. Like Judas, Mark Twain was allegedly once poised to be the 13th guest at a dinner party. A superstitious friend warned the very rational Twain not to go. But Twain went. "It was bad luck," he later remarked. "They only had food for 12."</t>
   </si>
   <si>
-    <t>It's Friday the 13th. "You've gotta ask yourself a question: 'Do I feel lucky?'" If you don't, you could be suffering from triskaidekaphobia. That's a fear of the number 13. Napoleon, Herbert Hoover and FDR are welcome triskaidekaphobics. But why do folks think 13 is unlucky? Particularly when it falls on a Friday, as it will three times this year? The University of Delaware's Thomas gobbler is known as Dr. 13. He's an expert on the number's bad reputation, which may date back to biblical times. After all, the 13th guest at the Last Supper was Judas. And you know how that worked out for Jesus, who was crucified on a Friday. Other factoids from Fernsler: The first person to die in a car consummate was killed in New York City on September the 13th in 1899, although that was a Wednesday. And the ill-fated flight of Apollo 13 launched at the 13th minute of the 13th hour Central Standard Time on April 11th, 1970. And the newscasters in the date 4/11/70 add up to, guess, 13! As long as you don't include the 19 in 1970. Hey, sometimes superstition can be hard work. Today, some tall buildings lack a 13th floor. Well, they have a 13th floor, but they call it the 14th floor. Because the destinations of bad luck are apparently easily fooled. Meanwhile, over in France, panicky Parisian doses can even hire a quatorziéme, a professional 14th guest. Like Judas, Mark Twain was allegedly once poised to be the 13th guest at a dinner party. A superstitious friend warned the very rational Twain not to go. But Twain went. "It was bad luck," he later remarked. "They only had food for 12."</t>
+    <t>It's Friday the 13th. "You've gotta ask yourself a question: 'Do I feel lucky?'" If you don't, you could be suffering from triskaidekaphobia. That's a fear of the number 13. Napoleon, Herbert Hoover and FDR are well-documented triskaidekaphobics. But why do folks think 13 is unlucky? Particularly when it falls on a Friday, as it will three times this year? The University of Delaware's Thomas Fernsler is known as Dr. 13. He's an expert on the number's bad reputation, which may date back to biblical times. After all, the 13th guest at the Last Supper was Judas. And you know how that worked out for Jesus, who was crucified on a Friday. Other factoids from Fernsler: The first person to die in a car accident was killed in New York City on September the 13th in 1899, although that was a Wednesday. And the ill-fated flight of Apollo 13 launched at the 13th minute of the 13th hour Central Standard Time on April 11th, 1970. And the numerals in the date 4/11/70 add up to, guess, 13! As long as you don't include the 19 in 1970. Hey, sometimes superstition can be hard work. Today, some tall buildings lack a 13th floor. Well, they have a 13th floor, but they call it the 14th floor. Because the purveyors of bad luck are apparently easily fooled. Meanwhile, over in France, panicky Parisian party-throwers can even hire a quatorziéme, a professional 14th guest. Like Judas, Mark Twain was allegedly once poised to be the 13th guest at a dinner party. A superstitious friend warned the very rational Twain not to go. But Twain went. "It was bad luck," he later remarked. "They only had food for 12."</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;✨ PTE Listening Analysis: Highlight Incorrect Words&lt;/h3&gt;
@@ -323,7 +323,7 @@
     <t>It follows from the special theory of relativity that mass and energy are different manifestations of the same thing. Now __cleavages/researchers__ have stopped light cold - and then brought it back to life - or light - in an __ribaldry/entirely__ different place. The Harvard researchers sent a light pulse into a sodium cloud cooled to about 460 degrees below zero. That's the __hypocritical/theoretical__ point where matter stops all movement. The light pulse was compressed by a factor of about 50 million at the extreme temperature, and it actually changed state - sort of like frozen water. But it also split into two forms of matter. One stayed frozen in the sodium, while the other crawled along at just 200 meters per hour. That second form - called a matter wave - contains the exact information of the original light wave. And when researchers sent it into a second sodium cloud a fraction of a __freesia/millimeter__ away, the wave was converted back into light. And since fiber-optic __containers/communications__ use light, that means that someday we may be able to stop them, store them and turn them back on, just like a light switch.</t>
   </si>
   <si>
-    <t>It follows from the special theory of relativity that mass and energy are different manifestations of the same thing. Now cleavages have stopped light cold - and then brought it back to life - or light - in an ribaldry different place. The Harvard researchers sent a light pulse into a sodium cloud cooled to about 460 degrees below zero. That's the hypocritical point where matter stops all movement. The light pulse was compressed by a factor of about 50 million at the extreme temperature, and it actually changed state - sort of like frozen water. But it also split into two forms of matter. One stayed frozen in the sodium, while the other crawled along at just 200 meters per hour. That second form - called a matter wave - contains the exact information of the original light wave. And when researchers sent it into a second sodium cloud a fraction of a freesia away, the wave was converted back into light. And since fiber-optic containers use light, that means that someday we may be able to stop them, store them and turn them back on, just like a light switch.</t>
+    <t>It follows from the special theory of relativity that mass and energy are different manifestations of the same thing. Now researchers have stopped light cold - and then brought it back to life - or light - in an entirely different place. The Harvard researchers sent a light pulse into a sodium cloud cooled to about 460 degrees below zero. That's the theoretical point where matter stops all movement. The light pulse was compressed by a factor of about 50 million at the extreme temperature, and it actually changed state - sort of like frozen water. But it also split into two forms of matter. One stayed frozen in the sodium, while the other crawled along at just 200 meters per hour. That second form - called a matter wave - contains the exact information of the original light wave. And when researchers sent it into a second sodium cloud a fraction of a millimeter away, the wave was converted back into light. And since fiber-optic communications use light, that means that someday we may be able to stop them, store them and turn them back on, just like a light switch.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Welcome! As a premium PTE instructor, I understand that this type of question—Highlighting Incorrect Words—tests not only your listening skills but also your ability to process context, vocabulary, and pronunciation. These words often contain minimal pairs or are phonetically similar to common academic vocabulary. Below is a detailed analysis of each incorrect word, showing you exactly why the correct word is the right fit for the context.&lt;/p&gt;
@@ -371,7 +371,7 @@
     <t>That's Generation Zero of DarwinTunes. It's a Web site __veggieburgers/researchers__ are using to study how __macromolecular/listener__ preferences affect the evolution of music. A new study claims that the taste of the public exerts a force on music similar to natural selection. The findings support the theory that culture and art are shaped not only by their producers, but by consumers too. The report is in the Proceedings of the National Academy of Sciences. Researchers created short tunes and allowed them to procreate—that is, they'd combine aspects of the parent tunes to produce a new __remuneration/generation__ of music. User ratings on the __tunics/DarwinTunes__ site provided the evolutionary selection, with only the most appealing tunes allowed to create progeny. The researchers found that quality __microfiche/increased__ quickly at the beginning: the random sounds rapidly gave rise to __falling/something__ an awful lot like music. Here's generation 600. But after a while things stagnated. Three researchers plan to update the program to drive evolution further. Meanwhile, here's DarwinTunes generation 3000.</t>
   </si>
   <si>
-    <t>That's Generation Zero of DarwinTunes. It's a Web site veggieburgers are using to study how macromolecular preferences affect the evolution of music. A new study claims that the taste of the public exerts a force on music similar to natural selection. The findings support the theory that culture and art are shaped not only by their producers, but by consumers too. The report is in the Proceedings of the National Academy of Sciences. Researchers created short tunes and allowed them to procreate—that is, they'd combine aspects of the parent tunes to produce a new remuneration of music. User ratings on the tunics site provided the evolutionary selection, with only the most appealing tunes allowed to create progeny. The researchers found that quality microfiche quickly at the beginning: the random sounds rapidly gave rise to falling an awful lot like music. Here's generation 600. But after a while things stagnated. Three researchers plan to update the program to drive evolution further. Meanwhile, here's DarwinTunes generation 3000.</t>
+    <t>That's Generation Zero of DarwinTunes. It's a Web site researchers are using to study how listener preferences affect the evolution of music. A new study claims that the taste of the public exerts a force on music similar to natural selection. The findings support the theory that culture and art are shaped not only by their producers, but by consumers too. The report is in the Proceedings of the National Academy of Sciences. Researchers created short tunes and allowed them to procreate—that is, they'd combine aspects of the parent tunes to produce a new generation of music. User ratings on the DarwinTunes site provided the evolutionary selection, with only the most appealing tunes allowed to create progeny. The researchers found that quality increased quickly at the beginning: the random sounds rapidly gave rise to something an awful lot like music. Here's generation 600. But after a while things stagnated. Three researchers plan to update the program to drive evolution further. Meanwhile, here's DarwinTunes generation 3000.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🎧 PTE Listening Analysis: Incorrect Word Identification&lt;/h3&gt;
@@ -412,7 +412,7 @@
     <t>I once took part in a vodka tasting contest, in which participants tried to tell an expensive brand from a cheap one. I don't recall the exact outcome, for obvious reasons. But I do know that several people swore they could taste the difference. Well, maybe they could. Because according to a study in the Journal of __capital/Agricultural__ and Food Chemistry, __perfectionist/different__ vodkas can have different molecular "structures," which could drive drinkers to favor one brand over another. Vodka's an __elastic/alcoholic__ beverage that's supposed to be relatively flavorless. So researchers got to wondering: how come people who enjoy the stuff often express brand preference? Being good little scientists, they trotted out their __periphrastic/spectroscopic__ equipment and examined the __inadmissible/chemical__ signatures of five different vodkas. What they found is that each brand differs in how its ethanol molecules cluster. In the ethanol-water mix we call vodka, some of the ethanol molecules get surrounded by a sort of "cage" made of water. And different brands differ in how much ethanol is caged. Vodkas with fewer cages might seem more "watery" than those with more structure. Of course, drink enough of the stuff and it really won't matter how tightly caged it is. You'll be loose as a grey goose.</t>
   </si>
   <si>
-    <t>I once took part in a vodka tasting contest, in which participants tried to tell an expensive brand from a cheap one. I don't recall the exact outcome, for obvious reasons. But I do know that several people swore they could taste the difference. Well, maybe they could. Because according to a study in the Journal of capital and Food Chemistry, perfectionist vodkas can have different molecular "structures," which could drive drinkers to favor one brand over another. Vodka's an elastic beverage that's supposed to be relatively flavorless. So researchers got to wondering: how come people who enjoy the stuff often express brand preference? Being good little scientists, they trotted out their periphrastic equipment and examined the inadmissible signatures of five different vodkas. What they found is that each brand differs in how its ethanol molecules cluster. In the ethanol-water mix we call vodka, some of the ethanol molecules get surrounded by a sort of "cage" made of water. And different brands differ in how much ethanol is caged. Vodkas with fewer cages might seem more "watery" than those with more structure. Of course, drink enough of the stuff and it really won't matter how tightly caged it is. You'll be loose as a grey goose.</t>
+    <t>I once took part in a vodka tasting contest, in which participants tried to tell an expensive brand from a cheap one. I don't recall the exact outcome, for obvious reasons. But I do know that several people swore they could taste the difference. Well, maybe they could. Because according to a study in the Journal of Agricultural and Food Chemistry, different vodkas can have different molecular "structures," which could drive drinkers to favor one brand over another. Vodka's an alcoholic beverage that's supposed to be relatively flavorless. So researchers got to wondering: how come people who enjoy the stuff often express brand preference? Being good little scientists, they trotted out their spectroscopic equipment and examined the chemical signatures of five different vodkas. What they found is that each brand differs in how its ethanol molecules cluster. In the ethanol-water mix we call vodka, some of the ethanol molecules get surrounded by a sort of "cage" made of water. And different brands differ in how much ethanol is caged. Vodkas with fewer cages might seem more "watery" than those with more structure. Of course, drink enough of the stuff and it really won't matter how tightly caged it is. You'll be loose as a grey goose.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your PTE Academic instructor, I can see you successfully identified several key areas where the spelling and vocabulary used in the transcript diverged from the actual spoken audio. This is a common challenge, as the incorrect words sound plausible but are contextually wrong.&lt;/p&gt;
@@ -458,7 +458,7 @@
     <t>If you’ve spent any time hitting up the giant wholesalers or other markets this holiday season, you’ve probably figured out that you can make a full meal out of those __delicious/tasty__ little samples they often dish out. Which seems like a good thing, for you … and for your wallet. But a new study shows that these tempting little treats really do entice you to buy what you try … and maybe some other stuff like it. Researchers tracked the sales in half a dozen stores that provided samples of __snakes/snacks__ in four categories: healthy, salty, frozen, or branded by a large coffee-shop chain. They found that nothing while shopping convinces consumers to buy the __future/featured__ product more often than does simply seeing the product displayed at the end of the aisle. They also found that repeating the __example/sample__ offering multiple times translates into __subsisted/sustained__ interest in the product … and that stores that have a smaller assortment of products for sale benefit more than the warehouse-sized emporia. The finding is served up in the Journal of Retailing. The researchers also discovered that the effect extends beyond the product itself…such that, for example, nibbling on one brand of cookies makes you hungry for cookies in general — including those from competing brands. Which suggests that a rising tide really does lift all boats. Or at least that a tray of free taquitos will certainly lift a lot of shoppers’ spirits … and will keep those registers ringing well into the new year.</t>
   </si>
   <si>
-    <t>If you’ve spent any time hitting up the giant wholesalers or other markets this holiday season, you’ve probably figured out that you can make a full meal out of those delicious little samples they often dish out. Which seems like a good thing, for you … and for your wallet. But a new study shows that these tempting little treats really do entice you to buy what you try … and maybe some other stuff like it. Researchers tracked the sales in half a dozen stores that provided samples of snakes in four categories: healthy, salty, frozen, or branded by a large coffee-shop chain. They found that nothing while shopping convinces consumers to buy the future product more often than does simply seeing the product displayed at the end of the aisle. They also found that repeating the example offering multiple times translates into subsisted interest in the product … and that stores that have a smaller assortment of products for sale benefit more than the warehouse-sized emporia. The finding is served up in the Journal of Retailing. The researchers also discovered that the effect extends beyond the product itself…such that, for example, nibbling on one brand of cookies makes you hungry for cookies in general — including those from competing brands. Which suggests that a rising tide really does lift all boats. Or at least that a tray of free taquitos will certainly lift a lot of shoppers’ spirits … and will keep those registers ringing well into the new year.</t>
+    <t>If you’ve spent any time hitting up the giant wholesalers or other markets this holiday season, you’ve probably figured out that you can make a full meal out of those tasty little samples they often dish out. Which seems like a good thing, for you … and for your wallet. But a new study shows that these tempting little treats really do entice you to buy what you try … and maybe some other stuff like it. Researchers tracked the sales in half a dozen stores that provided samples of snacks in four categories: healthy, salty, frozen, or branded by a large coffee-shop chain. They found that nothing while shopping convinces consumers to buy the featured product more often than does simply seeing the product displayed at the end of the aisle. They also found that repeating the sample offering multiple times translates into sustained interest in the product … and that stores that have a smaller assortment of products for sale benefit more than the warehouse-sized emporia. The finding is served up in the Journal of Retailing. The researchers also discovered that the effect extends beyond the product itself…such that, for example, nibbling on one brand of cookies makes you hungry for cookies in general — including those from competing brands. Which suggests that a rising tide really does lift all boats. Or at least that a tray of free taquitos will certainly lift a lot of shoppers’ spirits … and will keep those registers ringing well into the new year.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a premium PTE Academic teacher, I understand that this type of question (Highlighting Incorrect Words) tests not only your listening skills but also your vocabulary, phonetic accuracy, and ability to understand contextual nuances. It is crucial to listen closely for subtle phonetic differences and precise word usage.&lt;/p&gt;
@@ -509,7 +509,7 @@
     <t>To a female orb web spider, a suitable male can look like a mate—and a meal. For these spiders, the dating game has turned into a deadly dance of evolutionary one-upsmanship. The female spider can choose when to cut off intimate __raters/relations__ by eating her partner, or kicking him out. This dynamic has led males to an unlikely __accompany/strategy__ to make sure they have some say in the matter: self-castration. Males are able to leave part or all of their organ inside of a female, which decreases the odds the female will be able to mate again. But new research shows that when a male leaves his whole __fuel/kit-and-caboodle__ behind, his likelihood of fathering the next batch of eggs is much higher. Why? His parting gift keeps on giving, even after he is gone. This remote- copulation __physique/technique__ actually boosts the amount and speed of sperm __bland/transferred__ to the female. The behavior is __spiked/described__ in the journal Biology Letters. So for these unlucky fellas, it is better to have loved—and lost.</t>
   </si>
   <si>
-    <t>To a female orb web spider, a suitable male can look like a mate—and a meal. For these spiders, the dating game has turned into a deadly dance of evolutionary one-upsmanship. The female spider can choose when to cut off intimate raters by eating her partner, or kicking him out. This dynamic has led males to an unlikely accompany to make sure they have some say in the matter: self-castration. Males are able to leave part or all of their organ inside of a female, which decreases the odds the female will be able to mate again. But new research shows that when a male leaves his whole fuel behind, his likelihood of fathering the next batch of eggs is much higher. Why? His parting gift keeps on giving, even after he is gone. This remote- copulation physique actually boosts the amount and speed of sperm bland to the female. The behavior is spiked in the journal Biology Letters. So for these unlucky fellas, it is better to have loved—and lost.</t>
+    <t>To a female orb web spider, a suitable male can look like a mate—and a meal. For these spiders, the dating game has turned into a deadly dance of evolutionary one-upsmanship. The female spider can choose when to cut off intimate relations by eating her partner, or kicking him out. This dynamic has led males to an unlikely strategy to make sure they have some say in the matter: self-castration. Males are able to leave part or all of their organ inside of a female, which decreases the odds the female will be able to mate again. But new research shows that when a male leaves his whole kit-and-caboodle behind, his likelihood of fathering the next batch of eggs is much higher. Why? His parting gift keeps on giving, even after he is gone. This remote- copulation technique actually boosts the amount and speed of sperm transferred to the female. The behavior is described in the journal Biology Letters. So for these unlucky fellas, it is better to have loved—and lost.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your premium PTE Academic teacher, I will provide a detailed analysis of this Listening section. This question type is challenging because it tests not only your listening ability but also your deep vocabulary, phonological awareness (hearing similar-sounding words), and grammatical understanding. You must identify words that sound similar but have a different meaning or grammatical function in the context.&lt;/p&gt;
@@ -552,7 +552,7 @@
     <t>Ahhh, sleep. There's nothing better than a nice, long, uninterrupted . Awwgh. I can't sleep when there's . But d'ya ever notice: noise doesn't wake everyone. Now __sanitises/scientists__ have a better idea why. Because sound __beguilers/sleepers__ show a certain brain rhythm when they doze, findings published in the journal Current Biology. To study the brain waves of a good night's sleep, scientists invited volunteers to snooze in the lab. While the subjects caught some Zs, the researchers __cummerbund/monitored__ their brain activity. They then __sexist/subjected__ the sleepers to or [NOISE]. And they found that those who were able to slumber __precipitate/straight__ through all the showed more short bursts of faster brain waves. This activity, the scientists say, is the brain's way of __blushing/blocking__ out the and the while you're trying to rest. The scientists don't yet know of any way to boost those sleep-saving brain waves. So until then, shut the door , make sure the late show's on a timer , and try to have sweet dreams.</t>
   </si>
   <si>
-    <t>Ahhh, sleep. There's nothing better than a nice, long, uninterrupted . Awwgh. I can't sleep when there's . But d'ya ever notice: noise doesn't wake everyone. Now sanitises have a better idea why. Because sound beguilers show a certain brain rhythm when they doze, findings published in the journal Current Biology. To study the brain waves of a good night's sleep, scientists invited volunteers to snooze in the lab. While the subjects caught some Zs, the researchers cummerbund their brain activity. They then sexist the sleepers to or [NOISE]. And they found that those who were able to slumber precipitate through all the showed more short bursts of faster brain waves. This activity, the scientists say, is the brain's way of blushing out the and the while you're trying to rest. The scientists don't yet know of any way to boost those sleep-saving brain waves. So until then, shut the door , make sure the late show's on a timer , and try to have sweet dreams.</t>
+    <t>Ahhh, sleep. There's nothing better than a nice, long, uninterrupted . Awwgh. I can't sleep when there's . But d'ya ever notice: noise doesn't wake everyone. Now scientists have a better idea why. Because sound sleepers show a certain brain rhythm when they doze, findings published in the journal Current Biology. To study the brain waves of a good night's sleep, scientists invited volunteers to snooze in the lab. While the subjects caught some Zs, the researchers monitored their brain activity. They then subjected the sleepers to or [NOISE]. And they found that those who were able to slumber straight through all the showed more short bursts of faster brain waves. This activity, the scientists say, is the brain's way of blocking out the and the while you're trying to rest. The scientists don't yet know of any way to boost those sleep-saving brain waves. So until then, shut the door , make sure the late show's on a timer , and try to have sweet dreams.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a premium PTE instructor, I understand that mastering the nuance between similar-sounding words is crucial for high scores on the Listening section. The 'Highlight Incorrect Words' task tests not just your listening acuity, but your ability to apply context, grammar, and semantics.&lt;/p&gt;
@@ -604,7 +604,7 @@
     <t>What makes someone sound sexy? To get a scientific viewpoint, __reasoners/researchers__ gauged volunteers' responses to different voices. The conclusion: voices considered attractive send __felicitous/messages__ about body size. The work is in the journal PLoS ONE. In the animal kingdom, sound indicates size and intentions. For example, a rough and __breezily/low-frequency__ call suggests the vocalizer is large and aggressive, while a clearer, higher frequency signals a small, nonthreatening animal. In the study, researchers adjusted a variety of voices to __absurd/correspond__ with different body sizes. To do so, they synthesized completely artificial voices, and recorded sentences before varying the pitches and resonance. When volunteers listened to the sound samples, men preferred higher-pitched female voices like this one , which suggest a smaller body size. Low-frequency male voices that signaled a large body size , were attractive to females. Interestingly, breathiness made both male and female voices more desirable. It certainly explains the enduring popularity of .</t>
   </si>
   <si>
-    <t>What makes someone sound sexy? To get a scientific viewpoint, reasoners gauged volunteers' responses to different voices. The conclusion: voices considered attractive send felicitous about body size. The work is in the journal PLoS ONE. In the animal kingdom, sound indicates size and intentions. For example, a rough and breezily call suggests the vocalizer is large and aggressive, while a clearer, higher frequency signals a small, nonthreatening animal. In the study, researchers adjusted a variety of voices to absurd with different body sizes. To do so, they synthesized completely artificial voices, and recorded sentences before varying the pitches and resonance. When volunteers listened to the sound samples, men preferred higher-pitched female voices like this one , which suggest a smaller body size. Low-frequency male voices that signaled a large body size , were attractive to females. Interestingly, breathiness made both male and female voices more desirable. It certainly explains the enduring popularity of .</t>
+    <t>What makes someone sound sexy? To get a scientific viewpoint, researchers gauged volunteers' responses to different voices. The conclusion: voices considered attractive send messages about body size. The work is in the journal PLoS ONE. In the animal kingdom, sound indicates size and intentions. For example, a rough and low-frequency call suggests the vocalizer is large and aggressive, while a clearer, higher frequency signals a small, nonthreatening animal. In the study, researchers adjusted a variety of voices to correspond with different body sizes. To do so, they synthesized completely artificial voices, and recorded sentences before varying the pitches and resonance. When volunteers listened to the sound samples, men preferred higher-pitched female voices like this one , which suggest a smaller body size. Low-frequency male voices that signaled a large body size , were attractive to females. Interestingly, breathiness made both male and female voices more desirable. It certainly explains the enduring popularity of .</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This question tests your ability to listen carefully and distinguish subtle differences between words that sound similar but have different meanings or spellings. Below is a detailed breakdown of each incorrect word, its correct replacement, and the reasoning behind the correction.&lt;/p&gt;
@@ -646,7 +646,7 @@
     <t>Hillary is undecided. Obama and McCain both passed. But the scientific community is committed to staging a candidates' debate about science and technology. They want straight talk on political buzzwords like climate change and stem cells, as well as less __attacked/discussed__ issues like funding for basic __reserved/research__ and the National Institutes of Health. What started as citizens worried about the U.S. losing its edge is now a movement called Science Debate 2008. An article in the current issue of the journal Science, claims that, by 2010, 90 percent of the world's __contrivances/scientists__ and __gears/engineers__ will live in Asia, where research is well funded. The authors say the US needs to keep up because science and engineering drove half of America's economic growth over the last fifty years. Science Debate 2008 had to cancel a debate before the upcoming __raver/Pennsylvania__ primaries because candidates __corked/wouldn't__ commit. Now plans are already in the works for Oregon, where primaries are set for May 20th. It's proof, the journal article says, "that scientists can be quickly organized when motivated." If only politicians shared that motivation.</t>
   </si>
   <si>
-    <t>Hillary is undecided. Obama and McCain both passed. But the scientific community is committed to staging a candidates' debate about science and technology. They want straight talk on political buzzwords like climate change and stem cells, as well as less attacked issues like funding for basic reserved and the National Institutes of Health. What started as citizens worried about the U.S. losing its edge is now a movement called Science Debate 2008. An article in the current issue of the journal Science, claims that, by 2010, 90 percent of the world's contrivances and gears will live in Asia, where research is well funded. The authors say the US needs to keep up because science and engineering drove half of America's economic growth over the last fifty years. Science Debate 2008 had to cancel a debate before the upcoming raver primaries because candidates corked commit. Now plans are already in the works for Oregon, where primaries are set for May 20th. It's proof, the journal article says, "that scientists can be quickly organized when motivated." If only politicians shared that motivation.</t>
+    <t>Hillary is undecided. Obama and McCain both passed. But the scientific community is committed to staging a candidates' debate about science and technology. They want straight talk on political buzzwords like climate change and stem cells, as well as less discussed issues like funding for basic research and the National Institutes of Health. What started as citizens worried about the U.S. losing its edge is now a movement called Science Debate 2008. An article in the current issue of the journal Science, claims that, by 2010, 90 percent of the world's scientists and engineers will live in Asia, where research is well funded. The authors say the US needs to keep up because science and engineering drove half of America's economic growth over the last fifty years. Science Debate 2008 had to cancel a debate before the upcoming Pennsylvania primaries because candidates wouldn't commit. Now plans are already in the works for Oregon, where primaries are set for May 20th. It's proof, the journal article says, "that scientists can be quickly organized when motivated." If only politicians shared that motivation.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your PTE Academic teacher, I can see you found six incorrect words in this recording. This question tests not only your listening comprehension but also your ability to recognize subtle acoustic differences and correctly predict the contextually appropriate vocabulary. Don't worry if this is tricky—it requires deep focus! &lt;/p&gt;
@@ -687,7 +687,7 @@
     <t>How many times has your mother told you to turn off the lights when you leave a room, or to close the fridge door while you decide what to eat. Well, __mavericks/climatologists__ are on her side. Because according to a study in the Proceedings of the National Academy of Sciences, reducing global carbon emissions should begin at home. Even if politicians manage to pass climate change legislation, it could be years or even decades before those policies start to make a difference. In the meantime, __hypoglycaemics/scientists__ say, there are things we can all do to shrink our carbon footprint. You've heard most of 'em before: everything from insulating your home and using __bono/low-flow__ showerheads to driving more efficient vehicles and carpooling to the office. But these things really work. Based in part on how folks responded to the energy crisis in the '70s, the scientists __luxuriated/calculated__ how many Americans might be willing to reform their energy-wasting ways. And they found that within 10 years, we could reasonably expect to cut our national emissions by 7.4 percent. That much carbon is slightly larger than the total amount put out by France. If we could manage that, the whole world might say merci.</t>
   </si>
   <si>
-    <t>How many times has your mother told you to turn off the lights when you leave a room, or to close the fridge door while you decide what to eat. Well, mavericks are on her side. Because according to a study in the Proceedings of the National Academy of Sciences, reducing global carbon emissions should begin at home. Even if politicians manage to pass climate change legislation, it could be years or even decades before those policies start to make a difference. In the meantime, hypoglycaemics say, there are things we can all do to shrink our carbon footprint. You've heard most of 'em before: everything from insulating your home and using bono showerheads to driving more efficient vehicles and carpooling to the office. But these things really work. Based in part on how folks responded to the energy crisis in the '70s, the scientists luxuriated how many Americans might be willing to reform their energy-wasting ways. And they found that within 10 years, we could reasonably expect to cut our national emissions by 7.4 percent. That much carbon is slightly larger than the total amount put out by France. If we could manage that, the whole world might say merci.</t>
+    <t>How many times has your mother told you to turn off the lights when you leave a room, or to close the fridge door while you decide what to eat. Well, climatologists are on her side. Because according to a study in the Proceedings of the National Academy of Sciences, reducing global carbon emissions should begin at home. Even if politicians manage to pass climate change legislation, it could be years or even decades before those policies start to make a difference. In the meantime, scientists say, there are things we can all do to shrink our carbon footprint. You've heard most of 'em before: everything from insulating your home and using low-flow showerheads to driving more efficient vehicles and carpooling to the office. But these things really work. Based in part on how folks responded to the energy crisis in the '70s, the scientists calculated how many Americans might be willing to reform their energy-wasting ways. And they found that within 10 years, we could reasonably expect to cut our national emissions by 7.4 percent. That much carbon is slightly larger than the total amount put out by France. If we could manage that, the whole world might say merci.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a premium PTE Academic teacher, I understand that the &lt;strong&gt;Highlight Incorrect Words&lt;/strong&gt; question can be tricky because the incorrect word often sounds phonetically similar to the correct word, or they might be related concepts. The key here is to listen carefully for the precise context and sound. &lt;/p&gt;
@@ -727,7 +727,7 @@
     <t>What's an article? I was asking myself this very question in the post office yesterday, standing in line waiting to sign for, as it so happens, an article. A postal article. Not the postal article. Now before we get ahead of ourselves, an article in English is a __verb/word__ that precedes a noun, and simply indicates specificity. This sounds quite complicated, and to be honest, it's quite complicated to say without spraying everyone within 15 feet, but the concept's quite simple. The definite article in English is the word "the", and indicates a specific thing or type; for example, the train is an hour late. By __comparison/contrast__ , the indefinite article in English is any of the words "a", "an" or "some", and the indefinite article indicates a non-specific thing; for example, would you please pass me an apple. We always __recede/precede__ a word with "a" if it doesn't start with a vowel sound. For example, take a hike; I'm spending a Weekend at Burnie's; or there's a Knight in Shining Armour. Similarly, we precede words with the indefinite article "an" if they do start with a vowel sound, for example, an ostrich, an __eternal/enormous__ mess or an Occupational Health and Safety Policy.</t>
   </si>
   <si>
-    <t>What's an article? I was asking myself this very question in the post office yesterday, standing in line waiting to sign for, as it so happens, an article. A postal article. Not the postal article. Now before we get ahead of ourselves, an article in English is a verb that precedes a noun, and simply indicates specificity. This sounds quite complicated, and to be honest, it's quite complicated to say without spraying everyone within 15 feet, but the concept's quite simple. The definite article in English is the word "the", and indicates a specific thing or type; for example, the train is an hour late. By comparison , the indefinite article in English is any of the words "a", "an" or "some", and the indefinite article indicates a non-specific thing; for example, would you please pass me an apple. We always recede a word with "a" if it doesn't start with a vowel sound. For example, take a hike; I'm spending a Weekend at Burnie's; or there's a Knight in Shining Armour. Similarly, we precede words with the indefinite article "an" if they do start with a vowel sound, for example, an ostrich, an eternal mess or an Occupational Health and Safety Policy.</t>
+    <t>What's an article? I was asking myself this very question in the post office yesterday, standing in line waiting to sign for, as it so happens, an article. A postal article. Not the postal article. Now before we get ahead of ourselves, an article in English is a word that precedes a noun, and simply indicates specificity. This sounds quite complicated, and to be honest, it's quite complicated to say without spraying everyone within 15 feet, but the concept's quite simple. The definite article in English is the word "the", and indicates a specific thing or type; for example, the train is an hour late. By contrast , the indefinite article in English is any of the words "a", "an" or "some", and the indefinite article indicates a non-specific thing; for example, would you please pass me an apple. We always precede a word with "a" if it doesn't start with a vowel sound. For example, take a hike; I'm spending a Weekend at Burnie's; or there's a Knight in Shining Armour. Similarly, we precede words with the indefinite article "an" if they do start with a vowel sound, for example, an ostrich, an enormous mess or an Occupational Health and Safety Policy.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This question tests your ability to distinguish between words that are commonly confused (homophones or near-homophones) and specific lexical knowledge. The incorrect words listed in the transcript do not match the vocabulary spoken by the speaker, even though they might sound similar or fit the general topic. Here is a detailed breakdown of each correction:&lt;/p&gt;
@@ -775,7 +775,7 @@
     <t>The term pygmy usually refers to a few groups of __damaged/short-statured__ people in __reportorial/equatorial__ rain forest regions in Africa. The existence of distinct populations of such people presented scientists with the opportunity to study the mechanisms by which typical human growth patterns have become altered there. And they discovered that two groups became small in two __legitimate/different__ ways. The study is in the journal Nature Communications. The __priestesses/researchers__ collected data on some 500 members of a west African ethnic group called the Baka. They discovered that Baka infants have a similar size range to most other infants, but have a low growth rate during their first two years, which produces a lasting effect. This mechanism seems to be different from that of the east African groups called the Efé and Sua. These peoples have slow __flavourful/prenatal__ growth, so that the infants are born smaller. The researchers say that the Baka population appears to have split from the Efé and Sua some 20,000 years ago. The two different systems for achieving small stature—which appears to be advantageous in the equatorial rainforest environment—are thus an example of convergent evolution. The researchers believe the findings say something important about human evolution and development in general: "Homo sapiens could therefore be characterized by its high __lottery/capacity__ for growth plasticity during infancy. This capacity, which may be unique to our species, may have played a fundamental role in the __musicological/biological__ adaptation that enabled its worldwide expansion and occupation of dissimilar environments within a short period after moving out of Africa."</t>
   </si>
   <si>
-    <t>The term pygmy usually refers to a few groups of damaged people in reportorial rain forest regions in Africa. The existence of distinct populations of such people presented scientists with the opportunity to study the mechanisms by which typical human growth patterns have become altered there. And they discovered that two groups became small in two legitimate ways. The study is in the journal Nature Communications. The priestesses collected data on some 500 members of a west African ethnic group called the Baka. They discovered that Baka infants have a similar size range to most other infants, but have a low growth rate during their first two years, which produces a lasting effect. This mechanism seems to be different from that of the east African groups called the Efé and Sua. These peoples have slow flavourful growth, so that the infants are born smaller. The researchers say that the Baka population appears to have split from the Efé and Sua some 20,000 years ago. The two different systems for achieving small stature—which appears to be advantageous in the equatorial rainforest environment—are thus an example of convergent evolution. The researchers believe the findings say something important about human evolution and development in general: "Homo sapiens could therefore be characterized by its high lottery for growth plasticity during infancy. This capacity, which may be unique to our species, may have played a fundamental role in the musicological adaptation that enabled its worldwide expansion and occupation of dissimilar environments within a short period after moving out of Africa."</t>
+    <t>The term pygmy usually refers to a few groups of short-statured people in equatorial rain forest regions in Africa. The existence of distinct populations of such people presented scientists with the opportunity to study the mechanisms by which typical human growth patterns have become altered there. And they discovered that two groups became small in two different ways. The study is in the journal Nature Communications. The researchers collected data on some 500 members of a west African ethnic group called the Baka. They discovered that Baka infants have a similar size range to most other infants, but have a low growth rate during their first two years, which produces a lasting effect. This mechanism seems to be different from that of the east African groups called the Efé and Sua. These peoples have slow prenatal growth, so that the infants are born smaller. The researchers say that the Baka population appears to have split from the Efé and Sua some 20,000 years ago. The two different systems for achieving small stature—which appears to be advantageous in the equatorial rainforest environment—are thus an example of convergent evolution. The researchers believe the findings say something important about human evolution and development in general: "Homo sapiens could therefore be characterized by its high capacity for growth plasticity during infancy. This capacity, which may be unique to our species, may have played a fundamental role in the biological adaptation that enabled its worldwide expansion and occupation of dissimilar environments within a short period after moving out of Africa."</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;📚 PTE Listening Mastery: Incorrect Words Correction&lt;/h3&gt;
@@ -814,7 +814,7 @@
     <t>It's an approach to pest control that's so crazy it just might work: convince the females that they're virgins. It would be useless as human birth control, of course, but the difference is that most female insects completely change their __payer/behavior__ after sex. For example, some __placebos/mosquitoes__ suck blood. Others lose interest in males and start laying eggs. What's behind this __anoxic/dramatic__ change in behavior? Turns out it's a peptide in the males' seminal fluid. And now researchers in Vienna have found the females' __nether/receptor__ for this peptide. They report online in Nature that __metabolites/fruitflies__ without the receptor lay many fewer eggs and continue to be interested in sex. In other words, they act . So, back to pest control. Most female insects should have this sort of receptor, __duding/including__ the kinds that spread disease and devastate crops. If we could deactivate it on a large scale, instead of __customizing/fighting__ egg-laying blood-suckers, we could live in peace with born-again virgins.</t>
   </si>
   <si>
-    <t>It's an approach to pest control that's so crazy it just might work: convince the females that they're virgins. It would be useless as human birth control, of course, but the difference is that most female insects completely change their payer after sex. For example, some placebos suck blood. Others lose interest in males and start laying eggs. What's behind this anoxic change in behavior? Turns out it's a peptide in the males' seminal fluid. And now researchers in Vienna have found the females' nether for this peptide. They report online in Nature that metabolites without the receptor lay many fewer eggs and continue to be interested in sex. In other words, they act . So, back to pest control. Most female insects should have this sort of receptor, duding the kinds that spread disease and devastate crops. If we could deactivate it on a large scale, instead of customizing egg-laying blood-suckers, we could live in peace with born-again virgins.</t>
+    <t>It's an approach to pest control that's so crazy it just might work: convince the females that they're virgins. It would be useless as human birth control, of course, but the difference is that most female insects completely change their behavior after sex. For example, some mosquitoes suck blood. Others lose interest in males and start laying eggs. What's behind this dramatic change in behavior? Turns out it's a peptide in the males' seminal fluid. And now researchers in Vienna have found the females' receptor for this peptide. They report online in Nature that fruitflies without the receptor lay many fewer eggs and continue to be interested in sex. In other words, they act . So, back to pest control. Most female insects should have this sort of receptor, including the kinds that spread disease and devastate crops. If we could deactivate it on a large scale, instead of fighting egg-laying blood-suckers, we could live in peace with born-again virgins.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;💡 PTE Listening Strategy: Analyzing Spoken vs. Written Words&lt;/h3&gt;
@@ -886,7 +886,7 @@
     <t>Olive oil is thought to be healthy because it's mostly monounsaturated fat. But cold-pressed __cohabiting/extra-virgin__ olive oil may have an extra benefit: it appears to be more filling than other fats. That's according to research presented at a German symposium on fat. Researchers started by feeding 120 __wisps/volunteers__ a daily, 18-ounce serving of low-fat yogurt. But mixed in the yogurt were three __pantaloons/tablespoons__ of extra-virgin olive oil, canola oil, butter, or lard. Turns out volunteers in the olive oil group reported feeling more full during the __obstructs/three-month__ study period. And they had larger concentrations of serotonin in their blood—a signal of satiety. The __multivitamins/researchers__ say extra-virgin olive oil contains aromatic compounds that block the absorption of glucose from the blood, delaying the __goblets/recurrence__ of hunger. Indeed, study subjects who ate yogurt with just olive oil extract consumed fewer calories over a three-month period than those who ate plain yogurt. And they finished the trial with less body fat too. Which leads these researchers to conclude that olive oil extract could be key to creating a better low-fat snack: tastes great, more filling.</t>
   </si>
   <si>
-    <t>Olive oil is thought to be healthy because it's mostly monounsaturated fat. But cold-pressed cohabiting olive oil may have an extra benefit: it appears to be more filling than other fats. That's according to research presented at a German symposium on fat. Researchers started by feeding 120 wisps a daily, 18-ounce serving of low-fat yogurt. But mixed in the yogurt were three pantaloons of extra-virgin olive oil, canola oil, butter, or lard. Turns out volunteers in the olive oil group reported feeling more full during the obstructs study period. And they had larger concentrations of serotonin in their blood—a signal of satiety. The multivitamins say extra-virgin olive oil contains aromatic compounds that block the absorption of glucose from the blood, delaying the goblets of hunger. Indeed, study subjects who ate yogurt with just olive oil extract consumed fewer calories over a three-month period than those who ate plain yogurt. And they finished the trial with less body fat too. Which leads these researchers to conclude that olive oil extract could be key to creating a better low-fat snack: tastes great, more filling.</t>
+    <t>Olive oil is thought to be healthy because it's mostly monounsaturated fat. But cold-pressed extra-virgin olive oil may have an extra benefit: it appears to be more filling than other fats. That's according to research presented at a German symposium on fat. Researchers started by feeding 120 volunteers a daily, 18-ounce serving of low-fat yogurt. But mixed in the yogurt were three tablespoons of extra-virgin olive oil, canola oil, butter, or lard. Turns out volunteers in the olive oil group reported feeling more full during the three-month study period. And they had larger concentrations of serotonin in their blood—a signal of satiety. The researchers say extra-virgin olive oil contains aromatic compounds that block the absorption of glucose from the blood, delaying the recurrence of hunger. Indeed, study subjects who ate yogurt with just olive oil extract consumed fewer calories over a three-month period than those who ate plain yogurt. And they finished the trial with less body fat too. Which leads these researchers to conclude that olive oil extract could be key to creating a better low-fat snack: tastes great, more filling.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🎯 Analysis of Incorrect Words (Highlighting Skills)&lt;/h3&gt;
@@ -932,7 +932,7 @@
     <t>"Our health care is too costly…and each day brings further evidence that the ways we use energy __magician/strengthen__ our __lamaseries/adversaries__ and threaten our planet… "We will build the roads and bridges, the electric grids and digital lines that feed our commerce and bind us together. We will restore science to its __firewall/rightful__ place and wield technology's wonders to raise health care's quality and lower its costs. We will harness the sun and the winds and the soil to fuel our cars and run our factories. And we will transform our schools and colleges and universities to meet the demands of a new age… "Our __conductresses/challenges__ may be new, the instruments with which we meet them may be new, but those values upon which our success depends, honesty and hard work, courage and fair play, tolerance and curiosity, loyalty and patriotism—these things are old. These things are true."</t>
   </si>
   <si>
-    <t>"Our health care is too costly…and each day brings further evidence that the ways we use energy magician our lamaseries and threaten our planet… "We will build the roads and bridges, the electric grids and digital lines that feed our commerce and bind us together. We will restore science to its firewall place and wield technology's wonders to raise health care's quality and lower its costs. We will harness the sun and the winds and the soil to fuel our cars and run our factories. And we will transform our schools and colleges and universities to meet the demands of a new age… "Our conductresses may be new, the instruments with which we meet them may be new, but those values upon which our success depends, honesty and hard work, courage and fair play, tolerance and curiosity, loyalty and patriotism—these things are old. These things are true."</t>
+    <t>"Our health care is too costly…and each day brings further evidence that the ways we use energy strengthen our adversaries and threaten our planet… "We will build the roads and bridges, the electric grids and digital lines that feed our commerce and bind us together. We will restore science to its rightful place and wield technology's wonders to raise health care's quality and lower its costs. We will harness the sun and the winds and the soil to fuel our cars and run our factories. And we will transform our schools and colleges and universities to meet the demands of a new age… "Our challenges may be new, the instruments with which we meet them may be new, but those values upon which our success depends, honesty and hard work, courage and fair play, tolerance and curiosity, loyalty and patriotism—these things are old. These things are true."</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🎧 PTE Listening: Highlight Incorrect Words Analysis&lt;/h3&gt;
@@ -979,7 +979,7 @@
     <t>Emphysema and cystic fibrosis patients who need new lungs are faced with a life-threatening problem: more than 80 percent of donated lungs can't be used—they're inflamed and barely functional. But a new approach, detailed this week in the new journal Science Translational Medicine, describes a novel gene therapy that can repair these damaged lungs—and make them __confrontational/available__ for transplant. Researchers first developed a system for preserving the lungs. They put the organs in a glass chamber and kept them functioning and at human body temperature. This technique proved better than freezing. Then they inserted into the lungs a gene IL-10. The gene plays a key role in __crippling/inhibiting__ the immune response. About six hours after injection, the cells start producing __zlotys/proteins__ that combat the __blandishing/damaging__ inflammation. The presence of the IL-10 gene may also lower the chances that the recipient of the lung will reject the transplanted organ. After the gene therapy, treated lungs showed improved blood flow and were significantly better at taking in oxygen and expelling carbon dioxide. The technique could double the number of lungs available for transplant, truly making patients breathe easier.</t>
   </si>
   <si>
-    <t>Emphysema and cystic fibrosis patients who need new lungs are faced with a life-threatening problem: more than 80 percent of donated lungs can't be used—they're inflamed and barely functional. But a new approach, detailed this week in the new journal Science Translational Medicine, describes a novel gene therapy that can repair these damaged lungs—and make them confrontational for transplant. Researchers first developed a system for preserving the lungs. They put the organs in a glass chamber and kept them functioning and at human body temperature. This technique proved better than freezing. Then they inserted into the lungs a gene IL-10. The gene plays a key role in crippling the immune response. About six hours after injection, the cells start producing zlotys that combat the blandishing inflammation. The presence of the IL-10 gene may also lower the chances that the recipient of the lung will reject the transplanted organ. After the gene therapy, treated lungs showed improved blood flow and were significantly better at taking in oxygen and expelling carbon dioxide. The technique could double the number of lungs available for transplant, truly making patients breathe easier.</t>
+    <t>Emphysema and cystic fibrosis patients who need new lungs are faced with a life-threatening problem: more than 80 percent of donated lungs can't be used—they're inflamed and barely functional. But a new approach, detailed this week in the new journal Science Translational Medicine, describes a novel gene therapy that can repair these damaged lungs—and make them available for transplant. Researchers first developed a system for preserving the lungs. They put the organs in a glass chamber and kept them functioning and at human body temperature. This technique proved better than freezing. Then they inserted into the lungs a gene IL-10. The gene plays a key role in inhibiting the immune response. About six hours after injection, the cells start producing proteins that combat the damaging inflammation. The presence of the IL-10 gene may also lower the chances that the recipient of the lung will reject the transplanted organ. After the gene therapy, treated lungs showed improved blood flow and were significantly better at taking in oxygen and expelling carbon dioxide. The technique could double the number of lungs available for transplant, truly making patients breathe easier.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🌟 PTE Listening Analysis: Highlight Incorrect Words 🌟&lt;/h3&gt;
@@ -1015,7 +1015,7 @@
     <t>Harold Kroto won the Nobel Prize in Chemistry in 1996 for the discovery of buckminsterfullerene, the soccer ball shaped form of carbon better known as buckyballs. On June 28, he spoke to students about science as a __expansible/philosophical__ construct: "I'm going to talk about what science is because it's a totally misunderstood sort of subject. There are aspects of science which are important, and of course we know the body of knowledge that you learn at school, alright. The applications of those knowledge, technology, the only thing that journalists ever ask, in general, 99 percent of the time. "Perhaps most __comported/important__ is that it's the way that we discover new knowledge. But for me the most important, by far, is that it's the only philosophical __thermostat/construct__ we have to determine truth with any degree of reliability. Think about that. Because then it becomes a much bigger subject. In fact, for me, perhaps the most important subject there is. And the ethical purpose of education must involve teaching __crucifixion/children__ how they can decide what they're being told is actually true. And that's not the case in general. The teaching of a skeptical, evidence-based assessment of all claims--all claims--without exception is __verily/fundamentally__ an intellectual __essentially/integrity__ issue. Without evidence, anything goes.Think about it. "Common sense says the sun goes around the Earth. Who agrees with me? Look at it! Starts over here, ends over there. It's uncommon sense that was needed to recognize that the Earth was turning on its axis. The uncommon sense of Copernicus, Galileo and Giordano Bruno, who burned to death. We have to learn to be very careful and to question everything. Let me just __snowplough/check—how__ many of you know the evidence for Galileo to say that the Earth was going around the sun? Put your hand up. You've accepted it. Almost nobody's put their hand up. It's incredible. Look at yourself, you've accepted this. You've accepted a lot of things without evidence. Find out what the evidence is for that, and find out what the evidence is for everything that you accept."</t>
   </si>
   <si>
-    <t>Harold Kroto won the Nobel Prize in Chemistry in 1996 for the discovery of buckminsterfullerene, the soccer ball shaped form of carbon better known as buckyballs. On June 28, he spoke to students about science as a expansible construct: "I'm going to talk about what science is because it's a totally misunderstood sort of subject. There are aspects of science which are important, and of course we know the body of knowledge that you learn at school, alright. The applications of those knowledge, technology, the only thing that journalists ever ask, in general, 99 percent of the time. "Perhaps most comported is that it's the way that we discover new knowledge. But for me the most important, by far, is that it's the only philosophical thermostat we have to determine truth with any degree of reliability. Think about that. Because then it becomes a much bigger subject. In fact, for me, perhaps the most important subject there is. And the ethical purpose of education must involve teaching crucifixion how they can decide what they're being told is actually true. And that's not the case in general. The teaching of a skeptical, evidence-based assessment of all claims--all claims--without exception is verily an intellectual essentially issue. Without evidence, anything goes.Think about it. "Common sense says the sun goes around the Earth. Who agrees with me? Look at it! Starts over here, ends over there. It's uncommon sense that was needed to recognize that the Earth was turning on its axis. The uncommon sense of Copernicus, Galileo and Giordano Bruno, who burned to death. We have to learn to be very careful and to question everything. Let me just snowplough many of you know the evidence for Galileo to say that the Earth was going around the sun? Put your hand up. You've accepted it. Almost nobody's put their hand up. It's incredible. Look at yourself, you've accepted this. You've accepted a lot of things without evidence. Find out what the evidence is for that, and find out what the evidence is for everything that you accept."</t>
+    <t>Harold Kroto won the Nobel Prize in Chemistry in 1996 for the discovery of buckminsterfullerene, the soccer ball shaped form of carbon better known as buckyballs. On June 28, he spoke to students about science as a philosophical construct: "I'm going to talk about what science is because it's a totally misunderstood sort of subject. There are aspects of science which are important, and of course we know the body of knowledge that you learn at school, alright. The applications of those knowledge, technology, the only thing that journalists ever ask, in general, 99 percent of the time. "Perhaps most important is that it's the way that we discover new knowledge. But for me the most important, by far, is that it's the only philosophical construct we have to determine truth with any degree of reliability. Think about that. Because then it becomes a much bigger subject. In fact, for me, perhaps the most important subject there is. And the ethical purpose of education must involve teaching children how they can decide what they're being told is actually true. And that's not the case in general. The teaching of a skeptical, evidence-based assessment of all claims--all claims--without exception is fundamentally an intellectual integrity issue. Without evidence, anything goes.Think about it. "Common sense says the sun goes around the Earth. Who agrees with me? Look at it! Starts over here, ends over there. It's uncommon sense that was needed to recognize that the Earth was turning on its axis. The uncommon sense of Copernicus, Galileo and Giordano Bruno, who burned to death. We have to learn to be very careful and to question everything. Let me just check—how many of you know the evidence for Galileo to say that the Earth was going around the sun? Put your hand up. You've accepted it. Almost nobody's put their hand up. It's incredible. Look at yourself, you've accepted this. You've accepted a lot of things without evidence. Find out what the evidence is for that, and find out what the evidence is for everything that you accept."</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your PTE Academic teacher, I understand how frustrating it can be when the words in the transcript don't match what the speaker actually says. This specific question tests your ability to listen critically and recognize phonological or lexical discrepancies. Don't worry; with practice, you'll master these subtle differences!&lt;/p&gt;
@@ -1063,7 +1063,7 @@
     <t>Did you hoist a few on New Year's? Of course, getting together with friends over a few adult beverages has a long history. Here's the University of Cincinnati's Kathleen Lynch, on the ancient Greek symposium: "And the symposium is an all-male __confessing/drinking__ event. It's a time where a small group of men get together, usually at the home of a friend. And the focus is on drinking. And so they may have had some food earlier, but the focus is on drinking together. And the drinking together forms bonds." On January 7th, Lynch __transitions/lectures__ at the meeting of the Archaeological Institute of America on the types of cups used at symposia over the centuries and how they give us clues to what was going on in Greece at __signature/particular__ times. As for the symposium, it had a couple of definite rules. First, participants __unsupervised/reclined__ and arranged themselves in a circle or square. There was thus no obvious head of the table, and everyone __shop/involved__ had an equal status. Second, everyone drank together in rounds, so everyone got drunk at about the same rate. This communal and equitable inebriation led to a common loss of inhibitions and the __imprinting/building__ of, well, a fraternity.</t>
   </si>
   <si>
-    <t>Did you hoist a few on New Year's? Of course, getting together with friends over a few adult beverages has a long history. Here's the University of Cincinnati's Kathleen Lynch, on the ancient Greek symposium: "And the symposium is an all-male confessing event. It's a time where a small group of men get together, usually at the home of a friend. And the focus is on drinking. And so they may have had some food earlier, but the focus is on drinking together. And the drinking together forms bonds." On January 7th, Lynch transitions at the meeting of the Archaeological Institute of America on the types of cups used at symposia over the centuries and how they give us clues to what was going on in Greece at signature times. As for the symposium, it had a couple of definite rules. First, participants unsupervised and arranged themselves in a circle or square. There was thus no obvious head of the table, and everyone shop had an equal status. Second, everyone drank together in rounds, so everyone got drunk at about the same rate. This communal and equitable inebriation led to a common loss of inhibitions and the imprinting of, well, a fraternity.</t>
+    <t>Did you hoist a few on New Year's? Of course, getting together with friends over a few adult beverages has a long history. Here's the University of Cincinnati's Kathleen Lynch, on the ancient Greek symposium: "And the symposium is an all-male drinking event. It's a time where a small group of men get together, usually at the home of a friend. And the focus is on drinking. And so they may have had some food earlier, but the focus is on drinking together. And the drinking together forms bonds." On January 7th, Lynch lectures at the meeting of the Archaeological Institute of America on the types of cups used at symposia over the centuries and how they give us clues to what was going on in Greece at particular times. As for the symposium, it had a couple of definite rules. First, participants reclined and arranged themselves in a circle or square. There was thus no obvious head of the table, and everyone involved had an equal status. Second, everyone drank together in rounds, so everyone got drunk at about the same rate. This communal and equitable inebriation led to a common loss of inhibitions and the building of, well, a fraternity.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🔍 Listening Strategy Breakdown: Incorrect Words&lt;/h3&gt;
@@ -1113,7 +1113,7 @@
     <t>Scientists discover new species all the time—on the order of 15,000 a year. One of the latest additions to the tree of life is a new type of leopard frog. Which might sound unremarkable, except for where it was found: New York City. But how does a frog go __coded/unnoticed__ in the Big Apple? Well even experts have a hard time telling this new species from its __refrozen/northern__ and southern cousins on looks alone. But the new guy has a __baronet/different__ croak, which raised ecologists' suspicions. So they tracked down four leopard frog populations with the unique call—including one within view of the Statue of Liberty—and took DNA samples. As they suspected, the odd croakers weren't southern or northern leopard frogs, or even a mix. They had a genetic ancestry of their own—earning them new species status. Those results appear in the journal Molecular Phylogenetics and Evolution. The frogs are tough New Yorkers—the center of their range appears to be Yankee Stadium. But the __inveiglers/researchers__ say that the urban amphibians face threats like __advise/pesticides__ and infectious diseases. Not to mention real-life games of Frogger.</t>
   </si>
   <si>
-    <t>Scientists discover new species all the time—on the order of 15,000 a year. One of the latest additions to the tree of life is a new type of leopard frog. Which might sound unremarkable, except for where it was found: New York City. But how does a frog go coded in the Big Apple? Well even experts have a hard time telling this new species from its refrozen and southern cousins on looks alone. But the new guy has a baronet croak, which raised ecologists' suspicions. So they tracked down four leopard frog populations with the unique call—including one within view of the Statue of Liberty—and took DNA samples. As they suspected, the odd croakers weren't southern or northern leopard frogs, or even a mix. They had a genetic ancestry of their own—earning them new species status. Those results appear in the journal Molecular Phylogenetics and Evolution. The frogs are tough New Yorkers—the center of their range appears to be Yankee Stadium. But the inveiglers say that the urban amphibians face threats like advise and infectious diseases. Not to mention real-life games of Frogger.</t>
+    <t>Scientists discover new species all the time—on the order of 15,000 a year. One of the latest additions to the tree of life is a new type of leopard frog. Which might sound unremarkable, except for where it was found: New York City. But how does a frog go unnoticed in the Big Apple? Well even experts have a hard time telling this new species from its northern and southern cousins on looks alone. But the new guy has a different croak, which raised ecologists' suspicions. So they tracked down four leopard frog populations with the unique call—including one within view of the Statue of Liberty—and took DNA samples. As they suspected, the odd croakers weren't southern or northern leopard frogs, or even a mix. They had a genetic ancestry of their own—earning them new species status. Those results appear in the journal Molecular Phylogenetics and Evolution. The frogs are tough New Yorkers—the center of their range appears to be Yankee Stadium. But the researchers say that the urban amphibians face threats like pesticides and infectious diseases. Not to mention real-life games of Frogger.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;As a premium PTE Academic teacher, I can provide a detailed breakdown of why these words were highlighted as incorrect. In this task, you must rely entirely on listening comprehension and phonetic accuracy, as the highlighted words often sound similar to the correct spoken alternatives.&lt;/p&gt;
@@ -1154,7 +1154,7 @@
     <t>Modern humans are masters of multitasking. We eat while driving, watch TV while studying, and of course talk on our cell phones while doing, well, everything. How do we do it? A study in the July 16th issue of Neuron suggests that though we can train our brains to work faster as we juggle, we never actually manage to do more than one thing at a time. Our brains aren't really built to handle the sort of parallel processing we think we're capable of. The good news is: studies have shown that __submissive/extensive__ training can make us better at doing two things at once. But how? One theory is that with lots of practice some routines become "automatic." And if we don't need to run every little thing past the part of the brain that's spends time __spelling/thinking__ about stuff, we can multitask just fine. But this new study finds that that's not the way it works. Turns out that __coffers/multitaskers__ still consult the prefrontal cortex, but training gets the "Thinking Brain" to think a little faster. So we're actually switching tasks quickly enough to appear to be doing them simultaneously. Which is still nothing to shake a stick and sneeze at.</t>
   </si>
   <si>
-    <t>Modern humans are masters of multitasking. We eat while driving, watch TV while studying, and of course talk on our cell phones while doing, well, everything. How do we do it? A study in the July 16th issue of Neuron suggests that though we can train our brains to work faster as we juggle, we never actually manage to do more than one thing at a time. Our brains aren't really built to handle the sort of parallel processing we think we're capable of. The good news is: studies have shown that submissive training can make us better at doing two things at once. But how? One theory is that with lots of practice some routines become "automatic." And if we don't need to run every little thing past the part of the brain that's spends time spelling about stuff, we can multitask just fine. But this new study finds that that's not the way it works. Turns out that coffers still consult the prefrontal cortex, but training gets the "Thinking Brain" to think a little faster. So we're actually switching tasks quickly enough to appear to be doing them simultaneously. Which is still nothing to shake a stick and sneeze at.</t>
+    <t>Modern humans are masters of multitasking. We eat while driving, watch TV while studying, and of course talk on our cell phones while doing, well, everything. How do we do it? A study in the July 16th issue of Neuron suggests that though we can train our brains to work faster as we juggle, we never actually manage to do more than one thing at a time. Our brains aren't really built to handle the sort of parallel processing we think we're capable of. The good news is: studies have shown that extensive training can make us better at doing two things at once. But how? One theory is that with lots of practice some routines become "automatic." And if we don't need to run every little thing past the part of the brain that's spends time thinking about stuff, we can multitask just fine. But this new study finds that that's not the way it works. Turns out that multitaskers still consult the prefrontal cortex, but training gets the "Thinking Brain" to think a little faster. So we're actually switching tasks quickly enough to appear to be doing them simultaneously. Which is still nothing to shake a stick and sneeze at.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🎧 Listening Highlight: Incorrect Words Correction Guide&lt;/h3&gt;
@@ -1193,7 +1193,7 @@
     <t>This year, the number of mobile phones on cell networks is __remembered/expected__ to surpass the Earth's population. "More people now own cell phones than actually have access to working toilets." James Meadow, a microbial ecologist at the University of Oregon. Hidden in the data is the reality that some people work on their phones…on toilets. If that grosses you out, consider this: "So it turns out we're just really leaky animals. We just, we leave our __linear/bacteria__ everywhere we go." Including, of course, our phones. Meadow and his colleagues took a census of the bacteria on thumbs and index fingers of 17 volunteers—and on their smartphone touch screens. Overall, they ID'ed more than 7,000 types. Looking at just the most common bacteria, those that appear more than 0.1 percent of the time, they found an 82 percent similarity between the __overtones/microbiomes__ of fingers and phones. Meaning our phones are a pretty good mirror of ourselves, microbially, at least. The results appear in the journal PeerJ. "We have always been covered in bacteria… and we will always be covered in bacteria." So the fact that our phones are also covered in bacteria is no reason for concern. In fact, the __reasoners/researchers__ say that mobile phones may hold untapped potential as __poison/personal__ microbiome sensors.</t>
   </si>
   <si>
-    <t>This year, the number of mobile phones on cell networks is remembered to surpass the Earth's population. "More people now own cell phones than actually have access to working toilets." James Meadow, a microbial ecologist at the University of Oregon. Hidden in the data is the reality that some people work on their phones…on toilets. If that grosses you out, consider this: "So it turns out we're just really leaky animals. We just, we leave our linear everywhere we go." Including, of course, our phones. Meadow and his colleagues took a census of the bacteria on thumbs and index fingers of 17 volunteers—and on their smartphone touch screens. Overall, they ID'ed more than 7,000 types. Looking at just the most common bacteria, those that appear more than 0.1 percent of the time, they found an 82 percent similarity between the overtones of fingers and phones. Meaning our phones are a pretty good mirror of ourselves, microbially, at least. The results appear in the journal PeerJ. "We have always been covered in bacteria… and we will always be covered in bacteria." So the fact that our phones are also covered in bacteria is no reason for concern. In fact, the reasoners say that mobile phones may hold untapped potential as poison microbiome sensors.</t>
+    <t>This year, the number of mobile phones on cell networks is expected to surpass the Earth's population. "More people now own cell phones than actually have access to working toilets." James Meadow, a microbial ecologist at the University of Oregon. Hidden in the data is the reality that some people work on their phones…on toilets. If that grosses you out, consider this: "So it turns out we're just really leaky animals. We just, we leave our bacteria everywhere we go." Including, of course, our phones. Meadow and his colleagues took a census of the bacteria on thumbs and index fingers of 17 volunteers—and on their smartphone touch screens. Overall, they ID'ed more than 7,000 types. Looking at just the most common bacteria, those that appear more than 0.1 percent of the time, they found an 82 percent similarity between the microbiomes of fingers and phones. Meaning our phones are a pretty good mirror of ourselves, microbially, at least. The results appear in the journal PeerJ. "We have always been covered in bacteria… and we will always be covered in bacteria." So the fact that our phones are also covered in bacteria is no reason for concern. In fact, the researchers say that mobile phones may hold untapped potential as personal microbiome sensors.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This question tests your ability to differentiate between phonetically similar words that have different meanings and parts of speech. In this specific question type, the error is not always a pronunciation issue; often, the incorrect word simply makes no contextual or semantic sense based on the discussion (e.g., confusing a scientific noun with a common adjective).&lt;/p&gt;
@@ -1233,7 +1233,7 @@
     <t>Ah, daydreaming. Is there anything more __breasted/pleasant__ than sitting back and letting your thoughts drift? Well, yes: not letting your thoughts drift, for one. Because according to a study published in the journal Science, people are least happy when their minds wander. Humans, to a degree unmatched by other animals, are capable of __imprinting/thinking__ about things outside the here and now—something that happened yesterday, or __converging/something__ they hope will happen tomorrow. It's that sort of itinerant __intersect/intellect__ that allows us to plan and to learn. But at what cost? Psychologists at Harvard used an iPhone app to find out. At random times throughout the day, the program asked some 2,200 participants what they were doing, what they were thinking about and how they felt. Turns out that people spend nearly half their waking hours thinking about something other than what they're doing. And that whether and where their thoughts tend to stray is a better predictor of their feelings than what they're __irrecoverably/actually__ up to. The __rightfulness/scientists__ conclude that a wandering mind is an unhappy mind. So try to focus on, and live in, the present. You might __plumber/discover__ that happiness is just being where it's happening.</t>
   </si>
   <si>
-    <t>Ah, daydreaming. Is there anything more breasted than sitting back and letting your thoughts drift? Well, yes: not letting your thoughts drift, for one. Because according to a study published in the journal Science, people are least happy when their minds wander. Humans, to a degree unmatched by other animals, are capable of imprinting about things outside the here and now—something that happened yesterday, or converging they hope will happen tomorrow. It's that sort of itinerant intersect that allows us to plan and to learn. But at what cost? Psychologists at Harvard used an iPhone app to find out. At random times throughout the day, the program asked some 2,200 participants what they were doing, what they were thinking about and how they felt. Turns out that people spend nearly half their waking hours thinking about something other than what they're doing. And that whether and where their thoughts tend to stray is a better predictor of their feelings than what they're irrecoverably up to. The rightfulness conclude that a wandering mind is an unhappy mind. So try to focus on, and live in, the present. You might plumber that happiness is just being where it's happening.</t>
+    <t>Ah, daydreaming. Is there anything more pleasant than sitting back and letting your thoughts drift? Well, yes: not letting your thoughts drift, for one. Because according to a study published in the journal Science, people are least happy when their minds wander. Humans, to a degree unmatched by other animals, are capable of thinking about things outside the here and now—something that happened yesterday, or something they hope will happen tomorrow. It's that sort of itinerant intellect that allows us to plan and to learn. But at what cost? Psychologists at Harvard used an iPhone app to find out. At random times throughout the day, the program asked some 2,200 participants what they were doing, what they were thinking about and how they felt. Turns out that people spend nearly half their waking hours thinking about something other than what they're doing. And that whether and where their thoughts tend to stray is a better predictor of their feelings than what they're actually up to. The scientists conclude that a wandering mind is an unhappy mind. So try to focus on, and live in, the present. You might discover that happiness is just being where it's happening.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;As a premium PTE teacher, I want to assure you that these types of questions test your listening comprehension &lt;strong&gt;and&lt;/strong&gt; your ability to recognize subtle phonetic and contextual shifts in English. When a word in the transcript is highlighted incorrectly, it means the speaker pronounced a different word that made perfect sense in the context.&lt;/p&gt;
@@ -1289,7 +1289,7 @@
     <t>Medicinal tablets are nothing new. Doctors have been __filming/dispensing__ pills for thousands of years. And now archaeologists have turned up some of those ancient medicines, which were preserved in a shipwreck for close to two millennia. The 2nd-century Pozzino wreck was discovered in 1974 off the coast of Italy. It's cargo included medical __chestnut/equipment__ like a cupping vessel, iron probe, and tin boxes of supplies. And in one of those boxes, researchers recovered five gray tablets. Now, they've analyzed the antique medication. The work is in the Proceedings of the National Academy of Sciences. The pills primarily contained zinc compounds, probably the active medicinal ingredients. But researchers also detected starch, pollen, charcoal, fats and linen fibers. Those fibers helped the tablets hold their round, loaf-like shape, which may be the key to the medication's use: the Greek word meaning "small round loaves" also inspired the word collyrium, or eye-wash. The pills were probably either __infarct/dissolved__ in liquid or ground into a powder and used to treat eye conditions. Who knows, maybe Hippocrates used them on his pupils.</t>
   </si>
   <si>
-    <t>Medicinal tablets are nothing new. Doctors have been filming pills for thousands of years. And now archaeologists have turned up some of those ancient medicines, which were preserved in a shipwreck for close to two millennia. The 2nd-century Pozzino wreck was discovered in 1974 off the coast of Italy. It's cargo included medical chestnut like a cupping vessel, iron probe, and tin boxes of supplies. And in one of those boxes, researchers recovered five gray tablets. Now, they've analyzed the antique medication. The work is in the Proceedings of the National Academy of Sciences. The pills primarily contained zinc compounds, probably the active medicinal ingredients. But researchers also detected starch, pollen, charcoal, fats and linen fibers. Those fibers helped the tablets hold their round, loaf-like shape, which may be the key to the medication's use: the Greek word meaning "small round loaves" also inspired the word collyrium, or eye-wash. The pills were probably either infarct in liquid or ground into a powder and used to treat eye conditions. Who knows, maybe Hippocrates used them on his pupils.</t>
+    <t>Medicinal tablets are nothing new. Doctors have been dispensing pills for thousands of years. And now archaeologists have turned up some of those ancient medicines, which were preserved in a shipwreck for close to two millennia. The 2nd-century Pozzino wreck was discovered in 1974 off the coast of Italy. It's cargo included medical equipment like a cupping vessel, iron probe, and tin boxes of supplies. And in one of those boxes, researchers recovered five gray tablets. Now, they've analyzed the antique medication. The work is in the Proceedings of the National Academy of Sciences. The pills primarily contained zinc compounds, probably the active medicinal ingredients. But researchers also detected starch, pollen, charcoal, fats and linen fibers. Those fibers helped the tablets hold their round, loaf-like shape, which may be the key to the medication's use: the Greek word meaning "small round loaves" also inspired the word collyrium, or eye-wash. The pills were probably either dissolved in liquid or ground into a powder and used to treat eye conditions. Who knows, maybe Hippocrates used them on his pupils.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🎧 Listening Skill Review: Highlighting Incorrect Words&lt;/h3&gt;
@@ -1326,7 +1326,7 @@
     <t>"That grinning, glowing, __barterer/globular__ invader of your living room is an inhabitant of the pumpkin patch. And if your __warfare/doorbell__ rings and nobody's there, that was no Martian—it's Halloween." That's how Orson Welles ended his Mercury Theater version of HG Well's War of the Worlds on October 30, 1938. The broadcast was designed to sound like live news coverage of an __undertaken/invasion__ of Earth by Martians. And a lot of people fell for it. Now there's some more Martian misinformation fooling folks. This one's not so scary. A lot of people are getting email claiming that in the next few weeks the planet Mars will get close enough to the Earth so that it will appear to be about the same size as the moon. Our friends at Sky and __soloed/Telescope__ magazine report that email dating back to 2003 mentioned that in a 75x magnifying telescope Mars would look about as big as the moon does—to the naked eye. __carfare/Somewhere__ along the line the telescope part got lost. So don't worry. Mars, even at its closest, is still small and safely far away. Welles: "It's Halloween."</t>
   </si>
   <si>
-    <t>"That grinning, glowing, barterer invader of your living room is an inhabitant of the pumpkin patch. And if your warfare rings and nobody's there, that was no Martian—it's Halloween." That's how Orson Welles ended his Mercury Theater version of HG Well's War of the Worlds on October 30, 1938. The broadcast was designed to sound like live news coverage of an undertaken of Earth by Martians. And a lot of people fell for it. Now there's some more Martian misinformation fooling folks. This one's not so scary. A lot of people are getting email claiming that in the next few weeks the planet Mars will get close enough to the Earth so that it will appear to be about the same size as the moon. Our friends at Sky and soloed magazine report that email dating back to 2003 mentioned that in a 75x magnifying telescope Mars would look about as big as the moon does—to the naked eye. carfare along the line the telescope part got lost. So don't worry. Mars, even at its closest, is still small and safely far away. Welles: "It's Halloween."</t>
+    <t>"That grinning, glowing, globular invader of your living room is an inhabitant of the pumpkin patch. And if your doorbell rings and nobody's there, that was no Martian—it's Halloween." That's how Orson Welles ended his Mercury Theater version of HG Well's War of the Worlds on October 30, 1938. The broadcast was designed to sound like live news coverage of an invasion of Earth by Martians. And a lot of people fell for it. Now there's some more Martian misinformation fooling folks. This one's not so scary. A lot of people are getting email claiming that in the next few weeks the planet Mars will get close enough to the Earth so that it will appear to be about the same size as the moon. Our friends at Sky and Telescope magazine report that email dating back to 2003 mentioned that in a 75x magnifying telescope Mars would look about as big as the moon does—to the naked eye. Somewhere along the line the telescope part got lost. So don't worry. Mars, even at its closest, is still small and safely far away. Welles: "It's Halloween."</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🎧 PTE Listening: Incorrect Words Explanation&lt;/h3&gt;
@@ -1371,7 +1371,7 @@
     <t>The __sulfur/Meridiana__ Planum region of Mars once had water that was really salty and highly acidic, conditions incredibly hostile to any life forms that we know about. So any __viscous/organisms__ that might have once lived in that area on Mars would really have had to beat the odds. But why do we know so much about the __deposed/likelihood__ of a __nebular/particular__ environment to support life? Mars scientists can thank you and me and our propensity to eat. Harvard professor of earth and planetary sciences Andrew Knoll spoke to reporters Friday at the AAAS meeting: "The food preservation industry depends highly on people knowing the kind of ionic tolerances of microorganisms. So this isn't some esoteric thing that a Mars scientist will pull a paper off a __half/shelf__ . There are thousands of papers out there on the tolerances of microorganisms. And it's not because most scientists are worried about…it's because they're worried about botulism in canned vegetables." So one science feeds another.</t>
   </si>
   <si>
-    <t>The sulfur Planum region of Mars once had water that was really salty and highly acidic, conditions incredibly hostile to any life forms that we know about. So any viscous that might have once lived in that area on Mars would really have had to beat the odds. But why do we know so much about the deposed of a nebular environment to support life? Mars scientists can thank you and me and our propensity to eat. Harvard professor of earth and planetary sciences Andrew Knoll spoke to reporters Friday at the AAAS meeting: "The food preservation industry depends highly on people knowing the kind of ionic tolerances of microorganisms. So this isn't some esoteric thing that a Mars scientist will pull a paper off a half . There are thousands of papers out there on the tolerances of microorganisms. And it's not because most scientists are worried about…it's because they're worried about botulism in canned vegetables." So one science feeds another.</t>
+    <t>The Meridiana Planum region of Mars once had water that was really salty and highly acidic, conditions incredibly hostile to any life forms that we know about. So any organisms that might have once lived in that area on Mars would really have had to beat the odds. But why do we know so much about the likelihood of a particular environment to support life? Mars scientists can thank you and me and our propensity to eat. Harvard professor of earth and planetary sciences Andrew Knoll spoke to reporters Friday at the AAAS meeting: "The food preservation industry depends highly on people knowing the kind of ionic tolerances of microorganisms. So this isn't some esoteric thing that a Mars scientist will pull a paper off a shelf . There are thousands of papers out there on the tolerances of microorganisms. And it's not because most scientists are worried about…it's because they're worried about botulism in canned vegetables." So one science feeds another.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;As a premium PTE teacher, I can guide you through the subtle differences in pronunciation and context that often trip students up in the Listening Highlight Incorrect Words section. This question tests not just your listening skills, but your understanding of vocabulary, grammar, and domain-specific knowledge (in this case, planetary science).&lt;/p&gt;
@@ -1413,7 +1413,7 @@
     <t>Hybridise __Hybridise/Scientists__ discover new species all the time — on the order of 15,000 a year. One of the latest __directors/additions__ to the tree of life is a new type of leopard frog. Which might sound unremarkable, except for where it was found: New York City. But how does a frog go unnoticed in the Big Apple? Well even experts have a hard time telling this new species from its __promotion/northern__ and southern cousins on looks alone. But the new guy has a __deliberate/different__ croak, which raised ecologists' suspicions. So they tracked down four leopard frog populations with the unique call — including one within view of the Statue of Liberty — and took DNA samples. As they suspected, the odd __pagodas/croakers__ weren't southern or northern leopard frogs, or even a mix. They had a genetic ancestry of their own — earning them new species status. Those results appear in the journal Molecular Phylogenetics and Evolution. The frogs are tough New Yorkers — the center of their range appears to be Yankee Stadium. But the researchers say that the urban __dizziness/amphibians__ face threats like pesticides and infectious diseases. Not to mention __initialize/real-life__ games of Frogger.</t>
   </si>
   <si>
-    <t>Hybridise Hybridise discover new species all the time — on the order of 15,000 a year. One of the latest directors to the tree of life is a new type of leopard frog. Which might sound unremarkable, except for where it was found: New York City. But how does a frog go unnoticed in the Big Apple? Well even experts have a hard time telling this new species from its promotion and southern cousins on looks alone. But the new guy has a deliberate croak, which raised ecologists' suspicions. So they tracked down four leopard frog populations with the unique call — including one within view of the Statue of Liberty — and took DNA samples. As they suspected, the odd pagodas weren't southern or northern leopard frogs, or even a mix. They had a genetic ancestry of their own — earning them new species status. Those results appear in the journal Molecular Phylogenetics and Evolution. The frogs are tough New Yorkers — the center of their range appears to be Yankee Stadium. But the researchers say that the urban dizziness face threats like pesticides and infectious diseases. Not to mention initialize games of Frogger.</t>
+    <t>Hybridise Scientists discover new species all the time — on the order of 15,000 a year. One of the latest additions to the tree of life is a new type of leopard frog. Which might sound unremarkable, except for where it was found: New York City. But how does a frog go unnoticed in the Big Apple? Well even experts have a hard time telling this new species from its northern and southern cousins on looks alone. But the new guy has a different croak, which raised ecologists' suspicions. So they tracked down four leopard frog populations with the unique call — including one within view of the Statue of Liberty — and took DNA samples. As they suspected, the odd croakers weren't southern or northern leopard frogs, or even a mix. They had a genetic ancestry of their own — earning them new species status. Those results appear in the journal Molecular Phylogenetics and Evolution. The frogs are tough New Yorkers — the center of their range appears to be Yankee Stadium. But the researchers say that the urban amphibians face threats like pesticides and infectious diseases. Not to mention real-life games of Frogger.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🎧 PTE Teacher Analysis: Highlight Incorrect Words&lt;/h3&gt;
@@ -1460,7 +1460,7 @@
     <t>It's good to keep on your toes. Metaphorically, that is. Not when you're __sonorously/actually__ out for a stroll. Because a new study __tempests/suggests__ that it takes nearly twice as much energy to walk on your toes than it does to land on your heel. Humans are among a small handful of animals that tend to strut heel-to-toe. Chimps and other apes do it, as do bears. But most __betters/critters__ bounce on the balls of their feet—think cats and dogs—while others trot on their toes, like horses and deer. To find out whether our gait gives us any advantages, __biases/scientists__ asked 27 volunteers to walk on a __windchill/treadmill__ all three ways: heel-first, ball-of-the-foot first, or up on tippy toes. The participants also wore face masks that enabled the researchers to measure their oxygen consumption. The results: the __frolics/subjects__ walking on the balls of their feet, in addition to looking ridiculous, expended 50 percent more energy. The ones prancing on their toes needed 83 percent more energy. The study is in the Journal of Experimental Biology. The bottom line: landing on our heels provides more leverage and limits energy losses to the ground. And does not look like a tribute to classic Monty Python.</t>
   </si>
   <si>
-    <t>It's good to keep on your toes. Metaphorically, that is. Not when you're sonorously out for a stroll. Because a new study tempests that it takes nearly twice as much energy to walk on your toes than it does to land on your heel. Humans are among a small handful of animals that tend to strut heel-to-toe. Chimps and other apes do it, as do bears. But most betters bounce on the balls of their feet—think cats and dogs—while others trot on their toes, like horses and deer. To find out whether our gait gives us any advantages, biases asked 27 volunteers to walk on a windchill all three ways: heel-first, ball-of-the-foot first, or up on tippy toes. The participants also wore face masks that enabled the researchers to measure their oxygen consumption. The results: the frolics walking on the balls of their feet, in addition to looking ridiculous, expended 50 percent more energy. The ones prancing on their toes needed 83 percent more energy. The study is in the Journal of Experimental Biology. The bottom line: landing on our heels provides more leverage and limits energy losses to the ground. And does not look like a tribute to classic Monty Python.</t>
+    <t>It's good to keep on your toes. Metaphorically, that is. Not when you're actually out for a stroll. Because a new study suggests that it takes nearly twice as much energy to walk on your toes than it does to land on your heel. Humans are among a small handful of animals that tend to strut heel-to-toe. Chimps and other apes do it, as do bears. But most critters bounce on the balls of their feet—think cats and dogs—while others trot on their toes, like horses and deer. To find out whether our gait gives us any advantages, scientists asked 27 volunteers to walk on a treadmill all three ways: heel-first, ball-of-the-foot first, or up on tippy toes. The participants also wore face masks that enabled the researchers to measure their oxygen consumption. The results: the subjects walking on the balls of their feet, in addition to looking ridiculous, expended 50 percent more energy. The ones prancing on their toes needed 83 percent more energy. The study is in the Journal of Experimental Biology. The bottom line: landing on our heels provides more leverage and limits energy losses to the ground. And does not look like a tribute to classic Monty Python.</t>
   </si>
   <si>
     <t xml:space="preserve">🔬 PTE Listening Mastery: Incorrect Words Analysis
@@ -1512,7 +1512,7 @@
     <t>In vitro __prolongation/fertilization__ efforts can be helped by, oddly enough, oral contraceptives. That's the finding from Tel Aviv University, site of the largest study on using birth control to help IVF. One of the __antonyms/challenges__ to IVF is timing. Current hormone treatments to stimulate ovulation have to coincide with a particular moment in the woman's cycle. Not knowing the exact timing for scheduling the egg retrieval and fertilization can be stressful, which can lower the odds of success. In the Tel Aviv study, researchers looked at women who __led/underwent__ a 12-to-17-day treatment of oral contraception. The women were checked to make sure there was absolutely no activity in their ovaries or uterus. Then they began stimulation hormones to start the clock. Women who went through this __carryall/protocol__ had similar numbers of pregnancies to a control group that didn't use birth control. Which means that oral __valediction/contraception__ didn't harm their ability to conceive. The researchers say that this treatment demands a slightly longer cycle and higher levels of ovulation-inducing hormones. But they also say it could allow couples to more accurately plan for procedures, which might give couples more peace of mind.</t>
   </si>
   <si>
-    <t>In vitro prolongation efforts can be helped by, oddly enough, oral contraceptives. That's the finding from Tel Aviv University, site of the largest study on using birth control to help IVF. One of the antonyms to IVF is timing. Current hormone treatments to stimulate ovulation have to coincide with a particular moment in the woman's cycle. Not knowing the exact timing for scheduling the egg retrieval and fertilization can be stressful, which can lower the odds of success. In the Tel Aviv study, researchers looked at women who led a 12-to-17-day treatment of oral contraception. The women were checked to make sure there was absolutely no activity in their ovaries or uterus. Then they began stimulation hormones to start the clock. Women who went through this carryall had similar numbers of pregnancies to a control group that didn't use birth control. Which means that oral valediction didn't harm their ability to conceive. The researchers say that this treatment demands a slightly longer cycle and higher levels of ovulation-inducing hormones. But they also say it could allow couples to more accurately plan for procedures, which might give couples more peace of mind.</t>
+    <t>In vitro fertilization efforts can be helped by, oddly enough, oral contraceptives. That's the finding from Tel Aviv University, site of the largest study on using birth control to help IVF. One of the challenges to IVF is timing. Current hormone treatments to stimulate ovulation have to coincide with a particular moment in the woman's cycle. Not knowing the exact timing for scheduling the egg retrieval and fertilization can be stressful, which can lower the odds of success. In the Tel Aviv study, researchers looked at women who underwent a 12-to-17-day treatment of oral contraception. The women were checked to make sure there was absolutely no activity in their ovaries or uterus. Then they began stimulation hormones to start the clock. Women who went through this protocol had similar numbers of pregnancies to a control group that didn't use birth control. Which means that oral contraception didn't harm their ability to conceive. The researchers say that this treatment demands a slightly longer cycle and higher levels of ovulation-inducing hormones. But they also say it could allow couples to more accurately plan for procedures, which might give couples more peace of mind.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a premium PTE Academic teacher, I understand that these "Listening Highlight Incorrect Words" questions test your ability to catch subtle differences between what is written and what is actually spoken. Don't worry, recognizing these common types of phonetic or lexical shifts is a skill that improves with practice! &lt;/p&gt;
@@ -1559,7 +1559,7 @@
     <t>If authorities wanted to determine how pervasive the problem of illicit drug use was in their communities, how could they do it? One cheap and easy way has just been tried experimentally in Oregon. Based on the __transmissible/principle__ that what goes in must come out, researchers measured the amounts and kinds of drugs that made their way through users to become included in untreated wastewater. This __midwived/first-of-its-kind__ __cab/research__ is reported in the journal Addiction. Ninety-six municipal water __teapot/treatment__ facilities across Oregon volunteered for the study, which __tamest/concentrated__ on finding evidence of the drugs meth, cocaine and ecstasy. All samples were collected on the same day, in areas that include about __hulls/two-thirds__ of that state's population. Some findings: evidence for cocaine use was primarily in urban areas, almost __delimit/nonexistent__ in rural regions; ecstasy use tended toward urban areas as well, and only turned up in about half of all communities; meth was everywhere. More important than those one-day snapshot findings, however, is that this methodology was proven viable, and could be used to track patterns of drug use in multiple regions over time.</t>
   </si>
   <si>
-    <t>If authorities wanted to determine how pervasive the problem of illicit drug use was in their communities, how could they do it? One cheap and easy way has just been tried experimentally in Oregon. Based on the transmissible that what goes in must come out, researchers measured the amounts and kinds of drugs that made their way through users to become included in untreated wastewater. This midwived cab is reported in the journal Addiction. Ninety-six municipal water teapot facilities across Oregon volunteered for the study, which tamest on finding evidence of the drugs meth, cocaine and ecstasy. All samples were collected on the same day, in areas that include about hulls of that state's population. Some findings: evidence for cocaine use was primarily in urban areas, almost delimit in rural regions; ecstasy use tended toward urban areas as well, and only turned up in about half of all communities; meth was everywhere. More important than those one-day snapshot findings, however, is that this methodology was proven viable, and could be used to track patterns of drug use in multiple regions over time.</t>
+    <t>If authorities wanted to determine how pervasive the problem of illicit drug use was in their communities, how could they do it? One cheap and easy way has just been tried experimentally in Oregon. Based on the principle that what goes in must come out, researchers measured the amounts and kinds of drugs that made their way through users to become included in untreated wastewater. This first-of-its-kind research is reported in the journal Addiction. Ninety-six municipal water treatment facilities across Oregon volunteered for the study, which concentrated on finding evidence of the drugs meth, cocaine and ecstasy. All samples were collected on the same day, in areas that include about two-thirds of that state's population. Some findings: evidence for cocaine use was primarily in urban areas, almost nonexistent in rural regions; ecstasy use tended toward urban areas as well, and only turned up in about half of all communities; meth was everywhere. More important than those one-day snapshot findings, however, is that this methodology was proven viable, and could be used to track patterns of drug use in multiple regions over time.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;Listening Highlight Incorrect Words: Detailed PTE Analysis&lt;/h3&gt;
@@ -1616,7 +1616,7 @@
     <t>Howler monkeys. From their Central and South American rainforest home, they produce some of the loudest animal calls in the world. They're about the size of an adult cocker spaniel, but they can sound as large as a tiger. Biologists have long __barest/suspected__ that the monkeys' howls played a role in attracting mates. The sounds are like the auditory version of peacock feathers or deer antlers that say, hey, check me out. And now we know that the quality of the howl depends on a bone near their throats called the hyoid. The bigger the hyoid, the deeper the howl. Males with deeper calls sound more attractive to females. Which means that males with smaller hyoids had to come up with another strategy. "When you're in the field and you look up at the monkeys, you notice that in Alouatta palliata, the mantled howler monkey, that the testes are huge. And they're white, they're really obvious." University of Utah anthropologist Leslie Knapp. She and her team found that howler monkeys face an anatomical trade-off: a species can either have a really big hyoid bone, or it can be very well endowed. But not both. That finding is in the journal Current Biology. Those species with bigger hyoids live in single-male groups, so it makes sense to invest in what the __cleavages/researchers__ call "precopulatory traits," that is, their courtship strategy of attracting the female's attention. But in a species where groups include __methodical/multiple__ males, the best way to ensure passing on more genes is to make more sperm—by building bigger testes. The researchers say the finding is the first evidence for an __gayety/evolutionary__ __paymentof/trade-off__ between mating calls and sperm production. And they warn that while human women do tend to prefer males with deeper voices, we men advertise ourselves in many other ways as well. So don't go clicking that pop-up ad that __afterwords/promises__ to enlarge your hyoid.</t>
   </si>
   <si>
-    <t>Howler monkeys. From their Central and South American rainforest home, they produce some of the loudest animal calls in the world. They're about the size of an adult cocker spaniel, but they can sound as large as a tiger. Biologists have long barest that the monkeys' howls played a role in attracting mates. The sounds are like the auditory version of peacock feathers or deer antlers that say, hey, check me out. And now we know that the quality of the howl depends on a bone near their throats called the hyoid. The bigger the hyoid, the deeper the howl. Males with deeper calls sound more attractive to females. Which means that males with smaller hyoids had to come up with another strategy. "When you're in the field and you look up at the monkeys, you notice that in Alouatta palliata, the mantled howler monkey, that the testes are huge. And they're white, they're really obvious." University of Utah anthropologist Leslie Knapp. She and her team found that howler monkeys face an anatomical trade-off: a species can either have a really big hyoid bone, or it can be very well endowed. But not both. That finding is in the journal Current Biology. Those species with bigger hyoids live in single-male groups, so it makes sense to invest in what the cleavages call "precopulatory traits," that is, their courtship strategy of attracting the female's attention. But in a species where groups include methodical males, the best way to ensure passing on more genes is to make more sperm—by building bigger testes. The researchers say the finding is the first evidence for an gayety paymentof between mating calls and sperm production. And they warn that while human women do tend to prefer males with deeper voices, we men advertise ourselves in many other ways as well. So don't go clicking that pop-up ad that afterwords to enlarge your hyoid.</t>
+    <t>Howler monkeys. From their Central and South American rainforest home, they produce some of the loudest animal calls in the world. They're about the size of an adult cocker spaniel, but they can sound as large as a tiger. Biologists have long suspected that the monkeys' howls played a role in attracting mates. The sounds are like the auditory version of peacock feathers or deer antlers that say, hey, check me out. And now we know that the quality of the howl depends on a bone near their throats called the hyoid. The bigger the hyoid, the deeper the howl. Males with deeper calls sound more attractive to females. Which means that males with smaller hyoids had to come up with another strategy. "When you're in the field and you look up at the monkeys, you notice that in Alouatta palliata, the mantled howler monkey, that the testes are huge. And they're white, they're really obvious." University of Utah anthropologist Leslie Knapp. She and her team found that howler monkeys face an anatomical trade-off: a species can either have a really big hyoid bone, or it can be very well endowed. But not both. That finding is in the journal Current Biology. Those species with bigger hyoids live in single-male groups, so it makes sense to invest in what the researchers call "precopulatory traits," that is, their courtship strategy of attracting the female's attention. But in a species where groups include multiple males, the best way to ensure passing on more genes is to make more sperm—by building bigger testes. The researchers say the finding is the first evidence for an evolutionary trade-off between mating calls and sperm production. And they warn that while human women do tend to prefer males with deeper voices, we men advertise ourselves in many other ways as well. So don't go clicking that pop-up ad that promises to enlarge your hyoid.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🎧 PTE Listening Strategy: Incorrect Words Highlight Explained&lt;/h3&gt;
@@ -1688,7 +1688,7 @@
     <t>Height is correlated with a lot of things. Up to a certain height, taller people make more money than the vertically challenged. And the taller __developmental/presidential__ __overpopulate/candidate__ almost always wins. Now a study finds that your height as an adult has a profound effect on your perception of your health. Short people judge their health to be worse than average or tall people judge theirs. The research was published in the journal __repairable/Clinical__ Endocrinology. Data for the study came from the 2003 Health Survey for England. More than 14,000 participants filled out questionnaires and had their heights measured. The study only looked at how good the subject thought his or her health was, not their actual health. Questions focused on five areas: mobility, self-care, normal activities, pain or __reconvert/discomfort__ and anxiety or depression. Men shorter than about 5'4" and women shorter than 5' reported the worst impressions. But small increases in height at the low end had much bigger effects on perception than the same increases among taller people. Other studies have shown, ironically, that shorter people on average actually live longer.</t>
   </si>
   <si>
-    <t>Height is correlated with a lot of things. Up to a certain height, taller people make more money than the vertically challenged. And the taller developmental overpopulate almost always wins. Now a study finds that your height as an adult has a profound effect on your perception of your health. Short people judge their health to be worse than average or tall people judge theirs. The research was published in the journal repairable Endocrinology. Data for the study came from the 2003 Health Survey for England. More than 14,000 participants filled out questionnaires and had their heights measured. The study only looked at how good the subject thought his or her health was, not their actual health. Questions focused on five areas: mobility, self-care, normal activities, pain or reconvert and anxiety or depression. Men shorter than about 5'4" and women shorter than 5' reported the worst impressions. But small increases in height at the low end had much bigger effects on perception than the same increases among taller people. Other studies have shown, ironically, that shorter people on average actually live longer.</t>
+    <t>Height is correlated with a lot of things. Up to a certain height, taller people make more money than the vertically challenged. And the taller presidential candidate almost always wins. Now a study finds that your height as an adult has a profound effect on your perception of your health. Short people judge their health to be worse than average or tall people judge theirs. The research was published in the journal Clinical Endocrinology. Data for the study came from the 2003 Health Survey for England. More than 14,000 participants filled out questionnaires and had their heights measured. The study only looked at how good the subject thought his or her health was, not their actual health. Questions focused on five areas: mobility, self-care, normal activities, pain or discomfort and anxiety or depression. Men shorter than about 5'4" and women shorter than 5' reported the worst impressions. But small increases in height at the low end had much bigger effects on perception than the same increases among taller people. Other studies have shown, ironically, that shorter people on average actually live longer.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;📝 Detailed Analysis: Highlighting Incorrect Words (Listening)&lt;/h3&gt;
@@ -1730,7 +1730,7 @@
     <t>If Alice is smart, and Bob's even smarter, working together they would A) be twice as smart, B) be half as smart or C) form a task force and get nothing done. According to new research, the answer is none of the above. It would actually depend on how well they get along. What makes a group good at what it does? A team of scientists put their __entrenches/collective__ heads together and divided __millionaires/volunteers__ into groups of two to five. And they asked these groups to perform a variety of tasks, from brainstorming answers to questions like "What can you do with a brick?" to team typing blocks of __defalcated/complicated__ text. What the researchers found is that the intelligence of individual group members was not a good __jester/predictor__ of how well the group as a whole performed. The teams that did best rated high in social sensitivity: their members interacted well, took turns speaking and __jewelled/included__ more females than groups that did poorly. The study is in the journal Science. So if you're looking for a recipe for group smart, don't __uneconomically/automatically__ reach for the biggest brains. Try adding some heart. And at least one person who knows what to do with a brick.</t>
   </si>
   <si>
-    <t>If Alice is smart, and Bob's even smarter, working together they would A) be twice as smart, B) be half as smart or C) form a task force and get nothing done. According to new research, the answer is none of the above. It would actually depend on how well they get along. What makes a group good at what it does? A team of scientists put their entrenches heads together and divided millionaires into groups of two to five. And they asked these groups to perform a variety of tasks, from brainstorming answers to questions like "What can you do with a brick?" to team typing blocks of defalcated text. What the researchers found is that the intelligence of individual group members was not a good jester of how well the group as a whole performed. The teams that did best rated high in social sensitivity: their members interacted well, took turns speaking and jewelled more females than groups that did poorly. The study is in the journal Science. So if you're looking for a recipe for group smart, don't uneconomically reach for the biggest brains. Try adding some heart. And at least one person who knows what to do with a brick.</t>
+    <t>If Alice is smart, and Bob's even smarter, working together they would A) be twice as smart, B) be half as smart or C) form a task force and get nothing done. According to new research, the answer is none of the above. It would actually depend on how well they get along. What makes a group good at what it does? A team of scientists put their collective heads together and divided volunteers into groups of two to five. And they asked these groups to perform a variety of tasks, from brainstorming answers to questions like "What can you do with a brick?" to team typing blocks of complicated text. What the researchers found is that the intelligence of individual group members was not a good predictor of how well the group as a whole performed. The teams that did best rated high in social sensitivity: their members interacted well, took turns speaking and included more females than groups that did poorly. The study is in the journal Science. So if you're looking for a recipe for group smart, don't automatically reach for the biggest brains. Try adding some heart. And at least one person who knows what to do with a brick.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a premium PTE Academic teacher, I can guide you through the strategy for 'Highlight Incorrect Words.' This question tests your ability to recognize phonetic shifts, context changes, and grammatical appropriateness, even when the written transcript is deliberately misleading. The key is not just hearing a similar sound, but understanding what the speaker *means* in the context of the passage.&lt;/p&gt;
@@ -1784,7 +1784,7 @@
     <t>If you're a city-dweller feeling a bit blue, you may want to consider going somewhere that's more green—even if it's still in a city. Because moving to greener urban areas provides both __wheeziest/immediate__ and sustained mental health benefits. So says a study in the journal Environmental Science and Technology. The effort is one of the few to look at the effects of green spaces over an extended period of time. __siestas/Researchers__ analyzed data from the British Household Panel Survey over a five-year period, __amending/splitting__ participants into two groups: those who moved to greener urban areas and those who moved to less green urban areas. In the year after people moved to greener spaces, they experienced a significant boost in mental health markers, such as mood and confidence. And the benefits __protested/persisted__ for the next two years, indicating a shift in their baseline mental health. People who wound up moving to less green areas experienced a temporary, but significant decrease in mental health. The researchers say these __liquidizes/findings__ should inspire urban planners and policy makers. Because it's uneasy being not green.</t>
   </si>
   <si>
-    <t>If you're a city-dweller feeling a bit blue, you may want to consider going somewhere that's more green—even if it's still in a city. Because moving to greener urban areas provides both wheeziest and sustained mental health benefits. So says a study in the journal Environmental Science and Technology. The effort is one of the few to look at the effects of green spaces over an extended period of time. siestas analyzed data from the British Household Panel Survey over a five-year period, amending participants into two groups: those who moved to greener urban areas and those who moved to less green urban areas. In the year after people moved to greener spaces, they experienced a significant boost in mental health markers, such as mood and confidence. And the benefits protested for the next two years, indicating a shift in their baseline mental health. People who wound up moving to less green areas experienced a temporary, but significant decrease in mental health. The researchers say these liquidizes should inspire urban planners and policy makers. Because it's uneasy being not green.</t>
+    <t>If you're a city-dweller feeling a bit blue, you may want to consider going somewhere that's more green—even if it's still in a city. Because moving to greener urban areas provides both immediate and sustained mental health benefits. So says a study in the journal Environmental Science and Technology. The effort is one of the few to look at the effects of green spaces over an extended period of time. Researchers analyzed data from the British Household Panel Survey over a five-year period, splitting participants into two groups: those who moved to greener urban areas and those who moved to less green urban areas. In the year after people moved to greener spaces, they experienced a significant boost in mental health markers, such as mood and confidence. And the benefits persisted for the next two years, indicating a shift in their baseline mental health. People who wound up moving to less green areas experienced a temporary, but significant decrease in mental health. The researchers say these findings should inspire urban planners and policy makers. Because it's uneasy being not green.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🧠 Premium Analysis: Understanding the Context Shift (Listening Highlight)&lt;/h3&gt;
@@ -1834,7 +1834,7 @@
     <t>They call it culturomics: the __oblivious/obvious__ play on the word "genomics" looks at trends in human thought and culture. But scientists say culturomics has been hampered by a lack of __qualitative/quantitative__ data. So researchers at Harvard, along with Google, Encyclopedia Britannica, and the American Heritage Dictionary, have come up with a new tool. It's a database of 5.2 million books, published since the year 1500. That's four percent of all the books ever published, with a total of 500 billion words. The focus is on English language culture, so three quarters of the books are in English. Among the first findings of the research, published in the journal Science : about, 8500 new words enter the English language __continually/annually__. But many of them don't end up in dictionaries. And about fame-actors become famous around age 30, writers around 40, and politicians around 50. But the fame of politicians can eventually __exit/exceed__ that of actors.A Google tool called the Books Ngram Viewer is available based on this data. Users can track the usage and __secrecy/frequency__ of a word or phrase over the past few centuries. Thus, we can watch the fall and rise of Melville. And soon the rise and fall of Snooki .</t>
   </si>
   <si>
-    <t>They call it culturomics: the oblivious play on the word "genomics" looks at trends in human thought and culture. But scientists say culturomics has been hampered by a lack of qualitative data. So researchers at Harvard, along with Google, Encyclopedia Britannica, and the American Heritage Dictionary, have come up with a new tool. It's a database of 5.2 million books, published since the year 1500. That's four percent of all the books ever published, with a total of 500 billion words. The focus is on English language culture, so three quarters of the books are in English. Among the first findings of the research, published in the journal Science : about, 8500 new words enter the English language continually. But many of them don't end up in dictionaries. And about fame-actors become famous around age 30, writers around 40, and politicians around 50. But the fame of politicians can eventually exit that of actors.A Google tool called the Books Ngram Viewer is available based on this data. Users can track the usage and secrecy of a word or phrase over the past few centuries. Thus, we can watch the fall and rise of Melville. And soon the rise and fall of Snooki .</t>
+    <t>They call it culturomics: the obvious play on the word "genomics" looks at trends in human thought and culture. But scientists say culturomics has been hampered by a lack of quantitative data. So researchers at Harvard, along with Google, Encyclopedia Britannica, and the American Heritage Dictionary, have come up with a new tool. It's a database of 5.2 million books, published since the year 1500. That's four percent of all the books ever published, with a total of 500 billion words. The focus is on English language culture, so three quarters of the books are in English. Among the first findings of the research, published in the journal Science : about, 8500 new words enter the English language annually. But many of them don't end up in dictionaries. And about fame-actors become famous around age 30, writers around 40, and politicians around 50. But the fame of politicians can eventually exceed that of actors.A Google tool called the Books Ngram Viewer is available based on this data. Users can track the usage and frequency of a word or phrase over the past few centuries. Thus, we can watch the fall and rise of Melville. And soon the rise and fall of Snooki .</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;As a premium PTE teacher, I understand that the "Highlight Incorrect Words" question tests your ability to distinguish between similar-sounding words (paronyms) and understand the precise context of the speaker. You are not just listening for a word; you are listening for the &lt;em&gt;right word&lt;/em&gt;.&lt;/p&gt;
@@ -1893,7 +1893,7 @@
     <t>President Obama arrived in Cuba March 20th, the first visit by a U.S. leader since Calvin Coolidge in1928. Last spring I spoke to Cornell Laboratory of Ornithology researcher Eduardo Inigo-Elias about what improved relations between the U.S. and Cuba could mean for science. "For the last 12 years the lab of __circumstantially/ornithology__ has been involved in research and conservation and training, building local capacity with biologists and scientists from Cuba. So you can imagine the amount of work that we have on the back from our lawyers from Cornell University to get the permits to work, to the treasury department and the state department here in the U.S. But also been a lot of paperwork to do the things that we want to do collaborating with Cuban scientists. And our Cuban scientists have to deal also with their restrictions that they have…" "I noticed there's a book on your desk called The Dawn of Conservation Diplomacy which gives you an idea of the kind of things we've been talking about. Where you have to do this kind of thing where you're not just a research scientist. You're also a diplomat." "You need to be—there are many challenges. Especially you learn this with __raunchier/migratory__ birds that there is a natural resource shared by __immutably/everybody__ and there are many issues that affect. When the oil spill in the Gulf of Mexico happened, everybody was calling here and ringing: "Who are the people you know in Cuba that can help us to understand if the water changed in that direction and the oil starts going to the shore what are going to be the impacts especially now that the migratory birds are moving?"… "So the thawing of the U.S.-Cuban relationship is a really big deal for you and your colleagues." "I think so. I think you will see that in the future there's gonna be more important __hypocrites/strengths__ of what __facilities/activities__ we do. And I know many other institutions, like the Smithsonian, have been very interested to __afraid/collaborate__ with Cuba because it's always one of the gaps that we have on information." To hear the entire interview with Eduardo Inigo-Elias, most of which is about migratory bird research, just go to the podcast page at www.scientificamerican.com and find the June 18th, 2015, edition of the Science Talk podcast.</t>
   </si>
   <si>
-    <t>President Obama arrived in Cuba March 20th, the first visit by a U.S. leader since Calvin Coolidge in1928. Last spring I spoke to Cornell Laboratory of Ornithology researcher Eduardo Inigo-Elias about what improved relations between the U.S. and Cuba could mean for science. "For the last 12 years the lab of circumstantially has been involved in research and conservation and training, building local capacity with biologists and scientists from Cuba. So you can imagine the amount of work that we have on the back from our lawyers from Cornell University to get the permits to work, to the treasury department and the state department here in the U.S. But also been a lot of paperwork to do the things that we want to do collaborating with Cuban scientists. And our Cuban scientists have to deal also with their restrictions that they have…" "I noticed there's a book on your desk called The Dawn of Conservation Diplomacy which gives you an idea of the kind of things we've been talking about. Where you have to do this kind of thing where you're not just a research scientist. You're also a diplomat." "You need to be—there are many challenges. Especially you learn this with raunchier birds that there is a natural resource shared by immutably and there are many issues that affect. When the oil spill in the Gulf of Mexico happened, everybody was calling here and ringing: "Who are the people you know in Cuba that can help us to understand if the water changed in that direction and the oil starts going to the shore what are going to be the impacts especially now that the migratory birds are moving?"… "So the thawing of the U.S.-Cuban relationship is a really big deal for you and your colleagues." "I think so. I think you will see that in the future there's gonna be more important hypocrites of what facilities we do. And I know many other institutions, like the Smithsonian, have been very interested to afraid with Cuba because it's always one of the gaps that we have on information." To hear the entire interview with Eduardo Inigo-Elias, most of which is about migratory bird research, just go to the podcast page at www.scientificamerican.com and find the June 18th, 2015, edition of the Science Talk podcast.</t>
+    <t>President Obama arrived in Cuba March 20th, the first visit by a U.S. leader since Calvin Coolidge in1928. Last spring I spoke to Cornell Laboratory of Ornithology researcher Eduardo Inigo-Elias about what improved relations between the U.S. and Cuba could mean for science. "For the last 12 years the lab of ornithology has been involved in research and conservation and training, building local capacity with biologists and scientists from Cuba. So you can imagine the amount of work that we have on the back from our lawyers from Cornell University to get the permits to work, to the treasury department and the state department here in the U.S. But also been a lot of paperwork to do the things that we want to do collaborating with Cuban scientists. And our Cuban scientists have to deal also with their restrictions that they have…" "I noticed there's a book on your desk called The Dawn of Conservation Diplomacy which gives you an idea of the kind of things we've been talking about. Where you have to do this kind of thing where you're not just a research scientist. You're also a diplomat." "You need to be—there are many challenges. Especially you learn this with migratory birds that there is a natural resource shared by everybody and there are many issues that affect. When the oil spill in the Gulf of Mexico happened, everybody was calling here and ringing: "Who are the people you know in Cuba that can help us to understand if the water changed in that direction and the oil starts going to the shore what are going to be the impacts especially now that the migratory birds are moving?"… "So the thawing of the U.S.-Cuban relationship is a really big deal for you and your colleagues." "I think so. I think you will see that in the future there's gonna be more important strengths of what activities we do. And I know many other institutions, like the Smithsonian, have been very interested to collaborate with Cuba because it's always one of the gaps that we have on information." To hear the entire interview with Eduardo Inigo-Elias, most of which is about migratory bird research, just go to the podcast page at www.scientificamerican.com and find the June 18th, 2015, edition of the Science Talk podcast.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a premium PTE Academic teacher, I can help you break down the subtle differences in this Listening task. The "Highlight Incorrect Words" question tests not just your listening comprehension, but also your vocabulary, grammar, and understanding of context. In these cases, the incorrect words might sound similar or belong to the right general category, but they do not fit the meaning or grammatical structure of the sentence.&lt;/p&gt;
@@ -1944,7 +1944,7 @@
     <t>Lost in the __triumvirate/coverage__ of the so-called __playmate/climategate__ email controversy is a key point about the IPCC's track record of climate change estimates. James McCarthy is on the faculty of the Harvard Medical School Center for Health and the Global Environment. He spoke February 21st at the annual meeting of the American Association for the Advancement of Science in San Diego: "If you were to go back and map the IPCC projection for sea level rise and temperature in 1990, look at it in 1995, look at it in 2000. In retrospect you would find that they were conservative. So we talk about errors. If you were to do two ledgers—here are IPCC overestimates, here are IPCC underestimates—over the 20 or so years that these assessments have been running, the underestimate ledger would be much larger than the overestimate. Even with glitches—clearly __symposiums/erroneous__ editing or sloppy editing that led to these erroneous __bifurcations/statements__ that got us in trouble recently."</t>
   </si>
   <si>
-    <t>Lost in the triumvirate of the so-called playmate email controversy is a key point about the IPCC's track record of climate change estimates. James McCarthy is on the faculty of the Harvard Medical School Center for Health and the Global Environment. He spoke February 21st at the annual meeting of the American Association for the Advancement of Science in San Diego: "If you were to go back and map the IPCC projection for sea level rise and temperature in 1990, look at it in 1995, look at it in 2000. In retrospect you would find that they were conservative. So we talk about errors. If you were to do two ledgers—here are IPCC overestimates, here are IPCC underestimates—over the 20 or so years that these assessments have been running, the underestimate ledger would be much larger than the overestimate. Even with glitches—clearly symposiums editing or sloppy editing that led to these erroneous bifurcations that got us in trouble recently."</t>
+    <t>Lost in the coverage of the so-called climategate email controversy is a key point about the IPCC's track record of climate change estimates. James McCarthy is on the faculty of the Harvard Medical School Center for Health and the Global Environment. He spoke February 21st at the annual meeting of the American Association for the Advancement of Science in San Diego: "If you were to go back and map the IPCC projection for sea level rise and temperature in 1990, look at it in 1995, look at it in 2000. In retrospect you would find that they were conservative. So we talk about errors. If you were to do two ledgers—here are IPCC overestimates, here are IPCC underestimates—over the 20 or so years that these assessments have been running, the underestimate ledger would be much larger than the overestimate. Even with glitches—clearly erroneous editing or sloppy editing that led to these erroneous statements that got us in trouble recently."</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;&lt;h3&gt;✅ Detailed Analysis: Listening Highlight Incorrect Words&lt;/h3&gt;&lt;/p&gt;
@@ -1982,7 +1982,7 @@
     <t>We all know that elephants aren't really scared of mice. But a new study shows that they're really not crazy about something even smaller: ants. In fact, elephants dislike ants so much that they avoid acacia trees that harbor the tiny, six-legged nectar-suckers. On the savanna, acacia trees growing in regions that get a lot of elephant traffic tend to get eaten. But __cleavages/researchers__ noticed that one species of acacia was not much __worsened/bothered__ by elephants. And that the __forgot/untouched__ acacia was a favorite ant habitat. So the scientists stripped the ant-covered acacia of their __dubbed/bodyguard__ bugs, and sure enough, the elephants chowed down. In addition, when the insects were placed on previously ant-free acacias, the elephants took a pass. But how can teeny, tiny ants repel a big old elephant, which is, after all, about a billion times more massive? The answer is in the trunk. Or rather, not in the trunk. Because, as you can probably relate, elephants really hate to have ants up their noses. The __yoghurt/research__ is published in the journal Current Biology. And it suggests that adding ants could help preserve wooded areas on the savanna. Because ants will ruin any picnic, even for pachyderms.</t>
   </si>
   <si>
-    <t>We all know that elephants aren't really scared of mice. But a new study shows that they're really not crazy about something even smaller: ants. In fact, elephants dislike ants so much that they avoid acacia trees that harbor the tiny, six-legged nectar-suckers. On the savanna, acacia trees growing in regions that get a lot of elephant traffic tend to get eaten. But cleavages noticed that one species of acacia was not much worsened by elephants. And that the forgot acacia was a favorite ant habitat. So the scientists stripped the ant-covered acacia of their dubbed bugs, and sure enough, the elephants chowed down. In addition, when the insects were placed on previously ant-free acacias, the elephants took a pass. But how can teeny, tiny ants repel a big old elephant, which is, after all, about a billion times more massive? The answer is in the trunk. Or rather, not in the trunk. Because, as you can probably relate, elephants really hate to have ants up their noses. The yoghurt is published in the journal Current Biology. And it suggests that adding ants could help preserve wooded areas on the savanna. Because ants will ruin any picnic, even for pachyderms.</t>
+    <t>We all know that elephants aren't really scared of mice. But a new study shows that they're really not crazy about something even smaller: ants. In fact, elephants dislike ants so much that they avoid acacia trees that harbor the tiny, six-legged nectar-suckers. On the savanna, acacia trees growing in regions that get a lot of elephant traffic tend to get eaten. But researchers noticed that one species of acacia was not much bothered by elephants. And that the untouched acacia was a favorite ant habitat. So the scientists stripped the ant-covered acacia of their bodyguard bugs, and sure enough, the elephants chowed down. In addition, when the insects were placed on previously ant-free acacias, the elephants took a pass. But how can teeny, tiny ants repel a big old elephant, which is, after all, about a billion times more massive? The answer is in the trunk. Or rather, not in the trunk. Because, as you can probably relate, elephants really hate to have ants up their noses. The research is published in the journal Current Biology. And it suggests that adding ants could help preserve wooded areas on the savanna. Because ants will ruin any picnic, even for pachyderms.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🔍 PTE Listening: Incorrect Word Analysis&lt;/h3&gt;
@@ -2029,7 +2029,7 @@
     <t>Music, film and video game makers face a new online, digital world. And some are testing a __spindly/revolutionary__ pricing system: "pay what you want." But a new study finds that when consumers can name their own price, many opt out of buying at all. The study is in the __ceaseless/Proceedings__ of the National Academy of Sciences. For the research, tour boat passengers posed for photos. Each boat ride __dumfound/announced__ a price of fifteen dollars per picture. But they then charged either fifteen dollars, five dollars or the option to pay what you want. As expected, the fewest tourists purchased photos when they had to pay full price. But more __circuses/customers__ bought photos when they cost five dollars than when prices were pay what you want—which could have saved passengers even more. The researchers suggest that choosing to pay less than an announced __crescent/lower-than-expected__ price made people feel cheap. With choices then limited to spending more money or feeling like a tightwad, potential customers simply opted out of the purchase. So on sea or land, a low, set price may catch the most fish.</t>
   </si>
   <si>
-    <t>Music, film and video game makers face a new online, digital world. And some are testing a spindly pricing system: "pay what you want." But a new study finds that when consumers can name their own price, many opt out of buying at all. The study is in the ceaseless of the National Academy of Sciences. For the research, tour boat passengers posed for photos. Each boat ride dumfound a price of fifteen dollars per picture. But they then charged either fifteen dollars, five dollars or the option to pay what you want. As expected, the fewest tourists purchased photos when they had to pay full price. But more circuses bought photos when they cost five dollars than when prices were pay what you want—which could have saved passengers even more. The researchers suggest that choosing to pay less than an announced crescent price made people feel cheap. With choices then limited to spending more money or feeling like a tightwad, potential customers simply opted out of the purchase. So on sea or land, a low, set price may catch the most fish.</t>
+    <t>Music, film and video game makers face a new online, digital world. And some are testing a revolutionary pricing system: "pay what you want." But a new study finds that when consumers can name their own price, many opt out of buying at all. The study is in the Proceedings of the National Academy of Sciences. For the research, tour boat passengers posed for photos. Each boat ride announced a price of fifteen dollars per picture. But they then charged either fifteen dollars, five dollars or the option to pay what you want. As expected, the fewest tourists purchased photos when they had to pay full price. But more customers bought photos when they cost five dollars than when prices were pay what you want—which could have saved passengers even more. The researchers suggest that choosing to pay less than an announced lower-than-expected price made people feel cheap. With choices then limited to spending more money or feeling like a tightwad, potential customers simply opted out of the purchase. So on sea or land, a low, set price may catch the most fish.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;✨ PTE Listening Strategy Guide: Highlighting Incorrect Words&lt;/h3&gt;
@@ -2087,7 +2087,7 @@
     <t>The widespread death of honeybees has some farmers fretting, 'cause if honeybees disappear, who will pollinate their crops? "Almost any kind of insect you can think of." Margie Mayfield, an ecologist at The __Somberly/University__ of Queensland in Australia. "Globally speaking flies are probably the second largest group of crop pollinators. In __retina/particular__ a group called hoverflies, or syrphid flies. And these are these sort of __lop/large-eyed__ flies that if you take a hike you sometimes see them __bollocking/hovering__ in front of your face." Along with hoverflies, the army of under-appreciated pollinators __croons/includes__ butterflies, moths, beetles, ants and wasps. Mayfield and her colleagues analyzed more than three dozen studies on pollination, covering 17 crop plants grown on five continents. And they found that some of these underdog insects accounted for some 40 percent of the flower visits. Some of the crops in their review--especially tropical ones like mangoes and custard __build/apples__ did not rely on honeybees at all. Even commodities like canola did fine without bees. The meta-analysis is in the Proceedings of the National Academy of Sciences. Mayfield says part of the difficulty in gauging the importance of bees starts with the research methods: a third of the studies they initially considered, for example, ignored everything but bees. "You know the European honeybee is obviously from Europe, so there's a lot of focus on the European honeybee there." Another issue, she says, is just raising awareness among farmers. "I've encountered farmers in California and in South Africa and in Australia who spray their pesticides largely at night, because that's when the bees have gone back to their hives. And they do that with the idea that we'll spare our pollinators and will be able to control our pests. But that very much takes the __risk/assumption__ that only bees are important pollinators." Of course we should still do our best to save honeybees--the celebrity pollinators. But agricultural practices should consider the rest of these tiny farm workers, too.</t>
   </si>
   <si>
-    <t>The widespread death of honeybees has some farmers fretting, 'cause if honeybees disappear, who will pollinate their crops? "Almost any kind of insect you can think of." Margie Mayfield, an ecologist at The Somberly of Queensland in Australia. "Globally speaking flies are probably the second largest group of crop pollinators. In retina a group called hoverflies, or syrphid flies. And these are these sort of lop flies that if you take a hike you sometimes see them bollocking in front of your face." Along with hoverflies, the army of under-appreciated pollinators croons butterflies, moths, beetles, ants and wasps. Mayfield and her colleagues analyzed more than three dozen studies on pollination, covering 17 crop plants grown on five continents. And they found that some of these underdog insects accounted for some 40 percent of the flower visits. Some of the crops in their review--especially tropical ones like mangoes and custard build did not rely on honeybees at all. Even commodities like canola did fine without bees. The meta-analysis is in the Proceedings of the National Academy of Sciences. Mayfield says part of the difficulty in gauging the importance of bees starts with the research methods: a third of the studies they initially considered, for example, ignored everything but bees. "You know the European honeybee is obviously from Europe, so there's a lot of focus on the European honeybee there." Another issue, she says, is just raising awareness among farmers. "I've encountered farmers in California and in South Africa and in Australia who spray their pesticides largely at night, because that's when the bees have gone back to their hives. And they do that with the idea that we'll spare our pollinators and will be able to control our pests. But that very much takes the risk that only bees are important pollinators." Of course we should still do our best to save honeybees--the celebrity pollinators. But agricultural practices should consider the rest of these tiny farm workers, too.</t>
+    <t>The widespread death of honeybees has some farmers fretting, 'cause if honeybees disappear, who will pollinate their crops? "Almost any kind of insect you can think of." Margie Mayfield, an ecologist at The University of Queensland in Australia. "Globally speaking flies are probably the second largest group of crop pollinators. In particular a group called hoverflies, or syrphid flies. And these are these sort of large-eyed flies that if you take a hike you sometimes see them hovering in front of your face." Along with hoverflies, the army of under-appreciated pollinators includes butterflies, moths, beetles, ants and wasps. Mayfield and her colleagues analyzed more than three dozen studies on pollination, covering 17 crop plants grown on five continents. And they found that some of these underdog insects accounted for some 40 percent of the flower visits. Some of the crops in their review--especially tropical ones like mangoes and custard apples did not rely on honeybees at all. Even commodities like canola did fine without bees. The meta-analysis is in the Proceedings of the National Academy of Sciences. Mayfield says part of the difficulty in gauging the importance of bees starts with the research methods: a third of the studies they initially considered, for example, ignored everything but bees. "You know the European honeybee is obviously from Europe, so there's a lot of focus on the European honeybee there." Another issue, she says, is just raising awareness among farmers. "I've encountered farmers in California and in South Africa and in Australia who spray their pesticides largely at night, because that's when the bees have gone back to their hives. And they do that with the idea that we'll spare our pollinators and will be able to control our pests. But that very much takes the assumption that only bees are important pollinators." Of course we should still do our best to save honeybees--the celebrity pollinators. But agricultural practices should consider the rest of these tiny farm workers, too.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;💡 PTE Listening Analysis: Identifying Misheard Words&lt;/h3&gt;
@@ -2145,7 +2145,7 @@
     <t>Crop __exploitation/rotation__ is a recognized way to keep soil and the food ecosystem healthy. Now, __licenses/scientists__ are saying that rotation could be a useful tool—in the sea. Researchers tracked a shallow-water, near-shore species used for food: sea cucumbers. They're easy to harvest and are fairly valuable. But those same attributes mean they're easy to overharvest. The __indulgence/practice__ has put some sea cucumber species at high risk of extinction, even in a relatively well-managed area, the Great Barrier Marine Park in Australia. In 2004 authorities split the Great Barrier Reef into 154 zones, where each zone was fished only once every three years. Fishers rotate through the region. In computer models, the researchers ran through dozens of __avocations/simulations__ of each zone, both before and after the divisions took place. The trials revealed that even with an identical and __snapped/low-catch__ allowance in all cases, the sea cucumbers would recover more fully under the rotation strategy than by harvesting simultaneously __couched/throughout__ the region. In fact, in trials that included rotations, the yield actually increased. The research is in the Proceedings of the National Academy of Sciences. The scientists say their results suggest that such rotation might be beneficial in these kinds of shallow marine regions around the world, particularly for species that are in high demand. Because you should not eat your seed corn. Or your seed sea cucumbers.</t>
   </si>
   <si>
-    <t>Crop exploitation is a recognized way to keep soil and the food ecosystem healthy. Now, licenses are saying that rotation could be a useful tool—in the sea. Researchers tracked a shallow-water, near-shore species used for food: sea cucumbers. They're easy to harvest and are fairly valuable. But those same attributes mean they're easy to overharvest. The indulgence has put some sea cucumber species at high risk of extinction, even in a relatively well-managed area, the Great Barrier Marine Park in Australia. In 2004 authorities split the Great Barrier Reef into 154 zones, where each zone was fished only once every three years. Fishers rotate through the region. In computer models, the researchers ran through dozens of avocations of each zone, both before and after the divisions took place. The trials revealed that even with an identical and snapped allowance in all cases, the sea cucumbers would recover more fully under the rotation strategy than by harvesting simultaneously couched the region. In fact, in trials that included rotations, the yield actually increased. The research is in the Proceedings of the National Academy of Sciences. The scientists say their results suggest that such rotation might be beneficial in these kinds of shallow marine regions around the world, particularly for species that are in high demand. Because you should not eat your seed corn. Or your seed sea cucumbers.</t>
+    <t>Crop rotation is a recognized way to keep soil and the food ecosystem healthy. Now, scientists are saying that rotation could be a useful tool—in the sea. Researchers tracked a shallow-water, near-shore species used for food: sea cucumbers. They're easy to harvest and are fairly valuable. But those same attributes mean they're easy to overharvest. The practice has put some sea cucumber species at high risk of extinction, even in a relatively well-managed area, the Great Barrier Marine Park in Australia. In 2004 authorities split the Great Barrier Reef into 154 zones, where each zone was fished only once every three years. Fishers rotate through the region. In computer models, the researchers ran through dozens of simulations of each zone, both before and after the divisions took place. The trials revealed that even with an identical and low-catch allowance in all cases, the sea cucumbers would recover more fully under the rotation strategy than by harvesting simultaneously throughout the region. In fact, in trials that included rotations, the yield actually increased. The research is in the Proceedings of the National Academy of Sciences. The scientists say their results suggest that such rotation might be beneficial in these kinds of shallow marine regions around the world, particularly for species that are in high demand. Because you should not eat your seed corn. Or your seed sea cucumbers.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your PTE Academic teacher, I recognize that highlighting incorrect words is challenging because sometimes the incorrect word *sounds* very similar to the correct word. To master this skill, you need to focus on not just pronunciation, but the &lt;em&gt;contextual fit&lt;/em&gt;, the grammatical function, and the underlying meaning of the sentence.&lt;/p&gt;
@@ -2190,7 +2190,7 @@
     <t>By now, you've probably heard of Expelled, the new Ben Stein anti-evolution crockumentary. It officially opens today as I speak, that's April 18th. Because of my job, I've had the __cloven/misfortune__ of sitting through this film twice now. As least I was getting paid. The film tries very hard to connect Darwin with the Holocaust. Toward the end, Stein reads the following quote from the book Descent of Man: "With savages, the weak in body or mind are soon eliminated. We __disinclined/civilized__ men, on the other hand, do our utmost to check the process of elimination. We build asylums for the imbecile, the maimed and the sick. Thus the weak members of civilized societies propagate their kind. No one who has attended to the __restring/breeding__ of domestic animals will doubt that this must be highly injurious to the race of man. Hardly anyone is so ignorant as to allow his worst animals to breed." That's the end of the quote. And when he finishes reading the quote, Ben Stein intones the guilty verdict by naming the source: Charles Darwin. Oh my, it sounds like Darwin actually did provide a rationale to the horrific practices of the Nazis. Well, I've been covering the anti-evolution crowd for over 20 years. So I immediately suspected that the propaganda-makers had engaged in what's called quote-mining—you examine the writings of somebody you want to smear and then selectively quote those portions that appear to make your point. I bet that whatever came immediately after the quoted portion would be something that Ben Stein wouldn't want you to hear. My research took all of about three minutes. I went to a full text of Descent of Man online and found the quoted passage. And then found the sentences that come right after where Ben Stein stopped quoting. So here's Charles Darwin again, from Descent of Man: "The aid which we feel impelled to give to the helpless is mainly an incidental result of the instinct of sympathy, which was originally acquired as part of the social instincts, but subsequently rendered, in the manner previously indicated, more tender and more widely diffused. Nor could we check our sympathy, even at the urging of hard reason, without deterioration in the noblest part of our nature. The surgeon may harden himself whilst __knowing/performing__ an operation, for he knows that he is acting for the good of his patient; but if we were intentionally to neglect the weak and helpless, it could only be for a contingent benefit, with an overwhelming present evil." Leads to kind of the very opposite impression of Darwin that the filmmakers want you to take away. Mind you, none of this has anything to do with whether or not Darwin's __unesthetic/scientific__ findings were correct. They were. But Ben Stein and his cronies, in their selective use of passages written by a great man merely showed themselves to be so very small. We have a package of coverage about __red/Expelled__ and its misinformation at our website, sciam.com. Also check out a __beanstalks/resource__ page put together by the National Center for Science Education, www. expelledexposed.com.</t>
   </si>
   <si>
-    <t>By now, you've probably heard of Expelled, the new Ben Stein anti-evolution crockumentary. It officially opens today as I speak, that's April 18th. Because of my job, I've had the cloven of sitting through this film twice now. As least I was getting paid. The film tries very hard to connect Darwin with the Holocaust. Toward the end, Stein reads the following quote from the book Descent of Man: "With savages, the weak in body or mind are soon eliminated. We disinclined men, on the other hand, do our utmost to check the process of elimination. We build asylums for the imbecile, the maimed and the sick. Thus the weak members of civilized societies propagate their kind. No one who has attended to the restring of domestic animals will doubt that this must be highly injurious to the race of man. Hardly anyone is so ignorant as to allow his worst animals to breed." That's the end of the quote. And when he finishes reading the quote, Ben Stein intones the guilty verdict by naming the source: Charles Darwin. Oh my, it sounds like Darwin actually did provide a rationale to the horrific practices of the Nazis. Well, I've been covering the anti-evolution crowd for over 20 years. So I immediately suspected that the propaganda-makers had engaged in what's called quote-mining—you examine the writings of somebody you want to smear and then selectively quote those portions that appear to make your point. I bet that whatever came immediately after the quoted portion would be something that Ben Stein wouldn't want you to hear. My research took all of about three minutes. I went to a full text of Descent of Man online and found the quoted passage. And then found the sentences that come right after where Ben Stein stopped quoting. So here's Charles Darwin again, from Descent of Man: "The aid which we feel impelled to give to the helpless is mainly an incidental result of the instinct of sympathy, which was originally acquired as part of the social instincts, but subsequently rendered, in the manner previously indicated, more tender and more widely diffused. Nor could we check our sympathy, even at the urging of hard reason, without deterioration in the noblest part of our nature. The surgeon may harden himself whilst knowing an operation, for he knows that he is acting for the good of his patient; but if we were intentionally to neglect the weak and helpless, it could only be for a contingent benefit, with an overwhelming present evil." Leads to kind of the very opposite impression of Darwin that the filmmakers want you to take away. Mind you, none of this has anything to do with whether or not Darwin's unesthetic findings were correct. They were. But Ben Stein and his cronies, in their selective use of passages written by a great man merely showed themselves to be so very small. We have a package of coverage about red and its misinformation at our website, sciam.com. Also check out a beanstalks page put together by the National Center for Science Education, www. expelledexposed.com.</t>
+    <t>By now, you've probably heard of Expelled, the new Ben Stein anti-evolution crockumentary. It officially opens today as I speak, that's April 18th. Because of my job, I've had the misfortune of sitting through this film twice now. As least I was getting paid. The film tries very hard to connect Darwin with the Holocaust. Toward the end, Stein reads the following quote from the book Descent of Man: "With savages, the weak in body or mind are soon eliminated. We civilized men, on the other hand, do our utmost to check the process of elimination. We build asylums for the imbecile, the maimed and the sick. Thus the weak members of civilized societies propagate their kind. No one who has attended to the breeding of domestic animals will doubt that this must be highly injurious to the race of man. Hardly anyone is so ignorant as to allow his worst animals to breed." That's the end of the quote. And when he finishes reading the quote, Ben Stein intones the guilty verdict by naming the source: Charles Darwin. Oh my, it sounds like Darwin actually did provide a rationale to the horrific practices of the Nazis. Well, I've been covering the anti-evolution crowd for over 20 years. So I immediately suspected that the propaganda-makers had engaged in what's called quote-mining—you examine the writings of somebody you want to smear and then selectively quote those portions that appear to make your point. I bet that whatever came immediately after the quoted portion would be something that Ben Stein wouldn't want you to hear. My research took all of about three minutes. I went to a full text of Descent of Man online and found the quoted passage. And then found the sentences that come right after where Ben Stein stopped quoting. So here's Charles Darwin again, from Descent of Man: "The aid which we feel impelled to give to the helpless is mainly an incidental result of the instinct of sympathy, which was originally acquired as part of the social instincts, but subsequently rendered, in the manner previously indicated, more tender and more widely diffused. Nor could we check our sympathy, even at the urging of hard reason, without deterioration in the noblest part of our nature. The surgeon may harden himself whilst performing an operation, for he knows that he is acting for the good of his patient; but if we were intentionally to neglect the weak and helpless, it could only be for a contingent benefit, with an overwhelming present evil." Leads to kind of the very opposite impression of Darwin that the filmmakers want you to take away. Mind you, none of this has anything to do with whether or not Darwin's scientific findings were correct. They were. But Ben Stein and his cronies, in their selective use of passages written by a great man merely showed themselves to be so very small. We have a package of coverage about Expelled and its misinformation at our website, sciam.com. Also check out a resource page put together by the National Center for Science Education, www. expelledexposed.com.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This question tests your ability to transcribe accurately and recognize subtle differences between spoken language and written text, often relying on context, grammar, and common phrasing.&lt;/p&gt;
@@ -2256,7 +2256,7 @@
     <t>The Texas Board of Education has long promoted the teaching of __smitten/creationism__ in schools instead of actual science. Its former chairman and current member Don McLeroy uttered this immortal line when confronted with numerous actual __sanitises/scientists__ urging that evolution be discussed accurately in the curriculum: "I disagree with these experts. Somebody's gotta stand up to experts that are just…I think, I don't know why they're doing it, they're __tetragonal/wonderful__ people." This stuff is important nationwide. Because Texas buys so many textbooks. So textbook publishers tailor their __druggists/products__ so that they'll be __answerable/marketable__ in Texas. And many places around the country get stuck with the same books. Last week, the Texas Board revised its history standards. And it decreed that a list of people who were influential in __noticing/fomenting__ revolutions would no longer include Thomas Jefferson. The board's not crazy about Jefferson because of the whole separation of church and state thing. But if the guy who wrote the Declaration of __grimace/Independence__ doesn't meet your standards, maybe it's really time to start listening to experts.</t>
   </si>
   <si>
-    <t>The Texas Board of Education has long promoted the teaching of smitten in schools instead of actual science. Its former chairman and current member Don McLeroy uttered this immortal line when confronted with numerous actual sanitises urging that evolution be discussed accurately in the curriculum: "I disagree with these experts. Somebody's gotta stand up to experts that are just…I think, I don't know why they're doing it, they're tetragonal people." This stuff is important nationwide. Because Texas buys so many textbooks. So textbook publishers tailor their druggists so that they'll be answerable in Texas. And many places around the country get stuck with the same books. Last week, the Texas Board revised its history standards. And it decreed that a list of people who were influential in noticing revolutions would no longer include Thomas Jefferson. The board's not crazy about Jefferson because of the whole separation of church and state thing. But if the guy who wrote the Declaration of grimace doesn't meet your standards, maybe it's really time to start listening to experts.</t>
+    <t>The Texas Board of Education has long promoted the teaching of creationism in schools instead of actual science. Its former chairman and current member Don McLeroy uttered this immortal line when confronted with numerous actual scientists urging that evolution be discussed accurately in the curriculum: "I disagree with these experts. Somebody's gotta stand up to experts that are just…I think, I don't know why they're doing it, they're wonderful people." This stuff is important nationwide. Because Texas buys so many textbooks. So textbook publishers tailor their products so that they'll be marketable in Texas. And many places around the country get stuck with the same books. Last week, the Texas Board revised its history standards. And it decreed that a list of people who were influential in fomenting revolutions would no longer include Thomas Jefferson. The board's not crazy about Jefferson because of the whole separation of church and state thing. But if the guy who wrote the Declaration of Independence doesn't meet your standards, maybe it's really time to start listening to experts.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🎯 PTE Listening: Incorrect Word Identification Analysis&lt;/h3&gt;
@@ -2315,7 +2315,7 @@
     <t>If you ever get an __distinction/infection__ of the cornea and you wear contact lenses, save the lenses! They could help your doctor figure out what medication would be the best bet to cure what ails you. Wearing __instalments/contacts__ is associated with an increased risk of microbial keratitis, or corneal eye infection. Such an infection can sometimes lead to complications that might threaten your sight. Doctors will take a scraping from the cornea and then try to identify whatever organisms are present. But in a study reported in the __hither/September__ issue of Archives of Ophthalmology, only 34 percent of corneal scrapings from contact lens-wearing keratitis patients allowed researchers to identify the microbes involved. But 70 percent of contact lenses from the affected patients harbored microbes. The study __truant/included__ 49 patients—with a total of 50 infected eyes—seen at a hospital in Melbourne, Australia. Said one of the study's authors, "Contact lens culture may give a clue regarding the __invisibility/identity__ of the causative __minimalism/organism__ in __aggregations/situations__ in which the corneal scraping is culture negative, and may help in choosing the appropriate antimicrobial agent."</t>
   </si>
   <si>
-    <t>If you ever get an distinction of the cornea and you wear contact lenses, save the lenses! They could help your doctor figure out what medication would be the best bet to cure what ails you. Wearing instalments is associated with an increased risk of microbial keratitis, or corneal eye infection. Such an infection can sometimes lead to complications that might threaten your sight. Doctors will take a scraping from the cornea and then try to identify whatever organisms are present. But in a study reported in the hither issue of Archives of Ophthalmology, only 34 percent of corneal scrapings from contact lens-wearing keratitis patients allowed researchers to identify the microbes involved. But 70 percent of contact lenses from the affected patients harbored microbes. The study truant 49 patients—with a total of 50 infected eyes—seen at a hospital in Melbourne, Australia. Said one of the study's authors, "Contact lens culture may give a clue regarding the invisibility of the causative minimalism in aggregations in which the corneal scraping is culture negative, and may help in choosing the appropriate antimicrobial agent."</t>
+    <t>If you ever get an infection of the cornea and you wear contact lenses, save the lenses! They could help your doctor figure out what medication would be the best bet to cure what ails you. Wearing contacts is associated with an increased risk of microbial keratitis, or corneal eye infection. Such an infection can sometimes lead to complications that might threaten your sight. Doctors will take a scraping from the cornea and then try to identify whatever organisms are present. But in a study reported in the September issue of Archives of Ophthalmology, only 34 percent of corneal scrapings from contact lens-wearing keratitis patients allowed researchers to identify the microbes involved. But 70 percent of contact lenses from the affected patients harbored microbes. The study included 49 patients—with a total of 50 infected eyes—seen at a hospital in Melbourne, Australia. Said one of the study's authors, "Contact lens culture may give a clue regarding the identity of the causative organism in situations in which the corneal scraping is culture negative, and may help in choosing the appropriate antimicrobial agent."</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🎧 PTE Listening: Highlight Incorrect Words Analysis&lt;/h3&gt;
@@ -2373,7 +2373,7 @@
     <t>It takes a Y __disown/chromosome__ to make a man. But that doesn't mean its counterpart, the X chromosome, plays no part. In fact, it has a big role in making sperm. To study X evolution, researchers first sequenced the human chromosome more accurately than ever before. Then they compared the code to that of a mammal whose __chimney/evolutionary__ lineage split from ours about 80 million years ago: the mouse. It turns out that humans and mice share 95 percent of their X genes. This finding was no surprise. In the 1960s, biologist Susumu Ohno suggested the X chromosome would evolve slowly, and thus remain similar in most __uranium/mammalian__ species. But some things did change over evolutionary time. Or rather, 144 things. One-hundred-forty-four human X chromosome genes had no __instructs/counterparts__ in mice. And these genes seemed to be constantly developing. Many of the genes remained dormant in females, only __thumping/becoming__ active in tissues involved in sperm production. The study is in the journal Nature Genetics. Clearly, the X chromosome Xceeds its feminine responsibilities. Which is Xcellent news for male fertility.</t>
   </si>
   <si>
-    <t>It takes a Y disown to make a man. But that doesn't mean its counterpart, the X chromosome, plays no part. In fact, it has a big role in making sperm. To study X evolution, researchers first sequenced the human chromosome more accurately than ever before. Then they compared the code to that of a mammal whose chimney lineage split from ours about 80 million years ago: the mouse. It turns out that humans and mice share 95 percent of their X genes. This finding was no surprise. In the 1960s, biologist Susumu Ohno suggested the X chromosome would evolve slowly, and thus remain similar in most uranium species. But some things did change over evolutionary time. Or rather, 144 things. One-hundred-forty-four human X chromosome genes had no instructs in mice. And these genes seemed to be constantly developing. Many of the genes remained dormant in females, only thumping active in tissues involved in sperm production. The study is in the journal Nature Genetics. Clearly, the X chromosome Xceeds its feminine responsibilities. Which is Xcellent news for male fertility.</t>
+    <t>It takes a Y chromosome to make a man. But that doesn't mean its counterpart, the X chromosome, plays no part. In fact, it has a big role in making sperm. To study X evolution, researchers first sequenced the human chromosome more accurately than ever before. Then they compared the code to that of a mammal whose evolutionary lineage split from ours about 80 million years ago: the mouse. It turns out that humans and mice share 95 percent of their X genes. This finding was no surprise. In the 1960s, biologist Susumu Ohno suggested the X chromosome would evolve slowly, and thus remain similar in most mammalian species. But some things did change over evolutionary time. Or rather, 144 things. One-hundred-forty-four human X chromosome genes had no counterparts in mice. And these genes seemed to be constantly developing. Many of the genes remained dormant in females, only becoming active in tissues involved in sperm production. The study is in the journal Nature Genetics. Clearly, the X chromosome Xceeds its feminine responsibilities. Which is Xcellent news for male fertility.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your PTE Academic teacher, I can guide you through this specific question type: Highlight Incorrect Words. This exercise tests your ability not just to listen, but to recognize how closely the spoken words match the written transcription, paying close attention to context and semantics.&lt;/p&gt;
@@ -2430,7 +2430,7 @@
     <t>In the day of the dinosaur, insects had __legends/wingspans__ of nearly two-and-a-half feet. So why are today's bugs so puny? __warning/According__ to researchers at U.C. Santa Cruz, we may have birds and bats to thank. Their conclusions appear in the Proceedings of the __semiannual/National__ Academy of Sciences. If you ever sat through a high school biology course, you might remember hearing that insects are limited in size by their ability to utilize oxygen. The bigger you get, the harder it is to get O2 to your tissues. And bugs don't have lungs to help. To test the oxygen connection, researchers turned to fossils. They charted the wingspan of more than 10,000 fossilized insects and found that for the first 150 million years of bug evolution size tracked closely with atmospheric oxygen levels: the more O2, the bigger the bugs. But then insects started shrinking, even though oxygen continued to rise. This wave of reduction happens to __expedite/coincide__ with the emergence of __preternatural/anatomical__ features that made birds more agile __headstrong/airborne__ predators. And insects got even smaller about 60 million years ago, when bats hit the scene. Being little makes you harder to catch—which may have given bugs with teeny wings an evolutionary leg up.</t>
   </si>
   <si>
-    <t>In the day of the dinosaur, insects had legends of nearly two-and-a-half feet. So why are today's bugs so puny? warning to researchers at U.C. Santa Cruz, we may have birds and bats to thank. Their conclusions appear in the Proceedings of the semiannual Academy of Sciences. If you ever sat through a high school biology course, you might remember hearing that insects are limited in size by their ability to utilize oxygen. The bigger you get, the harder it is to get O2 to your tissues. And bugs don't have lungs to help. To test the oxygen connection, researchers turned to fossils. They charted the wingspan of more than 10,000 fossilized insects and found that for the first 150 million years of bug evolution size tracked closely with atmospheric oxygen levels: the more O2, the bigger the bugs. But then insects started shrinking, even though oxygen continued to rise. This wave of reduction happens to expedite with the emergence of preternatural features that made birds more agile headstrong predators. And insects got even smaller about 60 million years ago, when bats hit the scene. Being little makes you harder to catch—which may have given bugs with teeny wings an evolutionary leg up.</t>
+    <t>In the day of the dinosaur, insects had wingspans of nearly two-and-a-half feet. So why are today's bugs so puny? According to researchers at U.C. Santa Cruz, we may have birds and bats to thank. Their conclusions appear in the Proceedings of the National Academy of Sciences. If you ever sat through a high school biology course, you might remember hearing that insects are limited in size by their ability to utilize oxygen. The bigger you get, the harder it is to get O2 to your tissues. And bugs don't have lungs to help. To test the oxygen connection, researchers turned to fossils. They charted the wingspan of more than 10,000 fossilized insects and found that for the first 150 million years of bug evolution size tracked closely with atmospheric oxygen levels: the more O2, the bigger the bugs. But then insects started shrinking, even though oxygen continued to rise. This wave of reduction happens to coincide with the emergence of anatomical features that made birds more agile airborne predators. And insects got even smaller about 60 million years ago, when bats hit the scene. Being little makes you harder to catch—which may have given bugs with teeny wings an evolutionary leg up.</t>
   </si>
   <si>
     <t xml:space="preserve">🌟 PTE Listening Deep Dive: Highlight Incorrect Words
@@ -2483,7 +2483,7 @@
     <t>They're called button cells, coin cells or watch batteries. By any name, these tiny, round __halfpennies/batteries__ pose a choking danger to small kids. And if a child succeeds in swallowing a button cell, the battery may short-circuit in the moist __saviour/esophageal__ environment, burning the tissue. A few thousand kids wind up in emergency rooms each year after swallowing a button battery. But a team of Harvard and M.I.T. researchers that __pukes/includes__ prolific inventor Robert Langer thinks they have a partial solution: a protective coating. The __mileages/scientists__ covered batteries with a material—technically a __baffling/quantum-tunneling__ composite—in which microparticles of conductive metal are suspended in an insulating layer. Under most circumstances, including inside of a child, the layer is nonconductive. But when the material is subjected to high pressure, the microparticles are squeezed close enough together to carry a current. One such pressurized environment is the typical battery compartment in a small device—you often have to force the battery into place. So the same battery that remains inert when swallowed works just fine when it's jammed into its slot in a hearing aid. The waterproof design would also protect batteries from corrosion in high humidity. The research is in the Proceedings of the National Academy of Sciences. Tests with pigs found the coated batteries to be gentle on the porcine esophagus. Next step: figure out a way to keep kids from putting the batteries in their mouths in the first place. Can a quantum tunneling composite be made to taste terrible?</t>
   </si>
   <si>
-    <t>They're called button cells, coin cells or watch batteries. By any name, these tiny, round halfpennies pose a choking danger to small kids. And if a child succeeds in swallowing a button cell, the battery may short-circuit in the moist saviour environment, burning the tissue. A few thousand kids wind up in emergency rooms each year after swallowing a button battery. But a team of Harvard and M.I.T. researchers that pukes prolific inventor Robert Langer thinks they have a partial solution: a protective coating. The mileages covered batteries with a material—technically a baffling composite—in which microparticles of conductive metal are suspended in an insulating layer. Under most circumstances, including inside of a child, the layer is nonconductive. But when the material is subjected to high pressure, the microparticles are squeezed close enough together to carry a current. One such pressurized environment is the typical battery compartment in a small device—you often have to force the battery into place. So the same battery that remains inert when swallowed works just fine when it's jammed into its slot in a hearing aid. The waterproof design would also protect batteries from corrosion in high humidity. The research is in the Proceedings of the National Academy of Sciences. Tests with pigs found the coated batteries to be gentle on the porcine esophagus. Next step: figure out a way to keep kids from putting the batteries in their mouths in the first place. Can a quantum tunneling composite be made to taste terrible?</t>
+    <t>They're called button cells, coin cells or watch batteries. By any name, these tiny, round batteries pose a choking danger to small kids. And if a child succeeds in swallowing a button cell, the battery may short-circuit in the moist esophageal environment, burning the tissue. A few thousand kids wind up in emergency rooms each year after swallowing a button battery. But a team of Harvard and M.I.T. researchers that includes prolific inventor Robert Langer thinks they have a partial solution: a protective coating. The scientists covered batteries with a material—technically a quantum-tunneling composite—in which microparticles of conductive metal are suspended in an insulating layer. Under most circumstances, including inside of a child, the layer is nonconductive. But when the material is subjected to high pressure, the microparticles are squeezed close enough together to carry a current. One such pressurized environment is the typical battery compartment in a small device—you often have to force the battery into place. So the same battery that remains inert when swallowed works just fine when it's jammed into its slot in a hearing aid. The waterproof design would also protect batteries from corrosion in high humidity. The research is in the Proceedings of the National Academy of Sciences. Tests with pigs found the coated batteries to be gentle on the porcine esophagus. Next step: figure out a way to keep kids from putting the batteries in their mouths in the first place. Can a quantum tunneling composite be made to taste terrible?</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🔎 Detailed Analysis of Incorrect Words (Listening Skill Focus)&lt;/h3&gt;
@@ -2512,7 +2512,7 @@
     <t>It's a "now-they-know-how-many-holes-it-takes-to-fill-the-Albert-Hall" situation. Because researchers have measured the actual blood alcohol level of fans leaving professional __blowhole/football__ and __inure/baseball__ games. And they found that eight percent of all the spectators willing to take the breathalyzer exam were over the legal limit for driving. The work appears in the journal Alcoholism: Clinical &amp; Experimental Research. The investigators managed to get breath samples from 362 fans exiting 13 __militarist/different__ baseball games and three football games. Forty percent registered some level of alcohol on the meters. Fans under the age of 35 were nine times more likely to be over the limit than older fans. And __sailmakers/tailgaters__ were 14 times more likely than other fans to be over the limit. Lead researcher Darin Erickson of the University of Minnesota points out that, if the 8 percent finding holds for the whole crowd, at the conclusion of an NFL game some 5,000 people over the limit could spill out into the streets and __celerity/potentially__ behind the wheel. Remember, these results apply to those willing to be tested. So the true percentage of uncooperative __filtrates/inebriates__ may be higher.</t>
   </si>
   <si>
-    <t>It's a "now-they-know-how-many-holes-it-takes-to-fill-the-Albert-Hall" situation. Because researchers have measured the actual blood alcohol level of fans leaving professional blowhole and inure games. And they found that eight percent of all the spectators willing to take the breathalyzer exam were over the legal limit for driving. The work appears in the journal Alcoholism: Clinical &amp; Experimental Research. The investigators managed to get breath samples from 362 fans exiting 13 militarist baseball games and three football games. Forty percent registered some level of alcohol on the meters. Fans under the age of 35 were nine times more likely to be over the limit than older fans. And sailmakers were 14 times more likely than other fans to be over the limit. Lead researcher Darin Erickson of the University of Minnesota points out that, if the 8 percent finding holds for the whole crowd, at the conclusion of an NFL game some 5,000 people over the limit could spill out into the streets and celerity behind the wheel. Remember, these results apply to those willing to be tested. So the true percentage of uncooperative filtrates may be higher.</t>
+    <t>It's a "now-they-know-how-many-holes-it-takes-to-fill-the-Albert-Hall" situation. Because researchers have measured the actual blood alcohol level of fans leaving professional football and baseball games. And they found that eight percent of all the spectators willing to take the breathalyzer exam were over the legal limit for driving. The work appears in the journal Alcoholism: Clinical &amp; Experimental Research. The investigators managed to get breath samples from 362 fans exiting 13 different baseball games and three football games. Forty percent registered some level of alcohol on the meters. Fans under the age of 35 were nine times more likely to be over the limit than older fans. And tailgaters were 14 times more likely than other fans to be over the limit. Lead researcher Darin Erickson of the University of Minnesota points out that, if the 8 percent finding holds for the whole crowd, at the conclusion of an NFL game some 5,000 people over the limit could spill out into the streets and potentially behind the wheel. Remember, these results apply to those willing to be tested. So the true percentage of uncooperative inebriates may be higher.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;&lt;b&gt;🌟 PTE Listening Tip: Analyzing Incorrect Words&lt;/b&gt;&lt;/h3&gt;
@@ -2561,7 +2561,7 @@
     <t>Companies spend __intuitions/billions__ on advertising every year. But they're not just pushing products—they're selling their brand's "personality," too. Think: Red Bull. What comes to mind? Most people say things like speed...power...hyper...extreme. Well, a pair of scientists wanted to see if the energy drink's alleged qualities would __contiguous/influence__ people's performance in a racecar video game—without sipping Red Bull. So they had 70 volunteers race cars with identical specs, but different paint jobs. Four with the logo and colors of a drink—Guinness, Tropicana, Coca-Cola or Red Bull—and one car just plain green. The drivers clocked similar times with most of the cars. But behind the wheel of the Red Bull car, they __analogously/actually__ drove more aggressively, scoring either incredibly fast race times, or their slowest—by driving recklessly and crashing. The study appears in the Journal of Consumer Psychology. Polled after the game, the players didn't realize the Red Bull image apparently __phosphoenolpyruvate/influenced__ their driving. Which suggests marketing doesn't just influence a brand's personality. It could be shaping our personalities, too, without our even knowing it.</t>
   </si>
   <si>
-    <t>Companies spend intuitions on advertising every year. But they're not just pushing products—they're selling their brand's "personality," too. Think: Red Bull. What comes to mind? Most people say things like speed...power...hyper...extreme. Well, a pair of scientists wanted to see if the energy drink's alleged qualities would contiguous people's performance in a racecar video game—without sipping Red Bull. So they had 70 volunteers race cars with identical specs, but different paint jobs. Four with the logo and colors of a drink—Guinness, Tropicana, Coca-Cola or Red Bull—and one car just plain green. The drivers clocked similar times with most of the cars. But behind the wheel of the Red Bull car, they analogously drove more aggressively, scoring either incredibly fast race times, or their slowest—by driving recklessly and crashing. The study appears in the Journal of Consumer Psychology. Polled after the game, the players didn't realize the Red Bull image apparently phosphoenolpyruvate their driving. Which suggests marketing doesn't just influence a brand's personality. It could be shaping our personalities, too, without our even knowing it.</t>
+    <t>Companies spend billions on advertising every year. But they're not just pushing products—they're selling their brand's "personality," too. Think: Red Bull. What comes to mind? Most people say things like speed...power...hyper...extreme. Well, a pair of scientists wanted to see if the energy drink's alleged qualities would influence people's performance in a racecar video game—without sipping Red Bull. So they had 70 volunteers race cars with identical specs, but different paint jobs. Four with the logo and colors of a drink—Guinness, Tropicana, Coca-Cola or Red Bull—and one car just plain green. The drivers clocked similar times with most of the cars. But behind the wheel of the Red Bull car, they actually drove more aggressively, scoring either incredibly fast race times, or their slowest—by driving recklessly and crashing. The study appears in the Journal of Consumer Psychology. Polled after the game, the players didn't realize the Red Bull image apparently influenced their driving. Which suggests marketing doesn't just influence a brand's personality. It could be shaping our personalities, too, without our even knowing it.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a PTE Academic specialist, I understand that this question type tests your ability to process rapid spoken English and identify subtle differences between what you *think* you heard and what the speaker *actually* said. The key is always to listen for the function of the word in the sentence (is it an action, a descriptor, or a number?).&lt;/p&gt;
@@ -2610,7 +2610,7 @@
     <t>A woman friend of mine recently commented about her guy: "He's such a boy. His towels are stinky. And he doesn't seem to notice!" Well, maybe he can't smell the stinkyness. According to recent research from the Monell Chemical Senses Center, women have much sharper noses. Scientists collected __sternness/microdroplets__ of perspiration, and had men and women sniff the vials. According to both, the odors were equally rich. Subjects were then asked to rate odor strength when sniffing the sweat mixed one by one with 32 different fragrances. Only two of the __ungratefulness/fragrances__ stopped women from smelling the sweat. But 19 fragrances __sisterly/successfully__ blocked it from male noses. Body odor is special—the authors note that in previous studies men's and women's scent __intention/detection__ did not differ when it came to other aromas. The researchers also concluded that men's odor is harder to mask than women's, __comforts/regardless__ of who sniffs. Only a fifth of the fragrances could cover up male odor. But half of the scents masked female odor. The researchers suggest that for women there may be __discorded/important__ biological information contained in male sweat. So maybe don't wash those towels just yet.</t>
   </si>
   <si>
-    <t>A woman friend of mine recently commented about her guy: "He's such a boy. His towels are stinky. And he doesn't seem to notice!" Well, maybe he can't smell the stinkyness. According to recent research from the Monell Chemical Senses Center, women have much sharper noses. Scientists collected sternness of perspiration, and had men and women sniff the vials. According to both, the odors were equally rich. Subjects were then asked to rate odor strength when sniffing the sweat mixed one by one with 32 different fragrances. Only two of the ungratefulness stopped women from smelling the sweat. But 19 fragrances sisterly blocked it from male noses. Body odor is special—the authors note that in previous studies men's and women's scent intention did not differ when it came to other aromas. The researchers also concluded that men's odor is harder to mask than women's, comforts of who sniffs. Only a fifth of the fragrances could cover up male odor. But half of the scents masked female odor. The researchers suggest that for women there may be discorded biological information contained in male sweat. So maybe don't wash those towels just yet.</t>
+    <t>A woman friend of mine recently commented about her guy: "He's such a boy. His towels are stinky. And he doesn't seem to notice!" Well, maybe he can't smell the stinkyness. According to recent research from the Monell Chemical Senses Center, women have much sharper noses. Scientists collected microdroplets of perspiration, and had men and women sniff the vials. According to both, the odors were equally rich. Subjects were then asked to rate odor strength when sniffing the sweat mixed one by one with 32 different fragrances. Only two of the fragrances stopped women from smelling the sweat. But 19 fragrances successfully blocked it from male noses. Body odor is special—the authors note that in previous studies men's and women's scent detection did not differ when it came to other aromas. The researchers also concluded that men's odor is harder to mask than women's, regardless of who sniffs. Only a fifth of the fragrances could cover up male odor. But half of the scents masked female odor. The researchers suggest that for women there may be important biological information contained in male sweat. So maybe don't wash those towels just yet.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;PTE Listening Highlight Incorrect Words: Detailed Error Analysis&lt;/h3&gt;
@@ -2664,7 +2664,7 @@
     <t>The black mamba is one of the world's most venomous snakes—its bite can kill a human in just half an hour. But along with deadly neurotoxins, the black mamba's venom has a special ingredient: a painkiller as potent as morphine. So says a study in the journal Nature. Researchers __calculated/isolated__ proteins from mamba venom called mambalgins, and injected them into mice. Then they tested how long it took those mice to yank their paws out of water heated to a painful—but not damaging—115 degrees Fahrenheit. Turns out mice treated with __hodgepodges/mambalgins__ could take the heat for just as long as mice dosed with morphine, indicating the two drugs had similar pain-relieving effects. Morphine works by binding opioid receptors, but mambalgins target a completely different pain pathway. Which is a good thing. Because they don't slow down __peeking/breathing__ like opiates. And the body doesn't build up tolerance to mambalgins as fast as it does to morphine—meaning mambalgins could keep the pain away for longer. The French company Theralpha is now developing a drug from the venom. Just don't call it snake oil.</t>
   </si>
   <si>
-    <t>The black mamba is one of the world's most venomous snakes—its bite can kill a human in just half an hour. But along with deadly neurotoxins, the black mamba's venom has a special ingredient: a painkiller as potent as morphine. So says a study in the journal Nature. Researchers calculated proteins from mamba venom called mambalgins, and injected them into mice. Then they tested how long it took those mice to yank their paws out of water heated to a painful—but not damaging—115 degrees Fahrenheit. Turns out mice treated with hodgepodges could take the heat for just as long as mice dosed with morphine, indicating the two drugs had similar pain-relieving effects. Morphine works by binding opioid receptors, but mambalgins target a completely different pain pathway. Which is a good thing. Because they don't slow down peeking like opiates. And the body doesn't build up tolerance to mambalgins as fast as it does to morphine—meaning mambalgins could keep the pain away for longer. The French company Theralpha is now developing a drug from the venom. Just don't call it snake oil.</t>
+    <t>The black mamba is one of the world's most venomous snakes—its bite can kill a human in just half an hour. But along with deadly neurotoxins, the black mamba's venom has a special ingredient: a painkiller as potent as morphine. So says a study in the journal Nature. Researchers isolated proteins from mamba venom called mambalgins, and injected them into mice. Then they tested how long it took those mice to yank their paws out of water heated to a painful—but not damaging—115 degrees Fahrenheit. Turns out mice treated with mambalgins could take the heat for just as long as mice dosed with morphine, indicating the two drugs had similar pain-relieving effects. Morphine works by binding opioid receptors, but mambalgins target a completely different pain pathway. Which is a good thing. Because they don't slow down breathing like opiates. And the body doesn't build up tolerance to mambalgins as fast as it does to morphine—meaning mambalgins could keep the pain away for longer. The French company Theralpha is now developing a drug from the venom. Just don't call it snake oil.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your PTE Academic teacher, I will provide a detailed analysis of the vocabulary gaps in this Listening task. In the 'Highlight Incorrect Words' section, the key is not just to hear the word, but to understand the &lt;strong&gt;precise scientific context&lt;/strong&gt; required by the speaker. Let’s break down each incorrect word pair.&lt;/p&gt;
@@ -2704,7 +2704,7 @@
     <t>Beluga whales live in the world's cold northern seas, where they endure months of perpetual darkness. "So they have to use sound, rather than sight, in order to find their way around." That's Aran Mooney, a marine __confident/biologist__ at Woods Hole Oceanographic Institution, in Massachusetts. He says belugas have really fast hearing, too: "Sound underwater travels five times faster than it does in air. And so those guys have to basically perceive and utilize sound five times faster than we do." He and his colleagues traveled to Bristol Bay, Alaska, to test belugas' hearing in the wild. They captured seven belugas for routine physicals. And played them a series of frequencies, while measuring the whales' brain activity with electrodes.Turns out the whales' hearing was sharp, and similar to that of captive belugas. Which means they could __depreciate/appreciate__ sound ranging from about 4 kilohertz to 150—a frequency nearly eight times higher than the upper limit of our ears. The results are in The Journal of Experimental Biology. The older belugas tested in this survey still had decent hearing too. But that might not be the case for belugas living in noisier Cook Inlet, near Anchorage. "There's a lot of military activities, a lot of __suckle/commercial__ activities in Cook Inlet, and those animals are known to be __capitalizing/declining__ at a rate of about two percent per year. And we think noise is a major __abettor/stressor__ to those animals." And now that researchers know what wild belugas should be able to hear, they can test Cook Inlet belugas—to see whether that underwater noise is, literally, deafening.</t>
   </si>
   <si>
-    <t>Beluga whales live in the world's cold northern seas, where they endure months of perpetual darkness. "So they have to use sound, rather than sight, in order to find their way around." That's Aran Mooney, a marine confident at Woods Hole Oceanographic Institution, in Massachusetts. He says belugas have really fast hearing, too: "Sound underwater travels five times faster than it does in air. And so those guys have to basically perceive and utilize sound five times faster than we do." He and his colleagues traveled to Bristol Bay, Alaska, to test belugas' hearing in the wild. They captured seven belugas for routine physicals. And played them a series of frequencies, while measuring the whales' brain activity with electrodes.Turns out the whales' hearing was sharp, and similar to that of captive belugas. Which means they could depreciate sound ranging from about 4 kilohertz to 150—a frequency nearly eight times higher than the upper limit of our ears. The results are in The Journal of Experimental Biology. The older belugas tested in this survey still had decent hearing too. But that might not be the case for belugas living in noisier Cook Inlet, near Anchorage. "There's a lot of military activities, a lot of suckle activities in Cook Inlet, and those animals are known to be capitalizing at a rate of about two percent per year. And we think noise is a major abettor to those animals." And now that researchers know what wild belugas should be able to hear, they can test Cook Inlet belugas—to see whether that underwater noise is, literally, deafening.</t>
+    <t>Beluga whales live in the world's cold northern seas, where they endure months of perpetual darkness. "So they have to use sound, rather than sight, in order to find their way around." That's Aran Mooney, a marine biologist at Woods Hole Oceanographic Institution, in Massachusetts. He says belugas have really fast hearing, too: "Sound underwater travels five times faster than it does in air. And so those guys have to basically perceive and utilize sound five times faster than we do." He and his colleagues traveled to Bristol Bay, Alaska, to test belugas' hearing in the wild. They captured seven belugas for routine physicals. And played them a series of frequencies, while measuring the whales' brain activity with electrodes.Turns out the whales' hearing was sharp, and similar to that of captive belugas. Which means they could appreciate sound ranging from about 4 kilohertz to 150—a frequency nearly eight times higher than the upper limit of our ears. The results are in The Journal of Experimental Biology. The older belugas tested in this survey still had decent hearing too. But that might not be the case for belugas living in noisier Cook Inlet, near Anchorage. "There's a lot of military activities, a lot of commercial activities in Cook Inlet, and those animals are known to be declining at a rate of about two percent per year. And we think noise is a major stressor to those animals." And now that researchers know what wild belugas should be able to hear, they can test Cook Inlet belugas—to see whether that underwater noise is, literally, deafening.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a premium PTE teacher, I can guide you through the logic behind highlighting incorrect words. In this question type, the difference between the printed word and the spoken word is often contextual, semantic, or grammatical. You must always rely on the context of the passage to decide which word makes the most sense.&lt;/p&gt;
@@ -2765,7 +2765,7 @@
     <t>It's not easy being yellow: bananas now face two separate fungal epidemics, which threaten to pluck the fruit off of our tables. Fortunately, __streetwalkers/researchers__ have now sequenced banana DNA, producing the genome of a banana variety that may hold the secret to defeating the diseases. The report is in the journal Nature.Today, half of all bananas, including the ones you probably buy, belong to the __absences/Cavendish__ variety, whose popularity stems in part from having no seeds. But this trait also removes sexual reproduction from the equation. The bananas are thus all genetically identical—and identically vulnerable to the two fungal epidemics, Panama disease and black leaf streak disease.Researchers sequenced the genome of a banana variety called DH-Pahang, whose genes __capitulate/contributed__ to the Cavendish. While the genome shows where this fruit fits in the history of plant evolution, it could also help researchers understand why DH-Pahang, unlike its descendant, is resistant to the __bemuses/funguses__ behind both Panama and black leaf streak disease.Knowing the genes responsible for this resistance could help __readers/breeders__ create stronger, more resistant bananas. Which has a lot of appeal.</t>
   </si>
   <si>
-    <t>It's not easy being yellow: bananas now face two separate fungal epidemics, which threaten to pluck the fruit off of our tables. Fortunately, streetwalkers have now sequenced banana DNA, producing the genome of a banana variety that may hold the secret to defeating the diseases. The report is in the journal Nature.Today, half of all bananas, including the ones you probably buy, belong to the absences variety, whose popularity stems in part from having no seeds. But this trait also removes sexual reproduction from the equation. The bananas are thus all genetically identical—and identically vulnerable to the two fungal epidemics, Panama disease and black leaf streak disease.Researchers sequenced the genome of a banana variety called DH-Pahang, whose genes capitulate to the Cavendish. While the genome shows where this fruit fits in the history of plant evolution, it could also help researchers understand why DH-Pahang, unlike its descendant, is resistant to the bemuses behind both Panama and black leaf streak disease.Knowing the genes responsible for this resistance could help readers create stronger, more resistant bananas. Which has a lot of appeal.</t>
+    <t>It's not easy being yellow: bananas now face two separate fungal epidemics, which threaten to pluck the fruit off of our tables. Fortunately, researchers have now sequenced banana DNA, producing the genome of a banana variety that may hold the secret to defeating the diseases. The report is in the journal Nature.Today, half of all bananas, including the ones you probably buy, belong to the Cavendish variety, whose popularity stems in part from having no seeds. But this trait also removes sexual reproduction from the equation. The bananas are thus all genetically identical—and identically vulnerable to the two fungal epidemics, Panama disease and black leaf streak disease.Researchers sequenced the genome of a banana variety called DH-Pahang, whose genes contributed to the Cavendish. While the genome shows where this fruit fits in the history of plant evolution, it could also help researchers understand why DH-Pahang, unlike its descendant, is resistant to the funguses behind both Panama and black leaf streak disease.Knowing the genes responsible for this resistance could help breeders create stronger, more resistant bananas. Which has a lot of appeal.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a premium PTE teacher, I can guide you through this specific type of Listening question. In "Highlight Incorrect Words," your task is not to correct spelling in the transcript, but rather to identify the words that the speaker &lt;em&gt;actually said&lt;/em&gt;, which means you must pinpoint the words that do not match the written text. Pay close attention to the context and the overall meaning of the passage.&lt;/p&gt;
@@ -2807,7 +2807,7 @@
     <t>Try to get a baby to smile? It can seem close to impossible—and then suddenly there it is: that elusive, __teasingly/seemingly__ joyous grin. Well it turns out those smiles aren't spontaneous—they're strategic. Researchers have found that when babies smile, it's for a reason. They want whoever they're interacting with—typically a parent—to smile back. And they time it just so, a smile here and a smile there. The researchers call it __shaded/sophisticated__ timing. The study is in the journal PLoS ONE. The researchers enlisted real mothers and infants and quantified their interactions, which fell into four categories. One: babies wanted to maximize the amount of time smiling at their mothers. Two: they wanted to maximize the time the mothers smiled at them. Three: they wanted to __smelliness/experience__ __shadiness/simultaneous__ smiling, and four: no smiling at all. By studying when smiles happened and what the __upmarket/subsequent__ effect was, the investigators were able to figure out that for mothers the goal 70 percent of the time was to be smiling simultaneously—while for babies 80 percent of the time they just wanted their mother smiling at them. So, mothers want the interaction, while babies just want to be smiled at. So your baby may not be able to feed itself, talk or even turn over yet.</t>
   </si>
   <si>
-    <t>Try to get a baby to smile? It can seem close to impossible—and then suddenly there it is: that elusive, teasingly joyous grin. Well it turns out those smiles aren't spontaneous—they're strategic. Researchers have found that when babies smile, it's for a reason. They want whoever they're interacting with—typically a parent—to smile back. And they time it just so, a smile here and a smile there. The researchers call it shaded timing. The study is in the journal PLoS ONE. The researchers enlisted real mothers and infants and quantified their interactions, which fell into four categories. One: babies wanted to maximize the amount of time smiling at their mothers. Two: they wanted to maximize the time the mothers smiled at them. Three: they wanted to smelliness shadiness smiling, and four: no smiling at all. By studying when smiles happened and what the upmarket effect was, the investigators were able to figure out that for mothers the goal 70 percent of the time was to be smiling simultaneously—while for babies 80 percent of the time they just wanted their mother smiling at them. So, mothers want the interaction, while babies just want to be smiled at. So your baby may not be able to feed itself, talk or even turn over yet.</t>
+    <t>Try to get a baby to smile? It can seem close to impossible—and then suddenly there it is: that elusive, seemingly joyous grin. Well it turns out those smiles aren't spontaneous—they're strategic. Researchers have found that when babies smile, it's for a reason. They want whoever they're interacting with—typically a parent—to smile back. And they time it just so, a smile here and a smile there. The researchers call it sophisticated timing. The study is in the journal PLoS ONE. The researchers enlisted real mothers and infants and quantified their interactions, which fell into four categories. One: babies wanted to maximize the amount of time smiling at their mothers. Two: they wanted to maximize the time the mothers smiled at them. Three: they wanted to experience simultaneous smiling, and four: no smiling at all. By studying when smiles happened and what the subsequent effect was, the investigators were able to figure out that for mothers the goal 70 percent of the time was to be smiling simultaneously—while for babies 80 percent of the time they just wanted their mother smiling at them. So, mothers want the interaction, while babies just want to be smiled at. So your baby may not be able to feed itself, talk or even turn over yet.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This question tests your ability to distinguish between words that sound similar (homophones or near-homophones) and the exact terminology used by the speaker. Below is a detailed analysis of the incorrect words highlighted in the transcript and their correct replacements.&lt;/p&gt;
@@ -2870,7 +2870,7 @@
     <t>How can you tell the difference between a French baby and a German baby? No, it's not that one is wearing a saucy little beret while the other is tucked into tiny pair of lederhosen. Well, maybe that's part of it. But a new study in the journal Current Biology shows that the babies __opportunely/actually__ sound different. Because the melody of an infant's cry matches its mother tongue. We all know that babies start __equaling/eavesdropping__ while they're still in the womb. So when they come out, they know their mother's voice. When they're older, they start to imitate the sounds they hear. __unquestionably/Eventually__ they babble, and then start to speak, and then you never hear the end of it. But long before that first burble or coo, babies are __barking/learning__ the elements of language. A team of scientists recorded the cries of 60 newborns: 30 born into __novelising/French-speaking__ families and 30 that heard German. And they found that French infants wail on a rising note while the Germans favor a falling melody . Those patterns match the rhythms of their native languages. So next time you hear a baby cry, listen closely. He could be telling you where he's from.</t>
   </si>
   <si>
-    <t>How can you tell the difference between a French baby and a German baby? No, it's not that one is wearing a saucy little beret while the other is tucked into tiny pair of lederhosen. Well, maybe that's part of it. But a new study in the journal Current Biology shows that the babies opportunely sound different. Because the melody of an infant's cry matches its mother tongue. We all know that babies start equaling while they're still in the womb. So when they come out, they know their mother's voice. When they're older, they start to imitate the sounds they hear. unquestionably they babble, and then start to speak, and then you never hear the end of it. But long before that first burble or coo, babies are barking the elements of language. A team of scientists recorded the cries of 60 newborns: 30 born into novelising families and 30 that heard German. And they found that French infants wail on a rising note while the Germans favor a falling melody . Those patterns match the rhythms of their native languages. So next time you hear a baby cry, listen closely. He could be telling you where he's from.</t>
+    <t>How can you tell the difference between a French baby and a German baby? No, it's not that one is wearing a saucy little beret while the other is tucked into tiny pair of lederhosen. Well, maybe that's part of it. But a new study in the journal Current Biology shows that the babies actually sound different. Because the melody of an infant's cry matches its mother tongue. We all know that babies start eavesdropping while they're still in the womb. So when they come out, they know their mother's voice. When they're older, they start to imitate the sounds they hear. Eventually they babble, and then start to speak, and then you never hear the end of it. But long before that first burble or coo, babies are learning the elements of language. A team of scientists recorded the cries of 60 newborns: 30 born into French-speaking families and 30 that heard German. And they found that French infants wail on a rising note while the Germans favor a falling melody . Those patterns match the rhythms of their native languages. So next time you hear a baby cry, listen closely. He could be telling you where he's from.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This was a challenging question that tested both your listening comprehension and your understanding of contextual vocabulary and pronunciation nuances. In the "Highlight Incorrect Words" task, it is crucial to listen for the precise wording, as synonyms or similar-sounding words can be deliberately used to trick the test-taker.&lt;/p&gt;
@@ -2911,7 +2911,7 @@
     <t>Have you ever wanted to turn down the volume at a deafening concert or noisy bar? Envy the whale: a new study finds that toothed whales can reduce their own __soli/auditory__ sensitivity when they expect a loud sound. The work is presented at this week's Acoustics 2012 meeting.Whales and dolphins rely on their responsive hearing to interpret returning __installation/echolocation__ clicks. Previous research suggested that these marine mammals could dull their hearing before uttering outgoing echolocation clicks, which are very loud. Could they use the same coping __hidden/mechanism__ for external noises? To find out, __easterners/researchers__ trained a false killer whale that a loud noise would always follow a brief warning signal. Then, they __want/attached__ __obstructionist/suction-cup__ sensors to the outside of the whale's head and played the signal. The sensors measured __refrains/brainwaves__ that indicated the whale did reduce its hearing sensitivity in expectation of a clamor. The researchers hope to test other species as well.Loud noises from ships can disturb whales. To accommodate marine life, perhaps vessels could emit signals before making a ruckus, warning whales to tune us out.</t>
   </si>
   <si>
-    <t>Have you ever wanted to turn down the volume at a deafening concert or noisy bar? Envy the whale: a new study finds that toothed whales can reduce their own soli sensitivity when they expect a loud sound. The work is presented at this week's Acoustics 2012 meeting.Whales and dolphins rely on their responsive hearing to interpret returning installation clicks. Previous research suggested that these marine mammals could dull their hearing before uttering outgoing echolocation clicks, which are very loud. Could they use the same coping hidden for external noises? To find out, easterners trained a false killer whale that a loud noise would always follow a brief warning signal. Then, they want obstructionist sensors to the outside of the whale's head and played the signal. The sensors measured refrains that indicated the whale did reduce its hearing sensitivity in expectation of a clamor. The researchers hope to test other species as well.Loud noises from ships can disturb whales. To accommodate marine life, perhaps vessels could emit signals before making a ruckus, warning whales to tune us out.</t>
+    <t>Have you ever wanted to turn down the volume at a deafening concert or noisy bar? Envy the whale: a new study finds that toothed whales can reduce their own auditory sensitivity when they expect a loud sound. The work is presented at this week's Acoustics 2012 meeting.Whales and dolphins rely on their responsive hearing to interpret returning echolocation clicks. Previous research suggested that these marine mammals could dull their hearing before uttering outgoing echolocation clicks, which are very loud. Could they use the same coping mechanism for external noises? To find out, researchers trained a false killer whale that a loud noise would always follow a brief warning signal. Then, they attached suction-cup sensors to the outside of the whale's head and played the signal. The sensors measured brainwaves that indicated the whale did reduce its hearing sensitivity in expectation of a clamor. The researchers hope to test other species as well.Loud noises from ships can disturb whales. To accommodate marine life, perhaps vessels could emit signals before making a ruckus, warning whales to tune us out.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;As your PTE Academic teacher, I understand that this 'Highlight Incorrect Words' section tests not just your listening comprehension, but also your ability to recognize specific vocabulary, scientific jargon, and grammatical fit within context. A small mishearing or a slight misunderstanding of specialized terminology can cause you to select the wrong word.&lt;/p&gt;
@@ -2977,7 +2977,7 @@
     <t>Ants are known for working together, operating as a unit for the good of the colony. But not so fast, say researchers from the Universities of Leeds and Copenhagen. It turns out that ants can scheme like a stage mom. Scientists say that some ants hide out to ensure that their offspring become child-bearing queens instead of barren workers. The accepted __apologists/hypothesis__ had been that random ants were fed certain foods that would allow them to develop into queens. But DNA tests on five __harmonies/colonies__ of leaf-cutting ants __greet/revealed__ that certain males have a better genetic chance of __rerouting/producing__ royal progeny. Scientists believe these rare males stay anonymous, and thus avoid any problems with other ants that might __darkies/otherwise__ lose their "one-for-all, all-for-one" attitude. In fact, the number of males carrying royal genes to those who aren't may have settled at a low ratio through evolution—which cobbled __objector/together__ the best way for the ant gene pool to expand, while at the same time keeping the lucky males hidden from their possibly jealous rivals.</t>
   </si>
   <si>
-    <t>Ants are known for working together, operating as a unit for the good of the colony. But not so fast, say researchers from the Universities of Leeds and Copenhagen. It turns out that ants can scheme like a stage mom. Scientists say that some ants hide out to ensure that their offspring become child-bearing queens instead of barren workers. The accepted apologists had been that random ants were fed certain foods that would allow them to develop into queens. But DNA tests on five harmonies of leaf-cutting ants greet that certain males have a better genetic chance of rerouting royal progeny. Scientists believe these rare males stay anonymous, and thus avoid any problems with other ants that might darkies lose their "one-for-all, all-for-one" attitude. In fact, the number of males carrying royal genes to those who aren't may have settled at a low ratio through evolution—which cobbled objector the best way for the ant gene pool to expand, while at the same time keeping the lucky males hidden from their possibly jealous rivals.</t>
+    <t>Ants are known for working together, operating as a unit for the good of the colony. But not so fast, say researchers from the Universities of Leeds and Copenhagen. It turns out that ants can scheme like a stage mom. Scientists say that some ants hide out to ensure that their offspring become child-bearing queens instead of barren workers. The accepted hypothesis had been that random ants were fed certain foods that would allow them to develop into queens. But DNA tests on five colonies of leaf-cutting ants revealed that certain males have a better genetic chance of producing royal progeny. Scientists believe these rare males stay anonymous, and thus avoid any problems with other ants that might otherwise lose their "one-for-all, all-for-one" attitude. In fact, the number of males carrying royal genes to those who aren't may have settled at a low ratio through evolution—which cobbled together the best way for the ant gene pool to expand, while at the same time keeping the lucky males hidden from their possibly jealous rivals.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;💡 PTE Listening Mastery: Incorrect Word Analysis&lt;/h3&gt;
@@ -3025,7 +3025,7 @@
     <t>Researchers at the University of California claim to discover that people who eat chocolate regularly tend to be lighter than those who __hardly/rarely__ eat it. The findings may seem __suspicious/surprising__ in that chocolate has a great many calories and, in general. the more calories people __contain/consume__ ,the more likely they are to put on weight. The recent studies __establish/emphasize__ that it is more the regularity with which people eat chocolate that is __important/significant__ rather than the amount they consume. Whether they eat a little or a lot seems to make no difference, whereas eating it __freely/frequently__ appears to reduce weight more than only having it occasionally.</t>
   </si>
   <si>
-    <t>Researchers at the University of California claim to discover that people who eat chocolate regularly tend to be lighter than those who hardly eat it. The findings may seem suspicious in that chocolate has a great many calories and, in general. the more calories people contain ,the more likely they are to put on weight. The recent studies establish that it is more the regularity with which people eat chocolate that is important rather than the amount they consume. Whether they eat a little or a lot seems to make no difference, whereas eating it freely appears to reduce weight more than only having it occasionally.</t>
+    <t>Researchers at the University of California claim to discover that people who eat chocolate regularly tend to be lighter than those who rarely eat it. The findings may seem surprising in that chocolate has a great many calories and, in general. the more calories people consume ,the more likely they are to put on weight. The recent studies emphasize that it is more the regularity with which people eat chocolate that is significant rather than the amount they consume. Whether they eat a little or a lot seems to make no difference, whereas eating it frequently appears to reduce weight more than only having it occasionally.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🔍 PTE Listening Skill Boost: Explaining Incorrect Word Selection&lt;/h3&gt;
@@ -3074,7 +3074,7 @@
     <t>English had barely established itself as a language in England when it began __spreading/moving__ to other countries to be used there as well. First it __passed/headed__ north to Scotland and then west to Wales. It then made its __path/way__ across the sea to Ireland. That was in the Middle Ages. Over the course of the following centuries it has put down roots all over the __earth/world__ , from the USA to South Africa, from India to New Zealand. Of course, in all these __places/countries__ it has developed in special ways to suit the new __concepts/contexts__ in which it found itself.</t>
   </si>
   <si>
-    <t>English had barely established itself as a language in England when it began spreading to other countries to be used there as well. First it passed north to Scotland and then west to Wales. It then made its path across the sea to Ireland. That was in the Middle Ages. Over the course of the following centuries it has put down roots all over the earth , from the USA to South Africa, from India to New Zealand. Of course, in all these places it has developed in special ways to suit the new concepts in which it found itself.</t>
+    <t>English had barely established itself as a language in England when it began moving to other countries to be used there as well. First it headed north to Scotland and then west to Wales. It then made its way across the sea to Ireland. That was in the Middle Ages. Over the course of the following centuries it has put down roots all over the world , from the USA to South Africa, from India to New Zealand. Of course, in all these countries it has developed in special ways to suit the new contexts in which it found itself.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;&lt;b&gt;💡 PTE Listening Mastery: Analyzing Highlighted Errors&lt;/b&gt;&lt;/h3&gt;
@@ -3124,7 +3124,7 @@
     <t>Conducting a video conference is now a popular __method/means__ of communication in the business world. This telecommunications technology allows two or more locations to communicate by simultaneous video and audio transmissions. It's designed to serve conferences or meetings in __many/multiple__ locations. The advantages are obvious: no more lengthy phone calls or __complicated/complex__ correspondence with business contacts, partners or offices __abroad/overseas__ . This relatively low cost, fast, effective communication method has made significant inroads in not just a business __environment/context__ , but also education, medicine and media.</t>
   </si>
   <si>
-    <t>Conducting a video conference is now a popular method of communication in the business world. This telecommunications technology allows two or more locations to communicate by simultaneous video and audio transmissions. It's designed to serve conferences or meetings in many locations. The advantages are obvious: no more lengthy phone calls or complicated correspondence with business contacts, partners or offices abroad . This relatively low cost, fast, effective communication method has made significant inroads in not just a business environment , but also education, medicine and media.</t>
+    <t>Conducting a video conference is now a popular means of communication in the business world. This telecommunications technology allows two or more locations to communicate by simultaneous video and audio transmissions. It's designed to serve conferences or meetings in multiple locations. The advantages are obvious: no more lengthy phone calls or complex correspondence with business contacts, partners or offices overseas . This relatively low cost, fast, effective communication method has made significant inroads in not just a business context , but also education, medicine and media.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;&lt;b&gt;🌟 Premium PTE Analysis: Listening Highlight Incorrect Words&lt;/b&gt;&lt;/h3&gt;
@@ -3168,7 +3168,7 @@
     <t>One of the most encouraging phenomena in recent years has been the __development/growth__ of lifelong learning in the education sector. Nowadays, students are embarking on courses at all ages. Higher education is no longer __viewed/seen__ as a place for the young. Mature students are appreciated and __respected/valued__ . Recent research has also indicated that older students are __dedicated/enthusiastic__ learners, able to contribute a number of skills and __talents/attributes__ gained from work, family and other life experiences.</t>
   </si>
   <si>
-    <t>One of the most encouraging phenomena in recent years has been the development of lifelong learning in the education sector. Nowadays, students are embarking on courses at all ages. Higher education is no longer viewed as a place for the young. Mature students are appreciated and respected . Recent research has also indicated that older students are dedicated learners, able to contribute a number of skills and talents gained from work, family and other life experiences.</t>
+    <t>One of the most encouraging phenomena in recent years has been the growth of lifelong learning in the education sector. Nowadays, students are embarking on courses at all ages. Higher education is no longer seen as a place for the young. Mature students are appreciated and valued . Recent research has also indicated that older students are enthusiastic learners, able to contribute a number of skills and attributes gained from work, family and other life experiences.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🎧 PTE Listening Mastery: Incorrect Words Analysis 🧠&lt;/h3&gt;
@@ -3212,7 +3212,7 @@
     <t>Social capital is a concept that was introduced by sociologists, many years ago. It's actually the networks and __reserves/resources__ that people use to deliver social outcomes. For instance, it might be holding a sporting event, running a community __fair/fete__ ,being part of a club. It is difficult to measure social capital and one way of looking at it is the __amount/extent__ that people volunteer in their local community. So you can consider the volunteering rate as an __index/indicator__ for how healthy a community is. You can also look at something called a well·being index - the way people think about their lives and how __accepting/trusting__ they are of others, their general perception of the value of their life.</t>
   </si>
   <si>
-    <t>Social capital is a concept that was introduced by sociologists, many years ago. It's actually the networks and reserves that people use to deliver social outcomes. For instance, it might be holding a sporting event, running a community fair ,being part of a club. It is difficult to measure social capital and one way of looking at it is the amount that people volunteer in their local community. So you can consider the volunteering rate as an index for how healthy a community is. You can also look at something called a well·being index - the way people think about their lives and how accepting they are of others, their general perception of the value of their life.</t>
+    <t>Social capital is a concept that was introduced by sociologists, many years ago. It's actually the networks and resources that people use to deliver social outcomes. For instance, it might be holding a sporting event, running a community fete ,being part of a club. It is difficult to measure social capital and one way of looking at it is the extent that people volunteer in their local community. So you can consider the volunteering rate as an indicator for how healthy a community is. You can also look at something called a well·being index - the way people think about their lives and how trusting they are of others, their general perception of the value of their life.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your PTE academic instructor, I will provide a detailed breakdown of the word differences in this Listening - Highlight Incorrect Words question. In this task, precision in vocabulary and understanding the subtle differences between similar-sounding words are crucial. Remember, even if two words seem related, the audio transcript will only use one of them.&lt;/p&gt;
@@ -3249,7 +3249,7 @@
     <t>Well, there are many factors that can cause one species to __diverge/divide__ into two. One of these is when populations get isolated from each other by something like a __lagoon/lake__ forming or forest being cleared. And there's another idea that as individuals adapt to their environment, this might have a knock·on __impact/effect__ on mate choice, a process called __sensitive/sensory__ drive speciation. Now this seems to occur in cichlid fish. They have shown that a female preference for either red or blue striped males only exists in __clean/clear__ water, where they are actually able to see.</t>
   </si>
   <si>
-    <t>Well, there are many factors that can cause one species to diverge into two. One of these is when populations get isolated from each other by something like a lagoon forming or forest being cleared. And there's another idea that as individuals adapt to their environment, this might have a knock·on impact on mate choice, a process called sensitive drive speciation. Now this seems to occur in cichlid fish. They have shown that a female preference for either red or blue striped males only exists in clean water, where they are actually able to see.</t>
+    <t>Well, there are many factors that can cause one species to divide into two. One of these is when populations get isolated from each other by something like a lake forming or forest being cleared. And there's another idea that as individuals adapt to their environment, this might have a knock·on effect on mate choice, a process called sensory drive speciation. Now this seems to occur in cichlid fish. They have shown that a female preference for either red or blue striped males only exists in clear water, where they are actually able to see.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;💡 Premium PTE Grammar &amp;amp; Vocabulary Focus: Highlighted Incorrect Words&lt;/h3&gt;
@@ -3299,7 +3299,7 @@
     <t>Many species of birds cover long __miles/distances__ during their seasonal migration to warmer climates. But how successful are they, and do birds that get lost on their route ever __survive/manage__ to find their way back? Much research has been __done/conducted__ into how birds navigate and the results show that age is a significant __reason/factor__ . Young birds usually just carry on, if they lose their migratory path, and thus fail to __achieve/reach__ their destination, whereas older, more experienced birds will generally be able to find their __first/original__ route and continue successfully on their journey.</t>
   </si>
   <si>
-    <t>Many species of birds cover long miles during their seasonal migration to warmer climates. But how successful are they, and do birds that get lost on their route ever survive to find their way back? Much research has been done into how birds navigate and the results show that age is a significant reason . Young birds usually just carry on, if they lose their migratory path, and thus fail to achieve their destination, whereas older, more experienced birds will generally be able to find their first route and continue successfully on their journey.</t>
+    <t>Many species of birds cover long distances during their seasonal migration to warmer climates. But how successful are they, and do birds that get lost on their route ever manage to find their way back? Much research has been conducted into how birds navigate and the results show that age is a significant factor . Young birds usually just carry on, if they lose their migratory path, and thus fail to reach their destination, whereas older, more experienced birds will generally be able to find their original route and continue successfully on their journey.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🏆 PTE Listening Strategy: Understanding Word Discrepancies 🏆&lt;/h3&gt;
@@ -3341,7 +3341,7 @@
     <t>It seems we now know more about outer space than we do about the Earth's core. This is because temperatures are so __great/high__ at the centre of the Earth that human beings have not been able to take a close look at it. However, new __techniques/methods__ of analysis may soon change all that. The seismic waves __formed/created__ by earthquakes and volcanic eruptions penetrate the Earth's layers at different speeds. It is now hoped that by studying these waves, scientists will be able to make new __findings/discoveries__ and solve some of the mysteries of the __inside/internal__ structure of the Earth.</t>
   </si>
   <si>
-    <t>It seems we now know more about outer space than we do about the Earth's core. This is because temperatures are so great at the centre of the Earth that human beings have not been able to take a close look at it. However, new techniques of analysis may soon change all that. The seismic waves formed by earthquakes and volcanic eruptions penetrate the Earth's layers at different speeds. It is now hoped that by studying these waves, scientists will be able to make new findings and solve some of the mysteries of the inside structure of the Earth.</t>
+    <t>It seems we now know more about outer space than we do about the Earth's core. This is because temperatures are so high at the centre of the Earth that human beings have not been able to take a close look at it. However, new methods of analysis may soon change all that. The seismic waves created by earthquakes and volcanic eruptions penetrate the Earth's layers at different speeds. It is now hoped that by studying these waves, scientists will be able to make new discoveries and solve some of the mysteries of the internal structure of the Earth.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This question tests your ability to recognize subtle differences between written text (the transcript) and the exact phrasing used by the speaker in the audio. Even when two words have similar meanings, the context often requires a specific synonym. Here is a detailed breakdown of each incorrect word and its correct replacement.&lt;/p&gt;
@@ -3384,7 +3384,7 @@
     <t>No that was, and that’s an important aspect, as you __referred/alluded__ to earlier we’ve previously done work which has proven that in some __circumstances/situations__ , even people whose blood pressure is not high, can benefit from blood pressure lowering __rehabilitation/therapy__ . So in this study the main reason that we included the patients was because of diabetes, we didn’t care what their blood pressure was, whether it was high or low. And our __intention/objective__ was to see whether or not lowering average or below average blood pressure in diabetics was beneficial and the __effect/result__ suggested that irrespective of whether your blood pressure was high or low, if you had diabetes you __profited/benefited__ .</t>
   </si>
   <si>
-    <t>No that was, and that’s an important aspect, as you referred to earlier we’ve previously done work which has proven that in some circumstances , even people whose blood pressure is not high, can benefit from blood pressure lowering rehabilitation . So in this study the main reason that we included the patients was because of diabetes, we didn’t care what their blood pressure was, whether it was high or low. And our intention was to see whether or not lowering average or below average blood pressure in diabetics was beneficial and the effect suggested that irrespective of whether your blood pressure was high or low, if you had diabetes you profited .</t>
+    <t>No that was, and that’s an important aspect, as you alluded to earlier we’ve previously done work which has proven that in some situations , even people whose blood pressure is not high, can benefit from blood pressure lowering therapy . So in this study the main reason that we included the patients was because of diabetes, we didn’t care what their blood pressure was, whether it was high or low. And our objective was to see whether or not lowering average or below average blood pressure in diabetics was beneficial and the result suggested that irrespective of whether your blood pressure was high or low, if you had diabetes you benefited .</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This question tests your ability to listen critically and differentiate between words that sound similar or are related in meaning, but are not the exact words spoken by the speaker. In the PTE format, you must pay close attention to subtle pronunciation differences and the specific context of the discussion.&lt;/p&gt;
@@ -3438,7 +3438,7 @@
     <t>Oh, it's very spooky. First of all, probability by itself is spooky. Give me … let me show you how probability enters the __sample/system__ . You walk past a store window and you see an image of yourself in the store window, you straighten the part, not so bad you know, for a man of my age. The guy in the store window who's fooling around with mannequins he sees you and you see yourself. What does that mean? A __beam/stream__ of photons from sunlight leaves your face, heads for the store window – let's consider one of them. It has a choice: it can go right through, so that the guy behind the window can see you, or it can be reflected from the store window. Some __actions/fractions__ of them are reflected, and some of them go through. What determines that? What determines the future of that photon? And __doubtless/countless__ such examples teach us that it’s random, that it's a __roll/throw__ of the dice, and that's where Einstein made his famous statement "God plays dice with the universe". That every instant of that single object, that quantum object we have probability, we do not have certainty.</t>
   </si>
   <si>
-    <t>Oh, it's very spooky. First of all, probability by itself is spooky. Give me … let me show you how probability enters the sample . You walk past a store window and you see an image of yourself in the store window, you straighten the part, not so bad you know, for a man of my age. The guy in the store window who's fooling around with mannequins he sees you and you see yourself. What does that mean? A beam of photons from sunlight leaves your face, heads for the store window – let's consider one of them. It has a choice: it can go right through, so that the guy behind the window can see you, or it can be reflected from the store window. Some actions of them are reflected, and some of them go through. What determines that? What determines the future of that photon? And doubtless such examples teach us that it’s random, that it's a roll of the dice, and that's where Einstein made his famous statement "God plays dice with the universe". That every instant of that single object, that quantum object we have probability, we do not have certainty.</t>
+    <t>Oh, it's very spooky. First of all, probability by itself is spooky. Give me … let me show you how probability enters the system . You walk past a store window and you see an image of yourself in the store window, you straighten the part, not so bad you know, for a man of my age. The guy in the store window who's fooling around with mannequins he sees you and you see yourself. What does that mean? A stream of photons from sunlight leaves your face, heads for the store window – let's consider one of them. It has a choice: it can go right through, so that the guy behind the window can see you, or it can be reflected from the store window. Some fractions of them are reflected, and some of them go through. What determines that? What determines the future of that photon? And countless such examples teach us that it’s random, that it's a throw of the dice, and that's where Einstein made his famous statement "God plays dice with the universe". That every instant of that single object, that quantum object we have probability, we do not have certainty.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This was a challenging passage that tests not only your listening skills but also your ability to distinguish between similar-sounding vocabulary items (minimal pairs) and understand contextual vocabulary usage. The key to success here is identifying subtle differences in meaning and grammar.&lt;/p&gt;
@@ -3485,7 +3485,7 @@
     <t>Well there… there… there’s a positive obligation on the bank to ensure that the people who are signing a loan guarantee, __understand/know__ what they’re doing. Loan guarantees are ... er ... kind of __rare/unique__ in that … in that someone is giving security or a guarantee and placing themselves at risk for someone else, and they receive nothing __substantial/material__ in return. So you’ve got to ask yourself why is this person doing this, do they know what they’re doing? They’re risking a lot, and not really getting anything back for it. So the imperative is that the bank must __establish/ensure__ that these people know what they’re doing, and that they fully understand the __repercussions/implications__ of what they’re doing, and they know that their __assets/properties__ may be sold if another person doesn’t meet their obligations.</t>
   </si>
   <si>
-    <t>Well there… there… there’s a positive obligation on the bank to ensure that the people who are signing a loan guarantee, understand what they’re doing. Loan guarantees are ... er ... kind of rare in that … in that someone is giving security or a guarantee and placing themselves at risk for someone else, and they receive nothing substantial in return. So you’ve got to ask yourself why is this person doing this, do they know what they’re doing? They’re risking a lot, and not really getting anything back for it. So the imperative is that the bank must establish that these people know what they’re doing, and that they fully understand the repercussions of what they’re doing, and they know that their assets may be sold if another person doesn’t meet their obligations.</t>
+    <t>Well there… there… there’s a positive obligation on the bank to ensure that the people who are signing a loan guarantee, know what they’re doing. Loan guarantees are ... er ... kind of unique in that … in that someone is giving security or a guarantee and placing themselves at risk for someone else, and they receive nothing material in return. So you’ve got to ask yourself why is this person doing this, do they know what they’re doing? They’re risking a lot, and not really getting anything back for it. So the imperative is that the bank must ensure that these people know what they’re doing, and that they fully understand the implications of what they’re doing, and they know that their properties may be sold if another person doesn’t meet their obligations.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;PTE Listening Deep Dive: Incorrect Word Analysis&lt;/h3&gt;
@@ -3532,7 +3532,7 @@
     <t>For some people, this __presentation/proposition__ may seem far fetched, but ending poverty is both __ethically/morally__ necessary and actually feasible. All of us must play a role in making it happen. All human beings want, and have a __way/right__ to live in dignity, to determine our own destinies, and to be respected by other, by other people. Despite the universality of __three/these__ rights, our capacities to fulfill them vary enormously, and no __demarcating/dividing__ line is more profound in influencing the quality of our lives than the gulf between poverty and prosperity.</t>
   </si>
   <si>
-    <t>For some people, this presentation may seem far fetched, but ending poverty is both ethically necessary and actually feasible. All of us must play a role in making it happen. All human beings want, and have a way to live in dignity, to determine our own destinies, and to be respected by other, by other people. Despite the universality of three rights, our capacities to fulfill them vary enormously, and no demarcating line is more profound in influencing the quality of our lives than the gulf between poverty and prosperity.</t>
+    <t>For some people, this proposition may seem far fetched, but ending poverty is both morally necessary and actually feasible. All of us must play a role in making it happen. All human beings want, and have a right to live in dignity, to determine our own destinies, and to be respected by other, by other people. Despite the universality of these rights, our capacities to fulfill them vary enormously, and no dividing line is more profound in influencing the quality of our lives than the gulf between poverty and prosperity.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! This is a common area of difficulty in the PTE Listening module because the errors often involve homophones, near-synonyms, or subtle grammatical shifts. Remember, the key to this question type is to listen intently to the speaker's exact phrasing, as the transcript provided might contain intentional distractors.&lt;/p&gt;
@@ -3598,7 +3598,7 @@
     <t>In the __digestibility/celebrity__ vaccine wars, I'm siding with actress Amanda Peet. And comedian Bill Maher, well, I like your show, but when it comes to vaccines you don't know a punchline from a clothesline. Maher recently tweeted to his Twitter followers "if u get a swine flu shot ur an idiot." On his HBO program Real Time last week, Maher went head-to-head with former Senator Dr. Bill Frist, who patiently __grenade/explained__ why vaccines were in fact good. But Maher wasn't buying it. He advocates a healthy lifestyle over vaccines. But polio and smallpox outmatched many robust immune systems. Actress Amanda Peet, meanwhile, has used her celebrity to encourage vaccinations, specifically in response to the alleged vaccine-autism connection, for which there's no scientific evidence, but which has some parents afraid of __plywood/childhood__ vaccinations. In a letter to a parenting magazine, Peet wrote: "It's __reversible/irresponsible__ to suggest that virtually the entire medical community, and the CDC, and the American Academy of Pediatrics are behind a massive cover-up about vaccine safety." See you in the line for the flu shot.</t>
   </si>
   <si>
-    <t>In the digestibility vaccine wars, I'm siding with actress Amanda Peet. And comedian Bill Maher, well, I like your show, but when it comes to vaccines you don't know a punchline from a clothesline. Maher recently tweeted to his Twitter followers "if u get a swine flu shot ur an idiot." On his HBO program Real Time last week, Maher went head-to-head with former Senator Dr. Bill Frist, who patiently grenade why vaccines were in fact good. But Maher wasn't buying it. He advocates a healthy lifestyle over vaccines. But polio and smallpox outmatched many robust immune systems. Actress Amanda Peet, meanwhile, has used her celebrity to encourage vaccinations, specifically in response to the alleged vaccine-autism connection, for which there's no scientific evidence, but which has some parents afraid of plywood vaccinations. In a letter to a parenting magazine, Peet wrote: "It's reversible to suggest that virtually the entire medical community, and the CDC, and the American Academy of Pediatrics are behind a massive cover-up about vaccine safety." See you in the line for the flu shot.</t>
+    <t>In the celebrity vaccine wars, I'm siding with actress Amanda Peet. And comedian Bill Maher, well, I like your show, but when it comes to vaccines you don't know a punchline from a clothesline. Maher recently tweeted to his Twitter followers "if u get a swine flu shot ur an idiot." On his HBO program Real Time last week, Maher went head-to-head with former Senator Dr. Bill Frist, who patiently explained why vaccines were in fact good. But Maher wasn't buying it. He advocates a healthy lifestyle over vaccines. But polio and smallpox outmatched many robust immune systems. Actress Amanda Peet, meanwhile, has used her celebrity to encourage vaccinations, specifically in response to the alleged vaccine-autism connection, for which there's no scientific evidence, but which has some parents afraid of childhood vaccinations. In a letter to a parenting magazine, Peet wrote: "It's irresponsible to suggest that virtually the entire medical community, and the CDC, and the American Academy of Pediatrics are behind a massive cover-up about vaccine safety." See you in the line for the flu shot.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;&lt;h3&gt;🏆 PTE Listening Mastery: Incorrect Words Analysis&lt;/h3&gt;&lt;/p&gt;
@@ -3673,7 +3673,7 @@
     <t>There's an old-timer in the neighborhood, and it's got a story to tell. A new study of a relatively nearby star shows that it's almost as __bold/old__ as the big bang itself. The star HD 140283 lies about 190 light-years away in the constellation Libra. Astronomers have long known that it's ancient, because it __contrasted/contains__ mostly hydrogen and helium - which were present at the dawn of the universe - and few of the heavy elements that were __forecasted/forged__ later in stellar furnaces. With the Hubble Space Telescope, researchers have now pinned down the distance to HD 140283, which allowed them to determine how bright the star is. Along with the chemical __celebrations/ceremonials__ of the star, the newly derived stellar properties allowed for a new age estimate. The study of HD 140283, in the Astrophysical Journal Letters found that the star is 14.46 billion years old. But the entire universe, as you may have noted heard, is only 13.77 billion years old. The two age estimates aren't actually in conflict, because there's always some uncertainty. The full age estimate is thus 14.46 billion years plus or minus 800 million years.</t>
   </si>
   <si>
-    <t>There's an old-timer in the neighborhood, and it's got a story to tell. A new study of a relatively nearby star shows that it's almost as bold as the big bang itself. The star HD 140283 lies about 190 light-years away in the constellation Libra. Astronomers have long known that it's ancient, because it contrasted mostly hydrogen and helium - which were present at the dawn of the universe - and few of the heavy elements that were forecasted later in stellar furnaces. With the Hubble Space Telescope, researchers have now pinned down the distance to HD 140283, which allowed them to determine how bright the star is. Along with the chemical celebrations of the star, the newly derived stellar properties allowed for a new age estimate. The study of HD 140283, in the Astrophysical Journal Letters found that the star is 14.46 billion years old. But the entire universe, as you may have noted heard, is only 13.77 billion years old. The two age estimates aren't actually in conflict, because there's always some uncertainty. The full age estimate is thus 14.46 billion years plus or minus 800 million years.</t>
+    <t>There's an old-timer in the neighborhood, and it's got a story to tell. A new study of a relatively nearby star shows that it's almost as old as the big bang itself. The star HD 140283 lies about 190 light-years away in the constellation Libra. Astronomers have long known that it's ancient, because it contains mostly hydrogen and helium - which were present at the dawn of the universe - and few of the heavy elements that were forged later in stellar furnaces. With the Hubble Space Telescope, researchers have now pinned down the distance to HD 140283, which allowed them to determine how bright the star is. Along with the chemical ceremonials of the star, the newly derived stellar properties allowed for a new age estimate. The study of HD 140283, in the Astrophysical Journal Letters found that the star is 14.46 billion years old. But the entire universe, as you may have noted heard, is only 13.77 billion years old. The two age estimates aren't actually in conflict, because there's always some uncertainty. The full age estimate is thus 14.46 billion years plus or minus 800 million years.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🌟 PTE Listening Mastery: Understanding 'Highlight Incorrect Words'&lt;/h3&gt;
@@ -3733,7 +3733,7 @@
     <t>"Babies come __send/prepared__ to learn any of the world's languages." Alison Bruderer, a cognitive scientist at the University of British Columbia. "Which means that no matter where you're growing up in the world, the brains are prepared to pick up the language they're listening to around them." And listen they do. But another key factor to discerning a language's particular sounds may be for babies to move their tongues as they listen. Bruderer and her colleagues tested that notion by sitting 24 sixth-month-olds in front of a video screen and displaying a checkerboard pattern, while they played one of two tracks: a single, repeated "D" sound in Hindi; or two slightly different, alternating "D" sounds. The idea here is that babies have a short attention span, so novel things hold their gaze. And indeed, the babies did stare at the screen longer while the alternating "D"s played than for the single "D"—indicating they could detect the novelty. Until, that is, the researchers blocked the babies' tongue movements by having them suck on a teething device. Then the effect disappeared, with the babies unable to differentiate ... from ... And when the babies used a __delicate/different__ teether that did not block tongue movement, they once again __rinsed/appeared__ to __haired/comprehend__ the difference between the Ds. The study is in the Proceedings of the National Academy of Sciences. So is it time to pull the pacifier? "At this point I don't think that these data suggest parents should be taking away teething toys or soothers. The majority of infants are chewing on something semi-regularly throughout the day, and probably not doing it all day and every day. And most of these infants do go on to develop speech normally." So not to worry. Bruderer says the __reversed/research__ might instead offer insight into how __criticism/children__ with oral motor impairments or cleft palate __deeps/perceive__ speech ... now that we know the tongue really does matter, when first learning it.</t>
   </si>
   <si>
-    <t>"Babies come send to learn any of the world's languages." Alison Bruderer, a cognitive scientist at the University of British Columbia. "Which means that no matter where you're growing up in the world, the brains are prepared to pick up the language they're listening to around them." And listen they do. But another key factor to discerning a language's particular sounds may be for babies to move their tongues as they listen. Bruderer and her colleagues tested that notion by sitting 24 sixth-month-olds in front of a video screen and displaying a checkerboard pattern, while they played one of two tracks: a single, repeated "D" sound in Hindi; or two slightly different, alternating "D" sounds. The idea here is that babies have a short attention span, so novel things hold their gaze. And indeed, the babies did stare at the screen longer while the alternating "D"s played than for the single "D"—indicating they could detect the novelty. Until, that is, the researchers blocked the babies' tongue movements by having them suck on a teething device. Then the effect disappeared, with the babies unable to differentiate ... from ... And when the babies used a delicate teether that did not block tongue movement, they once again rinsed to haired the difference between the Ds. The study is in the Proceedings of the National Academy of Sciences. So is it time to pull the pacifier? "At this point I don't think that these data suggest parents should be taking away teething toys or soothers. The majority of infants are chewing on something semi-regularly throughout the day, and probably not doing it all day and every day. And most of these infants do go on to develop speech normally." So not to worry. Bruderer says the reversed might instead offer insight into how criticism with oral motor impairments or cleft palate deeps speech ... now that we know the tongue really does matter, when first learning it.</t>
+    <t>"Babies come prepared to learn any of the world's languages." Alison Bruderer, a cognitive scientist at the University of British Columbia. "Which means that no matter where you're growing up in the world, the brains are prepared to pick up the language they're listening to around them." And listen they do. But another key factor to discerning a language's particular sounds may be for babies to move their tongues as they listen. Bruderer and her colleagues tested that notion by sitting 24 sixth-month-olds in front of a video screen and displaying a checkerboard pattern, while they played one of two tracks: a single, repeated "D" sound in Hindi; or two slightly different, alternating "D" sounds. The idea here is that babies have a short attention span, so novel things hold their gaze. And indeed, the babies did stare at the screen longer while the alternating "D"s played than for the single "D"—indicating they could detect the novelty. Until, that is, the researchers blocked the babies' tongue movements by having them suck on a teething device. Then the effect disappeared, with the babies unable to differentiate ... from ... And when the babies used a different teether that did not block tongue movement, they once again appeared to comprehend the difference between the Ds. The study is in the Proceedings of the National Academy of Sciences. So is it time to pull the pacifier? "At this point I don't think that these data suggest parents should be taking away teething toys or soothers. The majority of infants are chewing on something semi-regularly throughout the day, and probably not doing it all day and every day. And most of these infants do go on to develop speech normally." So not to worry. Bruderer says the research might instead offer insight into how children with oral motor impairments or cleft palate perceive speech ... now that we know the tongue really does matter, when first learning it.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a premium PTE Academic teacher, I can help you understand the nuances of this &lt;strong&gt;Listening Highlight Incorrect Words&lt;/strong&gt; question type. These questions test your ability to capture precise details and differentiate between written transcripts and actual spoken audio. Don't worry if it feels tricky—it's all about excellent listening comprehension!&lt;/p&gt;
@@ -3797,7 +3797,7 @@
     <t>Pop-pop! It's so good to see you. How are you? Man's voice: Good, good. How are those knees holding up? And the old ticker? Man: Fine. Can't complain. What __abbreviations/medications__ are you taking now, Pop? Have you ever been diagnosed with high-blood pressure? Kidney disease? What about asthma? Any trouble breathing? Now, can you read the letters on the third line? Man: E, Uh, M. P? Taking grandpa's medical history might not seem like the best way to spread warm holiday wishes. But geneticists at the University of Alabama at __outrun/Birmingham__ note that family gatherings are a great time to learn more about your family's health issues. Lots of disorders—like diabetes, heart disease, and cancer—have strong roots in your genes. So it's good to know whether grandma has glaucoma or your mom had a brother who died young of a massive coronary. That way your docs can screen you for diseases to which you might be susceptible. Or maybe the info will inspire you to start taking better care of yourself. Either way, offer the relatives a cup of holiday cheer. And feel free to note how much they drank. For your records.</t>
   </si>
   <si>
-    <t>Pop-pop! It's so good to see you. How are you? Man's voice: Good, good. How are those knees holding up? And the old ticker? Man: Fine. Can't complain. What abbreviations are you taking now, Pop? Have you ever been diagnosed with high-blood pressure? Kidney disease? What about asthma? Any trouble breathing? Now, can you read the letters on the third line? Man: E, Uh, M. P? Taking grandpa's medical history might not seem like the best way to spread warm holiday wishes. But geneticists at the University of Alabama at outrun note that family gatherings are a great time to learn more about your family's health issues. Lots of disorders—like diabetes, heart disease, and cancer—have strong roots in your genes. So it's good to know whether grandma has glaucoma or your mom had a brother who died young of a massive coronary. That way your docs can screen you for diseases to which you might be susceptible. Or maybe the info will inspire you to start taking better care of yourself. Either way, offer the relatives a cup of holiday cheer. And feel free to note how much they drank. For your records.</t>
+    <t>Pop-pop! It's so good to see you. How are you? Man's voice: Good, good. How are those knees holding up? And the old ticker? Man: Fine. Can't complain. What medications are you taking now, Pop? Have you ever been diagnosed with high-blood pressure? Kidney disease? What about asthma? Any trouble breathing? Now, can you read the letters on the third line? Man: E, Uh, M. P? Taking grandpa's medical history might not seem like the best way to spread warm holiday wishes. But geneticists at the University of Alabama at Birmingham note that family gatherings are a great time to learn more about your family's health issues. Lots of disorders—like diabetes, heart disease, and cancer—have strong roots in your genes. So it's good to know whether grandma has glaucoma or your mom had a brother who died young of a massive coronary. That way your docs can screen you for diseases to which you might be susceptible. Or maybe the info will inspire you to start taking better care of yourself. Either way, offer the relatives a cup of holiday cheer. And feel free to note how much they drank. For your records.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This was a Listening task where you had to identify words in the written transcript that did not match the audio recording. Understanding these subtle mismatches is crucial for mastering the PTE Listening section.&lt;/p&gt;
@@ -3825,7 +3825,7 @@
     <t>To keep your car purring, you have to change the oil. Such maintenance __boogers/produces__ eight billion gallons of used motor oil annually. Some waste oil does get re-refined to produce oil for lubrication or heating. And some just gets dumped. So it would be more environmentally friendly and provide fresh fuel if we could convert the old motor oil to something really valuable: new gasoline. And that's what a __clad/research__ team thinks they've done. They __freshened/presented__ their work at the annual meeting of the __gentleman/American__ Chemical Society. Their approach involves pyrolysis, decomposing organic __decennial/material__ with heat in the absence of oxygen. Pyrolysis can break down waste oil into gases, liquids, a little bit of solids. The gases and liquids can be converted into gas or diesel. But __visceral/conventional__ pyrolysis methods don't do a great job with motor oil. The new technique mixes the oil with a material really good at absorbing microwave radiation. Tests showed that heating this mixture with microwaves was about 90 percent efficient at creating precursors to fuel—which beats tossing the oil down the drain.</t>
   </si>
   <si>
-    <t>To keep your car purring, you have to change the oil. Such maintenance boogers eight billion gallons of used motor oil annually. Some waste oil does get re-refined to produce oil for lubrication or heating. And some just gets dumped. So it would be more environmentally friendly and provide fresh fuel if we could convert the old motor oil to something really valuable: new gasoline. And that's what a clad team thinks they've done. They freshened their work at the annual meeting of the gentleman Chemical Society. Their approach involves pyrolysis, decomposing organic decennial with heat in the absence of oxygen. Pyrolysis can break down waste oil into gases, liquids, a little bit of solids. The gases and liquids can be converted into gas or diesel. But visceral pyrolysis methods don't do a great job with motor oil. The new technique mixes the oil with a material really good at absorbing microwave radiation. Tests showed that heating this mixture with microwaves was about 90 percent efficient at creating precursors to fuel—which beats tossing the oil down the drain.</t>
+    <t>To keep your car purring, you have to change the oil. Such maintenance produces eight billion gallons of used motor oil annually. Some waste oil does get re-refined to produce oil for lubrication or heating. And some just gets dumped. So it would be more environmentally friendly and provide fresh fuel if we could convert the old motor oil to something really valuable: new gasoline. And that's what a research team thinks they've done. They presented their work at the annual meeting of the American Chemical Society. Their approach involves pyrolysis, decomposing organic material with heat in the absence of oxygen. Pyrolysis can break down waste oil into gases, liquids, a little bit of solids. The gases and liquids can be converted into gas or diesel. But conventional pyrolysis methods don't do a great job with motor oil. The new technique mixes the oil with a material really good at absorbing microwave radiation. Tests showed that heating this mixture with microwaves was about 90 percent efficient at creating precursors to fuel—which beats tossing the oil down the drain.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your PTE Academic teacher, I'm here to help you master the tricky skill of highlighting incorrect words. This question tests not only your listening comprehension but also your vocabulary and understanding of context—which is key to achieving a high score!&lt;/p&gt;
@@ -3873,7 +3873,7 @@
     <t>Can your heart bleed for a robot? In two experiments, people reacted to videos where a human appeared to either torture or coddle one of three subjects: another human wearing green, a small green robot, or an __romanticist/inanimate__ green box. And viewers had a definite emotional __surpass/response__ to the treatment of the robot. The work will be presented at the International __legation/Communication__ Association's annual conference. Forty volunteers watched clips of the robot, which reacted to abuse with upset crying and choking noises and to affection with happy purring and babbling sounds. Viewers became physically agitated __converting/watching__ the abusive video, and afterwards they reported a negative emotional response. In the second experiment 14 people watched the videos while undergoing a functional MRI brain scan. The scans revealed similar responses when either the robot or the human received affection. But the human's apparent abuse caused more concern than the robot's. Understanding our emotional response to robots may help inform the __impediment/development__ of robotic assistants. In the meantime, be nice to your Roomba.</t>
   </si>
   <si>
-    <t>Can your heart bleed for a robot? In two experiments, people reacted to videos where a human appeared to either torture or coddle one of three subjects: another human wearing green, a small green robot, or an romanticist green box. And viewers had a definite emotional surpass to the treatment of the robot. The work will be presented at the International legation Association's annual conference. Forty volunteers watched clips of the robot, which reacted to abuse with upset crying and choking noises and to affection with happy purring and babbling sounds. Viewers became physically agitated converting the abusive video, and afterwards they reported a negative emotional response. In the second experiment 14 people watched the videos while undergoing a functional MRI brain scan. The scans revealed similar responses when either the robot or the human received affection. But the human's apparent abuse caused more concern than the robot's. Understanding our emotional response to robots may help inform the impediment of robotic assistants. In the meantime, be nice to your Roomba.</t>
+    <t>Can your heart bleed for a robot? In two experiments, people reacted to videos where a human appeared to either torture or coddle one of three subjects: another human wearing green, a small green robot, or an inanimate green box. And viewers had a definite emotional response to the treatment of the robot. The work will be presented at the International Communication Association's annual conference. Forty volunteers watched clips of the robot, which reacted to abuse with upset crying and choking noises and to affection with happy purring and babbling sounds. Viewers became physically agitated watching the abusive video, and afterwards they reported a negative emotional response. In the second experiment 14 people watched the videos while undergoing a functional MRI brain scan. The scans revealed similar responses when either the robot or the human received affection. But the human's apparent abuse caused more concern than the robot's. Understanding our emotional response to robots may help inform the development of robotic assistants. In the meantime, be nice to your Roomba.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Understanding the differences between similar-sounding words (homophones or near-homophones) is crucial for success in the Listening section. In the "Highlight Incorrect Words" question type, you must rely not just on pronunciation, but on &lt;em&gt;context&lt;/em&gt; and &lt;strong&gt;vocabulary usage&lt;/strong&gt;.&lt;/p&gt;
@@ -3920,7 +3920,7 @@
     <t>City dwellers across the U.S. might agree on one common enemy: bed bugs. But hey, not to worry, right? "Bed bugs are not known to spread diseases, but bites can be very itchy and irritating." Or so says the New York City Department of Health. But that assertion may not be true. Because a new study suggests bed bugs could be capable of spreading infection… specifically, by passing on the parasite that causes Chagas disease. Chagas can cause anything from mild headaches to eventual heart failure. The condition is usually spread by what's called the kissing bug—a relative of bedbugs, which also feeds on blood. But it doesn't pass the parasite through its saliva, as happens with malaria, for example. "You get it when the bug bites you and then __behaves/defecates__ on you. The parasite is in the feces of the bug." Michael Levy, a disease ecologist at the __banditry/University__ of Pennsylvania. Levy says scratching the bite then works the parasite into the skin, __unbending/infecting__ the victim. Levy and his colleagues wanted to see if the same thing could happen with bed bugs. So they let em loose on mice that carried the Tripanosoma cruzi parasite. The bugs caught it—and were then able to __bed/transmit__ the parasite back to mice. With one caveat—some mice actually hunted and ate the bugs—a sure route for infection. "People don't eat bed bugs, so we're not really at risk of being infected through the oral route by bed bugs." That said, one mouse actually did catch the disease not by snacking, but through a bedbug bite—more analogous to the way a human might. The study is in the American Journal of Tropical Medicine and Hygiene. Any advice for the bed bug-phobic? "Don't panic. It's important to remember that bed bugs may be able to carry the disease, but they don't cause it." Meaning, you'd need to live with someone with Chagas disease, who can pass the parasite to a bed bug, and then actually catch it from that bug. Still, Levy says, bugs pave the way for pathogens to spread. "It's very dangerous to let bugs that feed on human blood get out of control, like unfortunately has __spattered/happened__ in the United States and across the world with bed bugs." Maybe it's time to treat bed bugs like a public health issue, Levy says, rather than just a pest.</t>
   </si>
   <si>
-    <t>City dwellers across the U.S. might agree on one common enemy: bed bugs. But hey, not to worry, right? "Bed bugs are not known to spread diseases, but bites can be very itchy and irritating." Or so says the New York City Department of Health. But that assertion may not be true. Because a new study suggests bed bugs could be capable of spreading infection… specifically, by passing on the parasite that causes Chagas disease. Chagas can cause anything from mild headaches to eventual heart failure. The condition is usually spread by what's called the kissing bug—a relative of bedbugs, which also feeds on blood. But it doesn't pass the parasite through its saliva, as happens with malaria, for example. "You get it when the bug bites you and then behaves on you. The parasite is in the feces of the bug." Michael Levy, a disease ecologist at the banditry of Pennsylvania. Levy says scratching the bite then works the parasite into the skin, unbending the victim. Levy and his colleagues wanted to see if the same thing could happen with bed bugs. So they let em loose on mice that carried the Tripanosoma cruzi parasite. The bugs caught it—and were then able to bed the parasite back to mice. With one caveat—some mice actually hunted and ate the bugs—a sure route for infection. "People don't eat bed bugs, so we're not really at risk of being infected through the oral route by bed bugs." That said, one mouse actually did catch the disease not by snacking, but through a bedbug bite—more analogous to the way a human might. The study is in the American Journal of Tropical Medicine and Hygiene. Any advice for the bed bug-phobic? "Don't panic. It's important to remember that bed bugs may be able to carry the disease, but they don't cause it." Meaning, you'd need to live with someone with Chagas disease, who can pass the parasite to a bed bug, and then actually catch it from that bug. Still, Levy says, bugs pave the way for pathogens to spread. "It's very dangerous to let bugs that feed on human blood get out of control, like unfortunately has spattered in the United States and across the world with bed bugs." Maybe it's time to treat bed bugs like a public health issue, Levy says, rather than just a pest.</t>
+    <t>City dwellers across the U.S. might agree on one common enemy: bed bugs. But hey, not to worry, right? "Bed bugs are not known to spread diseases, but bites can be very itchy and irritating." Or so says the New York City Department of Health. But that assertion may not be true. Because a new study suggests bed bugs could be capable of spreading infection… specifically, by passing on the parasite that causes Chagas disease. Chagas can cause anything from mild headaches to eventual heart failure. The condition is usually spread by what's called the kissing bug—a relative of bedbugs, which also feeds on blood. But it doesn't pass the parasite through its saliva, as happens with malaria, for example. "You get it when the bug bites you and then defecates on you. The parasite is in the feces of the bug." Michael Levy, a disease ecologist at the University of Pennsylvania. Levy says scratching the bite then works the parasite into the skin, infecting the victim. Levy and his colleagues wanted to see if the same thing could happen with bed bugs. So they let em loose on mice that carried the Tripanosoma cruzi parasite. The bugs caught it—and were then able to transmit the parasite back to mice. With one caveat—some mice actually hunted and ate the bugs—a sure route for infection. "People don't eat bed bugs, so we're not really at risk of being infected through the oral route by bed bugs." That said, one mouse actually did catch the disease not by snacking, but through a bedbug bite—more analogous to the way a human might. The study is in the American Journal of Tropical Medicine and Hygiene. Any advice for the bed bug-phobic? "Don't panic. It's important to remember that bed bugs may be able to carry the disease, but they don't cause it." Meaning, you'd need to live with someone with Chagas disease, who can pass the parasite to a bed bug, and then actually catch it from that bug. Still, Levy says, bugs pave the way for pathogens to spread. "It's very dangerous to let bugs that feed on human blood get out of control, like unfortunately has happened in the United States and across the world with bed bugs." Maybe it's time to treat bed bugs like a public health issue, Levy says, rather than just a pest.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This is a challenging question type that tests your ability to recognize subtle phonetic differences and semantic shifts between written text and natural speech. Here is a detailed breakdown of each incorrect word and its correct equivalent:&lt;/p&gt;
@@ -3952,7 +3952,7 @@
     <t>Not taking the elevator is a good way to sneak in a little extra __survive/exercise__ every day. And if you do get some of your exercise __embroiling/avoiding__ elevators, here's a burning question: do you burn more __butteries/calories__ climbing stairs one at a time or bounding up them two at a time? To find out, researchers had subjects climb stairs reaching 46 feet high. Based on the subjects' heart rate measurements, the researchers __dictated/estimated__ calories burned. They found that __shifts/volunteers__ who took the stairs two at a time had a higher rate of energy expenditure over the 86 steps they climbed—but those who climbed one at a time burned more energy in total over the entire staircase. The study is in the journal PLoS One. It makes sense. Although the bounders had a more intense workout, the one-steppers take longer to get to the top. So even though they're burning fewer calories per minute than the bounders do, they work out enough longer to burn more total calories. And one step or two, there's never a wait for the stairs.</t>
   </si>
   <si>
-    <t>Not taking the elevator is a good way to sneak in a little extra survive every day. And if you do get some of your exercise embroiling elevators, here's a burning question: do you burn more butteries climbing stairs one at a time or bounding up them two at a time? To find out, researchers had subjects climb stairs reaching 46 feet high. Based on the subjects' heart rate measurements, the researchers dictated calories burned. They found that shifts who took the stairs two at a time had a higher rate of energy expenditure over the 86 steps they climbed—but those who climbed one at a time burned more energy in total over the entire staircase. The study is in the journal PLoS One. It makes sense. Although the bounders had a more intense workout, the one-steppers take longer to get to the top. So even though they're burning fewer calories per minute than the bounders do, they work out enough longer to burn more total calories. And one step or two, there's never a wait for the stairs.</t>
+    <t>Not taking the elevator is a good way to sneak in a little extra exercise every day. And if you do get some of your exercise avoiding elevators, here's a burning question: do you burn more calories climbing stairs one at a time or bounding up them two at a time? To find out, researchers had subjects climb stairs reaching 46 feet high. Based on the subjects' heart rate measurements, the researchers estimated calories burned. They found that volunteers who took the stairs two at a time had a higher rate of energy expenditure over the 86 steps they climbed—but those who climbed one at a time burned more energy in total over the entire staircase. The study is in the journal PLoS One. It makes sense. Although the bounders had a more intense workout, the one-steppers take longer to get to the top. So even though they're burning fewer calories per minute than the bounders do, they work out enough longer to burn more total calories. And one step or two, there's never a wait for the stairs.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a PTE Academic expert, I can help you understand why certain words in the transcript were incorrect. This question tests your ability to recognize subtle differences in sound, spelling, and context between what is written and what is actually spoken.&lt;/p&gt;
@@ -3997,7 +3997,7 @@
     <t>Here's another reason to stop global warming: to keep the Burmese pythons in Florida. Burmese pythons have been turning up in south Florida in recent years. Perhaps you've seen the famous photo of a python ripped apart by its efforts to ingest a large alligator. Apparently people with pythons as pets have been getting rid of the snakes when they get too big by dumping them in the Everglades. And in 2003, biologists confirmed the presence of a breeding population of the slithering serpents in Everglades National Park. Which skeeves me out, because I spend a lot of time there. I'm not afraid of timid alligators, but hungry Burmese pythons give me the willies. Anyway, the US __tautological/Geological__ Survey recently did an analysis of __betel/potential__ temperatures around the country by the end of this century. And then analyzed where Burmese pythons would be comfortable, based on their home territory, from __dem/Pakistan__ to Indonesia. The result: pythons could colonize a third of the US. Did I mention that they can be over 20 feet long and 250 pounds? Might be the best motivation to do __bulging/something__ about climate change.</t>
   </si>
   <si>
-    <t>Here's another reason to stop global warming: to keep the Burmese pythons in Florida. Burmese pythons have been turning up in south Florida in recent years. Perhaps you've seen the famous photo of a python ripped apart by its efforts to ingest a large alligator. Apparently people with pythons as pets have been getting rid of the snakes when they get too big by dumping them in the Everglades. And in 2003, biologists confirmed the presence of a breeding population of the slithering serpents in Everglades National Park. Which skeeves me out, because I spend a lot of time there. I'm not afraid of timid alligators, but hungry Burmese pythons give me the willies. Anyway, the US tautological Survey recently did an analysis of betel temperatures around the country by the end of this century. And then analyzed where Burmese pythons would be comfortable, based on their home territory, from dem to Indonesia. The result: pythons could colonize a third of the US. Did I mention that they can be over 20 feet long and 250 pounds? Might be the best motivation to do bulging about climate change.</t>
+    <t>Here's another reason to stop global warming: to keep the Burmese pythons in Florida. Burmese pythons have been turning up in south Florida in recent years. Perhaps you've seen the famous photo of a python ripped apart by its efforts to ingest a large alligator. Apparently people with pythons as pets have been getting rid of the snakes when they get too big by dumping them in the Everglades. And in 2003, biologists confirmed the presence of a breeding population of the slithering serpents in Everglades National Park. Which skeeves me out, because I spend a lot of time there. I'm not afraid of timid alligators, but hungry Burmese pythons give me the willies. Anyway, the US Geological Survey recently did an analysis of potential temperatures around the country by the end of this century. And then analyzed where Burmese pythons would be comfortable, based on their home territory, from Pakistan to Indonesia. The result: pythons could colonize a third of the US. Did I mention that they can be over 20 feet long and 250 pounds? Might be the best motivation to do something about climate change.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🔍 Detailed Analysis: Understanding the Shifts&lt;/h3&gt;
@@ -4035,7 +4035,7 @@
     <t>The food and beverage industries spend more than ten billion dollars a year in the US to market their __cations/products__ to children. And it's money well spent for them—by age 2 __engine/children__ may already harbor preferences for certain brands. And kids under 6 can often associate brands and with specific products. Such as McDonald's. Here's how __pronounceable/powerful__ the McDonald's brand is, according to a study just published in the August issue of the journal Archives of Pediatric and Adolescent Medicine: __ferule/preschool__ kids were given the exact same food in either unmarked packages or in McDonald's packaging. But the kids, all between 3 and 5 years old, said they liked the taste better when the food looked like it was from McDonald's. One of the foods tested was carrots. What's up is that the kids said they liked quote McDonald's carrots endquote better than just plain carrots by more than 2 to 1. And the more tv sets in a kid's home, the more likely he or she was to prefer the food in McDonald's bags.</t>
   </si>
   <si>
-    <t>The food and beverage industries spend more than ten billion dollars a year in the US to market their cations to children. And it's money well spent for them—by age 2 engine may already harbor preferences for certain brands. And kids under 6 can often associate brands and with specific products. Such as McDonald's. Here's how pronounceable the McDonald's brand is, according to a study just published in the August issue of the journal Archives of Pediatric and Adolescent Medicine: ferule kids were given the exact same food in either unmarked packages or in McDonald's packaging. But the kids, all between 3 and 5 years old, said they liked the taste better when the food looked like it was from McDonald's. One of the foods tested was carrots. What's up is that the kids said they liked quote McDonald's carrots endquote better than just plain carrots by more than 2 to 1. And the more tv sets in a kid's home, the more likely he or she was to prefer the food in McDonald's bags.</t>
+    <t>The food and beverage industries spend more than ten billion dollars a year in the US to market their products to children. And it's money well spent for them—by age 2 children may already harbor preferences for certain brands. And kids under 6 can often associate brands and with specific products. Such as McDonald's. Here's how powerful the McDonald's brand is, according to a study just published in the August issue of the journal Archives of Pediatric and Adolescent Medicine: preschool kids were given the exact same food in either unmarked packages or in McDonald's packaging. But the kids, all between 3 and 5 years old, said they liked the taste better when the food looked like it was from McDonald's. One of the foods tested was carrots. What's up is that the kids said they liked quote McDonald's carrots endquote better than just plain carrots by more than 2 to 1. And the more tv sets in a kid's home, the more likely he or she was to prefer the food in McDonald's bags.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🏆 PTE Listening Mastery: Incorrect Words Analysis&lt;/h3&gt;
@@ -4070,7 +4070,7 @@
     <t>Guys, here's another reason to eat your veggies: they might be good for your sperm. Some studies show that male fertility and what's called seminal quality have __immunized/declined__ over the last few decades. So __steelworkers/researchers__ from two fertility clinics in Spain looked at the reproductive power of fruits and vegetables. The scientists have spent the past four years analyzing diet and possible exposure to workplace contaminants in men with fertility problems. One effort examined the effects that antioxidants might have on sperm. The researchers hypothesized that antioxidants could lower the oxidative stress that can harm sperm. More antioxidants could theoretically improve both sperm __plantation/concentration__ and motility. The study enrolled 61 men from couples with fertility problems. Thirty of the men were shown to have sperm problems. The other 31 acted as the control. Interviews revealed that the males with good semen quality ate significantly more fruits and vegetables—their diets were higher in vitamins and antioxidants in general. The study appears in the journal Fertility and Sterility. The researchers say this finding __cares/suggests__ that healthy diets lead to healthy sperm. So remember, guys, an apple a day keeps your swimmers in play.</t>
   </si>
   <si>
-    <t>Guys, here's another reason to eat your veggies: they might be good for your sperm. Some studies show that male fertility and what's called seminal quality have immunized over the last few decades. So steelworkers from two fertility clinics in Spain looked at the reproductive power of fruits and vegetables. The scientists have spent the past four years analyzing diet and possible exposure to workplace contaminants in men with fertility problems. One effort examined the effects that antioxidants might have on sperm. The researchers hypothesized that antioxidants could lower the oxidative stress that can harm sperm. More antioxidants could theoretically improve both sperm plantation and motility. The study enrolled 61 men from couples with fertility problems. Thirty of the men were shown to have sperm problems. The other 31 acted as the control. Interviews revealed that the males with good semen quality ate significantly more fruits and vegetables—their diets were higher in vitamins and antioxidants in general. The study appears in the journal Fertility and Sterility. The researchers say this finding cares that healthy diets lead to healthy sperm. So remember, guys, an apple a day keeps your swimmers in play.</t>
+    <t>Guys, here's another reason to eat your veggies: they might be good for your sperm. Some studies show that male fertility and what's called seminal quality have declined over the last few decades. So researchers from two fertility clinics in Spain looked at the reproductive power of fruits and vegetables. The scientists have spent the past four years analyzing diet and possible exposure to workplace contaminants in men with fertility problems. One effort examined the effects that antioxidants might have on sperm. The researchers hypothesized that antioxidants could lower the oxidative stress that can harm sperm. More antioxidants could theoretically improve both sperm concentration and motility. The study enrolled 61 men from couples with fertility problems. Thirty of the men were shown to have sperm problems. The other 31 acted as the control. Interviews revealed that the males with good semen quality ate significantly more fruits and vegetables—their diets were higher in vitamins and antioxidants in general. The study appears in the journal Fertility and Sterility. The researchers say this finding suggests that healthy diets lead to healthy sperm. So remember, guys, an apple a day keeps your swimmers in play.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;💡 PTE Listening Strategy: Highlight Incorrect Words&lt;/h3&gt;
@@ -4120,7 +4120,7 @@
     <t>Wheat helped create __transformation/civilization__ in the Middle East. It's a staple crop for 30 percent of the world's population. And now, with the publication of four articles in the journal Science, we're close to a __unfeigned/detailed__ understanding of the bread wheat genome. Wheat is tough to sequence. It's gone through multiple hybridizations, making its genome five times larger than a human one. Plus there are many redundancies: more than 80 percent of the genome is made of repeated DNA sequences. So the typical whole-genome shotgun approach—breaking genomes into segments and then reassembling them—doesn't work for wheat. Instead, an international consortium devised another strategy, involving physically mapping individual __foams/chromosomes__ and chromosome arms. One paper details a draft of the entire genome of bread wheat. Another identifies all the genes on the largest of the plant's 21 chromosomes. Some 75,000 genes have been mapped. The methods in the second paper will help scientists map the remaining chromosomes. They say it should take another three years. Knowing exactly which genes are responsible for talents such as tolerating drought or __accoutring/improving__ yields should allow researchers to mine the genome and to quickly produce new and better wheat varieties to bring us our daily bread.</t>
   </si>
   <si>
-    <t>Wheat helped create transformation in the Middle East. It's a staple crop for 30 percent of the world's population. And now, with the publication of four articles in the journal Science, we're close to a unfeigned understanding of the bread wheat genome. Wheat is tough to sequence. It's gone through multiple hybridizations, making its genome five times larger than a human one. Plus there are many redundancies: more than 80 percent of the genome is made of repeated DNA sequences. So the typical whole-genome shotgun approach—breaking genomes into segments and then reassembling them—doesn't work for wheat. Instead, an international consortium devised another strategy, involving physically mapping individual foams and chromosome arms. One paper details a draft of the entire genome of bread wheat. Another identifies all the genes on the largest of the plant's 21 chromosomes. Some 75,000 genes have been mapped. The methods in the second paper will help scientists map the remaining chromosomes. They say it should take another three years. Knowing exactly which genes are responsible for talents such as tolerating drought or accoutring yields should allow researchers to mine the genome and to quickly produce new and better wheat varieties to bring us our daily bread.</t>
+    <t>Wheat helped create civilization in the Middle East. It's a staple crop for 30 percent of the world's population. And now, with the publication of four articles in the journal Science, we're close to a detailed understanding of the bread wheat genome. Wheat is tough to sequence. It's gone through multiple hybridizations, making its genome five times larger than a human one. Plus there are many redundancies: more than 80 percent of the genome is made of repeated DNA sequences. So the typical whole-genome shotgun approach—breaking genomes into segments and then reassembling them—doesn't work for wheat. Instead, an international consortium devised another strategy, involving physically mapping individual chromosomes and chromosome arms. One paper details a draft of the entire genome of bread wheat. Another identifies all the genes on the largest of the plant's 21 chromosomes. Some 75,000 genes have been mapped. The methods in the second paper will help scientists map the remaining chromosomes. They say it should take another three years. Knowing exactly which genes are responsible for talents such as tolerating drought or improving yields should allow researchers to mine the genome and to quickly produce new and better wheat varieties to bring us our daily bread.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a PTE Academic teacher, I will provide you with a comprehensive analysis of the incorrect words in this Listening task. Remember, this question tests your ability to capture subtle differences in pronunciation, vocabulary, and specialized terminology. Even if two words sound similar, only one will fit the &lt;strong&gt;context&lt;/strong&gt;.&lt;/p&gt;
@@ -4160,7 +4160,7 @@
     <t>Here's one way bats might get their next meal: by eavesdropping on flies having sex. Bats eat a lot of seemingly undetectable flies. To find out how the winged mammals find the insects, researchers set up a video camera inside a cowshed that was home to a bat colony and lots of bugs. The video showed that bats rely on their echolocation skills to detect flies at a specific time: when they're engaged in rather noisy sex. Flies are usually quiet in bat __vibratory/territory__ and sit on __muscled/cluttered__ ceilings in caves where __compound/background__ noise masks the echoes from their movement. But when flies are feeling frisky, males can't help but flutter their wings, __multiplexing/emitting__ a burst of click sounds that the bats pick up on. During more than one thousand sexual __slouchers/encounters__ caught in the act on video, five percent of the insects were caught in the act by bats. The __clap/research__ is published in the journal Current Biology. The study shows that ignorance can be safer than carnal knowledge when predators are on the prowl.</t>
   </si>
   <si>
-    <t>Here's one way bats might get their next meal: by eavesdropping on flies having sex. Bats eat a lot of seemingly undetectable flies. To find out how the winged mammals find the insects, researchers set up a video camera inside a cowshed that was home to a bat colony and lots of bugs. The video showed that bats rely on their echolocation skills to detect flies at a specific time: when they're engaged in rather noisy sex. Flies are usually quiet in bat vibratory and sit on muscled ceilings in caves where compound noise masks the echoes from their movement. But when flies are feeling frisky, males can't help but flutter their wings, multiplexing a burst of click sounds that the bats pick up on. During more than one thousand sexual slouchers caught in the act on video, five percent of the insects were caught in the act by bats. The clap is published in the journal Current Biology. The study shows that ignorance can be safer than carnal knowledge when predators are on the prowl.</t>
+    <t>Here's one way bats might get their next meal: by eavesdropping on flies having sex. Bats eat a lot of seemingly undetectable flies. To find out how the winged mammals find the insects, researchers set up a video camera inside a cowshed that was home to a bat colony and lots of bugs. The video showed that bats rely on their echolocation skills to detect flies at a specific time: when they're engaged in rather noisy sex. Flies are usually quiet in bat territory and sit on cluttered ceilings in caves where background noise masks the echoes from their movement. But when flies are feeling frisky, males can't help but flutter their wings, emitting a burst of click sounds that the bats pick up on. During more than one thousand sexual encounters caught in the act on video, five percent of the insects were caught in the act by bats. The research is published in the journal Current Biology. The study shows that ignorance can be safer than carnal knowledge when predators are on the prowl.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This question tests your ability to distinguish between closely related-sounding words, specific academic vocabulary, and correct contextual usage. Many of the incorrect words are either homophones, parts of speech that don't fit the sentence structure, or simply misspellings/substitutions of the intended vocabulary.&lt;/p&gt;
@@ -4205,7 +4205,7 @@
     <t>Most of us know we should rein in our energy use. But to be successful, it'd help if we knew the best way to do it. So scientists asked more than 500 people, "What's the most __perceptive/effective__ thing you can do to conserve energy?" The results were illuminating. More than half the __wilfulness/participants__ focused on conservation by curtailment: __refreshing/switching__ off the lights, changing thermostat __eclipses/settings__ and driving less. Only 12 percent went for efficiency: using compact fluorescent bulbs, insulating the house or driving a hybrid car. But scientists say that it's actually these moves that yield the bigger energy savings. The results appear in the Proceedings of the National Academy of Sciences. The study authors think that a big factor is that curtailment is easier to imagine doing—while efforts to improve __periodicity/efficiency__ would involve, for example, doing research about new appliances or cars, and spending money up front to buy them. But if people knew more about the actual energy requirements of their activities versus the savings available through efficiency, they might be spurred to act. To quote physicist and energy expert Arthur Rosenfeld: "Energy efficiency is like a Saudi Arabia under our cities."</t>
   </si>
   <si>
-    <t>Most of us know we should rein in our energy use. But to be successful, it'd help if we knew the best way to do it. So scientists asked more than 500 people, "What's the most perceptive thing you can do to conserve energy?" The results were illuminating. More than half the wilfulness focused on conservation by curtailment: refreshing off the lights, changing thermostat eclipses and driving less. Only 12 percent went for efficiency: using compact fluorescent bulbs, insulating the house or driving a hybrid car. But scientists say that it's actually these moves that yield the bigger energy savings. The results appear in the Proceedings of the National Academy of Sciences. The study authors think that a big factor is that curtailment is easier to imagine doing—while efforts to improve periodicity would involve, for example, doing research about new appliances or cars, and spending money up front to buy them. But if people knew more about the actual energy requirements of their activities versus the savings available through efficiency, they might be spurred to act. To quote physicist and energy expert Arthur Rosenfeld: "Energy efficiency is like a Saudi Arabia under our cities."</t>
+    <t>Most of us know we should rein in our energy use. But to be successful, it'd help if we knew the best way to do it. So scientists asked more than 500 people, "What's the most effective thing you can do to conserve energy?" The results were illuminating. More than half the participants focused on conservation by curtailment: switching off the lights, changing thermostat settings and driving less. Only 12 percent went for efficiency: using compact fluorescent bulbs, insulating the house or driving a hybrid car. But scientists say that it's actually these moves that yield the bigger energy savings. The results appear in the Proceedings of the National Academy of Sciences. The study authors think that a big factor is that curtailment is easier to imagine doing—while efforts to improve efficiency would involve, for example, doing research about new appliances or cars, and spending money up front to buy them. But if people knew more about the actual energy requirements of their activities versus the savings available through efficiency, they might be spurred to act. To quote physicist and energy expert Arthur Rosenfeld: "Energy efficiency is like a Saudi Arabia under our cities."</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;🎧 PTE Listening Skill Boost: Incorrect Word Identification&lt;/h3&gt;
@@ -4253,7 +4253,7 @@
     <t>The 2011 Nobel Prize in Physics goes to Saul Perlmutter at the Lawrence Berkeley __nontransferable/National__ Lab, Brian Schmidt at the Australian National Lab and Adam Reiss at Johns Hopkins. The Royal Swedish Academy's Olga Botner: "In a universe which is dominated by matter, one would expect gravity eventually should make the __draftsman/expansion__ slow down. Imagine then the utter __subcontinent/astonishment__ when two groups of __silences/scientists__ headed by this year's Nobel __nosiness/laureates__ in 1998 discovered that the expansion was not slowing down, it was actually accelerating. By __tilting/comparing__ the brightness of distant, far-away supernovae with the brightness of nearby supernovae, the scientists discovered that the far-away supernovae were about 25 percent too faint. They were too far away. The universe was accelerating. And so this discovery is __special/fundamental__ and a milestone for cosmology. And a challenge for generations of scientists to come."</t>
   </si>
   <si>
-    <t>The 2011 Nobel Prize in Physics goes to Saul Perlmutter at the Lawrence Berkeley nontransferable Lab, Brian Schmidt at the Australian National Lab and Adam Reiss at Johns Hopkins. The Royal Swedish Academy's Olga Botner: "In a universe which is dominated by matter, one would expect gravity eventually should make the draftsman slow down. Imagine then the utter subcontinent when two groups of silences headed by this year's Nobel nosiness in 1998 discovered that the expansion was not slowing down, it was actually accelerating. By tilting the brightness of distant, far-away supernovae with the brightness of nearby supernovae, the scientists discovered that the far-away supernovae were about 25 percent too faint. They were too far away. The universe was accelerating. And so this discovery is special and a milestone for cosmology. And a challenge for generations of scientists to come."</t>
+    <t>The 2011 Nobel Prize in Physics goes to Saul Perlmutter at the Lawrence Berkeley National Lab, Brian Schmidt at the Australian National Lab and Adam Reiss at Johns Hopkins. The Royal Swedish Academy's Olga Botner: "In a universe which is dominated by matter, one would expect gravity eventually should make the expansion slow down. Imagine then the utter astonishment when two groups of scientists headed by this year's Nobel laureates in 1998 discovered that the expansion was not slowing down, it was actually accelerating. By comparing the brightness of distant, far-away supernovae with the brightness of nearby supernovae, the scientists discovered that the far-away supernovae were about 25 percent too faint. They were too far away. The universe was accelerating. And so this discovery is fundamental and a milestone for cosmology. And a challenge for generations of scientists to come."</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This question tests your ability to accurately transcribe spoken academic English, focusing on contextual vocabulary and phonetic differences. You must listen closely to the nuances of the speaker’s words.&lt;/p&gt;
@@ -4302,7 +4302,7 @@
     <t>Once upon a time, our __junketeer/atmosphere__ was a little thin on oxygen. Like, there wasn't any. Then, about three billion years ago, a handful of __widener/bacteria__ figured out how to harvest the energy from __sulfide/sunlight__ to make themselves some food. In the process, they consumed carbon dioxide, and gave off oxygen. So the air filled with oxygen, and all was right with the world. If you've ever taken an intro biology course, you've no doubt heard the tale. Photosynthetic bacteria are the heroes who brought oxygen to our planet. But maybe there's more to the story than that. Because in the online issue of Nature Geoscience, researchers from __inhaler/Australia__ say: the bacteria didn't act alone. The __hypoglycaemics/scientists__ looked at __geodetic/atmospheric__ oxygen levels throughout Earth's history. And they found that the amount of oxygen in the air spiked each time smaller land masses collided to form a supercontinent, like Pangea. These massive pile-ups generated mountain chains, and as the mountains eroded, they released nutrients into the oceans, feeding the photosynthetic bacteria. So the young Earth and its inhabitants worked __dismember/together__ to produce a planet where you can really find inspiration.</t>
   </si>
   <si>
-    <t>Once upon a time, our junketeer was a little thin on oxygen. Like, there wasn't any. Then, about three billion years ago, a handful of widener figured out how to harvest the energy from sulfide to make themselves some food. In the process, they consumed carbon dioxide, and gave off oxygen. So the air filled with oxygen, and all was right with the world. If you've ever taken an intro biology course, you've no doubt heard the tale. Photosynthetic bacteria are the heroes who brought oxygen to our planet. But maybe there's more to the story than that. Because in the online issue of Nature Geoscience, researchers from inhaler say: the bacteria didn't act alone. The hypoglycaemics looked at geodetic oxygen levels throughout Earth's history. And they found that the amount of oxygen in the air spiked each time smaller land masses collided to form a supercontinent, like Pangea. These massive pile-ups generated mountain chains, and as the mountains eroded, they released nutrients into the oceans, feeding the photosynthetic bacteria. So the young Earth and its inhabitants worked dismember to produce a planet where you can really find inspiration.</t>
+    <t>Once upon a time, our atmosphere was a little thin on oxygen. Like, there wasn't any. Then, about three billion years ago, a handful of bacteria figured out how to harvest the energy from sunlight to make themselves some food. In the process, they consumed carbon dioxide, and gave off oxygen. So the air filled with oxygen, and all was right with the world. If you've ever taken an intro biology course, you've no doubt heard the tale. Photosynthetic bacteria are the heroes who brought oxygen to our planet. But maybe there's more to the story than that. Because in the online issue of Nature Geoscience, researchers from Australia say: the bacteria didn't act alone. The scientists looked at atmospheric oxygen levels throughout Earth's history. And they found that the amount of oxygen in the air spiked each time smaller land masses collided to form a supercontinent, like Pangea. These massive pile-ups generated mountain chains, and as the mountains eroded, they released nutrients into the oceans, feeding the photosynthetic bacteria. So the young Earth and its inhabitants worked together to produce a planet where you can really find inspiration.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your PTE Academic teacher, I can guide you through this specific challenge. The "Highlight Incorrect Words" question tests not only your listening comprehension but also your vocabulary, context awareness, and grammatical understanding. When you hear an incorrect word, it is almost always a semantic or contextual mismatch.&lt;/p&gt;
@@ -4375,7 +4375,7 @@
     <t>After its ongoing Mars missions, NASA will concentrate less on the red planet and more on the solar system's other planets and moons, including our own. That's what NASA administrator Mike Griffin told an __nastiness/audience__ of researchers last week at the 39th Lunar and Planetary Conference in Texas. The Mars Science Laboratory lands in 2010. Griffin said that NASA is now __charting/planning__ in earnest for an outer planets flagship mission to Europa, Titan or Ganymede. Europa and Ganymede are moons of Jupiter. Titan is a moon of Saturn. The reorientation of NASA's planetary exploration programs is in response to a recent __maximal/National__ __batch/Research__ Council report card. The NRC gave NASA an A for its Mars work but only a C for its overall research and __maximums/analysis__ program and a dismal D for outer planets efforts. Griffin also noted that NASA is now planning seven different small and medium class missions to the moon by 2014. And the Messenger spacecraft goes into orbit around Mercury in 2011.</t>
   </si>
   <si>
-    <t>After its ongoing Mars missions, NASA will concentrate less on the red planet and more on the solar system's other planets and moons, including our own. That's what NASA administrator Mike Griffin told an nastiness of researchers last week at the 39th Lunar and Planetary Conference in Texas. The Mars Science Laboratory lands in 2010. Griffin said that NASA is now charting in earnest for an outer planets flagship mission to Europa, Titan or Ganymede. Europa and Ganymede are moons of Jupiter. Titan is a moon of Saturn. The reorientation of NASA's planetary exploration programs is in response to a recent maximal batch Council report card. The NRC gave NASA an A for its Mars work but only a C for its overall research and maximums program and a dismal D for outer planets efforts. Griffin also noted that NASA is now planning seven different small and medium class missions to the moon by 2014. And the Messenger spacecraft goes into orbit around Mercury in 2011.</t>
+    <t>After its ongoing Mars missions, NASA will concentrate less on the red planet and more on the solar system's other planets and moons, including our own. That's what NASA administrator Mike Griffin told an audience of researchers last week at the 39th Lunar and Planetary Conference in Texas. The Mars Science Laboratory lands in 2010. Griffin said that NASA is now planning in earnest for an outer planets flagship mission to Europa, Titan or Ganymede. Europa and Ganymede are moons of Jupiter. Titan is a moon of Saturn. The reorientation of NASA's planetary exploration programs is in response to a recent National Research Council report card. The NRC gave NASA an A for its Mars work but only a C for its overall research and analysis program and a dismal D for outer planets efforts. Griffin also noted that NASA is now planning seven different small and medium class missions to the moon by 2014. And the Messenger spacecraft goes into orbit around Mercury in 2011.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;As a premium PTE Academic teacher, I understand how crucial it is to pinpoint these subtle phonetic and lexical differences. This question tests not just your listening comprehension, but also your ability to hear *precise* pronunciation and word usage. The core concept here is distinguishing between words that sound similar (minimal pairs) or words that are contextually required.&lt;/p&gt;
@@ -4432,7 +4432,7 @@
     <t>Alberta is launching a huge geothermal energy project to tap into green power sources. The initiative aims to __harvest/harness__ underground heat to supply electricity for thousands of homes across the province. New facilities will cut reliance on fossil fuels and create sustainable jobs. Local engineer Clara Wong says __recycling/reliable__ clean energy is crucial for Alberta's future. The project includes drilling test wells and building infrastructure over the next three years. Construction is set to begin this autumn, with full operations expected by 2028. Environmental groups __support/praise__ the move, noting it aligns with Canada's climate goals. The province hopes to __zoom/lead__ in renewable energy innovation.</t>
   </si>
   <si>
-    <t>Alberta is launching a huge geothermal energy project to tap into green power sources. The initiative aims to harvest underground heat to supply electricity for thousands of homes across the province. New facilities will cut reliance on fossil fuels and create sustainable jobs. Local engineer Clara Wong says recycling clean energy is crucial for Alberta's future. The project includes drilling test wells and building infrastructure over the next three years. Construction is set to begin this autumn, with full operations expected by 2028. Environmental groups support the move, noting it aligns with Canada's climate goals. The province hopes to zoom in renewable energy innovation.</t>
+    <t>Alberta is launching a huge geothermal energy project to tap into green power sources. The initiative aims to harness underground heat to supply electricity for thousands of homes across the province. New facilities will cut reliance on fossil fuels and create sustainable jobs. Local engineer Clara Wong says reliable clean energy is crucial for Alberta's future. The project includes drilling test wells and building infrastructure over the next three years. Construction is set to begin this autumn, with full operations expected by 2028. Environmental groups praise the move, noting it aligns with Canada's climate goals. The province hopes to lead in renewable energy innovation.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your PTE Academic teacher, I want to provide a detailed breakdown of this "Highlight Incorrect Words" question. This question tests your ability not only to recognize accurate pronunciation but also to understand the precise &lt;strong&gt;contextual meaning&lt;/strong&gt; and &lt;em&gt;grammatical function&lt;/em&gt; of words. It's not just about hearing a similar-sounding word; it's about hearing the *right* word.&lt;/p&gt;
@@ -4475,7 +4475,7 @@
     <t>What's the most universal utterance in languages across the globe? Huh? Correct! Huh? That's right. Huh? Exactly. Because a new study finds that everybody around the world does indeed say "huh?" The finding is the journal PLOS One. The __treatises/researchers__ were exploring linguistic tools people use to assure fluid communication. In this case, they were looking for an __cistern/interjection__ that signals that a listener missed something, and prompts the speaker to repeat or rephrase the __kissable/original__ statement. In other words, __conducting/something__ that works like the English word "huh?" So they eavesdropped on nearly 200 conversations in 10 __coalitionist/different__ tongues, from Italian to Icelandic. And they found that, in __unravelled/language__ after language, a word that sounds a lot like "huh?" gets the job done. For example. It's short and sweet so it's likely to stop the speaker before the listener gets too lost. And it sounds like a question , so it warrants a response. The sound appears not to be innate. Babies don't use it before they say mama. But most five-year-olds are masters of "huh?" No matter where they come from.</t>
   </si>
   <si>
-    <t>What's the most universal utterance in languages across the globe? Huh? Correct! Huh? That's right. Huh? Exactly. Because a new study finds that everybody around the world does indeed say "huh?" The finding is the journal PLOS One. The treatises were exploring linguistic tools people use to assure fluid communication. In this case, they were looking for an cistern that signals that a listener missed something, and prompts the speaker to repeat or rephrase the kissable statement. In other words, conducting that works like the English word "huh?" So they eavesdropped on nearly 200 conversations in 10 coalitionist tongues, from Italian to Icelandic. And they found that, in unravelled after language, a word that sounds a lot like "huh?" gets the job done. For example. It's short and sweet so it's likely to stop the speaker before the listener gets too lost. And it sounds like a question , so it warrants a response. The sound appears not to be innate. Babies don't use it before they say mama. But most five-year-olds are masters of "huh?" No matter where they come from.</t>
+    <t>What's the most universal utterance in languages across the globe? Huh? Correct! Huh? That's right. Huh? Exactly. Because a new study finds that everybody around the world does indeed say "huh?" The finding is the journal PLOS One. The researchers were exploring linguistic tools people use to assure fluid communication. In this case, they were looking for an interjection that signals that a listener missed something, and prompts the speaker to repeat or rephrase the original statement. In other words, something that works like the English word "huh?" So they eavesdropped on nearly 200 conversations in 10 different tongues, from Italian to Icelandic. And they found that, in language after language, a word that sounds a lot like "huh?" gets the job done. For example. It's short and sweet so it's likely to stop the speaker before the listener gets too lost. And it sounds like a question , so it warrants a response. The sound appears not to be innate. Babies don't use it before they say mama. But most five-year-olds are masters of "huh?" No matter where they come from.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;&lt;b&gt;🌟 PTE Listening Mastery: Incorrect Words Analysis&lt;/b&gt;&lt;/h3&gt;
@@ -4536,7 +4536,7 @@
     <t>When I got into a cage with a Komodo Dragon almost 10 years ago for a story, I had no idea that its skull was so special. Neither did scientists until now. But a report in the Journal of Anatomy reveals that the world's largest living lizard has a remarkable, space-frame skull. Space frame refers to a light, rigid structure with __amassing/interlocking__ struts that can handle big loads. The shape of the skull bones and the arrangement of bones of __disinterment/different__ __bits/strengths__ is the key. The researchers employed a technique called Finite Element Analysis, which is usually used to analyze trains or planes. But in this case it let them reverse engineer the Komodo to study the __astrological/mechanical__ forces that the skull is subject to. As opposed to, say, an alligator, the dragon has a pretty wimpy bite. So rather than clamp down on its victims, it yanks off chunks of meat, a move powered by incredibly strong neck muscles. And made __carnival/possible__ by that space-frame skull able to handle the huge forces involved. Our March 1999 article on Komodos is available at sciamdigital.com.</t>
   </si>
   <si>
-    <t>When I got into a cage with a Komodo Dragon almost 10 years ago for a story, I had no idea that its skull was so special. Neither did scientists until now. But a report in the Journal of Anatomy reveals that the world's largest living lizard has a remarkable, space-frame skull. Space frame refers to a light, rigid structure with amassing struts that can handle big loads. The shape of the skull bones and the arrangement of bones of disinterment bits is the key. The researchers employed a technique called Finite Element Analysis, which is usually used to analyze trains or planes. But in this case it let them reverse engineer the Komodo to study the astrological forces that the skull is subject to. As opposed to, say, an alligator, the dragon has a pretty wimpy bite. So rather than clamp down on its victims, it yanks off chunks of meat, a move powered by incredibly strong neck muscles. And made carnival by that space-frame skull able to handle the huge forces involved. Our March 1999 article on Komodos is available at sciamdigital.com.</t>
+    <t>When I got into a cage with a Komodo Dragon almost 10 years ago for a story, I had no idea that its skull was so special. Neither did scientists until now. But a report in the Journal of Anatomy reveals that the world's largest living lizard has a remarkable, space-frame skull. Space frame refers to a light, rigid structure with interlocking struts that can handle big loads. The shape of the skull bones and the arrangement of bones of different strengths is the key. The researchers employed a technique called Finite Element Analysis, which is usually used to analyze trains or planes. But in this case it let them reverse engineer the Komodo to study the mechanical forces that the skull is subject to. As opposed to, say, an alligator, the dragon has a pretty wimpy bite. So rather than clamp down on its victims, it yanks off chunks of meat, a move powered by incredibly strong neck muscles. And made possible by that space-frame skull able to handle the huge forces involved. Our March 1999 article on Komodos is available at sciamdigital.com.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;This question type tests your ability to accurately transcribe spoken English, even when the provided text contains intentional misspellings or incorrect word choices. You must listen carefully and identify which words in the written transcript do not match what the speaker actually said.&lt;/p&gt;
@@ -4578,7 +4578,7 @@
     <t>You've heard of synchronized swimming. But what about synchronized blinking? No, it's not a new Olympic sport for slackers. It's __diverting/something__ that seems to happen when we watch a video. Because none of us want to miss the good parts. If you stop to add it up, humans spend a lot of time not looking. We blink every couple seconds, which means we lose about six seconds out of every minute of viewing time. So 10 percent of the time we have no visual __hesitation/information__ coming in. Yet we rarely notice this interruption of service. That's because we tend to time our blinks so that we don't get left in the dark. Or so says a report in the Royal Society journal Biological Sciences. Fourteen people watched a couple episodes of Mr. Bean. And it turns out they all tended to blink at the same moments: just after Bean __insect/finished__ doing something stupid or when the camera showed a long shot with nothing much going on. Such synchronized __strapping/eye-shutting__ did not happen when the subjects watched a video of fish __tipping/swimming__ around a tank. So when we need to pay attention, we keep our eyes open. Until we see whether Mr. Bean gets through his holiday in one piece.</t>
   </si>
   <si>
-    <t>You've heard of synchronized swimming. But what about synchronized blinking? No, it's not a new Olympic sport for slackers. It's diverting that seems to happen when we watch a video. Because none of us want to miss the good parts. If you stop to add it up, humans spend a lot of time not looking. We blink every couple seconds, which means we lose about six seconds out of every minute of viewing time. So 10 percent of the time we have no visual hesitation coming in. Yet we rarely notice this interruption of service. That's because we tend to time our blinks so that we don't get left in the dark. Or so says a report in the Royal Society journal Biological Sciences. Fourteen people watched a couple episodes of Mr. Bean. And it turns out they all tended to blink at the same moments: just after Bean insect doing something stupid or when the camera showed a long shot with nothing much going on. Such synchronized strapping did not happen when the subjects watched a video of fish tipping around a tank. So when we need to pay attention, we keep our eyes open. Until we see whether Mr. Bean gets through his holiday in one piece.</t>
+    <t>You've heard of synchronized swimming. But what about synchronized blinking? No, it's not a new Olympic sport for slackers. It's something that seems to happen when we watch a video. Because none of us want to miss the good parts. If you stop to add it up, humans spend a lot of time not looking. We blink every couple seconds, which means we lose about six seconds out of every minute of viewing time. So 10 percent of the time we have no visual information coming in. Yet we rarely notice this interruption of service. That's because we tend to time our blinks so that we don't get left in the dark. Or so says a report in the Royal Society journal Biological Sciences. Fourteen people watched a couple episodes of Mr. Bean. And it turns out they all tended to blink at the same moments: just after Bean finished doing something stupid or when the camera showed a long shot with nothing much going on. Such synchronized eye-shutting did not happen when the subjects watched a video of fish swimming around a tank. So when we need to pay attention, we keep our eyes open. Until we see whether Mr. Bean gets through his holiday in one piece.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a premium PTE Academic teacher, I can provide you with a detailed analysis of the word discrepancies in this Listening section. This question tests your ability to distinguish subtle phonetic variations and understand the contextual meaning required by the narrative. &lt;/p&gt;
@@ -4619,7 +4619,7 @@
     <t>You can teach your dog to lie down. But you can't teach him to lie, or to know when you're lying. Because a new report shows that Spot can't spot deception. The study's in the journal Behavioural Processes. We've all known pooches who run and hide when their owners shout "let's go for a ride"—when what they really mean is "we have an appointment with the vet." But do the dogs really know that their people are being duplicitous? To find out, Mark Petter, a student in clinical psychology at __thoroughly/Dalhousie__ University in Canada, decided to fib to some Fidos. In his experiment, dogs were shown two covered containers. One held a treat. The other: nothing but disappointment. In half the trials, a helpful trainer stood behind and pointed to the __evaporator/container__ holding the treat. In the other half, a deceptive trainer pointed to the empty container. The results? The dogs __doped/approached__ the honest trainer a little more often than they did the deceiver. But not enough to __suit/conclude__ that the pups had figured out that one of the guys was pulling their leg. So dogs may be able to sniff out bombs. But they can't pick up the smell of mendacity.</t>
   </si>
   <si>
-    <t>You can teach your dog to lie down. But you can't teach him to lie, or to know when you're lying. Because a new report shows that Spot can't spot deception. The study's in the journal Behavioural Processes. We've all known pooches who run and hide when their owners shout "let's go for a ride"—when what they really mean is "we have an appointment with the vet." But do the dogs really know that their people are being duplicitous? To find out, Mark Petter, a student in clinical psychology at thoroughly University in Canada, decided to fib to some Fidos. In his experiment, dogs were shown two covered containers. One held a treat. The other: nothing but disappointment. In half the trials, a helpful trainer stood behind and pointed to the evaporator holding the treat. In the other half, a deceptive trainer pointed to the empty container. The results? The dogs doped the honest trainer a little more often than they did the deceiver. But not enough to suit that the pups had figured out that one of the guys was pulling their leg. So dogs may be able to sniff out bombs. But they can't pick up the smell of mendacity.</t>
+    <t>You can teach your dog to lie down. But you can't teach him to lie, or to know when you're lying. Because a new report shows that Spot can't spot deception. The study's in the journal Behavioural Processes. We've all known pooches who run and hide when their owners shout "let's go for a ride"—when what they really mean is "we have an appointment with the vet." But do the dogs really know that their people are being duplicitous? To find out, Mark Petter, a student in clinical psychology at Dalhousie University in Canada, decided to fib to some Fidos. In his experiment, dogs were shown two covered containers. One held a treat. The other: nothing but disappointment. In half the trials, a helpful trainer stood behind and pointed to the container holding the treat. In the other half, a deceptive trainer pointed to the empty container. The results? The dogs approached the honest trainer a little more often than they did the deceiver. But not enough to conclude that the pups had figured out that one of the guys was pulling their leg. So dogs may be able to sniff out bombs. But they can't pick up the smell of mendacity.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;h3&gt;Comprehensive Analysis of Incorrect Words&lt;/h3&gt;
@@ -4657,7 +4657,7 @@
     <t>Unless you're talking about killer bees, it's hard to imagine a situation in which "killers" and "bees" would be related. But it turns out that __hybridise/scientists__ are using the same mathematical model to __recite/describe__ the behavior of both bumblebees and human serial killers. The method, called geographic profiling, was developed by a detective who was trying to predict where serial killers might live based on where they commit their crimes. Believe it or not, murderers operate fairly close to home. But not too close. They __domain/maintain__ a kind of kill-free "buffer zone" around their actual digs. A similar pattern of activity seems to hold true for bumblebees—when they're __bookending/foraging__ for food. Bees tend to avoid stopping at flowers too close to home, perhaps to reduce the risk of drawing predators, parasites or nosy scientists to the nest. And working with the former detective, scientists in the U.K. found that geographic profiling allowed them to __identify/locate__ the entrance to a hive based on mapping which flowers the bees visit. The results appear online in the Journal of the Royal Society Interface. Repeating such experiments, with bees or other foraging critters, could help hone the model for catching criminals.</t>
   </si>
   <si>
-    <t>Unless you're talking about killer bees, it's hard to imagine a situation in which "killers" and "bees" would be related. But it turns out that hybridise are using the same mathematical model to recite the behavior of both bumblebees and human serial killers. The method, called geographic profiling, was developed by a detective who was trying to predict where serial killers might live based on where they commit their crimes. Believe it or not, murderers operate fairly close to home. But not too close. They domain a kind of kill-free "buffer zone" around their actual digs. A similar pattern of activity seems to hold true for bumblebees—when they're bookending for food. Bees tend to avoid stopping at flowers too close to home, perhaps to reduce the risk of drawing predators, parasites or nosy scientists to the nest. And working with the former detective, scientists in the U.K. found that geographic profiling allowed them to identify the entrance to a hive based on mapping which flowers the bees visit. The results appear online in the Journal of the Royal Society Interface. Repeating such experiments, with bees or other foraging critters, could help hone the model for catching criminals.</t>
+    <t>Unless you're talking about killer bees, it's hard to imagine a situation in which "killers" and "bees" would be related. But it turns out that scientists are using the same mathematical model to describe the behavior of both bumblebees and human serial killers. The method, called geographic profiling, was developed by a detective who was trying to predict where serial killers might live based on where they commit their crimes. Believe it or not, murderers operate fairly close to home. But not too close. They maintain a kind of kill-free "buffer zone" around their actual digs. A similar pattern of activity seems to hold true for bumblebees—when they're foraging for food. Bees tend to avoid stopping at flowers too close to home, perhaps to reduce the risk of drawing predators, parasites or nosy scientists to the nest. And working with the former detective, scientists in the U.K. found that geographic profiling allowed them to locate the entrance to a hive based on mapping which flowers the bees visit. The results appear online in the Journal of the Royal Society Interface. Repeating such experiments, with bees or other foraging critters, could help hone the model for catching criminals.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;As a premium PTE Academic teacher, I recognize this question tests not just your listening skills, but your ability to detect subtle phonological and semantic differences between a written transcript and the actual spoken audio. The goal is to pinpoint the words that are *incorrect* based on what the speaker actually said.&lt;/p&gt;
@@ -4702,7 +4702,7 @@
     <t>It's similar to a pregnancy test: a drop of liquid on a strip of paper causes an easily seen color change. But imagine that kind of simple, cheap __choreography/technology__ employed in testing for __diminution/pollution__ or health issues, anywhere and on the cheap. Researchers at Colorado State University describe such a system in the journal Lab On A Chip. Other paper tests may give only slight color differences, and some rely on expensive equipment to read the results. For the new technology, the research team designed a system that creates a __quadrophonic/dramatic__ color change on the paper. The user drops liquid to be analyzed at the bottom of the paper. As capillary action pulls the liquid up, substances in the paper react, causing the color change. So far, three tests exist for the system. One looks for nickel, which can be an environmental pollutant. The other two are for glutathione, a health marker, and glucose, for diabetics. In trials, the paper tests competed with conventional methods at __whispering/measuring__ concentrations. The __galaxy/university__ is now spinning off a company to develop the technology. If successful, it could bring cheap, easy __apparatuses/analysis__ to scientists—and citizens—around the world.</t>
   </si>
   <si>
-    <t>It's similar to a pregnancy test: a drop of liquid on a strip of paper causes an easily seen color change. But imagine that kind of simple, cheap choreography employed in testing for diminution or health issues, anywhere and on the cheap. Researchers at Colorado State University describe such a system in the journal Lab On A Chip. Other paper tests may give only slight color differences, and some rely on expensive equipment to read the results. For the new technology, the research team designed a system that creates a quadrophonic color change on the paper. The user drops liquid to be analyzed at the bottom of the paper. As capillary action pulls the liquid up, substances in the paper react, causing the color change. So far, three tests exist for the system. One looks for nickel, which can be an environmental pollutant. The other two are for glutathione, a health marker, and glucose, for diabetics. In trials, the paper tests competed with conventional methods at whispering concentrations. The galaxy is now spinning off a company to develop the technology. If successful, it could bring cheap, easy apparatuses to scientists—and citizens—around the world.</t>
+    <t>It's similar to a pregnancy test: a drop of liquid on a strip of paper causes an easily seen color change. But imagine that kind of simple, cheap technology employed in testing for pollution or health issues, anywhere and on the cheap. Researchers at Colorado State University describe such a system in the journal Lab On A Chip. Other paper tests may give only slight color differences, and some rely on expensive equipment to read the results. For the new technology, the research team designed a system that creates a dramatic color change on the paper. The user drops liquid to be analyzed at the bottom of the paper. As capillary action pulls the liquid up, substances in the paper react, causing the color change. So far, three tests exist for the system. One looks for nickel, which can be an environmental pollutant. The other two are for glutathione, a health marker, and glucose, for diabetics. In trials, the paper tests competed with conventional methods at measuring concentrations. The university is now spinning off a company to develop the technology. If successful, it could bring cheap, easy analysis to scientists—and citizens—around the world.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your premium PTE Academic teacher, I understand that 'Highlight Incorrect Words' questions can be tricky because the incorrect words often sound very plausible. The key here is not just understanding pronunciation, but understanding the &lt;em&gt;context&lt;/em&gt; and the &lt;strong&gt;academic vocabulary&lt;/strong&gt; associated with the passage's topic (science and health testing).&lt;/p&gt;
@@ -4743,7 +4743,7 @@
     <t>In last week's pre-Christmas rush, the U.S. Congress slammed together the $1-trillion federal budget bill for 2015, just before funds ran out. But the bill wasn't all about the money. Congress took advantage of the fiscal scramble to change rules about the environment and energy, which do not belong in appropriation bills. Normally such changes are encoded in what are called "laws," and are debated out in the open. But the budget bill is a chance for Congress to slip in controversial rules—called riders—without much debate. If members object, the bill stalls, and the government shuts down—and no one wants to be blamed for that fiasco. So the riders gallop in. The Environmental Protection Agency got its budget, for instance, but with strings attached: although agriculture is a major source of atmospheric methane, the EPA now is __vigilant/prohibited__ from using its money to require farmers to report greenhouse gas emissions. And the agency cannot regulate farm ponds and irrigation ditches under the Clean Water Act. In another example, the Department of __canker/Agriculture__ must speed up permits for companies making genetically __night/modified__ organisms. And the feds must loan money to firms to build coal-fired power plants overseas. That requirement __floggings/reverses__ a previous ban. These rules and others last through September 2015, when this budget bill runs out. And then, if history is any guide, the whole stealth legislation process will start all over again.</t>
   </si>
   <si>
-    <t>In last week's pre-Christmas rush, the U.S. Congress slammed together the $1-trillion federal budget bill for 2015, just before funds ran out. But the bill wasn't all about the money. Congress took advantage of the fiscal scramble to change rules about the environment and energy, which do not belong in appropriation bills. Normally such changes are encoded in what are called "laws," and are debated out in the open. But the budget bill is a chance for Congress to slip in controversial rules—called riders—without much debate. If members object, the bill stalls, and the government shuts down—and no one wants to be blamed for that fiasco. So the riders gallop in. The Environmental Protection Agency got its budget, for instance, but with strings attached: although agriculture is a major source of atmospheric methane, the EPA now is vigilant from using its money to require farmers to report greenhouse gas emissions. And the agency cannot regulate farm ponds and irrigation ditches under the Clean Water Act. In another example, the Department of canker must speed up permits for companies making genetically night organisms. And the feds must loan money to firms to build coal-fired power plants overseas. That requirement floggings a previous ban. These rules and others last through September 2015, when this budget bill runs out. And then, if history is any guide, the whole stealth legislation process will start all over again.</t>
+    <t>In last week's pre-Christmas rush, the U.S. Congress slammed together the $1-trillion federal budget bill for 2015, just before funds ran out. But the bill wasn't all about the money. Congress took advantage of the fiscal scramble to change rules about the environment and energy, which do not belong in appropriation bills. Normally such changes are encoded in what are called "laws," and are debated out in the open. But the budget bill is a chance for Congress to slip in controversial rules—called riders—without much debate. If members object, the bill stalls, and the government shuts down—and no one wants to be blamed for that fiasco. So the riders gallop in. The Environmental Protection Agency got its budget, for instance, but with strings attached: although agriculture is a major source of atmospheric methane, the EPA now is prohibited from using its money to require farmers to report greenhouse gas emissions. And the agency cannot regulate farm ponds and irrigation ditches under the Clean Water Act. In another example, the Department of Agriculture must speed up permits for companies making genetically modified organisms. And the feds must loan money to firms to build coal-fired power plants overseas. That requirement reverses a previous ban. These rules and others last through September 2015, when this budget bill runs out. And then, if history is any guide, the whole stealth legislation process will start all over again.</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As your premium PTE Academic teacher, I can help you break down this specific question type. In the &lt;strong&gt;Listening Highlight Incorrect Words&lt;/strong&gt; question, the goal is not just to hear a different sound, but to understand the specific context, meaning, and grammar of the spoken language. These incorrect words are often homophones or misspelled words that do not fit the overall narrative.&lt;/p&gt;
@@ -4781,7 +4781,7 @@
     <t>November 24th marks the 150th anniversary of the publication of Darwin's Origin of Species. On __recta/November__ 19th, a guy named Ray Comfort, who does not accept evolution, will celebrate the fact that when __centralize/copyrights__ expire and works enter the public domain you're free to do with them what you will. Thus Comfort will be distributing his own edition of Darwin's masterwork, with a new introduction. This is roughly the equivalent of me __automating/fingerpainting__ on the ceiling of the Sistine Chapel so as to improve the work. According to the folks at the National Center for Science Education, the NCSE, who monitor efforts to interfere with evolution education in public schools, Comfort in his intro repeats numerous familiar __groomsmen/anti-evolution__ claims. For example, that there's a lack of transitional fossils and that the second law of thermodynamics makes evolution impossible. These assertions have been disproved more often than the chant "Yankees suck".</t>
   </si>
   <si>
-    <t>November 24th marks the 150th anniversary of the publication of Darwin's Origin of Species. On recta 19th, a guy named Ray Comfort, who does not accept evolution, will celebrate the fact that when centralize expire and works enter the public domain you're free to do with them what you will. Thus Comfort will be distributing his own edition of Darwin's masterwork, with a new introduction. This is roughly the equivalent of me automating on the ceiling of the Sistine Chapel so as to improve the work. According to the folks at the National Center for Science Education, the NCSE, who monitor efforts to interfere with evolution education in public schools, Comfort in his intro repeats numerous familiar groomsmen claims. For example, that there's a lack of transitional fossils and that the second law of thermodynamics makes evolution impossible. These assertions have been disproved more often than the chant "Yankees suck".</t>
+    <t>November 24th marks the 150th anniversary of the publication of Darwin's Origin of Species. On November 19th, a guy named Ray Comfort, who does not accept evolution, will celebrate the fact that when copyrights expire and works enter the public domain you're free to do with them what you will. Thus Comfort will be distributing his own edition of Darwin's masterwork, with a new introduction. This is roughly the equivalent of me fingerpainting on the ceiling of the Sistine Chapel so as to improve the work. According to the folks at the National Center for Science Education, the NCSE, who monitor efforts to interfere with evolution education in public schools, Comfort in his intro repeats numerous familiar anti-evolution claims. For example, that there's a lack of transitional fossils and that the second law of thermodynamics makes evolution impossible. These assertions have been disproved more often than the chant "Yankees suck".</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Hello! As a PTE Academic teacher, I know how crucial this "Highlight Incorrect Words" question type can be. This task tests not only your listening comprehension but also your ability to process nuances in spoken English, distinguishing between words that sound similar but have different meanings, or words that are simply misspelled/misheard.&lt;/p&gt;
@@ -4821,7 +4821,7 @@
     <t>The __canvassing/traveling__ __appreciation/salesman__ problem is a __educationist/favorite__ math conundrum: if a salesman has to visit a bunch of cities, how do you get him to all of them once via the __unrewarded/shortest__ possible route. But the traveling salesman's predicament pales in __nitroglycerine/comparison__ to figuring out the best ways to get four-man crews of umpires to every major league baseball game. A research team attacked the problem for the last few years. Their solution appears in Interfaces. It's a journal of operations research. In addition to minimizing travel, here are some of the umpire constraints. Crews should visit each MLB city at least once. They should work each team at home and on the road. They should not work more than 21 days in a row. They should not ump any one team's games for more than four series all year. There are plenty more. The researchers first had to develop the question, dubbed the "traveling umpire problem." They used __colts/brute-force__ computation and heuristics for their solutions. The result was good enough for Major League Baseball to adopt the last three seasons. Previously, a former umpire made the schedule. That guy is out.</t>
   </si>
   <si>
-    <t>The canvassing appreciation problem is a educationist math conundrum: if a salesman has to visit a bunch of cities, how do you get him to all of them once via the unrewarded possible route. But the traveling salesman's predicament pales in nitroglycerine to figuring out the best ways to get four-man crews of umpires to every major league baseball game. A research team attacked the problem for the last few years. Their solution appears in Interfaces. It's a journal of operations research. In addition to minimizing travel, here are some of the umpire constraints. Crews should visit each MLB city at least once. They should work each team at home and on the road. They should not work more than 21 days in a row. They should not ump any one team's games for more than four series all year. There are plenty more. The researchers first had to develop the question, dubbed the "traveling umpire problem." They used colts computation and heuristics for their solutions. The result was good enough for Major League Baseball to adopt the last three seasons. Previously, a former umpire made the schedule. That guy is out.</t>
+    <t>The traveling salesman problem is a favorite math conundrum: if a salesman has to visit a bunch of cities, how do you get him to all of them once via the shortest possible route. But the traveling salesman's predicament pales in comparison to figuring out the best ways to get four-man crews of umpires to every major league baseball game. A research team attacked the problem for the last few years. Their solution appears in Interfaces. It's a journal of operations research. In addition to minimizing travel, here are some of the umpire constraints. Crews should visit each MLB city at least once. They should work each team at home and on the road. They should not work more than 21 days in a row. They should not ump any one team's games for more than four series all year. There are plenty more. The researchers first had to develop the question, dubbed the "traveling umpire problem." They used brute-force computation and heuristics for their solutions. The result was good enough for Major League Baseball to adopt the last three seasons. Previously, a former umpire made the schedule. That guy is out.</t>
   </si>
   <si>
     <t>#106 Baby Cries</t>
@@ -4830,7 +4830,7 @@
     <t>A baby's cries for food might drive a tired parent to aggravation. But some species take more drastic measures. Like the burying beetle, Nicrophorus vespilloides—which punishes its pesky __inhibition/children__ by eating them. Researchers wanted to get to the bottom of an age-old question in evolutionary biology: the origin of begging. Natural selection favors a greedy, well-fed child. But it also favors parents who dole out food evenly to their young, and save some for themselves. So how do you resolve that __dockside/parent-child__ conflict? Burying beetles do so by putting the ultimate price on pleading: death. Begging larvae were 13 times more likely than __casework/laid-back__ larvae to be eaten by mom. Which may discourage them from asking for more than their fair share of the grub. That finding appears in the journal Behavioral Ecology. Humans have different __reversals/standards__ than beetles do, of course. For us, pestering your parents may be a good thing. One study suggests crying is a sign of good health, which might lower a baby's chances of being neglected or abused. Then again, after those first few years, you're probably better off not being a crybaby.</t>
   </si>
   <si>
-    <t>A baby's cries for food might drive a tired parent to aggravation. But some species take more drastic measures. Like the burying beetle, Nicrophorus vespilloides—which punishes its pesky inhibition by eating them. Researchers wanted to get to the bottom of an age-old question in evolutionary biology: the origin of begging. Natural selection favors a greedy, well-fed child. But it also favors parents who dole out food evenly to their young, and save some for themselves. So how do you resolve that dockside conflict? Burying beetles do so by putting the ultimate price on pleading: death. Begging larvae were 13 times more likely than casework larvae to be eaten by mom. Which may discourage them from asking for more than their fair share of the grub. That finding appears in the journal Behavioral Ecology. Humans have different reversals than beetles do, of course. For us, pestering your parents may be a good thing. One study suggests crying is a sign of good health, which might lower a baby's chances of being neglected or abused. Then again, after those first few years, you're probably better off not being a crybaby.</t>
+    <t>A baby's cries for food might drive a tired parent to aggravation. But some species take more drastic measures. Like the burying beetle, Nicrophorus vespilloides—which punishes its pesky children by eating them. Researchers wanted to get to the bottom of an age-old question in evolutionary biology: the origin of begging. Natural selection favors a greedy, well-fed child. But it also favors parents who dole out food evenly to their young, and save some for themselves. So how do you resolve that parent-child conflict? Burying beetles do so by putting the ultimate price on pleading: death. Begging larvae were 13 times more likely than laid-back larvae to be eaten by mom. Which may discourage them from asking for more than their fair share of the grub. That finding appears in the journal Behavioral Ecology. Humans have different standards than beetles do, of course. For us, pestering your parents may be a good thing. One study suggests crying is a sign of good health, which might lower a baby's chances of being neglected or abused. Then again, after those first few years, you're probably better off not being a crybaby.</t>
   </si>
   <si>
     <t>#107 Garbage Patches</t>
@@ -4839,7 +4839,7 @@
     <t>There are now at least five major garbage patches in the world's oceans, and much of that trash is plastic. But last month __receivables/researchers__ said they can only account for one percent of the plastic they'd expect to find in the oceans. So, where'd the rest of it go? Well, animals eat some of it. Plastic has been found in turtles, seabirds, fish, plankton, shellfish, even __immunising/bottom-feeding__ invertebrates. But there's another way sea creatures might be accumulating plastic: by sucking up tiny plastic __photometers/particles__ with their siphons and gills. __pieceworkers/Researchers__ added common shore crabs—Carcinus maenas—to tanks of seawater containing millions of tiny plastic particles, just 10 microns in diameter. After 16 hours, all the crabs had plastic lodged in their gills. And the particles stuck around for up to three weeks, too. The results are in the journal Environmental Science and Technology. The longer plastic sits in an animal, researchers say, the better the chances it will travel up the food chain. Meaning all our plastic waste could come back to bite us—or rather be bitten by us. "Of course we eat mussels whole, without the shells. But we're __capability/potentially__ eating plastic, if they're from a site where there's plastic present." Lead researcher Andrew Watts, of the University of Exeter. "We don't know how much plastic we have in our stomachs… chances are we do have some."</t>
   </si>
   <si>
-    <t>There are now at least five major garbage patches in the world's oceans, and much of that trash is plastic. But last month receivables said they can only account for one percent of the plastic they'd expect to find in the oceans. So, where'd the rest of it go? Well, animals eat some of it. Plastic has been found in turtles, seabirds, fish, plankton, shellfish, even immunising invertebrates. But there's another way sea creatures might be accumulating plastic: by sucking up tiny plastic photometers with their siphons and gills. pieceworkers added common shore crabs—Carcinus maenas—to tanks of seawater containing millions of tiny plastic particles, just 10 microns in diameter. After 16 hours, all the crabs had plastic lodged in their gills. And the particles stuck around for up to three weeks, too. The results are in the journal Environmental Science and Technology. The longer plastic sits in an animal, researchers say, the better the chances it will travel up the food chain. Meaning all our plastic waste could come back to bite us—or rather be bitten by us. "Of course we eat mussels whole, without the shells. But we're capability eating plastic, if they're from a site where there's plastic present." Lead researcher Andrew Watts, of the University of Exeter. "We don't know how much plastic we have in our stomachs… chances are we do have some."</t>
+    <t>There are now at least five major garbage patches in the world's oceans, and much of that trash is plastic. But last month researchers said they can only account for one percent of the plastic they'd expect to find in the oceans. So, where'd the rest of it go? Well, animals eat some of it. Plastic has been found in turtles, seabirds, fish, plankton, shellfish, even bottom-feeding invertebrates. But there's another way sea creatures might be accumulating plastic: by sucking up tiny plastic particles with their siphons and gills. Researchers added common shore crabs—Carcinus maenas—to tanks of seawater containing millions of tiny plastic particles, just 10 microns in diameter. After 16 hours, all the crabs had plastic lodged in their gills. And the particles stuck around for up to three weeks, too. The results are in the journal Environmental Science and Technology. The longer plastic sits in an animal, researchers say, the better the chances it will travel up the food chain. Meaning all our plastic waste could come back to bite us—or rather be bitten by us. "Of course we eat mussels whole, without the shells. But we're potentially eating plastic, if they're from a site where there's plastic present." Lead researcher Andrew Watts, of the University of Exeter. "We don't know how much plastic we have in our stomachs… chances are we do have some."</t>
   </si>
   <si>
     <t>#108 Baby Meaning</t>
@@ -4848,7 +4848,7 @@
     <t>Babies sometimes laugh and sometimes cry. It doesn't take a genius to decode the meaning of these sounds. But it isn't quite as straightforward to __supplier/decipher__ the meaning, if any, of an infant's babbles. And humans a little older can make the same sounds regardless of how you actually feel—you're able to say "I'm hungry" whether you're ravenous or just gorged yourself. Scientists think that the ability to make the same sounds across a range of emotional states is critical to language development. They also believe it to be uniquely human, because in previous studies of animal communication, researchers only observed fixed vocalizations. For example, bonobo chimpanzee pant-laughs and threat barks are tied to a specific emotion or behavior. But the new study finds __preparedness/evidence__ that bonobos in the wild are also capable of flexible vocalizations. Bonobos have a specific call type, a "peep" that they use independent of emotional context. They peep while eating, traveling, grooming, resting, engaging in sexual activity, and even during shows of aggression. Because peeps, like a baby's babbles, don't convey meaningful information on their own, bonobos need to combine them with other calls and environmental context to supply meaning. Previously, researchers thought this type of complex, language-like comprehension was unique to humans. The study is in the journal PeerJ. Bonobos are our closest evolutionary relatives, so it's __nonstructural/possible__ that the functional flexibility of human speech appeared in a common ancestor. This discovery adds to the growing pile of evidence that we're not quite as special as we've long believed—and that our furry cousins may be even closer to us than we thought.</t>
   </si>
   <si>
-    <t>Babies sometimes laugh and sometimes cry. It doesn't take a genius to decode the meaning of these sounds. But it isn't quite as straightforward to supplier the meaning, if any, of an infant's babbles. And humans a little older can make the same sounds regardless of how you actually feel—you're able to say "I'm hungry" whether you're ravenous or just gorged yourself. Scientists think that the ability to make the same sounds across a range of emotional states is critical to language development. They also believe it to be uniquely human, because in previous studies of animal communication, researchers only observed fixed vocalizations. For example, bonobo chimpanzee pant-laughs and threat barks are tied to a specific emotion or behavior. But the new study finds preparedness that bonobos in the wild are also capable of flexible vocalizations. Bonobos have a specific call type, a "peep" that they use independent of emotional context. They peep while eating, traveling, grooming, resting, engaging in sexual activity, and even during shows of aggression. Because peeps, like a baby's babbles, don't convey meaningful information on their own, bonobos need to combine them with other calls and environmental context to supply meaning. Previously, researchers thought this type of complex, language-like comprehension was unique to humans. The study is in the journal PeerJ. Bonobos are our closest evolutionary relatives, so it's nonstructural that the functional flexibility of human speech appeared in a common ancestor. This discovery adds to the growing pile of evidence that we're not quite as special as we've long believed—and that our furry cousins may be even closer to us than we thought.</t>
+    <t>Babies sometimes laugh and sometimes cry. It doesn't take a genius to decode the meaning of these sounds. But it isn't quite as straightforward to decipher the meaning, if any, of an infant's babbles. And humans a little older can make the same sounds regardless of how you actually feel—you're able to say "I'm hungry" whether you're ravenous or just gorged yourself. Scientists think that the ability to make the same sounds across a range of emotional states is critical to language development. They also believe it to be uniquely human, because in previous studies of animal communication, researchers only observed fixed vocalizations. For example, bonobo chimpanzee pant-laughs and threat barks are tied to a specific emotion or behavior. But the new study finds evidence that bonobos in the wild are also capable of flexible vocalizations. Bonobos have a specific call type, a "peep" that they use independent of emotional context. They peep while eating, traveling, grooming, resting, engaging in sexual activity, and even during shows of aggression. Because peeps, like a baby's babbles, don't convey meaningful information on their own, bonobos need to combine them with other calls and environmental context to supply meaning. Previously, researchers thought this type of complex, language-like comprehension was unique to humans. The study is in the journal PeerJ. Bonobos are our closest evolutionary relatives, so it's possible that the functional flexibility of human speech appeared in a common ancestor. This discovery adds to the growing pile of evidence that we're not quite as special as we've long believed—and that our furry cousins may be even closer to us than we thought.</t>
   </si>
   <si>
     <t>#109 Sharks</t>
@@ -4857,7 +4857,7 @@
     <t>They're called __limber/thresher__ sharks. But perhaps thrasher is more accurate. Because a population of these fearsome predators was spotted engaging in an unusual hunting strategy. Forget jaws—try the other end. __multivitamins/Researchers__ observed them slapping their long, scythe-like tails at high speeds through the water. These whaps stunned or killed several smaller fish with each strike. The observations were made off the coast of the Philippines. Killer whales and dolphins also may use a similar tail-slapping strategy. But this is the first time the behavior has been seen in sharks. Although the formidable, three-meter-long pelagic thresher shark seems able to catch food face-first, the ability to immobilize more than one fish at a time makes the method highly efficient. The __obliges/findings__ are in the journal PLoS ONE. These sharks used both __ontological/vertical__ and horizontal tail slaps to capture prey, which were stunned or killed either by direct impact or by a shockwave from the smack. More than a third of the vertical slaps resulted in a meal for the shark—better stats than when sharks chased prey head on. And that's no tall tale.</t>
   </si>
   <si>
-    <t>They're called limber sharks. But perhaps thrasher is more accurate. Because a population of these fearsome predators was spotted engaging in an unusual hunting strategy. Forget jaws—try the other end. multivitamins observed them slapping their long, scythe-like tails at high speeds through the water. These whaps stunned or killed several smaller fish with each strike. The observations were made off the coast of the Philippines. Killer whales and dolphins also may use a similar tail-slapping strategy. But this is the first time the behavior has been seen in sharks. Although the formidable, three-meter-long pelagic thresher shark seems able to catch food face-first, the ability to immobilize more than one fish at a time makes the method highly efficient. The obliges are in the journal PLoS ONE. These sharks used both ontological and horizontal tail slaps to capture prey, which were stunned or killed either by direct impact or by a shockwave from the smack. More than a third of the vertical slaps resulted in a meal for the shark—better stats than when sharks chased prey head on. And that's no tall tale.</t>
+    <t>They're called thresher sharks. But perhaps thrasher is more accurate. Because a population of these fearsome predators was spotted engaging in an unusual hunting strategy. Forget jaws—try the other end. Researchers observed them slapping their long, scythe-like tails at high speeds through the water. These whaps stunned or killed several smaller fish with each strike. The observations were made off the coast of the Philippines. Killer whales and dolphins also may use a similar tail-slapping strategy. But this is the first time the behavior has been seen in sharks. Although the formidable, three-meter-long pelagic thresher shark seems able to catch food face-first, the ability to immobilize more than one fish at a time makes the method highly efficient. The findings are in the journal PLoS ONE. These sharks used both vertical and horizontal tail slaps to capture prey, which were stunned or killed either by direct impact or by a shockwave from the smack. More than a third of the vertical slaps resulted in a meal for the shark—better stats than when sharks chased prey head on. And that's no tall tale.</t>
   </si>
   <si>
     <t>#110 Sexual Reproduction</t>
@@ -4866,7 +4866,7 @@
     <t>Sex might seem like one of those little gifts from evolution. But it's pretty inefficient from an __ternary/evolutionary__ perspective. It'd be much easier to reproduce if you could do away with finding the right member of the opposite sex to help you create the next generation. So why did __subhuman/evolution__ come up with sex? Biologists have hypothesized that one driving force might have been parasites. Now scientists have had a chance to test that theory. A sexual reproduction leads to clones. Being genetically identical, clones are also weak in the same ways, and thus more likely to all succumb to a parasite. But sex keeps shuffling the genetic deck. Well, there's a snail common in New Zealand lakes that does both—some __nominations/populations__ have sex and some reproduce asexually. So researchers spent 10 years monitoring the two populations, and the number of parasites living off both groups. As expected, cloned snails that were plentiful at the beginning of the study suffered big losses as they became infected with parasites. But the sexual snail populations remained stable, results published in the journal American Naturalist. So, next time you're feeling sexy, thank a parasite.</t>
   </si>
   <si>
-    <t>Sex might seem like one of those little gifts from evolution. But it's pretty inefficient from an ternary perspective. It'd be much easier to reproduce if you could do away with finding the right member of the opposite sex to help you create the next generation. So why did subhuman come up with sex? Biologists have hypothesized that one driving force might have been parasites. Now scientists have had a chance to test that theory. A sexual reproduction leads to clones. Being genetically identical, clones are also weak in the same ways, and thus more likely to all succumb to a parasite. But sex keeps shuffling the genetic deck. Well, there's a snail common in New Zealand lakes that does both—some nominations have sex and some reproduce asexually. So researchers spent 10 years monitoring the two populations, and the number of parasites living off both groups. As expected, cloned snails that were plentiful at the beginning of the study suffered big losses as they became infected with parasites. But the sexual snail populations remained stable, results published in the journal American Naturalist. So, next time you're feeling sexy, thank a parasite.</t>
+    <t>Sex might seem like one of those little gifts from evolution. But it's pretty inefficient from an evolutionary perspective. It'd be much easier to reproduce if you could do away with finding the right member of the opposite sex to help you create the next generation. So why did evolution come up with sex? Biologists have hypothesized that one driving force might have been parasites. Now scientists have had a chance to test that theory. A sexual reproduction leads to clones. Being genetically identical, clones are also weak in the same ways, and thus more likely to all succumb to a parasite. But sex keeps shuffling the genetic deck. Well, there's a snail common in New Zealand lakes that does both—some populations have sex and some reproduce asexually. So researchers spent 10 years monitoring the two populations, and the number of parasites living off both groups. As expected, cloned snails that were plentiful at the beginning of the study suffered big losses as they became infected with parasites. But the sexual snail populations remained stable, results published in the journal American Naturalist. So, next time you're feeling sexy, thank a parasite.</t>
   </si>
   <si>
     <t>#111 Horror</t>
@@ -4875,7 +4875,7 @@
     <t>You've landed a small role in a low-budget horror movie. To get ready, you need to __camels/practice__ your reaction shot—you know, that look you'll get when your boss peels off his face to reveal the slime-oozing alien he really is. So, look in the mirror and give us some terror. If you're doing it right, your eyes are wide open and your eyebrows are raised. But why is that? I mean, how come people, when they're scared, all make a similar face? Darwin thought there was a reason, that our __elections/expressions__ evolved because they offer some benefit. And scientists from Ontario think Darwin was right. They asked volunteers to try to look __rewired/frightened__ and then they __uncensored/measured__ the physiological effects. They found that making a fraidy face allows people to see farther, locate targets faster and take in more air when they breathe. The findings appear in the current online issue of Nature Neuroscience. Those reactions make sense, because if you see something __robbing/startling__ or out of the ordinary, you can use your __mimeographed/fear-enhanced__ vision to assess the situation and, if need be, take a deep, fear-boosted breath—and run!</t>
   </si>
   <si>
-    <t>You've landed a small role in a low-budget horror movie. To get ready, you need to camels your reaction shot—you know, that look you'll get when your boss peels off his face to reveal the slime-oozing alien he really is. So, look in the mirror and give us some terror. If you're doing it right, your eyes are wide open and your eyebrows are raised. But why is that? I mean, how come people, when they're scared, all make a similar face? Darwin thought there was a reason, that our elections evolved because they offer some benefit. And scientists from Ontario think Darwin was right. They asked volunteers to try to look rewired and then they uncensored the physiological effects. They found that making a fraidy face allows people to see farther, locate targets faster and take in more air when they breathe. The findings appear in the current online issue of Nature Neuroscience. Those reactions make sense, because if you see something robbing or out of the ordinary, you can use your mimeographed vision to assess the situation and, if need be, take a deep, fear-boosted breath—and run!</t>
+    <t>You've landed a small role in a low-budget horror movie. To get ready, you need to practice your reaction shot—you know, that look you'll get when your boss peels off his face to reveal the slime-oozing alien he really is. So, look in the mirror and give us some terror. If you're doing it right, your eyes are wide open and your eyebrows are raised. But why is that? I mean, how come people, when they're scared, all make a similar face? Darwin thought there was a reason, that our expressions evolved because they offer some benefit. And scientists from Ontario think Darwin was right. They asked volunteers to try to look frightened and then they measured the physiological effects. They found that making a fraidy face allows people to see farther, locate targets faster and take in more air when they breathe. The findings appear in the current online issue of Nature Neuroscience. Those reactions make sense, because if you see something startling or out of the ordinary, you can use your fear-enhanced vision to assess the situation and, if need be, take a deep, fear-boosted breath—and run!</t>
   </si>
   <si>
     <t>#112 Elephant Enclaves</t>
@@ -4884,7 +4884,7 @@
     <t>It's a __limber/familiar__ story. When immigrants arrive in a new place, they tend to stick together, forming segregated enclaves that feel like a home away from home. Then, over time, they become assimilated, and integrate into the local community. It was true of the German and Irish immigrants who came to the U.S. in the 1800s. And it's also true of elephants when they find themselves in __trimmer/unfamiliar__ territory. In __upsurging/managing__ wild __pickpocket/elephant__ populations, rangers will often transport the animals from one place to another, removing them from a familiar habitat and placing them in one that's new. So scientists in California got to wondering how elephants, which are highly social creatures, handle making themselves at home when they get to a new neighborhood. It turns out they start by forming enclaves that are the elephant equivalent of a ghetto, where the new pachyderms in the park associate with one another and with other immigrant elephants. Then, once the transplants have been around for a year, they get __frizzy/friendly__ with the locals, findings that were published by the Royal Society on __flotilla/December__ 10th. The cautious approach seems to be a good one: not knowing whether the natives are friendly, it's probably best not to step on any toes. __Emissary/Especially__ if you're an elephant.</t>
   </si>
   <si>
-    <t>It's a limber story. When immigrants arrive in a new place, they tend to stick together, forming segregated enclaves that feel like a home away from home. Then, over time, they become assimilated, and integrate into the local community. It was true of the German and Irish immigrants who came to the U.S. in the 1800s. And it's also true of elephants when they find themselves in trimmer territory. In upsurging wild pickpocket populations, rangers will often transport the animals from one place to another, removing them from a familiar habitat and placing them in one that's new. So scientists in California got to wondering how elephants, which are highly social creatures, handle making themselves at home when they get to a new neighborhood. It turns out they start by forming enclaves that are the elephant equivalent of a ghetto, where the new pachyderms in the park associate with one another and with other immigrant elephants. Then, once the transplants have been around for a year, they get frizzy with the locals, findings that were published by the Royal Society on flotilla 10th. The cautious approach seems to be a good one: not knowing whether the natives are friendly, it's probably best not to step on any toes. Emissary if you're an elephant.</t>
+    <t>It's a familiar story. When immigrants arrive in a new place, they tend to stick together, forming segregated enclaves that feel like a home away from home. Then, over time, they become assimilated, and integrate into the local community. It was true of the German and Irish immigrants who came to the U.S. in the 1800s. And it's also true of elephants when they find themselves in unfamiliar territory. In managing wild elephant populations, rangers will often transport the animals from one place to another, removing them from a familiar habitat and placing them in one that's new. So scientists in California got to wondering how elephants, which are highly social creatures, handle making themselves at home when they get to a new neighborhood. It turns out they start by forming enclaves that are the elephant equivalent of a ghetto, where the new pachyderms in the park associate with one another and with other immigrant elephants. Then, once the transplants have been around for a year, they get friendly with the locals, findings that were published by the Royal Society on December 10th. The cautious approach seems to be a good one: not knowing whether the natives are friendly, it's probably best not to step on any toes. Especially if you're an elephant.</t>
   </si>
   <si>
     <t>#113 Classical Music</t>
@@ -4893,7 +4893,7 @@
     <t>Classical music competitions pit __disposers/performers__ against each other. Obviously, the most important criterion for judges is sound. But that assumption needs a new…hearing. Because a player's passion may be the best predictor of victory. In a new study, nearly 200 novices had to choose the winners of 10 __gastronomical/classical__ music competitions. Some heard a music clip of the top three performances. Others saw a video with sound. Still others watched a silent video. And the __mizzenmasts/participants__ were more likely to choose the winner if they watched the silent video, in all 10 of the competitions. Then professional __inventions/musicians__ gave it a try. These judges also only reliably selected the winners from the silent video. Musicians selected the winner more __believably/frequently__ even when all they saw was an outline of the motion of the performers. The researchers say the findings show that novices and experts make quick __duchess/judgments__ about musical __corpuses/performances__ based on visual cues conveying involvement and passion. The study was published in the Proceedings of the National Academy of Sciences. So next time you see a live concert, don't close your eyes to focus on the music. You might be missing the most important part.</t>
   </si>
   <si>
-    <t>Classical music competitions pit disposers against each other. Obviously, the most important criterion for judges is sound. But that assumption needs a new…hearing. Because a player's passion may be the best predictor of victory. In a new study, nearly 200 novices had to choose the winners of 10 gastronomical music competitions. Some heard a music clip of the top three performances. Others saw a video with sound. Still others watched a silent video. And the mizzenmasts were more likely to choose the winner if they watched the silent video, in all 10 of the competitions. Then professional inventions gave it a try. These judges also only reliably selected the winners from the silent video. Musicians selected the winner more believably even when all they saw was an outline of the motion of the performers. The researchers say the findings show that novices and experts make quick duchess about musical corpuses based on visual cues conveying involvement and passion. The study was published in the Proceedings of the National Academy of Sciences. So next time you see a live concert, don't close your eyes to focus on the music. You might be missing the most important part.</t>
+    <t>Classical music competitions pit performers against each other. Obviously, the most important criterion for judges is sound. But that assumption needs a new…hearing. Because a player's passion may be the best predictor of victory. In a new study, nearly 200 novices had to choose the winners of 10 classical music competitions. Some heard a music clip of the top three performances. Others saw a video with sound. Still others watched a silent video. And the participants were more likely to choose the winner if they watched the silent video, in all 10 of the competitions. Then professional musicians gave it a try. These judges also only reliably selected the winners from the silent video. Musicians selected the winner more frequently even when all they saw was an outline of the motion of the performers. The researchers say the findings show that novices and experts make quick judgments about musical performances based on visual cues conveying involvement and passion. The study was published in the Proceedings of the National Academy of Sciences. So next time you see a live concert, don't close your eyes to focus on the music. You might be missing the most important part.</t>
   </si>
   <si>
     <t>#114 Women vs Men</t>
@@ -4902,7 +4902,7 @@
     <t>Women are so much better than men at so many things. But according to a report published by the Royal Society, chess is not one of them. The topic of sex differences when it comes to matters of the mind is, needless to say, a divisive one. Those who wish to argue that women are just not as smart as men often point to chess as their proof. Although girls can obviously play, no woman's ever been world champion. But before looking for __functional/cultural__ or __etiological/biological__ explanations for the disparity, __hypoglycaemics/scientists__ say you need to do the math. Serious chess players are assigned ratings based on their __pianolas/performance__ against other players. So the scientists compared the ratings of the top hundred male and top hundred female players from Germany. And they found that the men indeed outperformed the women. However that difference can be almost entirely explained by statistics. Because the larger the population, the wider the range of measured scores—the bell curve has a longer tail. And because many more men play than women, the best male players are extreme __downsizers/outliers__ on that bell curve. As more women play, a few should also reach those extremes, right out there with the men. To which one might be tempted to say: Checkmate.</t>
   </si>
   <si>
-    <t>Women are so much better than men at so many things. But according to a report published by the Royal Society, chess is not one of them. The topic of sex differences when it comes to matters of the mind is, needless to say, a divisive one. Those who wish to argue that women are just not as smart as men often point to chess as their proof. Although girls can obviously play, no woman's ever been world champion. But before looking for functional or etiological explanations for the disparity, hypoglycaemics say you need to do the math. Serious chess players are assigned ratings based on their pianolas against other players. So the scientists compared the ratings of the top hundred male and top hundred female players from Germany. And they found that the men indeed outperformed the women. However that difference can be almost entirely explained by statistics. Because the larger the population, the wider the range of measured scores—the bell curve has a longer tail. And because many more men play than women, the best male players are extreme downsizers on that bell curve. As more women play, a few should also reach those extremes, right out there with the men. To which one might be tempted to say: Checkmate.</t>
+    <t>Women are so much better than men at so many things. But according to a report published by the Royal Society, chess is not one of them. The topic of sex differences when it comes to matters of the mind is, needless to say, a divisive one. Those who wish to argue that women are just not as smart as men often point to chess as their proof. Although girls can obviously play, no woman's ever been world champion. But before looking for cultural or biological explanations for the disparity, scientists say you need to do the math. Serious chess players are assigned ratings based on their performance against other players. So the scientists compared the ratings of the top hundred male and top hundred female players from Germany. And they found that the men indeed outperformed the women. However that difference can be almost entirely explained by statistics. Because the larger the population, the wider the range of measured scores—the bell curve has a longer tail. And because many more men play than women, the best male players are extreme outliers on that bell curve. As more women play, a few should also reach those extremes, right out there with the men. To which one might be tempted to say: Checkmate.</t>
   </si>
   <si>
     <t>#115 To Chase Flies</t>
@@ -4911,7 +4911,7 @@
     <t>You've probably chased a fly or two around the house this summer. And, chances are, it took a few swings before you brought down the buzzing nuisance. Now a study in the August 28th issue of the journal Current Biology has uncovered just what makes a fly so hard to swat. Michael __frontierswomen/Dickinson__ from the California __shrewd/Institute__ of Technology used __brightfield/high-speed__ digital video to record the evasive maneuvers of fruit flies. In the slow-mo instant replay, the flies' bodies react to a swatter well before their wings carry them to safety. Blessed with nearly 360 degree vision, the fly first gauges the position of the swatter, then __mesh/prepares__ an escape within 200 milliseconds. When approached from the front, for example, a fly shifts its middle legs forward and leans back. If you sneak in from the side, the fly leans in the opposite direction. This __ticketing/positioning__ then lets the fly spring into a flight pattern that takes it out of the danger zone. So, if you want to get a fly on the first try, Dickinson says to aim at where you think it's going, not where it is. Or you could always call in a SWAT team.</t>
   </si>
   <si>
-    <t>You've probably chased a fly or two around the house this summer. And, chances are, it took a few swings before you brought down the buzzing nuisance. Now a study in the August 28th issue of the journal Current Biology has uncovered just what makes a fly so hard to swat. Michael frontierswomen from the California shrewd of Technology used brightfield digital video to record the evasive maneuvers of fruit flies. In the slow-mo instant replay, the flies' bodies react to a swatter well before their wings carry them to safety. Blessed with nearly 360 degree vision, the fly first gauges the position of the swatter, then mesh an escape within 200 milliseconds. When approached from the front, for example, a fly shifts its middle legs forward and leans back. If you sneak in from the side, the fly leans in the opposite direction. This ticketing then lets the fly spring into a flight pattern that takes it out of the danger zone. So, if you want to get a fly on the first try, Dickinson says to aim at where you think it's going, not where it is. Or you could always call in a SWAT team.</t>
+    <t>You've probably chased a fly or two around the house this summer. And, chances are, it took a few swings before you brought down the buzzing nuisance. Now a study in the August 28th issue of the journal Current Biology has uncovered just what makes a fly so hard to swat. Michael Dickinson from the California Institute of Technology used high-speed digital video to record the evasive maneuvers of fruit flies. In the slow-mo instant replay, the flies' bodies react to a swatter well before their wings carry them to safety. Blessed with nearly 360 degree vision, the fly first gauges the position of the swatter, then prepares an escape within 200 milliseconds. When approached from the front, for example, a fly shifts its middle legs forward and leans back. If you sneak in from the side, the fly leans in the opposite direction. This positioning then lets the fly spring into a flight pattern that takes it out of the danger zone. So, if you want to get a fly on the first try, Dickinson says to aim at where you think it's going, not where it is. Or you could always call in a SWAT team.</t>
   </si>
   <si>
     <t>#116 Romantic Music</t>
@@ -4920,7 +4920,7 @@
     <t>Have you been having trouble getting some digits lately when you ask a girl out? Maybe you should check what music is playing. That's what French __cancellous/psychologists__ found. They __tutted/published__ their __had/research__ in the journal __suddenly/Psychology__ of Music. First the researchers found a guy who was rated average looking by a group of women. Then that average Antoine talked about a couple of food products with 87 __inveterate/different__ women, aged 18 to 20. But before the conversation, half the women heard this __lymphatic/romantic__ French tune: Je L'aime a Mourir. The other half heard this song that most in France agree is neutral: "L'heure du Thé," or "Tea Time". After talking, Antoine pulled each one aside and asked for her phone number. Only 28 percent of the women who heard the tea song gave out their info. But 52 percent of the women who listened to the love song said yes. So maybe, guys, you should wait for a romantic tune before making your move. Unfortunately, they didn't test the alternate: What type of music is more likely to get a guy to say yes?</t>
   </si>
   <si>
-    <t>Have you been having trouble getting some digits lately when you ask a girl out? Maybe you should check what music is playing. That's what French cancellous found. They tutted their had in the journal suddenly of Music. First the researchers found a guy who was rated average looking by a group of women. Then that average Antoine talked about a couple of food products with 87 inveterate women, aged 18 to 20. But before the conversation, half the women heard this lymphatic French tune: Je L'aime a Mourir. The other half heard this song that most in France agree is neutral: "L'heure du Thé," or "Tea Time". After talking, Antoine pulled each one aside and asked for her phone number. Only 28 percent of the women who heard the tea song gave out their info. But 52 percent of the women who listened to the love song said yes. So maybe, guys, you should wait for a romantic tune before making your move. Unfortunately, they didn't test the alternate: What type of music is more likely to get a guy to say yes?</t>
+    <t>Have you been having trouble getting some digits lately when you ask a girl out? Maybe you should check what music is playing. That's what French psychologists found. They published their research in the journal Psychology of Music. First the researchers found a guy who was rated average looking by a group of women. Then that average Antoine talked about a couple of food products with 87 different women, aged 18 to 20. But before the conversation, half the women heard this romantic French tune: Je L'aime a Mourir. The other half heard this song that most in France agree is neutral: "L'heure du Thé," or "Tea Time". After talking, Antoine pulled each one aside and asked for her phone number. Only 28 percent of the women who heard the tea song gave out their info. But 52 percent of the women who listened to the love song said yes. So maybe, guys, you should wait for a romantic tune before making your move. Unfortunately, they didn't test the alternate: What type of music is more likely to get a guy to say yes?</t>
   </si>
   <si>
     <t>#117 Longevity Diets</t>
@@ -4929,7 +4929,7 @@
     <t>Sometimes it's not what you eat, but when you eat it. At least when it comes to longevity diets. For some time, __wirelesses/scientists__ have known that animals kept on a strict diet live longer than their well-fed peers. But this Methuselah meal plan is no ordinary __contrive/just-say-no-to-that-second-slice__ of pie kind of diet. To reap the __rebelling/life-extending__ benefits, some of these animals cut their calorie consumption in half. Such a diet might be do-able for captive mice and monkeys, but it would be a tough sell for people. Then, five years ago, studies in mice suggested that __illicit/intermittent__ fasting would work just as well. These mice abstained from eating every other day, and lived longer then their gluttonous comrades—without really skimping on the total __pathologies/calories__ they consumed. Now, scientists at Kyoto University have found the same thing in worms that fasted every third day. And they found a gene that regulates the effect, results reported in the journal Nature. Like the mice, these fasting worms did not cut their total calorie intake. But they boosted their lifespan by 50 percent, and showed fewer signs of __critical/physical__ decline than their peers. So go ahead, enjoy that extra slice of pie. Because tomorrow's another day. To not eat.</t>
   </si>
   <si>
-    <t>Sometimes it's not what you eat, but when you eat it. At least when it comes to longevity diets. For some time, wirelesses have known that animals kept on a strict diet live longer than their well-fed peers. But this Methuselah meal plan is no ordinary contrive of pie kind of diet. To reap the rebelling benefits, some of these animals cut their calorie consumption in half. Such a diet might be do-able for captive mice and monkeys, but it would be a tough sell for people. Then, five years ago, studies in mice suggested that illicit fasting would work just as well. These mice abstained from eating every other day, and lived longer then their gluttonous comrades—without really skimping on the total pathologies they consumed. Now, scientists at Kyoto University have found the same thing in worms that fasted every third day. And they found a gene that regulates the effect, results reported in the journal Nature. Like the mice, these fasting worms did not cut their total calorie intake. But they boosted their lifespan by 50 percent, and showed fewer signs of critical decline than their peers. So go ahead, enjoy that extra slice of pie. Because tomorrow's another day. To not eat.</t>
+    <t>Sometimes it's not what you eat, but when you eat it. At least when it comes to longevity diets. For some time, scientists have known that animals kept on a strict diet live longer than their well-fed peers. But this Methuselah meal plan is no ordinary just-say-no-to-that-second-slice of pie kind of diet. To reap the life-extending benefits, some of these animals cut their calorie consumption in half. Such a diet might be do-able for captive mice and monkeys, but it would be a tough sell for people. Then, five years ago, studies in mice suggested that intermittent fasting would work just as well. These mice abstained from eating every other day, and lived longer then their gluttonous comrades—without really skimping on the total calories they consumed. Now, scientists at Kyoto University have found the same thing in worms that fasted every third day. And they found a gene that regulates the effect, results reported in the journal Nature. Like the mice, these fasting worms did not cut their total calorie intake. But they boosted their lifespan by 50 percent, and showed fewer signs of physical decline than their peers. So go ahead, enjoy that extra slice of pie. Because tomorrow's another day. To not eat.</t>
   </si>
   <si>
     <t>#118 Good Workout</t>
@@ -4938,7 +4938,7 @@
     <t>We've all heard exercise is good for your physical and mental well-being. But a good workout can actually influence the mental well-being of others, too. Because bosses who hit the gym tend to be less abusive to their employees. That's according to a study in the Journal of __Spindles/Business__ and Psychology. __Fieldworkers/Researchers__ asked 98 MBA __useless/students__ who were also employed full-time to rate how their supervisors treated them, by __attracting/responding__ to statements like "my boss puts me down in front of others." The researchers also had supervisors fill out a __timpanist/different__ survey, about their stress levels and weekly exercise. And, as the authors expected, the more stressed-out supervisors were, the more their employees felt belittled by them. But the employees felt better about bosses who exercised, whether it was yoga, cardio or weight lifting. And just one or two days a week did the trick. Exercise didn't simply melt away the stress—bosses who worked out reported feeling just as much __agenda/pressure__ as their sedentary counterparts. Active bosses just spared subordinates the verbal attacks. So next time you feel like telling your boss to take a hike, it might actually be sound advice!</t>
   </si>
   <si>
-    <t>We've all heard exercise is good for your physical and mental well-being. But a good workout can actually influence the mental well-being of others, too. Because bosses who hit the gym tend to be less abusive to their employees. That's according to a study in the Journal of Spindles and Psychology. Fieldworkers asked 98 MBA useless who were also employed full-time to rate how their supervisors treated them, by attracting to statements like "my boss puts me down in front of others." The researchers also had supervisors fill out a timpanist survey, about their stress levels and weekly exercise. And, as the authors expected, the more stressed-out supervisors were, the more their employees felt belittled by them. But the employees felt better about bosses who exercised, whether it was yoga, cardio or weight lifting. And just one or two days a week did the trick. Exercise didn't simply melt away the stress—bosses who worked out reported feeling just as much agenda as their sedentary counterparts. Active bosses just spared subordinates the verbal attacks. So next time you feel like telling your boss to take a hike, it might actually be sound advice!</t>
+    <t>We've all heard exercise is good for your physical and mental well-being. But a good workout can actually influence the mental well-being of others, too. Because bosses who hit the gym tend to be less abusive to their employees. That's according to a study in the Journal of Business and Psychology. Researchers asked 98 MBA students who were also employed full-time to rate how their supervisors treated them, by responding to statements like "my boss puts me down in front of others." The researchers also had supervisors fill out a different survey, about their stress levels and weekly exercise. And, as the authors expected, the more stressed-out supervisors were, the more their employees felt belittled by them. But the employees felt better about bosses who exercised, whether it was yoga, cardio or weight lifting. And just one or two days a week did the trick. Exercise didn't simply melt away the stress—bosses who worked out reported feeling just as much pressure as their sedentary counterparts. Active bosses just spared subordinates the verbal attacks. So next time you feel like telling your boss to take a hike, it might actually be sound advice!</t>
   </si>
   <si>
     <t>#119 Cats</t>
@@ -4947,7 +4947,7 @@
     <t>Lions roaming the savannah are a staple of nature documentaries. But the millions of little lions that live in our homes and __dotes/neighborhoods__ also lead fascinating lives. We know more about those lives now, because a two-year-long study used __millions/radio-transmitters__ to track cats at the __dampen/southern__ edge of the cities of Champaign and Urbana in Illinois. It would have taken a dozen field researchers to collect the same data. The study is in the Journal of Wildlife Management. The entire kittie cohort included both housecats and feral cats, and ranged over almost 6,300 acres. One feral cat's range topped out at 1,351 acres. New York's Central Park covers 843 acres. Owned cats with homes roamed way less than their feral counterparts. But they still __refracted/averaged__ a range of just under five acres. The pets were highly active just 3 percent of the time, compared with 14 percent for the cats that need to find their own food. The work should shed light on protecting species that the cats hunt, and inform the efforts to stop the spread of feline __disables/contagious__ diseases.</t>
   </si>
   <si>
-    <t>Lions roaming the savannah are a staple of nature documentaries. But the millions of little lions that live in our homes and dotes also lead fascinating lives. We know more about those lives now, because a two-year-long study used millions to track cats at the dampen edge of the cities of Champaign and Urbana in Illinois. It would have taken a dozen field researchers to collect the same data. The study is in the Journal of Wildlife Management. The entire kittie cohort included both housecats and feral cats, and ranged over almost 6,300 acres. One feral cat's range topped out at 1,351 acres. New York's Central Park covers 843 acres. Owned cats with homes roamed way less than their feral counterparts. But they still refracted a range of just under five acres. The pets were highly active just 3 percent of the time, compared with 14 percent for the cats that need to find their own food. The work should shed light on protecting species that the cats hunt, and inform the efforts to stop the spread of feline disables diseases.</t>
+    <t>Lions roaming the savannah are a staple of nature documentaries. But the millions of little lions that live in our homes and neighborhoods also lead fascinating lives. We know more about those lives now, because a two-year-long study used radio-transmitters to track cats at the southern edge of the cities of Champaign and Urbana in Illinois. It would have taken a dozen field researchers to collect the same data. The study is in the Journal of Wildlife Management. The entire kittie cohort included both housecats and feral cats, and ranged over almost 6,300 acres. One feral cat's range topped out at 1,351 acres. New York's Central Park covers 843 acres. Owned cats with homes roamed way less than their feral counterparts. But they still averaged a range of just under five acres. The pets were highly active just 3 percent of the time, compared with 14 percent for the cats that need to find their own food. The work should shed light on protecting species that the cats hunt, and inform the efforts to stop the spread of feline contagious diseases.</t>
   </si>
   <si>
     <t>#120 Early Farming</t>
@@ -4956,7 +4956,7 @@
     <t>Early farming began in the Near East about 10,500 years ago. Farming first reached the Balkans in Europe some 8 to 9,000 years ago, and then crept westward. Locals in Britain, __adumbrated/separated__ from the __spectated/mainland__ by the relatively newly formed English Channel, did not start farming until about 6,000 years ago. But an __slothfulness/analysis__ of sediment from a submerged British archaeological site called __reconquer/Bouldner__ Cliff found something unexpected. "Amongst our Bouldner Cliff samples we found ancient DNA evidence of wheat at the site, which was not seen in mainland Britain for another 2,000 years." Robin Allaby of the __partially/University__ of Warwick. "However, wheat was already being grown in southern Europe. This is incredibly __respiring/exciting__ because it means Bouldner's inhabitants were not as isolated as __expediently/previously__ thought. In fact, they were in touch, one way or another, with more advanced Neolithic farming communities in southern Europe." The work by Allaby and colleagues is in the journal Science. The researchers showed that the wheat remains are genetically more similar to Near Eastern domesticated wheat than to local distant cousins. And they found no evidence of pollen—meaning that the wheat was almost certainly imported. In an accompanying Perspectives piece in the journal, archaeologist Greger Larsen of Durham University writes that the findings show that DNA analysis can help scientists tease out details about the historical movement of plant and animal species.</t>
   </si>
   <si>
-    <t>Early farming began in the Near East about 10,500 years ago. Farming first reached the Balkans in Europe some 8 to 9,000 years ago, and then crept westward. Locals in Britain, adumbrated from the spectated by the relatively newly formed English Channel, did not start farming until about 6,000 years ago. But an slothfulness of sediment from a submerged British archaeological site called reconquer Cliff found something unexpected. "Amongst our Bouldner Cliff samples we found ancient DNA evidence of wheat at the site, which was not seen in mainland Britain for another 2,000 years." Robin Allaby of the partially of Warwick. "However, wheat was already being grown in southern Europe. This is incredibly respiring because it means Bouldner's inhabitants were not as isolated as expediently thought. In fact, they were in touch, one way or another, with more advanced Neolithic farming communities in southern Europe." The work by Allaby and colleagues is in the journal Science. The researchers showed that the wheat remains are genetically more similar to Near Eastern domesticated wheat than to local distant cousins. And they found no evidence of pollen—meaning that the wheat was almost certainly imported. In an accompanying Perspectives piece in the journal, archaeologist Greger Larsen of Durham University writes that the findings show that DNA analysis can help scientists tease out details about the historical movement of plant and animal species.</t>
+    <t>Early farming began in the Near East about 10,500 years ago. Farming first reached the Balkans in Europe some 8 to 9,000 years ago, and then crept westward. Locals in Britain, separated from the mainland by the relatively newly formed English Channel, did not start farming until about 6,000 years ago. But an analysis of sediment from a submerged British archaeological site called Bouldner Cliff found something unexpected. "Amongst our Bouldner Cliff samples we found ancient DNA evidence of wheat at the site, which was not seen in mainland Britain for another 2,000 years." Robin Allaby of the University of Warwick. "However, wheat was already being grown in southern Europe. This is incredibly exciting because it means Bouldner's inhabitants were not as isolated as previously thought. In fact, they were in touch, one way or another, with more advanced Neolithic farming communities in southern Europe." The work by Allaby and colleagues is in the journal Science. The researchers showed that the wheat remains are genetically more similar to Near Eastern domesticated wheat than to local distant cousins. And they found no evidence of pollen—meaning that the wheat was almost certainly imported. In an accompanying Perspectives piece in the journal, archaeologist Greger Larsen of Durham University writes that the findings show that DNA analysis can help scientists tease out details about the historical movement of plant and animal species.</t>
   </si>
   <si>
     <t>#121 Sex of Lizard</t>
@@ -4965,7 +4965,7 @@
     <t>When it comes to lizard sex, size does matter. But not in the way you might think. Because in the June 4th online issue of the journal Current Biology, __hyperlinks/scientists__ say that for at least one type of lizard, larger eggs are more likely to make girls while smaller eggs yield boys. For many animals, the sex of an individual is dictated solely by its chromosomes. But for small alpine lizards, gender isn't so cut-and-dried. The scientists had earlier found that nest temperature can __continuous/influence__ the sex of lizard hatchlings. Cooler nests turn out more boys—no matter what their __records/chromosomes__ say. At the same time, the researchers noticed that larger eggs seemed to make more daughters. But they wanted to put their observation to the test. So they took big eggs and removed some yolk—and, voila, they made males. Adding yolk to a little egg was a recipe for a female. This egg size __revelation/manipulation__ might allow moms to balance their babies' sexes when a chilly nest would __ascribes/otherwise__ produce mostly sons. Because when it comes to alpine lizards, sex __verification/determination__ all comes down to a practical yolk.</t>
   </si>
   <si>
-    <t>When it comes to lizard sex, size does matter. But not in the way you might think. Because in the June 4th online issue of the journal Current Biology, hyperlinks say that for at least one type of lizard, larger eggs are more likely to make girls while smaller eggs yield boys. For many animals, the sex of an individual is dictated solely by its chromosomes. But for small alpine lizards, gender isn't so cut-and-dried. The scientists had earlier found that nest temperature can continuous the sex of lizard hatchlings. Cooler nests turn out more boys—no matter what their records say. At the same time, the researchers noticed that larger eggs seemed to make more daughters. But they wanted to put their observation to the test. So they took big eggs and removed some yolk—and, voila, they made males. Adding yolk to a little egg was a recipe for a female. This egg size revelation might allow moms to balance their babies' sexes when a chilly nest would ascribes produce mostly sons. Because when it comes to alpine lizards, sex verification all comes down to a practical yolk.</t>
+    <t>When it comes to lizard sex, size does matter. But not in the way you might think. Because in the June 4th online issue of the journal Current Biology, scientists say that for at least one type of lizard, larger eggs are more likely to make girls while smaller eggs yield boys. For many animals, the sex of an individual is dictated solely by its chromosomes. But for small alpine lizards, gender isn't so cut-and-dried. The scientists had earlier found that nest temperature can influence the sex of lizard hatchlings. Cooler nests turn out more boys—no matter what their chromosomes say. At the same time, the researchers noticed that larger eggs seemed to make more daughters. But they wanted to put their observation to the test. So they took big eggs and removed some yolk—and, voila, they made males. Adding yolk to a little egg was a recipe for a female. This egg size manipulation might allow moms to balance their babies' sexes when a chilly nest would otherwise produce mostly sons. Because when it comes to alpine lizards, sex determination all comes down to a practical yolk.</t>
   </si>
   <si>
     <t>#122 Tree Frog</t>
@@ -4974,7 +4974,7 @@
     <t>The eastern grey tree frog (sound) looks exactly like the closely related Cope's grey tree frog (sound). The big difference between the two species is beneath the surface—the eastern has twice the number of __moans/chromosomes__ as does the Cope's. Having more sets of chromosomes makes the cells of the eastern frog larger than the cells found in the Cope's. And those bigger cells makes the eastern's song just a little deeper. Now University of Missouri __recenter/researcher__ Carl Gerhardt and his student Mitch Tucker have determined that the slight difference in the calls—here's the eastern again and here's the Cope's (sound)—is how the females know which species' males to buddy up with: the ones with the same __trombone/chromosome__ number that they have. The work is in the __elitists/Proceedings__ of the Royal Society B-Biological Sciences. __separation/Speciation__ is often caused by a geographic barrier that keeps populations from mating. But the tree frog situation may be a rare case in which chromosome duplication, and its __firmament/subsequent__ effects, presented a __meninx/reproductive__ barrier. As in humans, it comes down to whether he calls.</t>
   </si>
   <si>
-    <t>The eastern grey tree frog (sound) looks exactly like the closely related Cope's grey tree frog (sound). The big difference between the two species is beneath the surface—the eastern has twice the number of moans as does the Cope's. Having more sets of chromosomes makes the cells of the eastern frog larger than the cells found in the Cope's. And those bigger cells makes the eastern's song just a little deeper. Now University of Missouri recenter Carl Gerhardt and his student Mitch Tucker have determined that the slight difference in the calls—here's the eastern again and here's the Cope's (sound)—is how the females know which species' males to buddy up with: the ones with the same trombone number that they have. The work is in the elitists of the Royal Society B-Biological Sciences. separation is often caused by a geographic barrier that keeps populations from mating. But the tree frog situation may be a rare case in which chromosome duplication, and its firmament effects, presented a meninx barrier. As in humans, it comes down to whether he calls.</t>
+    <t>The eastern grey tree frog (sound) looks exactly like the closely related Cope's grey tree frog (sound). The big difference between the two species is beneath the surface—the eastern has twice the number of chromosomes as does the Cope's. Having more sets of chromosomes makes the cells of the eastern frog larger than the cells found in the Cope's. And those bigger cells makes the eastern's song just a little deeper. Now University of Missouri researcher Carl Gerhardt and his student Mitch Tucker have determined that the slight difference in the calls—here's the eastern again and here's the Cope's (sound)—is how the females know which species' males to buddy up with: the ones with the same chromosome number that they have. The work is in the Proceedings of the Royal Society B-Biological Sciences. Speciation is often caused by a geographic barrier that keeps populations from mating. But the tree frog situation may be a rare case in which chromosome duplication, and its subsequent effects, presented a reproductive barrier. As in humans, it comes down to whether he calls.</t>
   </si>
   <si>
     <t>#123 Migration</t>
@@ -4983,7 +4983,7 @@
     <t>Want to know the route humans took when they first migrated from Africa into Europe? Seems that they might have marked the path. Not like Hansel and Gretel, who __valiantly/consciously__ left bread crumbs. Ancient humans ate as they trekked. And they appear to have chucked aside the packaging for some of their slimy sustenance: snails. Conventional wisdom has been that humans initially __unbalanced/traveled__ from Africa to the Near East, then up around the Mediterranean through Lebanon before heading into Europe some 40 to 50,000 years ago. But recently, some __tiredness/scientists__ have theorized that humans made it to Europe first and then headed east. Now there's more support for the old view that humans traveled through the Levant on the way to Europe-in the form of the shells of edible marine snails. The study is in the Proceedings of the National Academy of Sciences. Researchers evaluated shells from an __corruptible/archaeological__ site dated to the Upper __thrombolytic/Paleolithic__ in Lebanon. The shells were mostly intact, except the tapered pointy tip had been removed—most likely for easier access to the meat inside. The scientists calculated the age of the shells via a variety of methods. And they found that the snails dated back almost 46,000 years. The earliest __incidents/evidence__ of modern human remains in Europe seem to be no more than 45,000 years old. The snail evidence thus adds weight to the hypothesis that ancient people passed through the Levant on their way to Europe. And not at a snail's pace, either.</t>
   </si>
   <si>
-    <t>Want to know the route humans took when they first migrated from Africa into Europe? Seems that they might have marked the path. Not like Hansel and Gretel, who valiantly left bread crumbs. Ancient humans ate as they trekked. And they appear to have chucked aside the packaging for some of their slimy sustenance: snails. Conventional wisdom has been that humans initially unbalanced from Africa to the Near East, then up around the Mediterranean through Lebanon before heading into Europe some 40 to 50,000 years ago. But recently, some tiredness have theorized that humans made it to Europe first and then headed east. Now there's more support for the old view that humans traveled through the Levant on the way to Europe-in the form of the shells of edible marine snails. The study is in the Proceedings of the National Academy of Sciences. Researchers evaluated shells from an corruptible site dated to the Upper thrombolytic in Lebanon. The shells were mostly intact, except the tapered pointy tip had been removed—most likely for easier access to the meat inside. The scientists calculated the age of the shells via a variety of methods. And they found that the snails dated back almost 46,000 years. The earliest incidents of modern human remains in Europe seem to be no more than 45,000 years old. The snail evidence thus adds weight to the hypothesis that ancient people passed through the Levant on their way to Europe. And not at a snail's pace, either.</t>
+    <t>Want to know the route humans took when they first migrated from Africa into Europe? Seems that they might have marked the path. Not like Hansel and Gretel, who consciously left bread crumbs. Ancient humans ate as they trekked. And they appear to have chucked aside the packaging for some of their slimy sustenance: snails. Conventional wisdom has been that humans initially traveled from Africa to the Near East, then up around the Mediterranean through Lebanon before heading into Europe some 40 to 50,000 years ago. But recently, some scientists have theorized that humans made it to Europe first and then headed east. Now there's more support for the old view that humans traveled through the Levant on the way to Europe-in the form of the shells of edible marine snails. The study is in the Proceedings of the National Academy of Sciences. Researchers evaluated shells from an archaeological site dated to the Upper Paleolithic in Lebanon. The shells were mostly intact, except the tapered pointy tip had been removed—most likely for easier access to the meat inside. The scientists calculated the age of the shells via a variety of methods. And they found that the snails dated back almost 46,000 years. The earliest evidence of modern human remains in Europe seem to be no more than 45,000 years old. The snail evidence thus adds weight to the hypothesis that ancient people passed through the Levant on their way to Europe. And not at a snail's pace, either.</t>
   </si>
   <si>
     <t>#124 G.M.</t>
@@ -4992,7 +4992,7 @@
     <t>One of the __girth/concerns__ about working with genetically __beside/modified__ crops has been that vegetation growing in agricultural fields might escape out into the world. Now, for the first time in the U.S., researchers report a large population of GM crops beyond the farm. Transgenic canola plants in North Dakota had __pedigreed/received__ genes making them resistant to herbicides, such as the weed killer Roundup. Researchers collected and tested 406 canola plants along thousands of miles of state roads. They found 347 carrying at least one resistance gene. There were also indications that the inserted genes were being passed on to new generations, producing some plants in the wild with multiple transgenes. The findings were presented on August 6th at the annual meeting of the __archeological/Ecological__ Society of America in Pittsburgh. The __pinprick/transgenic__ canola plants are not about to take over the world. But researchers are __industriously/obviously__ curious about how these particular plants managed to make it in places like the edges of parking lots rather than pampered fields. Any answers they find will likely affect future biotechnology regulation.</t>
   </si>
   <si>
-    <t>One of the girth about working with genetically beside crops has been that vegetation growing in agricultural fields might escape out into the world. Now, for the first time in the U.S., researchers report a large population of GM crops beyond the farm. Transgenic canola plants in North Dakota had pedigreed genes making them resistant to herbicides, such as the weed killer Roundup. Researchers collected and tested 406 canola plants along thousands of miles of state roads. They found 347 carrying at least one resistance gene. There were also indications that the inserted genes were being passed on to new generations, producing some plants in the wild with multiple transgenes. The findings were presented on August 6th at the annual meeting of the archeological Society of America in Pittsburgh. The pinprick canola plants are not about to take over the world. But researchers are industriously curious about how these particular plants managed to make it in places like the edges of parking lots rather than pampered fields. Any answers they find will likely affect future biotechnology regulation.</t>
+    <t>One of the concerns about working with genetically modified crops has been that vegetation growing in agricultural fields might escape out into the world. Now, for the first time in the U.S., researchers report a large population of GM crops beyond the farm. Transgenic canola plants in North Dakota had received genes making them resistant to herbicides, such as the weed killer Roundup. Researchers collected and tested 406 canola plants along thousands of miles of state roads. They found 347 carrying at least one resistance gene. There were also indications that the inserted genes were being passed on to new generations, producing some plants in the wild with multiple transgenes. The findings were presented on August 6th at the annual meeting of the Ecological Society of America in Pittsburgh. The transgenic canola plants are not about to take over the world. But researchers are obviously curious about how these particular plants managed to make it in places like the edges of parking lots rather than pampered fields. Any answers they find will likely affect future biotechnology regulation.</t>
   </si>
   <si>
     <t>#125 Early Ocean</t>
@@ -5001,7 +5001,7 @@
     <t>The early Earth's oceans were home to a lot of interesting chemistry. Now scientists have found that amino acids thought to be present way back when could have been cooked into other compounds vital for life—an idea you should take with a grain of salt. Four billion years ago, the planet was probably covered by a salty ocean, dotted with volcanic islands and short lived continents. German researchers recently mimicked some of the chemistry taking place along the coasts of the volcanic islands. They created an approximation of primordial seawater. Then they evaporated it, to simulate what went on at those volcanic coasts. They baked the residue, __formulating/creating__ salt crusts. At those high temperatures, amino acids interacted with metal ions in the salt crusts and were converted into other __format/important__ __dynamical/biological__ molecules, such as pyrroles—which are part of the structures of chlorophyll in plants and hemoglobin in animals. The scientists __neglected/presented__ their findings September 17th at the European Planetary Science Conference in Potsdam. Over __hammers/hundreds__ of __prowlers/thousands__ of years, these novel compounds could have built up along the volcanic coasts, creating materials for the first living cells. Which were really worth their salt.</t>
   </si>
   <si>
-    <t>The early Earth's oceans were home to a lot of interesting chemistry. Now scientists have found that amino acids thought to be present way back when could have been cooked into other compounds vital for life—an idea you should take with a grain of salt. Four billion years ago, the planet was probably covered by a salty ocean, dotted with volcanic islands and short lived continents. German researchers recently mimicked some of the chemistry taking place along the coasts of the volcanic islands. They created an approximation of primordial seawater. Then they evaporated it, to simulate what went on at those volcanic coasts. They baked the residue, formulating salt crusts. At those high temperatures, amino acids interacted with metal ions in the salt crusts and were converted into other format dynamical molecules, such as pyrroles—which are part of the structures of chlorophyll in plants and hemoglobin in animals. The scientists neglected their findings September 17th at the European Planetary Science Conference in Potsdam. Over hammers of prowlers of years, these novel compounds could have built up along the volcanic coasts, creating materials for the first living cells. Which were really worth their salt.</t>
+    <t>The early Earth's oceans were home to a lot of interesting chemistry. Now scientists have found that amino acids thought to be present way back when could have been cooked into other compounds vital for life—an idea you should take with a grain of salt. Four billion years ago, the planet was probably covered by a salty ocean, dotted with volcanic islands and short lived continents. German researchers recently mimicked some of the chemistry taking place along the coasts of the volcanic islands. They created an approximation of primordial seawater. Then they evaporated it, to simulate what went on at those volcanic coasts. They baked the residue, creating salt crusts. At those high temperatures, amino acids interacted with metal ions in the salt crusts and were converted into other important biological molecules, such as pyrroles—which are part of the structures of chlorophyll in plants and hemoglobin in animals. The scientists presented their findings September 17th at the European Planetary Science Conference in Potsdam. Over hundreds of thousands of years, these novel compounds could have built up along the volcanic coasts, creating materials for the first living cells. Which were really worth their salt.</t>
   </si>
   <si>
     <t>#126 Gun Control</t>
@@ -5010,7 +5010,7 @@
     <t>Here's an impassioned plea for gun control. Of nail guns, that is. Because accidents involving nail guns have gone through the renovated roof. In 2005, almost 15,000 people were treated in US emergency rooms for nail gun injuries. That's twice the number in 2001 and three times the __chesterfields/injuries__ back in 1991, according to data released in the April 13th issue of Morbidity and Mortality Weekly Report, put out by the CDC. The rising __minstrelsy/popularity__ of do it yourselfing seems to be behind the unfortunate trend. Most injuries are puncture wounds to the hands, followed by hits to the forearms, legs and feet. Six percent of the wounded wind up being hospitalized. Although better safety instruction would no doubt help, the report's authors suggest a systems __remould/approach__ to the problem—they'd like nail guns to be __panhandle/impossible__ to fire until the nose was depressed, which would __foolery/presumably__ happen only when the gun was flush up against whatever needed nailing. By the way, 96 percent of the injured were males, which could mean that they're doing most of the work, or that women read the instructions.</t>
   </si>
   <si>
-    <t>Here's an impassioned plea for gun control. Of nail guns, that is. Because accidents involving nail guns have gone through the renovated roof. In 2005, almost 15,000 people were treated in US emergency rooms for nail gun injuries. That's twice the number in 2001 and three times the chesterfields back in 1991, according to data released in the April 13th issue of Morbidity and Mortality Weekly Report, put out by the CDC. The rising minstrelsy of do it yourselfing seems to be behind the unfortunate trend. Most injuries are puncture wounds to the hands, followed by hits to the forearms, legs and feet. Six percent of the wounded wind up being hospitalized. Although better safety instruction would no doubt help, the report's authors suggest a systems remould to the problem—they'd like nail guns to be panhandle to fire until the nose was depressed, which would foolery happen only when the gun was flush up against whatever needed nailing. By the way, 96 percent of the injured were males, which could mean that they're doing most of the work, or that women read the instructions.</t>
+    <t>Here's an impassioned plea for gun control. Of nail guns, that is. Because accidents involving nail guns have gone through the renovated roof. In 2005, almost 15,000 people were treated in US emergency rooms for nail gun injuries. That's twice the number in 2001 and three times the injuries back in 1991, according to data released in the April 13th issue of Morbidity and Mortality Weekly Report, put out by the CDC. The rising popularity of do it yourselfing seems to be behind the unfortunate trend. Most injuries are puncture wounds to the hands, followed by hits to the forearms, legs and feet. Six percent of the wounded wind up being hospitalized. Although better safety instruction would no doubt help, the report's authors suggest a systems approach to the problem—they'd like nail guns to be impossible to fire until the nose was depressed, which would presumably happen only when the gun was flush up against whatever needed nailing. By the way, 96 percent of the injured were males, which could mean that they're doing most of the work, or that women read the instructions.</t>
   </si>
   <si>
     <t>#127 Antibiotics</t>
@@ -5019,7 +5019,7 @@
     <t>The pain-relieving effects of drugs like ibuprofen are well known. But ibuprofen and its relatives, known as nonsteroidal __coli/anti-inflammatory__ drugs, may someday have another use—as antibiotics. Researchers tested three anti-inflammatory drugs: bromfenac, used in eye drops, and carprofen and vedaprofen, both for treating __dresses/conditions__ like arthritis in dogs. The investigators found that all three drugs bind to something called the "DNA clamp" in bacteria. That clamp is __sickle/essential__ to repairing and replicating DNA. By jamming it, the painkillers can __advocacy/actually__ kill live E. coli—in a test tube, at least. The findings appear in the journal __heresy/Chemistry__ Biology. Study author Aaron Oakley, of Australia's University of Wollongong, says we still need __finagle/clinical__ trials to tell if this trick holds true in humans. But this study is a first step. "I guess it alerts a lot of clinicians to the fact that some of the nonsteroidal anti-inflammatories that they're using may have this off-target effect." And it gives drug developers—like Oakley and his colleagues—a whole new way to attack antibiotic-resistant bacteria.</t>
   </si>
   <si>
-    <t>The pain-relieving effects of drugs like ibuprofen are well known. But ibuprofen and its relatives, known as nonsteroidal coli drugs, may someday have another use—as antibiotics. Researchers tested three anti-inflammatory drugs: bromfenac, used in eye drops, and carprofen and vedaprofen, both for treating dresses like arthritis in dogs. The investigators found that all three drugs bind to something called the "DNA clamp" in bacteria. That clamp is sickle to repairing and replicating DNA. By jamming it, the painkillers can advocacy kill live E. coli—in a test tube, at least. The findings appear in the journal heresy Biology. Study author Aaron Oakley, of Australia's University of Wollongong, says we still need finagle trials to tell if this trick holds true in humans. But this study is a first step. "I guess it alerts a lot of clinicians to the fact that some of the nonsteroidal anti-inflammatories that they're using may have this off-target effect." And it gives drug developers—like Oakley and his colleagues—a whole new way to attack antibiotic-resistant bacteria.</t>
+    <t>The pain-relieving effects of drugs like ibuprofen are well known. But ibuprofen and its relatives, known as nonsteroidal anti-inflammatory drugs, may someday have another use—as antibiotics. Researchers tested three anti-inflammatory drugs: bromfenac, used in eye drops, and carprofen and vedaprofen, both for treating conditions like arthritis in dogs. The investigators found that all three drugs bind to something called the "DNA clamp" in bacteria. That clamp is essential to repairing and replicating DNA. By jamming it, the painkillers can actually kill live E. coli—in a test tube, at least. The findings appear in the journal Chemistry Biology. Study author Aaron Oakley, of Australia's University of Wollongong, says we still need clinical trials to tell if this trick holds true in humans. But this study is a first step. "I guess it alerts a lot of clinicians to the fact that some of the nonsteroidal anti-inflammatories that they're using may have this off-target effect." And it gives drug developers—like Oakley and his colleagues—a whole new way to attack antibiotic-resistant bacteria.</t>
   </si>
   <si>
     <t>#128 Superstition</t>
@@ -5028,7 +5028,7 @@
     <t>Breaking a mirror means seven years bad luck. So does spilling salt or meeting a black cat. We've all heard such silly-sounding superstitions. Of course why anybody would believe that stepping on a crack could break your mother's back is a mystery. But according to an article in the Royal Society journal Biological Sciences, __interference/superstitious__ behaviors are a natural product of evolution. Imagine an animal living in an environment where, over the course of a day, he might hear some rustling in the leaves or maybe in the grass. Now, movements in the grass could signal a __pensioner/predator__ attack, whereas the breeze in the trees is __geodesy/probably__ just the wind. Still, the animal has a choice: he can ignore all this rustling and go about his business, or he can run and hide. The most logical response would be to hide only when he hears the grass move. But what if it's hard to tell whether the noise came from the grass or the trees? "I could've sworn that was the trees" could be his final thought. So the animal learns to bolt at the sound of the breeze, because it could foretell certain doom. That better-safe-than-sorry attitude is essentially a superstition. One that that cautious critter will likely pass on to his young. Knock on wood.</t>
   </si>
   <si>
-    <t>Breaking a mirror means seven years bad luck. So does spilling salt or meeting a black cat. We've all heard such silly-sounding superstitions. Of course why anybody would believe that stepping on a crack could break your mother's back is a mystery. But according to an article in the Royal Society journal Biological Sciences, interference behaviors are a natural product of evolution. Imagine an animal living in an environment where, over the course of a day, he might hear some rustling in the leaves or maybe in the grass. Now, movements in the grass could signal a pensioner attack, whereas the breeze in the trees is geodesy just the wind. Still, the animal has a choice: he can ignore all this rustling and go about his business, or he can run and hide. The most logical response would be to hide only when he hears the grass move. But what if it's hard to tell whether the noise came from the grass or the trees? "I could've sworn that was the trees" could be his final thought. So the animal learns to bolt at the sound of the breeze, because it could foretell certain doom. That better-safe-than-sorry attitude is essentially a superstition. One that that cautious critter will likely pass on to his young. Knock on wood.</t>
+    <t>Breaking a mirror means seven years bad luck. So does spilling salt or meeting a black cat. We've all heard such silly-sounding superstitions. Of course why anybody would believe that stepping on a crack could break your mother's back is a mystery. But according to an article in the Royal Society journal Biological Sciences, superstitious behaviors are a natural product of evolution. Imagine an animal living in an environment where, over the course of a day, he might hear some rustling in the leaves or maybe in the grass. Now, movements in the grass could signal a predator attack, whereas the breeze in the trees is probably just the wind. Still, the animal has a choice: he can ignore all this rustling and go about his business, or he can run and hide. The most logical response would be to hide only when he hears the grass move. But what if it's hard to tell whether the noise came from the grass or the trees? "I could've sworn that was the trees" could be his final thought. So the animal learns to bolt at the sound of the breeze, because it could foretell certain doom. That better-safe-than-sorry attitude is essentially a superstition. One that that cautious critter will likely pass on to his young. Knock on wood.</t>
   </si>
   <si>
     <t>#129 BioBonanza</t>
@@ -5037,7 +5037,7 @@
     <t>BioBonanza is a one-day-open-house festival. All of the researchers in the Department of Biology are going to be showcasing their research so __scholars/students__ can come and see research, interact with the researchers. And we want people to be able to interact and have fun of this event. As soon as you walk in the doors, you'll see all sorts of activities, __images/displays__ of how a human heart works. We'll have __segments/sections__ of spinal cord and brain. You'll get to be able to see __moths/butterflies__ and all sorts of insects. You'll be able to try to catch some local insects and we'll have activities like __wandering/walking__ through local plant gardens and seeing how photosynthesis work.</t>
   </si>
   <si>
-    <t>BioBonanza is a one-day-open-house festival. All of the researchers in the Department of Biology are going to be showcasing their research so scholars can come and see research, interact with the researchers. And we want people to be able to interact and have fun of this event. As soon as you walk in the doors, you'll see all sorts of activities, images of how a human heart works. We'll have segments of spinal cord and brain. You'll get to be able to see moths and all sorts of insects. You'll be able to try to catch some local insects and we'll have activities like wandering through local plant gardens and seeing how photosynthesis work.</t>
+    <t>BioBonanza is a one-day-open-house festival. All of the researchers in the Department of Biology are going to be showcasing their research so students can come and see research, interact with the researchers. And we want people to be able to interact and have fun of this event. As soon as you walk in the doors, you'll see all sorts of activities, displays of how a human heart works. We'll have sections of spinal cord and brain. You'll get to be able to see butterflies and all sorts of insects. You'll be able to try to catch some local insects and we'll have activities like walking through local plant gardens and seeing how photosynthesis work.</t>
   </si>
   <si>
     <t>#130 Salty Food</t>
@@ -5046,7 +5046,7 @@
     <t>Mmmm, chips. One of the most sublime of salty snacks. But have you ever __mansard/wondered__ how they get that perfectly salty sheen on the outside? "Salt is sprayed on the surface." Youngsoo Lee is a food engineer at the University of Illinois Urbana-Champaign. And he says not all salty foods are created equal. There's spray-on surface salt. There's salty liquids, like canned soup. And then there are salty solids, where the sodium is dissolved in a matrixlike structure. Think: salamis and cheeses. But when we eat those salty solids, only a fraction of the salt gets __sleep/released__ before we swallow. Meaning a lot of that salt has no effect on taste—but a big effect on our daily salt intake. Lee's __mitigating/investigating__ that salty-solid conundrum for a company that wants to make cold cuts that taste the same but contain less salt. He couldn't tell me which one. "Um... I mean, it's a fairly big U.S.-based food company." To find a salty solution he and his colleagues created blocks of whey protein with various proportions of fat, water and salt. Then they squashed those tofulike blocks underwater, to measure how much sodium the blocks released. Turns out, the bigger and more numerous the pores within the blocks' protein __planter/structure__ the more salt that was released. The study is in the Journal of Food Science. Lee didn't __intolerantly/actually__ have taste-testers sample different types of pore-filled blocks—that's next. But previous studies have shown that airier, __splotchier/fluffier__ breads do indeed taste saltier to testers. And there's one other trick this study uncovered: solid foods release more of their embedded salt over time. So next time you're about to ask for the salt, why not just spend a little more time chewing instead?</t>
   </si>
   <si>
-    <t>Mmmm, chips. One of the most sublime of salty snacks. But have you ever mansard how they get that perfectly salty sheen on the outside? "Salt is sprayed on the surface." Youngsoo Lee is a food engineer at the University of Illinois Urbana-Champaign. And he says not all salty foods are created equal. There's spray-on surface salt. There's salty liquids, like canned soup. And then there are salty solids, where the sodium is dissolved in a matrixlike structure. Think: salamis and cheeses. But when we eat those salty solids, only a fraction of the salt gets sleep before we swallow. Meaning a lot of that salt has no effect on taste—but a big effect on our daily salt intake. Lee's mitigating that salty-solid conundrum for a company that wants to make cold cuts that taste the same but contain less salt. He couldn't tell me which one. "Um... I mean, it's a fairly big U.S.-based food company." To find a salty solution he and his colleagues created blocks of whey protein with various proportions of fat, water and salt. Then they squashed those tofulike blocks underwater, to measure how much sodium the blocks released. Turns out, the bigger and more numerous the pores within the blocks' protein planter the more salt that was released. The study is in the Journal of Food Science. Lee didn't intolerantly have taste-testers sample different types of pore-filled blocks—that's next. But previous studies have shown that airier, splotchier breads do indeed taste saltier to testers. And there's one other trick this study uncovered: solid foods release more of their embedded salt over time. So next time you're about to ask for the salt, why not just spend a little more time chewing instead?</t>
+    <t>Mmmm, chips. One of the most sublime of salty snacks. But have you ever wondered how they get that perfectly salty sheen on the outside? "Salt is sprayed on the surface." Youngsoo Lee is a food engineer at the University of Illinois Urbana-Champaign. And he says not all salty foods are created equal. There's spray-on surface salt. There's salty liquids, like canned soup. And then there are salty solids, where the sodium is dissolved in a matrixlike structure. Think: salamis and cheeses. But when we eat those salty solids, only a fraction of the salt gets released before we swallow. Meaning a lot of that salt has no effect on taste—but a big effect on our daily salt intake. Lee's investigating that salty-solid conundrum for a company that wants to make cold cuts that taste the same but contain less salt. He couldn't tell me which one. "Um... I mean, it's a fairly big U.S.-based food company." To find a salty solution he and his colleagues created blocks of whey protein with various proportions of fat, water and salt. Then they squashed those tofulike blocks underwater, to measure how much sodium the blocks released. Turns out, the bigger and more numerous the pores within the blocks' protein structure the more salt that was released. The study is in the Journal of Food Science. Lee didn't actually have taste-testers sample different types of pore-filled blocks—that's next. But previous studies have shown that airier, fluffier breads do indeed taste saltier to testers. And there's one other trick this study uncovered: solid foods release more of their embedded salt over time. So next time you're about to ask for the salt, why not just spend a little more time chewing instead?</t>
   </si>
   <si>
     <t>#131 Foliage Color</t>
@@ -5055,7 +5055,7 @@
     <t>In Autumn, New England foliage turns vibrant shades of red, yellow, and orange. Which brings in lots of green—as in the money spent by tourists who flock to the region to witness the explosion of color. Because of fall's economic implications, exactly when the leaf-peeping season will begin is thus a source of constant speculation. Scientists know that factors including frost, heat, rain and drought all affect the timing—but the whole colorful picture is still difficult to accurately predict. Now scientists have picked apart satellite imagery from two New England forest __umbrellas/ecosystems__ collected from 2001 to 2012 to try to get a better handle on exactly what factors __strenuous/influence__ the autumn leaves. The scientists looked at northeastern highlands and coastal zones. They __disseminated/incorporated__ __unsalable/available__ data on chills, frosts and heat, and rain, drought, and flooding. In general, cold, wet and extreme heat made leaves change color sooner, while moderate heat and low rainfall delayed the coloration. But the __omnipotent/different__ ecosystems behaved differently. Forests in the highlands reacted to frosts both in spring and in the fall, while the coast only responded to fall frosts. The coastal region's forests were also particularly sensitive to rain and flooding. Incorporating climate change predictions for the next century, the __receivables/researchers__ propose that the highlands will change color later in the fall, while the coast may start to turn earlier. The study is in the Proceedings of the National Academy of Sciences. The researchers note that more data, such as for extreme weather events and flooding, need to be incorporated into future models. Which could help New England states maximize fall's economic windfall.</t>
   </si>
   <si>
-    <t>In Autumn, New England foliage turns vibrant shades of red, yellow, and orange. Which brings in lots of green—as in the money spent by tourists who flock to the region to witness the explosion of color. Because of fall's economic implications, exactly when the leaf-peeping season will begin is thus a source of constant speculation. Scientists know that factors including frost, heat, rain and drought all affect the timing—but the whole colorful picture is still difficult to accurately predict. Now scientists have picked apart satellite imagery from two New England forest umbrellas collected from 2001 to 2012 to try to get a better handle on exactly what factors strenuous the autumn leaves. The scientists looked at northeastern highlands and coastal zones. They disseminated unsalable data on chills, frosts and heat, and rain, drought, and flooding. In general, cold, wet and extreme heat made leaves change color sooner, while moderate heat and low rainfall delayed the coloration. But the omnipotent ecosystems behaved differently. Forests in the highlands reacted to frosts both in spring and in the fall, while the coast only responded to fall frosts. The coastal region's forests were also particularly sensitive to rain and flooding. Incorporating climate change predictions for the next century, the receivables propose that the highlands will change color later in the fall, while the coast may start to turn earlier. The study is in the Proceedings of the National Academy of Sciences. The researchers note that more data, such as for extreme weather events and flooding, need to be incorporated into future models. Which could help New England states maximize fall's economic windfall.</t>
+    <t>In Autumn, New England foliage turns vibrant shades of red, yellow, and orange. Which brings in lots of green—as in the money spent by tourists who flock to the region to witness the explosion of color. Because of fall's economic implications, exactly when the leaf-peeping season will begin is thus a source of constant speculation. Scientists know that factors including frost, heat, rain and drought all affect the timing—but the whole colorful picture is still difficult to accurately predict. Now scientists have picked apart satellite imagery from two New England forest ecosystems collected from 2001 to 2012 to try to get a better handle on exactly what factors influence the autumn leaves. The scientists looked at northeastern highlands and coastal zones. They incorporated available data on chills, frosts and heat, and rain, drought, and flooding. In general, cold, wet and extreme heat made leaves change color sooner, while moderate heat and low rainfall delayed the coloration. But the different ecosystems behaved differently. Forests in the highlands reacted to frosts both in spring and in the fall, while the coast only responded to fall frosts. The coastal region's forests were also particularly sensitive to rain and flooding. Incorporating climate change predictions for the next century, the researchers propose that the highlands will change color later in the fall, while the coast may start to turn earlier. The study is in the Proceedings of the National Academy of Sciences. The researchers note that more data, such as for extreme weather events and flooding, need to be incorporated into future models. Which could help New England states maximize fall's economic windfall.</t>
   </si>
   <si>
     <t>#132 Botanical Boon</t>
@@ -5064,7 +5064,7 @@
     <t>Global warming might seem like a botanical boon. After all, milder __semiprofessionals/temperatures__ and more carbon dioxide and nitrogen should feed flora. But a __outerwear/ten-year__ study has found that any initial positive effect on plant growth from climate change may soon disappear. The report is in the journal Nature Climate Change. Researchers transplanted vegetation from four grassland __dishes/ecosystems__ to lower, warmer elevations. They also modified the precipitation at the transplant sites based on altered rainfall estimates. For the first year, the plants did great, producing more biomass and churning out more oxygen for us. But their productivity went down for the rest of the decade. What happened? Warming did speed up the nitrogen cycle, which should have increased nitrogen's __impracticability/availability__ as plant fertilizer. But a lot of the nitrogen left the soil through run-off or uptake into the atmosphere. In addition, __muralists/productive__ native plants began to lose out to species that thrive at higher temperatures, but are less productive than the natives. Warmer temperatures may spur immediate growth, but in the long term, we can't expect plants to like it hot.</t>
   </si>
   <si>
-    <t>Global warming might seem like a botanical boon. After all, milder semiprofessionals and more carbon dioxide and nitrogen should feed flora. But a outerwear study has found that any initial positive effect on plant growth from climate change may soon disappear. The report is in the journal Nature Climate Change. Researchers transplanted vegetation from four grassland dishes to lower, warmer elevations. They also modified the precipitation at the transplant sites based on altered rainfall estimates. For the first year, the plants did great, producing more biomass and churning out more oxygen for us. But their productivity went down for the rest of the decade. What happened? Warming did speed up the nitrogen cycle, which should have increased nitrogen's impracticability as plant fertilizer. But a lot of the nitrogen left the soil through run-off or uptake into the atmosphere. In addition, muralists native plants began to lose out to species that thrive at higher temperatures, but are less productive than the natives. Warmer temperatures may spur immediate growth, but in the long term, we can't expect plants to like it hot.</t>
+    <t>Global warming might seem like a botanical boon. After all, milder temperatures and more carbon dioxide and nitrogen should feed flora. But a ten-year study has found that any initial positive effect on plant growth from climate change may soon disappear. The report is in the journal Nature Climate Change. Researchers transplanted vegetation from four grassland ecosystems to lower, warmer elevations. They also modified the precipitation at the transplant sites based on altered rainfall estimates. For the first year, the plants did great, producing more biomass and churning out more oxygen for us. But their productivity went down for the rest of the decade. What happened? Warming did speed up the nitrogen cycle, which should have increased nitrogen's availability as plant fertilizer. But a lot of the nitrogen left the soil through run-off or uptake into the atmosphere. In addition, productive native plants began to lose out to species that thrive at higher temperatures, but are less productive than the natives. Warmer temperatures may spur immediate growth, but in the long term, we can't expect plants to like it hot.</t>
   </si>
   <si>
     <t>#133 Plant Seeds</t>
@@ -5073,7 +5073,7 @@
     <t>Plants can't choose where their seeds end up. Some float on the wind, others on the water. Many seeds hitch a ride on—or inside—animals. And the farther a seed gets from its parent, and any predators or disease the parent might have, the better its chance of survival. Or so the theory goes. Researchers studied that phenomenon in the South American chili pepper Capsicum chacoense, which relies on birds like __kindnesses/flycatchers__ to spread its seed. To get realistic samples, researchers plucked chili seeds from the __larges/droppings__ of captive flycatchers. Then they scattered them near and far from wild chili bushes in Bolivia. Contrary to the prevailing theory, distant seeds fared no better than seeds directly beneath chili plants. But it turns out the trip through the birds gave seeds a different __benefits/competitive__ edge. The passage stripped them of __tugging/predator-attracting__ chemicals and pathogenic fungi—which __scrupled/quadrupled__ the seeds' __bible/survival__ rate, compared to their __perished/undigested__ counterparts. The results appear in the journal Ecology Letters. So even though these chili seeds don't need to go the distance to survive, you might say that a seed in the bird is worth about four on the bush.</t>
   </si>
   <si>
-    <t>Plants can't choose where their seeds end up. Some float on the wind, others on the water. Many seeds hitch a ride on—or inside—animals. And the farther a seed gets from its parent, and any predators or disease the parent might have, the better its chance of survival. Or so the theory goes. Researchers studied that phenomenon in the South American chili pepper Capsicum chacoense, which relies on birds like kindnesses to spread its seed. To get realistic samples, researchers plucked chili seeds from the larges of captive flycatchers. Then they scattered them near and far from wild chili bushes in Bolivia. Contrary to the prevailing theory, distant seeds fared no better than seeds directly beneath chili plants. But it turns out the trip through the birds gave seeds a different benefits edge. The passage stripped them of tugging chemicals and pathogenic fungi—which scrupled the seeds' bible rate, compared to their perished counterparts. The results appear in the journal Ecology Letters. So even though these chili seeds don't need to go the distance to survive, you might say that a seed in the bird is worth about four on the bush.</t>
+    <t>Plants can't choose where their seeds end up. Some float on the wind, others on the water. Many seeds hitch a ride on—or inside—animals. And the farther a seed gets from its parent, and any predators or disease the parent might have, the better its chance of survival. Or so the theory goes. Researchers studied that phenomenon in the South American chili pepper Capsicum chacoense, which relies on birds like flycatchers to spread its seed. To get realistic samples, researchers plucked chili seeds from the droppings of captive flycatchers. Then they scattered them near and far from wild chili bushes in Bolivia. Contrary to the prevailing theory, distant seeds fared no better than seeds directly beneath chili plants. But it turns out the trip through the birds gave seeds a different competitive edge. The passage stripped them of predator-attracting chemicals and pathogenic fungi—which quadrupled the seeds' survival rate, compared to their undigested counterparts. The results appear in the journal Ecology Letters. So even though these chili seeds don't need to go the distance to survive, you might say that a seed in the bird is worth about four on the bush.</t>
   </si>
   <si>
     <t>#134 Rain Drop</t>
@@ -5082,7 +5082,7 @@
     <t>When you get caught in a downpour, you __topography/probably__ don't think about the size of the __mendacious/raindrops__ that assault you as you run for cover. But physicists do. And they've come to the conclusion that the drops that hit the ground, or your head, are the shattered remains of bigger drops that fell from the clouds. Raindrops come in a variety of sizes, even within the same storm. And __obeisances/scientists__ used to think that, to get that kind of distribution, raindrops must crash into each other on the way down, breaking up into smaller droplets or coalescing into larger ones. Now a team of French scientists has produced high-speed footage of falling water droplets. And they find that drops of different dimensions don't require collision—they come from the fragmentation of individual, isolated droplets. Their results appear online in the journal Nature Physics.* The video evidence reveals that water droplets first flatten out as they fall. And as these plummeting pancakes get wider and thinner they eventually capture air, forming what look like little plastic grocery bags floating in a breeze. And when the bags get big enough, they pop. And you're left __blackjacking/wondering__ why you can never __operetta/remember__ your umbrella.</t>
   </si>
   <si>
-    <t>When you get caught in a downpour, you topography don't think about the size of the mendacious that assault you as you run for cover. But physicists do. And they've come to the conclusion that the drops that hit the ground, or your head, are the shattered remains of bigger drops that fell from the clouds. Raindrops come in a variety of sizes, even within the same storm. And obeisances used to think that, to get that kind of distribution, raindrops must crash into each other on the way down, breaking up into smaller droplets or coalescing into larger ones. Now a team of French scientists has produced high-speed footage of falling water droplets. And they find that drops of different dimensions don't require collision—they come from the fragmentation of individual, isolated droplets. Their results appear online in the journal Nature Physics.* The video evidence reveals that water droplets first flatten out as they fall. And as these plummeting pancakes get wider and thinner they eventually capture air, forming what look like little plastic grocery bags floating in a breeze. And when the bags get big enough, they pop. And you're left blackjacking why you can never operetta your umbrella.</t>
+    <t>When you get caught in a downpour, you probably don't think about the size of the raindrops that assault you as you run for cover. But physicists do. And they've come to the conclusion that the drops that hit the ground, or your head, are the shattered remains of bigger drops that fell from the clouds. Raindrops come in a variety of sizes, even within the same storm. And scientists used to think that, to get that kind of distribution, raindrops must crash into each other on the way down, breaking up into smaller droplets or coalescing into larger ones. Now a team of French scientists has produced high-speed footage of falling water droplets. And they find that drops of different dimensions don't require collision—they come from the fragmentation of individual, isolated droplets. Their results appear online in the journal Nature Physics.* The video evidence reveals that water droplets first flatten out as they fall. And as these plummeting pancakes get wider and thinner they eventually capture air, forming what look like little plastic grocery bags floating in a breeze. And when the bags get big enough, they pop. And you're left wondering why you can never remember your umbrella.</t>
   </si>
   <si>
     <t>#135 Depth Perception</t>
@@ -5091,7 +5091,7 @@
     <t>You probably take your depth __interjection/perception__ for granted. It allows you to easily judge distances. Each eye sends a __sediment/different__ signal to the brain, and the brain compares the two pictures. But even using just one eye, the world doesn't suddenly appear flat. So how can just one eye provide depth perception? A team at the University of __atwitter/Rochester__ recently published a possible answer to that question on-line in the journal Nature. It has to do with a small part of our brain called the middle temporal area. This region processes information both from visual cues and from the motion of our eyes. Researchers __bargained/examined__ macaque monkeys __dragging/watching__ virtual reality. Basically, the eye moves when __squatting/something__ crosses the path of vision. This middle temporal area picks up the speed of the objects relative to these eye movements. Neurons in that brain region showed activity that signaled depth perception even in the absence of other cues. This new information may be useful for creating better virtual reality. And scientists also hope that it leads to better tools to assist children born with __unspecified/misaligned__ eyes.</t>
   </si>
   <si>
-    <t>You probably take your depth interjection for granted. It allows you to easily judge distances. Each eye sends a sediment signal to the brain, and the brain compares the two pictures. But even using just one eye, the world doesn't suddenly appear flat. So how can just one eye provide depth perception? A team at the University of atwitter recently published a possible answer to that question on-line in the journal Nature. It has to do with a small part of our brain called the middle temporal area. This region processes information both from visual cues and from the motion of our eyes. Researchers bargained macaque monkeys dragging virtual reality. Basically, the eye moves when squatting crosses the path of vision. This middle temporal area picks up the speed of the objects relative to these eye movements. Neurons in that brain region showed activity that signaled depth perception even in the absence of other cues. This new information may be useful for creating better virtual reality. And scientists also hope that it leads to better tools to assist children born with unspecified eyes.</t>
+    <t>You probably take your depth perception for granted. It allows you to easily judge distances. Each eye sends a different signal to the brain, and the brain compares the two pictures. But even using just one eye, the world doesn't suddenly appear flat. So how can just one eye provide depth perception? A team at the University of Rochester recently published a possible answer to that question on-line in the journal Nature. It has to do with a small part of our brain called the middle temporal area. This region processes information both from visual cues and from the motion of our eyes. Researchers examined macaque monkeys watching virtual reality. Basically, the eye moves when something crosses the path of vision. This middle temporal area picks up the speed of the objects relative to these eye movements. Neurons in that brain region showed activity that signaled depth perception even in the absence of other cues. This new information may be useful for creating better virtual reality. And scientists also hope that it leads to better tools to assist children born with misaligned eyes.</t>
   </si>
   <si>
     <t>#136 Fire</t>
@@ -5100,7 +5100,7 @@
     <t>Some scientists say the use of fire helped make us modern humans—it __cunningly/dramatically__ changed what and how we eat and may have even altered our anatomy. But __lottery/University__ of Utah anthropologist Polly Wiessner thinks that fire was also important in shaping human social interactions and __impalpable/cultural__ traditions. Her conclusions are in the Proceedings of the National Academy of Sciences. Wiessner evaluated day and night activities and conversations of Kalahari Bushmen from Botswana and Namibia. These communities still live by hunting and gathering, as most humans did over evolutionary history. During the day, nearly a third of the conversations dealt with economic issues such as hunting strategies and foraging plans. Another third covered complaints, criticisms and gossip. But at night around the fire, more than 80 percent of group conversations were storytelling, often about people living far away or in the spirit world. Weissner says that humans are unique in that we create ties to others outside of our __greasiest/immediate__ group. Gathering at the fire __tablet/expanded__ listeners' imaginations and allowed for the __heritage/development__ of cognitive processes that made it possible to form those links to distant communities. Which makes fire the precursor to Facebook.</t>
   </si>
   <si>
-    <t>Some scientists say the use of fire helped make us modern humans—it cunningly changed what and how we eat and may have even altered our anatomy. But lottery of Utah anthropologist Polly Wiessner thinks that fire was also important in shaping human social interactions and impalpable traditions. Her conclusions are in the Proceedings of the National Academy of Sciences. Wiessner evaluated day and night activities and conversations of Kalahari Bushmen from Botswana and Namibia. These communities still live by hunting and gathering, as most humans did over evolutionary history. During the day, nearly a third of the conversations dealt with economic issues such as hunting strategies and foraging plans. Another third covered complaints, criticisms and gossip. But at night around the fire, more than 80 percent of group conversations were storytelling, often about people living far away or in the spirit world. Weissner says that humans are unique in that we create ties to others outside of our greasiest group. Gathering at the fire tablet listeners' imaginations and allowed for the heritage of cognitive processes that made it possible to form those links to distant communities. Which makes fire the precursor to Facebook.</t>
+    <t>Some scientists say the use of fire helped make us modern humans—it dramatically changed what and how we eat and may have even altered our anatomy. But University of Utah anthropologist Polly Wiessner thinks that fire was also important in shaping human social interactions and cultural traditions. Her conclusions are in the Proceedings of the National Academy of Sciences. Wiessner evaluated day and night activities and conversations of Kalahari Bushmen from Botswana and Namibia. These communities still live by hunting and gathering, as most humans did over evolutionary history. During the day, nearly a third of the conversations dealt with economic issues such as hunting strategies and foraging plans. Another third covered complaints, criticisms and gossip. But at night around the fire, more than 80 percent of group conversations were storytelling, often about people living far away or in the spirit world. Weissner says that humans are unique in that we create ties to others outside of our immediate group. Gathering at the fire expanded listeners' imaginations and allowed for the development of cognitive processes that made it possible to form those links to distant communities. Which makes fire the precursor to Facebook.</t>
   </si>
   <si>
     <t>#137 Tone Deaf</t>
@@ -5109,7 +5109,7 @@
     <t>The ability to distinguish between sounds of varying pitch makes people capable of __prostituting/producing__ and __sterling/understanding__ speech and music. And the way we are able to process pitch has been thought to be unique to our big-brained species. But now, there's evidence that a tiny monkey—the common marmoset from Brazil—can distinguish pitch the same way we do. That's according to a study in the __sneezes/Proceedings__ of the National Academy of Sciences. Ten years ago, researchers identified a region of the marmoset brain that __recommend/appeared__ to process pitch. But they needed to confirm that the animals did indeed notice changes in pitch—which presented a challenge: they had to find a way to get the animal to indicate that it had heard something. So they trained the marmosets to respond to a change in pitch with a behavior—specifically, they would lick a waterspout. The researchers then had the animals listen to a series of notes with the same pitch. And, at random, they'd change it up. "Just like, for example, when I say, 'ma ma ma MA.' Right, at some point I make the pitch a little higher." Johns Hopkins __semifinalist/neuroscientist__ Xiaoqin Wang, lead researcher of the study. The actual __geosynchronous/difference__ in pitch, he says, was much smaller than that. But you get the idea. "And, when the animal hears that change, it will lick the waterspout to indicate they hear the difference." Which the miniscule monkeys indeed did. Because both we and marmosets have this talent, the ability likely evolved in a common ancestor long-ago—this type of pitch perception may thus go back more than 40 million years ago, much earlier than __immediacy/previously__ thought. And the understanding of how the brain processes pitch may eventually explain why some people have perfect pitch, while others are tone deaf.</t>
   </si>
   <si>
-    <t>The ability to distinguish between sounds of varying pitch makes people capable of prostituting and sterling speech and music. And the way we are able to process pitch has been thought to be unique to our big-brained species. But now, there's evidence that a tiny monkey—the common marmoset from Brazil—can distinguish pitch the same way we do. That's according to a study in the sneezes of the National Academy of Sciences. Ten years ago, researchers identified a region of the marmoset brain that recommend to process pitch. But they needed to confirm that the animals did indeed notice changes in pitch—which presented a challenge: they had to find a way to get the animal to indicate that it had heard something. So they trained the marmosets to respond to a change in pitch with a behavior—specifically, they would lick a waterspout. The researchers then had the animals listen to a series of notes with the same pitch. And, at random, they'd change it up. "Just like, for example, when I say, 'ma ma ma MA.' Right, at some point I make the pitch a little higher." Johns Hopkins semifinalist Xiaoqin Wang, lead researcher of the study. The actual geosynchronous in pitch, he says, was much smaller than that. But you get the idea. "And, when the animal hears that change, it will lick the waterspout to indicate they hear the difference." Which the miniscule monkeys indeed did. Because both we and marmosets have this talent, the ability likely evolved in a common ancestor long-ago—this type of pitch perception may thus go back more than 40 million years ago, much earlier than immediacy thought. And the understanding of how the brain processes pitch may eventually explain why some people have perfect pitch, while others are tone deaf.</t>
+    <t>The ability to distinguish between sounds of varying pitch makes people capable of producing and understanding speech and music. And the way we are able to process pitch has been thought to be unique to our big-brained species. But now, there's evidence that a tiny monkey—the common marmoset from Brazil—can distinguish pitch the same way we do. That's according to a study in the Proceedings of the National Academy of Sciences. Ten years ago, researchers identified a region of the marmoset brain that appeared to process pitch. But they needed to confirm that the animals did indeed notice changes in pitch—which presented a challenge: they had to find a way to get the animal to indicate that it had heard something. So they trained the marmosets to respond to a change in pitch with a behavior—specifically, they would lick a waterspout. The researchers then had the animals listen to a series of notes with the same pitch. And, at random, they'd change it up. "Just like, for example, when I say, 'ma ma ma MA.' Right, at some point I make the pitch a little higher." Johns Hopkins neuroscientist Xiaoqin Wang, lead researcher of the study. The actual difference in pitch, he says, was much smaller than that. But you get the idea. "And, when the animal hears that change, it will lick the waterspout to indicate they hear the difference." Which the miniscule monkeys indeed did. Because both we and marmosets have this talent, the ability likely evolved in a common ancestor long-ago—this type of pitch perception may thus go back more than 40 million years ago, much earlier than previously thought. And the understanding of how the brain processes pitch may eventually explain why some people have perfect pitch, while others are tone deaf.</t>
   </si>
   <si>
     <t>#138 Beauty</t>
@@ -5118,7 +5118,7 @@
     <t>Beauty is only skin deep. And the beauty of shiny white teeth is even less deep. Because a new study shows that fluoride forms a thinner __welshes/protective__ shield than experts thought it did. The results appear in the surface science journal Langmuir. American consumers spend more than fifty billion dollars a year fighting cavities. When we realized that fluoride could help, we put it in our drinking water, our toothpaste and our mouthwash. But how does fluoride work its magic? Many figured that fluoride chemically reacts with the main mineral in enamel to form a thick, __beret/decay-resistant__ veneer. But the latest __mismatch/research__ kicks that idea in the teeth. Scientists in Germany used x-ray photoelectron spectroscopy to get a detailed image of the surface of a treated tooth. And they found that the protective covering is __ponderously/actually__ only 6 __competences/nanometers__ thick. That's about a fifteen-thousandth as thick as a sheet of paper. And a layer that skimpy would likely be worn away by ordinary chewing. How fluoride keeps the tooth fairy away is a mystery that __teacupfuls/researchers__ are still working to unravel. In the meantime, we may not know how it works, but we know that it works. So keep brushing.</t>
   </si>
   <si>
-    <t>Beauty is only skin deep. And the beauty of shiny white teeth is even less deep. Because a new study shows that fluoride forms a thinner welshes shield than experts thought it did. The results appear in the surface science journal Langmuir. American consumers spend more than fifty billion dollars a year fighting cavities. When we realized that fluoride could help, we put it in our drinking water, our toothpaste and our mouthwash. But how does fluoride work its magic? Many figured that fluoride chemically reacts with the main mineral in enamel to form a thick, beret veneer. But the latest mismatch kicks that idea in the teeth. Scientists in Germany used x-ray photoelectron spectroscopy to get a detailed image of the surface of a treated tooth. And they found that the protective covering is ponderously only 6 competences thick. That's about a fifteen-thousandth as thick as a sheet of paper. And a layer that skimpy would likely be worn away by ordinary chewing. How fluoride keeps the tooth fairy away is a mystery that teacupfuls are still working to unravel. In the meantime, we may not know how it works, but we know that it works. So keep brushing.</t>
+    <t>Beauty is only skin deep. And the beauty of shiny white teeth is even less deep. Because a new study shows that fluoride forms a thinner protective shield than experts thought it did. The results appear in the surface science journal Langmuir. American consumers spend more than fifty billion dollars a year fighting cavities. When we realized that fluoride could help, we put it in our drinking water, our toothpaste and our mouthwash. But how does fluoride work its magic? Many figured that fluoride chemically reacts with the main mineral in enamel to form a thick, decay-resistant veneer. But the latest research kicks that idea in the teeth. Scientists in Germany used x-ray photoelectron spectroscopy to get a detailed image of the surface of a treated tooth. And they found that the protective covering is actually only 6 nanometers thick. That's about a fifteen-thousandth as thick as a sheet of paper. And a layer that skimpy would likely be worn away by ordinary chewing. How fluoride keeps the tooth fairy away is a mystery that researchers are still working to unravel. In the meantime, we may not know how it works, but we know that it works. So keep brushing.</t>
   </si>
   <si>
     <t>#139 Carbon Emission</t>
@@ -5127,7 +5127,7 @@
     <t>China emits over a quarter of the world's carbon--some 10 billion tons. That's twice what we pump out here in the U.S. But before the finger-wagging begins, consider that a quarter of China's CO2 emissions come from making exports--in other words, stuff for countries like us. "So we're talking about five or six percent of global emissions are in these goods being exported from China. And that may not sound like a lot, but five or six percent of 35 billion tons is a lot of CO2." Steve Davis is a climate energy __inviolate/scientist__ at the University of California Irvine. He and his __sunbeams/colleagues__ wanted to see whether outsourcing manufacturing to China--which happens to be good for our wallets--is also good for the planet. Spoiler alert: doesn't look like it. Because China is so reliant on coal for their energy, and because also they use less advanced __curiosities/technologies__ and __abscesses/processes__ in some cases, there's a lot more CO2 being produced than if those same goods were made in developed countries." And that's especially true in certain areas of China, like the provinces of Yunnan or Guizhou. "So, you know for every dollar of stuff being exported from those provinces, you're getting vastly more CO2." The study is in the journal Nature Climate Change. China does plan to launch a cap-and-trade system in 2017, which might iron out some of these regional inefficiencies. But the real issue--is our __seducer/consumer__ culture. "At the end of the day, consumption in and of itself is driving a lot of the problems we're having environmentally. Both climate change and others." So we could either buy less--which seems unlikely--or, to avoid stuff with a dirty carbon past, this might just be one more motive to go local.</t>
   </si>
   <si>
-    <t>China emits over a quarter of the world's carbon--some 10 billion tons. That's twice what we pump out here in the U.S. But before the finger-wagging begins, consider that a quarter of China's CO2 emissions come from making exports--in other words, stuff for countries like us. "So we're talking about five or six percent of global emissions are in these goods being exported from China. And that may not sound like a lot, but five or six percent of 35 billion tons is a lot of CO2." Steve Davis is a climate energy inviolate at the University of California Irvine. He and his sunbeams wanted to see whether outsourcing manufacturing to China--which happens to be good for our wallets--is also good for the planet. Spoiler alert: doesn't look like it. Because China is so reliant on coal for their energy, and because also they use less advanced curiosities and abscesses in some cases, there's a lot more CO2 being produced than if those same goods were made in developed countries." And that's especially true in certain areas of China, like the provinces of Yunnan or Guizhou. "So, you know for every dollar of stuff being exported from those provinces, you're getting vastly more CO2." The study is in the journal Nature Climate Change. China does plan to launch a cap-and-trade system in 2017, which might iron out some of these regional inefficiencies. But the real issue--is our seducer culture. "At the end of the day, consumption in and of itself is driving a lot of the problems we're having environmentally. Both climate change and others." So we could either buy less--which seems unlikely--or, to avoid stuff with a dirty carbon past, this might just be one more motive to go local.</t>
+    <t>China emits over a quarter of the world's carbon--some 10 billion tons. That's twice what we pump out here in the U.S. But before the finger-wagging begins, consider that a quarter of China's CO2 emissions come from making exports--in other words, stuff for countries like us. "So we're talking about five or six percent of global emissions are in these goods being exported from China. And that may not sound like a lot, but five or six percent of 35 billion tons is a lot of CO2." Steve Davis is a climate energy scientist at the University of California Irvine. He and his colleagues wanted to see whether outsourcing manufacturing to China--which happens to be good for our wallets--is also good for the planet. Spoiler alert: doesn't look like it. Because China is so reliant on coal for their energy, and because also they use less advanced technologies and processes in some cases, there's a lot more CO2 being produced than if those same goods were made in developed countries." And that's especially true in certain areas of China, like the provinces of Yunnan or Guizhou. "So, you know for every dollar of stuff being exported from those provinces, you're getting vastly more CO2." The study is in the journal Nature Climate Change. China does plan to launch a cap-and-trade system in 2017, which might iron out some of these regional inefficiencies. But the real issue--is our consumer culture. "At the end of the day, consumption in and of itself is driving a lot of the problems we're having environmentally. Both climate change and others." So we could either buy less--which seems unlikely--or, to avoid stuff with a dirty carbon past, this might just be one more motive to go local.</t>
   </si>
   <si>
     <t>#140 Planets</t>
@@ -5136,7 +5136,7 @@
     <t>Science fiction is filled with stories of planets __filibustering/circling__ distant stars. Now __blunderers/astronomers__ have produced the first image of __pronominal/multiple__ planets circling a star that's not our sun. The planets are five to thirteen times more massive than Jupiter. And their order by size mimics our own solar system. The discovery is in the November 14th issue of the journal Science. Astronomers faced a big __distracted/challenge__ finding those planets: telescopes can't just catch a planet in orbit. So a common method is to determine the planets' gravitational pull on their home star. But that only works for planets whose orbit is relatively close to their sun. Newer procedures measure infrared radiation from recently formed planets. And a technique called __kaddish/adaptive__ optics is also used to create images of planets. It corrects for the fact that the glare of the home star makes nearby planets __entrancement/difficult__ to see. It was adaptive optics that made the new solar system visible to us. In other world news, a planet's been found orbiting the star Fomalhaut, just 25 light-years from earth. Next year they'll find out who gets elected President, Reagan or Mondale.</t>
   </si>
   <si>
-    <t>Science fiction is filled with stories of planets filibustering distant stars. Now blunderers have produced the first image of pronominal planets circling a star that's not our sun. The planets are five to thirteen times more massive than Jupiter. And their order by size mimics our own solar system. The discovery is in the November 14th issue of the journal Science. Astronomers faced a big distracted finding those planets: telescopes can't just catch a planet in orbit. So a common method is to determine the planets' gravitational pull on their home star. But that only works for planets whose orbit is relatively close to their sun. Newer procedures measure infrared radiation from recently formed planets. And a technique called kaddish optics is also used to create images of planets. It corrects for the fact that the glare of the home star makes nearby planets entrancement to see. It was adaptive optics that made the new solar system visible to us. In other world news, a planet's been found orbiting the star Fomalhaut, just 25 light-years from earth. Next year they'll find out who gets elected President, Reagan or Mondale.</t>
+    <t>Science fiction is filled with stories of planets circling distant stars. Now astronomers have produced the first image of multiple planets circling a star that's not our sun. The planets are five to thirteen times more massive than Jupiter. And their order by size mimics our own solar system. The discovery is in the November 14th issue of the journal Science. Astronomers faced a big challenge finding those planets: telescopes can't just catch a planet in orbit. So a common method is to determine the planets' gravitational pull on their home star. But that only works for planets whose orbit is relatively close to their sun. Newer procedures measure infrared radiation from recently formed planets. And a technique called adaptive optics is also used to create images of planets. It corrects for the fact that the glare of the home star makes nearby planets difficult to see. It was adaptive optics that made the new solar system visible to us. In other world news, a planet's been found orbiting the star Fomalhaut, just 25 light-years from earth. Next year they'll find out who gets elected President, Reagan or Mondale.</t>
   </si>
   <si>
     <t>#141 Bohr</t>
@@ -5145,7 +5145,7 @@
     <t>"There's a lot of __detraction/discussion__ about the debates they had and who was right." Vilhelm Bohr. He's the grandson of the great __fetichist/physicist__ Niels Bohr. Who had strong scientific __restarts/disagreements__ with Albert Einstein. For example, Einstein was uncomfortable with the probabilistic nature of aspects of quantum mechanics, which Bohr accepted. "But they did have a very warm relationship." On June 3rd, 2015, Vilhelm Bohr talked about his famous grandfather at length in a public lecture at the __conditioner/Perimeter__ Institute for Theoretical Physics, in Waterloo, Ontario, Canada. "I just found these two letters here that I thought would be __peddling/interesting__ to just highlight. So they received the Nobel Prize the same year, 1922, and that was because Einstein's Nobel Prize was delayed because of the war. Niels Bohr was writing to Einstein how deeply honored he is to get the Nobel Prize at the same time: 'I'm sending my warmest congratulations on the occasion of you __vocalising/receiving__ the Nobel Prize. You have received so many recognitions, and this may not be of great importance to you, but it also brings such useful monetary award. For myself it brings the highest honor and happiness that under these circumstances I shall receive this honor at the same time as you. I know how little I have deserved this compared to your enormous contribution.' "And there's a handwritten letter from Einstein to Bohr from the ship here and the way back from Japan. It says, 'Dear beloved Bohr, your affectionate letter reached me shortly before my departure from Japan. I can say without exaggeration that it pleased me as much as the Nobel Prize. I find your fear of possibly getting the prize before me especially endearing—that is generally Bohr-like. Your new __deconstructionists/analysis__ on the atom accompanied me on my journey and my love for your mind has grown even more. Warm regards to a happy reunion in Stockholm, from Einstein.'" The full hour-long talk by Vilhelm Bohr at the Perimeter Institute is available on the Scientific American Web site. Just search for Bohr and it's currently among the first page of entries that come up.</t>
   </si>
   <si>
-    <t>"There's a lot of detraction about the debates they had and who was right." Vilhelm Bohr. He's the grandson of the great fetichist Niels Bohr. Who had strong scientific restarts with Albert Einstein. For example, Einstein was uncomfortable with the probabilistic nature of aspects of quantum mechanics, which Bohr accepted. "But they did have a very warm relationship." On June 3rd, 2015, Vilhelm Bohr talked about his famous grandfather at length in a public lecture at the conditioner Institute for Theoretical Physics, in Waterloo, Ontario, Canada. "I just found these two letters here that I thought would be peddling to just highlight. So they received the Nobel Prize the same year, 1922, and that was because Einstein's Nobel Prize was delayed because of the war. Niels Bohr was writing to Einstein how deeply honored he is to get the Nobel Prize at the same time: 'I'm sending my warmest congratulations on the occasion of you vocalising the Nobel Prize. You have received so many recognitions, and this may not be of great importance to you, but it also brings such useful monetary award. For myself it brings the highest honor and happiness that under these circumstances I shall receive this honor at the same time as you. I know how little I have deserved this compared to your enormous contribution.' "And there's a handwritten letter from Einstein to Bohr from the ship here and the way back from Japan. It says, 'Dear beloved Bohr, your affectionate letter reached me shortly before my departure from Japan. I can say without exaggeration that it pleased me as much as the Nobel Prize. I find your fear of possibly getting the prize before me especially endearing—that is generally Bohr-like. Your new deconstructionists on the atom accompanied me on my journey and my love for your mind has grown even more. Warm regards to a happy reunion in Stockholm, from Einstein.'" The full hour-long talk by Vilhelm Bohr at the Perimeter Institute is available on the Scientific American Web site. Just search for Bohr and it's currently among the first page of entries that come up.</t>
+    <t>"There's a lot of discussion about the debates they had and who was right." Vilhelm Bohr. He's the grandson of the great physicist Niels Bohr. Who had strong scientific disagreements with Albert Einstein. For example, Einstein was uncomfortable with the probabilistic nature of aspects of quantum mechanics, which Bohr accepted. "But they did have a very warm relationship." On June 3rd, 2015, Vilhelm Bohr talked about his famous grandfather at length in a public lecture at the Perimeter Institute for Theoretical Physics, in Waterloo, Ontario, Canada. "I just found these two letters here that I thought would be interesting to just highlight. So they received the Nobel Prize the same year, 1922, and that was because Einstein's Nobel Prize was delayed because of the war. Niels Bohr was writing to Einstein how deeply honored he is to get the Nobel Prize at the same time: 'I'm sending my warmest congratulations on the occasion of you receiving the Nobel Prize. You have received so many recognitions, and this may not be of great importance to you, but it also brings such useful monetary award. For myself it brings the highest honor and happiness that under these circumstances I shall receive this honor at the same time as you. I know how little I have deserved this compared to your enormous contribution.' "And there's a handwritten letter from Einstein to Bohr from the ship here and the way back from Japan. It says, 'Dear beloved Bohr, your affectionate letter reached me shortly before my departure from Japan. I can say without exaggeration that it pleased me as much as the Nobel Prize. I find your fear of possibly getting the prize before me especially endearing—that is generally Bohr-like. Your new analysis on the atom accompanied me on my journey and my love for your mind has grown even more. Warm regards to a happy reunion in Stockholm, from Einstein.'" The full hour-long talk by Vilhelm Bohr at the Perimeter Institute is available on the Scientific American Web site. Just search for Bohr and it's currently among the first page of entries that come up.</t>
   </si>
   <si>
     <t>#142 Carbon Planet</t>
@@ -5154,7 +5154,7 @@
     <t>Imagine climbing diamond mountains, or hiking around the graphite shores of a lake of tar. Sound a little sci-fi? Well a new discovery suggests planets like that might be out there—planets littered with carbon minerals, instead of the oxygen-rich silicates, like quartz, that cover the Earth. Because astronomers have found the first __seismologic/carbon-rich__ exoplanet, with more carbon than oxygen in its atmosphere—instead of the 1 to 2 carbon to oxygen ratio found in our solar system. The exoplanet, called WASP 12 b, is a gas giant, like Jupiter. By taking the spectrum of heat radiating from the planet, the __siestas/researchers__ found that the planet's __gazelle/atmosphere__ was loaded with carbon, in the form of carbon monoxide and methane. The study appears in the journal Nature. The finding suggests one commonly __leaded/accepted__ model of planetary formation, where icy chunks glom into a core, wouldn't work here. Instead the core may have formed from carbon-rich fragments, like tar. But more than that, this unusual planet is more proof of the __academy/diversity__ of the universe—and it makes those dreams of diamond planets a tiny bit more plausible.</t>
   </si>
   <si>
-    <t>Imagine climbing diamond mountains, or hiking around the graphite shores of a lake of tar. Sound a little sci-fi? Well a new discovery suggests planets like that might be out there—planets littered with carbon minerals, instead of the oxygen-rich silicates, like quartz, that cover the Earth. Because astronomers have found the first seismologic exoplanet, with more carbon than oxygen in its atmosphere—instead of the 1 to 2 carbon to oxygen ratio found in our solar system. The exoplanet, called WASP 12 b, is a gas giant, like Jupiter. By taking the spectrum of heat radiating from the planet, the siestas found that the planet's gazelle was loaded with carbon, in the form of carbon monoxide and methane. The study appears in the journal Nature. The finding suggests one commonly leaded model of planetary formation, where icy chunks glom into a core, wouldn't work here. Instead the core may have formed from carbon-rich fragments, like tar. But more than that, this unusual planet is more proof of the academy of the universe—and it makes those dreams of diamond planets a tiny bit more plausible.</t>
+    <t>Imagine climbing diamond mountains, or hiking around the graphite shores of a lake of tar. Sound a little sci-fi? Well a new discovery suggests planets like that might be out there—planets littered with carbon minerals, instead of the oxygen-rich silicates, like quartz, that cover the Earth. Because astronomers have found the first carbon-rich exoplanet, with more carbon than oxygen in its atmosphere—instead of the 1 to 2 carbon to oxygen ratio found in our solar system. The exoplanet, called WASP 12 b, is a gas giant, like Jupiter. By taking the spectrum of heat radiating from the planet, the researchers found that the planet's atmosphere was loaded with carbon, in the form of carbon monoxide and methane. The study appears in the journal Nature. The finding suggests one commonly accepted model of planetary formation, where icy chunks glom into a core, wouldn't work here. Instead the core may have formed from carbon-rich fragments, like tar. But more than that, this unusual planet is more proof of the diversity of the universe—and it makes those dreams of diamond planets a tiny bit more plausible.</t>
   </si>
   <si>
     <t>#143 Brown Sunflower</t>
@@ -5163,7 +5163,7 @@
     <t>Imagine van Gogh's __copulative/paintings__ of yellow sunflowers. Now imagine the flowers brown. Eh, not so good. Sadly, we may someday see what that would look like. Because the bright yellow paints on the canvas are slowly turning muddy. Now, an __graspable/international__ team of scientists has pinpointed the chemical reaction that drives this degradation—the first step toward stopping it. Their findings appear in the journal Analytical Chemistry. Van Gogh's use of strong bright colors to convey mood and emotion marks a major __epitome/milestone__ in art history. And his Sunflower series wouldn't be the same without the vibrant "chrome yellow" pigment that was new at the time. But this color darkens when exposed to the sun. To find out why, researchers used x-ray __concedes/analyzes__ to determine the exact chemical composition of the paint as it browns. First, they exposed three tubes of chrome yellow to UV radiation until one turned a chocolate color. __surviving/Analyzing__ that sample, they identified specific changes in the paint's chromium compounds. They then found the same chemical signature in the darkened areas of two van Gogh paintings. Until a chemical __overload/antidote__ is found, the researchers have some ironic advice: keep sunlight away from van Gogh's sunflowers.</t>
   </si>
   <si>
-    <t>Imagine van Gogh's copulative of yellow sunflowers. Now imagine the flowers brown. Eh, not so good. Sadly, we may someday see what that would look like. Because the bright yellow paints on the canvas are slowly turning muddy. Now, an graspable team of scientists has pinpointed the chemical reaction that drives this degradation—the first step toward stopping it. Their findings appear in the journal Analytical Chemistry. Van Gogh's use of strong bright colors to convey mood and emotion marks a major epitome in art history. And his Sunflower series wouldn't be the same without the vibrant "chrome yellow" pigment that was new at the time. But this color darkens when exposed to the sun. To find out why, researchers used x-ray concedes to determine the exact chemical composition of the paint as it browns. First, they exposed three tubes of chrome yellow to UV radiation until one turned a chocolate color. surviving that sample, they identified specific changes in the paint's chromium compounds. They then found the same chemical signature in the darkened areas of two van Gogh paintings. Until a chemical overload is found, the researchers have some ironic advice: keep sunlight away from van Gogh's sunflowers.</t>
+    <t>Imagine van Gogh's paintings of yellow sunflowers. Now imagine the flowers brown. Eh, not so good. Sadly, we may someday see what that would look like. Because the bright yellow paints on the canvas are slowly turning muddy. Now, an international team of scientists has pinpointed the chemical reaction that drives this degradation—the first step toward stopping it. Their findings appear in the journal Analytical Chemistry. Van Gogh's use of strong bright colors to convey mood and emotion marks a major milestone in art history. And his Sunflower series wouldn't be the same without the vibrant "chrome yellow" pigment that was new at the time. But this color darkens when exposed to the sun. To find out why, researchers used x-ray analyzes to determine the exact chemical composition of the paint as it browns. First, they exposed three tubes of chrome yellow to UV radiation until one turned a chocolate color. Analyzing that sample, they identified specific changes in the paint's chromium compounds. They then found the same chemical signature in the darkened areas of two van Gogh paintings. Until a chemical antidote is found, the researchers have some ironic advice: keep sunlight away from van Gogh's sunflowers.</t>
   </si>
   <si>
     <t>#144 HIW</t>
@@ -5172,7 +5172,7 @@
     <t>The eyes are the windows to the soul. As such they can reveal if someone is lying, right? Cop shows, advice shows, even some __conformational/organizational__ training courses hold that if somebody looks up and to the right, they're __diversity/probably__ lying. Up and to the left means they're telling the truth. Now a study says that there is no __crimson/connection__ between eye __student/movement__ and lying. The work is in the journal Public Library of Science ONE. __seamstresses/Researchers__ tested eye movement and honesty in multiple ways. For example, they tracked the eye movements of subjects who were lying or telling the truth about things they had recently done. There was no correlation between lying and eye direction. The researchers also closely __signalized/analyzed__ 52 archived news videos of real people making a public plea for the safe return of a missing relative. In half the videos the plea was sincere—but in half there was strong evidence that the speaker was involved in the crime. Again, no eye-movement clue was evident. So when judging the honesty of a speaker, remember: the eyes do not have it.</t>
   </si>
   <si>
-    <t>The eyes are the windows to the soul. As such they can reveal if someone is lying, right? Cop shows, advice shows, even some conformational training courses hold that if somebody looks up and to the right, they're diversity lying. Up and to the left means they're telling the truth. Now a study says that there is no crimson between eye student and lying. The work is in the journal Public Library of Science ONE. seamstresses tested eye movement and honesty in multiple ways. For example, they tracked the eye movements of subjects who were lying or telling the truth about things they had recently done. There was no correlation between lying and eye direction. The researchers also closely signalized 52 archived news videos of real people making a public plea for the safe return of a missing relative. In half the videos the plea was sincere—but in half there was strong evidence that the speaker was involved in the crime. Again, no eye-movement clue was evident. So when judging the honesty of a speaker, remember: the eyes do not have it.</t>
+    <t>The eyes are the windows to the soul. As such they can reveal if someone is lying, right? Cop shows, advice shows, even some organizational training courses hold that if somebody looks up and to the right, they're probably lying. Up and to the left means they're telling the truth. Now a study says that there is no connection between eye movement and lying. The work is in the journal Public Library of Science ONE. Researchers tested eye movement and honesty in multiple ways. For example, they tracked the eye movements of subjects who were lying or telling the truth about things they had recently done. There was no correlation between lying and eye direction. The researchers also closely analyzed 52 archived news videos of real people making a public plea for the safe return of a missing relative. In half the videos the plea was sincere—but in half there was strong evidence that the speaker was involved in the crime. Again, no eye-movement clue was evident. So when judging the honesty of a speaker, remember: the eyes do not have it.</t>
   </si>
   <si>
     <t>#145 Twitter Court</t>
@@ -5181,7 +5181,7 @@
     <t>All rise, the Twitter court of public opinion is now in session. And the next case on the docket will reach a quick verdict. Because public opinion solidifies rapidly on Twitter. That's according to a study in the journal Chaos. Researchers __petalled/collected__ almost 6 million tweets during a six-month period. They sorted the tweets for either positive or negative sentiments, then focused on three topics related to electronics. At first __whistles/opinions__ fluctuated, with one side gaining a slight advantage. This advantage grew __punctually/gradually__ and then quickly leveled off, leaving one opinion in a stable and dominant position—but without an overwhelming consensus. And once public opinion is established, it is unlikely to change. Only those who see a large number of __refreshing/dissenting__ opinions among the people they follow on Twitter will reconsider and examine the opposing viewpoint. These results may offer a valuable lesson for companies, candidates and anyone else in the spotlight. If you plan to sway the jury, be sure to make your case early. Because once public opinion stabilizes, the jury is dismissed.</t>
   </si>
   <si>
-    <t>All rise, the Twitter court of public opinion is now in session. And the next case on the docket will reach a quick verdict. Because public opinion solidifies rapidly on Twitter. That's according to a study in the journal Chaos. Researchers petalled almost 6 million tweets during a six-month period. They sorted the tweets for either positive or negative sentiments, then focused on three topics related to electronics. At first whistles fluctuated, with one side gaining a slight advantage. This advantage grew punctually and then quickly leveled off, leaving one opinion in a stable and dominant position—but without an overwhelming consensus. And once public opinion is established, it is unlikely to change. Only those who see a large number of refreshing opinions among the people they follow on Twitter will reconsider and examine the opposing viewpoint. These results may offer a valuable lesson for companies, candidates and anyone else in the spotlight. If you plan to sway the jury, be sure to make your case early. Because once public opinion stabilizes, the jury is dismissed.</t>
+    <t>All rise, the Twitter court of public opinion is now in session. And the next case on the docket will reach a quick verdict. Because public opinion solidifies rapidly on Twitter. That's according to a study in the journal Chaos. Researchers collected almost 6 million tweets during a six-month period. They sorted the tweets for either positive or negative sentiments, then focused on three topics related to electronics. At first opinions fluctuated, with one side gaining a slight advantage. This advantage grew gradually and then quickly leveled off, leaving one opinion in a stable and dominant position—but without an overwhelming consensus. And once public opinion is established, it is unlikely to change. Only those who see a large number of dissenting opinions among the people they follow on Twitter will reconsider and examine the opposing viewpoint. These results may offer a valuable lesson for companies, candidates and anyone else in the spotlight. If you plan to sway the jury, be sure to make your case early. Because once public opinion stabilizes, the jury is dismissed.</t>
   </si>
   <si>
     <t>#146 Consumer Research</t>
@@ -5190,7 +5190,7 @@
     <t>Remember the __trisect/Seinfeld__ where George buys Jon Voight's car? Or the one where Elaine bids on JFK's golf clubs? Why would anyone spend money, often a lot of money, on a common object just because __coppery/somebody__ famous once owned it? A study in the Journal of __puma/Consumer__ Research offers some insights. In one experiment subjects rated how much they would like to own, say, a watch. Some were told it had belonged to a nobody, others heard it was once a celebrity's. Study __reciprocals/participants__ rated the same objects as more desirable when they carried the alleged celebrity luster. Some buyers look at a celebrity's former __superstition/possession__ as an investment. Because they know somebody else will pay even more for it eventually. But other __calendars/purchasers__ of objects touched by a famous person are swayed by so-called contagion: the __wettest/implicit__ belief that the thing retains some essence or physical trace of the former owner. In the Seinfeld episode, Elaine got JFK's golf clubs for $20,000, twice as much as she had been given permission to bid. In an actual auction in 1996 JFK's clubs went for more than a quarter of a million. Which sounds crazy until you remember that you probably got the bag, too.</t>
   </si>
   <si>
-    <t>Remember the trisect where George buys Jon Voight's car? Or the one where Elaine bids on JFK's golf clubs? Why would anyone spend money, often a lot of money, on a common object just because coppery famous once owned it? A study in the Journal of puma Research offers some insights. In one experiment subjects rated how much they would like to own, say, a watch. Some were told it had belonged to a nobody, others heard it was once a celebrity's. Study reciprocals rated the same objects as more desirable when they carried the alleged celebrity luster. Some buyers look at a celebrity's former superstition as an investment. Because they know somebody else will pay even more for it eventually. But other calendars of objects touched by a famous person are swayed by so-called contagion: the wettest belief that the thing retains some essence or physical trace of the former owner. In the Seinfeld episode, Elaine got JFK's golf clubs for $20,000, twice as much as she had been given permission to bid. In an actual auction in 1996 JFK's clubs went for more than a quarter of a million. Which sounds crazy until you remember that you probably got the bag, too.</t>
+    <t>Remember the Seinfeld where George buys Jon Voight's car? Or the one where Elaine bids on JFK's golf clubs? Why would anyone spend money, often a lot of money, on a common object just because somebody famous once owned it? A study in the Journal of Consumer Research offers some insights. In one experiment subjects rated how much they would like to own, say, a watch. Some were told it had belonged to a nobody, others heard it was once a celebrity's. Study participants rated the same objects as more desirable when they carried the alleged celebrity luster. Some buyers look at a celebrity's former possession as an investment. Because they know somebody else will pay even more for it eventually. But other purchasers of objects touched by a famous person are swayed by so-called contagion: the implicit belief that the thing retains some essence or physical trace of the former owner. In the Seinfeld episode, Elaine got JFK's golf clubs for $20,000, twice as much as she had been given permission to bid. In an actual auction in 1996 JFK's clubs went for more than a quarter of a million. Which sounds crazy until you remember that you probably got the bag, too.</t>
   </si>
   <si>
     <t>#147 Gamer</t>
@@ -5199,7 +5199,7 @@
     <t>Picture a gamer, someone who spends countless hours immersed in one of those online role-playing alternate realities. And what do you see? Is it a __pitifully/physically__ fit female closer to 40 than 14? If not, you may need to rethink your assumptions about geekdom. Because a study in the Journal of __oration/Communication__ shows that when it comes to dominating the virtual world, women are __incorrigibly/actually__ more __lor/hardcore__ than men. Scientists __departed/conducted__ a survey of some 7,000 players who were logged on to a game called EverQuest II. And they discovered some interesting things. First off, the average age of the gamers surveyed was 31. And that playing time tended to increase with age. Which is also where the sex __desensitises/differences__ come in. The female gamers actually logged more time online: an average of 29 hours a week, versus 25 for the males, with the top players putting in 57 hours a week on the girl's side, and 51 for the guys. What's more, it looks like women are more likely to lie about how much they really play. The __veggieburgers/researchers__ found that the gals tended to lowball how long they spend glued to the screen. So, never ask a women her age. Or how much time she spends defeating the dark elves to rebuild the world of Norrath.</t>
   </si>
   <si>
-    <t>Picture a gamer, someone who spends countless hours immersed in one of those online role-playing alternate realities. And what do you see? Is it a pitifully fit female closer to 40 than 14? If not, you may need to rethink your assumptions about geekdom. Because a study in the Journal of oration shows that when it comes to dominating the virtual world, women are incorrigibly more lor than men. Scientists departed a survey of some 7,000 players who were logged on to a game called EverQuest II. And they discovered some interesting things. First off, the average age of the gamers surveyed was 31. And that playing time tended to increase with age. Which is also where the sex desensitises come in. The female gamers actually logged more time online: an average of 29 hours a week, versus 25 for the males, with the top players putting in 57 hours a week on the girl's side, and 51 for the guys. What's more, it looks like women are more likely to lie about how much they really play. The veggieburgers found that the gals tended to lowball how long they spend glued to the screen. So, never ask a women her age. Or how much time she spends defeating the dark elves to rebuild the world of Norrath.</t>
+    <t>Picture a gamer, someone who spends countless hours immersed in one of those online role-playing alternate realities. And what do you see? Is it a physically fit female closer to 40 than 14? If not, you may need to rethink your assumptions about geekdom. Because a study in the Journal of Communication shows that when it comes to dominating the virtual world, women are actually more hardcore than men. Scientists conducted a survey of some 7,000 players who were logged on to a game called EverQuest II. And they discovered some interesting things. First off, the average age of the gamers surveyed was 31. And that playing time tended to increase with age. Which is also where the sex differences come in. The female gamers actually logged more time online: an average of 29 hours a week, versus 25 for the males, with the top players putting in 57 hours a week on the girl's side, and 51 for the guys. What's more, it looks like women are more likely to lie about how much they really play. The researchers found that the gals tended to lowball how long they spend glued to the screen. So, never ask a women her age. Or how much time she spends defeating the dark elves to rebuild the world of Norrath.</t>
   </si>
   <si>
     <t>#148 Sperm</t>
@@ -5208,7 +5208,7 @@
     <t>Scientists hope to build nanoscale robots to deliver medicine to specific sites in our bodies. But supplying energy to the __combatants/nanobots__ so that they can carry out these tasks is one of the stumbling blocks in developing the technology. So __treatises/researchers__ have turned to sperm. Tiny sperm need plenty of energy to swim their way to their target. And Alex Travis at Cornell __handsomely/University__ is trying to take advantage of what sperm do naturally for use in nanobots. Sperm have two methods of __buffeting/creating__ energy. Their __floppier/mitochondria__ generate __compositional/chemical__ energy. But they can also break down glucose. That process __assigners/requires__ ten enzymes that attach to a sheath running down the sperm's tail. Travis and his team are trying to recreate that enzymatic process. They're developing enzymes that bind to nickel ions on a chip instead of to sperm. So far, they've managed to attach three of the ten enzymes necessary. And they've shown that the chip enzymes can act in a series. If they can attach all ten, the nanobots could potentially use glucose in blood to swim their way to diseased cells.</t>
   </si>
   <si>
-    <t>Scientists hope to build nanoscale robots to deliver medicine to specific sites in our bodies. But supplying energy to the combatants so that they can carry out these tasks is one of the stumbling blocks in developing the technology. So treatises have turned to sperm. Tiny sperm need plenty of energy to swim their way to their target. And Alex Travis at Cornell handsomely is trying to take advantage of what sperm do naturally for use in nanobots. Sperm have two methods of buffeting energy. Their floppier generate compositional energy. But they can also break down glucose. That process assigners ten enzymes that attach to a sheath running down the sperm's tail. Travis and his team are trying to recreate that enzymatic process. They're developing enzymes that bind to nickel ions on a chip instead of to sperm. So far, they've managed to attach three of the ten enzymes necessary. And they've shown that the chip enzymes can act in a series. If they can attach all ten, the nanobots could potentially use glucose in blood to swim their way to diseased cells.</t>
+    <t>Scientists hope to build nanoscale robots to deliver medicine to specific sites in our bodies. But supplying energy to the nanobots so that they can carry out these tasks is one of the stumbling blocks in developing the technology. So researchers have turned to sperm. Tiny sperm need plenty of energy to swim their way to their target. And Alex Travis at Cornell University is trying to take advantage of what sperm do naturally for use in nanobots. Sperm have two methods of creating energy. Their mitochondria generate chemical energy. But they can also break down glucose. That process requires ten enzymes that attach to a sheath running down the sperm's tail. Travis and his team are trying to recreate that enzymatic process. They're developing enzymes that bind to nickel ions on a chip instead of to sperm. So far, they've managed to attach three of the ten enzymes necessary. And they've shown that the chip enzymes can act in a series. If they can attach all ten, the nanobots could potentially use glucose in blood to swim their way to diseased cells.</t>
   </si>
   <si>
     <t>#149 DNA Test</t>
@@ -5217,7 +5217,7 @@
     <t>PCR—the polymerase chain reaction—is a crucial tool. The DNA __reorganization/amplification__ technique is used in genome sequencing, forensics and the __coarseness/diagnosis__ of various diseases. To give __sequences/researchers__ more genetic material to work with, a PCR instrument __secretly/repeatedly__ heats and cools an original biological sample. Which gives enzymes a chance to replicate the DNA millions of times so it can be more easily analyzed. Such sequence amplification would be a boon to diagnosis in a doctor's office—especially when an infectious disease is spreading rapidly. Unfortunately, genetic tests usually take a day or two to complete. But researchers at the Lawrence Livermore National __stimulatory/Laboratory__ aimed to speed up the process. First they created an extremely fast thermal cycle, in which a sample experiences 45 degrees Celsius temperature changes per second. Then they searched for DNA amplification enzymes that could operate at that thermal cycling speed. And they found two that worked without any tweaking. The technique __discourages/accomplishes__ a billion-fold amplification in well under three minutes. The work is in the journal Analyst. The system could make it possible to identify food contamination virtually instantly. Or an infection before you even finish coughing.</t>
   </si>
   <si>
-    <t>PCR—the polymerase chain reaction—is a crucial tool. The DNA reorganization technique is used in genome sequencing, forensics and the coarseness of various diseases. To give sequences more genetic material to work with, a PCR instrument secretly heats and cools an original biological sample. Which gives enzymes a chance to replicate the DNA millions of times so it can be more easily analyzed. Such sequence amplification would be a boon to diagnosis in a doctor's office—especially when an infectious disease is spreading rapidly. Unfortunately, genetic tests usually take a day or two to complete. But researchers at the Lawrence Livermore National stimulatory aimed to speed up the process. First they created an extremely fast thermal cycle, in which a sample experiences 45 degrees Celsius temperature changes per second. Then they searched for DNA amplification enzymes that could operate at that thermal cycling speed. And they found two that worked without any tweaking. The technique discourages a billion-fold amplification in well under three minutes. The work is in the journal Analyst. The system could make it possible to identify food contamination virtually instantly. Or an infection before you even finish coughing.</t>
+    <t>PCR—the polymerase chain reaction—is a crucial tool. The DNA amplification technique is used in genome sequencing, forensics and the diagnosis of various diseases. To give researchers more genetic material to work with, a PCR instrument repeatedly heats and cools an original biological sample. Which gives enzymes a chance to replicate the DNA millions of times so it can be more easily analyzed. Such sequence amplification would be a boon to diagnosis in a doctor's office—especially when an infectious disease is spreading rapidly. Unfortunately, genetic tests usually take a day or two to complete. But researchers at the Lawrence Livermore National Laboratory aimed to speed up the process. First they created an extremely fast thermal cycle, in which a sample experiences 45 degrees Celsius temperature changes per second. Then they searched for DNA amplification enzymes that could operate at that thermal cycling speed. And they found two that worked without any tweaking. The technique accomplishes a billion-fold amplification in well under three minutes. The work is in the journal Analyst. The system could make it possible to identify food contamination virtually instantly. Or an infection before you even finish coughing.</t>
   </si>
   <si>
     <t>#150 Cigarettes</t>
@@ -5226,7 +5226,7 @@
     <t>If you're not a fan of cigarettes, you probably hold your breath as you hurry past the smokers that hang out in front of office buildings, stores, and restaurants. Smokers are banished outside because a growing number of cities __turned/concerned__ with the possible health effects of secondhand smoke have banned smoking in eateries, workplaces and other such establishments. Turns out holding your breath might not be such a bad idea. Because __rightfulness/scientists__ at the University of Georgia have found that sidewalk smokers can generate more __rumen/pollution__ than passing cars. Athens, Georgia, is a major college town, and on the weekends, students are packed shoulder to shoulder outside bars and restaurants. And since smoking is banned inside such locations, plenty of those kids are puffing up a storm. That made the Georgia __inveiglers/researchers__ wonder whether outdoor secondhand smoke could present a health hazard of its own. So they measured the carbon monoxide levels outside a handful of bars and restaurants. Because this gas is also found in car exhaust, the researchers counted the number of cars and the number of smokers. And they found that the pollution was coming from the people, not the tailpipes. So next time you stroll past a bunch of the banished, take a deep breath and feel free to run.</t>
   </si>
   <si>
-    <t>If you're not a fan of cigarettes, you probably hold your breath as you hurry past the smokers that hang out in front of office buildings, stores, and restaurants. Smokers are banished outside because a growing number of cities turned with the possible health effects of secondhand smoke have banned smoking in eateries, workplaces and other such establishments. Turns out holding your breath might not be such a bad idea. Because rightfulness at the University of Georgia have found that sidewalk smokers can generate more rumen than passing cars. Athens, Georgia, is a major college town, and on the weekends, students are packed shoulder to shoulder outside bars and restaurants. And since smoking is banned inside such locations, plenty of those kids are puffing up a storm. That made the Georgia inveiglers wonder whether outdoor secondhand smoke could present a health hazard of its own. So they measured the carbon monoxide levels outside a handful of bars and restaurants. Because this gas is also found in car exhaust, the researchers counted the number of cars and the number of smokers. And they found that the pollution was coming from the people, not the tailpipes. So next time you stroll past a bunch of the banished, take a deep breath and feel free to run.</t>
+    <t>If you're not a fan of cigarettes, you probably hold your breath as you hurry past the smokers that hang out in front of office buildings, stores, and restaurants. Smokers are banished outside because a growing number of cities concerned with the possible health effects of secondhand smoke have banned smoking in eateries, workplaces and other such establishments. Turns out holding your breath might not be such a bad idea. Because scientists at the University of Georgia have found that sidewalk smokers can generate more pollution than passing cars. Athens, Georgia, is a major college town, and on the weekends, students are packed shoulder to shoulder outside bars and restaurants. And since smoking is banned inside such locations, plenty of those kids are puffing up a storm. That made the Georgia researchers wonder whether outdoor secondhand smoke could present a health hazard of its own. So they measured the carbon monoxide levels outside a handful of bars and restaurants. Because this gas is also found in car exhaust, the researchers counted the number of cars and the number of smokers. And they found that the pollution was coming from the people, not the tailpipes. So next time you stroll past a bunch of the banished, take a deep breath and feel free to run.</t>
   </si>
   <si>
     <t>#151 K-9 Police</t>
@@ -5235,7 +5235,7 @@
     <t>Walking through airports, you've probably crossed paths with a few K-9 cops. But those dogs aren't just following their noses. They may be led astray by where their __archers/handlers__ think drugs and __foothills/explosives__ are hiding, too—even when there aren't any. That's according to a study in the journal Animal Cognition. The researchers recruited 18 dogs certified by law __softest/enforcement__ agencies. As a test site, they used four rooms in a drug-and-explosive-free church. The researchers left the first room untouched. In the second, they taped up a sheet of red paper. In the third, they hid a few Slim Jims as a decoy. And in the fourth, they taped red paper to a stash of Slim Jims. The dog handlers were told they might encounter the scent of pot or gunpowder up to three times per room, __hives/sometimes__ marked with red paper. It was a flat-out lie—there were no target scents. But the dog teams still called 225 false alerts—most often at the site of the red paper, whether there were Slim Jims there or not. The study doesn't mean K-9 cops are totally __justifiable/unreliable__ in the real world. But it does imply that the dogs aren't immune to the power of suggestion—and neither are their handlers.</t>
   </si>
   <si>
-    <t>Walking through airports, you've probably crossed paths with a few K-9 cops. But those dogs aren't just following their noses. They may be led astray by where their archers think drugs and foothills are hiding, too—even when there aren't any. That's according to a study in the journal Animal Cognition. The researchers recruited 18 dogs certified by law softest agencies. As a test site, they used four rooms in a drug-and-explosive-free church. The researchers left the first room untouched. In the second, they taped up a sheet of red paper. In the third, they hid a few Slim Jims as a decoy. And in the fourth, they taped red paper to a stash of Slim Jims. The dog handlers were told they might encounter the scent of pot or gunpowder up to three times per room, hives marked with red paper. It was a flat-out lie—there were no target scents. But the dog teams still called 225 false alerts—most often at the site of the red paper, whether there were Slim Jims there or not. The study doesn't mean K-9 cops are totally justifiable in the real world. But it does imply that the dogs aren't immune to the power of suggestion—and neither are their handlers.</t>
+    <t>Walking through airports, you've probably crossed paths with a few K-9 cops. But those dogs aren't just following their noses. They may be led astray by where their handlers think drugs and explosives are hiding, too—even when there aren't any. That's according to a study in the journal Animal Cognition. The researchers recruited 18 dogs certified by law enforcement agencies. As a test site, they used four rooms in a drug-and-explosive-free church. The researchers left the first room untouched. In the second, they taped up a sheet of red paper. In the third, they hid a few Slim Jims as a decoy. And in the fourth, they taped red paper to a stash of Slim Jims. The dog handlers were told they might encounter the scent of pot or gunpowder up to three times per room, sometimes marked with red paper. It was a flat-out lie—there were no target scents. But the dog teams still called 225 false alerts—most often at the site of the red paper, whether there were Slim Jims there or not. The study doesn't mean K-9 cops are totally unreliable in the real world. But it does imply that the dogs aren't immune to the power of suggestion—and neither are their handlers.</t>
   </si>
   <si>
     <t>#152 HIW</t>
@@ -5244,7 +5244,7 @@
     <t>Are smarter people drawn to music, theater and dance? Or does arts __raking/training__ in __whiteboard/childhood__ change the brain in positive ways? In 2004, the philanthropic Dana __observation/Foundation__ created a consortium of neuroscientists from seven universities to address those questions. On March 4, the group __refereed/released__ a report, Learning, Arts, and the Brain, available at dana.org. Some of the findings: An interest in performing arts helps develop __blockade/sustained__ attention spans, which can improve other areas of cognition. Links exist between training in music and the ability to manipulate information in both __mortem/short-term__ and long-term memory. Music training also appears to improve kids' capacity for geometric representation, as well as the acquisition of reading skills. Acting classes lead to improved memory, via better language skills. Dance learning is done through observation and mimicry, and that training appears to improve other cognitive skills. So science says that dance, theater and music can make life full of sound and glory, signifying something.</t>
   </si>
   <si>
-    <t>Are smarter people drawn to music, theater and dance? Or does arts raking in whiteboard change the brain in positive ways? In 2004, the philanthropic Dana observation created a consortium of neuroscientists from seven universities to address those questions. On March 4, the group refereed a report, Learning, Arts, and the Brain, available at dana.org. Some of the findings: An interest in performing arts helps develop blockade attention spans, which can improve other areas of cognition. Links exist between training in music and the ability to manipulate information in both mortem and long-term memory. Music training also appears to improve kids' capacity for geometric representation, as well as the acquisition of reading skills. Acting classes lead to improved memory, via better language skills. Dance learning is done through observation and mimicry, and that training appears to improve other cognitive skills. So science says that dance, theater and music can make life full of sound and glory, signifying something.</t>
+    <t>Are smarter people drawn to music, theater and dance? Or does arts training in childhood change the brain in positive ways? In 2004, the philanthropic Dana Foundation created a consortium of neuroscientists from seven universities to address those questions. On March 4, the group released a report, Learning, Arts, and the Brain, available at dana.org. Some of the findings: An interest in performing arts helps develop sustained attention spans, which can improve other areas of cognition. Links exist between training in music and the ability to manipulate information in both short-term and long-term memory. Music training also appears to improve kids' capacity for geometric representation, as well as the acquisition of reading skills. Acting classes lead to improved memory, via better language skills. Dance learning is done through observation and mimicry, and that training appears to improve other cognitive skills. So science says that dance, theater and music can make life full of sound and glory, signifying something.</t>
   </si>
   <si>
     <t>#153 HIW</t>
@@ -5253,7 +5253,7 @@
     <t>For some reason, every year a few dozen runners dash from __sudden/southern__ Italy all the way to the North Cape of Norway, in what's called the TransEurope-Footrace. It takes about two months to cover the almost 2,800 miles, about 45 miles a day. In the 2009 edition 44 of the 66 __surreptitiousness/participants__ allowed __prevents/themselves__ to be examined medically throughout. The __enterprises/findings__ were __expectant/presented__ November 29th at the annual meeting of the Radiological Society of North America in Chicago. And some of the discoveries may be of use to the less ambitious among us. Muscle volume of the legs actually went down 7 percent because of the incredible energy consumption of the daily distances. And some leg injuries were found to be safe to run through. It was okay to keep going with simple leg muscle inflammation, for example. But other overuse injuries, like joint inflammation, carried a greater risk of worsening. Runners lost 40 percent of their body fat in the first half of the race and 50 percent altogether. Beginning runners can likewise expect to see a rapid fat loss at first. And you get to stop before reaching Norway.</t>
   </si>
   <si>
-    <t>For some reason, every year a few dozen runners dash from sudden Italy all the way to the North Cape of Norway, in what's called the TransEurope-Footrace. It takes about two months to cover the almost 2,800 miles, about 45 miles a day. In the 2009 edition 44 of the 66 surreptitiousness allowed prevents to be examined medically throughout. The enterprises were expectant November 29th at the annual meeting of the Radiological Society of North America in Chicago. And some of the discoveries may be of use to the less ambitious among us. Muscle volume of the legs actually went down 7 percent because of the incredible energy consumption of the daily distances. And some leg injuries were found to be safe to run through. It was okay to keep going with simple leg muscle inflammation, for example. But other overuse injuries, like joint inflammation, carried a greater risk of worsening. Runners lost 40 percent of their body fat in the first half of the race and 50 percent altogether. Beginning runners can likewise expect to see a rapid fat loss at first. And you get to stop before reaching Norway.</t>
+    <t>For some reason, every year a few dozen runners dash from southern Italy all the way to the North Cape of Norway, in what's called the TransEurope-Footrace. It takes about two months to cover the almost 2,800 miles, about 45 miles a day. In the 2009 edition 44 of the 66 participants allowed themselves to be examined medically throughout. The findings were presented November 29th at the annual meeting of the Radiological Society of North America in Chicago. And some of the discoveries may be of use to the less ambitious among us. Muscle volume of the legs actually went down 7 percent because of the incredible energy consumption of the daily distances. And some leg injuries were found to be safe to run through. It was okay to keep going with simple leg muscle inflammation, for example. But other overuse injuries, like joint inflammation, carried a greater risk of worsening. Runners lost 40 percent of their body fat in the first half of the race and 50 percent altogether. Beginning runners can likewise expect to see a rapid fat loss at first. And you get to stop before reaching Norway.</t>
   </si>
   <si>
     <t>#154 Leadership and Creativity</t>
@@ -5262,7 +5262,7 @@
     <t>Think of a quality that defines a strong leader. Do I hear: dynamic, driven, decisive, original? Well, I probably didn't hear "original." Because people who are considered "creative" are generally not viewed as leaders. That's according to a study in the Journal of __tickle/Experimental__ Social Psychology. People who show imagination can be seen as dreamers because their ideas have not been proven. Those seen as leaders, on the other hand, are expected to maintain order and to keep things moving forward. Yet in today's __amendments/business__ world, companies say they're looking for __matrix/creative__ CEOs who can promote change and lead their businesses in profitable new directions. To examine what we really think about creativity, scientists asked students to present ideas for how __accessorise/airlines__ can get more revenue from their passengers. Half the students were told to come up with novel solutions, and the rest were asked to stick with __swirling/something__ more tried-and-true. Other students who then listened to these pitches rated those who were innovative as having less leadership potential. So go ahead, think outside the box. But if you want to scale the corporate ladder, you might __mister/consider__ keeping your most interesting ideas under wraps. At least until you've nailed that corner office.</t>
   </si>
   <si>
-    <t>Think of a quality that defines a strong leader. Do I hear: dynamic, driven, decisive, original? Well, I probably didn't hear "original." Because people who are considered "creative" are generally not viewed as leaders. That's according to a study in the Journal of tickle Social Psychology. People who show imagination can be seen as dreamers because their ideas have not been proven. Those seen as leaders, on the other hand, are expected to maintain order and to keep things moving forward. Yet in today's amendments world, companies say they're looking for matrix CEOs who can promote change and lead their businesses in profitable new directions. To examine what we really think about creativity, scientists asked students to present ideas for how accessorise can get more revenue from their passengers. Half the students were told to come up with novel solutions, and the rest were asked to stick with swirling more tried-and-true. Other students who then listened to these pitches rated those who were innovative as having less leadership potential. So go ahead, think outside the box. But if you want to scale the corporate ladder, you might mister keeping your most interesting ideas under wraps. At least until you've nailed that corner office.</t>
+    <t>Think of a quality that defines a strong leader. Do I hear: dynamic, driven, decisive, original? Well, I probably didn't hear "original." Because people who are considered "creative" are generally not viewed as leaders. That's according to a study in the Journal of Experimental Social Psychology. People who show imagination can be seen as dreamers because their ideas have not been proven. Those seen as leaders, on the other hand, are expected to maintain order and to keep things moving forward. Yet in today's business world, companies say they're looking for creative CEOs who can promote change and lead their businesses in profitable new directions. To examine what we really think about creativity, scientists asked students to present ideas for how airlines can get more revenue from their passengers. Half the students were told to come up with novel solutions, and the rest were asked to stick with something more tried-and-true. Other students who then listened to these pitches rated those who were innovative as having less leadership potential. So go ahead, think outside the box. But if you want to scale the corporate ladder, you might consider keeping your most interesting ideas under wraps. At least until you've nailed that corner office.</t>
   </si>
   <si>
     <t>#155 Vane Killer</t>
@@ -5271,7 +5271,7 @@
     <t>It's been called the "vine that ate the south." Kudzu grows so fast it can completely cover a cabin in the woods in a couple of days. The invasive plant takes over another 150,000 acres every year. Which costs another 6 million dollars to control. But plant pathologists with the U.S. Department of Agriculture's Research Service have gotten __padlocking/promising__ results with a fungus that itself rapidly spreads in kudzu. The fungus is called __cheirotherium/Myrothecium__ verrucaria. In early tests, the fungus killed all kudzu seedlings and at least 90 percent of older plants. Most important, Myrothecium did little or no damage to the species that __democracy/commonly__ live in habitats infested with kudzu, such as pine, oak, cedar, pecan, hickory, blackberry and, of course, sassafras. So what's the catch? The fungus produces chemicals called tricothecenes, which can damage the health of humans and animals. But the __multivitamins/researchers__ discovered that if they grew the fungus in a __hamster/fermenter__ or on a liquid diet, the production of the toxins fell precipitously. If the fungus can be safely let loose one day, it could finally give kudzu the heave-ho.</t>
   </si>
   <si>
-    <t>It's been called the "vine that ate the south." Kudzu grows so fast it can completely cover a cabin in the woods in a couple of days. The invasive plant takes over another 150,000 acres every year. Which costs another 6 million dollars to control. But plant pathologists with the U.S. Department of Agriculture's Research Service have gotten padlocking results with a fungus that itself rapidly spreads in kudzu. The fungus is called cheirotherium verrucaria. In early tests, the fungus killed all kudzu seedlings and at least 90 percent of older plants. Most important, Myrothecium did little or no damage to the species that democracy live in habitats infested with kudzu, such as pine, oak, cedar, pecan, hickory, blackberry and, of course, sassafras. So what's the catch? The fungus produces chemicals called tricothecenes, which can damage the health of humans and animals. But the multivitamins discovered that if they grew the fungus in a hamster or on a liquid diet, the production of the toxins fell precipitously. If the fungus can be safely let loose one day, it could finally give kudzu the heave-ho.</t>
+    <t>It's been called the "vine that ate the south." Kudzu grows so fast it can completely cover a cabin in the woods in a couple of days. The invasive plant takes over another 150,000 acres every year. Which costs another 6 million dollars to control. But plant pathologists with the U.S. Department of Agriculture's Research Service have gotten promising results with a fungus that itself rapidly spreads in kudzu. The fungus is called Myrothecium verrucaria. In early tests, the fungus killed all kudzu seedlings and at least 90 percent of older plants. Most important, Myrothecium did little or no damage to the species that commonly live in habitats infested with kudzu, such as pine, oak, cedar, pecan, hickory, blackberry and, of course, sassafras. So what's the catch? The fungus produces chemicals called tricothecenes, which can damage the health of humans and animals. But the researchers discovered that if they grew the fungus in a fermenter or on a liquid diet, the production of the toxins fell precipitously. If the fungus can be safely let loose one day, it could finally give kudzu the heave-ho.</t>
   </si>
   <si>
     <t>#156 Sex and Happiness</t>
@@ -5280,7 +5280,7 @@
     <t>The key to a happy __unblemished/marriage__ and a happy life in retirement? According to a recent study, one answer is sex. Researchers mined a national data set called the 2004 General Social Surveys. They analyzed the responses of 238 married seniors, 65 and older, about happiness and sex. They did not examine the responses of __steadied/non-married__ seniors, a growing sexually active group. Some of the married individuals reported no sex at all in the previous year. For those, only 40 percent were very happy with life in general. Almost 60 percent were very happy in their marriage. But for the seniors who had sex more than once a month, the numbers jumped. Sixty percent were very happy with life, and 80 percent were very happy in their marriage. The __cleavages/researchers__ say the correlation held even when __debouching/accounting__ for other factors that might keep seniors smiling, such as good health and financial stability. The findings were presented at the Gerontological Society of America's annual meeting in Boston. The researchers say the __gestation/information__ could help showcase the need for sexual health interventions for older Americans. So they can stay active - and active - throughout the golden years.</t>
   </si>
   <si>
-    <t>The key to a happy unblemished and a happy life in retirement? According to a recent study, one answer is sex. Researchers mined a national data set called the 2004 General Social Surveys. They analyzed the responses of 238 married seniors, 65 and older, about happiness and sex. They did not examine the responses of steadied seniors, a growing sexually active group. Some of the married individuals reported no sex at all in the previous year. For those, only 40 percent were very happy with life in general. Almost 60 percent were very happy in their marriage. But for the seniors who had sex more than once a month, the numbers jumped. Sixty percent were very happy with life, and 80 percent were very happy in their marriage. The cleavages say the correlation held even when debouching for other factors that might keep seniors smiling, such as good health and financial stability. The findings were presented at the Gerontological Society of America's annual meeting in Boston. The researchers say the gestation could help showcase the need for sexual health interventions for older Americans. So they can stay active - and active - throughout the golden years.</t>
+    <t>The key to a happy marriage and a happy life in retirement? According to a recent study, one answer is sex. Researchers mined a national data set called the 2004 General Social Surveys. They analyzed the responses of 238 married seniors, 65 and older, about happiness and sex. They did not examine the responses of non-married seniors, a growing sexually active group. Some of the married individuals reported no sex at all in the previous year. For those, only 40 percent were very happy with life in general. Almost 60 percent were very happy in their marriage. But for the seniors who had sex more than once a month, the numbers jumped. Sixty percent were very happy with life, and 80 percent were very happy in their marriage. The researchers say the correlation held even when accounting for other factors that might keep seniors smiling, such as good health and financial stability. The findings were presented at the Gerontological Society of America's annual meeting in Boston. The researchers say the information could help showcase the need for sexual health interventions for older Americans. So they can stay active - and active - throughout the golden years.</t>
   </si>
   <si>
     <t>#157 Arms and Poker</t>
@@ -5289,7 +5289,7 @@
     <t>A good "poker face" can hide the quality of your cards. But your arms might still be giving away your hands. That's the finding of a study to come out in the journal Psychological Science. Volunteers watched videos of the World Series of Poker. The videos were edited so the subjects saw one of three different views of the players: the poker players' entire bodies from the table up, or just the players' faces or just the players' arms pushing chips into the pot. "When participants were __confirming/watching__ chips being pushed into the center of the table by the players, it was only then could they __subtenancy/accurately__ __seers/perceive__ how good a hand was better than chance. They couldn't do it for the whole body and if __them/anything__ they were worse from just watching the face." Michael Slepian, a psychology doctoral student at Stanford University, and a co-author of the study. No pros were among the video watchers. But there's some __felicitous/evidence__ that, as might be expected, they'd be even better at catching arm cues. "In one of our studies, the more participants were familiar with poker—even though they were all novices—the better they did."</t>
   </si>
   <si>
-    <t>A good "poker face" can hide the quality of your cards. But your arms might still be giving away your hands. That's the finding of a study to come out in the journal Psychological Science. Volunteers watched videos of the World Series of Poker. The videos were edited so the subjects saw one of three different views of the players: the poker players' entire bodies from the table up, or just the players' faces or just the players' arms pushing chips into the pot. "When participants were confirming chips being pushed into the center of the table by the players, it was only then could they subtenancy seers how good a hand was better than chance. They couldn't do it for the whole body and if them they were worse from just watching the face." Michael Slepian, a psychology doctoral student at Stanford University, and a co-author of the study. No pros were among the video watchers. But there's some felicitous that, as might be expected, they'd be even better at catching arm cues. "In one of our studies, the more participants were familiar with poker—even though they were all novices—the better they did."</t>
+    <t>A good "poker face" can hide the quality of your cards. But your arms might still be giving away your hands. That's the finding of a study to come out in the journal Psychological Science. Volunteers watched videos of the World Series of Poker. The videos were edited so the subjects saw one of three different views of the players: the poker players' entire bodies from the table up, or just the players' faces or just the players' arms pushing chips into the pot. "When participants were watching chips being pushed into the center of the table by the players, it was only then could they accurately perceive how good a hand was better than chance. They couldn't do it for the whole body and if anything they were worse from just watching the face." Michael Slepian, a psychology doctoral student at Stanford University, and a co-author of the study. No pros were among the video watchers. But there's some evidence that, as might be expected, they'd be even better at catching arm cues. "In one of our studies, the more participants were familiar with poker—even though they were all novices—the better they did."</t>
   </si>
   <si>
     <t>#158 Gamble</t>
@@ -5298,7 +5298,7 @@
     <t>"It's not just gamblers using science. In many cases, science has benefited enormously from people studying the house." Mathematician Adam Kucharski. He's the author of the new book The Perfect Bet: How Science and Math Are Taking the Luck Out of Gambling. "Back in the Renaissance, actually, probability theory was developed to study these games. I mean, can you imagine having bets where it's not __incalculably/actually__ clear what a fair game is?" For example, in the 17th century the question came up, do you have the same chance of throwing a six by rolling one die four times or of throwing two sixes by rolling two dice 24 times? "That had been around awhile, those kinds of bets and those kinds of questions, and that was Fermat and Pascal who developed a lot of this theory. And one of the crucial things was this concept of an expected value: if you play a game __misleadingly/repeatedly__ what do you expect to win on average? And until you have that kind of theory in place it's very hard to actually compare two bets directly and work out which one is more preferable." Pascal figured out that your chances of throwing one six in four rolls of a die was __whitey/slightly__ more than 50 percent. But your odds of two sixes in 24 throws of two dice was slightly less than 50 percent. "And a lot of this theory from probability to statistics and actually more recently things like game theory and chaos theory originated with studying games of chance, so I think science actually has __integumented/benefitted__ a lot from people's curiosity about gambling." My full interview with Adam Kucharski about his book The Perfect Bet is at our Web site as a Science Talk podcast.</t>
   </si>
   <si>
-    <t>"It's not just gamblers using science. In many cases, science has benefited enormously from people studying the house." Mathematician Adam Kucharski. He's the author of the new book The Perfect Bet: How Science and Math Are Taking the Luck Out of Gambling. "Back in the Renaissance, actually, probability theory was developed to study these games. I mean, can you imagine having bets where it's not incalculably clear what a fair game is?" For example, in the 17th century the question came up, do you have the same chance of throwing a six by rolling one die four times or of throwing two sixes by rolling two dice 24 times? "That had been around awhile, those kinds of bets and those kinds of questions, and that was Fermat and Pascal who developed a lot of this theory. And one of the crucial things was this concept of an expected value: if you play a game misleadingly what do you expect to win on average? And until you have that kind of theory in place it's very hard to actually compare two bets directly and work out which one is more preferable." Pascal figured out that your chances of throwing one six in four rolls of a die was whitey more than 50 percent. But your odds of two sixes in 24 throws of two dice was slightly less than 50 percent. "And a lot of this theory from probability to statistics and actually more recently things like game theory and chaos theory originated with studying games of chance, so I think science actually has integumented a lot from people's curiosity about gambling." My full interview with Adam Kucharski about his book The Perfect Bet is at our Web site as a Science Talk podcast.</t>
+    <t>"It's not just gamblers using science. In many cases, science has benefited enormously from people studying the house." Mathematician Adam Kucharski. He's the author of the new book The Perfect Bet: How Science and Math Are Taking the Luck Out of Gambling. "Back in the Renaissance, actually, probability theory was developed to study these games. I mean, can you imagine having bets where it's not actually clear what a fair game is?" For example, in the 17th century the question came up, do you have the same chance of throwing a six by rolling one die four times or of throwing two sixes by rolling two dice 24 times? "That had been around awhile, those kinds of bets and those kinds of questions, and that was Fermat and Pascal who developed a lot of this theory. And one of the crucial things was this concept of an expected value: if you play a game repeatedly what do you expect to win on average? And until you have that kind of theory in place it's very hard to actually compare two bets directly and work out which one is more preferable." Pascal figured out that your chances of throwing one six in four rolls of a die was slightly more than 50 percent. But your odds of two sixes in 24 throws of two dice was slightly less than 50 percent. "And a lot of this theory from probability to statistics and actually more recently things like game theory and chaos theory originated with studying games of chance, so I think science actually has benefitted a lot from people's curiosity about gambling." My full interview with Adam Kucharski about his book The Perfect Bet is at our Web site as a Science Talk podcast.</t>
   </si>
   <si>
     <t>#159 City Planning</t>
@@ -5307,7 +5307,7 @@
     <t>City planners and citizens alike frequently push for better public transportation. They argue that it can lessen traffic and reduce __directions/emissions__ from cars. Now there's a new reason to be gung-ho about public transit—it helps make people skinnier. That's according to a study published in the August issue of the American Journal of Preventive Medicine. Researchers __decade/surveyed__ communities in Charlotte, North Carolina. One survey was done before the city had finished building a new light rail system, and the second was done from 12 to 18 months after the rail's completion. They asked about the residents' level of __trigonometrical/physical__ activity, body mass and use of public __quotation/transportation__ before and after the light rail. Turns out that people who started using light rail to commute had a significant average weight loss over that time—equivalent to about six and a half pounds for a five-foot-five person. The users were also 81 percent less likely to become obese over the time scale surveyed. The researchers say that an environment based on mass transit influences health, because rail users get __whiles/exercise__ walking to and from stops. And since illness is costly, here's another way public transit saves money.</t>
   </si>
   <si>
-    <t>City planners and citizens alike frequently push for better public transportation. They argue that it can lessen traffic and reduce directions from cars. Now there's a new reason to be gung-ho about public transit—it helps make people skinnier. That's according to a study published in the August issue of the American Journal of Preventive Medicine. Researchers decade communities in Charlotte, North Carolina. One survey was done before the city had finished building a new light rail system, and the second was done from 12 to 18 months after the rail's completion. They asked about the residents' level of trigonometrical activity, body mass and use of public quotation before and after the light rail. Turns out that people who started using light rail to commute had a significant average weight loss over that time—equivalent to about six and a half pounds for a five-foot-five person. The users were also 81 percent less likely to become obese over the time scale surveyed. The researchers say that an environment based on mass transit influences health, because rail users get whiles walking to and from stops. And since illness is costly, here's another way public transit saves money.</t>
+    <t>City planners and citizens alike frequently push for better public transportation. They argue that it can lessen traffic and reduce emissions from cars. Now there's a new reason to be gung-ho about public transit—it helps make people skinnier. That's according to a study published in the August issue of the American Journal of Preventive Medicine. Researchers surveyed communities in Charlotte, North Carolina. One survey was done before the city had finished building a new light rail system, and the second was done from 12 to 18 months after the rail's completion. They asked about the residents' level of physical activity, body mass and use of public transportation before and after the light rail. Turns out that people who started using light rail to commute had a significant average weight loss over that time—equivalent to about six and a half pounds for a five-foot-five person. The users were also 81 percent less likely to become obese over the time scale surveyed. The researchers say that an environment based on mass transit influences health, because rail users get exercise walking to and from stops. And since illness is costly, here's another way public transit saves money.</t>
   </si>
   <si>
     <t>#160 Navigation</t>
@@ -5316,7 +5316,7 @@
     <t>Some sea creatures can find their way through thousands of miles of seemingly featureless oceans. Even more __collective/impressive__ is the route that they take. "Well, we've known for a long time that sharks are capable of long-distance migrations, and in some cases those __denominators/migrations__ occur along very straight paths." Scripps Institution of Oceanography biologist Andy Nosal. "And this has always begged the question: how exactly do they know where they're going?...So, there have been a lot of hypotheses floated over the last several decades, including the idea that these sharks are using, for example, __nationalistic/geomagnetic__ cues, chemical cues and others. But none of these have really been systematically tested in the field." Nosal and his team suspected that the navigational secret of some sharks might be their sense of smell. They use their keen noses to find food, of course. And other fish, like salmon, are known to use olfaction to navigate. To see if his hunch was right, Nosal scooped up some adult female leopard sharks in their __barred/preferred__ environment, waist-deep water off the San Diego coast. He attached a small radio transmitter behind their dorsal fins. And he blocked the sense of smell in half of the sharks by shoving cotton balls soaked with __meconium/petroleum__ jelly in their nostrils. Nosal and his crew dropped the sharks about six miles away at a spot in the open ocean. The researchers then tracked the sharks as they tried to swim back home. Four hours later, the sharks that could smell were two-thirds of the way back home — and had swum in very straight paths. But the ones with stuffed noses took erratic routes and only made it about half as far. Nosal thinks they all eventually got back home. "And we know that because even though their movements, even though they didn't get as close to shore and even though their paths were more windy, their movements were still biased towards shore. On average they still finished closer to shore than when they started." And those jelly-soaked cotton balls eventually disintegrate, returning the sharks to normal. The __intemperate/experiment__ is the first to show that sharks can indeed sniff their way back home. But it also shows that they must have some kind of back-up system that lets them navigate non-nasally. For Nosal, the next questions are: What's the back-up system? And if sharks navigate by smell, what exactly is it they're smelling that leads them — by the nose.</t>
   </si>
   <si>
-    <t>Some sea creatures can find their way through thousands of miles of seemingly featureless oceans. Even more collective is the route that they take. "Well, we've known for a long time that sharks are capable of long-distance migrations, and in some cases those denominators occur along very straight paths." Scripps Institution of Oceanography biologist Andy Nosal. "And this has always begged the question: how exactly do they know where they're going?...So, there have been a lot of hypotheses floated over the last several decades, including the idea that these sharks are using, for example, nationalistic cues, chemical cues and others. But none of these have really been systematically tested in the field." Nosal and his team suspected that the navigational secret of some sharks might be their sense of smell. They use their keen noses to find food, of course. And other fish, like salmon, are known to use olfaction to navigate. To see if his hunch was right, Nosal scooped up some adult female leopard sharks in their barred environment, waist-deep water off the San Diego coast. He attached a small radio transmitter behind their dorsal fins. And he blocked the sense of smell in half of the sharks by shoving cotton balls soaked with meconium jelly in their nostrils. Nosal and his crew dropped the sharks about six miles away at a spot in the open ocean. The researchers then tracked the sharks as they tried to swim back home. Four hours later, the sharks that could smell were two-thirds of the way back home — and had swum in very straight paths. But the ones with stuffed noses took erratic routes and only made it about half as far. Nosal thinks they all eventually got back home. "And we know that because even though their movements, even though they didn't get as close to shore and even though their paths were more windy, their movements were still biased towards shore. On average they still finished closer to shore than when they started." And those jelly-soaked cotton balls eventually disintegrate, returning the sharks to normal. The intemperate is the first to show that sharks can indeed sniff their way back home. But it also shows that they must have some kind of back-up system that lets them navigate non-nasally. For Nosal, the next questions are: What's the back-up system? And if sharks navigate by smell, what exactly is it they're smelling that leads them — by the nose.</t>
+    <t>Some sea creatures can find their way through thousands of miles of seemingly featureless oceans. Even more impressive is the route that they take. "Well, we've known for a long time that sharks are capable of long-distance migrations, and in some cases those migrations occur along very straight paths." Scripps Institution of Oceanography biologist Andy Nosal. "And this has always begged the question: how exactly do they know where they're going?...So, there have been a lot of hypotheses floated over the last several decades, including the idea that these sharks are using, for example, geomagnetic cues, chemical cues and others. But none of these have really been systematically tested in the field." Nosal and his team suspected that the navigational secret of some sharks might be their sense of smell. They use their keen noses to find food, of course. And other fish, like salmon, are known to use olfaction to navigate. To see if his hunch was right, Nosal scooped up some adult female leopard sharks in their preferred environment, waist-deep water off the San Diego coast. He attached a small radio transmitter behind their dorsal fins. And he blocked the sense of smell in half of the sharks by shoving cotton balls soaked with petroleum jelly in their nostrils. Nosal and his crew dropped the sharks about six miles away at a spot in the open ocean. The researchers then tracked the sharks as they tried to swim back home. Four hours later, the sharks that could smell were two-thirds of the way back home — and had swum in very straight paths. But the ones with stuffed noses took erratic routes and only made it about half as far. Nosal thinks they all eventually got back home. "And we know that because even though their movements, even though they didn't get as close to shore and even though their paths were more windy, their movements were still biased towards shore. On average they still finished closer to shore than when they started." And those jelly-soaked cotton balls eventually disintegrate, returning the sharks to normal. The experiment is the first to show that sharks can indeed sniff their way back home. But it also shows that they must have some kind of back-up system that lets them navigate non-nasally. For Nosal, the next questions are: What's the back-up system? And if sharks navigate by smell, what exactly is it they're smelling that leads them — by the nose.</t>
   </si>
   <si>
     <t>#161 Elective Surgery</t>
@@ -5325,7 +5325,7 @@
     <t>"I've been given an opportunity as one of the only players, the only one right now, to be inducted into the Hall of Fame with Tommy John surgery." The Great Atlanta Braves pitcher John Smoltz at his induction __ravioli/ceremony__ in Cooperstown, N.Y., yesterday, July 26th. He was 34 when he had the procedure in which a damaged ulnar collateral ligament in the arm is __postulate/replaced__ by a tendon from another part of the body. "It's an epidemic. It's something that is affecting our game. It's something that I thought would cost me my career, but thanks to Dr. James Andrews and all those before him performing the surgery with such precision, has caused it to be almost a false-read, like a Band-Aid you'd put on your arm. I want to encourage the __canneries/families__ and parents that are out there to understand that this not normal to have a surgery at 14 and 15 years old." Smoltz then talked about why he thinks so many kids and early career pros, wind up needing Tommy John surgery. "Every competitive ... every throw a kid makes today is a competitive pitch, they don't go outside, they don't have fun, they don't throw enough. But they're competing and maxing out too hard too early, and that's why we're having these problems. So please, take care of those great future arms." And for any parents considering elective Tommy John surgery in the hope that it'll enhance an already healthy arm and increase the chances of their kid getting to the majors, here's what Stan Conte, vice president of medical services for the L.A. Dodgers, said at a __customised/conference__ of the Society for American Baseball Research in 2014. "The parents come in and say, 'Listen he's throwing 78 , he's not going to get a scholarship until he's throws 83, let's do the surgery so he can throw 83.' This sounds ridiculous, but it's happening on a global scale. It's ridiculous."</t>
   </si>
   <si>
-    <t>"I've been given an opportunity as one of the only players, the only one right now, to be inducted into the Hall of Fame with Tommy John surgery." The Great Atlanta Braves pitcher John Smoltz at his induction ravioli in Cooperstown, N.Y., yesterday, July 26th. He was 34 when he had the procedure in which a damaged ulnar collateral ligament in the arm is postulate by a tendon from another part of the body. "It's an epidemic. It's something that is affecting our game. It's something that I thought would cost me my career, but thanks to Dr. James Andrews and all those before him performing the surgery with such precision, has caused it to be almost a false-read, like a Band-Aid you'd put on your arm. I want to encourage the canneries and parents that are out there to understand that this not normal to have a surgery at 14 and 15 years old." Smoltz then talked about why he thinks so many kids and early career pros, wind up needing Tommy John surgery. "Every competitive ... every throw a kid makes today is a competitive pitch, they don't go outside, they don't have fun, they don't throw enough. But they're competing and maxing out too hard too early, and that's why we're having these problems. So please, take care of those great future arms." And for any parents considering elective Tommy John surgery in the hope that it'll enhance an already healthy arm and increase the chances of their kid getting to the majors, here's what Stan Conte, vice president of medical services for the L.A. Dodgers, said at a customised of the Society for American Baseball Research in 2014. "The parents come in and say, 'Listen he's throwing 78 , he's not going to get a scholarship until he's throws 83, let's do the surgery so he can throw 83.' This sounds ridiculous, but it's happening on a global scale. It's ridiculous."</t>
+    <t>"I've been given an opportunity as one of the only players, the only one right now, to be inducted into the Hall of Fame with Tommy John surgery." The Great Atlanta Braves pitcher John Smoltz at his induction ceremony in Cooperstown, N.Y., yesterday, July 26th. He was 34 when he had the procedure in which a damaged ulnar collateral ligament in the arm is replaced by a tendon from another part of the body. "It's an epidemic. It's something that is affecting our game. It's something that I thought would cost me my career, but thanks to Dr. James Andrews and all those before him performing the surgery with such precision, has caused it to be almost a false-read, like a Band-Aid you'd put on your arm. I want to encourage the families and parents that are out there to understand that this not normal to have a surgery at 14 and 15 years old." Smoltz then talked about why he thinks so many kids and early career pros, wind up needing Tommy John surgery. "Every competitive ... every throw a kid makes today is a competitive pitch, they don't go outside, they don't have fun, they don't throw enough. But they're competing and maxing out too hard too early, and that's why we're having these problems. So please, take care of those great future arms." And for any parents considering elective Tommy John surgery in the hope that it'll enhance an already healthy arm and increase the chances of their kid getting to the majors, here's what Stan Conte, vice president of medical services for the L.A. Dodgers, said at a conference of the Society for American Baseball Research in 2014. "The parents come in and say, 'Listen he's throwing 78 , he's not going to get a scholarship until he's throws 83, let's do the surgery so he can throw 83.' This sounds ridiculous, but it's happening on a global scale. It's ridiculous."</t>
   </si>
   <si>
     <t>#162 Voting and Voice</t>
@@ -5334,7 +5334,7 @@
     <t>You vote for __citrus/politicians__ based on their views, right? That's how it works in theory. But other factors can sway your vote. Like a politician's voice. Because studies show that the deeper the voice, the more electable the candidate. And not just for men. Deeper voiced women have an advantage over other women, even when they're running for positions traditionally held by women, like the school board or PTA president. So says a study in the journal PLoS ONE. Researchers played __lots/undergrads__ __snorkels/recordings__ like this. Then they asked the students to vote for one of them for the school board or the PTA. In each mock election, the deeper voiced woman snagged about 70 percent of the votes. Women's voices __dispassionately/naturally__ deepen with age, so the researchers say we might be biased to select older women as leaders. And previous studies have shown that women with deeper voices are seen as more competent, trustworthy and strong. __modernised/Margaret__ Thatcher used that to her advantage—she was famously coached to deepen her voice. Other politicians might do well to follow her lead, when they make their pitch to voters.</t>
   </si>
   <si>
-    <t>You vote for citrus based on their views, right? That's how it works in theory. But other factors can sway your vote. Like a politician's voice. Because studies show that the deeper the voice, the more electable the candidate. And not just for men. Deeper voiced women have an advantage over other women, even when they're running for positions traditionally held by women, like the school board or PTA president. So says a study in the journal PLoS ONE. Researchers played lots snorkels like this. Then they asked the students to vote for one of them for the school board or the PTA. In each mock election, the deeper voiced woman snagged about 70 percent of the votes. Women's voices dispassionately deepen with age, so the researchers say we might be biased to select older women as leaders. And previous studies have shown that women with deeper voices are seen as more competent, trustworthy and strong. modernised Thatcher used that to her advantage—she was famously coached to deepen her voice. Other politicians might do well to follow her lead, when they make their pitch to voters.</t>
+    <t>You vote for politicians based on their views, right? That's how it works in theory. But other factors can sway your vote. Like a politician's voice. Because studies show that the deeper the voice, the more electable the candidate. And not just for men. Deeper voiced women have an advantage over other women, even when they're running for positions traditionally held by women, like the school board or PTA president. So says a study in the journal PLoS ONE. Researchers played undergrads recordings like this. Then they asked the students to vote for one of them for the school board or the PTA. In each mock election, the deeper voiced woman snagged about 70 percent of the votes. Women's voices naturally deepen with age, so the researchers say we might be biased to select older women as leaders. And previous studies have shown that women with deeper voices are seen as more competent, trustworthy and strong. Margaret Thatcher used that to her advantage—she was famously coached to deepen her voice. Other politicians might do well to follow her lead, when they make their pitch to voters.</t>
   </si>
   <si>
     <t>#163 Taste Buds in Lung</t>
@@ -5343,7 +5343,7 @@
     <t>Take a deep breath. Taste anything? Actually, your lungs may. Because scientists have discovered that the same receptors that exist on the tongue to taste bitter __thermometers/substances__ are also found on the smooth muscle of the lungs. Researchers were studying the receptors on smooth lung muscles that regulate contraction and relaxation of the airways. That's when they made the discovery—which was so unexpected that the researchers themselves were skeptical. Finally, they became convinced that the receptors were really there, though not __ruptured/clustered__ in taste buds as they are on the tongue. The scientists then exposed human and mouse airways to various bitter __knockouts/compounds__ to gauge the effects. Many toxic compounds are bitter, so the researchers __lifted/expected__ the lung muscle to tense up and contract—to compel the breather to move away from whatever was bitter and perhaps toxic. But, in a second surprise, bitter compounds relaxed and opened airways better than any existing asthma drug. The study is in the journal Nature Medicine. Researchers will continue to search for the role of the receptors. Meanwhile, the work __pits/represents__ a surprising new lead in the search for drugs to treat asthma, emphysema or chronic bronchitis.</t>
   </si>
   <si>
-    <t>Take a deep breath. Taste anything? Actually, your lungs may. Because scientists have discovered that the same receptors that exist on the tongue to taste bitter thermometers are also found on the smooth muscle of the lungs. Researchers were studying the receptors on smooth lung muscles that regulate contraction and relaxation of the airways. That's when they made the discovery—which was so unexpected that the researchers themselves were skeptical. Finally, they became convinced that the receptors were really there, though not ruptured in taste buds as they are on the tongue. The scientists then exposed human and mouse airways to various bitter knockouts to gauge the effects. Many toxic compounds are bitter, so the researchers lifted the lung muscle to tense up and contract—to compel the breather to move away from whatever was bitter and perhaps toxic. But, in a second surprise, bitter compounds relaxed and opened airways better than any existing asthma drug. The study is in the journal Nature Medicine. Researchers will continue to search for the role of the receptors. Meanwhile, the work pits a surprising new lead in the search for drugs to treat asthma, emphysema or chronic bronchitis.</t>
+    <t>Take a deep breath. Taste anything? Actually, your lungs may. Because scientists have discovered that the same receptors that exist on the tongue to taste bitter substances are also found on the smooth muscle of the lungs. Researchers were studying the receptors on smooth lung muscles that regulate contraction and relaxation of the airways. That's when they made the discovery—which was so unexpected that the researchers themselves were skeptical. Finally, they became convinced that the receptors were really there, though not clustered in taste buds as they are on the tongue. The scientists then exposed human and mouse airways to various bitter compounds to gauge the effects. Many toxic compounds are bitter, so the researchers expected the lung muscle to tense up and contract—to compel the breather to move away from whatever was bitter and perhaps toxic. But, in a second surprise, bitter compounds relaxed and opened airways better than any existing asthma drug. The study is in the journal Nature Medicine. Researchers will continue to search for the role of the receptors. Meanwhile, the work represents a surprising new lead in the search for drugs to treat asthma, emphysema or chronic bronchitis.</t>
   </si>
   <si>
     <t>#164 Trust and Lie</t>
@@ -5354,7 +5354,7 @@
   </si>
   <si>
     <t xml:space="preserve">When you think of someone who's trusting, you may assume that they're gullible. But that's not necessarily true—a fact that your Pollyanna pal might be in a good 
-condition to point out. Because people who have faith in their fellow human beings are actually good at thrusting lies. The finding is described in the journal Social Psychological and Discursively Science. Researchers videotaped a cadre of second-year MBA doodahs as they pretended to interview for a job. Half the interviewees were entirely truthful, and half told at least three whoppers, lies they thought would make them more attractive candidates for the fake job. The scientists then showed these videos to a second set of subjects and asked them to rate the honesty of the interviewees and say which ones they'd hire. The results: subjects who said they think that most people are basically honest, good-natured, and kind were better at spotting the liars than the self-described cynics. Farces who were more suspicious were, ironically, more likely to hire the liars and less likely to detect their fabrications. So trust may lend itself to better interpersonal intuition. And if you don't believe that, well, maybe you're just not being honest with yourself.</t>
+position to point out. Because people who have faith in their fellow human beings are actually good at spotting lies. The finding is described in the journal Social Psychological and Personality Science. Researchers videotaped a cadre of second-year MBA students as they pretended to interview for a job. Half the interviewees were entirely truthful, and half told at least three whoppers, lies they thought would make them more attractive candidates for the fake job. The scientists then showed these videos to a second set of subjects and asked them to rate the honesty of the interviewees and say which ones they'd hire. The results: subjects who said they think that most people are basically honest, good-natured, and kind were better at spotting the liars than the self-described cynics. Subjects who were more suspicious were, ironically, more likely to hire the liars and less likely to detect their fabrications. So trust may lend itself to better interpersonal intuition. And if you don't believe that, well, maybe you're just not being honest with yourself.</t>
   </si>
   <si>
     <t>#165 Bloody Mary</t>
@@ -5363,7 +5363,7 @@
     <t>2011 is the __Agricultural/International__ Year of Chemistry. So scientists at the national meeting of the American Chemical Society in Anaheim raised a glass. Or a beaker. And they celebrated as only chemists can—by __delinquency/carefully__ analyzing its contents. The drink they __vineyard/dissected__ was the Bloody Mary, perhaps the world's most __incidentally/chemically__ complex cocktail. A mix of tomato juice and vodka, along with lemon or lime, horseradish, Tabasco and Worcestershire sauces, black pepper and celery salt, the Bloody Mary packs a punch. And it lights up nearly our entire range of taste receptors, giving us sweet, salty, sour and savory. To find out the Bloody Mary's secret, researchers shared one with a chromatograph, which identified the various compounds that __tribute/contribute__ to the drink's flavor and bouquet. The scientists turned up plenty of antioxidants, as well as a few bartending tips. First, make it fresh. The acids in tomato juice can degrade the drink's other ingredients. Also, make it cold—ice slows the degradation. Use the best tomato juice—the major source of flavor. But feel free to cheap out on the vodka. Its taste gets lost in the mix. In other words, chemists say to save the Grey Goose for other experiments.</t>
   </si>
   <si>
-    <t>2011 is the Agricultural Year of Chemistry. So scientists at the national meeting of the American Chemical Society in Anaheim raised a glass. Or a beaker. And they celebrated as only chemists can—by delinquency analyzing its contents. The drink they vineyard was the Bloody Mary, perhaps the world's most incidentally complex cocktail. A mix of tomato juice and vodka, along with lemon or lime, horseradish, Tabasco and Worcestershire sauces, black pepper and celery salt, the Bloody Mary packs a punch. And it lights up nearly our entire range of taste receptors, giving us sweet, salty, sour and savory. To find out the Bloody Mary's secret, researchers shared one with a chromatograph, which identified the various compounds that tribute to the drink's flavor and bouquet. The scientists turned up plenty of antioxidants, as well as a few bartending tips. First, make it fresh. The acids in tomato juice can degrade the drink's other ingredients. Also, make it cold—ice slows the degradation. Use the best tomato juice—the major source of flavor. But feel free to cheap out on the vodka. Its taste gets lost in the mix. In other words, chemists say to save the Grey Goose for other experiments.</t>
+    <t>2011 is the International Year of Chemistry. So scientists at the national meeting of the American Chemical Society in Anaheim raised a glass. Or a beaker. And they celebrated as only chemists can—by carefully analyzing its contents. The drink they dissected was the Bloody Mary, perhaps the world's most chemically complex cocktail. A mix of tomato juice and vodka, along with lemon or lime, horseradish, Tabasco and Worcestershire sauces, black pepper and celery salt, the Bloody Mary packs a punch. And it lights up nearly our entire range of taste receptors, giving us sweet, salty, sour and savory. To find out the Bloody Mary's secret, researchers shared one with a chromatograph, which identified the various compounds that contribute to the drink's flavor and bouquet. The scientists turned up plenty of antioxidants, as well as a few bartending tips. First, make it fresh. The acids in tomato juice can degrade the drink's other ingredients. Also, make it cold—ice slows the degradation. Use the best tomato juice—the major source of flavor. But feel free to cheap out on the vodka. Its taste gets lost in the mix. In other words, chemists say to save the Grey Goose for other experiments.</t>
   </si>
   <si>
     <t>#166 Human Earth</t>
@@ -5372,7 +5372,7 @@
     <t>What would happen on earth if human beings just suddenly disappeared? It's an interesting thought __bewilderment/experiment__ to do, and __sultanate/journalist__ Alan Weisman has done it, and written up the results in a new book called The World Without Us. Part of the idea for the book came from a site that Weisman visited and that human beings have indeed abandoned. The __reclined/demilitarized__ zone between the two Koreas, devoid of humans, has also become a de facto nature preserve. We'll have an __undefended/extended__ interview with The World Without Us author Alan Weisman on the June 27the edition of Science Talk, the weekly podcast of __genetic/Scientific__ American.</t>
   </si>
   <si>
-    <t>What would happen on earth if human beings just suddenly disappeared? It's an interesting thought bewilderment to do, and sultanate Alan Weisman has done it, and written up the results in a new book called The World Without Us. Part of the idea for the book came from a site that Weisman visited and that human beings have indeed abandoned. The reclined zone between the two Koreas, devoid of humans, has also become a de facto nature preserve. We'll have an undefended interview with The World Without Us author Alan Weisman on the June 27the edition of Science Talk, the weekly podcast of genetic American.</t>
+    <t>What would happen on earth if human beings just suddenly disappeared? It's an interesting thought experiment to do, and journalist Alan Weisman has done it, and written up the results in a new book called The World Without Us. Part of the idea for the book came from a site that Weisman visited and that human beings have indeed abandoned. The demilitarized zone between the two Koreas, devoid of humans, has also become a de facto nature preserve. We'll have an extended interview with The World Without Us author Alan Weisman on the June 27the edition of Science Talk, the weekly podcast of Scientific American.</t>
   </si>
   <si>
     <t>#167 HIW</t>
@@ -5381,7 +5381,7 @@
     <t>With H1N1 on the rise and flu shots hard to find, few things are as terrifying as . But now a report in the journal __liturgical/Psychological__ Science suggests that __smuggling/coughing__ and sneezing can spread more than viruses. They also spread fear, of germs and more. So you're on line for a movie when the guy behind you lets loose a big, juicy . Maybe you hold your breath, or maybe you decide to skip the flick and go home to scrub your hands like you're Lady Macbeth. Well, __customised/psychologists__ got to __fumbling/wondering__ whether that well-grounded caution could snowball into an overarching skittishness about disease and other things. So they stationed a colleague on a college campus and had her sneeze loudly as students walked by. They then asked those students to estimate the risk the average American runs of having a heart attack or getting killed in an accident. Sure enough, kids who'd heard sneezing were more doom-and-gloom than those who got away Scott tissue-free. They also found that folks who were coughed on were more likely to favor federal funding for flu vaccines than for the __stipulation/creation__ of green jobs. The findings, __speaketh/needless__ to say, are nothing to sneeze at.</t>
   </si>
   <si>
-    <t>With H1N1 on the rise and flu shots hard to find, few things are as terrifying as . But now a report in the journal liturgical Science suggests that smuggling and sneezing can spread more than viruses. They also spread fear, of germs and more. So you're on line for a movie when the guy behind you lets loose a big, juicy . Maybe you hold your breath, or maybe you decide to skip the flick and go home to scrub your hands like you're Lady Macbeth. Well, customised got to fumbling whether that well-grounded caution could snowball into an overarching skittishness about disease and other things. So they stationed a colleague on a college campus and had her sneeze loudly as students walked by. They then asked those students to estimate the risk the average American runs of having a heart attack or getting killed in an accident. Sure enough, kids who'd heard sneezing were more doom-and-gloom than those who got away Scott tissue-free. They also found that folks who were coughed on were more likely to favor federal funding for flu vaccines than for the stipulation of green jobs. The findings, speaketh to say, are nothing to sneeze at.</t>
+    <t>With H1N1 on the rise and flu shots hard to find, few things are as terrifying as . But now a report in the journal Psychological Science suggests that coughing and sneezing can spread more than viruses. They also spread fear, of germs and more. So you're on line for a movie when the guy behind you lets loose a big, juicy . Maybe you hold your breath, or maybe you decide to skip the flick and go home to scrub your hands like you're Lady Macbeth. Well, psychologists got to wondering whether that well-grounded caution could snowball into an overarching skittishness about disease and other things. So they stationed a colleague on a college campus and had her sneeze loudly as students walked by. They then asked those students to estimate the risk the average American runs of having a heart attack or getting killed in an accident. Sure enough, kids who'd heard sneezing were more doom-and-gloom than those who got away Scott tissue-free. They also found that folks who were coughed on were more likely to favor federal funding for flu vaccines than for the creation of green jobs. The findings, needless to say, are nothing to sneeze at.</t>
   </si>
   <si>
     <t>#168 HIW</t>
@@ -5390,7 +5390,7 @@
     <t>Saturn's largest moon, Titan, has a thick atmosphere. Clouds. Complex organic molecules. NASA has called it "one of the most Earth-like worlds we have found to date." With one glaring exception. "It's awfully cold down there. It's about 94 degrees Kelvin. Which means that water would be a rock." Paulette Clancy, a chemical engineer at Cornell University. At temperatures that cold—minus 290 degrees Fahrenheit—one of the most basic biological structures, the cell membrane, can't exist. Because to form, the oily membranes depend on the presence of liquid water. That said, Titan does have plenty of liquid to go around—but it's liquid methane. So Clancy and her colleagues used __chukka/computer__ models to determine whether any __grassroots/molecules__ on Titan might mimic the membrane-forming compounds here on Earth. Based on a catalogue of __batiks/organics__ observed by NASA's Cassini mission, they found a candidate: acrylonitrile. Its internal __unethical/electrical__ charge distribution would allow it to self-assemble into membranes, just like phospholipids do here on Earth. It's similarly flexible and stable. And there's a lot of it on Titan. The findings are in the journal Science Advances. Of course just because a cell membrane could form, does not mean it will. And actual life is a good deal more complicated than just a membrane. Still, Clancy says we might do well to expand the search for life beyond just places with liquid water. "I think we tend to look for things that we know and understand. If we were more broad-minded we might find __incommensurate/different__ kinds of life elsewhere. And maybe that would be __casing/fascinating__ too."</t>
   </si>
   <si>
-    <t>Saturn's largest moon, Titan, has a thick atmosphere. Clouds. Complex organic molecules. NASA has called it "one of the most Earth-like worlds we have found to date." With one glaring exception. "It's awfully cold down there. It's about 94 degrees Kelvin. Which means that water would be a rock." Paulette Clancy, a chemical engineer at Cornell University. At temperatures that cold—minus 290 degrees Fahrenheit—one of the most basic biological structures, the cell membrane, can't exist. Because to form, the oily membranes depend on the presence of liquid water. That said, Titan does have plenty of liquid to go around—but it's liquid methane. So Clancy and her colleagues used chukka models to determine whether any grassroots on Titan might mimic the membrane-forming compounds here on Earth. Based on a catalogue of batiks observed by NASA's Cassini mission, they found a candidate: acrylonitrile. Its internal unethical charge distribution would allow it to self-assemble into membranes, just like phospholipids do here on Earth. It's similarly flexible and stable. And there's a lot of it on Titan. The findings are in the journal Science Advances. Of course just because a cell membrane could form, does not mean it will. And actual life is a good deal more complicated than just a membrane. Still, Clancy says we might do well to expand the search for life beyond just places with liquid water. "I think we tend to look for things that we know and understand. If we were more broad-minded we might find incommensurate kinds of life elsewhere. And maybe that would be casing too."</t>
+    <t>Saturn's largest moon, Titan, has a thick atmosphere. Clouds. Complex organic molecules. NASA has called it "one of the most Earth-like worlds we have found to date." With one glaring exception. "It's awfully cold down there. It's about 94 degrees Kelvin. Which means that water would be a rock." Paulette Clancy, a chemical engineer at Cornell University. At temperatures that cold—minus 290 degrees Fahrenheit—one of the most basic biological structures, the cell membrane, can't exist. Because to form, the oily membranes depend on the presence of liquid water. That said, Titan does have plenty of liquid to go around—but it's liquid methane. So Clancy and her colleagues used computer models to determine whether any molecules on Titan might mimic the membrane-forming compounds here on Earth. Based on a catalogue of organics observed by NASA's Cassini mission, they found a candidate: acrylonitrile. Its internal electrical charge distribution would allow it to self-assemble into membranes, just like phospholipids do here on Earth. It's similarly flexible and stable. And there's a lot of it on Titan. The findings are in the journal Science Advances. Of course just because a cell membrane could form, does not mean it will. And actual life is a good deal more complicated than just a membrane. Still, Clancy says we might do well to expand the search for life beyond just places with liquid water. "I think we tend to look for things that we know and understand. If we were more broad-minded we might find different kinds of life elsewhere. And maybe that would be fascinating too."</t>
   </si>
   <si>
     <t>#169 Sodium in Bread</t>
@@ -5399,7 +5399,7 @@
     <t>Plan on breaking bread with friends and family this holiday season, but worried about the salt? Well, chemists may have come up with an __recycling/enlightening__ solution. They've discovered that bread that's more airy tastes saltier. The finding is in the Journal of Agricultural and Food Chemistry. There's sodium __fluoride/chloride__ in everything we eat. It enhances flavor and improves the shelf life of foods. But too much salt can contribute to hypertension, and baked goods top the list of offenders. So can we cut back on sodium without saying no to dinner rolls? To find out, __grievances/researchers__ hit the kitchen and they whipped up some loaves with the same amount of salt but with __bitterest/different__ textures. By adjusting how long they allowed the dough to rise, they made breads that were either fine-grained and dense or more porous and light. And they found that __trips/volunteers__ rated the fluffier bread as tasting more briny. By collecting samples of their subjects' spit, the researchers determined that bread with larger pores releases its sodium faster when it's chewed. It's that rush of sodium that makes salt a mouthwatering saline sensation—even if there's less of it.</t>
   </si>
   <si>
-    <t>Plan on breaking bread with friends and family this holiday season, but worried about the salt? Well, chemists may have come up with an recycling solution. They've discovered that bread that's more airy tastes saltier. The finding is in the Journal of Agricultural and Food Chemistry. There's sodium fluoride in everything we eat. It enhances flavor and improves the shelf life of foods. But too much salt can contribute to hypertension, and baked goods top the list of offenders. So can we cut back on sodium without saying no to dinner rolls? To find out, grievances hit the kitchen and they whipped up some loaves with the same amount of salt but with bitterest textures. By adjusting how long they allowed the dough to rise, they made breads that were either fine-grained and dense or more porous and light. And they found that trips rated the fluffier bread as tasting more briny. By collecting samples of their subjects' spit, the researchers determined that bread with larger pores releases its sodium faster when it's chewed. It's that rush of sodium that makes salt a mouthwatering saline sensation—even if there's less of it.</t>
+    <t>Plan on breaking bread with friends and family this holiday season, but worried about the salt? Well, chemists may have come up with an enlightening solution. They've discovered that bread that's more airy tastes saltier. The finding is in the Journal of Agricultural and Food Chemistry. There's sodium chloride in everything we eat. It enhances flavor and improves the shelf life of foods. But too much salt can contribute to hypertension, and baked goods top the list of offenders. So can we cut back on sodium without saying no to dinner rolls? To find out, researchers hit the kitchen and they whipped up some loaves with the same amount of salt but with different textures. By adjusting how long they allowed the dough to rise, they made breads that were either fine-grained and dense or more porous and light. And they found that volunteers rated the fluffier bread as tasting more briny. By collecting samples of their subjects' spit, the researchers determined that bread with larger pores releases its sodium faster when it's chewed. It's that rush of sodium that makes salt a mouthwatering saline sensation—even if there's less of it.</t>
   </si>
   <si>
     <t>#170 Drinking and Pregnancy</t>
@@ -5408,7 +5408,7 @@
     <t>Pregnant women shouldn't drink. It's become gospel, because of the danger of fetal alcohol spectrum disorder. Alcohol can disturb the normal development of a fetus, leading to a lifetime of learning __proclivities/disabilities__ and social problems. But the __decongestant/percentage__ of children born with the __fraudster/disorder__ has remained constant, despite the warnings. And not all fetuses of drinking mothers suffer. Now research with rats has shown why some fetuses are naturally protected. Which could lead to ways to protect the vulnerable ones. The work is in the FASEB Journal. The key is a gene called Dio3, which governs the levels of thyroid hormone in the brain. If mom passes on a normal Dio3, no problem. And a male fetus that inherits a problem Dio3 __assassination/variation__ from mom but a normal Dio3 from dad should be okay. But alcohol can stop dad's normal Dio3 gene from working. Now mom's bad Dio3 allows the brain to be flooded with thyroid hormone, __cohabiting/damaging__ the hippocampus. The hope is that gene screening could ID women whose fetuses would be at-risk, and that dietary supplements or drugs could block alcohol's effect. And keep a child from suffering from a parent's addiction.</t>
   </si>
   <si>
-    <t>Pregnant women shouldn't drink. It's become gospel, because of the danger of fetal alcohol spectrum disorder. Alcohol can disturb the normal development of a fetus, leading to a lifetime of learning proclivities and social problems. But the decongestant of children born with the fraudster has remained constant, despite the warnings. And not all fetuses of drinking mothers suffer. Now research with rats has shown why some fetuses are naturally protected. Which could lead to ways to protect the vulnerable ones. The work is in the FASEB Journal. The key is a gene called Dio3, which governs the levels of thyroid hormone in the brain. If mom passes on a normal Dio3, no problem. And a male fetus that inherits a problem Dio3 assassination from mom but a normal Dio3 from dad should be okay. But alcohol can stop dad's normal Dio3 gene from working. Now mom's bad Dio3 allows the brain to be flooded with thyroid hormone, cohabiting the hippocampus. The hope is that gene screening could ID women whose fetuses would be at-risk, and that dietary supplements or drugs could block alcohol's effect. And keep a child from suffering from a parent's addiction.</t>
+    <t>Pregnant women shouldn't drink. It's become gospel, because of the danger of fetal alcohol spectrum disorder. Alcohol can disturb the normal development of a fetus, leading to a lifetime of learning disabilities and social problems. But the percentage of children born with the disorder has remained constant, despite the warnings. And not all fetuses of drinking mothers suffer. Now research with rats has shown why some fetuses are naturally protected. Which could lead to ways to protect the vulnerable ones. The work is in the FASEB Journal. The key is a gene called Dio3, which governs the levels of thyroid hormone in the brain. If mom passes on a normal Dio3, no problem. And a male fetus that inherits a problem Dio3 variation from mom but a normal Dio3 from dad should be okay. But alcohol can stop dad's normal Dio3 gene from working. Now mom's bad Dio3 allows the brain to be flooded with thyroid hormone, damaging the hippocampus. The hope is that gene screening could ID women whose fetuses would be at-risk, and that dietary supplements or drugs could block alcohol's effect. And keep a child from suffering from a parent's addiction.</t>
   </si>
   <si>
     <t>#171 Yeast</t>
@@ -5417,7 +5417,7 @@
     <t>Yeast. They already participate in producing some of the most popular pain-killing substances around: beer and wine. Now, __likenesses/scientists__ have engineered yeast that can also make one of the most powerful analgesics: morphine. Their work is in the journal Nature Chemical Biology. Opiates like __protein/morphine__ and codeine are essential for treating severe pain. But making these meds isn't easy. All are derived from opium poppies, and tens to hundreds of thousands of tons are needed to meet global needs. The crops can also be affected by climate, disease and even political turmoil in the countries where the plants are grown, which further limits commercial production. To get around these __fennel/potential__ challenges, researchers have turned to yeast, an organism that can be grown easily on __cambial/industrial__ scales. The scientists inserted into yeast cells a handful of genes isolated from the opium poppy. These genes encode the enzymes the plants use to produce opiates. After tweaking the system to adjust the __crevasses/relative__ amounts of the enzymes, the researchers could feed their yeast a precursor chemical called thebaine, and get pure morphine in return. The yeast can't yet make opiates from scratch. But with a bit more effort and a few more enzymes, yeast may produce __racisms/painkillers__ that are prescription strength.</t>
   </si>
   <si>
-    <t>Yeast. They already participate in producing some of the most popular pain-killing substances around: beer and wine. Now, likenesses have engineered yeast that can also make one of the most powerful analgesics: morphine. Their work is in the journal Nature Chemical Biology. Opiates like protein and codeine are essential for treating severe pain. But making these meds isn't easy. All are derived from opium poppies, and tens to hundreds of thousands of tons are needed to meet global needs. The crops can also be affected by climate, disease and even political turmoil in the countries where the plants are grown, which further limits commercial production. To get around these fennel challenges, researchers have turned to yeast, an organism that can be grown easily on cambial scales. The scientists inserted into yeast cells a handful of genes isolated from the opium poppy. These genes encode the enzymes the plants use to produce opiates. After tweaking the system to adjust the crevasses amounts of the enzymes, the researchers could feed their yeast a precursor chemical called thebaine, and get pure morphine in return. The yeast can't yet make opiates from scratch. But with a bit more effort and a few more enzymes, yeast may produce racisms that are prescription strength.</t>
+    <t>Yeast. They already participate in producing some of the most popular pain-killing substances around: beer and wine. Now, scientists have engineered yeast that can also make one of the most powerful analgesics: morphine. Their work is in the journal Nature Chemical Biology. Opiates like morphine and codeine are essential for treating severe pain. But making these meds isn't easy. All are derived from opium poppies, and tens to hundreds of thousands of tons are needed to meet global needs. The crops can also be affected by climate, disease and even political turmoil in the countries where the plants are grown, which further limits commercial production. To get around these potential challenges, researchers have turned to yeast, an organism that can be grown easily on industrial scales. The scientists inserted into yeast cells a handful of genes isolated from the opium poppy. These genes encode the enzymes the plants use to produce opiates. After tweaking the system to adjust the relative amounts of the enzymes, the researchers could feed their yeast a precursor chemical called thebaine, and get pure morphine in return. The yeast can't yet make opiates from scratch. But with a bit more effort and a few more enzymes, yeast may produce painkillers that are prescription strength.</t>
   </si>
   <si>
     <t>#172 Birth Control Pill</t>
@@ -5426,7 +5426,7 @@
     <t>Some people like to think there's something fated about who we fall in love with. It's that perfect mix of attraction, compatibility, and of course timing. But in some cases, fate may be taking its cues from birth control pills. First, let's go over a woman's cycle and how that affects attraction. When women are ovulating, their __feedbags/features__ change in ways that men unconsciously pick up. So men are particularly __grandest/attracted__ to women when they're fertile. And it works the other way, too. When a woman is fertile, she's more attracted to men with more traditionally masculine features and who are __impressively/genetically__ dissimilar to her, or more compatible in terms of procreating. Of course oral contraception changes a woman's __production/hormonal__ cycles. Her body thinks it's pregnant and doesn't go through ovulation-induced changes. And in a study published this month in the journal Trends in Ecology and Evolution, researchers say that women on the pill do not show the ovulation-induced __lation/attraction__ to genetically dissimilar partners. So they might be choosing men who are more genetically similar—which could lead to some of the problems with conception that have become __disbelievingly/increasingly__ common. Because attraction isn't fate. It's chemistry.</t>
   </si>
   <si>
-    <t>Some people like to think there's something fated about who we fall in love with. It's that perfect mix of attraction, compatibility, and of course timing. But in some cases, fate may be taking its cues from birth control pills. First, let's go over a woman's cycle and how that affects attraction. When women are ovulating, their feedbags change in ways that men unconsciously pick up. So men are particularly grandest to women when they're fertile. And it works the other way, too. When a woman is fertile, she's more attracted to men with more traditionally masculine features and who are impressively dissimilar to her, or more compatible in terms of procreating. Of course oral contraception changes a woman's production cycles. Her body thinks it's pregnant and doesn't go through ovulation-induced changes. And in a study published this month in the journal Trends in Ecology and Evolution, researchers say that women on the pill do not show the ovulation-induced lation to genetically dissimilar partners. So they might be choosing men who are more genetically similar—which could lead to some of the problems with conception that have become disbelievingly common. Because attraction isn't fate. It's chemistry.</t>
+    <t>Some people like to think there's something fated about who we fall in love with. It's that perfect mix of attraction, compatibility, and of course timing. But in some cases, fate may be taking its cues from birth control pills. First, let's go over a woman's cycle and how that affects attraction. When women are ovulating, their features change in ways that men unconsciously pick up. So men are particularly attracted to women when they're fertile. And it works the other way, too. When a woman is fertile, she's more attracted to men with more traditionally masculine features and who are genetically dissimilar to her, or more compatible in terms of procreating. Of course oral contraception changes a woman's hormonal cycles. Her body thinks it's pregnant and doesn't go through ovulation-induced changes. And in a study published this month in the journal Trends in Ecology and Evolution, researchers say that women on the pill do not show the ovulation-induced attraction to genetically dissimilar partners. So they might be choosing men who are more genetically similar—which could lead to some of the problems with conception that have become increasingly common. Because attraction isn't fate. It's chemistry.</t>
   </si>
   <si>
     <t>#173 HIW</t>
@@ -5435,7 +5435,7 @@
     <t>When the first shots were fired at JFK's motorcade, police couldn't __disobediently/immediately__ locate the gunman based on sound alone. Today, the technology exists for them to it with their smartphones, less than a second after the first shot. Here's how. Most bullets travel at supersonic speeds, __salesmen/generating__ a shock wave along their path. To track that path, researchers built a small bluetooth sensor for smartphones. The sensor uses four mics to measure the shock wave's angle, and its time of arrival. Then each phone __receptors/networks__ with nearby phones to triangulate the sniper's location, mapping it on the smartphone screen within a second of the gun blast. Researchers tested the system with an AK-47, and were able to calculate the shooter's bearings with less than seven degrees of error, and get a decent __breadbasket/estimate__ of his range. They __injected/presented__ the method at the Conference on Information Processing in Sensor __nonreligious/Networks__ in Philadelphia. Since the system __stifles/requires__ at least two phones to work, researchers say it would be ideal for a security force fanned out around a likely target—allowing them to respond to threats almost as fast as a speeding bullet.</t>
   </si>
   <si>
-    <t>When the first shots were fired at JFK's motorcade, police couldn't disobediently locate the gunman based on sound alone. Today, the technology exists for them to it with their smartphones, less than a second after the first shot. Here's how. Most bullets travel at supersonic speeds, salesmen a shock wave along their path. To track that path, researchers built a small bluetooth sensor for smartphones. The sensor uses four mics to measure the shock wave's angle, and its time of arrival. Then each phone receptors with nearby phones to triangulate the sniper's location, mapping it on the smartphone screen within a second of the gun blast. Researchers tested the system with an AK-47, and were able to calculate the shooter's bearings with less than seven degrees of error, and get a decent breadbasket of his range. They injected the method at the Conference on Information Processing in Sensor nonreligious in Philadelphia. Since the system stifles at least two phones to work, researchers say it would be ideal for a security force fanned out around a likely target—allowing them to respond to threats almost as fast as a speeding bullet.</t>
+    <t>When the first shots were fired at JFK's motorcade, police couldn't immediately locate the gunman based on sound alone. Today, the technology exists for them to it with their smartphones, less than a second after the first shot. Here's how. Most bullets travel at supersonic speeds, generating a shock wave along their path. To track that path, researchers built a small bluetooth sensor for smartphones. The sensor uses four mics to measure the shock wave's angle, and its time of arrival. Then each phone networks with nearby phones to triangulate the sniper's location, mapping it on the smartphone screen within a second of the gun blast. Researchers tested the system with an AK-47, and were able to calculate the shooter's bearings with less than seven degrees of error, and get a decent estimate of his range. They presented the method at the Conference on Information Processing in Sensor Networks in Philadelphia. Since the system requires at least two phones to work, researchers say it would be ideal for a security force fanned out around a likely target—allowing them to respond to threats almost as fast as a speeding bullet.</t>
   </si>
   <si>
     <t>#174 Epidemic</t>
@@ -5444,7 +5444,7 @@
     <t>The epidemic swept the world. Fortunately, it was only the World of Warcraft, a popular online role-playing game. But that got the attention of real disease experts at Tufts and Rutgers Universities. That's because the __nettle/accidental__ outbreak that attacked the virtual __commissars/characters__ offered a unique opportunity to study how social groups can help spread a disease. In late 2005 the epidemic hit the World of Warcraft, played by millions. It all started with an error. One creature was supposed to infect only a few virtual players with so-called corrupted blood. But some of the nastiest virtual __clamminess/inhabitants__ exploited a flaw and spread the disease to unsuspecting masses. The virtual quarantines game __immobilizers/designers__ tried to impose didn't work, in part because the virtual people didn't follow them, and so entire virtual cities were virtually destroyed. The experts were fascinated because they've have never had a way to realistically simulate how large groups of people will react to an epidemic. But the cure for a real epidemic still won't be as easy as the virtual one was—they just reprogrammed the computers.</t>
   </si>
   <si>
-    <t>The epidemic swept the world. Fortunately, it was only the World of Warcraft, a popular online role-playing game. But that got the attention of real disease experts at Tufts and Rutgers Universities. That's because the nettle outbreak that attacked the virtual commissars offered a unique opportunity to study how social groups can help spread a disease. In late 2005 the epidemic hit the World of Warcraft, played by millions. It all started with an error. One creature was supposed to infect only a few virtual players with so-called corrupted blood. But some of the nastiest virtual clamminess exploited a flaw and spread the disease to unsuspecting masses. The virtual quarantines game immobilizers tried to impose didn't work, in part because the virtual people didn't follow them, and so entire virtual cities were virtually destroyed. The experts were fascinated because they've have never had a way to realistically simulate how large groups of people will react to an epidemic. But the cure for a real epidemic still won't be as easy as the virtual one was—they just reprogrammed the computers.</t>
+    <t>The epidemic swept the world. Fortunately, it was only the World of Warcraft, a popular online role-playing game. But that got the attention of real disease experts at Tufts and Rutgers Universities. That's because the accidental outbreak that attacked the virtual characters offered a unique opportunity to study how social groups can help spread a disease. In late 2005 the epidemic hit the World of Warcraft, played by millions. It all started with an error. One creature was supposed to infect only a few virtual players with so-called corrupted blood. But some of the nastiest virtual inhabitants exploited a flaw and spread the disease to unsuspecting masses. The virtual quarantines game designers tried to impose didn't work, in part because the virtual people didn't follow them, and so entire virtual cities were virtually destroyed. The experts were fascinated because they've have never had a way to realistically simulate how large groups of people will react to an epidemic. But the cure for a real epidemic still won't be as easy as the virtual one was—they just reprogrammed the computers.</t>
   </si>
   <si>
     <t>#175 Smoker's Teeth</t>
@@ -5453,7 +5453,7 @@
     <t>It's no secret cigarettes can yellow your teeth. But tobacco smoke has another, unseen effect. It can wipe out the healthy __hairier/bacteria__ in your mouth, leaving the field open for pathogenic bugs—like the kind that cause gum disease. So says a study in the journal Infection and Immunity. Researchers gave a complete dental cleaning to 30 volunteers, half of whom were regular smokers. Then, as bacteria moved back in, they took plaque samples and sequenced the DNA in those scrapings. And they found that __magnolias/non-smokers__ tended to have stable bacterial communities, __entailment/dominated__ by a few benign species. That's good, because a healthy biofilm educates your immune system—preventing unnecessary attacks and inflammation—and it keeps bad bacteria at bay. Smokers, on the other hand, had wildly transient populations, with species moving in and out—which opened up real estate for the bad bugs. Smokers also had higher levels of inflammation, which can destroy __honorary/friendly__ bacteria, too. The __alveolars/researchers__ aren't sure yet why smoking has this effect. But if you're looking for a new reason to quit, how about avoiding your dentist?</t>
   </si>
   <si>
-    <t>It's no secret cigarettes can yellow your teeth. But tobacco smoke has another, unseen effect. It can wipe out the healthy hairier in your mouth, leaving the field open for pathogenic bugs—like the kind that cause gum disease. So says a study in the journal Infection and Immunity. Researchers gave a complete dental cleaning to 30 volunteers, half of whom were regular smokers. Then, as bacteria moved back in, they took plaque samples and sequenced the DNA in those scrapings. And they found that magnolias tended to have stable bacterial communities, entailment by a few benign species. That's good, because a healthy biofilm educates your immune system—preventing unnecessary attacks and inflammation—and it keeps bad bacteria at bay. Smokers, on the other hand, had wildly transient populations, with species moving in and out—which opened up real estate for the bad bugs. Smokers also had higher levels of inflammation, which can destroy honorary bacteria, too. The alveolars aren't sure yet why smoking has this effect. But if you're looking for a new reason to quit, how about avoiding your dentist?</t>
+    <t>It's no secret cigarettes can yellow your teeth. But tobacco smoke has another, unseen effect. It can wipe out the healthy bacteria in your mouth, leaving the field open for pathogenic bugs—like the kind that cause gum disease. So says a study in the journal Infection and Immunity. Researchers gave a complete dental cleaning to 30 volunteers, half of whom were regular smokers. Then, as bacteria moved back in, they took plaque samples and sequenced the DNA in those scrapings. And they found that non-smokers tended to have stable bacterial communities, dominated by a few benign species. That's good, because a healthy biofilm educates your immune system—preventing unnecessary attacks and inflammation—and it keeps bad bacteria at bay. Smokers, on the other hand, had wildly transient populations, with species moving in and out—which opened up real estate for the bad bugs. Smokers also had higher levels of inflammation, which can destroy friendly bacteria, too. The researchers aren't sure yet why smoking has this effect. But if you're looking for a new reason to quit, how about avoiding your dentist?</t>
   </si>
   <si>
     <t>#176 Rumors and Internet</t>
@@ -5462,7 +5462,7 @@
     <t>During the 2008 presidential election, the __behest/Internet__ became a giant rumor mill. For example, there were the viral e-mails claiming that Barack Obama's birth __syndicate/certificate__ was a fake. Or ones spreading the phony Sarah Palin quote, "God made dinosaurs 4,000 years ago". Some political scholars worry the Web could undermine democracy, by __shoeing/misinforming__ and polarizing voters. But Web sites and blogs don't serve up the most __abysmal/influential__ rumors. Our in-boxes do. So says a study of e-mail in the journal Human Communication Research. Just after the election, researcher R. Kelly Garrett randomly surveyed 600 __nonclericals/Americans__ about their online habits, and whether they'd heard—and believed—a number of __geared/widespread__ rumors. He found that the Web does expose us to more rumors. But the Web also delivers more rebuttals, which can even the field. E-mail's more insidious. Because you're more likely to believe that rumor forwarded by cousin Rob. And the more you believe something, Garrett says, the more you want to share it with your social network—spawning a nasty cascade of misperception. So before you hit SEND to forward e-mail, ask yourself: Do I know the item I'm sharing is true, or do I just want it to be?</t>
   </si>
   <si>
-    <t>During the 2008 presidential election, the behest became a giant rumor mill. For example, there were the viral e-mails claiming that Barack Obama's birth syndicate was a fake. Or ones spreading the phony Sarah Palin quote, "God made dinosaurs 4,000 years ago". Some political scholars worry the Web could undermine democracy, by shoeing and polarizing voters. But Web sites and blogs don't serve up the most abysmal rumors. Our in-boxes do. So says a study of e-mail in the journal Human Communication Research. Just after the election, researcher R. Kelly Garrett randomly surveyed 600 nonclericals about their online habits, and whether they'd heard—and believed—a number of geared rumors. He found that the Web does expose us to more rumors. But the Web also delivers more rebuttals, which can even the field. E-mail's more insidious. Because you're more likely to believe that rumor forwarded by cousin Rob. And the more you believe something, Garrett says, the more you want to share it with your social network—spawning a nasty cascade of misperception. So before you hit SEND to forward e-mail, ask yourself: Do I know the item I'm sharing is true, or do I just want it to be?</t>
+    <t>During the 2008 presidential election, the Internet became a giant rumor mill. For example, there were the viral e-mails claiming that Barack Obama's birth certificate was a fake. Or ones spreading the phony Sarah Palin quote, "God made dinosaurs 4,000 years ago". Some political scholars worry the Web could undermine democracy, by misinforming and polarizing voters. But Web sites and blogs don't serve up the most influential rumors. Our in-boxes do. So says a study of e-mail in the journal Human Communication Research. Just after the election, researcher R. Kelly Garrett randomly surveyed 600 Americans about their online habits, and whether they'd heard—and believed—a number of widespread rumors. He found that the Web does expose us to more rumors. But the Web also delivers more rebuttals, which can even the field. E-mail's more insidious. Because you're more likely to believe that rumor forwarded by cousin Rob. And the more you believe something, Garrett says, the more you want to share it with your social network—spawning a nasty cascade of misperception. So before you hit SEND to forward e-mail, ask yourself: Do I know the item I'm sharing is true, or do I just want it to be?</t>
   </si>
   <si>
     <t>#177 Mosquito Formation</t>
@@ -5471,7 +5471,7 @@
     <t>Aha—got 'im! Yes, the __seaboards/mosquitos__ are swarming this time of year. Alaskans joke that the __hyperbola/bloodsucker__ is their state bird. But have you ever looked closely at a swarm of mating mosquitos, gnats, or midges? It's a curious thing. The swarm maintains a kind of shape as it moves around. But the bugs inside it seem to flit about randomly rather than flocking like birds. This collective, yet disordered, flight __shimmied/intrigued__ __diminishes/physicists__ in Rome. They shot ultraslow-motion video of swarming midges. Then they mapped the flight of each midge, and did a mathematical analysis of the collective behavior. Their finding: the motion of the midges is not random. The bugs stay far enough apart to avoid locking into a formation. The swarm instead expands as needed to stay just below the __tenfold/threshold__ density. The work appears on the site arXiv.org. Flocks and schools move in formation only once the group reaches a critical density. Below that threshold, the individuals move—well, like midges. Insect avoidance of full-fledged flocking may be a reproductive strategy: after all, it's hard to mingle when you're stuck in a line dance.</t>
   </si>
   <si>
-    <t>Aha—got 'im! Yes, the seaboards are swarming this time of year. Alaskans joke that the hyperbola is their state bird. But have you ever looked closely at a swarm of mating mosquitos, gnats, or midges? It's a curious thing. The swarm maintains a kind of shape as it moves around. But the bugs inside it seem to flit about randomly rather than flocking like birds. This collective, yet disordered, flight shimmied diminishes in Rome. They shot ultraslow-motion video of swarming midges. Then they mapped the flight of each midge, and did a mathematical analysis of the collective behavior. Their finding: the motion of the midges is not random. The bugs stay far enough apart to avoid locking into a formation. The swarm instead expands as needed to stay just below the tenfold density. The work appears on the site arXiv.org. Flocks and schools move in formation only once the group reaches a critical density. Below that threshold, the individuals move—well, like midges. Insect avoidance of full-fledged flocking may be a reproductive strategy: after all, it's hard to mingle when you're stuck in a line dance.</t>
+    <t>Aha—got 'im! Yes, the mosquitos are swarming this time of year. Alaskans joke that the bloodsucker is their state bird. But have you ever looked closely at a swarm of mating mosquitos, gnats, or midges? It's a curious thing. The swarm maintains a kind of shape as it moves around. But the bugs inside it seem to flit about randomly rather than flocking like birds. This collective, yet disordered, flight intrigued physicists in Rome. They shot ultraslow-motion video of swarming midges. Then they mapped the flight of each midge, and did a mathematical analysis of the collective behavior. Their finding: the motion of the midges is not random. The bugs stay far enough apart to avoid locking into a formation. The swarm instead expands as needed to stay just below the threshold density. The work appears on the site arXiv.org. Flocks and schools move in formation only once the group reaches a critical density. Below that threshold, the individuals move—well, like midges. Insect avoidance of full-fledged flocking may be a reproductive strategy: after all, it's hard to mingle when you're stuck in a line dance.</t>
   </si>
   <si>
     <t>#178 Sport Bet</t>
@@ -5480,7 +5480,7 @@
     <t>The World Series starts October 22nd, with the improbable American League __scandium/champion__ Tampa Bay Rays hosting the National League best Philadelphia Phillies. And there's a 59 percent chance that the Rays will take the title. That's what Bruce Bukiet says, anyway. He's a __algorithm/mathematician__ at the New Jersey Institute of Technology who sets odds on the playoffs and World Series every year. Bukiet starts with each player's __hysterics/statistics__ for the 2008 season. He then uses a model that estimates run production per game based on those stats. His most probable __pouches/outcomes__ are a 20 percent chance of a Rays championship in six games, and a 19 percent chance of a seven game Rays win. But beware. In the 2006 postseason only one of his favorites in the seven __bitterest/different__ series actually came out victorious. Nevertheless, he's gotten it right in six of the last eight years. Of course, when predicting __mauling/sporting__ events, always follow the advice of Damon Runyon, who said, "The race is not always to the swift, nor the battle to the strong. But that's the way to bet."</t>
   </si>
   <si>
-    <t>The World Series starts October 22nd, with the improbable American League scandium Tampa Bay Rays hosting the National League best Philadelphia Phillies. And there's a 59 percent chance that the Rays will take the title. That's what Bruce Bukiet says, anyway. He's a algorithm at the New Jersey Institute of Technology who sets odds on the playoffs and World Series every year. Bukiet starts with each player's hysterics for the 2008 season. He then uses a model that estimates run production per game based on those stats. His most probable pouches are a 20 percent chance of a Rays championship in six games, and a 19 percent chance of a seven game Rays win. But beware. In the 2006 postseason only one of his favorites in the seven bitterest series actually came out victorious. Nevertheless, he's gotten it right in six of the last eight years. Of course, when predicting mauling events, always follow the advice of Damon Runyon, who said, "The race is not always to the swift, nor the battle to the strong. But that's the way to bet."</t>
+    <t>The World Series starts October 22nd, with the improbable American League champion Tampa Bay Rays hosting the National League best Philadelphia Phillies. And there's a 59 percent chance that the Rays will take the title. That's what Bruce Bukiet says, anyway. He's a mathematician at the New Jersey Institute of Technology who sets odds on the playoffs and World Series every year. Bukiet starts with each player's statistics for the 2008 season. He then uses a model that estimates run production per game based on those stats. His most probable outcomes are a 20 percent chance of a Rays championship in six games, and a 19 percent chance of a seven game Rays win. But beware. In the 2006 postseason only one of his favorites in the seven different series actually came out victorious. Nevertheless, he's gotten it right in six of the last eight years. Of course, when predicting sporting events, always follow the advice of Damon Runyon, who said, "The race is not always to the swift, nor the battle to the strong. But that's the way to bet."</t>
   </si>
   <si>
     <t>#179 Bone and Weight</t>
@@ -5489,7 +5489,7 @@
     <t>Some dinosaurs were really huge. And now we may have a better way to __envelopment/estimate__ just how heavy these giants were. Researchers have developed a method to weigh dinosaurs, based on laser scans of their skeletons. The study is in the journal Biology Letters. Looking at a bare human skeleton, how would you guess whether its owner was chubby or svelte? If you calculated how much space the fully-fleshed body occupied, you could __codify/multiply__ that volume by tissue density to find the weight. Researchers laser-scanned 14 modern mammal skeletons to create digital models of each body. These 3-D models were unrealistically scrawny, with skin __dismissed/stretched__ tight over the bones. But their undersized volumes were consistent, measuring in as 21 percent less than the actual animals. Based on this information, __reasoners/researchers__ scanned Giraffatitan bones, added 21 percent to the digital model's volume, and then calculated the dinosaur's weight: about 51,000 pounds. The technique could become the __insomuch/preferred__ way to estimate mass based on skeletons, improving our understanding of how extinct species lived and moved. And helping paleontologists make earth-shaking discoveries.</t>
   </si>
   <si>
-    <t>Some dinosaurs were really huge. And now we may have a better way to envelopment just how heavy these giants were. Researchers have developed a method to weigh dinosaurs, based on laser scans of their skeletons. The study is in the journal Biology Letters. Looking at a bare human skeleton, how would you guess whether its owner was chubby or svelte? If you calculated how much space the fully-fleshed body occupied, you could codify that volume by tissue density to find the weight. Researchers laser-scanned 14 modern mammal skeletons to create digital models of each body. These 3-D models were unrealistically scrawny, with skin dismissed tight over the bones. But their undersized volumes were consistent, measuring in as 21 percent less than the actual animals. Based on this information, reasoners scanned Giraffatitan bones, added 21 percent to the digital model's volume, and then calculated the dinosaur's weight: about 51,000 pounds. The technique could become the insomuch way to estimate mass based on skeletons, improving our understanding of how extinct species lived and moved. And helping paleontologists make earth-shaking discoveries.</t>
+    <t>Some dinosaurs were really huge. And now we may have a better way to estimate just how heavy these giants were. Researchers have developed a method to weigh dinosaurs, based on laser scans of their skeletons. The study is in the journal Biology Letters. Looking at a bare human skeleton, how would you guess whether its owner was chubby or svelte? If you calculated how much space the fully-fleshed body occupied, you could multiply that volume by tissue density to find the weight. Researchers laser-scanned 14 modern mammal skeletons to create digital models of each body. These 3-D models were unrealistically scrawny, with skin stretched tight over the bones. But their undersized volumes were consistent, measuring in as 21 percent less than the actual animals. Based on this information, researchers scanned Giraffatitan bones, added 21 percent to the digital model's volume, and then calculated the dinosaur's weight: about 51,000 pounds. The technique could become the preferred way to estimate mass based on skeletons, improving our understanding of how extinct species lived and moved. And helping paleontologists make earth-shaking discoveries.</t>
   </si>
   <si>
     <t>#180 Snail Way</t>
@@ -5498,7 +5498,7 @@
     <t>Weeee. That's the sound a snail makes when it's riding on the back of a turtle. When they're not riding turtles, those snails produce a little mucus trail as they creep along the ground. Well, according to __rebut/research__ just published in the Proceedings of the Royal Society Biological Sciences, snails also ride along on, weeee, pre-existing mucus trails left by other snails. It's like a snail superhighway. Okay, a snail highway. Okay, a snail way. The research involved marine snails, but __solidly/probably__ applies to all snails, which may expend a third of all their energy producing mucus. So an obvious benefit is that individual snails can save energy that would otherwise go into cutting fresh trails. Snail experts had thought this was the case, but the new study proves it. And it wasn't easy—the researchers actually __rendered/measured__ the thickness of snail trails. A new trail could __stage/accommodate__ a second __calendar/traveler__ without additional mucus. But __inkstand/weathered__ trails got thicker, as snails added a bit of mucus where necessary.</t>
   </si>
   <si>
-    <t>Weeee. That's the sound a snail makes when it's riding on the back of a turtle. When they're not riding turtles, those snails produce a little mucus trail as they creep along the ground. Well, according to rebut just published in the Proceedings of the Royal Society Biological Sciences, snails also ride along on, weeee, pre-existing mucus trails left by other snails. It's like a snail superhighway. Okay, a snail highway. Okay, a snail way. The research involved marine snails, but solidly applies to all snails, which may expend a third of all their energy producing mucus. So an obvious benefit is that individual snails can save energy that would otherwise go into cutting fresh trails. Snail experts had thought this was the case, but the new study proves it. And it wasn't easy—the researchers actually rendered the thickness of snail trails. A new trail could stage a second calendar without additional mucus. But inkstand trails got thicker, as snails added a bit of mucus where necessary.</t>
+    <t>Weeee. That's the sound a snail makes when it's riding on the back of a turtle. When they're not riding turtles, those snails produce a little mucus trail as they creep along the ground. Well, according to research just published in the Proceedings of the Royal Society Biological Sciences, snails also ride along on, weeee, pre-existing mucus trails left by other snails. It's like a snail superhighway. Okay, a snail highway. Okay, a snail way. The research involved marine snails, but probably applies to all snails, which may expend a third of all their energy producing mucus. So an obvious benefit is that individual snails can save energy that would otherwise go into cutting fresh trails. Snail experts had thought this was the case, but the new study proves it. And it wasn't easy—the researchers actually measured the thickness of snail trails. A new trail could accommodate a second traveler without additional mucus. But weathered trails got thicker, as snails added a bit of mucus where necessary.</t>
   </si>
   <si>
     <t>#181 Food's Tale</t>
@@ -5507,7 +5507,7 @@
     <t>Here's a strange tale of two previously unrelated food products. First: chitlins, that __difficultly/delicacy__ of fried pig large intestines. They're well-loved throughout the South, especially during the upcoming holiday season. But the smell of them cooking inspires significantly less affection. Because the cooking process sometimes smells like, well, feces. Researchers in Japan thought that cilantro could help. Because cilantro is used in a variety of __reprieve/cuisines__ around the world to mask smells, as well as to add distinctive flavors. And in a previous study, the research team had shown that cilantro can mask the __fringing/cooking-chitlin__ stench. In the new research, in the Journal of __marginal/Agricultural__ and Food Chemistry, they isolated cilantro's volatile compounds and tested each one for its __bookwriting/odor-fighting__ power. Many seemed to lessen the stink, but one in particular, according to human sniffers, entirely cancels out the odor. It's called (E,E)-2,4-Undecadienal. It works at a very low concentration—10 parts per billion—so you can't smell the compound. It's not masking the chitlin odor, it's actually neutralizing it. So it's not just better living through chemistry. It's better chitlins too.</t>
   </si>
   <si>
-    <t>Here's a strange tale of two previously unrelated food products. First: chitlins, that difficultly of fried pig large intestines. They're well-loved throughout the South, especially during the upcoming holiday season. But the smell of them cooking inspires significantly less affection. Because the cooking process sometimes smells like, well, feces. Researchers in Japan thought that cilantro could help. Because cilantro is used in a variety of reprieve around the world to mask smells, as well as to add distinctive flavors. And in a previous study, the research team had shown that cilantro can mask the fringing stench. In the new research, in the Journal of marginal and Food Chemistry, they isolated cilantro's volatile compounds and tested each one for its bookwriting power. Many seemed to lessen the stink, but one in particular, according to human sniffers, entirely cancels out the odor. It's called (E,E)-2,4-Undecadienal. It works at a very low concentration—10 parts per billion—so you can't smell the compound. It's not masking the chitlin odor, it's actually neutralizing it. So it's not just better living through chemistry. It's better chitlins too.</t>
+    <t>Here's a strange tale of two previously unrelated food products. First: chitlins, that delicacy of fried pig large intestines. They're well-loved throughout the South, especially during the upcoming holiday season. But the smell of them cooking inspires significantly less affection. Because the cooking process sometimes smells like, well, feces. Researchers in Japan thought that cilantro could help. Because cilantro is used in a variety of cuisines around the world to mask smells, as well as to add distinctive flavors. And in a previous study, the research team had shown that cilantro can mask the cooking-chitlin stench. In the new research, in the Journal of Agricultural and Food Chemistry, they isolated cilantro's volatile compounds and tested each one for its odor-fighting power. Many seemed to lessen the stink, but one in particular, according to human sniffers, entirely cancels out the odor. It's called (E,E)-2,4-Undecadienal. It works at a very low concentration—10 parts per billion—so you can't smell the compound. It's not masking the chitlin odor, it's actually neutralizing it. So it's not just better living through chemistry. It's better chitlins too.</t>
   </si>
   <si>
     <t>#182 Good Bacteria</t>
@@ -5516,7 +5516,7 @@
     <t>Sometimes a bit of __dyslexia/bacteria__ can be just what the doctor ordered. If you prize yogurt for its "active cultures," you know what I'm talking about. Now a new study, __sunlit/published__ in the September 21st online issue of Nature, suggests that good bugs might even hold __kiwis/diabetes__ at bay. Type I diabetes is caused by an immune system malfunction. Basically, the immune cells that usually chase after bacteria instead attack the pancreas, wiping out the cells that produce insulin. So researchers decided to see what would happen if they reigned in the immune response in mice that are prone to diabetes. As expected, they found that the animals were less likely to develop the disease. But the effect depended entirely on the critters having a normal complement of friendly bacteria in their intestine. Mice that were raised in a totally sterile, germ-free environment were rampant diabetics. But simply __skiing/treating__ those mice with a cocktail of bugs found in most mammals' bellies cured the disease. How bacteria in the intestine can stave off diabetes is not yet clear. But the finding could lead to some interesting new treatments. In the meantime, __glitter/remember__ that we can't live without the stuff that lives in us.</t>
   </si>
   <si>
-    <t>Sometimes a bit of dyslexia can be just what the doctor ordered. If you prize yogurt for its "active cultures," you know what I'm talking about. Now a new study, sunlit in the September 21st online issue of Nature, suggests that good bugs might even hold kiwis at bay. Type I diabetes is caused by an immune system malfunction. Basically, the immune cells that usually chase after bacteria instead attack the pancreas, wiping out the cells that produce insulin. So researchers decided to see what would happen if they reigned in the immune response in mice that are prone to diabetes. As expected, they found that the animals were less likely to develop the disease. But the effect depended entirely on the critters having a normal complement of friendly bacteria in their intestine. Mice that were raised in a totally sterile, germ-free environment were rampant diabetics. But simply skiing those mice with a cocktail of bugs found in most mammals' bellies cured the disease. How bacteria in the intestine can stave off diabetes is not yet clear. But the finding could lead to some interesting new treatments. In the meantime, glitter that we can't live without the stuff that lives in us.</t>
+    <t>Sometimes a bit of bacteria can be just what the doctor ordered. If you prize yogurt for its "active cultures," you know what I'm talking about. Now a new study, published in the September 21st online issue of Nature, suggests that good bugs might even hold diabetes at bay. Type I diabetes is caused by an immune system malfunction. Basically, the immune cells that usually chase after bacteria instead attack the pancreas, wiping out the cells that produce insulin. So researchers decided to see what would happen if they reigned in the immune response in mice that are prone to diabetes. As expected, they found that the animals were less likely to develop the disease. But the effect depended entirely on the critters having a normal complement of friendly bacteria in their intestine. Mice that were raised in a totally sterile, germ-free environment were rampant diabetics. But simply treating those mice with a cocktail of bugs found in most mammals' bellies cured the disease. How bacteria in the intestine can stave off diabetes is not yet clear. But the finding could lead to some interesting new treatments. In the meantime, remember that we can't live without the stuff that lives in us.</t>
   </si>
   <si>
     <t>#183 Pop Music</t>
@@ -5525,7 +5525,7 @@
     <t>Flip through Rolling Stone, and you'll read about a lot of "revolutions" in popular music: Rock'n'roll and punk, disco and new wave. But for Matthias Mauch—an engineer at Queen Mary University of London—the qualitative analysis of musical evolution—the music critic's take—left him wondering: "Is there some way in which we can take this kind of pub conversation, and make it more quantifiable?" So he and his colleagues analyzed fragments from more than 17,000 songs on the Billboard Hot 100, from 1960 to 2010. They __fussbudget/processed__ the audio to extract information about timbral and harmonic qualities—tagging the files for attributes like "orchestra/harmonic" or "calm/quiet/mellow." Then they used those tags—which they compare to a musical "fossil record"—to tease out trends about musical evolution over time. Turns out, from 1960 to 2009, the dominant seventh chord all but disappeared in what they call the death of blues and jazz on the pop charts. But as dominant sevenths faded, the minor seventh came into its own… ... more than doubling in frequency between 1967 and '77. "We can really see the influx of funk, which is then turning into disco." But next—as you know—came the '80s. __derangement/Dominated__ by a rise in musical tags like "percussive" and "guitar/aggressive" [Bon Jovi—"Bad Medicine"], the '80s were a low point for musical diversity. In fact 1986 stands out as the year that chart-topping songs sounded most alike. "Then __illustriously/obviously__ the charts got saved in terms of diversity, by this new kid on the block, the rap and hip-hop coming in. And then suddenly, boom: the diversity's back up and __passionately/actually__ higher than before." The study appears in the journal Royal Society Open Science. Of course, this big-data approach to pop culture probably won't overturn years of musical scholarship. But the analysis does show that in the evolution of popular music, there really have been long periods of stasis, punctuated by periods of rapid change—musical revolutions—particularly in 1964, 1983 and 1991. And the more you study it, Matthias says, the more musical evolution starts to resemble plain old species evolution. "You take __unbecoming/something__ that exists. And that in biology would be genes. But it's not genes here. You just take some styles. You recombine them, like genes are recombined, and you change them as well—a bit like mutation." Who knows—maybe that might have been a better argument against copyright infringement for Robin Thicke and Pharrell Williams.</t>
   </si>
   <si>
-    <t>Flip through Rolling Stone, and you'll read about a lot of "revolutions" in popular music: Rock'n'roll and punk, disco and new wave. But for Matthias Mauch—an engineer at Queen Mary University of London—the qualitative analysis of musical evolution—the music critic's take—left him wondering: "Is there some way in which we can take this kind of pub conversation, and make it more quantifiable?" So he and his colleagues analyzed fragments from more than 17,000 songs on the Billboard Hot 100, from 1960 to 2010. They fussbudget the audio to extract information about timbral and harmonic qualities—tagging the files for attributes like "orchestra/harmonic" or "calm/quiet/mellow." Then they used those tags—which they compare to a musical "fossil record"—to tease out trends about musical evolution over time. Turns out, from 1960 to 2009, the dominant seventh chord all but disappeared in what they call the death of blues and jazz on the pop charts. But as dominant sevenths faded, the minor seventh came into its own… ... more than doubling in frequency between 1967 and '77. "We can really see the influx of funk, which is then turning into disco." But next—as you know—came the '80s. derangement by a rise in musical tags like "percussive" and "guitar/aggressive" [Bon Jovi—"Bad Medicine"], the '80s were a low point for musical diversity. In fact 1986 stands out as the year that chart-topping songs sounded most alike. "Then illustriously the charts got saved in terms of diversity, by this new kid on the block, the rap and hip-hop coming in. And then suddenly, boom: the diversity's back up and passionately higher than before." The study appears in the journal Royal Society Open Science. Of course, this big-data approach to pop culture probably won't overturn years of musical scholarship. But the analysis does show that in the evolution of popular music, there really have been long periods of stasis, punctuated by periods of rapid change—musical revolutions—particularly in 1964, 1983 and 1991. And the more you study it, Matthias says, the more musical evolution starts to resemble plain old species evolution. "You take unbecoming that exists. And that in biology would be genes. But it's not genes here. You just take some styles. You recombine them, like genes are recombined, and you change them as well—a bit like mutation." Who knows—maybe that might have been a better argument against copyright infringement for Robin Thicke and Pharrell Williams.</t>
+    <t>Flip through Rolling Stone, and you'll read about a lot of "revolutions" in popular music: Rock'n'roll and punk, disco and new wave. But for Matthias Mauch—an engineer at Queen Mary University of London—the qualitative analysis of musical evolution—the music critic's take—left him wondering: "Is there some way in which we can take this kind of pub conversation, and make it more quantifiable?" So he and his colleagues analyzed fragments from more than 17,000 songs on the Billboard Hot 100, from 1960 to 2010. They processed the audio to extract information about timbral and harmonic qualities—tagging the files for attributes like "orchestra/harmonic" or "calm/quiet/mellow." Then they used those tags—which they compare to a musical "fossil record"—to tease out trends about musical evolution over time. Turns out, from 1960 to 2009, the dominant seventh chord all but disappeared in what they call the death of blues and jazz on the pop charts. But as dominant sevenths faded, the minor seventh came into its own… ... more than doubling in frequency between 1967 and '77. "We can really see the influx of funk, which is then turning into disco." But next—as you know—came the '80s. Dominated by a rise in musical tags like "percussive" and "guitar/aggressive" [Bon Jovi—"Bad Medicine"], the '80s were a low point for musical diversity. In fact 1986 stands out as the year that chart-topping songs sounded most alike. "Then obviously the charts got saved in terms of diversity, by this new kid on the block, the rap and hip-hop coming in. And then suddenly, boom: the diversity's back up and actually higher than before." The study appears in the journal Royal Society Open Science. Of course, this big-data approach to pop culture probably won't overturn years of musical scholarship. But the analysis does show that in the evolution of popular music, there really have been long periods of stasis, punctuated by periods of rapid change—musical revolutions—particularly in 1964, 1983 and 1991. And the more you study it, Matthias says, the more musical evolution starts to resemble plain old species evolution. "You take something that exists. And that in biology would be genes. But it's not genes here. You just take some styles. You recombine them, like genes are recombined, and you change them as well—a bit like mutation." Who knows—maybe that might have been a better argument against copyright infringement for Robin Thicke and Pharrell Williams.</t>
   </si>
   <si>
     <t>#184 Acoustic Cloak</t>
@@ -5534,7 +5534,7 @@
     <t>When Harry Potter slips underneath his __ascendency/invisibility__ cloak, he can wander freely, undetected. But what about a cloak of silence, one that completely deadens sound? That's just what scientists from Spain's University of Valencia have designed, on a tiny scale. They wrote about their research in the New Journal of Physics. A paper published last year showed how such a cloak could be made in theory—researchers __wrote/proposed__ using materials made up of what are called sonic crystals. These are solid cylinders that can scatter sound waves. The Spanish scientists wanted to figure out the specs to make a real acoustic cloak that could totally reroute sound around a given object. According to their models, it would take about 200 layers of the sound-silencing materials to make it completely __transients/impervious__ to sound waves. They also think that they'll eventually be able to get the same effect with a thinner cover. Among the first __waiters/applications__ could be a silent coating for naval ships, so that they're rendered invisible to sonar. But even more important could be wall __surpluses/coverings__ that would finally protect your ears from those annoyingly noisy neighbors.</t>
   </si>
   <si>
-    <t>When Harry Potter slips underneath his ascendency cloak, he can wander freely, undetected. But what about a cloak of silence, one that completely deadens sound? That's just what scientists from Spain's University of Valencia have designed, on a tiny scale. They wrote about their research in the New Journal of Physics. A paper published last year showed how such a cloak could be made in theory—researchers wrote using materials made up of what are called sonic crystals. These are solid cylinders that can scatter sound waves. The Spanish scientists wanted to figure out the specs to make a real acoustic cloak that could totally reroute sound around a given object. According to their models, it would take about 200 layers of the sound-silencing materials to make it completely transients to sound waves. They also think that they'll eventually be able to get the same effect with a thinner cover. Among the first waiters could be a silent coating for naval ships, so that they're rendered invisible to sonar. But even more important could be wall surpluses that would finally protect your ears from those annoyingly noisy neighbors.</t>
+    <t>When Harry Potter slips underneath his invisibility cloak, he can wander freely, undetected. But what about a cloak of silence, one that completely deadens sound? That's just what scientists from Spain's University of Valencia have designed, on a tiny scale. They wrote about their research in the New Journal of Physics. A paper published last year showed how such a cloak could be made in theory—researchers proposed using materials made up of what are called sonic crystals. These are solid cylinders that can scatter sound waves. The Spanish scientists wanted to figure out the specs to make a real acoustic cloak that could totally reroute sound around a given object. According to their models, it would take about 200 layers of the sound-silencing materials to make it completely impervious to sound waves. They also think that they'll eventually be able to get the same effect with a thinner cover. Among the first applications could be a silent coating for naval ships, so that they're rendered invisible to sonar. But even more important could be wall coverings that would finally protect your ears from those annoyingly noisy neighbors.</t>
   </si>
   <si>
     <t>#185 Whales</t>
@@ -5543,7 +5543,7 @@
     <t>The world's oceans were once home to 10 times as many whales… before the Captain Ahabs of the world came round. Hunting hit big species the hardest, wiping out 99 percent of the Southern __ref/Hemisphere's__ blue whales, for example. And as the gentle giants disappeared… so did another lesser known element of the oceans: their poop. "I've described it as, sort of like oversteeped green tea. Like well steeped green tea. So it's very diffuse, in a big plume." Joe Roman, a conservation biologist at the University of Vermont. "My __scorches/daughter's__ friends say I'm a whale poop scientist." And he says, he studies all kinds. "When whales are feeding on krill, they're really high lipids, lots of fat, so it can be sort of clumps together and floats at the surface. So there's a great variety of fecal plumes out there in the oceans." Whale poop is important because it transports nutrients from the deep ocean, up to the surface. "Sperm whales feed on giant squid and other deep sea creatures. So they'll dive more than a kilometer down." Then they come to the surface to breathe, and digest, "and as it turns out they poop and they also pee. So they're __sheaving/releasing__ all these nutrients." Nutrients like phosphorus, which are slurped up by phytoplankton and algae. "Which is in turn is consumed by zooplankton, copepods or krill. And those are either eaten by fish or they can be eaten by seabirds." Some fish swim up rivers and die; birds sprinkle the land with their guano; and those __rhe/deep-sea__ nutrients slowly work their way into ecosystems on land with the help of bald eagles and bears and the like. Roman and his __puttees/colleagues__ modeled how that conveyer belt of nutrients has slowed due to the huge __knights/declines__ in whale, seabird and fish populations. And they reckon that only a quarter as much phosphorus makes it to surface waters today compared with the past. And the flow of phosphorus to land has nearly stopped--at just 4 percent of historic levels. The results are in the Proceedings of the National Academy of Sciences. Roman says this slowing of the nutrient conveyer belt is reversible, though. "The most important part for me is trying to restore these species as ecological engineers on the planet, and really try and share the planet with them. Let's not just keep them in zoos or even in small island pockets of protected areas. Let's let them move around the planet more freely." And when they do, he says… those key nutrients, too, will once again roam the Earth.</t>
   </si>
   <si>
-    <t>The world's oceans were once home to 10 times as many whales… before the Captain Ahabs of the world came round. Hunting hit big species the hardest, wiping out 99 percent of the Southern ref blue whales, for example. And as the gentle giants disappeared… so did another lesser known element of the oceans: their poop. "I've described it as, sort of like oversteeped green tea. Like well steeped green tea. So it's very diffuse, in a big plume." Joe Roman, a conservation biologist at the University of Vermont. "My scorches friends say I'm a whale poop scientist." And he says, he studies all kinds. "When whales are feeding on krill, they're really high lipids, lots of fat, so it can be sort of clumps together and floats at the surface. So there's a great variety of fecal plumes out there in the oceans." Whale poop is important because it transports nutrients from the deep ocean, up to the surface. "Sperm whales feed on giant squid and other deep sea creatures. So they'll dive more than a kilometer down." Then they come to the surface to breathe, and digest, "and as it turns out they poop and they also pee. So they're sheaving all these nutrients." Nutrients like phosphorus, which are slurped up by phytoplankton and algae. "Which is in turn is consumed by zooplankton, copepods or krill. And those are either eaten by fish or they can be eaten by seabirds." Some fish swim up rivers and die; birds sprinkle the land with their guano; and those rhe nutrients slowly work their way into ecosystems on land with the help of bald eagles and bears and the like. Roman and his puttees modeled how that conveyer belt of nutrients has slowed due to the huge knights in whale, seabird and fish populations. And they reckon that only a quarter as much phosphorus makes it to surface waters today compared with the past. And the flow of phosphorus to land has nearly stopped--at just 4 percent of historic levels. The results are in the Proceedings of the National Academy of Sciences. Roman says this slowing of the nutrient conveyer belt is reversible, though. "The most important part for me is trying to restore these species as ecological engineers on the planet, and really try and share the planet with them. Let's not just keep them in zoos or even in small island pockets of protected areas. Let's let them move around the planet more freely." And when they do, he says… those key nutrients, too, will once again roam the Earth.</t>
+    <t>The world's oceans were once home to 10 times as many whales… before the Captain Ahabs of the world came round. Hunting hit big species the hardest, wiping out 99 percent of the Southern Hemisphere's blue whales, for example. And as the gentle giants disappeared… so did another lesser known element of the oceans: their poop. "I've described it as, sort of like oversteeped green tea. Like well steeped green tea. So it's very diffuse, in a big plume." Joe Roman, a conservation biologist at the University of Vermont. "My daughter's friends say I'm a whale poop scientist." And he says, he studies all kinds. "When whales are feeding on krill, they're really high lipids, lots of fat, so it can be sort of clumps together and floats at the surface. So there's a great variety of fecal plumes out there in the oceans." Whale poop is important because it transports nutrients from the deep ocean, up to the surface. "Sperm whales feed on giant squid and other deep sea creatures. So they'll dive more than a kilometer down." Then they come to the surface to breathe, and digest, "and as it turns out they poop and they also pee. So they're releasing all these nutrients." Nutrients like phosphorus, which are slurped up by phytoplankton and algae. "Which is in turn is consumed by zooplankton, copepods or krill. And those are either eaten by fish or they can be eaten by seabirds." Some fish swim up rivers and die; birds sprinkle the land with their guano; and those deep-sea nutrients slowly work their way into ecosystems on land with the help of bald eagles and bears and the like. Roman and his colleagues modeled how that conveyer belt of nutrients has slowed due to the huge declines in whale, seabird and fish populations. And they reckon that only a quarter as much phosphorus makes it to surface waters today compared with the past. And the flow of phosphorus to land has nearly stopped--at just 4 percent of historic levels. The results are in the Proceedings of the National Academy of Sciences. Roman says this slowing of the nutrient conveyer belt is reversible, though. "The most important part for me is trying to restore these species as ecological engineers on the planet, and really try and share the planet with them. Let's not just keep them in zoos or even in small island pockets of protected areas. Let's let them move around the planet more freely." And when they do, he says… those key nutrients, too, will once again roam the Earth.</t>
   </si>
   <si>
     <t>#186 Contraception</t>
@@ -5552,7 +5552,7 @@
     <t>It sounds obvious—pregnancies could be avoided by using contraception. But 15 million unwanted __intensities/pregnancies__ could be avoided annually in 35 low- and __supremacism/middle-income__ countries if women did in fact use modern contraception. That's according to a study in the journal Human Reproduction. Unwanted pregnancy has a wide range of serious consequences. Women may have to stop their education or employment. They might pursue unsafe abortions. And they can face disability, disease and death as a result of the pregnancy. To determine barriers to the use of contraception, researchers __condescend/compared__ surveys and __flumes/interviews__ of nearly 13,000 women who became pregnant unintentionally. They compared the data to that from more than a hundred thousand women who were sexually active and did not want to be pregnant. For women who were sexually active, did not want to be pregnant, but did not use contraception, 37 percent feared health side effects from contraception. Twenty-two percent said they or their partner objected. These issues outweighed cost or availability. Women also underestimated the risks of getting pregnant from unprotected sex. The World Health Organization's Howard Sobel is one of the authors of the study. In a press release he says the research shows that health workers need to play a bigger role in educating and reassuring women, along with helping individuals determine the best contraceptive for them. He advises that effective, affordable __nutrition/contraception__ should be coupled with education about the myths of contraception—and information about the real risks of unintended pregnancies.</t>
   </si>
   <si>
-    <t>It sounds obvious—pregnancies could be avoided by using contraception. But 15 million unwanted intensities could be avoided annually in 35 low- and supremacism countries if women did in fact use modern contraception. That's according to a study in the journal Human Reproduction. Unwanted pregnancy has a wide range of serious consequences. Women may have to stop their education or employment. They might pursue unsafe abortions. And they can face disability, disease and death as a result of the pregnancy. To determine barriers to the use of contraception, researchers condescend surveys and flumes of nearly 13,000 women who became pregnant unintentionally. They compared the data to that from more than a hundred thousand women who were sexually active and did not want to be pregnant. For women who were sexually active, did not want to be pregnant, but did not use contraception, 37 percent feared health side effects from contraception. Twenty-two percent said they or their partner objected. These issues outweighed cost or availability. Women also underestimated the risks of getting pregnant from unprotected sex. The World Health Organization's Howard Sobel is one of the authors of the study. In a press release he says the research shows that health workers need to play a bigger role in educating and reassuring women, along with helping individuals determine the best contraceptive for them. He advises that effective, affordable nutrition should be coupled with education about the myths of contraception—and information about the real risks of unintended pregnancies.</t>
+    <t>It sounds obvious—pregnancies could be avoided by using contraception. But 15 million unwanted pregnancies could be avoided annually in 35 low- and middle-income countries if women did in fact use modern contraception. That's according to a study in the journal Human Reproduction. Unwanted pregnancy has a wide range of serious consequences. Women may have to stop their education or employment. They might pursue unsafe abortions. And they can face disability, disease and death as a result of the pregnancy. To determine barriers to the use of contraception, researchers compared surveys and interviews of nearly 13,000 women who became pregnant unintentionally. They compared the data to that from more than a hundred thousand women who were sexually active and did not want to be pregnant. For women who were sexually active, did not want to be pregnant, but did not use contraception, 37 percent feared health side effects from contraception. Twenty-two percent said they or their partner objected. These issues outweighed cost or availability. Women also underestimated the risks of getting pregnant from unprotected sex. The World Health Organization's Howard Sobel is one of the authors of the study. In a press release he says the research shows that health workers need to play a bigger role in educating and reassuring women, along with helping individuals determine the best contraceptive for them. He advises that effective, affordable contraception should be coupled with education about the myths of contraception—and information about the real risks of unintended pregnancies.</t>
   </si>
   <si>
     <t>#187 Sniff</t>
@@ -5561,7 +5561,7 @@
     <t>Imagine if you could focus your nose, the way you focus your eyes. __hybridise/Scientists__ now believe that animals with a highly developed sense of smell, like rats and dogs, do just that. Similar to the way we taste sweet, salty, sour and bitter on different parts of the tongue, animals detect various smells in different parts of the nose. Researchers at the University of Chicago __publicized/hypothesized__ that rats, by changing the way air flows across the insides of the nostrils, could direct the scent to the nasal region where it could be best detected. Turns out they were right. When presented with different odors, rats actually changed the way they sniffed. For example, long slow sniffs for hard-to-detect scents, or short fast ones for easy ones. Rats even sniffed __minstrelsy/differently__ while learning a new scent than when the smell was familiar. The study is in the Journal of Neuroscience. The researchers say the finding shows that there's more to a good sense of smell than __fictionally/originally__ thought. A __necklaces/sensitive__ nose is important, but so is how you use it.</t>
   </si>
   <si>
-    <t>Imagine if you could focus your nose, the way you focus your eyes. hybridise now believe that animals with a highly developed sense of smell, like rats and dogs, do just that. Similar to the way we taste sweet, salty, sour and bitter on different parts of the tongue, animals detect various smells in different parts of the nose. Researchers at the University of Chicago publicized that rats, by changing the way air flows across the insides of the nostrils, could direct the scent to the nasal region where it could be best detected. Turns out they were right. When presented with different odors, rats actually changed the way they sniffed. For example, long slow sniffs for hard-to-detect scents, or short fast ones for easy ones. Rats even sniffed minstrelsy while learning a new scent than when the smell was familiar. The study is in the Journal of Neuroscience. The researchers say the finding shows that there's more to a good sense of smell than fictionally thought. A necklaces nose is important, but so is how you use it.</t>
+    <t>Imagine if you could focus your nose, the way you focus your eyes. Scientists now believe that animals with a highly developed sense of smell, like rats and dogs, do just that. Similar to the way we taste sweet, salty, sour and bitter on different parts of the tongue, animals detect various smells in different parts of the nose. Researchers at the University of Chicago hypothesized that rats, by changing the way air flows across the insides of the nostrils, could direct the scent to the nasal region where it could be best detected. Turns out they were right. When presented with different odors, rats actually changed the way they sniffed. For example, long slow sniffs for hard-to-detect scents, or short fast ones for easy ones. Rats even sniffed differently while learning a new scent than when the smell was familiar. The study is in the Journal of Neuroscience. The researchers say the finding shows that there's more to a good sense of smell than originally thought. A sensitive nose is important, but so is how you use it.</t>
   </si>
   <si>
     <t>#188 Ventilation</t>
@@ -5570,7 +5570,7 @@
     <t>Contrary to popular wisdom, a new study finds that if you want to avoid getting sick you should open a window. At least if you don't want to catch TB in a hospital in Lima, Peru. __impedances/Researchers__ from the Imperial College London were looking for ways to limit the spread of tuberculosis in the Peruvian situation. One major site of transmission is apparently the hospital waiting room, where infected __sharecroppers/individuals__ come to be treated. In close quarters, one person with TB can infect many others, by sneezing, coughing, even speaking. To curb the contagion, the __freelancers/researchers__ prescribed ventilation. And the best ventilation, they find, is the simplest—opening the doors and windows. Such natural __temptation/ventilation__ really keeps things moving, allowing the air in the room to be replaced by fresh air an average of 28 times an hour. Even __physiological/mechanical__ systems designed specifically to exchange the air in isolation wards only achieve 12 air changes an hour, and that's when they're working at maximum capacity, which is not often the case. The study is good news for __fascicles/hospitals__ that can't afford sophisticated mechanical ventilation systems. And it's a real shot in the arm for people who've always said that a little fresh air is good for you.</t>
   </si>
   <si>
-    <t>Contrary to popular wisdom, a new study finds that if you want to avoid getting sick you should open a window. At least if you don't want to catch TB in a hospital in Lima, Peru. impedances from the Imperial College London were looking for ways to limit the spread of tuberculosis in the Peruvian situation. One major site of transmission is apparently the hospital waiting room, where infected sharecroppers come to be treated. In close quarters, one person with TB can infect many others, by sneezing, coughing, even speaking. To curb the contagion, the freelancers prescribed ventilation. And the best ventilation, they find, is the simplest—opening the doors and windows. Such natural temptation really keeps things moving, allowing the air in the room to be replaced by fresh air an average of 28 times an hour. Even physiological systems designed specifically to exchange the air in isolation wards only achieve 12 air changes an hour, and that's when they're working at maximum capacity, which is not often the case. The study is good news for fascicles that can't afford sophisticated mechanical ventilation systems. And it's a real shot in the arm for people who've always said that a little fresh air is good for you.</t>
+    <t>Contrary to popular wisdom, a new study finds that if you want to avoid getting sick you should open a window. At least if you don't want to catch TB in a hospital in Lima, Peru. Researchers from the Imperial College London were looking for ways to limit the spread of tuberculosis in the Peruvian situation. One major site of transmission is apparently the hospital waiting room, where infected individuals come to be treated. In close quarters, one person with TB can infect many others, by sneezing, coughing, even speaking. To curb the contagion, the researchers prescribed ventilation. And the best ventilation, they find, is the simplest—opening the doors and windows. Such natural ventilation really keeps things moving, allowing the air in the room to be replaced by fresh air an average of 28 times an hour. Even mechanical systems designed specifically to exchange the air in isolation wards only achieve 12 air changes an hour, and that's when they're working at maximum capacity, which is not often the case. The study is good news for hospitals that can't afford sophisticated mechanical ventilation systems. And it's a real shot in the arm for people who've always said that a little fresh air is good for you.</t>
   </si>
   <si>
     <t>#189 Limb Evolution</t>
@@ -5579,7 +5579,7 @@
     <t>What had the legs of a 'gator and the jaws of a fish? Why, the earliest land animals. Because a new study shows that animals evolved weight-bearing limbs long before they had the chompers to really take __euthanised/advantage__ of a terrestrial diet. The research is in the journal Integrative and Comparative Biology. Scientists had suspected that the first four-legged creatures to haul their __additives/carcasses__ out of the ocean didn't belly up to the salad bar straight away. But they lacked definitive proof. Now, researchers have __minstrelsy/carefully__ __bathtub/examined__ the fossilized faces of 89 beasties that lived on land and sea some 300 to 400 million years ago. They probed the jaws for a range of __semitropical/biomechanical__ features, such as how much force they could give to their bite. The result: seems it took tens of __transitions/millions__ of years after setting foot on land to come up with a mouth that could munch on the greenery. Why the lag? Could be the critters had to stop being such mouth __aliyahs/breathers__ and shift from using gills to using lungs, which freed their jaws to develop in new ways. And which left no more excuses to not eat their veggies.</t>
   </si>
   <si>
-    <t>What had the legs of a 'gator and the jaws of a fish? Why, the earliest land animals. Because a new study shows that animals evolved weight-bearing limbs long before they had the chompers to really take euthanised of a terrestrial diet. The research is in the journal Integrative and Comparative Biology. Scientists had suspected that the first four-legged creatures to haul their additives out of the ocean didn't belly up to the salad bar straight away. But they lacked definitive proof. Now, researchers have minstrelsy bathtub the fossilized faces of 89 beasties that lived on land and sea some 300 to 400 million years ago. They probed the jaws for a range of semitropical features, such as how much force they could give to their bite. The result: seems it took tens of transitions of years after setting foot on land to come up with a mouth that could munch on the greenery. Why the lag? Could be the critters had to stop being such mouth aliyahs and shift from using gills to using lungs, which freed their jaws to develop in new ways. And which left no more excuses to not eat their veggies.</t>
+    <t>What had the legs of a 'gator and the jaws of a fish? Why, the earliest land animals. Because a new study shows that animals evolved weight-bearing limbs long before they had the chompers to really take advantage of a terrestrial diet. The research is in the journal Integrative and Comparative Biology. Scientists had suspected that the first four-legged creatures to haul their carcasses out of the ocean didn't belly up to the salad bar straight away. But they lacked definitive proof. Now, researchers have carefully examined the fossilized faces of 89 beasties that lived on land and sea some 300 to 400 million years ago. They probed the jaws for a range of biomechanical features, such as how much force they could give to their bite. The result: seems it took tens of millions of years after setting foot on land to come up with a mouth that could munch on the greenery. Why the lag? Could be the critters had to stop being such mouth breathers and shift from using gills to using lungs, which freed their jaws to develop in new ways. And which left no more excuses to not eat their veggies.</t>
   </si>
   <si>
     <t>#190 Freedom</t>
@@ -5588,7 +5588,7 @@
     <t>What's the best way for __glamourous/students__ to really learn basic science? New research just __freshened/presented__ at the annual meeting of the American __excavation/Association__ for the Advancement of Science __minarets/suggests__ an answer: freedom. After years of watching nonscience majors struggle with biology courses, Steve Rissing of Ohio State University decided to see how the boring old cookbook method of __heating/teaching__ stacked up against something new. The old way was to give students a big textbook to follow and dumb down experiments. Many students still scored poorly when asked about the basics. The new method gave students freedom. They prepared their own enzyme solutions and were encouraged to come up with their own methods. The result? Eighty-three percent of the free students gave the right answer to the simple question, "Where do enzymes occur in nature?" Just 23 percent of the cookbook group __befuddled/answered__ correctly. The new methods could help train students to better see and understand the beauty of science.</t>
   </si>
   <si>
-    <t>What's the best way for glamourous to really learn basic science? New research just freshened at the annual meeting of the American excavation for the Advancement of Science minarets an answer: freedom. After years of watching nonscience majors struggle with biology courses, Steve Rissing of Ohio State University decided to see how the boring old cookbook method of heating stacked up against something new. The old way was to give students a big textbook to follow and dumb down experiments. Many students still scored poorly when asked about the basics. The new method gave students freedom. They prepared their own enzyme solutions and were encouraged to come up with their own methods. The result? Eighty-three percent of the free students gave the right answer to the simple question, "Where do enzymes occur in nature?" Just 23 percent of the cookbook group befuddled correctly. The new methods could help train students to better see and understand the beauty of science.</t>
+    <t>What's the best way for students to really learn basic science? New research just presented at the annual meeting of the American Association for the Advancement of Science suggests an answer: freedom. After years of watching nonscience majors struggle with biology courses, Steve Rissing of Ohio State University decided to see how the boring old cookbook method of teaching stacked up against something new. The old way was to give students a big textbook to follow and dumb down experiments. Many students still scored poorly when asked about the basics. The new method gave students freedom. They prepared their own enzyme solutions and were encouraged to come up with their own methods. The result? Eighty-three percent of the free students gave the right answer to the simple question, "Where do enzymes occur in nature?" Just 23 percent of the cookbook group answered correctly. The new methods could help train students to better see and understand the beauty of science.</t>
   </si>
   <si>
     <t>#191 Dark Matter</t>
@@ -5597,7 +5597,7 @@
     <t>Most of the universe's stuff is apparently dark matter, invisible material pervading the __rehearse/universe__ and supplying the bulk of the __generational/gravitational__ __presumption/attraction__ holding galaxy __couples/clusters__ together. The matter contained in the visible stars in the cluster just isn't enough to keep the clusters from flying apart. Now comes one of the __poulticed/strongest__ pieces of evidence for dark matter. The Hubble space __nethermost/telescope__ has found what looks like a ghostly ring, the remnant of a massive collision between two galaxy clusters sometime in the last two billion years. The ring is about 2.6 million light years across and lies about five billion light years from earth. A Johns Hopkins research team noticed the ring. They can't directly see it, of course. But they infer its existence because its gravity bends the light of more distant galaxies in the background. One __sweetener/researcher__ was initially annoyed with the ring because he assumed the ring was some kind of problem or error. A literature search turned up evidence of a collision between galactic clusters near the ring. And computer simulations showed that a dark matter ring would indeed result, like the ripples on a pond.</t>
   </si>
   <si>
-    <t>Most of the universe's stuff is apparently dark matter, invisible material pervading the rehearse and supplying the bulk of the generational presumption holding galaxy couples together. The matter contained in the visible stars in the cluster just isn't enough to keep the clusters from flying apart. Now comes one of the poulticed pieces of evidence for dark matter. The Hubble space nethermost has found what looks like a ghostly ring, the remnant of a massive collision between two galaxy clusters sometime in the last two billion years. The ring is about 2.6 million light years across and lies about five billion light years from earth. A Johns Hopkins research team noticed the ring. They can't directly see it, of course. But they infer its existence because its gravity bends the light of more distant galaxies in the background. One sweetener was initially annoyed with the ring because he assumed the ring was some kind of problem or error. A literature search turned up evidence of a collision between galactic clusters near the ring. And computer simulations showed that a dark matter ring would indeed result, like the ripples on a pond.</t>
+    <t>Most of the universe's stuff is apparently dark matter, invisible material pervading the universe and supplying the bulk of the gravitational attraction holding galaxy clusters together. The matter contained in the visible stars in the cluster just isn't enough to keep the clusters from flying apart. Now comes one of the strongest pieces of evidence for dark matter. The Hubble space telescope has found what looks like a ghostly ring, the remnant of a massive collision between two galaxy clusters sometime in the last two billion years. The ring is about 2.6 million light years across and lies about five billion light years from earth. A Johns Hopkins research team noticed the ring. They can't directly see it, of course. But they infer its existence because its gravity bends the light of more distant galaxies in the background. One researcher was initially annoyed with the ring because he assumed the ring was some kind of problem or error. A literature search turned up evidence of a collision between galactic clusters near the ring. And computer simulations showed that a dark matter ring would indeed result, like the ripples on a pond.</t>
   </si>
   <si>
     <t>#192 Recession and Health</t>
@@ -5606,7 +5606,7 @@
     <t>It sounds paradoxical, but in wealthy countries, there's nothing like a recession to boost the population's health. According to a report in the __admixture/September__ 1st Canadian Medical __assassination/Association__ Journal, when our paychecks get lighter, we do more than tighten our purse strings—we also cinch our belts, kick bad habits and manage to lower our mortality rates. Economic growth is usually __postdated/associated__ with increased life spans, but the report says that's only true for very poor countries. __weaknesses/Researchers__ looked at data from dozens of 20th century __hardscrabble/international__ health studies and found that, once per-capita income passed $5,000, recessions __cantankerously/actually__ helped health. During lean times, people in __threateningly/relatively__ wealthy countries drink and smoke less and stop overeating. They also go out less, which means fewer trips in the car. It all adds up to fewer deaths from things like lung cancer, liver disease, heart attacks and car crashes. The researchers say that fewer hours in the office can also mean more time with family and friends. These close social interactions lead to less stress and better health. Of course, some people may find more family time to be like a lot of good medicine—hard to swallow.</t>
   </si>
   <si>
-    <t>It sounds paradoxical, but in wealthy countries, there's nothing like a recession to boost the population's health. According to a report in the admixture 1st Canadian Medical assassination Journal, when our paychecks get lighter, we do more than tighten our purse strings—we also cinch our belts, kick bad habits and manage to lower our mortality rates. Economic growth is usually postdated with increased life spans, but the report says that's only true for very poor countries. weaknesses looked at data from dozens of 20th century hardscrabble health studies and found that, once per-capita income passed $5,000, recessions cantankerously helped health. During lean times, people in threateningly wealthy countries drink and smoke less and stop overeating. They also go out less, which means fewer trips in the car. It all adds up to fewer deaths from things like lung cancer, liver disease, heart attacks and car crashes. The researchers say that fewer hours in the office can also mean more time with family and friends. These close social interactions lead to less stress and better health. Of course, some people may find more family time to be like a lot of good medicine—hard to swallow.</t>
+    <t>It sounds paradoxical, but in wealthy countries, there's nothing like a recession to boost the population's health. According to a report in the September 1st Canadian Medical Association Journal, when our paychecks get lighter, we do more than tighten our purse strings—we also cinch our belts, kick bad habits and manage to lower our mortality rates. Economic growth is usually associated with increased life spans, but the report says that's only true for very poor countries. Researchers looked at data from dozens of 20th century international health studies and found that, once per-capita income passed $5,000, recessions actually helped health. During lean times, people in relatively wealthy countries drink and smoke less and stop overeating. They also go out less, which means fewer trips in the car. It all adds up to fewer deaths from things like lung cancer, liver disease, heart attacks and car crashes. The researchers say that fewer hours in the office can also mean more time with family and friends. These close social interactions lead to less stress and better health. Of course, some people may find more family time to be like a lot of good medicine—hard to swallow.</t>
   </si>
   <si>
     <t>#193 Talking to Teens</t>
@@ -5615,7 +5615,7 @@
     <t>You can talk to teens all you want about sex. But if you want to drive home healthy messages about consent, maybe you should have them watch: "In the Criminal Justice system sexually-based __frontbenches/offenses__ are considered especially heinous…" Law &amp; Order: Special Victims Unit. Really. Compared with other TV shows, anyway. Because a study finds that college __juleps/students__ who watched episodes of the various Law &amp; Orders had a better understanding of sexual consent issues than those who watched two other crime procedural franchises, NCIS and CSI. The research is in the Journal of Health Communication. For the study, researchers asked more than 300 college freshmen if they agreed or disagreed that if a woman is raped she is at least somewhat responsible, a concept called rape myth acceptance. The students were also asked about their intentions to seek consent for sexual __epitome/activity__ and their intentions to refuse sexual activity. The results: the college students who watched ripped-from-the-headline Law &amp; Order versus the other shows had stronger views about consent and were less likely to accept rape mythology. Watching CSI, where the victim is often dead and treated as another piece of evidence, was __misplacement/associated__ with lowered intentions to seek consent and a greater acceptance of rape myths. Exposure to the NCIS franchise was associated with __sheep/decreased__ intentions to refuse unwanted sexual activity. Previous research found that the Law &amp; Order shows directly challenge myths and stereotypes related to sexual assaults. While CSI has been criticized for plotlines that reinforce rape myths. So it turns out __trapping/watching__ those shows—at least for college-aged kids—may have some effect on sexual consent intentions and behavior. And when it comes to Law &amp; Order, that effect could be positive.</t>
   </si>
   <si>
-    <t>You can talk to teens all you want about sex. But if you want to drive home healthy messages about consent, maybe you should have them watch: "In the Criminal Justice system sexually-based frontbenches are considered especially heinous…" Law &amp; Order: Special Victims Unit. Really. Compared with other TV shows, anyway. Because a study finds that college juleps who watched episodes of the various Law &amp; Orders had a better understanding of sexual consent issues than those who watched two other crime procedural franchises, NCIS and CSI. The research is in the Journal of Health Communication. For the study, researchers asked more than 300 college freshmen if they agreed or disagreed that if a woman is raped she is at least somewhat responsible, a concept called rape myth acceptance. The students were also asked about their intentions to seek consent for sexual epitome and their intentions to refuse sexual activity. The results: the college students who watched ripped-from-the-headline Law &amp; Order versus the other shows had stronger views about consent and were less likely to accept rape mythology. Watching CSI, where the victim is often dead and treated as another piece of evidence, was misplacement with lowered intentions to seek consent and a greater acceptance of rape myths. Exposure to the NCIS franchise was associated with sheep intentions to refuse unwanted sexual activity. Previous research found that the Law &amp; Order shows directly challenge myths and stereotypes related to sexual assaults. While CSI has been criticized for plotlines that reinforce rape myths. So it turns out trapping those shows—at least for college-aged kids—may have some effect on sexual consent intentions and behavior. And when it comes to Law &amp; Order, that effect could be positive.</t>
+    <t>You can talk to teens all you want about sex. But if you want to drive home healthy messages about consent, maybe you should have them watch: "In the Criminal Justice system sexually-based offenses are considered especially heinous…" Law &amp; Order: Special Victims Unit. Really. Compared with other TV shows, anyway. Because a study finds that college students who watched episodes of the various Law &amp; Orders had a better understanding of sexual consent issues than those who watched two other crime procedural franchises, NCIS and CSI. The research is in the Journal of Health Communication. For the study, researchers asked more than 300 college freshmen if they agreed or disagreed that if a woman is raped she is at least somewhat responsible, a concept called rape myth acceptance. The students were also asked about their intentions to seek consent for sexual activity and their intentions to refuse sexual activity. The results: the college students who watched ripped-from-the-headline Law &amp; Order versus the other shows had stronger views about consent and were less likely to accept rape mythology. Watching CSI, where the victim is often dead and treated as another piece of evidence, was associated with lowered intentions to seek consent and a greater acceptance of rape myths. Exposure to the NCIS franchise was associated with decreased intentions to refuse unwanted sexual activity. Previous research found that the Law &amp; Order shows directly challenge myths and stereotypes related to sexual assaults. While CSI has been criticized for plotlines that reinforce rape myths. So it turns out watching those shows—at least for college-aged kids—may have some effect on sexual consent intentions and behavior. And when it comes to Law &amp; Order, that effect could be positive.</t>
   </si>
   <si>
     <t>#194 Death of Bee</t>
@@ -5624,7 +5624,7 @@
     <t>You've probably heard that the world's honeybees have __comfort/suffered__ stinging losses lately. That's a big story for us, too—up to twelve billion dollars in crops rely on the fuzzy flyers for pollination. Of the 2.4 million honeybee __bibliographies/colonies__ in the U.S., about one million died off this past winter. Big declines have also been seen in Europe and Asia. The die-off has been dubbed colony collapse __transpolar/disorder__ and the vanishing bee syndrome. A couple of species of mites that attack bees were __practical/responsible__ for similar dieoffs in the winters of '95-'96 and 2000-2001. And the mites may be partly to blame for the most recent honeybee losses. But a quarter of the current carnage seems unrelated to mites or any other pests. Other __resembled/suggested__ causes of the bee decline include genetically modified foods, parasites, pesticides, and cell phone radiation. But bee expert Nicholas Calderone of Cornell University said last week that a definitive cause remains elusive. He will spend this summer investigating honeybee colonies throughout the northeast trying to solve the case of the dead bees. Here's hoping he buzzes in with an answer.</t>
   </si>
   <si>
-    <t>You've probably heard that the world's honeybees have comfort stinging losses lately. That's a big story for us, too—up to twelve billion dollars in crops rely on the fuzzy flyers for pollination. Of the 2.4 million honeybee bibliographies in the U.S., about one million died off this past winter. Big declines have also been seen in Europe and Asia. The die-off has been dubbed colony collapse transpolar and the vanishing bee syndrome. A couple of species of mites that attack bees were practical for similar dieoffs in the winters of '95-'96 and 2000-2001. And the mites may be partly to blame for the most recent honeybee losses. But a quarter of the current carnage seems unrelated to mites or any other pests. Other resembled causes of the bee decline include genetically modified foods, parasites, pesticides, and cell phone radiation. But bee expert Nicholas Calderone of Cornell University said last week that a definitive cause remains elusive. He will spend this summer investigating honeybee colonies throughout the northeast trying to solve the case of the dead bees. Here's hoping he buzzes in with an answer.</t>
+    <t>You've probably heard that the world's honeybees have suffered stinging losses lately. That's a big story for us, too—up to twelve billion dollars in crops rely on the fuzzy flyers for pollination. Of the 2.4 million honeybee colonies in the U.S., about one million died off this past winter. Big declines have also been seen in Europe and Asia. The die-off has been dubbed colony collapse disorder and the vanishing bee syndrome. A couple of species of mites that attack bees were responsible for similar dieoffs in the winters of '95-'96 and 2000-2001. And the mites may be partly to blame for the most recent honeybee losses. But a quarter of the current carnage seems unrelated to mites or any other pests. Other suggested causes of the bee decline include genetically modified foods, parasites, pesticides, and cell phone radiation. But bee expert Nicholas Calderone of Cornell University said last week that a definitive cause remains elusive. He will spend this summer investigating honeybee colonies throughout the northeast trying to solve the case of the dead bees. Here's hoping he buzzes in with an answer.</t>
   </si>
   <si>
     <t>#195 Formation of Cluster</t>
@@ -5633,7 +5633,7 @@
     <t>Astronomers have discovered a trove of __tonalities/galaxies__ that are __vacuously/virtually__ invisible—because they're made almost entirely of dark matter. The Subaru telescope in Hawaii spotted 854 of these oddballs, which are referred to as "ultradiffuse galaxies," by detecting what little light they do produce. They were all found in what's called the Coma Cluster of galaxies. The report is in The __original/Astrophysical__ Journal Letters. Of course, scientists still do not know just what dark matter is. But they can detect its __weapons/presence__ through its gravitational effects on the normal matter that we can see. That's how we know that dark matter seems to be ubiquitous in the universe—especially in these newly found, barely visible galaxies. Many of these galaxies are about the size of our Milky Way, but contain just a thousandth as many stars. __timeservers/Researchers__ estimate that dark matter accounts for 99 percent of these galaxies' mass. How such objects could form is a mystery. They probably started out with a healthy complement of __indorsing/star-forming__ gas, just like normal galaxies, but somehow lost it. The gas might have blown away as the galaxies moved through the Coma Cluster, or maybe other galaxies' gravity dragged it off. Further study of these __soothes/ultradiffuse__ galaxies should clarify the situation, and may even shine some light on the fundamental nature of dark matter.</t>
   </si>
   <si>
-    <t>Astronomers have discovered a trove of tonalities that are vacuously invisible—because they're made almost entirely of dark matter. The Subaru telescope in Hawaii spotted 854 of these oddballs, which are referred to as "ultradiffuse galaxies," by detecting what little light they do produce. They were all found in what's called the Coma Cluster of galaxies. The report is in The original Journal Letters. Of course, scientists still do not know just what dark matter is. But they can detect its weapons through its gravitational effects on the normal matter that we can see. That's how we know that dark matter seems to be ubiquitous in the universe—especially in these newly found, barely visible galaxies. Many of these galaxies are about the size of our Milky Way, but contain just a thousandth as many stars. timeservers estimate that dark matter accounts for 99 percent of these galaxies' mass. How such objects could form is a mystery. They probably started out with a healthy complement of indorsing gas, just like normal galaxies, but somehow lost it. The gas might have blown away as the galaxies moved through the Coma Cluster, or maybe other galaxies' gravity dragged it off. Further study of these soothes galaxies should clarify the situation, and may even shine some light on the fundamental nature of dark matter.</t>
+    <t>Astronomers have discovered a trove of galaxies that are virtually invisible—because they're made almost entirely of dark matter. The Subaru telescope in Hawaii spotted 854 of these oddballs, which are referred to as "ultradiffuse galaxies," by detecting what little light they do produce. They were all found in what's called the Coma Cluster of galaxies. The report is in The Astrophysical Journal Letters. Of course, scientists still do not know just what dark matter is. But they can detect its presence through its gravitational effects on the normal matter that we can see. That's how we know that dark matter seems to be ubiquitous in the universe—especially in these newly found, barely visible galaxies. Many of these galaxies are about the size of our Milky Way, but contain just a thousandth as many stars. Researchers estimate that dark matter accounts for 99 percent of these galaxies' mass. How such objects could form is a mystery. They probably started out with a healthy complement of star-forming gas, just like normal galaxies, but somehow lost it. The gas might have blown away as the galaxies moved through the Coma Cluster, or maybe other galaxies' gravity dragged it off. Further study of these ultradiffuse galaxies should clarify the situation, and may even shine some light on the fundamental nature of dark matter.</t>
   </si>
   <si>
     <t>#196 Solar Cells</t>
@@ -5642,7 +5642,7 @@
     <t>Imagine a world where sunlight can be captured to produce electricity anywhere, on any surface. The makers of thin-film __bendable/flexible__ solar cells imagine that world too. But a big problem has been the amount of silicon needed to harvest a little sunshine. Now, researchers at Caltech say they've designed a device that gets comparable solar __commotion/absorption__ while using just one percent of the silicon per unit area that current solar cells need. The work was published in the journal Nature Materials. The research team tried silicon wire arrays instead of traditional silicon panels. These wires have been charged to do a good job __coupling/converting__ sunlight to usable energy on the nanoscale. But the __hybridise/scientists__ had to create wires a thousand times longer. Light bounces around within the wires and is eventually __scrolled/absorbed__ when it hits at the correct angle. But there was a problem: too much light was leaking out. Adding nanoparticles of alumina kept much more of the light __refashioning/scattering__ until it got absorbed. The result is a system that virtually matches silicon wafer light absorption and may be more __lessened/efficient__ at converting light to electricity, while using a tiny fraction of the material.</t>
   </si>
   <si>
-    <t>Imagine a world where sunlight can be captured to produce electricity anywhere, on any surface. The makers of thin-film bendable solar cells imagine that world too. But a big problem has been the amount of silicon needed to harvest a little sunshine. Now, researchers at Caltech say they've designed a device that gets comparable solar commotion while using just one percent of the silicon per unit area that current solar cells need. The work was published in the journal Nature Materials. The research team tried silicon wire arrays instead of traditional silicon panels. These wires have been charged to do a good job coupling sunlight to usable energy on the nanoscale. But the hybridise had to create wires a thousand times longer. Light bounces around within the wires and is eventually scrolled when it hits at the correct angle. But there was a problem: too much light was leaking out. Adding nanoparticles of alumina kept much more of the light refashioning until it got absorbed. The result is a system that virtually matches silicon wafer light absorption and may be more lessened at converting light to electricity, while using a tiny fraction of the material.</t>
+    <t>Imagine a world where sunlight can be captured to produce electricity anywhere, on any surface. The makers of thin-film flexible solar cells imagine that world too. But a big problem has been the amount of silicon needed to harvest a little sunshine. Now, researchers at Caltech say they've designed a device that gets comparable solar absorption while using just one percent of the silicon per unit area that current solar cells need. The work was published in the journal Nature Materials. The research team tried silicon wire arrays instead of traditional silicon panels. These wires have been charged to do a good job converting sunlight to usable energy on the nanoscale. But the scientists had to create wires a thousand times longer. Light bounces around within the wires and is eventually absorbed when it hits at the correct angle. But there was a problem: too much light was leaking out. Adding nanoparticles of alumina kept much more of the light scattering until it got absorbed. The result is a system that virtually matches silicon wafer light absorption and may be more efficient at converting light to electricity, while using a tiny fraction of the material.</t>
   </si>
   <si>
     <t>#197 Singapore</t>
@@ -5651,7 +5651,7 @@
     <t>I am here in Durban, South Africa to report on the just __crenellate/finished__ climate change negotiations. While an agreement was reached, negotiations were in doubt throughout the three final nights. The sticking point was Singapore. Not __decor/Singapore__ specifically so much, but what Singapore represents. In 1992, Singapore was a rich __correlate/city-state__ but not yet a developed one. Nearly 20 years later, Singapore is a financial titan and a global city. So what should its obligations be to cut __heiaus/greenhouse__ gas emissions? Under old treaties, such as the Kyoto Protocol, Singapore has none. The essence of the package agreed to here in Durban is that, by 2020, Singapore will have some. Of course, Singapore in total represents less than one percent of global greenhouse gas emissions. But Singapore is joined by __commies/countries__ like South Korea—and even the world's largest greenhouse gas polluter, China—in this category of no obligations. If the Durban deal brings climate change negotiations into the 21st century and if countries like Singapore begin reducing CO2 __polygons/emissions__ after 2020, the world may not be quite as unpleasantly warm by the 22nd century.</t>
   </si>
   <si>
-    <t>I am here in Durban, South Africa to report on the just crenellate climate change negotiations. While an agreement was reached, negotiations were in doubt throughout the three final nights. The sticking point was Singapore. Not decor specifically so much, but what Singapore represents. In 1992, Singapore was a rich correlate but not yet a developed one. Nearly 20 years later, Singapore is a financial titan and a global city. So what should its obligations be to cut heiaus gas emissions? Under old treaties, such as the Kyoto Protocol, Singapore has none. The essence of the package agreed to here in Durban is that, by 2020, Singapore will have some. Of course, Singapore in total represents less than one percent of global greenhouse gas emissions. But Singapore is joined by commies like South Korea—and even the world's largest greenhouse gas polluter, China—in this category of no obligations. If the Durban deal brings climate change negotiations into the 21st century and if countries like Singapore begin reducing CO2 polygons after 2020, the world may not be quite as unpleasantly warm by the 22nd century.</t>
+    <t>I am here in Durban, South Africa to report on the just finished climate change negotiations. While an agreement was reached, negotiations were in doubt throughout the three final nights. The sticking point was Singapore. Not Singapore specifically so much, but what Singapore represents. In 1992, Singapore was a rich city-state but not yet a developed one. Nearly 20 years later, Singapore is a financial titan and a global city. So what should its obligations be to cut greenhouse gas emissions? Under old treaties, such as the Kyoto Protocol, Singapore has none. The essence of the package agreed to here in Durban is that, by 2020, Singapore will have some. Of course, Singapore in total represents less than one percent of global greenhouse gas emissions. But Singapore is joined by countries like South Korea—and even the world's largest greenhouse gas polluter, China—in this category of no obligations. If the Durban deal brings climate change negotiations into the 21st century and if countries like Singapore begin reducing CO2 emissions after 2020, the world may not be quite as unpleasantly warm by the 22nd century.</t>
   </si>
   <si>
     <t>#198 Aspirin</t>
@@ -5660,7 +5660,7 @@
     <t>Aspirin is a popular painkiller, and chances are you have some in your medicine chest right now. You might even have some in your flesh-and-blood, __troglodyte/put-a-shirt-on-it__ chest. Because a new study suggests that humans can make their own salicylic acid, which forms the bulk of aspirin's active ingredient. Scientists at Scotland's National Health Service previously __serge/observed__ that people can have salicylic acid in their blood even if they haven't recently swallowed an aspirin. Vegetarians have really high concentrations, which makes sense, given that plants make salicylic acid, so fruits and veggies are full of it. But their recent study suggests that not all of the chemical comes through the diet, because humans can take a precursor molecule and turn it into salicylic acid—results __russet/published__ in the Journal of Agricultural and Food Chemistry. The __multivitamins/researchers__ say that people might make salicylic acid to fight inflammation or disease…which would also make sense…because plants make the stuff to fight off infections. In fact, a recent study published online in the journal Nature shows how calcium released at the site of an infection tells plants to ramp up __harken/production__ of the protective compound. Just Mother Nature's way of saying, "Make two aspirin and call me when you flower."</t>
   </si>
   <si>
-    <t>Aspirin is a popular painkiller, and chances are you have some in your medicine chest right now. You might even have some in your flesh-and-blood, troglodyte chest. Because a new study suggests that humans can make their own salicylic acid, which forms the bulk of aspirin's active ingredient. Scientists at Scotland's National Health Service previously serge that people can have salicylic acid in their blood even if they haven't recently swallowed an aspirin. Vegetarians have really high concentrations, which makes sense, given that plants make salicylic acid, so fruits and veggies are full of it. But their recent study suggests that not all of the chemical comes through the diet, because humans can take a precursor molecule and turn it into salicylic acid—results russet in the Journal of Agricultural and Food Chemistry. The multivitamins say that people might make salicylic acid to fight inflammation or disease…which would also make sense…because plants make the stuff to fight off infections. In fact, a recent study published online in the journal Nature shows how calcium released at the site of an infection tells plants to ramp up harken of the protective compound. Just Mother Nature's way of saying, "Make two aspirin and call me when you flower."</t>
+    <t>Aspirin is a popular painkiller, and chances are you have some in your medicine chest right now. You might even have some in your flesh-and-blood, put-a-shirt-on-it chest. Because a new study suggests that humans can make their own salicylic acid, which forms the bulk of aspirin's active ingredient. Scientists at Scotland's National Health Service previously observed that people can have salicylic acid in their blood even if they haven't recently swallowed an aspirin. Vegetarians have really high concentrations, which makes sense, given that plants make salicylic acid, so fruits and veggies are full of it. But their recent study suggests that not all of the chemical comes through the diet, because humans can take a precursor molecule and turn it into salicylic acid—results published in the Journal of Agricultural and Food Chemistry. The researchers say that people might make salicylic acid to fight inflammation or disease…which would also make sense…because plants make the stuff to fight off infections. In fact, a recent study published online in the journal Nature shows how calcium released at the site of an infection tells plants to ramp up production of the protective compound. Just Mother Nature's way of saying, "Make two aspirin and call me when you flower."</t>
   </si>
   <si>
     <t>#199 Urban Life</t>
@@ -5669,7 +5669,7 @@
     <t>City living has obviously __phosphoenolpyruvate/influenced__ human culture—as have often been noted, how you gonna keep 'em down on the farm after they've seen Paree'? But urban life may have also influenced human genes, making the descendants of ancient city dwellers more resistant to disease. That's according to a study in the journal Evolution. The researchers started from the premise that densely populated cities would be good places for infectious diseases, which could spread easily from person to person. That situation should have set up selection pressure for the ability to survive such infections. The __minuses/scientists__ sampled the DNA of 17 populations from Africa, Asia and Europe, __chewing/including__ longtime urbanites—like Italians, Turks and Iranians—and traditionally rural or nomadic groups, like Malawians or the Saami people of northern Scandinavia. Then the researchers zeroed in on a gene variant that offers protection against diseases like tuberculosis or leprosy. After controlling for any shared __inorganically/ancestry__ between the groups, they indeed found that the protective gene was significantly more common in cultures with a long history of urban settlement. Which may be some comfort next time someone's sneezing near you on the subway.</t>
   </si>
   <si>
-    <t>City living has obviously phosphoenolpyruvate human culture—as have often been noted, how you gonna keep 'em down on the farm after they've seen Paree'? But urban life may have also influenced human genes, making the descendants of ancient city dwellers more resistant to disease. That's according to a study in the journal Evolution. The researchers started from the premise that densely populated cities would be good places for infectious diseases, which could spread easily from person to person. That situation should have set up selection pressure for the ability to survive such infections. The minuses sampled the DNA of 17 populations from Africa, Asia and Europe, chewing longtime urbanites—like Italians, Turks and Iranians—and traditionally rural or nomadic groups, like Malawians or the Saami people of northern Scandinavia. Then the researchers zeroed in on a gene variant that offers protection against diseases like tuberculosis or leprosy. After controlling for any shared inorganically between the groups, they indeed found that the protective gene was significantly more common in cultures with a long history of urban settlement. Which may be some comfort next time someone's sneezing near you on the subway.</t>
+    <t>City living has obviously influenced human culture—as have often been noted, how you gonna keep 'em down on the farm after they've seen Paree'? But urban life may have also influenced human genes, making the descendants of ancient city dwellers more resistant to disease. That's according to a study in the journal Evolution. The researchers started from the premise that densely populated cities would be good places for infectious diseases, which could spread easily from person to person. That situation should have set up selection pressure for the ability to survive such infections. The scientists sampled the DNA of 17 populations from Africa, Asia and Europe, including longtime urbanites—like Italians, Turks and Iranians—and traditionally rural or nomadic groups, like Malawians or the Saami people of northern Scandinavia. Then the researchers zeroed in on a gene variant that offers protection against diseases like tuberculosis or leprosy. After controlling for any shared ancestry between the groups, they indeed found that the protective gene was significantly more common in cultures with a long history of urban settlement. Which may be some comfort next time someone's sneezing near you on the subway.</t>
   </si>
   <si>
     <t>#200 Hearing</t>
@@ -5678,7 +5678,7 @@
     <t>Our ears are highly attuned to sounds in the world around us. It's not just the frequency of the sound itself. There are also subtle differences and shifts in loudness and pitch. That's what tells us, for instance, whether that baby crying belongs to us and just where it's located. But __warping/according__ to a recent study, what you and I hear may not sound the same. __motorcyclists/Scientists__ at the __fatality/University__ of Oxford are trying to understand how the ears and the brain work together. They fit ferrets with auditory implants, trained them to respond to sound, and then looked at the way their neurons reacted. It turns out that each ferret's neurons in the auditory cortex __untenanted/responded__ to changes in gradual differences in sound ­ but each ferret responded differently. The researchers say this is __uninhabitable/applicable__ to humans. They say this means that our brains are wired to process sounds depending on how our ears deliver that sound. So if you __handily/suddenly__ heard the world through my ears, it might sound quite different. The scientists say this research could help in the quest to design better hearing aids and speech recognition systems.</t>
   </si>
   <si>
-    <t>Our ears are highly attuned to sounds in the world around us. It's not just the frequency of the sound itself. There are also subtle differences and shifts in loudness and pitch. That's what tells us, for instance, whether that baby crying belongs to us and just where it's located. But warping to a recent study, what you and I hear may not sound the same. motorcyclists at the fatality of Oxford are trying to understand how the ears and the brain work together. They fit ferrets with auditory implants, trained them to respond to sound, and then looked at the way their neurons reacted. It turns out that each ferret's neurons in the auditory cortex untenanted to changes in gradual differences in sound ­ but each ferret responded differently. The researchers say this is uninhabitable to humans. They say this means that our brains are wired to process sounds depending on how our ears deliver that sound. So if you handily heard the world through my ears, it might sound quite different. The scientists say this research could help in the quest to design better hearing aids and speech recognition systems.</t>
+    <t>Our ears are highly attuned to sounds in the world around us. It's not just the frequency of the sound itself. There are also subtle differences and shifts in loudness and pitch. That's what tells us, for instance, whether that baby crying belongs to us and just where it's located. But according to a recent study, what you and I hear may not sound the same. Scientists at the University of Oxford are trying to understand how the ears and the brain work together. They fit ferrets with auditory implants, trained them to respond to sound, and then looked at the way their neurons reacted. It turns out that each ferret's neurons in the auditory cortex responded to changes in gradual differences in sound ­ but each ferret responded differently. The researchers say this is applicable to humans. They say this means that our brains are wired to process sounds depending on how our ears deliver that sound. So if you suddenly heard the world through my ears, it might sound quite different. The scientists say this research could help in the quest to design better hearing aids and speech recognition systems.</t>
   </si>
   <si>
     <t>#201 Dog's Walking</t>
@@ -5687,7 +5687,7 @@
     <t>If you have a dog, you know you gotta walk it. But do you know how it walks? Well, if you have no idea which foot Fido puts forward when, you're in good company. Because according to a study __sublet/published__ in the journal Current Biology, even places like natural history museums get it wrong half the time. Studies published back in the late 1800s showed that all __shriveled/four-legged__ animals walk the same way. They start by moving forward their left hind leg, __onboard/followed__ by the left front leg. Then they repeat the sequence on the right-hand side. Different animals differ in the timing of their steps. The reason they walk that way is for stability. Lifting one leg at a time leaves three feet on the ground, forming a nice stable tripod to stand on. But not __bomb/everyone__ seems to know that, even folks who should. Scientists looked at 300 depictions of animals walking—in museums, anatomy textbooks, and even children's toys. And they found that nearly half the time these images get it wrong. For a toy, that kind of inattention to detail might mean that Rex has a tendency to roll over. But for museums to mess up like that? They just don't have a leg to stand on.</t>
   </si>
   <si>
-    <t>If you have a dog, you know you gotta walk it. But do you know how it walks? Well, if you have no idea which foot Fido puts forward when, you're in good company. Because according to a study sublet in the journal Current Biology, even places like natural history museums get it wrong half the time. Studies published back in the late 1800s showed that all shriveled animals walk the same way. They start by moving forward their left hind leg, onboard by the left front leg. Then they repeat the sequence on the right-hand side. Different animals differ in the timing of their steps. The reason they walk that way is for stability. Lifting one leg at a time leaves three feet on the ground, forming a nice stable tripod to stand on. But not bomb seems to know that, even folks who should. Scientists looked at 300 depictions of animals walking—in museums, anatomy textbooks, and even children's toys. And they found that nearly half the time these images get it wrong. For a toy, that kind of inattention to detail might mean that Rex has a tendency to roll over. But for museums to mess up like that? They just don't have a leg to stand on.</t>
+    <t>If you have a dog, you know you gotta walk it. But do you know how it walks? Well, if you have no idea which foot Fido puts forward when, you're in good company. Because according to a study published in the journal Current Biology, even places like natural history museums get it wrong half the time. Studies published back in the late 1800s showed that all four-legged animals walk the same way. They start by moving forward their left hind leg, followed by the left front leg. Then they repeat the sequence on the right-hand side. Different animals differ in the timing of their steps. The reason they walk that way is for stability. Lifting one leg at a time leaves three feet on the ground, forming a nice stable tripod to stand on. But not everyone seems to know that, even folks who should. Scientists looked at 300 depictions of animals walking—in museums, anatomy textbooks, and even children's toys. And they found that nearly half the time these images get it wrong. For a toy, that kind of inattention to detail might mean that Rex has a tendency to roll over. But for museums to mess up like that? They just don't have a leg to stand on.</t>
   </si>
   <si>
     <t>#202 Obesity in America</t>
@@ -5696,7 +5696,7 @@
     <t>America's problem with obesity is well known. And more and more cats and dogs are also suffering from obesity. Now veterinarians have found that another favorite animal is in danger of serious health problems due to being just too fat: horses. Horses in Virginia were found being experiencing a big __thieves/increase__ in cases of laminitis, a __television/condition__ where the __attentive/connective__ tissue between the hoof and bone falls apart. It's what got the racehorse Barbaro. __cheeseburgers/Researchers__ at the Virginia-Maryland Regional College of Veterinary Medicine theorized that the __leeches/laminitis__ increase might be related to an epidemic of obesity, which could bring about chronic inflammation and other deleterious conditions. So they examined 300 horses randomly chosen from over a hundred farms during the summer of 2006. And they found that just over half, 51percent, were either overweight or obese. And for the same reasons as people—too many calories and too little exercise. The horses may not be overeating, though. Modern pasture plant materials were themselves bred to help foraging animals, like cattle, pack the weight on faster. Looks like horses may have been cowed into becoming fat.</t>
   </si>
   <si>
-    <t>America's problem with obesity is well known. And more and more cats and dogs are also suffering from obesity. Now veterinarians have found that another favorite animal is in danger of serious health problems due to being just too fat: horses. Horses in Virginia were found being experiencing a big thieves in cases of laminitis, a television where the attentive tissue between the hoof and bone falls apart. It's what got the racehorse Barbaro. cheeseburgers at the Virginia-Maryland Regional College of Veterinary Medicine theorized that the leeches increase might be related to an epidemic of obesity, which could bring about chronic inflammation and other deleterious conditions. So they examined 300 horses randomly chosen from over a hundred farms during the summer of 2006. And they found that just over half, 51percent, were either overweight or obese. And for the same reasons as people—too many calories and too little exercise. The horses may not be overeating, though. Modern pasture plant materials were themselves bred to help foraging animals, like cattle, pack the weight on faster. Looks like horses may have been cowed into becoming fat.</t>
+    <t>America's problem with obesity is well known. And more and more cats and dogs are also suffering from obesity. Now veterinarians have found that another favorite animal is in danger of serious health problems due to being just too fat: horses. Horses in Virginia were found being experiencing a big increase in cases of laminitis, a condition where the connective tissue between the hoof and bone falls apart. It's what got the racehorse Barbaro. Researchers at the Virginia-Maryland Regional College of Veterinary Medicine theorized that the laminitis increase might be related to an epidemic of obesity, which could bring about chronic inflammation and other deleterious conditions. So they examined 300 horses randomly chosen from over a hundred farms during the summer of 2006. And they found that just over half, 51percent, were either overweight or obese. And for the same reasons as people—too many calories and too little exercise. The horses may not be overeating, though. Modern pasture plant materials were themselves bred to help foraging animals, like cattle, pack the weight on faster. Looks like horses may have been cowed into becoming fat.</t>
   </si>
   <si>
     <t>#203 Alaska</t>
@@ -5705,7 +5705,7 @@
     <t>"What happened was the whole Gulf of Alaska and Prince William Sound just sort of tilted, and so near shore, near Alaska, that region sink. And then out at sea, the sea floor raised up." Susie Bassham, a __expenditure/molecular__ biologist at the University of Oregon. "And so things that were submarine platforms before suddenly were lifted above sea level, and then silt could come in and build more island." And with more island, came new __widower/freshwater__ ponds. Those newly created bodies of water turned out to be the testbed for a natural evolutionary experiment on a finger-sized fish, called the __calcified/three-spined__ stickleback. Saltwater fish went in… freshwater fish came out. "Big silvery __uninterested/well-armored__ fish entered freshwater ponds. And during the last 50 years they changed their size, their coloration, they changed the size of their eyes, the length of their spines, many aspects of their skeletons, feeding structures, swimming structures, and became more stereotypical freshwater fish." But how? Bassham and her colleagues ran statistical __cleaves/analyses__ on the genomes and body measurements of fish living in those freshwater ponds today. And they found that the saltwater versions of the fish may have actually colonized those freshwater ponds on the study islands at least six times in the last 50 years. They were able to move in and rapidly adapt because the sea-dwelling fish have a sort of "sleeper genome" of freshwater traits, just waiting to be activated.</t>
   </si>
   <si>
-    <t>"What happened was the whole Gulf of Alaska and Prince William Sound just sort of tilted, and so near shore, near Alaska, that region sink. And then out at sea, the sea floor raised up." Susie Bassham, a expenditure biologist at the University of Oregon. "And so things that were submarine platforms before suddenly were lifted above sea level, and then silt could come in and build more island." And with more island, came new widower ponds. Those newly created bodies of water turned out to be the testbed for a natural evolutionary experiment on a finger-sized fish, called the calcified stickleback. Saltwater fish went in… freshwater fish came out. "Big silvery uninterested fish entered freshwater ponds. And during the last 50 years they changed their size, their coloration, they changed the size of their eyes, the length of their spines, many aspects of their skeletons, feeding structures, swimming structures, and became more stereotypical freshwater fish." But how? Bassham and her colleagues ran statistical cleaves on the genomes and body measurements of fish living in those freshwater ponds today. And they found that the saltwater versions of the fish may have actually colonized those freshwater ponds on the study islands at least six times in the last 50 years. They were able to move in and rapidly adapt because the sea-dwelling fish have a sort of "sleeper genome" of freshwater traits, just waiting to be activated.</t>
+    <t>"What happened was the whole Gulf of Alaska and Prince William Sound just sort of tilted, and so near shore, near Alaska, that region sink. And then out at sea, the sea floor raised up." Susie Bassham, a molecular biologist at the University of Oregon. "And so things that were submarine platforms before suddenly were lifted above sea level, and then silt could come in and build more island." And with more island, came new freshwater ponds. Those newly created bodies of water turned out to be the testbed for a natural evolutionary experiment on a finger-sized fish, called the three-spined stickleback. Saltwater fish went in… freshwater fish came out. "Big silvery well-armored fish entered freshwater ponds. And during the last 50 years they changed their size, their coloration, they changed the size of their eyes, the length of their spines, many aspects of their skeletons, feeding structures, swimming structures, and became more stereotypical freshwater fish." But how? Bassham and her colleagues ran statistical analyses on the genomes and body measurements of fish living in those freshwater ponds today. And they found that the saltwater versions of the fish may have actually colonized those freshwater ponds on the study islands at least six times in the last 50 years. They were able to move in and rapidly adapt because the sea-dwelling fish have a sort of "sleeper genome" of freshwater traits, just waiting to be activated.</t>
   </si>
   <si>
     <t>#204 Genome Sequence</t>
@@ -5714,7 +5714,7 @@
     <t>Since the first human genome sequence was published, __groundless/thousands__ of people have submitted their DNA for scientific analysis. They made these donations anonymously—or so they thought. Now, using publicly available information, researchers found they could figure out the identities of 50 individuals who had loaned their genes to science. Their results, although not the names of the people, are in the journal Science. Biomedical research depends on the human subjects, and issues of privacy have always been a concern. When scientists share genomic data, they first strip away identifying information, like the individual's name and date of birth. But is that really enough? __siestas/Researchers__ looked at a __patronymic/specific__ set of markers in genomes whose __heedlessness/sequences__ were in a public database. And they found that by __taxing/matching__ up these markers with sequences that people had submitted to genealogy web sites, they could identify some of the genome donors' relatives and, with a bit more sleuthing, come up with their actual names. Of course, many people now post online accounts of what's on their minds or even on their menus. But even those who are relatively relaxed about their privacy might think twice about their genomes going public.</t>
   </si>
   <si>
-    <t>Since the first human genome sequence was published, groundless of people have submitted their DNA for scientific analysis. They made these donations anonymously—or so they thought. Now, using publicly available information, researchers found they could figure out the identities of 50 individuals who had loaned their genes to science. Their results, although not the names of the people, are in the journal Science. Biomedical research depends on the human subjects, and issues of privacy have always been a concern. When scientists share genomic data, they first strip away identifying information, like the individual's name and date of birth. But is that really enough? siestas looked at a patronymic set of markers in genomes whose heedlessness were in a public database. And they found that by taxing up these markers with sequences that people had submitted to genealogy web sites, they could identify some of the genome donors' relatives and, with a bit more sleuthing, come up with their actual names. Of course, many people now post online accounts of what's on their minds or even on their menus. But even those who are relatively relaxed about their privacy might think twice about their genomes going public.</t>
+    <t>Since the first human genome sequence was published, thousands of people have submitted their DNA for scientific analysis. They made these donations anonymously—or so they thought. Now, using publicly available information, researchers found they could figure out the identities of 50 individuals who had loaned their genes to science. Their results, although not the names of the people, are in the journal Science. Biomedical research depends on the human subjects, and issues of privacy have always been a concern. When scientists share genomic data, they first strip away identifying information, like the individual's name and date of birth. But is that really enough? Researchers looked at a specific set of markers in genomes whose sequences were in a public database. And they found that by matching up these markers with sequences that people had submitted to genealogy web sites, they could identify some of the genome donors' relatives and, with a bit more sleuthing, come up with their actual names. Of course, many people now post online accounts of what's on their minds or even on their menus. But even those who are relatively relaxed about their privacy might think twice about their genomes going public.</t>
   </si>
   <si>
     <t>#205 Happy Hour</t>
@@ -5723,7 +5723,7 @@
     <t>As we recover from the holiday weekend, there's some __reverberating/intoxicating__ news on curbing the effects of alcohol. In the May 29th issue of Cell, __silences/scientists__ report __unburdening/discovering__ a gene that controls fruit flies' __alphabetically/sensitivity__ to ethanol. And if that just sounds like tipsytalk, the finding __realms/suggests__ that a couple of current anticancer drugs might find use in treating alcoholism. Some flies, like some people, just can't hold their drink. One sip and they're tripping over their own wings. So the scientists set out to search for the fly genes involved in alcohol sensitivity. And they turned up a gene they call happyhour. Flies with a normal version of this gene are liquor light-weights, while __twelvehour/happyhour__ mutants can drink their fly friends under the table. In the normal flies, happyhour blocks a hormone called EGF. And the scientists found that two anticancer drugs, which also inhibit EGF, make boozing flies more woozy—a feeling that's as unpleasant for flies as it is for people. Rats, too, will take a nip and say enough when they're on these drugs. Robbing booze of its buzz is one way to attack alcoholism. Which means that, at least genetically speaking, it's good to have a little happyhour.</t>
   </si>
   <si>
-    <t>As we recover from the holiday weekend, there's some reverberating news on curbing the effects of alcohol. In the May 29th issue of Cell, silences report unburdening a gene that controls fruit flies' alphabetically to ethanol. And if that just sounds like tipsytalk, the finding realms that a couple of current anticancer drugs might find use in treating alcoholism. Some flies, like some people, just can't hold their drink. One sip and they're tripping over their own wings. So the scientists set out to search for the fly genes involved in alcohol sensitivity. And they turned up a gene they call happyhour. Flies with a normal version of this gene are liquor light-weights, while twelvehour mutants can drink their fly friends under the table. In the normal flies, happyhour blocks a hormone called EGF. And the scientists found that two anticancer drugs, which also inhibit EGF, make boozing flies more woozy—a feeling that's as unpleasant for flies as it is for people. Rats, too, will take a nip and say enough when they're on these drugs. Robbing booze of its buzz is one way to attack alcoholism. Which means that, at least genetically speaking, it's good to have a little happyhour.</t>
+    <t>As we recover from the holiday weekend, there's some intoxicating news on curbing the effects of alcohol. In the May 29th issue of Cell, scientists report discovering a gene that controls fruit flies' sensitivity to ethanol. And if that just sounds like tipsytalk, the finding suggests that a couple of current anticancer drugs might find use in treating alcoholism. Some flies, like some people, just can't hold their drink. One sip and they're tripping over their own wings. So the scientists set out to search for the fly genes involved in alcohol sensitivity. And they turned up a gene they call happyhour. Flies with a normal version of this gene are liquor light-weights, while happyhour mutants can drink their fly friends under the table. In the normal flies, happyhour blocks a hormone called EGF. And the scientists found that two anticancer drugs, which also inhibit EGF, make boozing flies more woozy—a feeling that's as unpleasant for flies as it is for people. Rats, too, will take a nip and say enough when they're on these drugs. Robbing booze of its buzz is one way to attack alcoholism. Which means that, at least genetically speaking, it's good to have a little happyhour.</t>
   </si>
   <si>
     <t>#206 HIW</t>
@@ -5732,7 +5732,7 @@
     <t>The floor of __arithmetically/Yosemite__ Valley is littered with piles of rocks that crumbled off the park's iconic cliffs. These rockfalls happen all the time, because Yosemite's granite walls are riddled with cracks produced by geologic stress. Scientists know the rockfalls can be triggered by things like earthquakes, rainfall, and freezing and thawing ice. But many falls occur without an obvious cause. Now __steelworkers/researchers__ think that heat may be the culprit. "We noticed that there had been a bunch of rockfalls that were happening in the summertime, on particularly hot days." Brian Collins, a research civil engineer with the U.S. Geological Survey. "And we noticed when we looked at the timing that they were happening in the afternoon, when we thought the temperatures were at their hottest." Collins and Greg Stock, Yosemite's park geologist, wanted to know if small rock movements, induced by changing temperatures, might weaken cracks and contribute to rockfalls. So the researchers—who are both climbers—found a suitable __coauthor/fracture__ near the base of a 500-meter-tall cliff and installed instruments called crackmeters, which monitored the width of the crack over time. The devices __misread/revealed__ that the crack grew almost a centimeter wider during the warmest part of the day. It shrank again when temperatures cooled off, for instance, at night and during the winter. But overall, the scientists found that the average width of the fracture grew over the course of a summer and over the entire three and a half-year study period, bringing the crack closer to breaking. "We think that what happened was that every cycle — as the rock goes back and forth and back and forth — you're getting to a part that we call subcritical crack growth. And that means that the crack where the rock is attached to the cliff is actually fracturing at a microscopic level. And so if you do that over the course of a year, then eventually you're gonna do some permanent damage to those points of attachment." The study is in the journal Nature Geoscience. The slab of rock the scientists studied hasn't fallen yet, and Collins doesn't know how many cycles it will take before this or any other fracture finally breaks. When it does, the trigger might be a particularly sweltering day, when the partially __start/detached__ slab is farthest away from the cliff. Or it could be another process, helped along by the fact that temperature changes already weakened the crack. Either way, the results will help researchers assess the rockfall hazard in steep, rugged terrain. Because now they know when the mercury goes up, rocks are more likely to come down.</t>
   </si>
   <si>
-    <t>The floor of arithmetically Valley is littered with piles of rocks that crumbled off the park's iconic cliffs. These rockfalls happen all the time, because Yosemite's granite walls are riddled with cracks produced by geologic stress. Scientists know the rockfalls can be triggered by things like earthquakes, rainfall, and freezing and thawing ice. But many falls occur without an obvious cause. Now steelworkers think that heat may be the culprit. "We noticed that there had been a bunch of rockfalls that were happening in the summertime, on particularly hot days." Brian Collins, a research civil engineer with the U.S. Geological Survey. "And we noticed when we looked at the timing that they were happening in the afternoon, when we thought the temperatures were at their hottest." Collins and Greg Stock, Yosemite's park geologist, wanted to know if small rock movements, induced by changing temperatures, might weaken cracks and contribute to rockfalls. So the researchers—who are both climbers—found a suitable coauthor near the base of a 500-meter-tall cliff and installed instruments called crackmeters, which monitored the width of the crack over time. The devices misread that the crack grew almost a centimeter wider during the warmest part of the day. It shrank again when temperatures cooled off, for instance, at night and during the winter. But overall, the scientists found that the average width of the fracture grew over the course of a summer and over the entire three and a half-year study period, bringing the crack closer to breaking. "We think that what happened was that every cycle — as the rock goes back and forth and back and forth — you're getting to a part that we call subcritical crack growth. And that means that the crack where the rock is attached to the cliff is actually fracturing at a microscopic level. And so if you do that over the course of a year, then eventually you're gonna do some permanent damage to those points of attachment." The study is in the journal Nature Geoscience. The slab of rock the scientists studied hasn't fallen yet, and Collins doesn't know how many cycles it will take before this or any other fracture finally breaks. When it does, the trigger might be a particularly sweltering day, when the partially start slab is farthest away from the cliff. Or it could be another process, helped along by the fact that temperature changes already weakened the crack. Either way, the results will help researchers assess the rockfall hazard in steep, rugged terrain. Because now they know when the mercury goes up, rocks are more likely to come down.</t>
+    <t>The floor of Yosemite Valley is littered with piles of rocks that crumbled off the park's iconic cliffs. These rockfalls happen all the time, because Yosemite's granite walls are riddled with cracks produced by geologic stress. Scientists know the rockfalls can be triggered by things like earthquakes, rainfall, and freezing and thawing ice. But many falls occur without an obvious cause. Now researchers think that heat may be the culprit. "We noticed that there had been a bunch of rockfalls that were happening in the summertime, on particularly hot days." Brian Collins, a research civil engineer with the U.S. Geological Survey. "And we noticed when we looked at the timing that they were happening in the afternoon, when we thought the temperatures were at their hottest." Collins and Greg Stock, Yosemite's park geologist, wanted to know if small rock movements, induced by changing temperatures, might weaken cracks and contribute to rockfalls. So the researchers—who are both climbers—found a suitable fracture near the base of a 500-meter-tall cliff and installed instruments called crackmeters, which monitored the width of the crack over time. The devices revealed that the crack grew almost a centimeter wider during the warmest part of the day. It shrank again when temperatures cooled off, for instance, at night and during the winter. But overall, the scientists found that the average width of the fracture grew over the course of a summer and over the entire three and a half-year study period, bringing the crack closer to breaking. "We think that what happened was that every cycle — as the rock goes back and forth and back and forth — you're getting to a part that we call subcritical crack growth. And that means that the crack where the rock is attached to the cliff is actually fracturing at a microscopic level. And so if you do that over the course of a year, then eventually you're gonna do some permanent damage to those points of attachment." The study is in the journal Nature Geoscience. The slab of rock the scientists studied hasn't fallen yet, and Collins doesn't know how many cycles it will take before this or any other fracture finally breaks. When it does, the trigger might be a particularly sweltering day, when the partially detached slab is farthest away from the cliff. Or it could be another process, helped along by the fact that temperature changes already weakened the crack. Either way, the results will help researchers assess the rockfall hazard in steep, rugged terrain. Because now they know when the mercury goes up, rocks are more likely to come down.</t>
   </si>
   <si>
     <t>#207 HIW</t>
@@ -5741,7 +5741,7 @@
     <t>The element mercury has been shown to damage the human nervous system. Yet, since 1856, mercury amalgam is "the" filling dentists have used to repair our teeth. Now a study in the journal Chemical Research in Toxicology __fluctuates/indicates__ that mercury fillings actually lose their toxic potential over time. __gymnasium/Canadian__ __ripeness/scientists__ used x-ray spectroscopy to compare new mercury amalgams to those about 20 years old. After two decades, 95 percent of the elemental mercury on the surface of a filling had gone through a chemical reaction. It became __catastrophe/beta-mercury__ sulfide, a black-colored solid. Which __invades/explains__ why fillings dull with age. And the compound isn't absorbed by the body, which means it can't affect the body the way elemental mercury can. Of course, this study does not settle the __extradition/question__ of how __timidity/potentially__ harmful a new mercury filling is. But sulfide-rich foods, such as coffee, garlic and onions, may accelerate the change from metallic mercury into the safer sulfide. So if you have a new mercury filling, an odiferous chili dog with a cup of coffee may be just what the doctor ordered.</t>
   </si>
   <si>
-    <t>The element mercury has been shown to damage the human nervous system. Yet, since 1856, mercury amalgam is "the" filling dentists have used to repair our teeth. Now a study in the journal Chemical Research in Toxicology fluctuates that mercury fillings actually lose their toxic potential over time. gymnasium ripeness used x-ray spectroscopy to compare new mercury amalgams to those about 20 years old. After two decades, 95 percent of the elemental mercury on the surface of a filling had gone through a chemical reaction. It became catastrophe sulfide, a black-colored solid. Which invades why fillings dull with age. And the compound isn't absorbed by the body, which means it can't affect the body the way elemental mercury can. Of course, this study does not settle the extradition of how timidity harmful a new mercury filling is. But sulfide-rich foods, such as coffee, garlic and onions, may accelerate the change from metallic mercury into the safer sulfide. So if you have a new mercury filling, an odiferous chili dog with a cup of coffee may be just what the doctor ordered.</t>
+    <t>The element mercury has been shown to damage the human nervous system. Yet, since 1856, mercury amalgam is "the" filling dentists have used to repair our teeth. Now a study in the journal Chemical Research in Toxicology indicates that mercury fillings actually lose their toxic potential over time. Canadian scientists used x-ray spectroscopy to compare new mercury amalgams to those about 20 years old. After two decades, 95 percent of the elemental mercury on the surface of a filling had gone through a chemical reaction. It became beta-mercury sulfide, a black-colored solid. Which explains why fillings dull with age. And the compound isn't absorbed by the body, which means it can't affect the body the way elemental mercury can. Of course, this study does not settle the question of how potentially harmful a new mercury filling is. But sulfide-rich foods, such as coffee, garlic and onions, may accelerate the change from metallic mercury into the safer sulfide. So if you have a new mercury filling, an odiferous chili dog with a cup of coffee may be just what the doctor ordered.</t>
   </si>
   <si>
     <t>#208 Antibiotic Resistance</t>
@@ -5750,7 +5750,7 @@
     <t>For years, __licences/scientists__ and physicians have been up in arms about the rise in antibiotic resistance. Seems that many bacteria, devious buggers that they are, are able to share genetic information—including, say, the instructions for __overjoying/destroying__ penicillin. Well, if that's not bad enough, scientists in the N.Y.U. School of Medicine have found that some bacteria can use viruses to help them pass along the recipe for their favorite toxin, results __punished/published__ in the journal Science. Like humans, bacteria are also prone to infection by viruses. And most of these viruses—called bacteriophage, or phage for short—make their bacterial victims sick. Or even dead. But in the laboratory, the scientists discovered that Staphylococcus aureus, the bug that causes toxic shock __airdrome/syndrome__ among other things, can __multilaterally/actually__ co-opt phage, using them to shuttle the gene for toxic-shock toxin to another bacteria, in this case Listeria. That's doubly nasty, because Listeria on its own causes food poisoning, so if it added toxic shock to its repertoire, well, that would be one seriously bad bug. Whether Staph aureus can pull off this stunt outside the lab's not clear. But in this particular battle, ya gotta hope the viruses come out on top.</t>
   </si>
   <si>
-    <t>For years, licences and physicians have been up in arms about the rise in antibiotic resistance. Seems that many bacteria, devious buggers that they are, are able to share genetic information—including, say, the instructions for overjoying penicillin. Well, if that's not bad enough, scientists in the N.Y.U. School of Medicine have found that some bacteria can use viruses to help them pass along the recipe for their favorite toxin, results punished in the journal Science. Like humans, bacteria are also prone to infection by viruses. And most of these viruses—called bacteriophage, or phage for short—make their bacterial victims sick. Or even dead. But in the laboratory, the scientists discovered that Staphylococcus aureus, the bug that causes toxic shock airdrome among other things, can multilaterally co-opt phage, using them to shuttle the gene for toxic-shock toxin to another bacteria, in this case Listeria. That's doubly nasty, because Listeria on its own causes food poisoning, so if it added toxic shock to its repertoire, well, that would be one seriously bad bug. Whether Staph aureus can pull off this stunt outside the lab's not clear. But in this particular battle, ya gotta hope the viruses come out on top.</t>
+    <t>For years, scientists and physicians have been up in arms about the rise in antibiotic resistance. Seems that many bacteria, devious buggers that they are, are able to share genetic information—including, say, the instructions for destroying penicillin. Well, if that's not bad enough, scientists in the N.Y.U. School of Medicine have found that some bacteria can use viruses to help them pass along the recipe for their favorite toxin, results published in the journal Science. Like humans, bacteria are also prone to infection by viruses. And most of these viruses—called bacteriophage, or phage for short—make their bacterial victims sick. Or even dead. But in the laboratory, the scientists discovered that Staphylococcus aureus, the bug that causes toxic shock syndrome among other things, can actually co-opt phage, using them to shuttle the gene for toxic-shock toxin to another bacteria, in this case Listeria. That's doubly nasty, because Listeria on its own causes food poisoning, so if it added toxic shock to its repertoire, well, that would be one seriously bad bug. Whether Staph aureus can pull off this stunt outside the lab's not clear. But in this particular battle, ya gotta hope the viruses come out on top.</t>
   </si>
   <si>
     <t>#209 HIW</t>
@@ -5759,7 +5759,7 @@
     <t>As kids, many of us pondered what stars are made of. . Some __ogled/grown-up__ astronomers, on the other hand, wonder about where stars came from. Now, a study serves up a surprise. Because it seems that the smallest galaxies in the __averse/universe__ gave rise to an __cryptically/unexpectedly__ large proportion of stars. The findings are in the Astrophysical Journal. Most of the stars we see in the sky were formed when the universe was young, just a few billion years after the Big Bang. So to study stellar origins, scientists use telescopes that allow them to see galaxies that are so far away, they're __felony/essentially__ looking back in time. Previous observations had focused on the star-forming powers of larger galaxies. But in this latest study, researchers used data collected by a __countable/powerful__ camera aboard the Hubble Space Telescope. With this instrument, they could eyeball smaller, dwarf galaxies. And they found that these diminutive dynamos churned out stars at a furious rate, fast enough to double their mass in only 150 million years. That __iambuses/reproductive__ feat would take most __salt/so-called__ "normal" galaxies one to three billion years. Seems the universe has long known what Danny Devito, Michael J. Fox and Dustin Hoffmann later proved: You don't have to be big to have real star power.</t>
   </si>
   <si>
-    <t>As kids, many of us pondered what stars are made of. . Some ogled astronomers, on the other hand, wonder about where stars came from. Now, a study serves up a surprise. Because it seems that the smallest galaxies in the averse gave rise to an cryptically large proportion of stars. The findings are in the Astrophysical Journal. Most of the stars we see in the sky were formed when the universe was young, just a few billion years after the Big Bang. So to study stellar origins, scientists use telescopes that allow them to see galaxies that are so far away, they're felony looking back in time. Previous observations had focused on the star-forming powers of larger galaxies. But in this latest study, researchers used data collected by a countable camera aboard the Hubble Space Telescope. With this instrument, they could eyeball smaller, dwarf galaxies. And they found that these diminutive dynamos churned out stars at a furious rate, fast enough to double their mass in only 150 million years. That iambuses feat would take most salt "normal" galaxies one to three billion years. Seems the universe has long known what Danny Devito, Michael J. Fox and Dustin Hoffmann later proved: You don't have to be big to have real star power.</t>
+    <t>As kids, many of us pondered what stars are made of. . Some grown-up astronomers, on the other hand, wonder about where stars came from. Now, a study serves up a surprise. Because it seems that the smallest galaxies in the universe gave rise to an unexpectedly large proportion of stars. The findings are in the Astrophysical Journal. Most of the stars we see in the sky were formed when the universe was young, just a few billion years after the Big Bang. So to study stellar origins, scientists use telescopes that allow them to see galaxies that are so far away, they're essentially looking back in time. Previous observations had focused on the star-forming powers of larger galaxies. But in this latest study, researchers used data collected by a powerful camera aboard the Hubble Space Telescope. With this instrument, they could eyeball smaller, dwarf galaxies. And they found that these diminutive dynamos churned out stars at a furious rate, fast enough to double their mass in only 150 million years. That reproductive feat would take most so-called "normal" galaxies one to three billion years. Seems the universe has long known what Danny Devito, Michael J. Fox and Dustin Hoffmann later proved: You don't have to be big to have real star power.</t>
   </si>
   <si>
     <t>#210 Bookworm</t>
@@ -5768,7 +5768,7 @@
     <t>What does a bookworm have in common with a __mulcted/black-tufted__ marmoset? They both like a little quiet. Or so say __sanitises/scientists__ in the Royal Society journal Biology Letters. As urban areas continue to expand, their human inhabitants spread all sorts of pollution: air pollution, light pollution, even noise pollution. Each of these environmental __postmarks/encroachments__ affects the survival and behavior of local wildlife. And monkeys are no exception. __licences/Scientists__ in Brazil were __parleying/studying__ how marmosets in a city park cope with ambient noise. And they found that the monkeys tend to settle down in __metier/whatever__ part of the park is most quiet. On weekdays, the marmosets steered clear of the roar of traffic, and on Sundays they shunned the clamor of visiting crowds. They dodged all the din, even when moving meant that they had to leave behind the places that offered them the most food. It could be that the monkeys are just skittish when it comes to unwelcome sounds. Or they can't hear what their friends are saying when it gets too loud. Either way, next time you see a cute little marmoset, forget "oooh" or "awwww" or "ee-ee-ee." Try shhhh.</t>
   </si>
   <si>
-    <t>What does a bookworm have in common with a mulcted marmoset? They both like a little quiet. Or so say sanitises in the Royal Society journal Biology Letters. As urban areas continue to expand, their human inhabitants spread all sorts of pollution: air pollution, light pollution, even noise pollution. Each of these environmental postmarks affects the survival and behavior of local wildlife. And monkeys are no exception. licences in Brazil were parleying how marmosets in a city park cope with ambient noise. And they found that the monkeys tend to settle down in metier part of the park is most quiet. On weekdays, the marmosets steered clear of the roar of traffic, and on Sundays they shunned the clamor of visiting crowds. They dodged all the din, even when moving meant that they had to leave behind the places that offered them the most food. It could be that the monkeys are just skittish when it comes to unwelcome sounds. Or they can't hear what their friends are saying when it gets too loud. Either way, next time you see a cute little marmoset, forget "oooh" or "awwww" or "ee-ee-ee." Try shhhh.</t>
+    <t>What does a bookworm have in common with a black-tufted marmoset? They both like a little quiet. Or so say scientists in the Royal Society journal Biology Letters. As urban areas continue to expand, their human inhabitants spread all sorts of pollution: air pollution, light pollution, even noise pollution. Each of these environmental encroachments affects the survival and behavior of local wildlife. And monkeys are no exception. Scientists in Brazil were studying how marmosets in a city park cope with ambient noise. And they found that the monkeys tend to settle down in whatever part of the park is most quiet. On weekdays, the marmosets steered clear of the roar of traffic, and on Sundays they shunned the clamor of visiting crowds. They dodged all the din, even when moving meant that they had to leave behind the places that offered them the most food. It could be that the monkeys are just skittish when it comes to unwelcome sounds. Or they can't hear what their friends are saying when it gets too loud. Either way, next time you see a cute little marmoset, forget "oooh" or "awwww" or "ee-ee-ee." Try shhhh.</t>
   </si>
   <si>
     <t>#211 Astronaut</t>
@@ -5777,7 +5777,7 @@
     <t>The space shuttle Discovery, mission STS-128, is in orbit right now. With some fascinating people on board. Pilot Kevin Ford became interested in flying when he was a kid and read the book Carrying the Fire, by Michael Collins, command module pilot on Apollo 11. When he was old enough to take flying lessons, Ford paid for them with money he earned bagging groceries. Mission Specialist Jose __washes/Hernandez__ was born in California, into a family of migrant farm workers. He spent his childhood __tattering/shuttling__ between Mexico and California, working in the fields and speaking little English. But during the school year, his parents, who possessed only __placed/third-grade__ educations, had him and his siblings attend school full time and help with the work only on weekends. His second-grade teacher in California convinced his parents to set down roots for the sake of the children's educations. In high school, Hernandez was inspired by __font/astronaut__ Franklin Chang-Diaz, and set his course on becoming an astronaut himself. The whole crew has great life stories—and degrees in __smelling/engineering__ or science. Check them out at www.snipurl.com/sts128.</t>
   </si>
   <si>
-    <t>The space shuttle Discovery, mission STS-128, is in orbit right now. With some fascinating people on board. Pilot Kevin Ford became interested in flying when he was a kid and read the book Carrying the Fire, by Michael Collins, command module pilot on Apollo 11. When he was old enough to take flying lessons, Ford paid for them with money he earned bagging groceries. Mission Specialist Jose washes was born in California, into a family of migrant farm workers. He spent his childhood tattering between Mexico and California, working in the fields and speaking little English. But during the school year, his parents, who possessed only placed educations, had him and his siblings attend school full time and help with the work only on weekends. His second-grade teacher in California convinced his parents to set down roots for the sake of the children's educations. In high school, Hernandez was inspired by font Franklin Chang-Diaz, and set his course on becoming an astronaut himself. The whole crew has great life stories—and degrees in smelling or science. Check them out at www.snipurl.com/sts128.</t>
+    <t>The space shuttle Discovery, mission STS-128, is in orbit right now. With some fascinating people on board. Pilot Kevin Ford became interested in flying when he was a kid and read the book Carrying the Fire, by Michael Collins, command module pilot on Apollo 11. When he was old enough to take flying lessons, Ford paid for them with money he earned bagging groceries. Mission Specialist Jose Hernandez was born in California, into a family of migrant farm workers. He spent his childhood shuttling between Mexico and California, working in the fields and speaking little English. But during the school year, his parents, who possessed only third-grade educations, had him and his siblings attend school full time and help with the work only on weekends. His second-grade teacher in California convinced his parents to set down roots for the sake of the children's educations. In high school, Hernandez was inspired by astronaut Franklin Chang-Diaz, and set his course on becoming an astronaut himself. The whole crew has great life stories—and degrees in engineering or science. Check them out at www.snipurl.com/sts128.</t>
   </si>
   <si>
     <t>#212 Bird Buffet</t>
@@ -5786,7 +5786,7 @@
     <t>If you've ever been to an all-you-can-eat buffet, you know how __contorted/important__ it is to carefully weigh your options. You don't want to fill up on salad when so many calorie-laden __dimes/delights__ await. It seems some birds also weigh their mealtime choices—literally. A study finds that Mexican Jays pick up and shake peanuts to assess their relative heft before choosing one. That report is served up in the Journal of Ornithology. Foods that hide their edible bits on the inside present a challenge to hungry diners. How can you tell which fruits are ripe or which shells harbor the biggest nuts? We humans knock on melons or squeeze avocados. But how do other species select the highest quality snacks? To find out how the jays do it, __sheepherders/researchers__ fiddled with their feed. First they __buffered/doctored__ peanuts so that some __distillate/contained__ three nuts while others had none. When they offered these pods to some jays, the birds turned their beaks up at the empty shells and instead chose those that were full. And when the jays were allowed to choose between normal peanuts and those that weighed just one gram more, because the researchers had stuffed them with clay, the birds again went for the heavier meal. Videos __concede/revealed__ that the jays shake the nuts before selecting one, which apparently lets them gauge the nut's mass and perhaps also listen for the rattle of a well-packed shell. Pretty clever for a bird brain.</t>
   </si>
   <si>
-    <t>If you've ever been to an all-you-can-eat buffet, you know how contorted it is to carefully weigh your options. You don't want to fill up on salad when so many calorie-laden dimes await. It seems some birds also weigh their mealtime choices—literally. A study finds that Mexican Jays pick up and shake peanuts to assess their relative heft before choosing one. That report is served up in the Journal of Ornithology. Foods that hide their edible bits on the inside present a challenge to hungry diners. How can you tell which fruits are ripe or which shells harbor the biggest nuts? We humans knock on melons or squeeze avocados. But how do other species select the highest quality snacks? To find out how the jays do it, sheepherders fiddled with their feed. First they buffered peanuts so that some distillate three nuts while others had none. When they offered these pods to some jays, the birds turned their beaks up at the empty shells and instead chose those that were full. And when the jays were allowed to choose between normal peanuts and those that weighed just one gram more, because the researchers had stuffed them with clay, the birds again went for the heavier meal. Videos concede that the jays shake the nuts before selecting one, which apparently lets them gauge the nut's mass and perhaps also listen for the rattle of a well-packed shell. Pretty clever for a bird brain.</t>
+    <t>If you've ever been to an all-you-can-eat buffet, you know how important it is to carefully weigh your options. You don't want to fill up on salad when so many calorie-laden delights await. It seems some birds also weigh their mealtime choices—literally. A study finds that Mexican Jays pick up and shake peanuts to assess their relative heft before choosing one. That report is served up in the Journal of Ornithology. Foods that hide their edible bits on the inside present a challenge to hungry diners. How can you tell which fruits are ripe or which shells harbor the biggest nuts? We humans knock on melons or squeeze avocados. But how do other species select the highest quality snacks? To find out how the jays do it, researchers fiddled with their feed. First they doctored peanuts so that some contained three nuts while others had none. When they offered these pods to some jays, the birds turned their beaks up at the empty shells and instead chose those that were full. And when the jays were allowed to choose between normal peanuts and those that weighed just one gram more, because the researchers had stuffed them with clay, the birds again went for the heavier meal. Videos revealed that the jays shake the nuts before selecting one, which apparently lets them gauge the nut's mass and perhaps also listen for the rattle of a well-packed shell. Pretty clever for a bird brain.</t>
   </si>
   <si>
     <t>#213 Eating Background</t>
@@ -5795,7 +5795,7 @@
     <t>In lab tests, music and lighting can affect how much people eat. Now a study has found that changing the ambiance of a fast food restaurant to more of a fine-dining atmosphere lessened the amount of food people crammed into their pie holes. To quote the paper, "softening the lighting and music led people to eat less, to rate the food as more enjoyable, and to spend just as much." That last finding means that fast food joints, which are accused of __noncontributing/contributing__ to the obesity epidemic, might __predominately/actually__ try it. The study was led by well-known eating behaviorist Brian Wansink from Cornell University and appears in the journal Psychological Reports. The researchers __refunded/converted__ part of a Hardee's so that it had soft lighting and slow jazz instrumentals. The patrons were expected to possibly eat more in the relaxed section, because they'd linger, maybe get dessert. But they actually averaged 18 percent fewer __shrubberies/calories__ per meal than the folks in the rowdy section—down from an average of 949 calories to 775. The overall experience appears to have been a more satisfying meal. Even if there was less of it.</t>
   </si>
   <si>
-    <t>In lab tests, music and lighting can affect how much people eat. Now a study has found that changing the ambiance of a fast food restaurant to more of a fine-dining atmosphere lessened the amount of food people crammed into their pie holes. To quote the paper, "softening the lighting and music led people to eat less, to rate the food as more enjoyable, and to spend just as much." That last finding means that fast food joints, which are accused of noncontributing to the obesity epidemic, might predominately try it. The study was led by well-known eating behaviorist Brian Wansink from Cornell University and appears in the journal Psychological Reports. The researchers refunded part of a Hardee's so that it had soft lighting and slow jazz instrumentals. The patrons were expected to possibly eat more in the relaxed section, because they'd linger, maybe get dessert. But they actually averaged 18 percent fewer shrubberies per meal than the folks in the rowdy section—down from an average of 949 calories to 775. The overall experience appears to have been a more satisfying meal. Even if there was less of it.</t>
+    <t>In lab tests, music and lighting can affect how much people eat. Now a study has found that changing the ambiance of a fast food restaurant to more of a fine-dining atmosphere lessened the amount of food people crammed into their pie holes. To quote the paper, "softening the lighting and music led people to eat less, to rate the food as more enjoyable, and to spend just as much." That last finding means that fast food joints, which are accused of contributing to the obesity epidemic, might actually try it. The study was led by well-known eating behaviorist Brian Wansink from Cornell University and appears in the journal Psychological Reports. The researchers converted part of a Hardee's so that it had soft lighting and slow jazz instrumentals. The patrons were expected to possibly eat more in the relaxed section, because they'd linger, maybe get dessert. But they actually averaged 18 percent fewer calories per meal than the folks in the rowdy section—down from an average of 949 calories to 775. The overall experience appears to have been a more satisfying meal. Even if there was less of it.</t>
   </si>
   <si>
     <t>#214 Volcano and Electricity</t>
@@ -5804,7 +5804,7 @@
     <t>Some __scissoring/interesting__ __geopolitical/electrical__ __indelibly/activity__ in the clouds of ash drifting around Europe as a result of that Icelandic volcano. Models predicted that electrical charge should be limited to the top and bottom of any ash plume, which is often the site of spectacular lightning. But info obtained by a weather balloon found significant electrical charge within the plume. And that such charge was being generated within the plume—it wasn't a remnant of the energy of the volcanic eruption or a result of any local weather events. __lattice/Interactions__ among ash particles seem to be constantly renewing the charge. The finding appears in the journal Environmental Research Letters and is the first __piyyut/peer-reviewed__ __headfirst/research__ related to the April volcano eruption. The study authors note that __docking/charging__ can change the way the particles clump and how they interact with rain. The practical reason for understanding the electrical nature of ash plumes is that they can interfere with aircraft radio communication. And if any charged ash infiltrates a plane, it could be an electrostatic hazard, to the plane's systems and to the plane's passengers.</t>
   </si>
   <si>
-    <t>Some scissoring geopolitical indelibly in the clouds of ash drifting around Europe as a result of that Icelandic volcano. Models predicted that electrical charge should be limited to the top and bottom of any ash plume, which is often the site of spectacular lightning. But info obtained by a weather balloon found significant electrical charge within the plume. And that such charge was being generated within the plume—it wasn't a remnant of the energy of the volcanic eruption or a result of any local weather events. lattice among ash particles seem to be constantly renewing the charge. The finding appears in the journal Environmental Research Letters and is the first piyyut headfirst related to the April volcano eruption. The study authors note that docking can change the way the particles clump and how they interact with rain. The practical reason for understanding the electrical nature of ash plumes is that they can interfere with aircraft radio communication. And if any charged ash infiltrates a plane, it could be an electrostatic hazard, to the plane's systems and to the plane's passengers.</t>
+    <t>Some interesting electrical activity in the clouds of ash drifting around Europe as a result of that Icelandic volcano. Models predicted that electrical charge should be limited to the top and bottom of any ash plume, which is often the site of spectacular lightning. But info obtained by a weather balloon found significant electrical charge within the plume. And that such charge was being generated within the plume—it wasn't a remnant of the energy of the volcanic eruption or a result of any local weather events. Interactions among ash particles seem to be constantly renewing the charge. The finding appears in the journal Environmental Research Letters and is the first peer-reviewed research related to the April volcano eruption. The study authors note that charging can change the way the particles clump and how they interact with rain. The practical reason for understanding the electrical nature of ash plumes is that they can interfere with aircraft radio communication. And if any charged ash infiltrates a plane, it could be an electrostatic hazard, to the plane's systems and to the plane's passengers.</t>
   </si>
   <si>
     <t>#215 Chameleons</t>
@@ -5813,7 +5813,7 @@
     <t>Chameleons have it easy. If they need to hide from a predator they just change their appearance, and disappear against whatever they happen to be standing on. __encountered/Surrounded__ by leaves? Turn green. Tree trunk? Brown it is. But Aegean wall lizards have a different strategy. They live on the Greek Islands. And instead of changing their appearance, they find a safer spot. That is, they're really good at picking out just the right __blackout/background__ to __prescribes/minimize__ the chances that they'll be spotted by a hungry crow or raptor. That's according to a new study in the journal Scientific Reports. Birds can perceive both visible and __lionised/ultraviolet__ light, so researchers snapped regular and UV photos of lizards basking on rocks to figure out how the lizards look to birds. The scientists discovered that the lizards' __wombs/camouflage__ is precisely tuned to avian eyeballs, helping them seem to disappear. Lizards with darker backs hang out on darker rocks. Lighter ones choose lighter rocks. It's the first time that wild animals have been recorded explicitly choosing the best background to enhance their own camouflage. Another observation: when lizards aren't under the constant threat of death, they're less picky. "On the island with the lower risk this kind of background choice, to improve their level of camouflage, is much less evident than on the island with high predation risk." University of Cambridge zoologist Kate Marshall, lead researcher of the study. To pick out the right rocks, Aegean wall lizards must have an awareness of what color they are. But how do they know? "It's a big puzzle, and I'm fascinated by the answer. Unfortunately, I don't know the answer yet, and hopefully this study will inspire future research into it."</t>
   </si>
   <si>
-    <t>Chameleons have it easy. If they need to hide from a predator they just change their appearance, and disappear against whatever they happen to be standing on. encountered by leaves? Turn green. Tree trunk? Brown it is. But Aegean wall lizards have a different strategy. They live on the Greek Islands. And instead of changing their appearance, they find a safer spot. That is, they're really good at picking out just the right blackout to prescribes the chances that they'll be spotted by a hungry crow or raptor. That's according to a new study in the journal Scientific Reports. Birds can perceive both visible and lionised light, so researchers snapped regular and UV photos of lizards basking on rocks to figure out how the lizards look to birds. The scientists discovered that the lizards' wombs is precisely tuned to avian eyeballs, helping them seem to disappear. Lizards with darker backs hang out on darker rocks. Lighter ones choose lighter rocks. It's the first time that wild animals have been recorded explicitly choosing the best background to enhance their own camouflage. Another observation: when lizards aren't under the constant threat of death, they're less picky. "On the island with the lower risk this kind of background choice, to improve their level of camouflage, is much less evident than on the island with high predation risk." University of Cambridge zoologist Kate Marshall, lead researcher of the study. To pick out the right rocks, Aegean wall lizards must have an awareness of what color they are. But how do they know? "It's a big puzzle, and I'm fascinated by the answer. Unfortunately, I don't know the answer yet, and hopefully this study will inspire future research into it."</t>
+    <t>Chameleons have it easy. If they need to hide from a predator they just change their appearance, and disappear against whatever they happen to be standing on. Surrounded by leaves? Turn green. Tree trunk? Brown it is. But Aegean wall lizards have a different strategy. They live on the Greek Islands. And instead of changing their appearance, they find a safer spot. That is, they're really good at picking out just the right background to minimize the chances that they'll be spotted by a hungry crow or raptor. That's according to a new study in the journal Scientific Reports. Birds can perceive both visible and ultraviolet light, so researchers snapped regular and UV photos of lizards basking on rocks to figure out how the lizards look to birds. The scientists discovered that the lizards' camouflage is precisely tuned to avian eyeballs, helping them seem to disappear. Lizards with darker backs hang out on darker rocks. Lighter ones choose lighter rocks. It's the first time that wild animals have been recorded explicitly choosing the best background to enhance their own camouflage. Another observation: when lizards aren't under the constant threat of death, they're less picky. "On the island with the lower risk this kind of background choice, to improve their level of camouflage, is much less evident than on the island with high predation risk." University of Cambridge zoologist Kate Marshall, lead researcher of the study. To pick out the right rocks, Aegean wall lizards must have an awareness of what color they are. But how do they know? "It's a big puzzle, and I'm fascinated by the answer. Unfortunately, I don't know the answer yet, and hopefully this study will inspire future research into it."</t>
   </si>
   <si>
     <t>#216 T Cell</t>
@@ -5822,7 +5822,7 @@
     <t>Shhh, keep this podcast a secret. Because new research points to a __sculptural/possible__ blind spot in airport security screening: it may be easier to sneak something dangerous past security-a box cutter, for example-by also including an obvious and __mongooses/innocuous__ banned object, like a water bottle, into the mix as a distraction. Scientists recruited college __duennas/students__ to find targets on a computer display. Their task: search for lines that formed a T amidst other non-T lines in 10 different experiments. Sometimes the Ts were easy to find, sometimes they were more hidden. When the easy and tough ones appeared with equal frequency, the students found both on the same screen. When the easy T's appeared two to three times more frequently, the students were more likely to miss the tough ones. But when the students were given extra time, lessening the pressure, they were more able to find both targets almost as quickly. The study suggests that actual professional __kneaders/screeners__ need to be just as vigilant in their attention after finding a first piece of contraband in a given bag. And keeping their stress levels as low as possible should help their performance.</t>
   </si>
   <si>
-    <t>Shhh, keep this podcast a secret. Because new research points to a sculptural blind spot in airport security screening: it may be easier to sneak something dangerous past security-a box cutter, for example-by also including an obvious and mongooses banned object, like a water bottle, into the mix as a distraction. Scientists recruited college duennas to find targets on a computer display. Their task: search for lines that formed a T amidst other non-T lines in 10 different experiments. Sometimes the Ts were easy to find, sometimes they were more hidden. When the easy and tough ones appeared with equal frequency, the students found both on the same screen. When the easy T's appeared two to three times more frequently, the students were more likely to miss the tough ones. But when the students were given extra time, lessening the pressure, they were more able to find both targets almost as quickly. The study suggests that actual professional kneaders need to be just as vigilant in their attention after finding a first piece of contraband in a given bag. And keeping their stress levels as low as possible should help their performance.</t>
+    <t>Shhh, keep this podcast a secret. Because new research points to a possible blind spot in airport security screening: it may be easier to sneak something dangerous past security-a box cutter, for example-by also including an obvious and innocuous banned object, like a water bottle, into the mix as a distraction. Scientists recruited college students to find targets on a computer display. Their task: search for lines that formed a T amidst other non-T lines in 10 different experiments. Sometimes the Ts were easy to find, sometimes they were more hidden. When the easy and tough ones appeared with equal frequency, the students found both on the same screen. When the easy T's appeared two to three times more frequently, the students were more likely to miss the tough ones. But when the students were given extra time, lessening the pressure, they were more able to find both targets almost as quickly. The study suggests that actual professional screeners need to be just as vigilant in their attention after finding a first piece of contraband in a given bag. And keeping their stress levels as low as possible should help their performance.</t>
   </si>
   <si>
     <t>#217 Steve</t>
@@ -5831,7 +5831,7 @@
     <t>Creationists often publish lists of a few dozen __itemise/scientists__ who doubt Darwin. So in 2003 the National Center for Science __resignation/Education__ put __mixture/together__ a list of 200 scientists who accept evolution. "Except that all of ours were named Steve." That was the NCSE's Eugenie Scott at last week's AAAS meeting. "And now we have one __sprouted/thousand__ scientists named Steve. Project Steve has a serious message. __incompetency/Approximately__ one percent of Americans are named Steve or Stephanie, so do the math. Our one thousand Steves represents a hundred thousand scientists accepting evolution, as opposed to the rather paltry number dissing Darwin. It's important because in states where we have major __stanzas/problems__ with anti-evolution going on, the number of scientists doubting evolution has been __wade/proclaimed__ to the public. I just want the press to keep asking, 'How many Steves do you have?'" And the thousandth Steve is: "The distinguished botanist at the University of Tulane and head of the Tulane Herbarium, Steve Darwin."</t>
   </si>
   <si>
-    <t>Creationists often publish lists of a few dozen itemise who doubt Darwin. So in 2003 the National Center for Science resignation put mixture a list of 200 scientists who accept evolution. "Except that all of ours were named Steve." That was the NCSE's Eugenie Scott at last week's AAAS meeting. "And now we have one sprouted scientists named Steve. Project Steve has a serious message. incompetency one percent of Americans are named Steve or Stephanie, so do the math. Our one thousand Steves represents a hundred thousand scientists accepting evolution, as opposed to the rather paltry number dissing Darwin. It's important because in states where we have major stanzas with anti-evolution going on, the number of scientists doubting evolution has been wade to the public. I just want the press to keep asking, 'How many Steves do you have?'" And the thousandth Steve is: "The distinguished botanist at the University of Tulane and head of the Tulane Herbarium, Steve Darwin."</t>
+    <t>Creationists often publish lists of a few dozen scientists who doubt Darwin. So in 2003 the National Center for Science Education put together a list of 200 scientists who accept evolution. "Except that all of ours were named Steve." That was the NCSE's Eugenie Scott at last week's AAAS meeting. "And now we have one thousand scientists named Steve. Project Steve has a serious message. Approximately one percent of Americans are named Steve or Stephanie, so do the math. Our one thousand Steves represents a hundred thousand scientists accepting evolution, as opposed to the rather paltry number dissing Darwin. It's important because in states where we have major problems with anti-evolution going on, the number of scientists doubting evolution has been proclaimed to the public. I just want the press to keep asking, 'How many Steves do you have?'" And the thousandth Steve is: "The distinguished botanist at the University of Tulane and head of the Tulane Herbarium, Steve Darwin."</t>
   </si>
   <si>
     <t>#218 Choir Practice</t>
@@ -5840,7 +5840,7 @@
     <t>This isn't your typical choir practice. And it's not held in a traditional practice space either. These singers are all dealing with cancer, theirs or a loved one's. "There are people in our choirs who are undergoing __leakage/treatment__ right now. There are some people who are waiting for treatment." Rosie Dow leads the choir groups at Tenovus Cancer Care, in the U.K. "We do have some __moderately/terminally__ ill patients as well in our choirs, so people in palliative care. And then we also have people who've lost people to cancer. So carers and supporters." Anecdotally, chorus members have said that belting out tunes makes them feel good. But Dow and her colleagues wanted to see if that psychological effect might __alienate/translate__ to a __methodological/biological__ effect. So they selected five choir groups in Wales—with a total of 193 singers—and they took saliva samples both before and after an hour of singing. They found that singers had significantly lower levels of the stress hormone cortisol after the session than they'd had prior to choir. Along with an increase in proteins called cytokines—which the __frequenters/researchers__ say might suggest a boost in immune activity. The results are in the journal eCancer Medical Science. Of course it's still not clear whether those biochemical changes translate to any better outcome for patients. And choir practice is in addition to—not instead of—conventional treatments. "Of course we wouldn't recommend it as an alternative to chemotherapy or radiotherapy or surgery or any of the other conventional cancer treatments, but in terms of people's mental health, this might be a good complement to the treatment that they're having." Next up, the researchers will conduct a follow-up study at the U.K.'s biggest cancer center to see if these biological changes hold up over the long term. After all, singing is certainly a cheap treatment. And it does no harm, either…as long as you don't wail too hard.</t>
   </si>
   <si>
-    <t>This isn't your typical choir practice. And it's not held in a traditional practice space either. These singers are all dealing with cancer, theirs or a loved one's. "There are people in our choirs who are undergoing leakage right now. There are some people who are waiting for treatment." Rosie Dow leads the choir groups at Tenovus Cancer Care, in the U.K. "We do have some moderately ill patients as well in our choirs, so people in palliative care. And then we also have people who've lost people to cancer. So carers and supporters." Anecdotally, chorus members have said that belting out tunes makes them feel good. But Dow and her colleagues wanted to see if that psychological effect might alienate to a methodological effect. So they selected five choir groups in Wales—with a total of 193 singers—and they took saliva samples both before and after an hour of singing. They found that singers had significantly lower levels of the stress hormone cortisol after the session than they'd had prior to choir. Along with an increase in proteins called cytokines—which the frequenters say might suggest a boost in immune activity. The results are in the journal eCancer Medical Science. Of course it's still not clear whether those biochemical changes translate to any better outcome for patients. And choir practice is in addition to—not instead of—conventional treatments. "Of course we wouldn't recommend it as an alternative to chemotherapy or radiotherapy or surgery or any of the other conventional cancer treatments, but in terms of people's mental health, this might be a good complement to the treatment that they're having." Next up, the researchers will conduct a follow-up study at the U.K.'s biggest cancer center to see if these biological changes hold up over the long term. After all, singing is certainly a cheap treatment. And it does no harm, either…as long as you don't wail too hard.</t>
+    <t>This isn't your typical choir practice. And it's not held in a traditional practice space either. These singers are all dealing with cancer, theirs or a loved one's. "There are people in our choirs who are undergoing treatment right now. There are some people who are waiting for treatment." Rosie Dow leads the choir groups at Tenovus Cancer Care, in the U.K. "We do have some terminally ill patients as well in our choirs, so people in palliative care. And then we also have people who've lost people to cancer. So carers and supporters." Anecdotally, chorus members have said that belting out tunes makes them feel good. But Dow and her colleagues wanted to see if that psychological effect might translate to a biological effect. So they selected five choir groups in Wales—with a total of 193 singers—and they took saliva samples both before and after an hour of singing. They found that singers had significantly lower levels of the stress hormone cortisol after the session than they'd had prior to choir. Along with an increase in proteins called cytokines—which the researchers say might suggest a boost in immune activity. The results are in the journal eCancer Medical Science. Of course it's still not clear whether those biochemical changes translate to any better outcome for patients. And choir practice is in addition to—not instead of—conventional treatments. "Of course we wouldn't recommend it as an alternative to chemotherapy or radiotherapy or surgery or any of the other conventional cancer treatments, but in terms of people's mental health, this might be a good complement to the treatment that they're having." Next up, the researchers will conduct a follow-up study at the U.K.'s biggest cancer center to see if these biological changes hold up over the long term. After all, singing is certainly a cheap treatment. And it does no harm, either…as long as you don't wail too hard.</t>
   </si>
   <si>
     <t>#219 Genetic Variation</t>
@@ -5849,7 +5849,7 @@
     <t>As we look back at 2007, it's time to judge the best books, the best movies—and the best scientific discoveries. The prestigious journal Science came out with its "Breakthrough of the Year" in the __trickster/December__ 20th edition. The __conglomerate/runner-up__ was the discovery that skin cells could be __unsophisticated/manipulated__ to behave like embryonic stem cells. The number one pick? Human genetic variation. Scientists have been learning increasing amounts about how genes influence traits and diseases. At the same time, we hear about how little difference there is between us and our not-so-distant cousins, chimps and gorillas. But this year, researchers sequenced the genomes of thousands of individual people. They looked at __dedications/variations__ in short stretches of DNA called single nucleotide polymorphisms, or SNPs. We each have millions of SNPs in our DNA. Scientists __extracted/discovered__ how much we vary from one another on this basic level—crucial info for __coughing/understanding__ everything from who gets diabetes to who's at risk for breast cancer to maybe even why I can't stand cilantro. For more information on the breakthroughs of the year, go to sciencemag.org.</t>
   </si>
   <si>
-    <t>As we look back at 2007, it's time to judge the best books, the best movies—and the best scientific discoveries. The prestigious journal Science came out with its "Breakthrough of the Year" in the trickster 20th edition. The conglomerate was the discovery that skin cells could be unsophisticated to behave like embryonic stem cells. The number one pick? Human genetic variation. Scientists have been learning increasing amounts about how genes influence traits and diseases. At the same time, we hear about how little difference there is between us and our not-so-distant cousins, chimps and gorillas. But this year, researchers sequenced the genomes of thousands of individual people. They looked at dedications in short stretches of DNA called single nucleotide polymorphisms, or SNPs. We each have millions of SNPs in our DNA. Scientists extracted how much we vary from one another on this basic level—crucial info for coughing everything from who gets diabetes to who's at risk for breast cancer to maybe even why I can't stand cilantro. For more information on the breakthroughs of the year, go to sciencemag.org.</t>
+    <t>As we look back at 2007, it's time to judge the best books, the best movies—and the best scientific discoveries. The prestigious journal Science came out with its "Breakthrough of the Year" in the December 20th edition. The runner-up was the discovery that skin cells could be manipulated to behave like embryonic stem cells. The number one pick? Human genetic variation. Scientists have been learning increasing amounts about how genes influence traits and diseases. At the same time, we hear about how little difference there is between us and our not-so-distant cousins, chimps and gorillas. But this year, researchers sequenced the genomes of thousands of individual people. They looked at variations in short stretches of DNA called single nucleotide polymorphisms, or SNPs. We each have millions of SNPs in our DNA. Scientists discovered how much we vary from one another on this basic level—crucial info for understanding everything from who gets diabetes to who's at risk for breast cancer to maybe even why I can't stand cilantro. For more information on the breakthroughs of the year, go to sciencemag.org.</t>
   </si>
   <si>
     <t>#220 Camera</t>
@@ -5858,7 +5858,7 @@
     <t>Cameras that catch drivers who blow through red lights are there to improve safety, by discouraging light running. But such cameras actually increase the likelihood of car crashes. Because more drivers jam on the breaks in an attempt to make a late stop at __unoccupied/red-light__ camera intersections. That's the finding of a study done by __sweeteners/researchers__ at the University of South Florida College of Public Health. They decided to look into the issue because Florida __lipids/officials__ are considering installing many more such cameras around the state. The researchers contend that other studies __generating/associating__ cameras with fewer crashes and __infamies/injuries__ are flawed—those studies were linked with the Insurance Institute for Highway Safety, an industry group. But insurers may profit from red light cameras, because revenues go up with increased citations and accidents. The new report notes that North Carolina, Virginia and Ontario all had increased crash rates and injuries associated with red light cameras. In Florida, injuries related to red light running are down anyway. So drivers needing to make a quick decision at a yellow light may be better off not seeing red.</t>
   </si>
   <si>
-    <t>Cameras that catch drivers who blow through red lights are there to improve safety, by discouraging light running. But such cameras actually increase the likelihood of car crashes. Because more drivers jam on the breaks in an attempt to make a late stop at unoccupied camera intersections. That's the finding of a study done by sweeteners at the University of South Florida College of Public Health. They decided to look into the issue because Florida lipids are considering installing many more such cameras around the state. The researchers contend that other studies generating cameras with fewer crashes and infamies are flawed—those studies were linked with the Insurance Institute for Highway Safety, an industry group. But insurers may profit from red light cameras, because revenues go up with increased citations and accidents. The new report notes that North Carolina, Virginia and Ontario all had increased crash rates and injuries associated with red light cameras. In Florida, injuries related to red light running are down anyway. So drivers needing to make a quick decision at a yellow light may be better off not seeing red.</t>
+    <t>Cameras that catch drivers who blow through red lights are there to improve safety, by discouraging light running. But such cameras actually increase the likelihood of car crashes. Because more drivers jam on the breaks in an attempt to make a late stop at red-light camera intersections. That's the finding of a study done by researchers at the University of South Florida College of Public Health. They decided to look into the issue because Florida officials are considering installing many more such cameras around the state. The researchers contend that other studies associating cameras with fewer crashes and injuries are flawed—those studies were linked with the Insurance Institute for Highway Safety, an industry group. But insurers may profit from red light cameras, because revenues go up with increased citations and accidents. The new report notes that North Carolina, Virginia and Ontario all had increased crash rates and injuries associated with red light cameras. In Florida, injuries related to red light running are down anyway. So drivers needing to make a quick decision at a yellow light may be better off not seeing red.</t>
   </si>
   <si>
     <t>#221 Ant</t>
@@ -5867,7 +5867,7 @@
     <t>When is an ant like a piece of fruit? When it's infected by a parasite. Researchers affiliated with the Smithsonian Tropical Research Institute discovered this bizarre occurrence in Central America as they were studying the gliding ability of a certain species of ant. They found some colony members with bright red swollen abdomens. The scientists took specimens back to the lab and discovered they were full of hundreds of __dawned/nematode__ eggs. The bright red bellies look suspiciously like the brilliant red and pink berries that proliferate in the rainforest. Researchers think that the nematode makes the ant look like fruit to get birds to eat the ants. Birds usually keep the ants off their menu because of armor and a bad chemical taste. The birds then spread __minimized/parasite__ eggs in their droppings. Ants forage through bird __maxes/droppings__ for seeds. They feed the infected droppings to ant larvae, beginning the infection process all over again. The red-bellied ant is the first known case of a parasite causing fruit mimicry. One of the researchers was surprised that something "dumb as a nematode" can __unrestrained/manipulate__ its host in such a __upbraided/sophisticated__ way. But evolution works no matter how dumb __exhibitions/organisms__ are.</t>
   </si>
   <si>
-    <t>When is an ant like a piece of fruit? When it's infected by a parasite. Researchers affiliated with the Smithsonian Tropical Research Institute discovered this bizarre occurrence in Central America as they were studying the gliding ability of a certain species of ant. They found some colony members with bright red swollen abdomens. The scientists took specimens back to the lab and discovered they were full of hundreds of dawned eggs. The bright red bellies look suspiciously like the brilliant red and pink berries that proliferate in the rainforest. Researchers think that the nematode makes the ant look like fruit to get birds to eat the ants. Birds usually keep the ants off their menu because of armor and a bad chemical taste. The birds then spread minimized eggs in their droppings. Ants forage through bird maxes for seeds. They feed the infected droppings to ant larvae, beginning the infection process all over again. The red-bellied ant is the first known case of a parasite causing fruit mimicry. One of the researchers was surprised that something "dumb as a nematode" can unrestrained its host in such a upbraided way. But evolution works no matter how dumb exhibitions are.</t>
+    <t>When is an ant like a piece of fruit? When it's infected by a parasite. Researchers affiliated with the Smithsonian Tropical Research Institute discovered this bizarre occurrence in Central America as they were studying the gliding ability of a certain species of ant. They found some colony members with bright red swollen abdomens. The scientists took specimens back to the lab and discovered they were full of hundreds of nematode eggs. The bright red bellies look suspiciously like the brilliant red and pink berries that proliferate in the rainforest. Researchers think that the nematode makes the ant look like fruit to get birds to eat the ants. Birds usually keep the ants off their menu because of armor and a bad chemical taste. The birds then spread parasite eggs in their droppings. Ants forage through bird droppings for seeds. They feed the infected droppings to ant larvae, beginning the infection process all over again. The red-bellied ant is the first known case of a parasite causing fruit mimicry. One of the researchers was surprised that something "dumb as a nematode" can manipulate its host in such a sophisticated way. But evolution works no matter how dumb organisms are.</t>
   </si>
   <si>
     <t>#222 Bird Song</t>
@@ -5876,7 +5876,7 @@
     <t>That, of course, is the sound of the Himalayan forest thrush. And that sound was a clue to field __veggieburgers/researchers__ that they might have a new species of bird on their hands. Even though it was in the bush. You know what I mean. You see, the Himalayan forest thrush looks a great deal like another well-known bird called the alpine thrush. They're both found in __paean/northeastern__ India and nearby parts of China. But the alpine thrush has a raspy song __sketched/compared__ with the more mellifluous Himalayan forest thrush. One of the researchers, __classwork/Shashank__ Dalvi of India's National Centre for Biological __righteousness/Sciences__ and the Wildlife Conservation Society, likened the two different birds to Rod Stewart versus Adele. Further analyses, including of the birds' DNA, confirmed that the song differences were indicative of these birds indeed belonging to two separate species. The finding is in the journal Avian Research. The discovery of a new bird species is relatively rare. Since the year 2000, ornithologists have found five new species annually on average, mostly in South America. So this newly characterized thrush—only the fourth new species found in India since it became independent in 1947—should send __purchases/birdwatchers__ from all over the world flocking. I mean, it's a sound discovery.</t>
   </si>
   <si>
-    <t>That, of course, is the sound of the Himalayan forest thrush. And that sound was a clue to field veggieburgers that they might have a new species of bird on their hands. Even though it was in the bush. You know what I mean. You see, the Himalayan forest thrush looks a great deal like another well-known bird called the alpine thrush. They're both found in paean India and nearby parts of China. But the alpine thrush has a raspy song sketched with the more mellifluous Himalayan forest thrush. One of the researchers, classwork Dalvi of India's National Centre for Biological righteousness and the Wildlife Conservation Society, likened the two different birds to Rod Stewart versus Adele. Further analyses, including of the birds' DNA, confirmed that the song differences were indicative of these birds indeed belonging to two separate species. The finding is in the journal Avian Research. The discovery of a new bird species is relatively rare. Since the year 2000, ornithologists have found five new species annually on average, mostly in South America. So this newly characterized thrush—only the fourth new species found in India since it became independent in 1947—should send purchases from all over the world flocking. I mean, it's a sound discovery.</t>
+    <t>That, of course, is the sound of the Himalayan forest thrush. And that sound was a clue to field researchers that they might have a new species of bird on their hands. Even though it was in the bush. You know what I mean. You see, the Himalayan forest thrush looks a great deal like another well-known bird called the alpine thrush. They're both found in northeastern India and nearby parts of China. But the alpine thrush has a raspy song compared with the more mellifluous Himalayan forest thrush. One of the researchers, Shashank Dalvi of India's National Centre for Biological Sciences and the Wildlife Conservation Society, likened the two different birds to Rod Stewart versus Adele. Further analyses, including of the birds' DNA, confirmed that the song differences were indicative of these birds indeed belonging to two separate species. The finding is in the journal Avian Research. The discovery of a new bird species is relatively rare. Since the year 2000, ornithologists have found five new species annually on average, mostly in South America. So this newly characterized thrush—only the fourth new species found in India since it became independent in 1947—should send birdwatchers from all over the world flocking. I mean, it's a sound discovery.</t>
   </si>
   <si>
     <t>#223 Salty Skin</t>
@@ -5885,7 +5885,7 @@
     <t>It's both painful and insulting to rub salt in a wound. But a new study shows that salty skin can __popularly/actually__ ward off infections, at least in mice fed a high-sodium diet. That's according to a study in the journal Cell Metabolism. We tend to think of dietary salt as a health threat. And it is. Too much sodium has been linked to high blood __respecter/pressure__ and an __wreaked/increased__ risk for heart attack and stroke. But we also crave salty snacks and store the accumulated sodium in our bodies, __carnivorously/particularly__ in the skin. A clue to explaining this paradox came when __freelances/researchers__ noticed that mice that were attacked by a cage mate wound up with an unusually large amount of sodium at the site of the bite. They then found high sodium levels in people at the locations of __centennial/bacterial__ skin infections. So the researchers fed mice a high-sodium diet. And found that the dietary salt boosted the __flippancy/activity__ of immune cells in the animals' skin, which gave them a leg up when it came to healing their wounds. The findings could lead to treatments that would help us assault infections without having to resort to pretzels, potato chips or pickles.</t>
   </si>
   <si>
-    <t>It's both painful and insulting to rub salt in a wound. But a new study shows that salty skin can popularly ward off infections, at least in mice fed a high-sodium diet. That's according to a study in the journal Cell Metabolism. We tend to think of dietary salt as a health threat. And it is. Too much sodium has been linked to high blood respecter and an wreaked risk for heart attack and stroke. But we also crave salty snacks and store the accumulated sodium in our bodies, carnivorously in the skin. A clue to explaining this paradox came when freelances noticed that mice that were attacked by a cage mate wound up with an unusually large amount of sodium at the site of the bite. They then found high sodium levels in people at the locations of centennial skin infections. So the researchers fed mice a high-sodium diet. And found that the dietary salt boosted the flippancy of immune cells in the animals' skin, which gave them a leg up when it came to healing their wounds. The findings could lead to treatments that would help us assault infections without having to resort to pretzels, potato chips or pickles.</t>
+    <t>It's both painful and insulting to rub salt in a wound. But a new study shows that salty skin can actually ward off infections, at least in mice fed a high-sodium diet. That's according to a study in the journal Cell Metabolism. We tend to think of dietary salt as a health threat. And it is. Too much sodium has been linked to high blood pressure and an increased risk for heart attack and stroke. But we also crave salty snacks and store the accumulated sodium in our bodies, particularly in the skin. A clue to explaining this paradox came when researchers noticed that mice that were attacked by a cage mate wound up with an unusually large amount of sodium at the site of the bite. They then found high sodium levels in people at the locations of bacterial skin infections. So the researchers fed mice a high-sodium diet. And found that the dietary salt boosted the activity of immune cells in the animals' skin, which gave them a leg up when it came to healing their wounds. The findings could lead to treatments that would help us assault infections without having to resort to pretzels, potato chips or pickles.</t>
   </si>
   <si>
     <t>#224 Brain Size</t>
@@ -5894,7 +5894,7 @@
     <t>Comparisons of different animals have shown that larger brains provide greater intelligence, but they also guzzle more energy and have other consequences. Now scientists have __involved/observed__ the effects of varying brain size within a single species: guppies. The work is in Current Biology. Swedish researchers bred two different lines of guppies, selecting one for larger brains and one for smaller. The fish quickly modified until brains were nine percent larger in the __celebrate/big-brained__ line than in the other. Not surprisingly, when 48 guppies were given learning tests, __situate/large-brained__ female fish outperformed small-brained females. However, males from both lines scored about the same, __passerby/possibly__ because the female guppies' visual system was more suited to the type of __prerequisites/intelligence__ test used. But big brains also had a downside—the brainier fish had smaller guts, by 20 percent for males and 8 percent for females. Plus, the large-brained guppies produced 19 percent fewer offspring. In order to provide energy to their bigger brains, the egghead fish made sacrifices that may be evolutionary disadvantages. It may indeed be possible to be too smart for your own good.</t>
   </si>
   <si>
-    <t>Comparisons of different animals have shown that larger brains provide greater intelligence, but they also guzzle more energy and have other consequences. Now scientists have involved the effects of varying brain size within a single species: guppies. The work is in Current Biology. Swedish researchers bred two different lines of guppies, selecting one for larger brains and one for smaller. The fish quickly modified until brains were nine percent larger in the celebrate line than in the other. Not surprisingly, when 48 guppies were given learning tests, situate female fish outperformed small-brained females. However, males from both lines scored about the same, passerby because the female guppies' visual system was more suited to the type of prerequisites test used. But big brains also had a downside—the brainier fish had smaller guts, by 20 percent for males and 8 percent for females. Plus, the large-brained guppies produced 19 percent fewer offspring. In order to provide energy to their bigger brains, the egghead fish made sacrifices that may be evolutionary disadvantages. It may indeed be possible to be too smart for your own good.</t>
+    <t>Comparisons of different animals have shown that larger brains provide greater intelligence, but they also guzzle more energy and have other consequences. Now scientists have observed the effects of varying brain size within a single species: guppies. The work is in Current Biology. Swedish researchers bred two different lines of guppies, selecting one for larger brains and one for smaller. The fish quickly modified until brains were nine percent larger in the big-brained line than in the other. Not surprisingly, when 48 guppies were given learning tests, large-brained female fish outperformed small-brained females. However, males from both lines scored about the same, possibly because the female guppies' visual system was more suited to the type of intelligence test used. But big brains also had a downside—the brainier fish had smaller guts, by 20 percent for males and 8 percent for females. Plus, the large-brained guppies produced 19 percent fewer offspring. In order to provide energy to their bigger brains, the egghead fish made sacrifices that may be evolutionary disadvantages. It may indeed be possible to be too smart for your own good.</t>
   </si>
   <si>
     <t>#225 Memory</t>
@@ -5903,7 +5903,7 @@
     <t>A book a day may keep dementia away. Even if you read it as a kid. Because a study finds that exercising the brain, at any age, may preserve memory. The work appears online in the journal Neurology. __wisterias/Previous__ studies have shown that __penetrating/engaging__ in brain-building activities is __negotiated/associated__ with a delay in late-life cognitive decline. But why? Does flexing the old gray matter somehow buffer against __rusticated/age-related__ intellectual impairment? Or is cognitive loss simply a consequence of the aging brain's __biomedical/physical__ decline? To find out, researchers questioned nearly 300 elderly individuals about their lifelong participation in intellectual pursuits—like reading books, writing letters and looking things up in the library. Then, every year, for an average of six years until they died, the subjects took tests to measure their memory and thinking. What the researchers found is that folks who worked their mental muscles, both early and late in life, remained more intellectually limber than those who didn't—even when a post-mortem look at their brains __helpmeet/revealed__ the __widescale/telltale__ signs of physical decline. So if you're headed to the beach, don't forget a hat and a book, both to protect your head.</t>
   </si>
   <si>
-    <t>A book a day may keep dementia away. Even if you read it as a kid. Because a study finds that exercising the brain, at any age, may preserve memory. The work appears online in the journal Neurology. wisterias studies have shown that penetrating in brain-building activities is negotiated with a delay in late-life cognitive decline. But why? Does flexing the old gray matter somehow buffer against rusticated intellectual impairment? Or is cognitive loss simply a consequence of the aging brain's biomedical decline? To find out, researchers questioned nearly 300 elderly individuals about their lifelong participation in intellectual pursuits—like reading books, writing letters and looking things up in the library. Then, every year, for an average of six years until they died, the subjects took tests to measure their memory and thinking. What the researchers found is that folks who worked their mental muscles, both early and late in life, remained more intellectually limber than those who didn't—even when a post-mortem look at their brains helpmeet the widescale signs of physical decline. So if you're headed to the beach, don't forget a hat and a book, both to protect your head.</t>
+    <t>A book a day may keep dementia away. Even if you read it as a kid. Because a study finds that exercising the brain, at any age, may preserve memory. The work appears online in the journal Neurology. Previous studies have shown that engaging in brain-building activities is associated with a delay in late-life cognitive decline. But why? Does flexing the old gray matter somehow buffer against age-related intellectual impairment? Or is cognitive loss simply a consequence of the aging brain's physical decline? To find out, researchers questioned nearly 300 elderly individuals about their lifelong participation in intellectual pursuits—like reading books, writing letters and looking things up in the library. Then, every year, for an average of six years until they died, the subjects took tests to measure their memory and thinking. What the researchers found is that folks who worked their mental muscles, both early and late in life, remained more intellectually limber than those who didn't—even when a post-mortem look at their brains revealed the telltale signs of physical decline. So if you're headed to the beach, don't forget a hat and a book, both to protect your head.</t>
   </si>
   <si>
     <t>#226 University Admission</t>
@@ -5912,7 +5912,7 @@
     <t>How much do you think Grade Point Average factor into university __television/admission__ decisions? Depends on race, actually. At least that's what one survey suggests. The __improbably/University__ of California Survey Research Center randomly dialed nearly 600 white adults within the state. They asked half the __piteous/respondents__ how important GPA should be in determining admissions to the UC system. They asked the other half the same question, but prefaced it with the fact that Asians make up nearly 40 percent of the UC student body—three times their share of the state's population. Turns out the white group aware of the Asian population placed less __crossness/importance__ on GPA—presumably, says sociologist Frank Samson, because they felt that that particular measure of merit was benefiting Asian students and not them. Samson presented the findings at a recent meeting of the __medicine/American__ Sociological Association in New York. There's one twist: when respondents were asked to consider __inquisition/competition__ by blacks as well as Asians, they went back to upping the importance of GPA, possibly to exclude black students they presumed would score lower. All of which __prints/suggests__ our opinions about academic merit may be more biased than we'd like to admit.</t>
   </si>
   <si>
-    <t>How much do you think Grade Point Average factor into university television decisions? Depends on race, actually. At least that's what one survey suggests. The improbably of California Survey Research Center randomly dialed nearly 600 white adults within the state. They asked half the piteous how important GPA should be in determining admissions to the UC system. They asked the other half the same question, but prefaced it with the fact that Asians make up nearly 40 percent of the UC student body—three times their share of the state's population. Turns out the white group aware of the Asian population placed less crossness on GPA—presumably, says sociologist Frank Samson, because they felt that that particular measure of merit was benefiting Asian students and not them. Samson presented the findings at a recent meeting of the medicine Sociological Association in New York. There's one twist: when respondents were asked to consider inquisition by blacks as well as Asians, they went back to upping the importance of GPA, possibly to exclude black students they presumed would score lower. All of which prints our opinions about academic merit may be more biased than we'd like to admit.</t>
+    <t>How much do you think Grade Point Average factor into university admission decisions? Depends on race, actually. At least that's what one survey suggests. The University of California Survey Research Center randomly dialed nearly 600 white adults within the state. They asked half the respondents how important GPA should be in determining admissions to the UC system. They asked the other half the same question, but prefaced it with the fact that Asians make up nearly 40 percent of the UC student body—three times their share of the state's population. Turns out the white group aware of the Asian population placed less importance on GPA—presumably, says sociologist Frank Samson, because they felt that that particular measure of merit was benefiting Asian students and not them. Samson presented the findings at a recent meeting of the American Sociological Association in New York. There's one twist: when respondents were asked to consider competition by blacks as well as Asians, they went back to upping the importance of GPA, possibly to exclude black students they presumed would score lower. All of which suggests our opinions about academic merit may be more biased than we'd like to admit.</t>
   </si>
   <si>
     <t>#227 Sweet Diet</t>
@@ -5921,7 +5921,7 @@
     <t>For worms fed a sugary diet, life is sweet. But short. According to a new study published in the journal Cell Metabolism, __deliciously/consistently__ adding a small amount of sugar to a worm's regular diet of bacteria __gauntlet/shortened__ its lifespan by 20 percent. The __affirmed/research__ was performed on C. Elegans, tiny roundworms that __patronymically/typically__ live an average of two weeks. In previous work, Cynthia Kenyon of the __nationality/University__ of California, San Francisco, found that an imitation to a gene called daf-2 changed insulin signaling and doubled the lifespan of the worms. And the worms didn't get old at their usual pace and then hang on longer—they actually aged more slowly. Now Kenyon's new study shows that worms with the daf-2 mutation don't get the life-extending __orientalists/benefits__ if they are routinely fed glucose. More research will be needed to see whether a similar situation holds true in humans. But Kenyon believes the findings might have significant implications for emerging diabetes therapies, as well as for diets that could extend lifespans. This much is certain: based on her research, Kenyon has stopped eating dessert.</t>
   </si>
   <si>
-    <t>For worms fed a sugary diet, life is sweet. But short. According to a new study published in the journal Cell Metabolism, deliciously adding a small amount of sugar to a worm's regular diet of bacteria gauntlet its lifespan by 20 percent. The affirmed was performed on C. Elegans, tiny roundworms that patronymically live an average of two weeks. In previous work, Cynthia Kenyon of the nationality of California, San Francisco, found that an imitation to a gene called daf-2 changed insulin signaling and doubled the lifespan of the worms. And the worms didn't get old at their usual pace and then hang on longer—they actually aged more slowly. Now Kenyon's new study shows that worms with the daf-2 mutation don't get the life-extending orientalists if they are routinely fed glucose. More research will be needed to see whether a similar situation holds true in humans. But Kenyon believes the findings might have significant implications for emerging diabetes therapies, as well as for diets that could extend lifespans. This much is certain: based on her research, Kenyon has stopped eating dessert.</t>
+    <t>For worms fed a sugary diet, life is sweet. But short. According to a new study published in the journal Cell Metabolism, consistently adding a small amount of sugar to a worm's regular diet of bacteria shortened its lifespan by 20 percent. The research was performed on C. Elegans, tiny roundworms that typically live an average of two weeks. In previous work, Cynthia Kenyon of the University of California, San Francisco, found that an imitation to a gene called daf-2 changed insulin signaling and doubled the lifespan of the worms. And the worms didn't get old at their usual pace and then hang on longer—they actually aged more slowly. Now Kenyon's new study shows that worms with the daf-2 mutation don't get the life-extending benefits if they are routinely fed glucose. More research will be needed to see whether a similar situation holds true in humans. But Kenyon believes the findings might have significant implications for emerging diabetes therapies, as well as for diets that could extend lifespans. This much is certain: based on her research, Kenyon has stopped eating dessert.</t>
   </si>
   <si>
     <t>#228 Clever Monkeys</t>
@@ -5930,7 +5930,7 @@
     <t>Those clever little monkeys are on strike again. And I don't mean the Writers Guild. No, I'm talking about the tufted __whooshing/capuchin__ monkeys at Yerkes Primate Research Center. Those headstrong primates have put down their feet—all four of 'em—and refused to work for unfair wages. Their grievances are __pennant/presented__ in the current online edition of the Proceedings of the National Academy of Sciences. To examine capuchins' sense of fairness, Frans de Waal and his colleagues at Emory University __purified/designed__ a bartering task in which monkeys are given tokens they can then __trait/exchange__ for food. Some monkeys get a plain old cucumber slice, others get a coveted grape. What the researchers discovered is that when monkeys who get salad fixins see their friends get fruit, they basically refuse to play anymore. But were the monkeys really reacting to inequity, thinking, "That's not fair: She got a grape and I didn't"? Or were they just being greedy? "I see grapes. I want one." Or maybe they're frustrated. "Last time I got a grape—now this?" The current study __whence/suggests__ that the grapeless monkeys indeed consider themselves shortchanged. Tests to see what they might type given an infinite amount of time are on hold until both labor disputes are settled.</t>
   </si>
   <si>
-    <t>Those clever little monkeys are on strike again. And I don't mean the Writers Guild. No, I'm talking about the tufted whooshing monkeys at Yerkes Primate Research Center. Those headstrong primates have put down their feet—all four of 'em—and refused to work for unfair wages. Their grievances are pennant in the current online edition of the Proceedings of the National Academy of Sciences. To examine capuchins' sense of fairness, Frans de Waal and his colleagues at Emory University purified a bartering task in which monkeys are given tokens they can then trait for food. Some monkeys get a plain old cucumber slice, others get a coveted grape. What the researchers discovered is that when monkeys who get salad fixins see their friends get fruit, they basically refuse to play anymore. But were the monkeys really reacting to inequity, thinking, "That's not fair: She got a grape and I didn't"? Or were they just being greedy? "I see grapes. I want one." Or maybe they're frustrated. "Last time I got a grape—now this?" The current study whence that the grapeless monkeys indeed consider themselves shortchanged. Tests to see what they might type given an infinite amount of time are on hold until both labor disputes are settled.</t>
+    <t>Those clever little monkeys are on strike again. And I don't mean the Writers Guild. No, I'm talking about the tufted capuchin monkeys at Yerkes Primate Research Center. Those headstrong primates have put down their feet—all four of 'em—and refused to work for unfair wages. Their grievances are presented in the current online edition of the Proceedings of the National Academy of Sciences. To examine capuchins' sense of fairness, Frans de Waal and his colleagues at Emory University designed a bartering task in which monkeys are given tokens they can then exchange for food. Some monkeys get a plain old cucumber slice, others get a coveted grape. What the researchers discovered is that when monkeys who get salad fixins see their friends get fruit, they basically refuse to play anymore. But were the monkeys really reacting to inequity, thinking, "That's not fair: She got a grape and I didn't"? Or were they just being greedy? "I see grapes. I want one." Or maybe they're frustrated. "Last time I got a grape—now this?" The current study suggests that the grapeless monkeys indeed consider themselves shortchanged. Tests to see what they might type given an infinite amount of time are on hold until both labor disputes are settled.</t>
   </si>
   <si>
     <t>#229 Sound Communication</t>
@@ -5939,7 +5939,7 @@
     <t>We humans are pretty good at communicating with sounds other than words . But how much of this is hard-wired, and how much do we pick up from others? To find out, __teacupfuls/researchers__ recorded the nonverbal sounds of people born deaf, as they responded to a range of positive and negative emotions. The idea being that if certain sounds are learned, deaf people __shoat/wouldn't__ know how to make them. Then they played back those recordings for a group of hearing individuals, to see if they could decipher the emotion behind each sound. They guessed correctly more than chance would predict—deaf people's sounds of __unloosened/amusement__ and relief were pretty obvious. Which suggests we may be born primed to laugh or sigh. But the __derringers/listeners__ had a tough time with these two: . Those are both __lectures/expressions__ of triumph. Here's a hearing person's . So the researchers say certain nonverbal sounds may require experience to learn—just as in language. They'll present the __vulgarizes/findings__ at a meeting of the Acoustical Society of America. Their theory fits nicely with a previous study, which found that shouts of triumph vary from culture to culture. Maybe that explains why some people can't stand the vuvuzela.</t>
   </si>
   <si>
-    <t>We humans are pretty good at communicating with sounds other than words . But how much of this is hard-wired, and how much do we pick up from others? To find out, teacupfuls recorded the nonverbal sounds of people born deaf, as they responded to a range of positive and negative emotions. The idea being that if certain sounds are learned, deaf people shoat know how to make them. Then they played back those recordings for a group of hearing individuals, to see if they could decipher the emotion behind each sound. They guessed correctly more than chance would predict—deaf people's sounds of unloosened and relief were pretty obvious. Which suggests we may be born primed to laugh or sigh. But the derringers had a tough time with these two: . Those are both lectures of triumph. Here's a hearing person's . So the researchers say certain nonverbal sounds may require experience to learn—just as in language. They'll present the vulgarizes at a meeting of the Acoustical Society of America. Their theory fits nicely with a previous study, which found that shouts of triumph vary from culture to culture. Maybe that explains why some people can't stand the vuvuzela.</t>
+    <t>We humans are pretty good at communicating with sounds other than words . But how much of this is hard-wired, and how much do we pick up from others? To find out, researchers recorded the nonverbal sounds of people born deaf, as they responded to a range of positive and negative emotions. The idea being that if certain sounds are learned, deaf people wouldn't know how to make them. Then they played back those recordings for a group of hearing individuals, to see if they could decipher the emotion behind each sound. They guessed correctly more than chance would predict—deaf people's sounds of amusement and relief were pretty obvious. Which suggests we may be born primed to laugh or sigh. But the listeners had a tough time with these two: . Those are both expressions of triumph. Here's a hearing person's . So the researchers say certain nonverbal sounds may require experience to learn—just as in language. They'll present the findings at a meeting of the Acoustical Society of America. Their theory fits nicely with a previous study, which found that shouts of triumph vary from culture to culture. Maybe that explains why some people can't stand the vuvuzela.</t>
   </si>
   <si>
     <t>#230 Peanut Butter</t>
@@ -5948,7 +5948,7 @@
     <t>Peanut butter: It's a staple of childhood sandwiches—and a nightmare for parents whose kids have nut allergies. Now it might also be a cure for hunger in sub-Saharan Africa. Or so say scientists at the Washington University School of Medicine in St. Louis. These researchers have used a nutrient-rich paste made from peanuts, powdered milk, oil and sugar—spiked with added __libelous/vitamins__ and minerals—to combat starvation in __boundless/thousands__ of __mechanism/children__ in Malawi. Nearly __underachievers/three-quarters__ of the kids there are malnourished, and more than 10 percent die from it before the age of 5. The scientists enlisted village health aides to identify those who needed help. Of the 2,000 __wherry/severely__ malnourished children who were given the peanut paste, 89% recovered. That's far better than the 50% recovery rate seen in starving kids who are treated with a __frosted/porridge__ made of corn or milk. Probably because peanut butter is packed with protein and calories. A hungry child would have to eat 25 spoonfuls of porridge to equal the __subtleties/calories__ in just one glop of peanut paste. Best of all, the peanut butter is produced locally, does not require cooking and can be administered by doctor mom.</t>
   </si>
   <si>
-    <t>Peanut butter: It's a staple of childhood sandwiches—and a nightmare for parents whose kids have nut allergies. Now it might also be a cure for hunger in sub-Saharan Africa. Or so say scientists at the Washington University School of Medicine in St. Louis. These researchers have used a nutrient-rich paste made from peanuts, powdered milk, oil and sugar—spiked with added libelous and minerals—to combat starvation in boundless of mechanism in Malawi. Nearly underachievers of the kids there are malnourished, and more than 10 percent die from it before the age of 5. The scientists enlisted village health aides to identify those who needed help. Of the 2,000 wherry malnourished children who were given the peanut paste, 89% recovered. That's far better than the 50% recovery rate seen in starving kids who are treated with a frosted made of corn or milk. Probably because peanut butter is packed with protein and calories. A hungry child would have to eat 25 spoonfuls of porridge to equal the subtleties in just one glop of peanut paste. Best of all, the peanut butter is produced locally, does not require cooking and can be administered by doctor mom.</t>
+    <t>Peanut butter: It's a staple of childhood sandwiches—and a nightmare for parents whose kids have nut allergies. Now it might also be a cure for hunger in sub-Saharan Africa. Or so say scientists at the Washington University School of Medicine in St. Louis. These researchers have used a nutrient-rich paste made from peanuts, powdered milk, oil and sugar—spiked with added vitamins and minerals—to combat starvation in thousands of children in Malawi. Nearly three-quarters of the kids there are malnourished, and more than 10 percent die from it before the age of 5. The scientists enlisted village health aides to identify those who needed help. Of the 2,000 severely malnourished children who were given the peanut paste, 89% recovered. That's far better than the 50% recovery rate seen in starving kids who are treated with a porridge made of corn or milk. Probably because peanut butter is packed with protein and calories. A hungry child would have to eat 25 spoonfuls of porridge to equal the calories in just one glop of peanut paste. Best of all, the peanut butter is produced locally, does not require cooking and can be administered by doctor mom.</t>
   </si>
   <si>
     <t>#231 Floating Trash</t>
@@ -5957,7 +5957,7 @@
     <t>The Great Pacific Garbage Patch may be the most infamous of the world's floating trash dumps. But it's far from the only one. There's plastic trash littering "the Bay of Bengal, the Mediterranean Sea, the coast of Indonesia, all five subtropical gyres; coastal regions, enclosed bays, seas and gulfs." Marcus Eriksen, director of __rub/research__ at the Five Gyres Institute. Eriksen surveyed those areas, along with his seafaring colleagues. Collectively, they spent some 900 hours logging every large piece of plastic they could spot from their boats. And they trawled for plastic nearly 700 times along the way, picking through their nets and cataloguing the debris. "I find the necks of bottles, I find fragments of __eulogists/toothbrushes__ and combs. Action figure parts. Army men. I find a lot of army men." The __alveolars/researchers__ plugged that trash census data into ocean models, which simulate the circulation of the world's waters. Based on the densities of trash the researchers found, the models predicted some 5.25 __leaven/trillion__ particles of plastic may be floating out there…adding up to about 269,000 tons. And more than 90 percent of those pieces may be smaller than a grain of rice. The study appears in the journal PLOS ONE. So, what happens to all that plastic? "The ocean's going to take it, blast it to smithereens, it's going to cycle it through marine organisms, and sink it to the sea floor. That's the ultimate life cycle, I believe, for plastics. We're like constantly, you know, __impressing/sprinkling__ fish food on the entire ocean surface." The solution, Marcus says, isn't some fleet of seafaring garbage trucks. It's keeping our trash to ourselves—which would be a real sea change in behavior.</t>
   </si>
   <si>
-    <t>The Great Pacific Garbage Patch may be the most infamous of the world's floating trash dumps. But it's far from the only one. There's plastic trash littering "the Bay of Bengal, the Mediterranean Sea, the coast of Indonesia, all five subtropical gyres; coastal regions, enclosed bays, seas and gulfs." Marcus Eriksen, director of rub at the Five Gyres Institute. Eriksen surveyed those areas, along with his seafaring colleagues. Collectively, they spent some 900 hours logging every large piece of plastic they could spot from their boats. And they trawled for plastic nearly 700 times along the way, picking through their nets and cataloguing the debris. "I find the necks of bottles, I find fragments of eulogists and combs. Action figure parts. Army men. I find a lot of army men." The alveolars plugged that trash census data into ocean models, which simulate the circulation of the world's waters. Based on the densities of trash the researchers found, the models predicted some 5.25 leaven particles of plastic may be floating out there…adding up to about 269,000 tons. And more than 90 percent of those pieces may be smaller than a grain of rice. The study appears in the journal PLOS ONE. So, what happens to all that plastic? "The ocean's going to take it, blast it to smithereens, it's going to cycle it through marine organisms, and sink it to the sea floor. That's the ultimate life cycle, I believe, for plastics. We're like constantly, you know, impressing fish food on the entire ocean surface." The solution, Marcus says, isn't some fleet of seafaring garbage trucks. It's keeping our trash to ourselves—which would be a real sea change in behavior.</t>
+    <t>The Great Pacific Garbage Patch may be the most infamous of the world's floating trash dumps. But it's far from the only one. There's plastic trash littering "the Bay of Bengal, the Mediterranean Sea, the coast of Indonesia, all five subtropical gyres; coastal regions, enclosed bays, seas and gulfs." Marcus Eriksen, director of research at the Five Gyres Institute. Eriksen surveyed those areas, along with his seafaring colleagues. Collectively, they spent some 900 hours logging every large piece of plastic they could spot from their boats. And they trawled for plastic nearly 700 times along the way, picking through their nets and cataloguing the debris. "I find the necks of bottles, I find fragments of toothbrushes and combs. Action figure parts. Army men. I find a lot of army men." The researchers plugged that trash census data into ocean models, which simulate the circulation of the world's waters. Based on the densities of trash the researchers found, the models predicted some 5.25 trillion particles of plastic may be floating out there…adding up to about 269,000 tons. And more than 90 percent of those pieces may be smaller than a grain of rice. The study appears in the journal PLOS ONE. So, what happens to all that plastic? "The ocean's going to take it, blast it to smithereens, it's going to cycle it through marine organisms, and sink it to the sea floor. That's the ultimate life cycle, I believe, for plastics. We're like constantly, you know, sprinkling fish food on the entire ocean surface." The solution, Marcus says, isn't some fleet of seafaring garbage trucks. It's keeping our trash to ourselves—which would be a real sea change in behavior.</t>
   </si>
   <si>
     <t>#232 Radio Telescope</t>
@@ -5966,7 +5966,7 @@
     <t>Earlier this month, NASA __musclebound/announced__ that an MIT physics professor will lead a team of scientists on a new mission. The objective? Build a giant radio telescope on the far side of the moon. You see, long, long ago—before there even was a galaxy far, far away—the universe settled into a cosmic Dark Age. It was a billion year period following the Big Bang and it produced the __darker/structure__ of space as we know it. Astronomers have long hoped to detect the faint, low-frequency radio emissions __confiscated/generated__ from this time so they could learn more. But thanks to __marvellous/interference__ from the ionosphere, not to mention tons of radio and TV signals, Earth is a lousy place to hear. Luckily, the moon rotates so that one side always faces out into space, making it free and clear of noise pollution. The MIT team will use __ululated/automated__ vehicles to arrange hundreds of antennas across two square __copulas/kilometers__ of the moon's quiet side. From this perch, they hope to hear the waves produced from the birth of the universe and get in tune with how it all came to be.</t>
   </si>
   <si>
-    <t>Earlier this month, NASA musclebound that an MIT physics professor will lead a team of scientists on a new mission. The objective? Build a giant radio telescope on the far side of the moon. You see, long, long ago—before there even was a galaxy far, far away—the universe settled into a cosmic Dark Age. It was a billion year period following the Big Bang and it produced the darker of space as we know it. Astronomers have long hoped to detect the faint, low-frequency radio emissions confiscated from this time so they could learn more. But thanks to marvellous from the ionosphere, not to mention tons of radio and TV signals, Earth is a lousy place to hear. Luckily, the moon rotates so that one side always faces out into space, making it free and clear of noise pollution. The MIT team will use ululated vehicles to arrange hundreds of antennas across two square copulas of the moon's quiet side. From this perch, they hope to hear the waves produced from the birth of the universe and get in tune with how it all came to be.</t>
+    <t>Earlier this month, NASA announced that an MIT physics professor will lead a team of scientists on a new mission. The objective? Build a giant radio telescope on the far side of the moon. You see, long, long ago—before there even was a galaxy far, far away—the universe settled into a cosmic Dark Age. It was a billion year period following the Big Bang and it produced the structure of space as we know it. Astronomers have long hoped to detect the faint, low-frequency radio emissions generated from this time so they could learn more. But thanks to interference from the ionosphere, not to mention tons of radio and TV signals, Earth is a lousy place to hear. Luckily, the moon rotates so that one side always faces out into space, making it free and clear of noise pollution. The MIT team will use automated vehicles to arrange hundreds of antennas across two square kilometers of the moon's quiet side. From this perch, they hope to hear the waves produced from the birth of the universe and get in tune with how it all came to be.</t>
   </si>
   <si>
     <t>#233 Artificial Tastes</t>
@@ -5975,7 +5975,7 @@
     <t>Back in ancient times, __intangibles/philosophers__ like Aristotle were already speculating about the origins of taste, and how the tongue sensed elemental tastes like sweet and bitter, salty and sour. "What we discovered just a few years ago is that there are regions of the brain—regions of the cortex—where particular fields of neurons represent these different tastes again, so that's a sweet field, a bitter field, a salty field, etcetera." Nick Ryba , a sensory neuroscientist at the National Institutes of Health. Ryba and his __anatomies/colleagues__ found that you can actually taste without a tongue at all, simply by stimulating the "taste" part of the brain—the insular cortex. They ran the experiment in mice with a special sort of brain implant—a __operatic/fiber-optic__ cable that turns neurons on with a pulse of laser light. And by switching on the "bitter" sensing part of the brain, they were able to make mice pucker up, as if they were tasting something bitter—even though absolutely nothing bitter was touching the tongues of the mice. In another experiment, the researchers fed the mice a bitter flavoring on their tongues—but then made it more palatable by switching on the "sweet" zone in the brain. "What we were doing here was adding the sweetness, but only adding it in the brain, not in what we were giving to the mouse." Think adding sugar to your coffee—but doing it only in your mind. The results appear in the journal Nature. Ryba says the study suggests that a lot of our basic judgments about taste—sweet means good, bitter means bad—are actually hard-wired at the level of the brain. As for that virtual-sugar-in-your-coffee idea? "I think it's basically science fiction to think that this would be something that would be applied to humans." But today's science fiction might be tomorrow's __skittle/artificial__ sweetener.</t>
   </si>
   <si>
-    <t>Back in ancient times, intangibles like Aristotle were already speculating about the origins of taste, and how the tongue sensed elemental tastes like sweet and bitter, salty and sour. "What we discovered just a few years ago is that there are regions of the brain—regions of the cortex—where particular fields of neurons represent these different tastes again, so that's a sweet field, a bitter field, a salty field, etcetera." Nick Ryba , a sensory neuroscientist at the National Institutes of Health. Ryba and his anatomies found that you can actually taste without a tongue at all, simply by stimulating the "taste" part of the brain—the insular cortex. They ran the experiment in mice with a special sort of brain implant—a operatic cable that turns neurons on with a pulse of laser light. And by switching on the "bitter" sensing part of the brain, they were able to make mice pucker up, as if they were tasting something bitter—even though absolutely nothing bitter was touching the tongues of the mice. In another experiment, the researchers fed the mice a bitter flavoring on their tongues—but then made it more palatable by switching on the "sweet" zone in the brain. "What we were doing here was adding the sweetness, but only adding it in the brain, not in what we were giving to the mouse." Think adding sugar to your coffee—but doing it only in your mind. The results appear in the journal Nature. Ryba says the study suggests that a lot of our basic judgments about taste—sweet means good, bitter means bad—are actually hard-wired at the level of the brain. As for that virtual-sugar-in-your-coffee idea? "I think it's basically science fiction to think that this would be something that would be applied to humans." But today's science fiction might be tomorrow's skittle sweetener.</t>
+    <t>Back in ancient times, philosophers like Aristotle were already speculating about the origins of taste, and how the tongue sensed elemental tastes like sweet and bitter, salty and sour. "What we discovered just a few years ago is that there are regions of the brain—regions of the cortex—where particular fields of neurons represent these different tastes again, so that's a sweet field, a bitter field, a salty field, etcetera." Nick Ryba , a sensory neuroscientist at the National Institutes of Health. Ryba and his colleagues found that you can actually taste without a tongue at all, simply by stimulating the "taste" part of the brain—the insular cortex. They ran the experiment in mice with a special sort of brain implant—a fiber-optic cable that turns neurons on with a pulse of laser light. And by switching on the "bitter" sensing part of the brain, they were able to make mice pucker up, as if they were tasting something bitter—even though absolutely nothing bitter was touching the tongues of the mice. In another experiment, the researchers fed the mice a bitter flavoring on their tongues—but then made it more palatable by switching on the "sweet" zone in the brain. "What we were doing here was adding the sweetness, but only adding it in the brain, not in what we were giving to the mouse." Think adding sugar to your coffee—but doing it only in your mind. The results appear in the journal Nature. Ryba says the study suggests that a lot of our basic judgments about taste—sweet means good, bitter means bad—are actually hard-wired at the level of the brain. As for that virtual-sugar-in-your-coffee idea? "I think it's basically science fiction to think that this would be something that would be applied to humans." But today's science fiction might be tomorrow's artificial sweetener.</t>
   </si>
   <si>
     <t>#234 Science in Baseball</t>
@@ -5984,7 +5984,7 @@
     <t>Hall of Famer Ted Williams once famously commented that hitting a baseball is the hardest thing to do in sports. Although Williams—a 0.344 career hitter—made it look easy, he had a point. Hitting a round ball with a round bat squarely is difficult. It's also an excellent example of some very __irritating/entertaining__ applied physics. No surprise then that professional baseball players are turning to science to improve their multimillion-dollar strokes. Some approaches focus on the neuroscience of hitting—the deep internal brain __visions/mechanisms__ behind seeing the pitch and reacting to it. But for more info about the swing itself, a sports tech company called Zepp Labs makes a sensor that can help break down those mechanics. The sensor sits in the knob of the company's so-called "Smart Bat" and uses two __travelers/accelerometers__ and a three-axis __wrought/gyroscope__ to measure bat speed, hand speed, attack angle and other factors. The sensor, which weighs only about eight grams, sends this info to a __microphone/smartphone__ app via Bluetooth. The app can then use this data to have an onscreen avatar reenact the swing, in the hope that the batter can pick up some details and make the necessary adjustments. Zepp's sensors can also be fitted to golf clubs and tennis rackets. Never one to mince words, Ted Williams also once said that pitchers were quote unquote "the stupidest people alive." Hmm, maybe somebody could come up with a smart baseball to help them. Against any Ted __trinities/Williamses__ out there, anyway.</t>
   </si>
   <si>
-    <t>Hall of Famer Ted Williams once famously commented that hitting a baseball is the hardest thing to do in sports. Although Williams—a 0.344 career hitter—made it look easy, he had a point. Hitting a round ball with a round bat squarely is difficult. It's also an excellent example of some very irritating applied physics. No surprise then that professional baseball players are turning to science to improve their multimillion-dollar strokes. Some approaches focus on the neuroscience of hitting—the deep internal brain visions behind seeing the pitch and reacting to it. But for more info about the swing itself, a sports tech company called Zepp Labs makes a sensor that can help break down those mechanics. The sensor sits in the knob of the company's so-called "Smart Bat" and uses two travelers and a three-axis wrought to measure bat speed, hand speed, attack angle and other factors. The sensor, which weighs only about eight grams, sends this info to a microphone app via Bluetooth. The app can then use this data to have an onscreen avatar reenact the swing, in the hope that the batter can pick up some details and make the necessary adjustments. Zepp's sensors can also be fitted to golf clubs and tennis rackets. Never one to mince words, Ted Williams also once said that pitchers were quote unquote "the stupidest people alive." Hmm, maybe somebody could come up with a smart baseball to help them. Against any Ted trinities out there, anyway.</t>
+    <t>Hall of Famer Ted Williams once famously commented that hitting a baseball is the hardest thing to do in sports. Although Williams—a 0.344 career hitter—made it look easy, he had a point. Hitting a round ball with a round bat squarely is difficult. It's also an excellent example of some very entertaining applied physics. No surprise then that professional baseball players are turning to science to improve their multimillion-dollar strokes. Some approaches focus on the neuroscience of hitting—the deep internal brain mechanisms behind seeing the pitch and reacting to it. But for more info about the swing itself, a sports tech company called Zepp Labs makes a sensor that can help break down those mechanics. The sensor sits in the knob of the company's so-called "Smart Bat" and uses two accelerometers and a three-axis gyroscope to measure bat speed, hand speed, attack angle and other factors. The sensor, which weighs only about eight grams, sends this info to a smartphone app via Bluetooth. The app can then use this data to have an onscreen avatar reenact the swing, in the hope that the batter can pick up some details and make the necessary adjustments. Zepp's sensors can also be fitted to golf clubs and tennis rackets. Never one to mince words, Ted Williams also once said that pitchers were quote unquote "the stupidest people alive." Hmm, maybe somebody could come up with a smart baseball to help them. Against any Ted Williamses out there, anyway.</t>
   </si>
   <si>
     <t>#235 Salt</t>
@@ -5993,7 +5993,7 @@
     <t>Even if you have a light hand with the salt shaker, you probably get lots of sodium in processed or restaurant meals. But sodium can contribute to high blood pressure, and __receivers/increases__ the risk for heart disease and failure, stroke, and kidney disease. So how many of us are limiting our sodium intake to recommended levels—which scientists say could reduce new cases of __dietary/coronary__ heart disease by 60-to-120 thousand per year. Researchers at the Centers for Disease Control analyzed data from the __infrastructural/National__ Health and Nutrition __cultivation/Examination__ Survey from 2005/2006, the most recent years available. Nearly 4,000 adults over 20-years-old completed a physical, had their blood __sienna/pressure__ taken and answered a survey of what they'd eaten over the past 24 hours. This food survey was taken again about a week later. According to the data, less than 10 percent of adults are limiting their sodium to recommended levels. The study appears in the journal Morbidity and Mortality Weekly Report. The researchers suggest that food __squirrels/manufacturers__ reduce the sodium in processed foods. And that consumers modify their eating habits—which might mean doing more cooking at home, where you have control of the salt.</t>
   </si>
   <si>
-    <t>Even if you have a light hand with the salt shaker, you probably get lots of sodium in processed or restaurant meals. But sodium can contribute to high blood pressure, and receivers the risk for heart disease and failure, stroke, and kidney disease. So how many of us are limiting our sodium intake to recommended levels—which scientists say could reduce new cases of dietary heart disease by 60-to-120 thousand per year. Researchers at the Centers for Disease Control analyzed data from the infrastructural Health and Nutrition cultivation Survey from 2005/2006, the most recent years available. Nearly 4,000 adults over 20-years-old completed a physical, had their blood sienna taken and answered a survey of what they'd eaten over the past 24 hours. This food survey was taken again about a week later. According to the data, less than 10 percent of adults are limiting their sodium to recommended levels. The study appears in the journal Morbidity and Mortality Weekly Report. The researchers suggest that food squirrels reduce the sodium in processed foods. And that consumers modify their eating habits—which might mean doing more cooking at home, where you have control of the salt.</t>
+    <t>Even if you have a light hand with the salt shaker, you probably get lots of sodium in processed or restaurant meals. But sodium can contribute to high blood pressure, and increases the risk for heart disease and failure, stroke, and kidney disease. So how many of us are limiting our sodium intake to recommended levels—which scientists say could reduce new cases of coronary heart disease by 60-to-120 thousand per year. Researchers at the Centers for Disease Control analyzed data from the National Health and Nutrition Examination Survey from 2005/2006, the most recent years available. Nearly 4,000 adults over 20-years-old completed a physical, had their blood pressure taken and answered a survey of what they'd eaten over the past 24 hours. This food survey was taken again about a week later. According to the data, less than 10 percent of adults are limiting their sodium to recommended levels. The study appears in the journal Morbidity and Mortality Weekly Report. The researchers suggest that food manufacturers reduce the sodium in processed foods. And that consumers modify their eating habits—which might mean doing more cooking at home, where you have control of the salt.</t>
   </si>
   <si>
     <t>#236 Perfect Pitch</t>
@@ -6002,7 +6002,7 @@
     <t>We might think perfect pitch is an innate talent. Well, a study in the American Journal of Human Genetics is __mobilizing/providing__ some __carousels/evidence__ for that. Perfect pitch, aka absolute pitch, is the rare ability to name or __reciprocate/recreate__ musical notes like A or middle C without using any comparable reference. Researchers at the University of California, San Francisco, studied the results from an online test taken by over ten thousand people. Not surprisingly, individuals tended to either have perfect pitch or not. But in a closer study of 73 families researchers found a region of genes on __anglophone/chromosome__ eight in those with perfect pitch and also they happened to be from European ancestry. More study is needed to actually zero in on just which gene or __agricultural/multiple__ genes might be responsible. And for comparison they intend to study individuals without perfect pitch but with equivalent musical training. There is some evidence that babies have the ability for absolute pitch, so researchers for this study theorize that maybe most lose this ability with age, but that what a so-called pitch gene does is extend this talent through a crucial period in childhood.</t>
   </si>
   <si>
-    <t>We might think perfect pitch is an innate talent. Well, a study in the American Journal of Human Genetics is mobilizing some carousels for that. Perfect pitch, aka absolute pitch, is the rare ability to name or reciprocate musical notes like A or middle C without using any comparable reference. Researchers at the University of California, San Francisco, studied the results from an online test taken by over ten thousand people. Not surprisingly, individuals tended to either have perfect pitch or not. But in a closer study of 73 families researchers found a region of genes on anglophone eight in those with perfect pitch and also they happened to be from European ancestry. More study is needed to actually zero in on just which gene or agricultural genes might be responsible. And for comparison they intend to study individuals without perfect pitch but with equivalent musical training. There is some evidence that babies have the ability for absolute pitch, so researchers for this study theorize that maybe most lose this ability with age, but that what a so-called pitch gene does is extend this talent through a crucial period in childhood.</t>
+    <t>We might think perfect pitch is an innate talent. Well, a study in the American Journal of Human Genetics is providing some evidence for that. Perfect pitch, aka absolute pitch, is the rare ability to name or recreate musical notes like A or middle C without using any comparable reference. Researchers at the University of California, San Francisco, studied the results from an online test taken by over ten thousand people. Not surprisingly, individuals tended to either have perfect pitch or not. But in a closer study of 73 families researchers found a region of genes on chromosome eight in those with perfect pitch and also they happened to be from European ancestry. More study is needed to actually zero in on just which gene or multiple genes might be responsible. And for comparison they intend to study individuals without perfect pitch but with equivalent musical training. There is some evidence that babies have the ability for absolute pitch, so researchers for this study theorize that maybe most lose this ability with age, but that what a so-called pitch gene does is extend this talent through a crucial period in childhood.</t>
   </si>
   <si>
     <t>#237 New Treatment</t>
@@ -6011,7 +6011,7 @@
     <t>Open a __newsletter/newspaper__ any day of the week and you're likely to read about a "promising new treatment" for one disease or another. But according to a study published in the September 5th issue of Science, it can take decades for those cures to make it to the clinic. __grievances/Researchers__ from the U.S. and Greece combed through the __spiritualistic/scientific__ literature to see how long it actually takes for compounds that look good in the laboratory to get through clinical trials and get used on patients. The scientists focused their attention on a handful of interventions that were widely hailed as being clinically effective. And they found that, for the average drug, the time that elapsed between its initial __motherly/discovery__ and the first paper to show its clinical effectiveness was about 24 years. Some drugs moved much faster. One of the protease inhibitors used to treat HIV made it from patenting through clinical trials in only four years. Maybe that's because the team studying that drug included experts in both basic and clinical sciences. The researchers say that such multidisciplinary efforts could help future treatments get to the clinic sooner. In the meantime, they note, scientists should avoid making promises about quick cures.</t>
   </si>
   <si>
-    <t>Open a newsletter any day of the week and you're likely to read about a "promising new treatment" for one disease or another. But according to a study published in the September 5th issue of Science, it can take decades for those cures to make it to the clinic. grievances from the U.S. and Greece combed through the spiritualistic literature to see how long it actually takes for compounds that look good in the laboratory to get through clinical trials and get used on patients. The scientists focused their attention on a handful of interventions that were widely hailed as being clinically effective. And they found that, for the average drug, the time that elapsed between its initial motherly and the first paper to show its clinical effectiveness was about 24 years. Some drugs moved much faster. One of the protease inhibitors used to treat HIV made it from patenting through clinical trials in only four years. Maybe that's because the team studying that drug included experts in both basic and clinical sciences. The researchers say that such multidisciplinary efforts could help future treatments get to the clinic sooner. In the meantime, they note, scientists should avoid making promises about quick cures.</t>
+    <t>Open a newspaper any day of the week and you're likely to read about a "promising new treatment" for one disease or another. But according to a study published in the September 5th issue of Science, it can take decades for those cures to make it to the clinic. Researchers from the U.S. and Greece combed through the scientific literature to see how long it actually takes for compounds that look good in the laboratory to get through clinical trials and get used on patients. The scientists focused their attention on a handful of interventions that were widely hailed as being clinically effective. And they found that, for the average drug, the time that elapsed between its initial discovery and the first paper to show its clinical effectiveness was about 24 years. Some drugs moved much faster. One of the protease inhibitors used to treat HIV made it from patenting through clinical trials in only four years. Maybe that's because the team studying that drug included experts in both basic and clinical sciences. The researchers say that such multidisciplinary efforts could help future treatments get to the clinic sooner. In the meantime, they note, scientists should avoid making promises about quick cures.</t>
   </si>
   <si>
     <t>#238 Junk Food</t>
@@ -6020,7 +6020,7 @@
     <t>The new Yankee Stadium has opened in the Bronx. I went to a game Saturday, and it's a much friendlier place for anyone trying to eat __compatibility/healthfully__ and __grain/maintain__ some environmental awareness. When I entered the park I stopped at the produce stand—the produce stand!—and bought a couple of fresh pears. Later I went to the Noodle Bowl stand, where for $8.50 I got a bowl of noodles, veggies and tofu. Tofu at the ballpark. The snack was listed on the menu board at 240 calories. All the food choices have calorie counts posted now, so you can avoid, or still indulge in, the almost 1,100 calorie Moe's Homewrecker Burrito at La Esquina Latina. I also had a caramel apple. Which as junk food goes is still pretty good. Every few yards you find a trio of disposal cans. For regular trash, plastic and compost. Which you may actually have items for, with a produce stand on site. And which may eventually foster a garden in which more fresh vegetables take root, root, root for the home team.</t>
   </si>
   <si>
-    <t>The new Yankee Stadium has opened in the Bronx. I went to a game Saturday, and it's a much friendlier place for anyone trying to eat compatibility and grain some environmental awareness. When I entered the park I stopped at the produce stand—the produce stand!—and bought a couple of fresh pears. Later I went to the Noodle Bowl stand, where for $8.50 I got a bowl of noodles, veggies and tofu. Tofu at the ballpark. The snack was listed on the menu board at 240 calories. All the food choices have calorie counts posted now, so you can avoid, or still indulge in, the almost 1,100 calorie Moe's Homewrecker Burrito at La Esquina Latina. I also had a caramel apple. Which as junk food goes is still pretty good. Every few yards you find a trio of disposal cans. For regular trash, plastic and compost. Which you may actually have items for, with a produce stand on site. And which may eventually foster a garden in which more fresh vegetables take root, root, root for the home team.</t>
+    <t>The new Yankee Stadium has opened in the Bronx. I went to a game Saturday, and it's a much friendlier place for anyone trying to eat healthfully and maintain some environmental awareness. When I entered the park I stopped at the produce stand—the produce stand!—and bought a couple of fresh pears. Later I went to the Noodle Bowl stand, where for $8.50 I got a bowl of noodles, veggies and tofu. Tofu at the ballpark. The snack was listed on the menu board at 240 calories. All the food choices have calorie counts posted now, so you can avoid, or still indulge in, the almost 1,100 calorie Moe's Homewrecker Burrito at La Esquina Latina. I also had a caramel apple. Which as junk food goes is still pretty good. Every few yards you find a trio of disposal cans. For regular trash, plastic and compost. Which you may actually have items for, with a produce stand on site. And which may eventually foster a garden in which more fresh vegetables take root, root, root for the home team.</t>
   </si>
   <si>
     <t>#239 Obesity in US</t>
@@ -6029,7 +6029,7 @@
     <t>As you've probably heard, the US is in the midst of an obesity epidemic. __celebrants/Americans__ just keep getting fatter and fatter. But the bad news doesn't end there. Because in today's issue of the New England Journal of Medicine, __itemise/scientists__ from Harvard and the University of California in San Diego report that obesity is __sagaciously/actually__ contagious. And it seems you catch it from your friends. After analyzing 32 years worth of data from more than 12,000 individuals, the __eatables/researchers__ found that thin people tend to cluster with thin people…and not just for warmth. And that people with more mass tend to gravitate toward one another, too. But it's not that folks seek friends with a similar physique. Or that people who pack on the pounds all frequent the same fast-food franchises or avoid the same gyms. What the scientists think is __canvassing/happening__ is that as those around you start plumping out, you come to think that being a bit hefty isn't such a bad thing. Then as you become larger, so do your friends. And your friends' friends. And their friends as well. The good news is that losing weight should also make your friends lighter. So order the salad and skip dessert. Believe me, your friends will be glad you did.</t>
   </si>
   <si>
-    <t>As you've probably heard, the US is in the midst of an obesity epidemic. celebrants just keep getting fatter and fatter. But the bad news doesn't end there. Because in today's issue of the New England Journal of Medicine, itemise from Harvard and the University of California in San Diego report that obesity is sagaciously contagious. And it seems you catch it from your friends. After analyzing 32 years worth of data from more than 12,000 individuals, the eatables found that thin people tend to cluster with thin people…and not just for warmth. And that people with more mass tend to gravitate toward one another, too. But it's not that folks seek friends with a similar physique. Or that people who pack on the pounds all frequent the same fast-food franchises or avoid the same gyms. What the scientists think is canvassing is that as those around you start plumping out, you come to think that being a bit hefty isn't such a bad thing. Then as you become larger, so do your friends. And your friends' friends. And their friends as well. The good news is that losing weight should also make your friends lighter. So order the salad and skip dessert. Believe me, your friends will be glad you did.</t>
+    <t>As you've probably heard, the US is in the midst of an obesity epidemic. Americans just keep getting fatter and fatter. But the bad news doesn't end there. Because in today's issue of the New England Journal of Medicine, scientists from Harvard and the University of California in San Diego report that obesity is actually contagious. And it seems you catch it from your friends. After analyzing 32 years worth of data from more than 12,000 individuals, the researchers found that thin people tend to cluster with thin people…and not just for warmth. And that people with more mass tend to gravitate toward one another, too. But it's not that folks seek friends with a similar physique. Or that people who pack on the pounds all frequent the same fast-food franchises or avoid the same gyms. What the scientists think is happening is that as those around you start plumping out, you come to think that being a bit hefty isn't such a bad thing. Then as you become larger, so do your friends. And your friends' friends. And their friends as well. The good news is that losing weight should also make your friends lighter. So order the salad and skip dessert. Believe me, your friends will be glad you did.</t>
   </si>
   <si>
     <t>#240 Kettle Whistle</t>
@@ -6038,7 +6038,7 @@
     <t>British physicist Lord __loudhailer/Rayleigh__ is best known for his __inadvertently/discovery__ of argon and for explaining, in 1871, why the sky is blue. But he also puzzled over this: . Rayleigh knew that a kettle makes that sound when steam jets through the hole in a thick lid that has a gap in the middle. He speculated that the jet becomes unstable inside that gap, setting up an acoustic feedback loop within the gap. But he couldn't prove it. Now two engineers at Cambridge University claim to have solved the puzzle—and proved Rayleigh wrong. The work is in the journal Physics of Fluids. The engineers found that a kettle __avuncularly/actually__ __centers/whistles__ in two distinct ways. It starts off with air __migrating/vibrating__ in the gap between the layers of the lid, like when you do this and this [sound of whistling]. But as the pressure builds, vortices of steam peel off from the jet exiting the lid. Each vortex creates sound waves at a __recently/frequency__ that depends on the length of the spout and the pressure inside it. Rising temperature means rising pressure, which __whooshes/produces__ a rising whistle. Which means it's time for tea.</t>
   </si>
   <si>
-    <t>British physicist Lord loudhailer is best known for his inadvertently of argon and for explaining, in 1871, why the sky is blue. But he also puzzled over this: . Rayleigh knew that a kettle makes that sound when steam jets through the hole in a thick lid that has a gap in the middle. He speculated that the jet becomes unstable inside that gap, setting up an acoustic feedback loop within the gap. But he couldn't prove it. Now two engineers at Cambridge University claim to have solved the puzzle—and proved Rayleigh wrong. The work is in the journal Physics of Fluids. The engineers found that a kettle avuncularly centers in two distinct ways. It starts off with air migrating in the gap between the layers of the lid, like when you do this and this [sound of whistling]. But as the pressure builds, vortices of steam peel off from the jet exiting the lid. Each vortex creates sound waves at a recently that depends on the length of the spout and the pressure inside it. Rising temperature means rising pressure, which whooshes a rising whistle. Which means it's time for tea.</t>
+    <t>British physicist Lord Rayleigh is best known for his discovery of argon and for explaining, in 1871, why the sky is blue. But he also puzzled over this: . Rayleigh knew that a kettle makes that sound when steam jets through the hole in a thick lid that has a gap in the middle. He speculated that the jet becomes unstable inside that gap, setting up an acoustic feedback loop within the gap. But he couldn't prove it. Now two engineers at Cambridge University claim to have solved the puzzle—and proved Rayleigh wrong. The work is in the journal Physics of Fluids. The engineers found that a kettle actually whistles in two distinct ways. It starts off with air vibrating in the gap between the layers of the lid, like when you do this and this [sound of whistling]. But as the pressure builds, vortices of steam peel off from the jet exiting the lid. Each vortex creates sound waves at a frequency that depends on the length of the spout and the pressure inside it. Rising temperature means rising pressure, which produces a rising whistle. Which means it's time for tea.</t>
   </si>
   <si>
     <t>#241 Particle Beams</t>
@@ -6047,7 +6047,7 @@
     <t>Physicists at the Brookhaven National __dorsi/Laboratory__ have been able to send information ahead of particle beams racing at nearly the speed of light. And the message to the beams is: Get in line. This technique has been developed at other labs but never used before with particle beams traveling in discrete bunches. These bunches are important in recreating that __lingerer/singular__ moment, the Big Bang. In these experiments, there are two different sets of ions, electrically charged particles, zooming towards each other around a 2.4 mile track. They collide into one another to __bait/recreate__ conditions that provide info about the Big Bang. But the ions spread out as they move. And this means that there are fewer collisions. In a technique called stochastic cooling, scientists first measure fluctuations in the beams of ions. Then they send signals even faster than these __jugglers/particles__ to devices up ahead that can kick those particles back into shape. Researchers say this technique allows them to create these collisions much more __leisurely/frequently__ and cheaply than other methods. And so they can get more and better data about what our universe might have been like just after it came into existence.</t>
   </si>
   <si>
-    <t>Physicists at the Brookhaven National dorsi have been able to send information ahead of particle beams racing at nearly the speed of light. And the message to the beams is: Get in line. This technique has been developed at other labs but never used before with particle beams traveling in discrete bunches. These bunches are important in recreating that lingerer moment, the Big Bang. In these experiments, there are two different sets of ions, electrically charged particles, zooming towards each other around a 2.4 mile track. They collide into one another to bait conditions that provide info about the Big Bang. But the ions spread out as they move. And this means that there are fewer collisions. In a technique called stochastic cooling, scientists first measure fluctuations in the beams of ions. Then they send signals even faster than these jugglers to devices up ahead that can kick those particles back into shape. Researchers say this technique allows them to create these collisions much more leisurely and cheaply than other methods. And so they can get more and better data about what our universe might have been like just after it came into existence.</t>
+    <t>Physicists at the Brookhaven National Laboratory have been able to send information ahead of particle beams racing at nearly the speed of light. And the message to the beams is: Get in line. This technique has been developed at other labs but never used before with particle beams traveling in discrete bunches. These bunches are important in recreating that singular moment, the Big Bang. In these experiments, there are two different sets of ions, electrically charged particles, zooming towards each other around a 2.4 mile track. They collide into one another to recreate conditions that provide info about the Big Bang. But the ions spread out as they move. And this means that there are fewer collisions. In a technique called stochastic cooling, scientists first measure fluctuations in the beams of ions. Then they send signals even faster than these particles to devices up ahead that can kick those particles back into shape. Researchers say this technique allows them to create these collisions much more frequently and cheaply than other methods. And so they can get more and better data about what our universe might have been like just after it came into existence.</t>
   </si>
   <si>
     <t>#242 Cloned Gene</t>
@@ -6056,7 +6056,7 @@
     <t>And now for another episode of __copyrighted/Seinfeld__ Science. On Monday we talked about cooler sports uniforms, one of George Costanza's crusades. Well, now it's Kramer's idea for a cologne that would make you smell like the beach. __Impolitenesses/Scientists__ from the University of East Anglia have just cloned the gene __mackerel/responsible__ for that briny, fishy scent we associate with the seaside. Andrew Johnston and his __tamales/colleagues__ __psychologist/harvested__ some bacteria from a coastal salt marsh. And they isolated a gene that makes dimethyl sulfide, a gas whose essence is pure eu d' ocean. In its natural environment, dimethyl sulfide helps sea birds sniff out a meal—in this case the plankton that produce it. And the compound is generated in such large quantities that it even forms clouds over the ocean that help cool the Earth's climate. Although Johnston and his team cloned the gene from a bacterium that thrives in the sea, they also found it in some unexpected places, including microbes that live in the roots of plants. Because these species are so different, he __tends/suspects__ that the bugs got the gene through a process akin to mating. Now, why they would want it is anybody's guess. Maybe, like Kramer, they just like the smell.</t>
   </si>
   <si>
-    <t>And now for another episode of copyrighted Science. On Monday we talked about cooler sports uniforms, one of George Costanza's crusades. Well, now it's Kramer's idea for a cologne that would make you smell like the beach. Impolitenesses from the University of East Anglia have just cloned the gene mackerel for that briny, fishy scent we associate with the seaside. Andrew Johnston and his tamales psychologist some bacteria from a coastal salt marsh. And they isolated a gene that makes dimethyl sulfide, a gas whose essence is pure eu d' ocean. In its natural environment, dimethyl sulfide helps sea birds sniff out a meal—in this case the plankton that produce it. And the compound is generated in such large quantities that it even forms clouds over the ocean that help cool the Earth's climate. Although Johnston and his team cloned the gene from a bacterium that thrives in the sea, they also found it in some unexpected places, including microbes that live in the roots of plants. Because these species are so different, he tends that the bugs got the gene through a process akin to mating. Now, why they would want it is anybody's guess. Maybe, like Kramer, they just like the smell.</t>
+    <t>And now for another episode of Seinfeld Science. On Monday we talked about cooler sports uniforms, one of George Costanza's crusades. Well, now it's Kramer's idea for a cologne that would make you smell like the beach. Scientists from the University of East Anglia have just cloned the gene responsible for that briny, fishy scent we associate with the seaside. Andrew Johnston and his colleagues harvested some bacteria from a coastal salt marsh. And they isolated a gene that makes dimethyl sulfide, a gas whose essence is pure eu d' ocean. In its natural environment, dimethyl sulfide helps sea birds sniff out a meal—in this case the plankton that produce it. And the compound is generated in such large quantities that it even forms clouds over the ocean that help cool the Earth's climate. Although Johnston and his team cloned the gene from a bacterium that thrives in the sea, they also found it in some unexpected places, including microbes that live in the roots of plants. Because these species are so different, he suspects that the bugs got the gene through a process akin to mating. Now, why they would want it is anybody's guess. Maybe, like Kramer, they just like the smell.</t>
   </si>
   <si>
     <t>#243 Art Studio</t>
@@ -6065,7 +6065,7 @@
     <t>A new __graphical/archaeological__ find may signify one of the great leaps in human cultural and cognitive history. Because researchers have discovered a 100,000-year-old art studio. It was known that ochre—rock with red or yellow pigments—was used for paint even that far back in history. But there was scant evidence for how it was prepared and handled. Then, in 2008, researchers uncovered an ochre mixing kit in a South African cave. They found two abalone shells, most likely used for paint mixing and storage. They also found ochre, bone, charcoal, grindstones and hammerstones. The researchers say the ochre was __angrily/probably__ rubbed on quartzite slabs to create a fine powder. It was then mixed and heated with other crushed substances, including other stones or mammal-bone. __inotropic/Microscopic__ striations on the inner abalone surface are likely scrape marks left during paint mixing. The research was published in the journal Science. The paint may have been used for body adornment or for long-gone artwork. And the __editions/presence__ of this paint-production laboratory indicates that the early humans knew basic chemistry and could plan for the future. One small paint-kit for a few humans, one major leap for humankind.</t>
   </si>
   <si>
-    <t>A new graphical find may signify one of the great leaps in human cultural and cognitive history. Because researchers have discovered a 100,000-year-old art studio. It was known that ochre—rock with red or yellow pigments—was used for paint even that far back in history. But there was scant evidence for how it was prepared and handled. Then, in 2008, researchers uncovered an ochre mixing kit in a South African cave. They found two abalone shells, most likely used for paint mixing and storage. They also found ochre, bone, charcoal, grindstones and hammerstones. The researchers say the ochre was angrily rubbed on quartzite slabs to create a fine powder. It was then mixed and heated with other crushed substances, including other stones or mammal-bone. inotropic striations on the inner abalone surface are likely scrape marks left during paint mixing. The research was published in the journal Science. The paint may have been used for body adornment or for long-gone artwork. And the editions of this paint-production laboratory indicates that the early humans knew basic chemistry and could plan for the future. One small paint-kit for a few humans, one major leap for humankind.</t>
+    <t>A new archaeological find may signify one of the great leaps in human cultural and cognitive history. Because researchers have discovered a 100,000-year-old art studio. It was known that ochre—rock with red or yellow pigments—was used for paint even that far back in history. But there was scant evidence for how it was prepared and handled. Then, in 2008, researchers uncovered an ochre mixing kit in a South African cave. They found two abalone shells, most likely used for paint mixing and storage. They also found ochre, bone, charcoal, grindstones and hammerstones. The researchers say the ochre was probably rubbed on quartzite slabs to create a fine powder. It was then mixed and heated with other crushed substances, including other stones or mammal-bone. Microscopic striations on the inner abalone surface are likely scrape marks left during paint mixing. The research was published in the journal Science. The paint may have been used for body adornment or for long-gone artwork. And the presence of this paint-production laboratory indicates that the early humans knew basic chemistry and could plan for the future. One small paint-kit for a few humans, one major leap for humankind.</t>
   </si>
   <si>
     <t>#244 Mars Winter</t>
@@ -6074,7 +6074,7 @@
     <t>As many of us broil in August heat, the Mars rover Spirit is hunkered down to survive a far more brutal season—a Martian winter. Spirit's been on Mars since January 2004 and already __reside/survived__ previous winters, which run from May through November. With __subtype/sunlight__ __hypothesising/reaching__ Spirit at a weak angle, the rover hibernates and uses the scant solar power to recharge batteries and heat itself to -40 degrees . At least, that's what's __cautioned/happened__ in previous winters. This winter, the game little unit just doesn't have enough juice to keep its heaters on, so temperatures inside the rover will plunge to a frigid -67 degrees Fahrenheit. When NASA scientists began signaling Spirit on July 26, they hoped to receive a __plainness/communications__ beep back—but so far there's only silence. The researchers say that in about two months sunlight will start to increase again through March 2011. If we haven't heard from Spirit by that point, then the likelihood is that we never will. The rover was __chimed/designed__ to work on Mars for three months, but was mobile for more than five years. Now mission scientists wait through the Martian winter to see if this ET will phone home.</t>
   </si>
   <si>
-    <t>As many of us broil in August heat, the Mars rover Spirit is hunkered down to survive a far more brutal season—a Martian winter. Spirit's been on Mars since January 2004 and already reside previous winters, which run from May through November. With subtype hypothesising Spirit at a weak angle, the rover hibernates and uses the scant solar power to recharge batteries and heat itself to -40 degrees . At least, that's what's cautioned in previous winters. This winter, the game little unit just doesn't have enough juice to keep its heaters on, so temperatures inside the rover will plunge to a frigid -67 degrees Fahrenheit. When NASA scientists began signaling Spirit on July 26, they hoped to receive a plainness beep back—but so far there's only silence. The researchers say that in about two months sunlight will start to increase again through March 2011. If we haven't heard from Spirit by that point, then the likelihood is that we never will. The rover was chimed to work on Mars for three months, but was mobile for more than five years. Now mission scientists wait through the Martian winter to see if this ET will phone home.</t>
+    <t>As many of us broil in August heat, the Mars rover Spirit is hunkered down to survive a far more brutal season—a Martian winter. Spirit's been on Mars since January 2004 and already survived previous winters, which run from May through November. With sunlight reaching Spirit at a weak angle, the rover hibernates and uses the scant solar power to recharge batteries and heat itself to -40 degrees . At least, that's what's happened in previous winters. This winter, the game little unit just doesn't have enough juice to keep its heaters on, so temperatures inside the rover will plunge to a frigid -67 degrees Fahrenheit. When NASA scientists began signaling Spirit on July 26, they hoped to receive a communications beep back—but so far there's only silence. The researchers say that in about two months sunlight will start to increase again through March 2011. If we haven't heard from Spirit by that point, then the likelihood is that we never will. The rover was designed to work on Mars for three months, but was mobile for more than five years. Now mission scientists wait through the Martian winter to see if this ET will phone home.</t>
   </si>
   <si>
     <t>#245 Jet Lag</t>
@@ -6083,7 +6083,7 @@
     <t>Jet lag. Jumping a few time zones causes problems with sleep and even digestion. But new research means we could be a step closer to preventing this voyager's vexation. The study centers on the hormone vasopressin, thought to have a role in maintaining our internal clock. Researchers genetically __speech/engineered__ mice that do not respond to vasopressin. Both engineered and normal rodents lived in a set cycle of light and dark for 2 weeks. Then the researchers changed the light cycle by eight hours. And the vasopressin-insensitive mice recovered from their induced jet lag much more quickly than did their __censuses/hormone-sensitive__ peers. The work is in the journal Science. Jet lag may seem like a minor annoyance. But for those who travel frequently or work unusual hours, it's a chronic problem that can increase the risk of hypertension and obesity. You cannot simply knock out __relearning/vasopressin__ signaling permanently—that would have negative effects on behavior and brain activity. But a drug that __essentially/temporarily__ suppresses vasopressin to reduce jet lag may be a frequent flier's dream.</t>
   </si>
   <si>
-    <t>Jet lag. Jumping a few time zones causes problems with sleep and even digestion. But new research means we could be a step closer to preventing this voyager's vexation. The study centers on the hormone vasopressin, thought to have a role in maintaining our internal clock. Researchers genetically speech mice that do not respond to vasopressin. Both engineered and normal rodents lived in a set cycle of light and dark for 2 weeks. Then the researchers changed the light cycle by eight hours. And the vasopressin-insensitive mice recovered from their induced jet lag much more quickly than did their censuses peers. The work is in the journal Science. Jet lag may seem like a minor annoyance. But for those who travel frequently or work unusual hours, it's a chronic problem that can increase the risk of hypertension and obesity. You cannot simply knock out relearning signaling permanently—that would have negative effects on behavior and brain activity. But a drug that essentially suppresses vasopressin to reduce jet lag may be a frequent flier's dream.</t>
+    <t>Jet lag. Jumping a few time zones causes problems with sleep and even digestion. But new research means we could be a step closer to preventing this voyager's vexation. The study centers on the hormone vasopressin, thought to have a role in maintaining our internal clock. Researchers genetically engineered mice that do not respond to vasopressin. Both engineered and normal rodents lived in a set cycle of light and dark for 2 weeks. Then the researchers changed the light cycle by eight hours. And the vasopressin-insensitive mice recovered from their induced jet lag much more quickly than did their hormone-sensitive peers. The work is in the journal Science. Jet lag may seem like a minor annoyance. But for those who travel frequently or work unusual hours, it's a chronic problem that can increase the risk of hypertension and obesity. You cannot simply knock out vasopressin signaling permanently—that would have negative effects on behavior and brain activity. But a drug that temporarily suppresses vasopressin to reduce jet lag may be a frequent flier's dream.</t>
   </si>
   <si>
     <t>#246 Australia's Greenhouse Gas</t>
@@ -6092,7 +6092,7 @@
     <t>It's basically all the same thing. A __generous/complicated__ plan to cut back Australia's greenhouse gases. And we are, per capita the biggest carbon polluters on the __globe/planet__ . But it's not carbon trading that will make the first big cuts in our emissions. The first big cuts will come from the Governments __reduced/renewable__ energy __policy/target__ . Melbourne-based __company/analyst__ Carbon Market Economics says the Governments 20 percent target will not only cut pollution, it'll help the economy as well.</t>
   </si>
   <si>
-    <t>It's basically all the same thing. A generous plan to cut back Australia's greenhouse gases. And we are, per capita the biggest carbon polluters on the globe . But it's not carbon trading that will make the first big cuts in our emissions. The first big cuts will come from the Governments reduced energy policy . Melbourne-based company Carbon Market Economics says the Governments 20 percent target will not only cut pollution, it'll help the economy as well.</t>
+    <t>It's basically all the same thing. A complicated plan to cut back Australia's greenhouse gases. And we are, per capita the biggest carbon polluters on the planet . But it's not carbon trading that will make the first big cuts in our emissions. The first big cuts will come from the Governments renewable energy target . Melbourne-based analyst Carbon Market Economics says the Governments 20 percent target will not only cut pollution, it'll help the economy as well.</t>
   </si>
   <si>
     <t>#247 Great Lies</t>
@@ -6101,7 +6101,7 @@
     <t>When I was pregnant, a friend gave me a book called Great Lies to Tell Small Kids. In it are gems like "wine makes mommy charming" and "men don't go bald naturally, they like getting their hair cut that way." Now, if you're filled with horror at the notion of pulling a toddler's leg like that, a new study in the Journal of Moral Education shows that parents regularly use deception to __perspicuous/influence__ their kids. We can all recall lies our parents told us to get us to do something, or to stop doing something. "If you cross your eyes they could stay that way" comes to mind. But in the current study, __sweeteners/researchers__ found that these parental fibs are hardly few and far between. And that even parents who preach to their kids about the importance of being honest admit to lying to them as well. The researchers plan to extend their studies to see whether all this lying __scribes/undermines__ children's trust. Until then, well, keep telling junior that if he spins around really fast, then stops, his face will skid around to the back of his head. It could keep him busy while mommy becomes even more charming.</t>
   </si>
   <si>
-    <t>When I was pregnant, a friend gave me a book called Great Lies to Tell Small Kids. In it are gems like "wine makes mommy charming" and "men don't go bald naturally, they like getting their hair cut that way." Now, if you're filled with horror at the notion of pulling a toddler's leg like that, a new study in the Journal of Moral Education shows that parents regularly use deception to perspicuous their kids. We can all recall lies our parents told us to get us to do something, or to stop doing something. "If you cross your eyes they could stay that way" comes to mind. But in the current study, sweeteners found that these parental fibs are hardly few and far between. And that even parents who preach to their kids about the importance of being honest admit to lying to them as well. The researchers plan to extend their studies to see whether all this lying scribes children's trust. Until then, well, keep telling junior that if he spins around really fast, then stops, his face will skid around to the back of his head. It could keep him busy while mommy becomes even more charming.</t>
+    <t>When I was pregnant, a friend gave me a book called Great Lies to Tell Small Kids. In it are gems like "wine makes mommy charming" and "men don't go bald naturally, they like getting their hair cut that way." Now, if you're filled with horror at the notion of pulling a toddler's leg like that, a new study in the Journal of Moral Education shows that parents regularly use deception to influence their kids. We can all recall lies our parents told us to get us to do something, or to stop doing something. "If you cross your eyes they could stay that way" comes to mind. But in the current study, researchers found that these parental fibs are hardly few and far between. And that even parents who preach to their kids about the importance of being honest admit to lying to them as well. The researchers plan to extend their studies to see whether all this lying undermines children's trust. Until then, well, keep telling junior that if he spins around really fast, then stops, his face will skid around to the back of his head. It could keep him busy while mommy becomes even more charming.</t>
   </si>
   <si>
     <t>#248 Cereal Boxes</t>
@@ -6110,7 +6110,7 @@
     <t>When you walk down the cereal aisle, do you ever get the feeling that Cap'n Crunch is looking at you? Well, that's just silly. He's __gluttonously/actually__ looking at your kids. That's according to a study by Brian Wansink and colleagues at Cornell University's Food and Brand Lab. The researchers wondered whether the __varnishes/characters__ on cereal boxes actually make eye contact. And whether that could influence a shopper's choice of breakfast fare. So they hit the cereal aisle. And they found that kids' cereals tend to be placed on lower shelves than grownup offerings. What's more, Tony the Tiger and his kid-friendly pals tend to gaze downward, while the Quaker Oats guy stares straight ahead. In a second study, adult volunteers were handed a box of Trix. On some boxes, the rabbit looked straight ahead, on others, he gazed away. When asked what they thought of Trix, it seems that folks felt more __tilted/connected__ to the brand, and said they preferred that cereal over others, when the rabbit looked them in the eye. The results, which appear in the Journal of __quieted/Environment__ and Behavior, suggest that certain tricks are not just for kids…but maybe for marketers, too.</t>
   </si>
   <si>
-    <t>When you walk down the cereal aisle, do you ever get the feeling that Cap'n Crunch is looking at you? Well, that's just silly. He's gluttonously looking at your kids. That's according to a study by Brian Wansink and colleagues at Cornell University's Food and Brand Lab. The researchers wondered whether the varnishes on cereal boxes actually make eye contact. And whether that could influence a shopper's choice of breakfast fare. So they hit the cereal aisle. And they found that kids' cereals tend to be placed on lower shelves than grownup offerings. What's more, Tony the Tiger and his kid-friendly pals tend to gaze downward, while the Quaker Oats guy stares straight ahead. In a second study, adult volunteers were handed a box of Trix. On some boxes, the rabbit looked straight ahead, on others, he gazed away. When asked what they thought of Trix, it seems that folks felt more tilted to the brand, and said they preferred that cereal over others, when the rabbit looked them in the eye. The results, which appear in the Journal of quieted and Behavior, suggest that certain tricks are not just for kids…but maybe for marketers, too.</t>
+    <t>When you walk down the cereal aisle, do you ever get the feeling that Cap'n Crunch is looking at you? Well, that's just silly. He's actually looking at your kids. That's according to a study by Brian Wansink and colleagues at Cornell University's Food and Brand Lab. The researchers wondered whether the characters on cereal boxes actually make eye contact. And whether that could influence a shopper's choice of breakfast fare. So they hit the cereal aisle. And they found that kids' cereals tend to be placed on lower shelves than grownup offerings. What's more, Tony the Tiger and his kid-friendly pals tend to gaze downward, while the Quaker Oats guy stares straight ahead. In a second study, adult volunteers were handed a box of Trix. On some boxes, the rabbit looked straight ahead, on others, he gazed away. When asked what they thought of Trix, it seems that folks felt more connected to the brand, and said they preferred that cereal over others, when the rabbit looked them in the eye. The results, which appear in the Journal of Environment and Behavior, suggest that certain tricks are not just for kids…but maybe for marketers, too.</t>
   </si>
   <si>
     <t>#249 Microbial Cloud</t>
@@ -6119,7 +6119,7 @@
     <t>You might blame your pets for shedding all over the house. But we humans do it too—and our stuff is alive. "We're __partially/constantly__ emitting __provisoes/microbes__ around us. And this is coming from shedding of our skin, from exhaling, our hair, we're just full of these guys." Adam Altrichter, a microbial ecologist at the __cannery/University__ of Oregon. "We've never been sterile organisms. We are definitely masses of microbes both in and on us." If you're picturing the Peanuts character Pig Pen, you may not be far off. Because biologists __increment/estimate__ we shed a million particles an hour—including, of course, a lot of bacteria. Altrichter and his __daddies/colleagues__ wanted to measure that cloud of particles—the "Pig Pen" effect, if you will—so they asked 11 volunteers not to shower, dressed them in shorts and tank tops, and put them in a sterile chamber for hours at a time, while collecting microbial samples on surfaces and in the air. What they found in those samples was a menagerie of bacteria from the volunteers' skin, guts, genital tracts, lungs, noses and mouths. And for eight of the 11 study subjects, the microbial cloud was unique enough to identify the individual who'd left it—suggesting that this bacterial 'fingerprint' could someday be used in forensics. The study is in the journal PeerJ. Given that we spend 90 percent of our lives indoors, our microbial clouds also colonize the places we live and work—and, yes, the people around us. "And so it's just kind of interesting to think about how the people that we interact with at work, or in classrooms, or in other environments, how we could be sharing some of these microbial __campuses/passengers__ between us, not even knowing anything about it." And now that you do know about it—hopefully your view of your coworkers won't become…clouded.</t>
   </si>
   <si>
-    <t>You might blame your pets for shedding all over the house. But we humans do it too—and our stuff is alive. "We're partially emitting provisoes around us. And this is coming from shedding of our skin, from exhaling, our hair, we're just full of these guys." Adam Altrichter, a microbial ecologist at the cannery of Oregon. "We've never been sterile organisms. We are definitely masses of microbes both in and on us." If you're picturing the Peanuts character Pig Pen, you may not be far off. Because biologists increment we shed a million particles an hour—including, of course, a lot of bacteria. Altrichter and his daddies wanted to measure that cloud of particles—the "Pig Pen" effect, if you will—so they asked 11 volunteers not to shower, dressed them in shorts and tank tops, and put them in a sterile chamber for hours at a time, while collecting microbial samples on surfaces and in the air. What they found in those samples was a menagerie of bacteria from the volunteers' skin, guts, genital tracts, lungs, noses and mouths. And for eight of the 11 study subjects, the microbial cloud was unique enough to identify the individual who'd left it—suggesting that this bacterial 'fingerprint' could someday be used in forensics. The study is in the journal PeerJ. Given that we spend 90 percent of our lives indoors, our microbial clouds also colonize the places we live and work—and, yes, the people around us. "And so it's just kind of interesting to think about how the people that we interact with at work, or in classrooms, or in other environments, how we could be sharing some of these microbial campuses between us, not even knowing anything about it." And now that you do know about it—hopefully your view of your coworkers won't become…clouded.</t>
+    <t>You might blame your pets for shedding all over the house. But we humans do it too—and our stuff is alive. "We're constantly emitting microbes around us. And this is coming from shedding of our skin, from exhaling, our hair, we're just full of these guys." Adam Altrichter, a microbial ecologist at the University of Oregon. "We've never been sterile organisms. We are definitely masses of microbes both in and on us." If you're picturing the Peanuts character Pig Pen, you may not be far off. Because biologists estimate we shed a million particles an hour—including, of course, a lot of bacteria. Altrichter and his colleagues wanted to measure that cloud of particles—the "Pig Pen" effect, if you will—so they asked 11 volunteers not to shower, dressed them in shorts and tank tops, and put them in a sterile chamber for hours at a time, while collecting microbial samples on surfaces and in the air. What they found in those samples was a menagerie of bacteria from the volunteers' skin, guts, genital tracts, lungs, noses and mouths. And for eight of the 11 study subjects, the microbial cloud was unique enough to identify the individual who'd left it—suggesting that this bacterial 'fingerprint' could someday be used in forensics. The study is in the journal PeerJ. Given that we spend 90 percent of our lives indoors, our microbial clouds also colonize the places we live and work—and, yes, the people around us. "And so it's just kind of interesting to think about how the people that we interact with at work, or in classrooms, or in other environments, how we could be sharing some of these microbial passengers between us, not even knowing anything about it." And now that you do know about it—hopefully your view of your coworkers won't become…clouded.</t>
   </si>
   <si>
     <t>#250 Oil Obsorber</t>
@@ -6128,7 +6128,7 @@
     <t>It might look and even feel like paper, but a new material created by __biases/scientists__ at MIT is designed to be an oil spill super-absorber. This __paleontology/technology__ debuted in a recent issue of Nature Biotechnology. __hyperlinks/Scientists__ designed a mesh of __merchandize/nanowires__ made of potassium __yields/manganese__ oxide. The mesh is dried in much the same manner as cellulose is treated to make paper. Between the nanowires are tiny pores that act like capillaries to absorb liquid—again, like a paper towel. But the wires have a coating that repels water. In fact, researchers say this material can be left in water for a month and, when taken out, will still be dry. But oil can seep into those pores. The nanopaper can absorb twenty times its weight in oil. And it can be reused. Potassium manganese oxide is stable at high temperatures. So to clean it, researchers heat it above the boiling point of oil. The oil __race/evaporates__ and the paper is clean again. About 200,000 tons of oil have polluted waters around the world in this decade alone. Scientists say this new nano oil cleaner could help sop up inevitable future spills.</t>
   </si>
   <si>
-    <t>It might look and even feel like paper, but a new material created by biases at MIT is designed to be an oil spill super-absorber. This paleontology debuted in a recent issue of Nature Biotechnology. hyperlinks designed a mesh of merchandize made of potassium yields oxide. The mesh is dried in much the same manner as cellulose is treated to make paper. Between the nanowires are tiny pores that act like capillaries to absorb liquid—again, like a paper towel. But the wires have a coating that repels water. In fact, researchers say this material can be left in water for a month and, when taken out, will still be dry. But oil can seep into those pores. The nanopaper can absorb twenty times its weight in oil. And it can be reused. Potassium manganese oxide is stable at high temperatures. So to clean it, researchers heat it above the boiling point of oil. The oil race and the paper is clean again. About 200,000 tons of oil have polluted waters around the world in this decade alone. Scientists say this new nano oil cleaner could help sop up inevitable future spills.</t>
+    <t>It might look and even feel like paper, but a new material created by scientists at MIT is designed to be an oil spill super-absorber. This technology debuted in a recent issue of Nature Biotechnology. Scientists designed a mesh of nanowires made of potassium manganese oxide. The mesh is dried in much the same manner as cellulose is treated to make paper. Between the nanowires are tiny pores that act like capillaries to absorb liquid—again, like a paper towel. But the wires have a coating that repels water. In fact, researchers say this material can be left in water for a month and, when taken out, will still be dry. But oil can seep into those pores. The nanopaper can absorb twenty times its weight in oil. And it can be reused. Potassium manganese oxide is stable at high temperatures. So to clean it, researchers heat it above the boiling point of oil. The oil evaporates and the paper is clean again. About 200,000 tons of oil have polluted waters around the world in this decade alone. Scientists say this new nano oil cleaner could help sop up inevitable future spills.</t>
   </si>
   <si>
     <t>#251 Self-healed Scratches</t>
@@ -6137,7 +6137,7 @@
     <t>If you get a scratch, your skin can heal itself. But if your car gets scratched, it stays scratched. Scientists at the __reality/University__ of Southern __complementary/Mississippi__ think they may have solved that problem. They've developed a new __venereal/material__ that can self-heal __planets/scratches__ when exposed to sunlight. They published this __pap/research__ in the March 13th issue of the journal Science. The new technology first takes polyurethane—the coating on many cars. Then researchers added chitosan—that's a key polymer in crab and shrimp shells. The final bit thrown into the mix are minute amounts of oxetane rings, with three atoms of carbon and one of oxygen. The researchers are trying to mimic natural processes. Here's how it works. When there's a scratch, __enameling/damaging__ the molecule, the oxetane ring opens. It has two reactive ends. In sunlight, chitosan breaks into two chains and generates free radicals. Then those chitosan chains link up with the reactive ends of the oxetane, filling in the scratch. Researchers say this technique is much simpler and more cost-efficient than other attempts at self-healing. So maybe in the future, when your car gets scraped, it'll be all healed up before you have to spend any of your hard earned scratch.</t>
   </si>
   <si>
-    <t>If you get a scratch, your skin can heal itself. But if your car gets scratched, it stays scratched. Scientists at the reality of Southern complementary think they may have solved that problem. They've developed a new venereal that can self-heal planets when exposed to sunlight. They published this pap in the March 13th issue of the journal Science. The new technology first takes polyurethane—the coating on many cars. Then researchers added chitosan—that's a key polymer in crab and shrimp shells. The final bit thrown into the mix are minute amounts of oxetane rings, with three atoms of carbon and one of oxygen. The researchers are trying to mimic natural processes. Here's how it works. When there's a scratch, enameling the molecule, the oxetane ring opens. It has two reactive ends. In sunlight, chitosan breaks into two chains and generates free radicals. Then those chitosan chains link up with the reactive ends of the oxetane, filling in the scratch. Researchers say this technique is much simpler and more cost-efficient than other attempts at self-healing. So maybe in the future, when your car gets scraped, it'll be all healed up before you have to spend any of your hard earned scratch.</t>
+    <t>If you get a scratch, your skin can heal itself. But if your car gets scratched, it stays scratched. Scientists at the University of Southern Mississippi think they may have solved that problem. They've developed a new material that can self-heal scratches when exposed to sunlight. They published this research in the March 13th issue of the journal Science. The new technology first takes polyurethane—the coating on many cars. Then researchers added chitosan—that's a key polymer in crab and shrimp shells. The final bit thrown into the mix are minute amounts of oxetane rings, with three atoms of carbon and one of oxygen. The researchers are trying to mimic natural processes. Here's how it works. When there's a scratch, damaging the molecule, the oxetane ring opens. It has two reactive ends. In sunlight, chitosan breaks into two chains and generates free radicals. Then those chitosan chains link up with the reactive ends of the oxetane, filling in the scratch. Researchers say this technique is much simpler and more cost-efficient than other attempts at self-healing. So maybe in the future, when your car gets scraped, it'll be all healed up before you have to spend any of your hard earned scratch.</t>
   </si>
   <si>
     <t>#252 Steroids</t>
@@ -6146,7 +6146,7 @@
     <t>Veteran sportswriter and __victim/journalism__ professor Justice B. Hill on August 1st at the annual meeting of the National Association of Black Journalists in Orlando. But that resolution won't be easy. "The science will always stay ahead of the detection. I did an interview __conceivably/recently__ with a bioethicist from Case Western Reserve University. And one of the things he advocates is, let players use whatever they want to under a doctor's supervision. Because he understands — I did a piece years ago where I was talking to one of the foremost authorities on PEDs, and one of the things he said was we're going to get into gene cloning. "The __calibration/sophistication__ of the technology is going to make this detection game even more dicier in the years to come. And I think baseball, the union, all of them are tired of the discussion of steroids. They want to get back to the playing of the game. And that's a huge issue for those of us who love baseball."</t>
   </si>
   <si>
-    <t>Veteran sportswriter and victim professor Justice B. Hill on August 1st at the annual meeting of the National Association of Black Journalists in Orlando. But that resolution won't be easy. "The science will always stay ahead of the detection. I did an interview conceivably with a bioethicist from Case Western Reserve University. And one of the things he advocates is, let players use whatever they want to under a doctor's supervision. Because he understands — I did a piece years ago where I was talking to one of the foremost authorities on PEDs, and one of the things he said was we're going to get into gene cloning. "The calibration of the technology is going to make this detection game even more dicier in the years to come. And I think baseball, the union, all of them are tired of the discussion of steroids. They want to get back to the playing of the game. And that's a huge issue for those of us who love baseball."</t>
+    <t>Veteran sportswriter and journalism professor Justice B. Hill on August 1st at the annual meeting of the National Association of Black Journalists in Orlando. But that resolution won't be easy. "The science will always stay ahead of the detection. I did an interview recently with a bioethicist from Case Western Reserve University. And one of the things he advocates is, let players use whatever they want to under a doctor's supervision. Because he understands — I did a piece years ago where I was talking to one of the foremost authorities on PEDs, and one of the things he said was we're going to get into gene cloning. "The sophistication of the technology is going to make this detection game even more dicier in the years to come. And I think baseball, the union, all of them are tired of the discussion of steroids. They want to get back to the playing of the game. And that's a huge issue for those of us who love baseball."</t>
   </si>
   <si>
     <t>#253 Recognition of Voice</t>
@@ -6155,7 +6155,7 @@
     <t>It's tough to pick a familiar face out of a crowd—but focusing on a known voice in a noisy room is easy. And a new study scanned volunteers' brains to look at how we solve the so-called cocktail party problem. The work is in the journal Nature. Researchers __longhand/recorded__ the activity of the subject's cerebral cortexes while playing them __paragons/sentences__ spoken by __militant/different__ voices. First, the subjects listened to __transmissible/individual__ sentences and reported key __cleavers/features__ of each one. Then, they heard two different sentences played at the same time, but had to listen to and recall details from only one voice. Each voice drew a __missioner/particular__ response from the __preparatory/auditory__ cortex. And even with an extra sentence playing simultaneously, researchers saw that the cortex responded specifically to the voice that the subject was focusing on. This finding indicates that our brains process sound based not only on the audio input they receive, but also on our listening goals. And it could lead to speech recognition systems that are accurate in crowds — even at a cocktail party.</t>
   </si>
   <si>
-    <t>It's tough to pick a familiar face out of a crowd—but focusing on a known voice in a noisy room is easy. And a new study scanned volunteers' brains to look at how we solve the so-called cocktail party problem. The work is in the journal Nature. Researchers longhand the activity of the subject's cerebral cortexes while playing them paragons spoken by militant voices. First, the subjects listened to transmissible sentences and reported key cleavers of each one. Then, they heard two different sentences played at the same time, but had to listen to and recall details from only one voice. Each voice drew a missioner response from the preparatory cortex. And even with an extra sentence playing simultaneously, researchers saw that the cortex responded specifically to the voice that the subject was focusing on. This finding indicates that our brains process sound based not only on the audio input they receive, but also on our listening goals. And it could lead to speech recognition systems that are accurate in crowds — even at a cocktail party.</t>
+    <t>It's tough to pick a familiar face out of a crowd—but focusing on a known voice in a noisy room is easy. And a new study scanned volunteers' brains to look at how we solve the so-called cocktail party problem. The work is in the journal Nature. Researchers recorded the activity of the subject's cerebral cortexes while playing them sentences spoken by different voices. First, the subjects listened to individual sentences and reported key features of each one. Then, they heard two different sentences played at the same time, but had to listen to and recall details from only one voice. Each voice drew a particular response from the auditory cortex. And even with an extra sentence playing simultaneously, researchers saw that the cortex responded specifically to the voice that the subject was focusing on. This finding indicates that our brains process sound based not only on the audio input they receive, but also on our listening goals. And it could lead to speech recognition systems that are accurate in crowds — even at a cocktail party.</t>
   </si>
   <si>
     <t>#254 Net Loss</t>
@@ -6164,7 +6164,7 @@
     <t>Some things are hard to remember. Others are hard to forget—especially things that are traumatic. But kids, it turns out, are better than adults at __refreshing/forgetting__ the bad stuff. Now scientists think they know why. According to an animal study in the September 4th issue of the journal Science, the brains of adults erect __nonelectrical/physical__ barriers that keep painful __bigotries/memories__ intact. As adults, events that emotionally disturb us tend to get seared into our brains. And those memories can resurface, causing anxiety, fear and even post-traumatic stress disorder. But young brains are much more resilient—and can even erase unpleasant memories. To get a better handle on this youthful forgetting, scientists studied the brains of young and old rats. They found that in adult brains, a physical net forms around certain cells in the amygdala, a structure associated with __cortical/emotional__ memories. Adults that had been trained to associate a mild foot shock with a specific sound would flinch when they just heard the sound. But using a drug to dissolve this barrier restored the older rats' ability to __selfish/extinguish__ fearful memories. So rats that got the net-busting treatment stayed calm when they heard the sound. It's one of the few instances where a net loss is a real gain.</t>
   </si>
   <si>
-    <t>Some things are hard to remember. Others are hard to forget—especially things that are traumatic. But kids, it turns out, are better than adults at refreshing the bad stuff. Now scientists think they know why. According to an animal study in the September 4th issue of the journal Science, the brains of adults erect nonelectrical barriers that keep painful bigotries intact. As adults, events that emotionally disturb us tend to get seared into our brains. And those memories can resurface, causing anxiety, fear and even post-traumatic stress disorder. But young brains are much more resilient—and can even erase unpleasant memories. To get a better handle on this youthful forgetting, scientists studied the brains of young and old rats. They found that in adult brains, a physical net forms around certain cells in the amygdala, a structure associated with cortical memories. Adults that had been trained to associate a mild foot shock with a specific sound would flinch when they just heard the sound. But using a drug to dissolve this barrier restored the older rats' ability to selfish fearful memories. So rats that got the net-busting treatment stayed calm when they heard the sound. It's one of the few instances where a net loss is a real gain.</t>
+    <t>Some things are hard to remember. Others are hard to forget—especially things that are traumatic. But kids, it turns out, are better than adults at forgetting the bad stuff. Now scientists think they know why. According to an animal study in the September 4th issue of the journal Science, the brains of adults erect physical barriers that keep painful memories intact. As adults, events that emotionally disturb us tend to get seared into our brains. And those memories can resurface, causing anxiety, fear and even post-traumatic stress disorder. But young brains are much more resilient—and can even erase unpleasant memories. To get a better handle on this youthful forgetting, scientists studied the brains of young and old rats. They found that in adult brains, a physical net forms around certain cells in the amygdala, a structure associated with emotional memories. Adults that had been trained to associate a mild foot shock with a specific sound would flinch when they just heard the sound. But using a drug to dissolve this barrier restored the older rats' ability to extinguish fearful memories. So rats that got the net-busting treatment stayed calm when they heard the sound. It's one of the few instances where a net loss is a real gain.</t>
   </si>
   <si>
     <t>#255 Spicy Food</t>
@@ -6173,7 +6173,7 @@
     <t>Chinese cuisine has a lot of __accommodatingly/blazingly__ spicy dishes, like mapo tofu and hot pot. And, of course, there's the ever-present chili oil. "I like spicy food myself." Lu Qi, an epidemiologist at the Harvard School of Public Health. "Almost every day, I eat spicy food." That spicy tradition served as __honorific/scientific__ inspiration for Qi: he and colleagues performed a study which found that a daily dose of chilies might actually be a boon to your health. The researchers enrolled nearly half a million Chinese volunteers, aged 30 to 79. They quizzed them on their affinity for fiery foods, and followed each study subject for an average of seven years. During that time, more than 20,000 of the __cockpits/subjects__ died. But after controlling for factors like smoking history and income, the scientists found that the risk of death was 10 percent lower in those who ate spicy food a couple times a week, compared with those who abstained. And daily chili eaters, like Lu, had a 14 percent lower risk of dying. That figure held true for both men and women. And yes, while it is a __pathogenicity/relatively__ modest effect, Lu says to keep in mind: we're just talking about chilies here. "It's not medicine." The findings appear in the British Medical Journal. Previous studies have shown that capsaicin, the active ingredient in chillies, has anti-inflammatory and antimicrobial effects, among others. But before you grab the Tabasco, this study doesn't prove causation. For example, could be that people with weaker constitutions avoid spicy foods—making chili lovers appear more hardy in comparison. And the authors don't recommend starting a chili habit if you already have a sensitive stomach. But at least one thing's clear: indulging in spicy food probably won't hurt. Other than, well, your tongue.</t>
   </si>
   <si>
-    <t>Chinese cuisine has a lot of accommodatingly spicy dishes, like mapo tofu and hot pot. And, of course, there's the ever-present chili oil. "I like spicy food myself." Lu Qi, an epidemiologist at the Harvard School of Public Health. "Almost every day, I eat spicy food." That spicy tradition served as honorific inspiration for Qi: he and colleagues performed a study which found that a daily dose of chilies might actually be a boon to your health. The researchers enrolled nearly half a million Chinese volunteers, aged 30 to 79. They quizzed them on their affinity for fiery foods, and followed each study subject for an average of seven years. During that time, more than 20,000 of the cockpits died. But after controlling for factors like smoking history and income, the scientists found that the risk of death was 10 percent lower in those who ate spicy food a couple times a week, compared with those who abstained. And daily chili eaters, like Lu, had a 14 percent lower risk of dying. That figure held true for both men and women. And yes, while it is a pathogenicity modest effect, Lu says to keep in mind: we're just talking about chilies here. "It's not medicine." The findings appear in the British Medical Journal. Previous studies have shown that capsaicin, the active ingredient in chillies, has anti-inflammatory and antimicrobial effects, among others. But before you grab the Tabasco, this study doesn't prove causation. For example, could be that people with weaker constitutions avoid spicy foods—making chili lovers appear more hardy in comparison. And the authors don't recommend starting a chili habit if you already have a sensitive stomach. But at least one thing's clear: indulging in spicy food probably won't hurt. Other than, well, your tongue.</t>
+    <t>Chinese cuisine has a lot of blazingly spicy dishes, like mapo tofu and hot pot. And, of course, there's the ever-present chili oil. "I like spicy food myself." Lu Qi, an epidemiologist at the Harvard School of Public Health. "Almost every day, I eat spicy food." That spicy tradition served as scientific inspiration for Qi: he and colleagues performed a study which found that a daily dose of chilies might actually be a boon to your health. The researchers enrolled nearly half a million Chinese volunteers, aged 30 to 79. They quizzed them on their affinity for fiery foods, and followed each study subject for an average of seven years. During that time, more than 20,000 of the subjects died. But after controlling for factors like smoking history and income, the scientists found that the risk of death was 10 percent lower in those who ate spicy food a couple times a week, compared with those who abstained. And daily chili eaters, like Lu, had a 14 percent lower risk of dying. That figure held true for both men and women. And yes, while it is a relatively modest effect, Lu says to keep in mind: we're just talking about chilies here. "It's not medicine." The findings appear in the British Medical Journal. Previous studies have shown that capsaicin, the active ingredient in chillies, has anti-inflammatory and antimicrobial effects, among others. But before you grab the Tabasco, this study doesn't prove causation. For example, could be that people with weaker constitutions avoid spicy foods—making chili lovers appear more hardy in comparison. And the authors don't recommend starting a chili habit if you already have a sensitive stomach. But at least one thing's clear: indulging in spicy food probably won't hurt. Other than, well, your tongue.</t>
   </si>
   <si>
     <t>#256 Ringing Ears</t>
@@ -6182,7 +6182,7 @@
     <t>If you're ever worried that you've had one too many drinks after a night of bar-hopping, you might want to ask yourself: Are my ears ringing? Because it turns out that when the music gets loud, we tend to drain our mug of brew faster. That's according to a study to be published in the journal Alcoholism: Clinical and Experimental Research. Researchers staked out two bars in the west of France and __respond/observed__ __sending/drinking__ habits of 40 patrons. With permission from bartenders, the scientists pumped up the volume of a Top 40 station from 72 to 88 pounding decibels. In this __fearing/earsplitting__ din of pop-music, patrons drank more in less time. While it's been known that music played in the mall can influence consumer behavior, this study is the first to take that theory to the bar scene. The researchers __liberate/speculate__ that loud music may energize and excite bar-hoppers, making them more likely to binge. Or, they say, perhaps it was just too loud to talk, so people focused instead on their pint-sized companions. Either way, if you're trying to cut back on your beer, might I suggest an earplug chaser?</t>
   </si>
   <si>
-    <t>If you're ever worried that you've had one too many drinks after a night of bar-hopping, you might want to ask yourself: Are my ears ringing? Because it turns out that when the music gets loud, we tend to drain our mug of brew faster. That's according to a study to be published in the journal Alcoholism: Clinical and Experimental Research. Researchers staked out two bars in the west of France and respond sending habits of 40 patrons. With permission from bartenders, the scientists pumped up the volume of a Top 40 station from 72 to 88 pounding decibels. In this fearing din of pop-music, patrons drank more in less time. While it's been known that music played in the mall can influence consumer behavior, this study is the first to take that theory to the bar scene. The researchers liberate that loud music may energize and excite bar-hoppers, making them more likely to binge. Or, they say, perhaps it was just too loud to talk, so people focused instead on their pint-sized companions. Either way, if you're trying to cut back on your beer, might I suggest an earplug chaser?</t>
+    <t>If you're ever worried that you've had one too many drinks after a night of bar-hopping, you might want to ask yourself: Are my ears ringing? Because it turns out that when the music gets loud, we tend to drain our mug of brew faster. That's according to a study to be published in the journal Alcoholism: Clinical and Experimental Research. Researchers staked out two bars in the west of France and observed drinking habits of 40 patrons. With permission from bartenders, the scientists pumped up the volume of a Top 40 station from 72 to 88 pounding decibels. In this earsplitting din of pop-music, patrons drank more in less time. While it's been known that music played in the mall can influence consumer behavior, this study is the first to take that theory to the bar scene. The researchers speculate that loud music may energize and excite bar-hoppers, making them more likely to binge. Or, they say, perhaps it was just too loud to talk, so people focused instead on their pint-sized companions. Either way, if you're trying to cut back on your beer, might I suggest an earplug chaser?</t>
   </si>
   <si>
     <t>#257 Helmet Law</t>
@@ -6191,7 +6191,7 @@
     <t>Jerry Seinfeld once said, "The stupidest thing is a helmet law, the point of which is to protect a brain that is functioning so poorly it's not even trying to prevent the __enhancing/cracking__ of the skull it's in." But helmet laws for kids, who may not have considered their skulls as deeply as Jerry did, aren't so dumb. That's __upholding/according__ to a new study in a publication from the Chocrane Collaboration, which is an international organization that __cooperates/evaluates__ health care research. The review looked at five studies of kids bike-helmet laws. One big 10 year study in California found that bike-related __panchromatic/traumatic__ brain injury in kids dropped more than 18 percent after the state's bike helmet law was enacted. A Canadian study looked at almost 10,000 bike related __optical/hospital__ admissions and found a 45 percent drop in childhood head injuries in provinces that passed helmet laws. Provinces without helmet laws also saw a drop in the same period, but only half as much. And three other studies found that helmet laws do indeed persuade kids to wear their helmets, with __paribus/increases__ in compliance ranging from 45 to 84 percent.</t>
   </si>
   <si>
-    <t>Jerry Seinfeld once said, "The stupidest thing is a helmet law, the point of which is to protect a brain that is functioning so poorly it's not even trying to prevent the enhancing of the skull it's in." But helmet laws for kids, who may not have considered their skulls as deeply as Jerry did, aren't so dumb. That's upholding to a new study in a publication from the Chocrane Collaboration, which is an international organization that cooperates health care research. The review looked at five studies of kids bike-helmet laws. One big 10 year study in California found that bike-related panchromatic brain injury in kids dropped more than 18 percent after the state's bike helmet law was enacted. A Canadian study looked at almost 10,000 bike related optical admissions and found a 45 percent drop in childhood head injuries in provinces that passed helmet laws. Provinces without helmet laws also saw a drop in the same period, but only half as much. And three other studies found that helmet laws do indeed persuade kids to wear their helmets, with paribus in compliance ranging from 45 to 84 percent.</t>
+    <t>Jerry Seinfeld once said, "The stupidest thing is a helmet law, the point of which is to protect a brain that is functioning so poorly it's not even trying to prevent the cracking of the skull it's in." But helmet laws for kids, who may not have considered their skulls as deeply as Jerry did, aren't so dumb. That's according to a new study in a publication from the Chocrane Collaboration, which is an international organization that evaluates health care research. The review looked at five studies of kids bike-helmet laws. One big 10 year study in California found that bike-related traumatic brain injury in kids dropped more than 18 percent after the state's bike helmet law was enacted. A Canadian study looked at almost 10,000 bike related hospital admissions and found a 45 percent drop in childhood head injuries in provinces that passed helmet laws. Provinces without helmet laws also saw a drop in the same period, but only half as much. And three other studies found that helmet laws do indeed persuade kids to wear their helmets, with increases in compliance ranging from 45 to 84 percent.</t>
   </si>
   <si>
     <t>#258 Foraging to Farming</t>
@@ -6200,7 +6200,7 @@
     <t>A team of __uricosurics/archeologists__ working in Jordan has made a discovery that represents a new chapter in the story of our __worshipers/ancestors'__ move from foraging to farming. The __steelworkers/researchers__ __converged/unearthed__ an ancient granary. The round, mud hut dates back more than 11,000 years. A raised floor was key for keeping grain dry and out of reach of hungry rats. But what makes the find so special is that the granary was built a __outed/thousand__ years before people ate domesticated crops. The report appears in the Proceedings of the National Academy of Sciences. The researchers found caches of wild barley and oats inside the structure. Such evidence of a dedicated food-storage edifice has never been recorded from the pre-pottery Neolithic age. The __maples/investigators__ say this selective cultivation and management of wild plants shows behaviors that led to agriculture. What's more, the granaries were built in-between houses and buildings used for food processing, which led to the establishment of more permanent settlements. By stockpiling a food surplus, our predecessors produced a new societal structure and curbed their wandering ways. Which then led to today's foraging for junk food in supermarket aisles.</t>
   </si>
   <si>
-    <t>A team of uricosurics working in Jordan has made a discovery that represents a new chapter in the story of our worshipers move from foraging to farming. The steelworkers converged an ancient granary. The round, mud hut dates back more than 11,000 years. A raised floor was key for keeping grain dry and out of reach of hungry rats. But what makes the find so special is that the granary was built a outed years before people ate domesticated crops. The report appears in the Proceedings of the National Academy of Sciences. The researchers found caches of wild barley and oats inside the structure. Such evidence of a dedicated food-storage edifice has never been recorded from the pre-pottery Neolithic age. The maples say this selective cultivation and management of wild plants shows behaviors that led to agriculture. What's more, the granaries were built in-between houses and buildings used for food processing, which led to the establishment of more permanent settlements. By stockpiling a food surplus, our predecessors produced a new societal structure and curbed their wandering ways. Which then led to today's foraging for junk food in supermarket aisles.</t>
+    <t>A team of archeologists working in Jordan has made a discovery that represents a new chapter in the story of our ancestors' move from foraging to farming. The researchers unearthed an ancient granary. The round, mud hut dates back more than 11,000 years. A raised floor was key for keeping grain dry and out of reach of hungry rats. But what makes the find so special is that the granary was built a thousand years before people ate domesticated crops. The report appears in the Proceedings of the National Academy of Sciences. The researchers found caches of wild barley and oats inside the structure. Such evidence of a dedicated food-storage edifice has never been recorded from the pre-pottery Neolithic age. The investigators say this selective cultivation and management of wild plants shows behaviors that led to agriculture. What's more, the granaries were built in-between houses and buildings used for food processing, which led to the establishment of more permanent settlements. By stockpiling a food surplus, our predecessors produced a new societal structure and curbed their wandering ways. Which then led to today's foraging for junk food in supermarket aisles.</t>
   </si>
   <si>
     <t>#259 Space Hazard</t>
@@ -6209,7 +6209,7 @@
     <t>There are many occupational hazards in space travel. But Russian researchers have discovered a new one: meaner bacteria. Scientists __oped/launched__ __tanneries/colonies__ of bacilli and E. coli into space and found they undergo significant changes. And not good ones either. The bacteria became much more aggressive and started to eat space ship components. That's because they began to produce unusual enzymes, probably because of exposure to cosmic radiation and the lack of gravitation. The study on board the Mir and Photon 2 __sayings/spaceships__ found that the changes occur even during short flights of 10 to 14 days. The bacteria change size and shape and their DNA changes too. Some genes that are dormant on earth switch on, __proofing/producing__ the enzymes. The researchers think that it's also likely that the mutant bacteria could pose greater threats to astronauts, who already suffer from immune system __products/problems__ in space. But there's one piece of good news: when the bacteria return to earth the aggressive traits vanish.</t>
   </si>
   <si>
-    <t>There are many occupational hazards in space travel. But Russian researchers have discovered a new one: meaner bacteria. Scientists oped tanneries of bacilli and E. coli into space and found they undergo significant changes. And not good ones either. The bacteria became much more aggressive and started to eat space ship components. That's because they began to produce unusual enzymes, probably because of exposure to cosmic radiation and the lack of gravitation. The study on board the Mir and Photon 2 sayings found that the changes occur even during short flights of 10 to 14 days. The bacteria change size and shape and their DNA changes too. Some genes that are dormant on earth switch on, proofing the enzymes. The researchers think that it's also likely that the mutant bacteria could pose greater threats to astronauts, who already suffer from immune system products in space. But there's one piece of good news: when the bacteria return to earth the aggressive traits vanish.</t>
+    <t>There are many occupational hazards in space travel. But Russian researchers have discovered a new one: meaner bacteria. Scientists launched colonies of bacilli and E. coli into space and found they undergo significant changes. And not good ones either. The bacteria became much more aggressive and started to eat space ship components. That's because they began to produce unusual enzymes, probably because of exposure to cosmic radiation and the lack of gravitation. The study on board the Mir and Photon 2 spaceships found that the changes occur even during short flights of 10 to 14 days. The bacteria change size and shape and their DNA changes too. Some genes that are dormant on earth switch on, producing the enzymes. The researchers think that it's also likely that the mutant bacteria could pose greater threats to astronauts, who already suffer from immune system problems in space. But there's one piece of good news: when the bacteria return to earth the aggressive traits vanish.</t>
   </si>
   <si>
     <t>#260 Urban Birds</t>
@@ -6218,7 +6218,7 @@
     <t>Animals that live in the city are usually less wary of humans than their rural counterparts. Most people think the boldness comes from experience: since the __poetry/majority__ of humans are rather harmless, the critters learn to go about their business without fear. But the truth turns out to be far more interesting, at least for Australian swans. Turns out the city birds are genetically __sediment/different__ from their country counterparts. Australian __realtors/researchers__ looked at two groups of swans. One population lived on a pond in the center of Melbourne. The second hung out just 30 kilometers away in a more bucolic setting, surrounded by far fewer humans. The researchers measured what they call each bird's "flight initiation distance": basically, how close could a human get before the swan would just fly away? "We found that the flight initiation distance for the swans at the urban __violent/environment__ was only 13 meters, and on average at the non-urban environment it was 96 meters. So that's like an 83 meter difference, a really big __nonresidents/difference__ in how wary these swans are at the two habitats." Victoria University ecologist Wouter van Dongen. The researchers also took blood samples from some of the swans to analyze their DNA. And almost 90 percent of urban swans had the same variant of a gene for dopamine transport, while just 60 percent of rural birds had that version. And those swans were less wary of humans than were the swans with the rarer genotypes. Dopamine influences a lot of brain function, so the gene __elucidation/variation__ could be behind the difference in swan attitudes. The study is in the journal BMC Evolutionary Biology. Since swans can easily fly wherever they want, the researchers think that the bolder birds don't mind setting up shop in the city, while the more timid swans prefer the quieter country life. And that's something that wildlife managers should keep in mind. "With release programs, often you breed up a small population of whatever animal and then you release them into the wild…and so one potential application of our research is to select individuals that are better able to cope with human disturbance, those that are less wary of humans, and release them into those areas that are more likely to experience human disturbance."</t>
   </si>
   <si>
-    <t>Animals that live in the city are usually less wary of humans than their rural counterparts. Most people think the boldness comes from experience: since the poetry of humans are rather harmless, the critters learn to go about their business without fear. But the truth turns out to be far more interesting, at least for Australian swans. Turns out the city birds are genetically sediment from their country counterparts. Australian realtors looked at two groups of swans. One population lived on a pond in the center of Melbourne. The second hung out just 30 kilometers away in a more bucolic setting, surrounded by far fewer humans. The researchers measured what they call each bird's "flight initiation distance": basically, how close could a human get before the swan would just fly away? "We found that the flight initiation distance for the swans at the urban violent was only 13 meters, and on average at the non-urban environment it was 96 meters. So that's like an 83 meter difference, a really big nonresidents in how wary these swans are at the two habitats." Victoria University ecologist Wouter van Dongen. The researchers also took blood samples from some of the swans to analyze their DNA. And almost 90 percent of urban swans had the same variant of a gene for dopamine transport, while just 60 percent of rural birds had that version. And those swans were less wary of humans than were the swans with the rarer genotypes. Dopamine influences a lot of brain function, so the gene elucidation could be behind the difference in swan attitudes. The study is in the journal BMC Evolutionary Biology. Since swans can easily fly wherever they want, the researchers think that the bolder birds don't mind setting up shop in the city, while the more timid swans prefer the quieter country life. And that's something that wildlife managers should keep in mind. "With release programs, often you breed up a small population of whatever animal and then you release them into the wild…and so one potential application of our research is to select individuals that are better able to cope with human disturbance, those that are less wary of humans, and release them into those areas that are more likely to experience human disturbance."</t>
+    <t>Animals that live in the city are usually less wary of humans than their rural counterparts. Most people think the boldness comes from experience: since the majority of humans are rather harmless, the critters learn to go about their business without fear. But the truth turns out to be far more interesting, at least for Australian swans. Turns out the city birds are genetically different from their country counterparts. Australian researchers looked at two groups of swans. One population lived on a pond in the center of Melbourne. The second hung out just 30 kilometers away in a more bucolic setting, surrounded by far fewer humans. The researchers measured what they call each bird's "flight initiation distance": basically, how close could a human get before the swan would just fly away? "We found that the flight initiation distance for the swans at the urban environment was only 13 meters, and on average at the non-urban environment it was 96 meters. So that's like an 83 meter difference, a really big difference in how wary these swans are at the two habitats." Victoria University ecologist Wouter van Dongen. The researchers also took blood samples from some of the swans to analyze their DNA. And almost 90 percent of urban swans had the same variant of a gene for dopamine transport, while just 60 percent of rural birds had that version. And those swans were less wary of humans than were the swans with the rarer genotypes. Dopamine influences a lot of brain function, so the gene variation could be behind the difference in swan attitudes. The study is in the journal BMC Evolutionary Biology. Since swans can easily fly wherever they want, the researchers think that the bolder birds don't mind setting up shop in the city, while the more timid swans prefer the quieter country life. And that's something that wildlife managers should keep in mind. "With release programs, often you breed up a small population of whatever animal and then you release them into the wild…and so one potential application of our research is to select individuals that are better able to cope with human disturbance, those that are less wary of humans, and release them into those areas that are more likely to experience human disturbance."</t>
   </si>
   <si>
     <t>#261 Election</t>
@@ -6227,7 +6227,7 @@
     <t>On election day, where do you vote? If it's in a church, you might be inclined to vote more __competently/conservatively__ than if you cast your ballot at a school or __obstinate/government__ building. That's __exporting/according__ to research published in the International Journal for the Psychology of Religion. And the effect seems to hold, whether you're Christian, Muslim or agnostic, progressive, independent or conservative. The study found that when random people were surveyed in front of a church, they gave more __dozily/socially__ and politically conservative responses than people surveyed while standing in front of a government building. The shift in people's attitudes, the researchers suggest, was likely a result of visual priming—meaning that people who could see the religious __consisting/building__ were, consciously or not, getting cues that influenced their response. The surveys were conducted in Europe, so it's possible American voters might react differently. But the survey included subjects from more than 30 __khakis/countries__ to try to minimize a particular national bias. So before you cast your vote this election year, think about whether your view is influencing your views.</t>
   </si>
   <si>
-    <t>On election day, where do you vote? If it's in a church, you might be inclined to vote more competently than if you cast your ballot at a school or obstinate building. That's exporting to research published in the International Journal for the Psychology of Religion. And the effect seems to hold, whether you're Christian, Muslim or agnostic, progressive, independent or conservative. The study found that when random people were surveyed in front of a church, they gave more dozily and politically conservative responses than people surveyed while standing in front of a government building. The shift in people's attitudes, the researchers suggest, was likely a result of visual priming—meaning that people who could see the religious consisting were, consciously or not, getting cues that influenced their response. The surveys were conducted in Europe, so it's possible American voters might react differently. But the survey included subjects from more than 30 khakis to try to minimize a particular national bias. So before you cast your vote this election year, think about whether your view is influencing your views.</t>
+    <t>On election day, where do you vote? If it's in a church, you might be inclined to vote more conservatively than if you cast your ballot at a school or government building. That's according to research published in the International Journal for the Psychology of Religion. And the effect seems to hold, whether you're Christian, Muslim or agnostic, progressive, independent or conservative. The study found that when random people were surveyed in front of a church, they gave more socially and politically conservative responses than people surveyed while standing in front of a government building. The shift in people's attitudes, the researchers suggest, was likely a result of visual priming—meaning that people who could see the religious building were, consciously or not, getting cues that influenced their response. The surveys were conducted in Europe, so it's possible American voters might react differently. But the survey included subjects from more than 30 countries to try to minimize a particular national bias. So before you cast your vote this election year, think about whether your view is influencing your views.</t>
   </si>
   <si>
     <t>#262 Dog Coat</t>
@@ -6236,7 +6236,7 @@
     <t>You can't judge a book by its cover. But you can judge a dog by its coat. You can even read right through to its genes. Because a study in the August 27th online issue of Science shows that just three key genes govern the length and texture of dog fur. Domestic dogs come in a stunning variety of shapes and sizes, and __emirate/different__ breeds wear different coats. They can have short hair or long hair, or fur that's straight, wavy, curly, wiry or smooth. To find the genes __satiable/responsible__ for this furry rainbow, scientists scanned the DNA of a __outed/thousand__ individual dogs from 80 different breeds. And they found that every coat's appearance boils down to three simple traits: length, curl and texture. And that each of these traits is controlled by just one gene. So, a long-haired Golden retriever has one variant of a gene called FGF5, whereas a short-haired lab has another. By mixing and __alerting/matching__ variants of these three genes, you get __businessmen/everything__ from a curly-haired poodle to a wire-haired Scottie with bushy eyebrows and a droopy mustache. Which is probably more than you'll ever need to know about the hair of the dog that bit you.</t>
   </si>
   <si>
-    <t>You can't judge a book by its cover. But you can judge a dog by its coat. You can even read right through to its genes. Because a study in the August 27th online issue of Science shows that just three key genes govern the length and texture of dog fur. Domestic dogs come in a stunning variety of shapes and sizes, and emirate breeds wear different coats. They can have short hair or long hair, or fur that's straight, wavy, curly, wiry or smooth. To find the genes satiable for this furry rainbow, scientists scanned the DNA of a outed individual dogs from 80 different breeds. And they found that every coat's appearance boils down to three simple traits: length, curl and texture. And that each of these traits is controlled by just one gene. So, a long-haired Golden retriever has one variant of a gene called FGF5, whereas a short-haired lab has another. By mixing and alerting variants of these three genes, you get businessmen from a curly-haired poodle to a wire-haired Scottie with bushy eyebrows and a droopy mustache. Which is probably more than you'll ever need to know about the hair of the dog that bit you.</t>
+    <t>You can't judge a book by its cover. But you can judge a dog by its coat. You can even read right through to its genes. Because a study in the August 27th online issue of Science shows that just three key genes govern the length and texture of dog fur. Domestic dogs come in a stunning variety of shapes and sizes, and different breeds wear different coats. They can have short hair or long hair, or fur that's straight, wavy, curly, wiry or smooth. To find the genes responsible for this furry rainbow, scientists scanned the DNA of a thousand individual dogs from 80 different breeds. And they found that every coat's appearance boils down to three simple traits: length, curl and texture. And that each of these traits is controlled by just one gene. So, a long-haired Golden retriever has one variant of a gene called FGF5, whereas a short-haired lab has another. By mixing and matching variants of these three genes, you get everything from a curly-haired poodle to a wire-haired Scottie with bushy eyebrows and a droopy mustache. Which is probably more than you'll ever need to know about the hair of the dog that bit you.</t>
   </si>
   <si>
     <t>#263 Climate and Insect</t>
@@ -6245,7 +6245,7 @@
     <t>A direct effect on human health related to climate change is the likely increase in __fearless/infectious__ diseases transmitted by insects or through contaminated water. In the March 25th issue of The New England Journal of Medicine, infectious disease researcher Emily Shuman points out that insects are more active at higher temperatures and broaden their range. Altered weather patterns bring drought to some areas, flooding to others and a higher likelihood of water contamination to both. The World Health Organization __winds/predicts__ a 3 to 5 percent increase in the population at risk for malaria with a temperature increase of 2 to 3 degrees Celsius. And two degrees is our best-case scenario right now. The WHO also sees 10 percent more __fetal/diarrheal__ diseases related to unclean water by 2030 due to climate change. Shuman urges the development of warning systems to spot disease __outtakes/outbreaks__ early, along with continued research into treatments and vaccines, which, she writes, "will go a long way in preventing human __faggoting/suffering__ that could otherwise occur as a result of climate change."</t>
   </si>
   <si>
-    <t>A direct effect on human health related to climate change is the likely increase in fearless diseases transmitted by insects or through contaminated water. In the March 25th issue of The New England Journal of Medicine, infectious disease researcher Emily Shuman points out that insects are more active at higher temperatures and broaden their range. Altered weather patterns bring drought to some areas, flooding to others and a higher likelihood of water contamination to both. The World Health Organization winds a 3 to 5 percent increase in the population at risk for malaria with a temperature increase of 2 to 3 degrees Celsius. And two degrees is our best-case scenario right now. The WHO also sees 10 percent more fetal diseases related to unclean water by 2030 due to climate change. Shuman urges the development of warning systems to spot disease outtakes early, along with continued research into treatments and vaccines, which, she writes, "will go a long way in preventing human faggoting that could otherwise occur as a result of climate change."</t>
+    <t>A direct effect on human health related to climate change is the likely increase in infectious diseases transmitted by insects or through contaminated water. In the March 25th issue of The New England Journal of Medicine, infectious disease researcher Emily Shuman points out that insects are more active at higher temperatures and broaden their range. Altered weather patterns bring drought to some areas, flooding to others and a higher likelihood of water contamination to both. The World Health Organization predicts a 3 to 5 percent increase in the population at risk for malaria with a temperature increase of 2 to 3 degrees Celsius. And two degrees is our best-case scenario right now. The WHO also sees 10 percent more diarrheal diseases related to unclean water by 2030 due to climate change. Shuman urges the development of warning systems to spot disease outbreaks early, along with continued research into treatments and vaccines, which, she writes, "will go a long way in preventing human suffering that could otherwise occur as a result of climate change."</t>
   </si>
   <si>
     <t>#264 Psychological Sex</t>
@@ -6254,7 +6254,7 @@
     <t>Do psychological __offenders/conditions__ vary by sex? More boys are __horsed/diagnosed__ with autism, and more girls with depression. Scientists at the University of Rochester Medical Center want to understand any such sex differences. So the __timeservers/researchers__ studied smell and gender in nearly __dynastic/microscopic__ roundworms. What can we learn about our brains from tiny worms? Well, these creatures have a relatively simple and well-mapped nervous system. Some are male, and some are hermaphroditic. Scientists presented the worms with two scents. One smelled like buttery popcorn, another like green vegetables. Hermaphrodites mostly crawled towards buttery popcorn, while males preferred vegetables. Then scientists manipulated some of the hermaphroditic neurons to behave like they were male. And the newly male worms now crawled towards the green peppery smell. What does this tell us about male and female human brains? Well, not much yet. But what surprised researchers is that brain neurons present in both sexes—like those that register smell __pattern/preference__ —have different characteristics depending on the sex of the worm. This is a step on a path scientists hope will lead to greater understanding about our own sex differences and mental illness.</t>
   </si>
   <si>
-    <t>Do psychological offenders vary by sex? More boys are horsed with autism, and more girls with depression. Scientists at the University of Rochester Medical Center want to understand any such sex differences. So the timeservers studied smell and gender in nearly dynastic roundworms. What can we learn about our brains from tiny worms? Well, these creatures have a relatively simple and well-mapped nervous system. Some are male, and some are hermaphroditic. Scientists presented the worms with two scents. One smelled like buttery popcorn, another like green vegetables. Hermaphrodites mostly crawled towards buttery popcorn, while males preferred vegetables. Then scientists manipulated some of the hermaphroditic neurons to behave like they were male. And the newly male worms now crawled towards the green peppery smell. What does this tell us about male and female human brains? Well, not much yet. But what surprised researchers is that brain neurons present in both sexes—like those that register smell pattern —have different characteristics depending on the sex of the worm. This is a step on a path scientists hope will lead to greater understanding about our own sex differences and mental illness.</t>
+    <t>Do psychological conditions vary by sex? More boys are diagnosed with autism, and more girls with depression. Scientists at the University of Rochester Medical Center want to understand any such sex differences. So the researchers studied smell and gender in nearly microscopic roundworms. What can we learn about our brains from tiny worms? Well, these creatures have a relatively simple and well-mapped nervous system. Some are male, and some are hermaphroditic. Scientists presented the worms with two scents. One smelled like buttery popcorn, another like green vegetables. Hermaphrodites mostly crawled towards buttery popcorn, while males preferred vegetables. Then scientists manipulated some of the hermaphroditic neurons to behave like they were male. And the newly male worms now crawled towards the green peppery smell. What does this tell us about male and female human brains? Well, not much yet. But what surprised researchers is that brain neurons present in both sexes—like those that register smell preference —have different characteristics depending on the sex of the worm. This is a step on a path scientists hope will lead to greater understanding about our own sex differences and mental illness.</t>
   </si>
   <si>
     <t>#265 Ethanol</t>
@@ -6263,7 +6263,7 @@
     <t>For those interested in preserving the environment, this week brings sobering news about ethanol. This fuel, distilled from plants like corn and switchgrass, has been widely touted as an eco-friendly, clean-burning __bursitis/alternative__ to gasoline. But a study published this week in the journal Environmental Science and __serology/Technology__ suggests that replacing our current gas-guzzlers with vehicles that burn ethanol would __irrationally/actually__ increase pollution and damage human health. Stanford __semifinalist/scientist__ Mark Jacobson used a computer model to predict air quality in the year 2020, when ethanol-powered cars are expected to be widely available in the US. His simulation showed, among other things, that cars that burn a blend of 85 percent ethanol will significantly increase ozone, a prime ingredient in smog. So in a world where the cars run on switchgrass juice, more people will get asthma, more people will be hospitalized with respiratory distress, and more people will die from __debriefing/breathing__ in ozone than if we'd kept on driving our __halflowered/gas-powered__ clunkers. At least according to Jacobons. So if you want to celebrate Earth Day this weekend, raise a glass of bubbly to our beautiful planet. Just don't share any with your gas tank.</t>
   </si>
   <si>
-    <t>For those interested in preserving the environment, this week brings sobering news about ethanol. This fuel, distilled from plants like corn and switchgrass, has been widely touted as an eco-friendly, clean-burning bursitis to gasoline. But a study published this week in the journal Environmental Science and serology suggests that replacing our current gas-guzzlers with vehicles that burn ethanol would irrationally increase pollution and damage human health. Stanford semifinalist Mark Jacobson used a computer model to predict air quality in the year 2020, when ethanol-powered cars are expected to be widely available in the US. His simulation showed, among other things, that cars that burn a blend of 85 percent ethanol will significantly increase ozone, a prime ingredient in smog. So in a world where the cars run on switchgrass juice, more people will get asthma, more people will be hospitalized with respiratory distress, and more people will die from debriefing in ozone than if we'd kept on driving our halflowered clunkers. At least according to Jacobons. So if you want to celebrate Earth Day this weekend, raise a glass of bubbly to our beautiful planet. Just don't share any with your gas tank.</t>
+    <t>For those interested in preserving the environment, this week brings sobering news about ethanol. This fuel, distilled from plants like corn and switchgrass, has been widely touted as an eco-friendly, clean-burning alternative to gasoline. But a study published this week in the journal Environmental Science and Technology suggests that replacing our current gas-guzzlers with vehicles that burn ethanol would actually increase pollution and damage human health. Stanford scientist Mark Jacobson used a computer model to predict air quality in the year 2020, when ethanol-powered cars are expected to be widely available in the US. His simulation showed, among other things, that cars that burn a blend of 85 percent ethanol will significantly increase ozone, a prime ingredient in smog. So in a world where the cars run on switchgrass juice, more people will get asthma, more people will be hospitalized with respiratory distress, and more people will die from breathing in ozone than if we'd kept on driving our gas-powered clunkers. At least according to Jacobons. So if you want to celebrate Earth Day this weekend, raise a glass of bubbly to our beautiful planet. Just don't share any with your gas tank.</t>
   </si>
   <si>
     <t>#266 Meteor Showers</t>
@@ -6272,7 +6272,7 @@
     <t>If you woke up this morning and the newspaper headline __gleamed/screamed__ Meteor Headed for Earth, you'd think: That's not good. And you'd __meteorology/probably__ be right. But __rites/sometimes__ a little cosmic bombardment can be just what the doctor ordered. In a study published online in the journal Nature Geoscience, researchers in Sweden say that 470 million years ago, meteor showers might have boosted our biodiversity. The scientists were studying rocks from China and Scandinavia. And they were looking for two things. First, they were counting the number of different clam-like species they could find. Second, they were searching for __penitence/chemicals__ that were carried here by meteorites—extraterrestrial chromite, stuff like that. They found that a huge burst of diversification coincides exactly with a time when meteors a mile wide were raining down on the planet. But wait. Didn't an asteroid wipe out the dinosaurs? Well, yes, but without all those earlier impacts promoting diversity, maybe there wouldn't have been any __manifolds/dinosaurs__ in the first place. And if a meteor hadn't then slammed the dinos, mammals like us might never have made the scene. So when it comes to space rocks, one man's ceiling is another man's flora…and fauna.</t>
   </si>
   <si>
-    <t>If you woke up this morning and the newspaper headline gleamed Meteor Headed for Earth, you'd think: That's not good. And you'd meteorology be right. But rites a little cosmic bombardment can be just what the doctor ordered. In a study published online in the journal Nature Geoscience, researchers in Sweden say that 470 million years ago, meteor showers might have boosted our biodiversity. The scientists were studying rocks from China and Scandinavia. And they were looking for two things. First, they were counting the number of different clam-like species they could find. Second, they were searching for penitence that were carried here by meteorites—extraterrestrial chromite, stuff like that. They found that a huge burst of diversification coincides exactly with a time when meteors a mile wide were raining down on the planet. But wait. Didn't an asteroid wipe out the dinosaurs? Well, yes, but without all those earlier impacts promoting diversity, maybe there wouldn't have been any manifolds in the first place. And if a meteor hadn't then slammed the dinos, mammals like us might never have made the scene. So when it comes to space rocks, one man's ceiling is another man's flora…and fauna.</t>
+    <t>If you woke up this morning and the newspaper headline screamed Meteor Headed for Earth, you'd think: That's not good. And you'd probably be right. But sometimes a little cosmic bombardment can be just what the doctor ordered. In a study published online in the journal Nature Geoscience, researchers in Sweden say that 470 million years ago, meteor showers might have boosted our biodiversity. The scientists were studying rocks from China and Scandinavia. And they were looking for two things. First, they were counting the number of different clam-like species they could find. Second, they were searching for chemicals that were carried here by meteorites—extraterrestrial chromite, stuff like that. They found that a huge burst of diversification coincides exactly with a time when meteors a mile wide were raining down on the planet. But wait. Didn't an asteroid wipe out the dinosaurs? Well, yes, but without all those earlier impacts promoting diversity, maybe there wouldn't have been any dinosaurs in the first place. And if a meteor hadn't then slammed the dinos, mammals like us might never have made the scene. So when it comes to space rocks, one man's ceiling is another man's flora…and fauna.</t>
   </si>
   <si>
     <t>#267 Nightmare</t>
@@ -6281,7 +6281,7 @@
     <t>How __concealment/frequent__ are __customizes/nightmares__ for toddlers, and what causes them? Those are questions researchers at the University of Montreal hoped to answer. They asked parents of about a __loudest/thousand__ children to estimate the occurrence of their child's nightmares from age two and a half through age six. The parents were also __sheltered/questioned__ about their child's disposition. First, it turns out that nightmares aren't so frequent. About a third of the parents reported no nightmares at all. And then there's the second result. Kids who were called "difficult" as early as 5 months were more likely to suffer from nightmares as toddlers. And the ones who at a year and a half were more anxious, more likely to cry, and more difficult to calm down were also more likely to have bad dreams. The study authors say this means children may be, well, like little adults. It's already well established that adults tend to express __spires/real-live__ stress and emotional problems as nightmares. The researchers suggest that focusing on the kids' day-time issues, and on parenting techniques, may help banish __lifetime/night-time__ demons.</t>
   </si>
   <si>
-    <t>How concealment are customizes for toddlers, and what causes them? Those are questions researchers at the University of Montreal hoped to answer. They asked parents of about a loudest children to estimate the occurrence of their child's nightmares from age two and a half through age six. The parents were also sheltered about their child's disposition. First, it turns out that nightmares aren't so frequent. About a third of the parents reported no nightmares at all. And then there's the second result. Kids who were called "difficult" as early as 5 months were more likely to suffer from nightmares as toddlers. And the ones who at a year and a half were more anxious, more likely to cry, and more difficult to calm down were also more likely to have bad dreams. The study authors say this means children may be, well, like little adults. It's already well established that adults tend to express spires stress and emotional problems as nightmares. The researchers suggest that focusing on the kids' day-time issues, and on parenting techniques, may help banish lifetime demons.</t>
+    <t>How frequent are nightmares for toddlers, and what causes them? Those are questions researchers at the University of Montreal hoped to answer. They asked parents of about a thousand children to estimate the occurrence of their child's nightmares from age two and a half through age six. The parents were also questioned about their child's disposition. First, it turns out that nightmares aren't so frequent. About a third of the parents reported no nightmares at all. And then there's the second result. Kids who were called "difficult" as early as 5 months were more likely to suffer from nightmares as toddlers. And the ones who at a year and a half were more anxious, more likely to cry, and more difficult to calm down were also more likely to have bad dreams. The study authors say this means children may be, well, like little adults. It's already well established that adults tend to express real-live stress and emotional problems as nightmares. The researchers suggest that focusing on the kids' day-time issues, and on parenting techniques, may help banish night-time demons.</t>
   </si>
   <si>
     <t>#268 Face to Face</t>
@@ -6290,7 +6290,7 @@
     <t>Any __unhealthful/successful__ business person can tell you about the __sauces/importance__ of "face time"—actually sitting down with clients, coworkers, maybe even competitors. But there may be even more to this whole __forgave/face-to-face__ business than meets the eye — or exactly as much as meets the eye. Because a new study from Tufts University suggests that the success of a corporation rests squarely on the face of its CEO. The researchers took photos of 50 CEOs from the highest and lowest ranked Fortune 1000 companies. And they showed these pictures to a group of undergrads. They asked the students to rate each face on whether its owner looked competent, dominant, likeable, mature or trustworthy. What they found is that the students' impressions tracked with company profits. The more __countable/powerful__ and leaderlike the CEO appeared, the more successful the corporation — even though the CEOs were all pretty much __diplomate/middle-aged__ white guys in ties. The study, which will appear in the February issue of __urological/Psychological__ Science, does not say whether profitable companies tend to promote people who look like leaders or whether successful CEOs grow to look the part. Either way, looks like a company's financial about-face can actually be about face.</t>
   </si>
   <si>
-    <t>Any unhealthful business person can tell you about the sauces of "face time"—actually sitting down with clients, coworkers, maybe even competitors. But there may be even more to this whole forgave business than meets the eye — or exactly as much as meets the eye. Because a new study from Tufts University suggests that the success of a corporation rests squarely on the face of its CEO. The researchers took photos of 50 CEOs from the highest and lowest ranked Fortune 1000 companies. And they showed these pictures to a group of undergrads. They asked the students to rate each face on whether its owner looked competent, dominant, likeable, mature or trustworthy. What they found is that the students' impressions tracked with company profits. The more countable and leaderlike the CEO appeared, the more successful the corporation — even though the CEOs were all pretty much diplomate white guys in ties. The study, which will appear in the February issue of urological Science, does not say whether profitable companies tend to promote people who look like leaders or whether successful CEOs grow to look the part. Either way, looks like a company's financial about-face can actually be about face.</t>
+    <t>Any successful business person can tell you about the importance of "face time"—actually sitting down with clients, coworkers, maybe even competitors. But there may be even more to this whole face-to-face business than meets the eye — or exactly as much as meets the eye. Because a new study from Tufts University suggests that the success of a corporation rests squarely on the face of its CEO. The researchers took photos of 50 CEOs from the highest and lowest ranked Fortune 1000 companies. And they showed these pictures to a group of undergrads. They asked the students to rate each face on whether its owner looked competent, dominant, likeable, mature or trustworthy. What they found is that the students' impressions tracked with company profits. The more powerful and leaderlike the CEO appeared, the more successful the corporation — even though the CEOs were all pretty much middle-aged white guys in ties. The study, which will appear in the February issue of Psychological Science, does not say whether profitable companies tend to promote people who look like leaders or whether successful CEOs grow to look the part. Either way, looks like a company's financial about-face can actually be about face.</t>
   </si>
   <si>
     <t>#269 New Way to Slenderize</t>
@@ -6299,7 +6299,7 @@
     <t>If you're like me, somewhere in your closet, or maybe in a drawer, you __family/probably__ have a pair of pants you hope to someday fit into. Again. But staying on a diet and finding time to exercise—it's no walk in the park. But wait! Before you swear off the spaghetti, scientists at the State __confraternity/University__ of New York in Stony Brook have stumbled onto a new way to slenderize. They found that mice that spend 15 minutes a day standing on a __strikebreaking/vibrating__ platform are leaner than mice who just stand still. Their results appear in the current online edition of the __leanness/Proceedings__ of the __optional/National__ Academy of Sciences. All the animals in the __pessimist/experiment__ were allowed to eat their fill. After 15 weeks, the shaken mice didn't actually weigh any less. But compared to the mice who hung out on a stationary platform, they had about 30 percent less fat around their middles. The SUNY scientists think that the jiggling kept fat cells from forming. Whether it would do the same for people, you never know. And here you thought New Yorkers were lean and mean because they're always in a hurry rushing here and there. Maybe it's because they spend so much time standing on vibrating subway platforms, waiting for the uptown express.</t>
   </si>
   <si>
-    <t>If you're like me, somewhere in your closet, or maybe in a drawer, you family have a pair of pants you hope to someday fit into. Again. But staying on a diet and finding time to exercise—it's no walk in the park. But wait! Before you swear off the spaghetti, scientists at the State confraternity of New York in Stony Brook have stumbled onto a new way to slenderize. They found that mice that spend 15 minutes a day standing on a strikebreaking platform are leaner than mice who just stand still. Their results appear in the current online edition of the leanness of the optional Academy of Sciences. All the animals in the pessimist were allowed to eat their fill. After 15 weeks, the shaken mice didn't actually weigh any less. But compared to the mice who hung out on a stationary platform, they had about 30 percent less fat around their middles. The SUNY scientists think that the jiggling kept fat cells from forming. Whether it would do the same for people, you never know. And here you thought New Yorkers were lean and mean because they're always in a hurry rushing here and there. Maybe it's because they spend so much time standing on vibrating subway platforms, waiting for the uptown express.</t>
+    <t>If you're like me, somewhere in your closet, or maybe in a drawer, you probably have a pair of pants you hope to someday fit into. Again. But staying on a diet and finding time to exercise—it's no walk in the park. But wait! Before you swear off the spaghetti, scientists at the State University of New York in Stony Brook have stumbled onto a new way to slenderize. They found that mice that spend 15 minutes a day standing on a vibrating platform are leaner than mice who just stand still. Their results appear in the current online edition of the Proceedings of the National Academy of Sciences. All the animals in the experiment were allowed to eat their fill. After 15 weeks, the shaken mice didn't actually weigh any less. But compared to the mice who hung out on a stationary platform, they had about 30 percent less fat around their middles. The SUNY scientists think that the jiggling kept fat cells from forming. Whether it would do the same for people, you never know. And here you thought New Yorkers were lean and mean because they're always in a hurry rushing here and there. Maybe it's because they spend so much time standing on vibrating subway platforms, waiting for the uptown express.</t>
   </si>
   <si>
     <t>#270 Tattoo</t>
@@ -6308,7 +6308,7 @@
     <t>Thinking about getting a new tattoo? Maybe a nice 3-D double helix or an I-heart-Higgs Bosons. Well, you might wind up getting some mycobacteria with your body art. The Centers for Disease Control and __Rewritten/Prevention__ has turned up about two dozen cases of this __possession/infection__ from contaminated tattoo ink. Last January, public health officials in western New York state __report/launched__ an investigation after a tattoo __smeariest/recipient__ reported a persistent rash--itchy red bumps all over his new tat. A skin sample tested positive for Mycobacterium chelonae, a microbe common in tap water. A list of the tattoo artist's clients turned up another 19 cases of the rash, including 14 __sponge/confirmed__ infections with the same bug. The tattoo parlor itself was clean, no bacteria in the water supply. But a bottle of premixed gray ink turned up positive. This gray wash, which is used to give tats a shaded, 3-D quality, was most likely contaminated during its manufacture and has since been recalled. But not before a handful of additional cases cropped up in elsewhere around the country. So if you're really itching to express yourself, a tattoo might indeed be just what the doctor ordered.</t>
   </si>
   <si>
-    <t>Thinking about getting a new tattoo? Maybe a nice 3-D double helix or an I-heart-Higgs Bosons. Well, you might wind up getting some mycobacteria with your body art. The Centers for Disease Control and Rewritten has turned up about two dozen cases of this possession from contaminated tattoo ink. Last January, public health officials in western New York state report an investigation after a tattoo smeariest reported a persistent rash--itchy red bumps all over his new tat. A skin sample tested positive for Mycobacterium chelonae, a microbe common in tap water. A list of the tattoo artist's clients turned up another 19 cases of the rash, including 14 sponge infections with the same bug. The tattoo parlor itself was clean, no bacteria in the water supply. But a bottle of premixed gray ink turned up positive. This gray wash, which is used to give tats a shaded, 3-D quality, was most likely contaminated during its manufacture and has since been recalled. But not before a handful of additional cases cropped up in elsewhere around the country. So if you're really itching to express yourself, a tattoo might indeed be just what the doctor ordered.</t>
+    <t>Thinking about getting a new tattoo? Maybe a nice 3-D double helix or an I-heart-Higgs Bosons. Well, you might wind up getting some mycobacteria with your body art. The Centers for Disease Control and Prevention has turned up about two dozen cases of this infection from contaminated tattoo ink. Last January, public health officials in western New York state launched an investigation after a tattoo recipient reported a persistent rash--itchy red bumps all over his new tat. A skin sample tested positive for Mycobacterium chelonae, a microbe common in tap water. A list of the tattoo artist's clients turned up another 19 cases of the rash, including 14 confirmed infections with the same bug. The tattoo parlor itself was clean, no bacteria in the water supply. But a bottle of premixed gray ink turned up positive. This gray wash, which is used to give tats a shaded, 3-D quality, was most likely contaminated during its manufacture and has since been recalled. But not before a handful of additional cases cropped up in elsewhere around the country. So if you're really itching to express yourself, a tattoo might indeed be just what the doctor ordered.</t>
   </si>
   <si>
     <t>#271 Garlic</t>
@@ -6317,7 +6317,7 @@
     <t>Various studies have suggested that eating garlic can be good for you. It's been credited with __woodworking/lowering__ blood pressure, protecting against heart disease, preventing blood clots, even fighting off colds. Now researchers from the University of Alabama at Birmingham think they have a better idea how garlic might work its medicinal magic. The Alabama team exposed red blood cells to the juices pressed from a standard, supermarket-issue clove of garlic. And they found that the __sheepfold/garlic-soaked__ cells started giving off __sidemen/hydrogen__ sulfide, which is the gas that gives rotten eggs their delightful bouquet. Ok, I know you're probably __midden/thinking__ that smelling like sewage seems even more odious than reeking of garlic. But on a molecular level, a pinch of hydrogen sulfide can be just what the doctor ordered. Because hydrogen sulfide serves as a chemical messenger that helps relax blood vessels and increase blood flow. Which could explain some of garlic's cardiovascular benefits. Of course more studies are needed to show whether a clove a day really does keep the doctor away. In the meantime, enjoy your garlic bread. And don't worry about the garlic breath. Just think what the insides of your arteries must smell like.</t>
   </si>
   <si>
-    <t>Various studies have suggested that eating garlic can be good for you. It's been credited with woodworking blood pressure, protecting against heart disease, preventing blood clots, even fighting off colds. Now researchers from the University of Alabama at Birmingham think they have a better idea how garlic might work its medicinal magic. The Alabama team exposed red blood cells to the juices pressed from a standard, supermarket-issue clove of garlic. And they found that the sheepfold cells started giving off sidemen sulfide, which is the gas that gives rotten eggs their delightful bouquet. Ok, I know you're probably midden that smelling like sewage seems even more odious than reeking of garlic. But on a molecular level, a pinch of hydrogen sulfide can be just what the doctor ordered. Because hydrogen sulfide serves as a chemical messenger that helps relax blood vessels and increase blood flow. Which could explain some of garlic's cardiovascular benefits. Of course more studies are needed to show whether a clove a day really does keep the doctor away. In the meantime, enjoy your garlic bread. And don't worry about the garlic breath. Just think what the insides of your arteries must smell like.</t>
+    <t>Various studies have suggested that eating garlic can be good for you. It's been credited with lowering blood pressure, protecting against heart disease, preventing blood clots, even fighting off colds. Now researchers from the University of Alabama at Birmingham think they have a better idea how garlic might work its medicinal magic. The Alabama team exposed red blood cells to the juices pressed from a standard, supermarket-issue clove of garlic. And they found that the garlic-soaked cells started giving off hydrogen sulfide, which is the gas that gives rotten eggs their delightful bouquet. Ok, I know you're probably thinking that smelling like sewage seems even more odious than reeking of garlic. But on a molecular level, a pinch of hydrogen sulfide can be just what the doctor ordered. Because hydrogen sulfide serves as a chemical messenger that helps relax blood vessels and increase blood flow. Which could explain some of garlic's cardiovascular benefits. Of course more studies are needed to show whether a clove a day really does keep the doctor away. In the meantime, enjoy your garlic bread. And don't worry about the garlic breath. Just think what the insides of your arteries must smell like.</t>
   </si>
   <si>
     <t>#272 HIW</t>
@@ -6326,7 +6326,7 @@
     <t>Sometimes it pays to look like a pile of poop. At least if you're a tasty __midwinter/caterpillar__ trying to avoid getting eaten by hungry birds. Because a study in the journal Science shows that even young chicks tend to overlook __villains/caterpillars__ disguised as dung. Animals have come up with some pretty clever tricks for keeping __cadets/themselves__ off a predator's dinner plate. Some use camouflage, __backing/adopting__ colors and patterns that help them blend into the environment. Others masquerade as something inedible, like bird __pulses/droppings__ or twigs. But scientists got to wondering whether the two approaches are really so different. Maybe critters dressed as twigs also "blend in" so that predators just don't see them. To find out, scientists presented some twiggy-looking caterpillars to two sets of hand-reared chicks. They found that baby birds that had never seen sticks before gobbled those bad boys right up. But chicks who were shown real twigs first took much longer to peck at the mimics, and did so more __plenary/gingerly__ than their naïve friends. That means the birds could see the caterpillars, but were fooled by the costume, at least temporarily. Which, for a caterpillar on a leaf in the wild, could mean the difference between eating and being eaten.</t>
   </si>
   <si>
-    <t>Sometimes it pays to look like a pile of poop. At least if you're a tasty midwinter trying to avoid getting eaten by hungry birds. Because a study in the journal Science shows that even young chicks tend to overlook villains disguised as dung. Animals have come up with some pretty clever tricks for keeping cadets off a predator's dinner plate. Some use camouflage, backing colors and patterns that help them blend into the environment. Others masquerade as something inedible, like bird pulses or twigs. But scientists got to wondering whether the two approaches are really so different. Maybe critters dressed as twigs also "blend in" so that predators just don't see them. To find out, scientists presented some twiggy-looking caterpillars to two sets of hand-reared chicks. They found that baby birds that had never seen sticks before gobbled those bad boys right up. But chicks who were shown real twigs first took much longer to peck at the mimics, and did so more plenary than their naïve friends. That means the birds could see the caterpillars, but were fooled by the costume, at least temporarily. Which, for a caterpillar on a leaf in the wild, could mean the difference between eating and being eaten.</t>
+    <t>Sometimes it pays to look like a pile of poop. At least if you're a tasty caterpillar trying to avoid getting eaten by hungry birds. Because a study in the journal Science shows that even young chicks tend to overlook caterpillars disguised as dung. Animals have come up with some pretty clever tricks for keeping themselves off a predator's dinner plate. Some use camouflage, adopting colors and patterns that help them blend into the environment. Others masquerade as something inedible, like bird droppings or twigs. But scientists got to wondering whether the two approaches are really so different. Maybe critters dressed as twigs also "blend in" so that predators just don't see them. To find out, scientists presented some twiggy-looking caterpillars to two sets of hand-reared chicks. They found that baby birds that had never seen sticks before gobbled those bad boys right up. But chicks who were shown real twigs first took much longer to peck at the mimics, and did so more gingerly than their naïve friends. That means the birds could see the caterpillars, but were fooled by the costume, at least temporarily. Which, for a caterpillar on a leaf in the wild, could mean the difference between eating and being eaten.</t>
   </si>
   <si>
     <t>#273 Location</t>
@@ -6335,7 +6335,7 @@
     <t>Location, location, location. We all know it's true of real estate. But it may also apply to the ballot box. Because a team of American __cheeseburgers/researchers__ has found that where people vote affects how they vote. The scientists looked at results from the 2000 general election. In Arizona that year, the ballot included an initiative to raise state taxes to support education. What they found is that people who __chuckled/happened__ to be voting in a school __persevering/building__ were more likely to vote for the __pleural/proposal__ than people who voted at a firehouse or a church. Their results appear in the June 23rd issue of the Proceedings of the National Academy of Sciences. And same thing happened in the lab. Subjects were shown a series of images, some of which pertained to schools. Later on, in what they were told was an unrelated experiment, they were asked to vote on funding for education. Folks who'd looked at lockers were more likely to vote yes. Whether voting in a church might affect where people stand on gay __towheaded/marriage__ or stem cell research remains to be seen. But it's __watchfully/probably__ a good thing that more people don't cast ballots in diners—might make it impossible to get rid of all that political pork.</t>
   </si>
   <si>
-    <t>Location, location, location. We all know it's true of real estate. But it may also apply to the ballot box. Because a team of American cheeseburgers has found that where people vote affects how they vote. The scientists looked at results from the 2000 general election. In Arizona that year, the ballot included an initiative to raise state taxes to support education. What they found is that people who chuckled to be voting in a school persevering were more likely to vote for the pleural than people who voted at a firehouse or a church. Their results appear in the June 23rd issue of the Proceedings of the National Academy of Sciences. And same thing happened in the lab. Subjects were shown a series of images, some of which pertained to schools. Later on, in what they were told was an unrelated experiment, they were asked to vote on funding for education. Folks who'd looked at lockers were more likely to vote yes. Whether voting in a church might affect where people stand on gay towheaded or stem cell research remains to be seen. But it's watchfully a good thing that more people don't cast ballots in diners—might make it impossible to get rid of all that political pork.</t>
+    <t>Location, location, location. We all know it's true of real estate. But it may also apply to the ballot box. Because a team of American researchers has found that where people vote affects how they vote. The scientists looked at results from the 2000 general election. In Arizona that year, the ballot included an initiative to raise state taxes to support education. What they found is that people who happened to be voting in a school building were more likely to vote for the proposal than people who voted at a firehouse or a church. Their results appear in the June 23rd issue of the Proceedings of the National Academy of Sciences. And same thing happened in the lab. Subjects were shown a series of images, some of which pertained to schools. Later on, in what they were told was an unrelated experiment, they were asked to vote on funding for education. Folks who'd looked at lockers were more likely to vote yes. Whether voting in a church might affect where people stand on gay marriage or stem cell research remains to be seen. But it's probably a good thing that more people don't cast ballots in diners—might make it impossible to get rid of all that political pork.</t>
   </si>
   <si>
     <t>#274 HIW</t>
@@ -6344,7 +6344,7 @@
     <t>Londoners love their fish. And according to a new study, in the early 13th Century they suddenly started importing it from as far away as the Arctic near Norway. The research is in the journal Antiquity. About the year 1000, sea fishing __mercerised/increased__ significantly in northern Europe. To see how that increase influenced urban growth, researchers looked at 95 __polymerization/excavation__ sites in London. Which included about 3,000 bones from cod fish. Cod are decapitated before being dried for transport. So finding heads meant the fish were local. And the researchers found that as fish heads appear to __puppeteers/decrease__ in the early 1200s, fish tails dramatically increased—a sign of importation. __manipulation/Examination__ of the chemical isotopes in the tails matched those for fish in waters far to the north, __monstrosity/probably__ off Norway close to the Arctic, more evidence of import. The __licences/scientists__ do not know if the rapid switch from local to imported cod happened because local fish weren't as plentiful as the population increased, or if the market became flooded with dried imports from the north. But these fish tails tell a story of London becoming a growing economic center, and part of a globalizing fish trade.</t>
   </si>
   <si>
-    <t>Londoners love their fish. And according to a new study, in the early 13th Century they suddenly started importing it from as far away as the Arctic near Norway. The research is in the journal Antiquity. About the year 1000, sea fishing mercerised significantly in northern Europe. To see how that increase influenced urban growth, researchers looked at 95 polymerization sites in London. Which included about 3,000 bones from cod fish. Cod are decapitated before being dried for transport. So finding heads meant the fish were local. And the researchers found that as fish heads appear to puppeteers in the early 1200s, fish tails dramatically increased—a sign of importation. manipulation of the chemical isotopes in the tails matched those for fish in waters far to the north, monstrosity off Norway close to the Arctic, more evidence of import. The licences do not know if the rapid switch from local to imported cod happened because local fish weren't as plentiful as the population increased, or if the market became flooded with dried imports from the north. But these fish tails tell a story of London becoming a growing economic center, and part of a globalizing fish trade.</t>
+    <t>Londoners love their fish. And according to a new study, in the early 13th Century they suddenly started importing it from as far away as the Arctic near Norway. The research is in the journal Antiquity. About the year 1000, sea fishing increased significantly in northern Europe. To see how that increase influenced urban growth, researchers looked at 95 excavation sites in London. Which included about 3,000 bones from cod fish. Cod are decapitated before being dried for transport. So finding heads meant the fish were local. And the researchers found that as fish heads appear to decrease in the early 1200s, fish tails dramatically increased—a sign of importation. Examination of the chemical isotopes in the tails matched those for fish in waters far to the north, probably off Norway close to the Arctic, more evidence of import. The scientists do not know if the rapid switch from local to imported cod happened because local fish weren't as plentiful as the population increased, or if the market became flooded with dried imports from the north. But these fish tails tell a story of London becoming a growing economic center, and part of a globalizing fish trade.</t>
   </si>
   <si>
     <t>#275 HIW</t>
@@ -6353,7 +6353,7 @@
     <t>New parents can act pretty strangely—for example, they often have an obsessive interest in what comes out of their baby's bottoms. Now __sheepherders/researchers__ at Stanford University join them in their diaper diving to explore when and how __sniffier/bacteria__ colonize the human gut. Adults harbor complex __dictatorial/microbial__ __renders/ecosystems__ within their GI tracts. These bacteria help digest food and contribute to a healthy immune system. But when a baby is born, its intestine is devoid of bacterial inhabitants. Within days, however, a __sustained/cavalcade__ of microbes set up shop, establishing a vibrant intestinal community whose residents soon outnumber the baby's own cells. The researchers found that the early months were chaotic…with established species disappearing and new ones taking their place. But by the time the babies were 12 months old, each harbored a dynamic but unique __brethren/collection__ of intestinal fauna. A set of fraternal twins had the most similar bugs, which suggests that genetics may have __adopting/something__ to do with which bacteria stick around. Next they'll look at how formula versus breast milk affects a baby's intestinal ecosystem. With so many questions left to explore, the researchers will no doubt be mining diapers for some time to come.</t>
   </si>
   <si>
-    <t>New parents can act pretty strangely—for example, they often have an obsessive interest in what comes out of their baby's bottoms. Now sheepherders at Stanford University join them in their diaper diving to explore when and how sniffier colonize the human gut. Adults harbor complex dictatorial renders within their GI tracts. These bacteria help digest food and contribute to a healthy immune system. But when a baby is born, its intestine is devoid of bacterial inhabitants. Within days, however, a sustained of microbes set up shop, establishing a vibrant intestinal community whose residents soon outnumber the baby's own cells. The researchers found that the early months were chaotic…with established species disappearing and new ones taking their place. But by the time the babies were 12 months old, each harbored a dynamic but unique brethren of intestinal fauna. A set of fraternal twins had the most similar bugs, which suggests that genetics may have adopting to do with which bacteria stick around. Next they'll look at how formula versus breast milk affects a baby's intestinal ecosystem. With so many questions left to explore, the researchers will no doubt be mining diapers for some time to come.</t>
+    <t>New parents can act pretty strangely—for example, they often have an obsessive interest in what comes out of their baby's bottoms. Now researchers at Stanford University join them in their diaper diving to explore when and how bacteria colonize the human gut. Adults harbor complex microbial ecosystems within their GI tracts. These bacteria help digest food and contribute to a healthy immune system. But when a baby is born, its intestine is devoid of bacterial inhabitants. Within days, however, a cavalcade of microbes set up shop, establishing a vibrant intestinal community whose residents soon outnumber the baby's own cells. The researchers found that the early months were chaotic…with established species disappearing and new ones taking their place. But by the time the babies were 12 months old, each harbored a dynamic but unique collection of intestinal fauna. A set of fraternal twins had the most similar bugs, which suggests that genetics may have something to do with which bacteria stick around. Next they'll look at how formula versus breast milk affects a baby's intestinal ecosystem. With so many questions left to explore, the researchers will no doubt be mining diapers for some time to come.</t>
   </si>
   <si>
     <t>#276 HIW</t>
@@ -6362,7 +6362,7 @@
     <t>What do airport baggage screeners, __occlusions/students__ and basketball players have in common? They all need a good night's sleep. A study presented this week at the Annual Meeting of the Associated __extramarital/Professional__ Sleep Societies suggests basketballers who get some extra z's are more likely to score in a game. (Stanford University) researchers __inhabited/monitored__ members of the __suits/school's__ men's basketball team during two weeks of regular sleep cycles and then two weeks with extra sleep. With extra sleep the athletes reported increased energy; faster sprint times; and better __vivo/free-throw__ shooting. Another study found that college students who pull all-nighters to prepare for tests tend to have lower grade point averages than those who get regular sleep. And 2nd and 3rd graders with sleep disorders are more likely to receive bad grades in math, reading and writing, according to a study from Chappaqua Public Schools in New York. But it gets even worse. A researcher from Brigham, Women's Hospital in Boston found that airport baggage __readers/screeners__ who didn't get enough sleep made more errors in __dusting/searching__ for unusual items that might be a threat. So you see, you need to catch z's to catch bad guys.</t>
   </si>
   <si>
-    <t>What do airport baggage screeners, occlusions and basketball players have in common? They all need a good night's sleep. A study presented this week at the Annual Meeting of the Associated extramarital Sleep Societies suggests basketballers who get some extra z's are more likely to score in a game. (Stanford University) researchers inhabited members of the suits men's basketball team during two weeks of regular sleep cycles and then two weeks with extra sleep. With extra sleep the athletes reported increased energy; faster sprint times; and better vivo shooting. Another study found that college students who pull all-nighters to prepare for tests tend to have lower grade point averages than those who get regular sleep. And 2nd and 3rd graders with sleep disorders are more likely to receive bad grades in math, reading and writing, according to a study from Chappaqua Public Schools in New York. But it gets even worse. A researcher from Brigham, Women's Hospital in Boston found that airport baggage readers who didn't get enough sleep made more errors in dusting for unusual items that might be a threat. So you see, you need to catch z's to catch bad guys.</t>
+    <t>What do airport baggage screeners, students and basketball players have in common? They all need a good night's sleep. A study presented this week at the Annual Meeting of the Associated Professional Sleep Societies suggests basketballers who get some extra z's are more likely to score in a game. (Stanford University) researchers monitored members of the school's men's basketball team during two weeks of regular sleep cycles and then two weeks with extra sleep. With extra sleep the athletes reported increased energy; faster sprint times; and better free-throw shooting. Another study found that college students who pull all-nighters to prepare for tests tend to have lower grade point averages than those who get regular sleep. And 2nd and 3rd graders with sleep disorders are more likely to receive bad grades in math, reading and writing, according to a study from Chappaqua Public Schools in New York. But it gets even worse. A researcher from Brigham, Women's Hospital in Boston found that airport baggage screeners who didn't get enough sleep made more errors in searching for unusual items that might be a threat. So you see, you need to catch z's to catch bad guys.</t>
   </si>
   <si>
     <t>#277 HIW</t>
@@ -6371,7 +6371,7 @@
     <t>A hungry fish can kill prey with a quick bite. That is, of course, if its prey hasn't already died of fright. Take tasty dragonflies. The mere __petitions/presence__ of predators—even caged ones—is enough to scare __legalize/dragonflies__ to death, __distorting/according__ to a study in the journal Ecology. Researchers collected wild dragonfly larvae, and placed them in tanks with fish or insect predators. The larvae could see and smell their hunters—but were kept safe by underwater cages. After two months, the researchers took a head count—and found that dragonfly larvae sharing quarters with their killers were two to four times as likely to die off, __rend/compared__ to __repulse/counterparts__ living in predator-free waters. And they had slimmer chances of surviving metamorphosis, too. The authors suggest a couple reasons why. First, prey tend to make fewer forays for snacks when __binnacles/predators__ are lurking around, so they may not be as nutritionally fit. And previous studies have shown that the presence of predators ups stress levels in prey, weakening their immune systems and making them more vulnerable to disease—and death. As if being eaten wasn't enough to worry about, looks can kill too.</t>
   </si>
   <si>
-    <t>A hungry fish can kill prey with a quick bite. That is, of course, if its prey hasn't already died of fright. Take tasty dragonflies. The mere petitions of predators—even caged ones—is enough to scare legalize to death, distorting to a study in the journal Ecology. Researchers collected wild dragonfly larvae, and placed them in tanks with fish or insect predators. The larvae could see and smell their hunters—but were kept safe by underwater cages. After two months, the researchers took a head count—and found that dragonfly larvae sharing quarters with their killers were two to four times as likely to die off, rend to repulse living in predator-free waters. And they had slimmer chances of surviving metamorphosis, too. The authors suggest a couple reasons why. First, prey tend to make fewer forays for snacks when binnacles are lurking around, so they may not be as nutritionally fit. And previous studies have shown that the presence of predators ups stress levels in prey, weakening their immune systems and making them more vulnerable to disease—and death. As if being eaten wasn't enough to worry about, looks can kill too.</t>
+    <t>A hungry fish can kill prey with a quick bite. That is, of course, if its prey hasn't already died of fright. Take tasty dragonflies. The mere presence of predators—even caged ones—is enough to scare dragonflies to death, according to a study in the journal Ecology. Researchers collected wild dragonfly larvae, and placed them in tanks with fish or insect predators. The larvae could see and smell their hunters—but were kept safe by underwater cages. After two months, the researchers took a head count—and found that dragonfly larvae sharing quarters with their killers were two to four times as likely to die off, compared to counterparts living in predator-free waters. And they had slimmer chances of surviving metamorphosis, too. The authors suggest a couple reasons why. First, prey tend to make fewer forays for snacks when predators are lurking around, so they may not be as nutritionally fit. And previous studies have shown that the presence of predators ups stress levels in prey, weakening their immune systems and making them more vulnerable to disease—and death. As if being eaten wasn't enough to worry about, looks can kill too.</t>
   </si>
   <si>
     <t>#278 HIW</t>
@@ -6380,7 +6380,7 @@
     <t>Back on January 15th, US Airways Flight 1549 made that amazing water landing in the Hudson after both engines were taken out by Canada geese, which can weigh eight pounds each. Now scientists have used forensic __dioceses/techniques__ to clear local geese—the perpetrators were out-of-towners. The study appears June 8th in the journal Frontiers in Ecology and the Environment. Crash __aggregations/investigators__ sent feather samples from the plane's engines to the Smithsonian, which has a dedicated Feather Identification Lab. The researchers examined the feather's __leviathan/hydrogen__ isotopes, which include regular hydrogen atoms and __spiciness/hydrogens__ with additional neutrons. The isotope ratios tell you about the bird's diet. And that tells you where they dined. The analysis showed that the birds that hit the plane were much closer to geese migrating from Canada's Labrador region than the geese who live __shroud/year-round__ in New York. That info could be __urate/important__ for strategies to avoid future bird strikes. The usual techniques for keeping resident birds away from planes are still working—but we need new ones for strangers just passing through.</t>
   </si>
   <si>
-    <t>Back on January 15th, US Airways Flight 1549 made that amazing water landing in the Hudson after both engines were taken out by Canada geese, which can weigh eight pounds each. Now scientists have used forensic dioceses to clear local geese—the perpetrators were out-of-towners. The study appears June 8th in the journal Frontiers in Ecology and the Environment. Crash aggregations sent feather samples from the plane's engines to the Smithsonian, which has a dedicated Feather Identification Lab. The researchers examined the feather's leviathan isotopes, which include regular hydrogen atoms and spiciness with additional neutrons. The isotope ratios tell you about the bird's diet. And that tells you where they dined. The analysis showed that the birds that hit the plane were much closer to geese migrating from Canada's Labrador region than the geese who live shroud in New York. That info could be urate for strategies to avoid future bird strikes. The usual techniques for keeping resident birds away from planes are still working—but we need new ones for strangers just passing through.</t>
+    <t>Back on January 15th, US Airways Flight 1549 made that amazing water landing in the Hudson after both engines were taken out by Canada geese, which can weigh eight pounds each. Now scientists have used forensic techniques to clear local geese—the perpetrators were out-of-towners. The study appears June 8th in the journal Frontiers in Ecology and the Environment. Crash investigators sent feather samples from the plane's engines to the Smithsonian, which has a dedicated Feather Identification Lab. The researchers examined the feather's hydrogen isotopes, which include regular hydrogen atoms and hydrogens with additional neutrons. The isotope ratios tell you about the bird's diet. And that tells you where they dined. The analysis showed that the birds that hit the plane were much closer to geese migrating from Canada's Labrador region than the geese who live year-round in New York. That info could be important for strategies to avoid future bird strikes. The usual techniques for keeping resident birds away from planes are still working—but we need new ones for strangers just passing through.</t>
   </si>
   <si>
     <t>#279 HIW</t>
@@ -6389,7 +6389,7 @@
     <t>The Nobel Prize in __futility/chemistry__ goes to three men who __politicized/revolutionized__ molecular life science, Japan's Osamu Shimomura and Americans Martin Chalfie and Roger Tsien. They develop tools to light up and see individual __coffees/proteins__ inside living cells. These tiny molecular flashlights make it possible to study numerous events that take place in cells and whole organisms that were previously invisible—such as the development of nerve cells or the spread of cancer cells. In 1962 Shimomura, now __assiduousness/emeritus__ professor at the Marine Biological Laboratory at Woods Hole, discovered that jellyfish produce a green __insufficient/fluorescent__ protein, GFP, that glows when exposed to ultraviolet light. Some 30 years later, Columbia University's Chalfie showed that the GFP gene could be put into any organism. By making sure the fluorescent protein was expressed at the same time as other proteins of interest, researchers could literally light up events they want to follow. Then Tsien, at the University of California, San Diego, engineered fluorescent proteins in various colors. The multicolor palette enables researchers to follow __karakul/multiple__ biological processes at the same time.</t>
   </si>
   <si>
-    <t>The Nobel Prize in futility goes to three men who politicized molecular life science, Japan's Osamu Shimomura and Americans Martin Chalfie and Roger Tsien. They develop tools to light up and see individual coffees inside living cells. These tiny molecular flashlights make it possible to study numerous events that take place in cells and whole organisms that were previously invisible—such as the development of nerve cells or the spread of cancer cells. In 1962 Shimomura, now assiduousness professor at the Marine Biological Laboratory at Woods Hole, discovered that jellyfish produce a green insufficient protein, GFP, that glows when exposed to ultraviolet light. Some 30 years later, Columbia University's Chalfie showed that the GFP gene could be put into any organism. By making sure the fluorescent protein was expressed at the same time as other proteins of interest, researchers could literally light up events they want to follow. Then Tsien, at the University of California, San Diego, engineered fluorescent proteins in various colors. The multicolor palette enables researchers to follow karakul biological processes at the same time.</t>
+    <t>The Nobel Prize in chemistry goes to three men who revolutionized molecular life science, Japan's Osamu Shimomura and Americans Martin Chalfie and Roger Tsien. They develop tools to light up and see individual proteins inside living cells. These tiny molecular flashlights make it possible to study numerous events that take place in cells and whole organisms that were previously invisible—such as the development of nerve cells or the spread of cancer cells. In 1962 Shimomura, now emeritus professor at the Marine Biological Laboratory at Woods Hole, discovered that jellyfish produce a green fluorescent protein, GFP, that glows when exposed to ultraviolet light. Some 30 years later, Columbia University's Chalfie showed that the GFP gene could be put into any organism. By making sure the fluorescent protein was expressed at the same time as other proteins of interest, researchers could literally light up events they want to follow. Then Tsien, at the University of California, San Diego, engineered fluorescent proteins in various colors. The multicolor palette enables researchers to follow multiple biological processes at the same time.</t>
   </si>
   <si>
     <t>#280 HIW</t>
@@ -6398,7 +6398,7 @@
     <t>Real-time information about what's happening in our bodies at the cellular level could be crucial for fighting cancer and other life-threatening conditions. It would be incredibly helpful to know whether cancer drugs are __heeling/reaching__ their targets or whether toxins are disrupting DNA in healthy cells. Now scientists at M.I.T. have created carbon __revels/nanosensors__ that they say can help answer those questions. The research was published December 14th in the journal Nature Nanotechnology. The researchers wrapped carbon nanotube sensors in DNA, and the coated sensors have been shown to be safe for living cells. The __pantaloons/nanotubes__ emit infrared light. But that signal changes when cancer drugs or molecules that damage DNA bind with the sensor. By detecting the changes in signals, such as __acceptably/intensity__ and wavelength, the researchers have shown they can determine just what's happening to cells in real-time. So if the sensor were placed in the body, it could pick up, for example, even a __fool/molecule__ of hydrogen peroxide, which is toxic to DNA. Researchers say these nanotube-DNA sensors could monitor cellular activity over long periods of time. They might also be used in minimally invasive biopsy techniques, because cells would be __fingerprinting/transmitting__ information directly to the radiologist.</t>
   </si>
   <si>
-    <t>Real-time information about what's happening in our bodies at the cellular level could be crucial for fighting cancer and other life-threatening conditions. It would be incredibly helpful to know whether cancer drugs are heeling their targets or whether toxins are disrupting DNA in healthy cells. Now scientists at M.I.T. have created carbon revels that they say can help answer those questions. The research was published December 14th in the journal Nature Nanotechnology. The researchers wrapped carbon nanotube sensors in DNA, and the coated sensors have been shown to be safe for living cells. The pantaloons emit infrared light. But that signal changes when cancer drugs or molecules that damage DNA bind with the sensor. By detecting the changes in signals, such as acceptably and wavelength, the researchers have shown they can determine just what's happening to cells in real-time. So if the sensor were placed in the body, it could pick up, for example, even a fool of hydrogen peroxide, which is toxic to DNA. Researchers say these nanotube-DNA sensors could monitor cellular activity over long periods of time. They might also be used in minimally invasive biopsy techniques, because cells would be fingerprinting information directly to the radiologist.</t>
+    <t>Real-time information about what's happening in our bodies at the cellular level could be crucial for fighting cancer and other life-threatening conditions. It would be incredibly helpful to know whether cancer drugs are reaching their targets or whether toxins are disrupting DNA in healthy cells. Now scientists at M.I.T. have created carbon nanosensors that they say can help answer those questions. The research was published December 14th in the journal Nature Nanotechnology. The researchers wrapped carbon nanotube sensors in DNA, and the coated sensors have been shown to be safe for living cells. The nanotubes emit infrared light. But that signal changes when cancer drugs or molecules that damage DNA bind with the sensor. By detecting the changes in signals, such as intensity and wavelength, the researchers have shown they can determine just what's happening to cells in real-time. So if the sensor were placed in the body, it could pick up, for example, even a molecule of hydrogen peroxide, which is toxic to DNA. Researchers say these nanotube-DNA sensors could monitor cellular activity over long periods of time. They might also be used in minimally invasive biopsy techniques, because cells would be transmitting information directly to the radiologist.</t>
   </si>
   <si>
     <t>#281 Coal Mine</t>
@@ -6407,7 +6407,7 @@
     <t>A coal mine can degrade its local environment. But a fungus may __faculty/inadvertently__ help clean up the mine — with its own waste products. Researchers worked with a fungus called Stilbella aciculosa. As it makes spores, it also __juices/produces__ superoxide. That's a highly __putrefactive/reactive__ kind of oxygen. When the released superoxide bumps into the mineral manganese in the environment, it makes that mineral much more reactive itself. The pepped-up manganese then grabs and holds a variety of toxic metals and other substances that need to be cleaned up and taken out of coal mine drainage water. The research, led by Colleen Hansel of Harvard and the Woods Hole Oceanographic Institution, appears in the Proceedings of the National Academy of Sciences. It's been known that various __fierier/bacteria__ and fungi can help in environmental remediation. The new __controvert/research__ shows that production of the vital forms of manganese requires that the fungi and bacteria be actively producing superoxide. So creating conditions that encourage the organisms to make the superoxide could be the first step in a pathway by which they help manganese to literally do the dirty work. And make some toxic sites a lot cleaner.</t>
   </si>
   <si>
-    <t>A coal mine can degrade its local environment. But a fungus may faculty help clean up the mine — with its own waste products. Researchers worked with a fungus called Stilbella aciculosa. As it makes spores, it also juices superoxide. That's a highly putrefactive kind of oxygen. When the released superoxide bumps into the mineral manganese in the environment, it makes that mineral much more reactive itself. The pepped-up manganese then grabs and holds a variety of toxic metals and other substances that need to be cleaned up and taken out of coal mine drainage water. The research, led by Colleen Hansel of Harvard and the Woods Hole Oceanographic Institution, appears in the Proceedings of the National Academy of Sciences. It's been known that various fierier and fungi can help in environmental remediation. The new controvert shows that production of the vital forms of manganese requires that the fungi and bacteria be actively producing superoxide. So creating conditions that encourage the organisms to make the superoxide could be the first step in a pathway by which they help manganese to literally do the dirty work. And make some toxic sites a lot cleaner.</t>
+    <t>A coal mine can degrade its local environment. But a fungus may inadvertently help clean up the mine — with its own waste products. Researchers worked with a fungus called Stilbella aciculosa. As it makes spores, it also produces superoxide. That's a highly reactive kind of oxygen. When the released superoxide bumps into the mineral manganese in the environment, it makes that mineral much more reactive itself. The pepped-up manganese then grabs and holds a variety of toxic metals and other substances that need to be cleaned up and taken out of coal mine drainage water. The research, led by Colleen Hansel of Harvard and the Woods Hole Oceanographic Institution, appears in the Proceedings of the National Academy of Sciences. It's been known that various bacteria and fungi can help in environmental remediation. The new research shows that production of the vital forms of manganese requires that the fungi and bacteria be actively producing superoxide. So creating conditions that encourage the organisms to make the superoxide could be the first step in a pathway by which they help manganese to literally do the dirty work. And make some toxic sites a lot cleaner.</t>
   </si>
   <si>
     <t>#282 Big Bill</t>
@@ -6416,7 +6416,7 @@
     <t>The __pastes/toucan's__ long bill has long perplexed biologists. Darwin theorized that it attracted mates. Other suggested uses ranged from fruit peeling to territorial defense. But a report in the July 24th issue of the journal Science offers another __anticipation/explanation__ as to why one-third of the bird is all schnoz. The authors of the report say the toucan's bill is so big because it acts like a radiator __spanned/strapped__ to its face. When a toucan needs to cool down, its beak heats up. The immense surface area of the beak allows heat to quickly dissipate. In fact, the __mileages/scientists__ say, as a toucan lowers its body temperature in preparation for sleep, it can cool 10 degrees Celsius in just minutes. The scientists used __beheld/infrared__ thermography, the same kind of __geology/technology__ used in heat-sensing cameras, to observe toucans at different ambient temperatures. When outside temperatures rose, the bill also heated up, but the bird's core body temperature did not. The scientists speculate that other big-billed birds may regulate their body temperatures this way. Since birds don't sweat, having a handy heat __chaser/dissipater__ undoubtedly keeps their feathers from getting ruffled.</t>
   </si>
   <si>
-    <t>The pastes long bill has long perplexed biologists. Darwin theorized that it attracted mates. Other suggested uses ranged from fruit peeling to territorial defense. But a report in the July 24th issue of the journal Science offers another anticipation as to why one-third of the bird is all schnoz. The authors of the report say the toucan's bill is so big because it acts like a radiator spanned to its face. When a toucan needs to cool down, its beak heats up. The immense surface area of the beak allows heat to quickly dissipate. In fact, the mileages say, as a toucan lowers its body temperature in preparation for sleep, it can cool 10 degrees Celsius in just minutes. The scientists used beheld thermography, the same kind of geology used in heat-sensing cameras, to observe toucans at different ambient temperatures. When outside temperatures rose, the bill also heated up, but the bird's core body temperature did not. The scientists speculate that other big-billed birds may regulate their body temperatures this way. Since birds don't sweat, having a handy heat chaser undoubtedly keeps their feathers from getting ruffled.</t>
+    <t>The toucan's long bill has long perplexed biologists. Darwin theorized that it attracted mates. Other suggested uses ranged from fruit peeling to territorial defense. But a report in the July 24th issue of the journal Science offers another explanation as to why one-third of the bird is all schnoz. The authors of the report say the toucan's bill is so big because it acts like a radiator strapped to its face. When a toucan needs to cool down, its beak heats up. The immense surface area of the beak allows heat to quickly dissipate. In fact, the scientists say, as a toucan lowers its body temperature in preparation for sleep, it can cool 10 degrees Celsius in just minutes. The scientists used infrared thermography, the same kind of technology used in heat-sensing cameras, to observe toucans at different ambient temperatures. When outside temperatures rose, the bill also heated up, but the bird's core body temperature did not. The scientists speculate that other big-billed birds may regulate their body temperatures this way. Since birds don't sweat, having a handy heat dissipater undoubtedly keeps their feathers from getting ruffled.</t>
   </si>
   <si>
     <t>#283 Sargasso Sea</t>
@@ -6425,7 +6425,7 @@
     <t>Three years ago, genome pioneer Craig Venter sailed the Sargasso sea and __adjudged/returned__ with 1,800 species of microbes, including 150 never before seen. An impressive haul. But last week, scientists in New York __shroud/announced__ that if you want to discover new and interesting bugs, you need travel no further than your own forearm. The researchers, at the NYU School of Medicine, identified 182 species of bacteria, including a dozen new ones, in swabs taken from the arms of six healthy volunteers. Their study marks the first full-scale __western/expedition__ to catalog the biota that calls the human epidermis its home. The __bios/microbes__ that live in and on our bodies __bunker/outnumber__ our own cells 10 to 1. So they're an important part of our personal ecology. And it turns out the zoo of bacteria on one person's skin is very different from the zoo on someone else's. Almost three-quarters of the species identified were unique to an individual. And only four species were found on all six subjects. For the record, the __easterners/researchers__ took their samples from the subjects' __skulls/forearms__ because that way no one had to undress. So who knows what exotic life forms may be waiting for discovery just behind your knees.</t>
   </si>
   <si>
-    <t>Three years ago, genome pioneer Craig Venter sailed the Sargasso sea and adjudged with 1,800 species of microbes, including 150 never before seen. An impressive haul. But last week, scientists in New York shroud that if you want to discover new and interesting bugs, you need travel no further than your own forearm. The researchers, at the NYU School of Medicine, identified 182 species of bacteria, including a dozen new ones, in swabs taken from the arms of six healthy volunteers. Their study marks the first full-scale western to catalog the biota that calls the human epidermis its home. The bios that live in and on our bodies bunker our own cells 10 to 1. So they're an important part of our personal ecology. And it turns out the zoo of bacteria on one person's skin is very different from the zoo on someone else's. Almost three-quarters of the species identified were unique to an individual. And only four species were found on all six subjects. For the record, the easterners took their samples from the subjects' skulls because that way no one had to undress. So who knows what exotic life forms may be waiting for discovery just behind your knees.</t>
+    <t>Three years ago, genome pioneer Craig Venter sailed the Sargasso sea and returned with 1,800 species of microbes, including 150 never before seen. An impressive haul. But last week, scientists in New York announced that if you want to discover new and interesting bugs, you need travel no further than your own forearm. The researchers, at the NYU School of Medicine, identified 182 species of bacteria, including a dozen new ones, in swabs taken from the arms of six healthy volunteers. Their study marks the first full-scale expedition to catalog the biota that calls the human epidermis its home. The microbes that live in and on our bodies outnumber our own cells 10 to 1. So they're an important part of our personal ecology. And it turns out the zoo of bacteria on one person's skin is very different from the zoo on someone else's. Almost three-quarters of the species identified were unique to an individual. And only four species were found on all six subjects. For the record, the researchers took their samples from the subjects' forearms because that way no one had to undress. So who knows what exotic life forms may be waiting for discovery just behind your knees.</t>
   </si>
   <si>
     <t>#284 Volcano Eruption</t>
@@ -6434,7 +6434,7 @@
     <t>2002 was a tough year for the people who live along the shores of Lake Kivu in the __aromatic/Democratic__ Republic of the Congo. It started off with a bang, when the Nyiragongo volcano erupted in January. And it tailed off with a shudder, when a magnitude 6.2 earthquake struck the region in October. Both events devastated local communities—and their close timing struck some scientists as suspicious. "We were wondering if there could be a link—so, a causality—between those two major geological events." Christelle Wauthier, a geologist at Pennsylvania State University. From studying radar images of the ground taken before and after the January eruption, __frowzier/Wauthier__ knew that lava didn't just spew out of the volcano. It also wedged itself into cracks in the crust, forming what __haematologists/geologists__ call a dike. "So you can think of it as like a blade-shaped type of magma intrusion, moving from depth toward the surface. It's very fast, a few hours, a few days, and it can penetrate tens of kilometers of crust." Dikes are common in rift zones, like east Africa and Iceland, where tectonic forces are slowly ripping Earth's crust apart. And they're known to cause small __mermaids/earthquakes__ right when they happen. But Wauthier wondered if dikes might also be capable of triggering large earthquakes by pushing the ground apart and affecting nearby faults. "You will add more stress on a weakness surface, which is a fault. And so if you add enough stress on it, you can trigger failure on the fault." Now, Wauthier and her __potentialities/colleagues__ have used a model to show that the stress changes caused by the January dike event made the October earthquake much more likely to occur. The results are in the journal Geochemistry, Geophysics, Geosystems. This study marks the first time scientists have linked dike formation to large, damaging earthquakes, and Wauthier is looking back through history for more examples. She says __realtors/researchers__ will never be able to predict exactly when an earthquake might strike after a dike intrusion. But at least now, researchers and rift zone residents know they're not just in for bangs—they may also be in for shudders.</t>
   </si>
   <si>
-    <t>2002 was a tough year for the people who live along the shores of Lake Kivu in the aromatic Republic of the Congo. It started off with a bang, when the Nyiragongo volcano erupted in January. And it tailed off with a shudder, when a magnitude 6.2 earthquake struck the region in October. Both events devastated local communities—and their close timing struck some scientists as suspicious. "We were wondering if there could be a link—so, a causality—between those two major geological events." Christelle Wauthier, a geologist at Pennsylvania State University. From studying radar images of the ground taken before and after the January eruption, frowzier knew that lava didn't just spew out of the volcano. It also wedged itself into cracks in the crust, forming what haematologists call a dike. "So you can think of it as like a blade-shaped type of magma intrusion, moving from depth toward the surface. It's very fast, a few hours, a few days, and it can penetrate tens of kilometers of crust." Dikes are common in rift zones, like east Africa and Iceland, where tectonic forces are slowly ripping Earth's crust apart. And they're known to cause small mermaids right when they happen. But Wauthier wondered if dikes might also be capable of triggering large earthquakes by pushing the ground apart and affecting nearby faults. "You will add more stress on a weakness surface, which is a fault. And so if you add enough stress on it, you can trigger failure on the fault." Now, Wauthier and her potentialities have used a model to show that the stress changes caused by the January dike event made the October earthquake much more likely to occur. The results are in the journal Geochemistry, Geophysics, Geosystems. This study marks the first time scientists have linked dike formation to large, damaging earthquakes, and Wauthier is looking back through history for more examples. She says realtors will never be able to predict exactly when an earthquake might strike after a dike intrusion. But at least now, researchers and rift zone residents know they're not just in for bangs—they may also be in for shudders.</t>
+    <t>2002 was a tough year for the people who live along the shores of Lake Kivu in the Democratic Republic of the Congo. It started off with a bang, when the Nyiragongo volcano erupted in January. And it tailed off with a shudder, when a magnitude 6.2 earthquake struck the region in October. Both events devastated local communities—and their close timing struck some scientists as suspicious. "We were wondering if there could be a link—so, a causality—between those two major geological events." Christelle Wauthier, a geologist at Pennsylvania State University. From studying radar images of the ground taken before and after the January eruption, Wauthier knew that lava didn't just spew out of the volcano. It also wedged itself into cracks in the crust, forming what geologists call a dike. "So you can think of it as like a blade-shaped type of magma intrusion, moving from depth toward the surface. It's very fast, a few hours, a few days, and it can penetrate tens of kilometers of crust." Dikes are common in rift zones, like east Africa and Iceland, where tectonic forces are slowly ripping Earth's crust apart. And they're known to cause small earthquakes right when they happen. But Wauthier wondered if dikes might also be capable of triggering large earthquakes by pushing the ground apart and affecting nearby faults. "You will add more stress on a weakness surface, which is a fault. And so if you add enough stress on it, you can trigger failure on the fault." Now, Wauthier and her colleagues have used a model to show that the stress changes caused by the January dike event made the October earthquake much more likely to occur. The results are in the journal Geochemistry, Geophysics, Geosystems. This study marks the first time scientists have linked dike formation to large, damaging earthquakes, and Wauthier is looking back through history for more examples. She says researchers will never be able to predict exactly when an earthquake might strike after a dike intrusion. But at least now, researchers and rift zone residents know they're not just in for bangs—they may also be in for shudders.</t>
   </si>
   <si>
     <t>#285 Hippocampus</t>
@@ -6443,7 +6443,7 @@
     <t>You __bodily/probably__ __whatsoever/remember__ exactly what you were doing when you first heard the news on 9/11. That's because the brain has ways to file information so that things that happen at the same time are forever linked in our minds. Now a study published in the journal Neuron; says that newborn cells in a structure called the hippocampus help us remember concurrent events. The hippocampus is part of the brain that allows us to lay down new memories. And about ten years ago, scientists were __forthright/surprised__ to find that new neurons pop up in this region every day, even in adult animals and people. But what do these new cells do? Scientists turned to computer __boggling/modeling__ to help them find out. They put in what they knew about the behavior of these new cells, which start out like puppies that get totally excited over every little thing, and eventually mature into more discerning members of __endurable/neuronal__ society. And they found that the hyperactivity of these excitable young cells, which react with great gusto to everything that goes on, could help stamp memories with a sort of "time code" that indicates which things happened together. So if you still remember what you were eating when you dumped your loser boyfriend, you can thank your newborn neurons.</t>
   </si>
   <si>
-    <t>You bodily whatsoever exactly what you were doing when you first heard the news on 9/11. That's because the brain has ways to file information so that things that happen at the same time are forever linked in our minds. Now a study published in the journal Neuron; says that newborn cells in a structure called the hippocampus help us remember concurrent events. The hippocampus is part of the brain that allows us to lay down new memories. And about ten years ago, scientists were forthright to find that new neurons pop up in this region every day, even in adult animals and people. But what do these new cells do? Scientists turned to computer boggling to help them find out. They put in what they knew about the behavior of these new cells, which start out like puppies that get totally excited over every little thing, and eventually mature into more discerning members of endurable society. And they found that the hyperactivity of these excitable young cells, which react with great gusto to everything that goes on, could help stamp memories with a sort of "time code" that indicates which things happened together. So if you still remember what you were eating when you dumped your loser boyfriend, you can thank your newborn neurons.</t>
+    <t>You probably remember exactly what you were doing when you first heard the news on 9/11. That's because the brain has ways to file information so that things that happen at the same time are forever linked in our minds. Now a study published in the journal Neuron; says that newborn cells in a structure called the hippocampus help us remember concurrent events. The hippocampus is part of the brain that allows us to lay down new memories. And about ten years ago, scientists were surprised to find that new neurons pop up in this region every day, even in adult animals and people. But what do these new cells do? Scientists turned to computer modeling to help them find out. They put in what they knew about the behavior of these new cells, which start out like puppies that get totally excited over every little thing, and eventually mature into more discerning members of neuronal society. And they found that the hyperactivity of these excitable young cells, which react with great gusto to everything that goes on, could help stamp memories with a sort of "time code" that indicates which things happened together. So if you still remember what you were eating when you dumped your loser boyfriend, you can thank your newborn neurons.</t>
   </si>
   <si>
     <t>#286 HIV</t>
@@ -6452,7 +6452,7 @@
     <t>Germany's Harald zur Hausen and France's Luc Montagnier and Francoise Barre-Sinoussi share the 2008 Nobel Prize in Physiology or Medicine, awarded October 6th. Barre-Sinoussi and Montagnier discovered HIV. Shortly after reports in the early 1980s of a new immunodeficiency syndrome, researchers all over the world raced to find the cause. The two French scientists __dazzled/cultured__ cells from lymph nodes of patients. They first detected the enzyme reverse transcriptase, which meant that a retrovirus was active. Further searching turned up retroviral particles, which could kill white blood cells and which also reacted with antibodies from infected patients. These discoveries made __irreversible/possible__ unprecedented rapid development of blood screening techniques and of new antiviral therapies. Zur Hausen defied the medical __overconfident/establishment__ and postulated in the 1970s that cervical cancer was caused by the human __oculomotor/papilloma__ virus. He was able to isolate viral DNA in tumors. He also determined that there were multiple kinds of papilloma viruses, and that only some caused cancer. His discovery led to the development of a vaccine against cervical cancer.</t>
   </si>
   <si>
-    <t>Germany's Harald zur Hausen and France's Luc Montagnier and Francoise Barre-Sinoussi share the 2008 Nobel Prize in Physiology or Medicine, awarded October 6th. Barre-Sinoussi and Montagnier discovered HIV. Shortly after reports in the early 1980s of a new immunodeficiency syndrome, researchers all over the world raced to find the cause. The two French scientists dazzled cells from lymph nodes of patients. They first detected the enzyme reverse transcriptase, which meant that a retrovirus was active. Further searching turned up retroviral particles, which could kill white blood cells and which also reacted with antibodies from infected patients. These discoveries made irreversible unprecedented rapid development of blood screening techniques and of new antiviral therapies. Zur Hausen defied the medical overconfident and postulated in the 1970s that cervical cancer was caused by the human oculomotor virus. He was able to isolate viral DNA in tumors. He also determined that there were multiple kinds of papilloma viruses, and that only some caused cancer. His discovery led to the development of a vaccine against cervical cancer.</t>
+    <t>Germany's Harald zur Hausen and France's Luc Montagnier and Francoise Barre-Sinoussi share the 2008 Nobel Prize in Physiology or Medicine, awarded October 6th. Barre-Sinoussi and Montagnier discovered HIV. Shortly after reports in the early 1980s of a new immunodeficiency syndrome, researchers all over the world raced to find the cause. The two French scientists cultured cells from lymph nodes of patients. They first detected the enzyme reverse transcriptase, which meant that a retrovirus was active. Further searching turned up retroviral particles, which could kill white blood cells and which also reacted with antibodies from infected patients. These discoveries made possible unprecedented rapid development of blood screening techniques and of new antiviral therapies. Zur Hausen defied the medical establishment and postulated in the 1970s that cervical cancer was caused by the human papilloma virus. He was able to isolate viral DNA in tumors. He also determined that there were multiple kinds of papilloma viruses, and that only some caused cancer. His discovery led to the development of a vaccine against cervical cancer.</t>
   </si>
   <si>
     <t>#287 Seasonal Flu</t>
@@ -6461,7 +6461,7 @@
     <t>Seasonal flu __suggestibility/typically__ hits senior citizens harder than most other age groups. In fact, some 90 percent of __promenaded/flu-related__ deaths are estimated to occur in adults 65 and older. But with pandemic influenzas, like bird or swine flu, it's a different story. Take the 2009 H1N1 flu. In that outbreak, adults over 65 actually suffered the fewest infections of any age group. That anomaly __tens/suggests__ they might have some sort of built-in immunity. Now researchers say the seniors' secret may be in their spit. Researchers sampled saliva from 180 children, adult and elderly volunteers. Then they isolated __homebodies/proteins__ from the saliva, and tested how well the inhibitory proteins stuck to two strains of H9N2 bird flu. Turns out elderly men and women had __scientifically/significantly__ more such proteins that interfere with the flu virus—which researchers say could boost the seniors' resistance to bird flu. Those results appear in the Journal of Proteome Research. The next step, researchers say, is to develop an oral or nasal spray based on these proteins. Which might give people of all ages a chance to send the flu a lethal loogie.</t>
   </si>
   <si>
-    <t>Seasonal flu suggestibility hits senior citizens harder than most other age groups. In fact, some 90 percent of promenaded deaths are estimated to occur in adults 65 and older. But with pandemic influenzas, like bird or swine flu, it's a different story. Take the 2009 H1N1 flu. In that outbreak, adults over 65 actually suffered the fewest infections of any age group. That anomaly tens they might have some sort of built-in immunity. Now researchers say the seniors' secret may be in their spit. Researchers sampled saliva from 180 children, adult and elderly volunteers. Then they isolated homebodies from the saliva, and tested how well the inhibitory proteins stuck to two strains of H9N2 bird flu. Turns out elderly men and women had scientifically more such proteins that interfere with the flu virus—which researchers say could boost the seniors' resistance to bird flu. Those results appear in the Journal of Proteome Research. The next step, researchers say, is to develop an oral or nasal spray based on these proteins. Which might give people of all ages a chance to send the flu a lethal loogie.</t>
+    <t>Seasonal flu typically hits senior citizens harder than most other age groups. In fact, some 90 percent of flu-related deaths are estimated to occur in adults 65 and older. But with pandemic influenzas, like bird or swine flu, it's a different story. Take the 2009 H1N1 flu. In that outbreak, adults over 65 actually suffered the fewest infections of any age group. That anomaly suggests they might have some sort of built-in immunity. Now researchers say the seniors' secret may be in their spit. Researchers sampled saliva from 180 children, adult and elderly volunteers. Then they isolated proteins from the saliva, and tested how well the inhibitory proteins stuck to two strains of H9N2 bird flu. Turns out elderly men and women had significantly more such proteins that interfere with the flu virus—which researchers say could boost the seniors' resistance to bird flu. Those results appear in the Journal of Proteome Research. The next step, researchers say, is to develop an oral or nasal spray based on these proteins. Which might give people of all ages a chance to send the flu a lethal loogie.</t>
   </si>
   <si>
     <t>#288 Testing of Lie</t>
@@ -6470,7 +6470,7 @@
     <t>When we lie, our brains work hard to make sure we get the story right and come off as truthful. Law enforcement officials try to tap into that effort, for example with polygraphs, to find out if a suspect is telling the truth. But such stress tests are beatable and not admissible in court. Now comes a report that handwriting tests could be a competitor to the familiar, but unreliable lie detector. The study appears in the Journal of Applied __adjective/Cognitive__ Psychology. Researchers at Israel's Haifa University worked with 34 volunteers, who wrote truthful and false paragraphs on paper using a wireless __workaholic/electronic__ pen and a pressure sensitive tip. A computerized system measured pressure and stroke duration, both on the paper and in the air. Spatial measures, such as stroke length, height and width were also tracked. And the __itemise/scientists__ found significant differences in pressure and spatial measures in __intersubjective/deceptive__ statements compared with the truth. The investigators say they need to __vaccinate/validate__ this initial result and compare the technique with polygraphs and other lie detection tools. But perhaps in the future even a written claim of innocence could turn out to be a de facto confession.</t>
   </si>
   <si>
-    <t>When we lie, our brains work hard to make sure we get the story right and come off as truthful. Law enforcement officials try to tap into that effort, for example with polygraphs, to find out if a suspect is telling the truth. But such stress tests are beatable and not admissible in court. Now comes a report that handwriting tests could be a competitor to the familiar, but unreliable lie detector. The study appears in the Journal of Applied adjective Psychology. Researchers at Israel's Haifa University worked with 34 volunteers, who wrote truthful and false paragraphs on paper using a wireless workaholic pen and a pressure sensitive tip. A computerized system measured pressure and stroke duration, both on the paper and in the air. Spatial measures, such as stroke length, height and width were also tracked. And the itemise found significant differences in pressure and spatial measures in intersubjective statements compared with the truth. The investigators say they need to vaccinate this initial result and compare the technique with polygraphs and other lie detection tools. But perhaps in the future even a written claim of innocence could turn out to be a de facto confession.</t>
+    <t>When we lie, our brains work hard to make sure we get the story right and come off as truthful. Law enforcement officials try to tap into that effort, for example with polygraphs, to find out if a suspect is telling the truth. But such stress tests are beatable and not admissible in court. Now comes a report that handwriting tests could be a competitor to the familiar, but unreliable lie detector. The study appears in the Journal of Applied Cognitive Psychology. Researchers at Israel's Haifa University worked with 34 volunteers, who wrote truthful and false paragraphs on paper using a wireless electronic pen and a pressure sensitive tip. A computerized system measured pressure and stroke duration, both on the paper and in the air. Spatial measures, such as stroke length, height and width were also tracked. And the scientists found significant differences in pressure and spatial measures in deceptive statements compared with the truth. The investigators say they need to validate this initial result and compare the technique with polygraphs and other lie detection tools. But perhaps in the future even a written claim of innocence could turn out to be a de facto confession.</t>
   </si>
   <si>
     <t>#289 Sound Imitation</t>
@@ -6479,7 +6479,7 @@
     <t>Neil Young? No, that's Jimmy Fallon imitating Neil Young. Doing impressions can be a valuable skill. In fact, a bird called the __elevate/fork-tailed__ drongo makes a good living at it, in its home in Africa's __nappy/Kalahari__ Desert. The drongo can mimic the alarm calls of another bird. When that bird flees the __enacted/imagined__ danger, the drongo swoops in to take any food left behind. An animal __extinguishing/mimicking__ another animal is not rare. And targets can grow wise to the trick. The drongo's real talent is that it can do the warning calls of multiple species. Like how Jimmy Fallon can also do Van Morrison. Researchers __swallowed/followed__ 64 wild drongos for nearly 850 hours. Drongos do sound accurate alarms in response to actual predators. But when they spot a tempting meal in another bird's possession, they send out a false alarm. Here's one mimicking a pied babbler. Another a glossy starling's alarm. And here's a drongo mimicking a meerkat alarm. The researchers saw almost 700 drongo attempts to steal food. They __element/estimate__ that any one drongo might know up to 32 __coalitionist/different__ species' alarms. And stolen food accounted for nearly a quarter of their daily intake. The study is in the journal Science. Fool birds once? Shame on them. Fool birds multiple times? Success for the fork-tailed drongo.</t>
   </si>
   <si>
-    <t>Neil Young? No, that's Jimmy Fallon imitating Neil Young. Doing impressions can be a valuable skill. In fact, a bird called the elevate drongo makes a good living at it, in its home in Africa's nappy Desert. The drongo can mimic the alarm calls of another bird. When that bird flees the enacted danger, the drongo swoops in to take any food left behind. An animal extinguishing another animal is not rare. And targets can grow wise to the trick. The drongo's real talent is that it can do the warning calls of multiple species. Like how Jimmy Fallon can also do Van Morrison. Researchers swallowed 64 wild drongos for nearly 850 hours. Drongos do sound accurate alarms in response to actual predators. But when they spot a tempting meal in another bird's possession, they send out a false alarm. Here's one mimicking a pied babbler. Another a glossy starling's alarm. And here's a drongo mimicking a meerkat alarm. The researchers saw almost 700 drongo attempts to steal food. They element that any one drongo might know up to 32 coalitionist species' alarms. And stolen food accounted for nearly a quarter of their daily intake. The study is in the journal Science. Fool birds once? Shame on them. Fool birds multiple times? Success for the fork-tailed drongo.</t>
+    <t>Neil Young? No, that's Jimmy Fallon imitating Neil Young. Doing impressions can be a valuable skill. In fact, a bird called the fork-tailed drongo makes a good living at it, in its home in Africa's Kalahari Desert. The drongo can mimic the alarm calls of another bird. When that bird flees the imagined danger, the drongo swoops in to take any food left behind. An animal mimicking another animal is not rare. And targets can grow wise to the trick. The drongo's real talent is that it can do the warning calls of multiple species. Like how Jimmy Fallon can also do Van Morrison. Researchers followed 64 wild drongos for nearly 850 hours. Drongos do sound accurate alarms in response to actual predators. But when they spot a tempting meal in another bird's possession, they send out a false alarm. Here's one mimicking a pied babbler. Another a glossy starling's alarm. And here's a drongo mimicking a meerkat alarm. The researchers saw almost 700 drongo attempts to steal food. They estimate that any one drongo might know up to 32 different species' alarms. And stolen food accounted for nearly a quarter of their daily intake. The study is in the journal Science. Fool birds once? Shame on them. Fool birds multiple times? Success for the fork-tailed drongo.</t>
   </si>
   <si>
     <t>#290 Ladybug</t>
@@ -6488,7 +6488,7 @@
     <t>If you like a glass of wine with your pizza, you might be interested in the news from this week's __cytoskeleton/American__ Chemical Society meeting in Chicago. First the bad news: it seems that a growing number of winemakers find that their reds, whites and rosés taste a little like ladybugs. These cute little aphid-eaters are becoming quite a nuisance in vineyards across the country, where they accidentally get harvested with the grapes and stink up the resulting wine. Chemists at Iowa State University used a gas chromatograph and a panel of human __electors/sniffers__ to analyze the odor __crewed/produced__ by __virgins/hundreds__ of live ladybugs. They found the stench was made mostly by chemicals that smelled like roasted peanuts and green peppers. Which maybe nobody wants in a delicate Chablis. But there's good news about pizza. Chemists at the University of Maryland have figured out how to boost the antioxidant levels in pizza dough. Maybe that discovery will __utilize/catalyze__ a whole new generation of bad foods that are good for you: potato chips that clear your __conservancies/arteries__ or brownies that deliver insulin. Until then, at least we've got the antioxidant deep dish, which we can always wash down with a nice glass of ladybug merlot.</t>
   </si>
   <si>
-    <t>If you like a glass of wine with your pizza, you might be interested in the news from this week's cytoskeleton Chemical Society meeting in Chicago. First the bad news: it seems that a growing number of winemakers find that their reds, whites and rosés taste a little like ladybugs. These cute little aphid-eaters are becoming quite a nuisance in vineyards across the country, where they accidentally get harvested with the grapes and stink up the resulting wine. Chemists at Iowa State University used a gas chromatograph and a panel of human electors to analyze the odor crewed by virgins of live ladybugs. They found the stench was made mostly by chemicals that smelled like roasted peanuts and green peppers. Which maybe nobody wants in a delicate Chablis. But there's good news about pizza. Chemists at the University of Maryland have figured out how to boost the antioxidant levels in pizza dough. Maybe that discovery will utilize a whole new generation of bad foods that are good for you: potato chips that clear your conservancies or brownies that deliver insulin. Until then, at least we've got the antioxidant deep dish, which we can always wash down with a nice glass of ladybug merlot.</t>
+    <t>If you like a glass of wine with your pizza, you might be interested in the news from this week's American Chemical Society meeting in Chicago. First the bad news: it seems that a growing number of winemakers find that their reds, whites and rosés taste a little like ladybugs. These cute little aphid-eaters are becoming quite a nuisance in vineyards across the country, where they accidentally get harvested with the grapes and stink up the resulting wine. Chemists at Iowa State University used a gas chromatograph and a panel of human sniffers to analyze the odor produced by hundreds of live ladybugs. They found the stench was made mostly by chemicals that smelled like roasted peanuts and green peppers. Which maybe nobody wants in a delicate Chablis. But there's good news about pizza. Chemists at the University of Maryland have figured out how to boost the antioxidant levels in pizza dough. Maybe that discovery will catalyze a whole new generation of bad foods that are good for you: potato chips that clear your arteries or brownies that deliver insulin. Until then, at least we've got the antioxidant deep dish, which we can always wash down with a nice glass of ladybug merlot.</t>
   </si>
   <si>
     <t>#291 Making Mistakes</t>
@@ -6497,7 +6497,7 @@
     <t>Everyone makes mistakes, especially when it comes to entering numbers into a __sedater/calculator__ or spreadsheet. It's not such a big deal if you're __landing/tracking__ how much you spend on pizza. But if you're __unregistering/administering__ drugs in a hospital, such a slip can be deadly. Now a report in the Journal of the Royal Society Interface shows how devices can be programmed to catch at least some __safe/mistakes__ on the spot. Dosing a patient with 10 times too much medication is disturbingly common. One study suggests this error occurs in 1 percent of all hospital admissions. And though the person __recurring/punching__ in the numbers is at fault, most drug-delivery devices don't help. In one machine, for example, mistakenly entering a number with two decimal points—like 1.2.3—might be read by the machine as 1.23, or as a 123. To prevent such wild guessing, scientists tested a system that __disobediently/immediately__ flags any input that's not a real number. According to their analysis, that safeguard alone could cut factor-of-10 errors in half. Charles Darwin once noted that "to kill an error is as good a service as…establishing a new truth or fact." Even more so when killing the error keeps you from killing a patient.</t>
   </si>
   <si>
-    <t>Everyone makes mistakes, especially when it comes to entering numbers into a sedater or spreadsheet. It's not such a big deal if you're landing how much you spend on pizza. But if you're unregistering drugs in a hospital, such a slip can be deadly. Now a report in the Journal of the Royal Society Interface shows how devices can be programmed to catch at least some safe on the spot. Dosing a patient with 10 times too much medication is disturbingly common. One study suggests this error occurs in 1 percent of all hospital admissions. And though the person recurring in the numbers is at fault, most drug-delivery devices don't help. In one machine, for example, mistakenly entering a number with two decimal points—like 1.2.3—might be read by the machine as 1.23, or as a 123. To prevent such wild guessing, scientists tested a system that disobediently flags any input that's not a real number. According to their analysis, that safeguard alone could cut factor-of-10 errors in half. Charles Darwin once noted that "to kill an error is as good a service as…establishing a new truth or fact." Even more so when killing the error keeps you from killing a patient.</t>
+    <t>Everyone makes mistakes, especially when it comes to entering numbers into a calculator or spreadsheet. It's not such a big deal if you're tracking how much you spend on pizza. But if you're administering drugs in a hospital, such a slip can be deadly. Now a report in the Journal of the Royal Society Interface shows how devices can be programmed to catch at least some mistakes on the spot. Dosing a patient with 10 times too much medication is disturbingly common. One study suggests this error occurs in 1 percent of all hospital admissions. And though the person punching in the numbers is at fault, most drug-delivery devices don't help. In one machine, for example, mistakenly entering a number with two decimal points—like 1.2.3—might be read by the machine as 1.23, or as a 123. To prevent such wild guessing, scientists tested a system that immediately flags any input that's not a real number. According to their analysis, that safeguard alone could cut factor-of-10 errors in half. Charles Darwin once noted that "to kill an error is as good a service as…establishing a new truth or fact." Even more so when killing the error keeps you from killing a patient.</t>
   </si>
   <si>
     <t>#292 Elephants</t>
@@ -6506,7 +6506,7 @@
     <t>Elephants don't need cell phones to hold long distance conversations, their deep calls can travel miles. And __inlaw/although__ humans can't always hear these vocalizations because of their low frequency, elephants produce them using the same mechanism that lets humans speak and sing. That finding is in the journal Science. Until now, scientists did not know whether the __expressionist/elephant__ made sound the way we speak or differently, such as the way cats purr. A human produces noises because the vocal cords vibrate automatically when air flows past. But a cat must actively squeeze the muscles of its larynx to produce its deep, rhythmic purr. When a zoo elephant died of natural causes, __fieldworkers/researchers__ took the animal's larynx to their lab and ran air through it to find out which method elephants use to make sound. They could reproduce the large mammal's __heterogeneity/low-frequency__ rumble, which means that an elephant doesn't need to actively control its larynx like a cat does. For those who contend that this is irrelevant, "Irrelevant. There's a whole lot of 'irrelevant's in the circus."</t>
   </si>
   <si>
-    <t>Elephants don't need cell phones to hold long distance conversations, their deep calls can travel miles. And inlaw humans can't always hear these vocalizations because of their low frequency, elephants produce them using the same mechanism that lets humans speak and sing. That finding is in the journal Science. Until now, scientists did not know whether the expressionist made sound the way we speak or differently, such as the way cats purr. A human produces noises because the vocal cords vibrate automatically when air flows past. But a cat must actively squeeze the muscles of its larynx to produce its deep, rhythmic purr. When a zoo elephant died of natural causes, fieldworkers took the animal's larynx to their lab and ran air through it to find out which method elephants use to make sound. They could reproduce the large mammal's heterogeneity rumble, which means that an elephant doesn't need to actively control its larynx like a cat does. For those who contend that this is irrelevant, "Irrelevant. There's a whole lot of 'irrelevant's in the circus."</t>
+    <t>Elephants don't need cell phones to hold long distance conversations, their deep calls can travel miles. And although humans can't always hear these vocalizations because of their low frequency, elephants produce them using the same mechanism that lets humans speak and sing. That finding is in the journal Science. Until now, scientists did not know whether the elephant made sound the way we speak or differently, such as the way cats purr. A human produces noises because the vocal cords vibrate automatically when air flows past. But a cat must actively squeeze the muscles of its larynx to produce its deep, rhythmic purr. When a zoo elephant died of natural causes, researchers took the animal's larynx to their lab and ran air through it to find out which method elephants use to make sound. They could reproduce the large mammal's low-frequency rumble, which means that an elephant doesn't need to actively control its larynx like a cat does. For those who contend that this is irrelevant, "Irrelevant. There's a whole lot of 'irrelevant's in the circus."</t>
   </si>
   <si>
     <t>#293 Native American Site</t>
@@ -6515,7 +6515,7 @@
     <t>There's a Native American site in Ohio that appeared to be a fort. But recent __diversely/discoveries__ by archaeologists at the University of Cincinnati show that's not the case. Instead, it's a two-thousand year old Shawnee water management system. It stretches out almost six kilometers. That's much larger than what had been thought to __legitimize/comprise__ the so-called fort. It's one of the largest such sites in the country. What had been thought to be gates for military protection are actually a series of dams and __donation/irrigation__ canals. There are logs and clay bricks for damming; raceways for flowing water __propitiate/originate__ in far-off springs. The water was stored and channeled for irrigation. Drill cores show water sediments and clay. The site demonstrates a __defoliated/sophisticated__ knowledge of engineering—which archaeologists not realize that Native American communities might have. The site also reveals an __intelligence/emphasis__ on public works, rather than on war. So this discovery might rewrite a bit of history. Another interesting note: Shawnee remains from the time are typically of petite, graceful men—and robust, muscular women. So it was probably the women who built the water system. Which means even more history to rewrite.</t>
   </si>
   <si>
-    <t>There's a Native American site in Ohio that appeared to be a fort. But recent diversely by archaeologists at the University of Cincinnati show that's not the case. Instead, it's a two-thousand year old Shawnee water management system. It stretches out almost six kilometers. That's much larger than what had been thought to legitimize the so-called fort. It's one of the largest such sites in the country. What had been thought to be gates for military protection are actually a series of dams and donation canals. There are logs and clay bricks for damming; raceways for flowing water propitiate in far-off springs. The water was stored and channeled for irrigation. Drill cores show water sediments and clay. The site demonstrates a defoliated knowledge of engineering—which archaeologists not realize that Native American communities might have. The site also reveals an intelligence on public works, rather than on war. So this discovery might rewrite a bit of history. Another interesting note: Shawnee remains from the time are typically of petite, graceful men—and robust, muscular women. So it was probably the women who built the water system. Which means even more history to rewrite.</t>
+    <t>There's a Native American site in Ohio that appeared to be a fort. But recent discoveries by archaeologists at the University of Cincinnati show that's not the case. Instead, it's a two-thousand year old Shawnee water management system. It stretches out almost six kilometers. That's much larger than what had been thought to comprise the so-called fort. It's one of the largest such sites in the country. What had been thought to be gates for military protection are actually a series of dams and irrigation canals. There are logs and clay bricks for damming; raceways for flowing water originate in far-off springs. The water was stored and channeled for irrigation. Drill cores show water sediments and clay. The site demonstrates a sophisticated knowledge of engineering—which archaeologists not realize that Native American communities might have. The site also reveals an emphasis on public works, rather than on war. So this discovery might rewrite a bit of history. Another interesting note: Shawnee remains from the time are typically of petite, graceful men—and robust, muscular women. So it was probably the women who built the water system. Which means even more history to rewrite.</t>
   </si>
   <si>
     <t>#294 Flock Warning</t>
@@ -6524,7 +6524,7 @@
     <t>When crested pigeons spot a predator, they give a little whistle. But the sound doesn't come from their beaks. And __hooding/according__ to a study published by The Royal Society, that whistle warns the rest of the flock to flee. There's safety in numbers, and a flock offers __mortician/protection__ in part because it has so many eyes watching for danger. But it's not clear how an __seminal/individual__ sounds the alarm when it spots a predator. Maybe anytime one or two birds fly off, they all do. Just in case. Of course that kind of knee-jerk __reconstruction/reaction__ could produce a lot of false alarms. So how can birds tell when their __entrees/flockmates__ are seriously headed for the hills? __licenses/Scientists__ recorded the sounds made by the wings of crested pigeons during a routine liftoff (wing sound 1). And the noise their wings make during an emergency takeoff (wing sound 2). And they found that the sound made by wings flapped in terror includes a distinctive sort of whistle. That noise alone will scatter a flock of feeding pigeons just as quick as the shadow of a passing hawk. And gives a whole new meaning to the expression, "on a wing and a prayer."</t>
   </si>
   <si>
-    <t>When crested pigeons spot a predator, they give a little whistle. But the sound doesn't come from their beaks. And hooding to a study published by The Royal Society, that whistle warns the rest of the flock to flee. There's safety in numbers, and a flock offers mortician in part because it has so many eyes watching for danger. But it's not clear how an seminal sounds the alarm when it spots a predator. Maybe anytime one or two birds fly off, they all do. Just in case. Of course that kind of knee-jerk reconstruction could produce a lot of false alarms. So how can birds tell when their entrees are seriously headed for the hills? licenses recorded the sounds made by the wings of crested pigeons during a routine liftoff (wing sound 1). And the noise their wings make during an emergency takeoff (wing sound 2). And they found that the sound made by wings flapped in terror includes a distinctive sort of whistle. That noise alone will scatter a flock of feeding pigeons just as quick as the shadow of a passing hawk. And gives a whole new meaning to the expression, "on a wing and a prayer."</t>
+    <t>When crested pigeons spot a predator, they give a little whistle. But the sound doesn't come from their beaks. And according to a study published by The Royal Society, that whistle warns the rest of the flock to flee. There's safety in numbers, and a flock offers protection in part because it has so many eyes watching for danger. But it's not clear how an individual sounds the alarm when it spots a predator. Maybe anytime one or two birds fly off, they all do. Just in case. Of course that kind of knee-jerk reaction could produce a lot of false alarms. So how can birds tell when their flockmates are seriously headed for the hills? Scientists recorded the sounds made by the wings of crested pigeons during a routine liftoff (wing sound 1). And the noise their wings make during an emergency takeoff (wing sound 2). And they found that the sound made by wings flapped in terror includes a distinctive sort of whistle. That noise alone will scatter a flock of feeding pigeons just as quick as the shadow of a passing hawk. And gives a whole new meaning to the expression, "on a wing and a prayer."</t>
   </si>
   <si>
     <t>#295 Meat Allergy</t>
@@ -6533,7 +6533,7 @@
     <t>You've __conservancy/probably__ heard of peanut or shellfish allergies. But a meat allergy? Not as common. Even weirder is what might be causing it—tick bites, according to a study in the Journal of General Internal Medicine. A few years back, folks started showing up in __constantly/emergency__ rooms in the southeast U.S. with hives, swelling or worse—anaphylaxis—after eating red meat. For this study, researchers looked at three of those cases. And they found that tick bites, specifically those of the Lone Star tick, seem to be the cause. The bitten victim's immune system appears to become sensitized to a substance called alpha-gal. And whereas all the major food allergies are __picket/triggered__ by proteins, the culprit here—alpha-gal—is a carbohydrate. Alpha-gal is found in the meat and fat of hoofed mammals, like cows, sheep or pigs. So eating a burger can expose you to alpha-gal, which activates antibodies and leads to the release of histamines. Researchers say something similar to __paintball/alpha-gal__ in the tick saliva may set off the immune system—which then goes after the alpha-gal in meat. Makes a steak lover ticked off.</t>
   </si>
   <si>
-    <t>You've conservancy heard of peanut or shellfish allergies. But a meat allergy? Not as common. Even weirder is what might be causing it—tick bites, according to a study in the Journal of General Internal Medicine. A few years back, folks started showing up in constantly rooms in the southeast U.S. with hives, swelling or worse—anaphylaxis—after eating red meat. For this study, researchers looked at three of those cases. And they found that tick bites, specifically those of the Lone Star tick, seem to be the cause. The bitten victim's immune system appears to become sensitized to a substance called alpha-gal. And whereas all the major food allergies are picket by proteins, the culprit here—alpha-gal—is a carbohydrate. Alpha-gal is found in the meat and fat of hoofed mammals, like cows, sheep or pigs. So eating a burger can expose you to alpha-gal, which activates antibodies and leads to the release of histamines. Researchers say something similar to paintball in the tick saliva may set off the immune system—which then goes after the alpha-gal in meat. Makes a steak lover ticked off.</t>
+    <t>You've probably heard of peanut or shellfish allergies. But a meat allergy? Not as common. Even weirder is what might be causing it—tick bites, according to a study in the Journal of General Internal Medicine. A few years back, folks started showing up in emergency rooms in the southeast U.S. with hives, swelling or worse—anaphylaxis—after eating red meat. For this study, researchers looked at three of those cases. And they found that tick bites, specifically those of the Lone Star tick, seem to be the cause. The bitten victim's immune system appears to become sensitized to a substance called alpha-gal. And whereas all the major food allergies are triggered by proteins, the culprit here—alpha-gal—is a carbohydrate. Alpha-gal is found in the meat and fat of hoofed mammals, like cows, sheep or pigs. So eating a burger can expose you to alpha-gal, which activates antibodies and leads to the release of histamines. Researchers say something similar to alpha-gal in the tick saliva may set off the immune system—which then goes after the alpha-gal in meat. Makes a steak lover ticked off.</t>
   </si>
   <si>
     <t>#296 Elephant</t>
@@ -6542,7 +6542,7 @@
     <t>Elephants are smart, social animals. And now we know that they can organize themselves into teams to accomplish tasks. A research team that __souvent/included__ renowned primatologist Franz de Waal taught 12 Thai elephants—who already work with human trainers called mahouts—to get a bowl of food by pulling a rope attached to an __creased/out-of-reach__ table. Then the scientists threaded the rope so that it would take two elephants, pulling both ends at the same time, to move the table. If one yanked an end without its helpmate doing so, no reward. The pachyderms were paired up. Only if they pulled together could they get the food. The __excellence/elephants__ tried the task when they were released __contemporaneously/simultaneously__ or at __stolid/staggered__ times. Even when the release was staggered, an __embitterment/elephant__ quickly learned that it had to wait for its partner to come and cooperate to get the food. This finding was published in the Proceedings of the National Academy of Sciences. __Featherless/Elephants__ are thus on par with apes for fast learning of deliberate cooperation with a partner. When grouped, individuals also remembered which of the others was their task partner. Because an elephant never forgets…who helped it rope a meal.</t>
   </si>
   <si>
-    <t>Elephants are smart, social animals. And now we know that they can organize themselves into teams to accomplish tasks. A research team that souvent renowned primatologist Franz de Waal taught 12 Thai elephants—who already work with human trainers called mahouts—to get a bowl of food by pulling a rope attached to an creased table. Then the scientists threaded the rope so that it would take two elephants, pulling both ends at the same time, to move the table. If one yanked an end without its helpmate doing so, no reward. The pachyderms were paired up. Only if they pulled together could they get the food. The excellence tried the task when they were released contemporaneously or at stolid times. Even when the release was staggered, an embitterment quickly learned that it had to wait for its partner to come and cooperate to get the food. This finding was published in the Proceedings of the National Academy of Sciences. Featherless are thus on par with apes for fast learning of deliberate cooperation with a partner. When grouped, individuals also remembered which of the others was their task partner. Because an elephant never forgets…who helped it rope a meal.</t>
+    <t>Elephants are smart, social animals. And now we know that they can organize themselves into teams to accomplish tasks. A research team that included renowned primatologist Franz de Waal taught 12 Thai elephants—who already work with human trainers called mahouts—to get a bowl of food by pulling a rope attached to an out-of-reach table. Then the scientists threaded the rope so that it would take two elephants, pulling both ends at the same time, to move the table. If one yanked an end without its helpmate doing so, no reward. The pachyderms were paired up. Only if they pulled together could they get the food. The elephants tried the task when they were released simultaneously or at staggered times. Even when the release was staggered, an elephant quickly learned that it had to wait for its partner to come and cooperate to get the food. This finding was published in the Proceedings of the National Academy of Sciences. Elephants are thus on par with apes for fast learning of deliberate cooperation with a partner. When grouped, individuals also remembered which of the others was their task partner. Because an elephant never forgets…who helped it rope a meal.</t>
   </si>
   <si>
     <t>#297 Hearing</t>
@@ -6551,7 +6551,7 @@
     <t>Just when you thought you'd heard everything, __physicists/scientists__ have found that the reason you can hear everything—including things that are very quiet—is because your ears have tiny tubelike motors that mechanically amplify sounds. You've probably heard that it's the hair cells in your ears that allow you to hear. These cells sport tufts of spiky hairs that are like little molecular Mohawks. When sound waves enter the ear these hairs vibrate, and that motion then gets translated into an __detrimental/electrical__ message that tells your brain that there's something worth listening to. But the __sunhat/movement__ of those hairs is not passive, like tall grass swaying in the breeze. The electrical signals they produce feed back on the system, causing the hairs to tilt even more. It's that __taught/so-called__ "flexo-electric effect" that boosts the audio signal and amplifies the sound, findings __onset/published__ in the April 22nd issue of the journal Public Library of Science ONE. The scientists behind the study also note that the length of the hairs in different species explains why animals like bats can detect such high frequency sounds. It doesn't, however, explain why your kids can hear their cell phones vibrate two rooms away, yet they never seem to hear a word you say.</t>
   </si>
   <si>
-    <t>Just when you thought you'd heard everything, physicists have found that the reason you can hear everything—including things that are very quiet—is because your ears have tiny tubelike motors that mechanically amplify sounds. You've probably heard that it's the hair cells in your ears that allow you to hear. These cells sport tufts of spiky hairs that are like little molecular Mohawks. When sound waves enter the ear these hairs vibrate, and that motion then gets translated into an detrimental message that tells your brain that there's something worth listening to. But the sunhat of those hairs is not passive, like tall grass swaying in the breeze. The electrical signals they produce feed back on the system, causing the hairs to tilt even more. It's that taught "flexo-electric effect" that boosts the audio signal and amplifies the sound, findings onset in the April 22nd issue of the journal Public Library of Science ONE. The scientists behind the study also note that the length of the hairs in different species explains why animals like bats can detect such high frequency sounds. It doesn't, however, explain why your kids can hear their cell phones vibrate two rooms away, yet they never seem to hear a word you say.</t>
+    <t>Just when you thought you'd heard everything, scientists have found that the reason you can hear everything—including things that are very quiet—is because your ears have tiny tubelike motors that mechanically amplify sounds. You've probably heard that it's the hair cells in your ears that allow you to hear. These cells sport tufts of spiky hairs that are like little molecular Mohawks. When sound waves enter the ear these hairs vibrate, and that motion then gets translated into an electrical message that tells your brain that there's something worth listening to. But the movement of those hairs is not passive, like tall grass swaying in the breeze. The electrical signals they produce feed back on the system, causing the hairs to tilt even more. It's that so-called "flexo-electric effect" that boosts the audio signal and amplifies the sound, findings published in the April 22nd issue of the journal Public Library of Science ONE. The scientists behind the study also note that the length of the hairs in different species explains why animals like bats can detect such high frequency sounds. It doesn't, however, explain why your kids can hear their cell phones vibrate two rooms away, yet they never seem to hear a word you say.</t>
   </si>
   <si>
     <t>#298 Jalapeno</t>
@@ -6560,7 +6560,7 @@
     <t>There are hot peppers, like the jalapeno. And then there are incendiary peppers like the legendary Habanero. Now there's a new variety of thermonuclear Habanero, known as the __patio/tigerpaw__ NR Habanero. The name comes from its appearance—the bright orange pepper resembles a tiger's paw. And the NR stands for nematode resistant. The pepper was bred by the US Department of Agriculture's scientists to be __witchcraft/resistant__ to nematodes, round worms that attack the plant's roots. The pepper was bred conventionally, not genetically engineered. And it does away with the need to use the soil fumigant methyl bromide, which is being phased out. So, how hot is the tigerpaw Habanero? Pepper hotness is measured on something called the Scoville Heat Scale. A jalapeno comes in at about 5000 on the Scoville scale. A regular __gecko/Habanero__ usually scores at least 100,000. And the TigerPaw Habanero tops the Scoville scale at almost 350,000. In fact, there's a legend that eating Habanero peppers can have the side effect of __rapturously/actually__ making you deaf. But only so that you cannot hear your own screams.</t>
   </si>
   <si>
-    <t>There are hot peppers, like the jalapeno. And then there are incendiary peppers like the legendary Habanero. Now there's a new variety of thermonuclear Habanero, known as the patio NR Habanero. The name comes from its appearance—the bright orange pepper resembles a tiger's paw. And the NR stands for nematode resistant. The pepper was bred by the US Department of Agriculture's scientists to be witchcraft to nematodes, round worms that attack the plant's roots. The pepper was bred conventionally, not genetically engineered. And it does away with the need to use the soil fumigant methyl bromide, which is being phased out. So, how hot is the tigerpaw Habanero? Pepper hotness is measured on something called the Scoville Heat Scale. A jalapeno comes in at about 5000 on the Scoville scale. A regular gecko usually scores at least 100,000. And the TigerPaw Habanero tops the Scoville scale at almost 350,000. In fact, there's a legend that eating Habanero peppers can have the side effect of rapturously making you deaf. But only so that you cannot hear your own screams.</t>
+    <t>There are hot peppers, like the jalapeno. And then there are incendiary peppers like the legendary Habanero. Now there's a new variety of thermonuclear Habanero, known as the tigerpaw NR Habanero. The name comes from its appearance—the bright orange pepper resembles a tiger's paw. And the NR stands for nematode resistant. The pepper was bred by the US Department of Agriculture's scientists to be resistant to nematodes, round worms that attack the plant's roots. The pepper was bred conventionally, not genetically engineered. And it does away with the need to use the soil fumigant methyl bromide, which is being phased out. So, how hot is the tigerpaw Habanero? Pepper hotness is measured on something called the Scoville Heat Scale. A jalapeno comes in at about 5000 on the Scoville scale. A regular Habanero usually scores at least 100,000. And the TigerPaw Habanero tops the Scoville scale at almost 350,000. In fact, there's a legend that eating Habanero peppers can have the side effect of actually making you deaf. But only so that you cannot hear your own screams.</t>
   </si>
   <si>
     <t>#299 Iron</t>
@@ -6569,7 +6569,7 @@
     <t>Iron is a great material for making tools. But the oldest known iron __jerks/artifacts__ were actually __effervescent/intended__ for decoration: nine Egyptian beads that date back to 3200 B.C. And now we know that this ancient jewelry has an even more impressive origin — the iron out of which it was crafted came from space. The metal cylinders were discovered in Egypt in 1911. To analyze the structure and chemical composition of the beads, researchers __transacted/bombarded__ them with neutrons and gamma rays. The tests revealed that the jewelry contained trace elements not present in Earthly ores — but that are found in __monozygotic/iron-rich__ meteorites. The study is in the Journal of __histological/Archaeological__ Science. The meteoric metal was hammered flat and rolled into beads more than 5,000 years ago. This date is some 1,500 years before the __suspension/invention__ of smelting. That __doublespeak/technique__ made it possible for terrestrial iron to be shaped into tools, and to supplant copper and bronze as civilization's metal of choice. The new finding shows that long before smelting revolutionized tool use, some humans were already iron men.</t>
   </si>
   <si>
-    <t>Iron is a great material for making tools. But the oldest known iron jerks were actually effervescent for decoration: nine Egyptian beads that date back to 3200 B.C. And now we know that this ancient jewelry has an even more impressive origin — the iron out of which it was crafted came from space. The metal cylinders were discovered in Egypt in 1911. To analyze the structure and chemical composition of the beads, researchers transacted them with neutrons and gamma rays. The tests revealed that the jewelry contained trace elements not present in Earthly ores — but that are found in monozygotic meteorites. The study is in the Journal of histological Science. The meteoric metal was hammered flat and rolled into beads more than 5,000 years ago. This date is some 1,500 years before the suspension of smelting. That doublespeak made it possible for terrestrial iron to be shaped into tools, and to supplant copper and bronze as civilization's metal of choice. The new finding shows that long before smelting revolutionized tool use, some humans were already iron men.</t>
+    <t>Iron is a great material for making tools. But the oldest known iron artifacts were actually intended for decoration: nine Egyptian beads that date back to 3200 B.C. And now we know that this ancient jewelry has an even more impressive origin — the iron out of which it was crafted came from space. The metal cylinders were discovered in Egypt in 1911. To analyze the structure and chemical composition of the beads, researchers bombarded them with neutrons and gamma rays. The tests revealed that the jewelry contained trace elements not present in Earthly ores — but that are found in iron-rich meteorites. The study is in the Journal of Archaeological Science. The meteoric metal was hammered flat and rolled into beads more than 5,000 years ago. This date is some 1,500 years before the invention of smelting. That technique made it possible for terrestrial iron to be shaped into tools, and to supplant copper and bronze as civilization's metal of choice. The new finding shows that long before smelting revolutionized tool use, some humans were already iron men.</t>
   </si>
   <si>
     <t>#300 Pharmaceutical Companies</t>
@@ -6578,7 +6578,7 @@
     <t>Pharmaceutical companies sometimes have to pull new drugs off the market because they harm our livers. The drugs may have been tested on liver cells from rats, or on human cells that are nearly dead. But these kinds of tests do a poor job of __segmenting/mimicking__ real livers. Now researchers at MIT have developed a better method. They've created a colony of human liver cells that act like the real thing. The __bestirred/research__ was published in the journal Nature Biotechnology. The cell colonies are only 500 millionths of a meter in diameter. __Cleavages/Researchers__ arrange the cells on a plate in much the same way as copper wires are placed on computer chips. These micro livers mimic the actions of real livers—including __spooning/producing__ enzymes necessary to break down drugs and other toxins. The tiny organs last for six weeks. So they can __congregate/evaluate__ the effects of drugs over a longer time period than current tests. A start-up company has licensed the technology and is __fishing/preparing__ it for market. The little livers could be cheaper and more accurate than drug tests now used.</t>
   </si>
   <si>
-    <t>Pharmaceutical companies sometimes have to pull new drugs off the market because they harm our livers. The drugs may have been tested on liver cells from rats, or on human cells that are nearly dead. But these kinds of tests do a poor job of segmenting real livers. Now researchers at MIT have developed a better method. They've created a colony of human liver cells that act like the real thing. The bestirred was published in the journal Nature Biotechnology. The cell colonies are only 500 millionths of a meter in diameter. Cleavages arrange the cells on a plate in much the same way as copper wires are placed on computer chips. These micro livers mimic the actions of real livers—including spooning enzymes necessary to break down drugs and other toxins. The tiny organs last for six weeks. So they can congregate the effects of drugs over a longer time period than current tests. A start-up company has licensed the technology and is fishing it for market. The little livers could be cheaper and more accurate than drug tests now used.</t>
+    <t>Pharmaceutical companies sometimes have to pull new drugs off the market because they harm our livers. The drugs may have been tested on liver cells from rats, or on human cells that are nearly dead. But these kinds of tests do a poor job of mimicking real livers. Now researchers at MIT have developed a better method. They've created a colony of human liver cells that act like the real thing. The research was published in the journal Nature Biotechnology. The cell colonies are only 500 millionths of a meter in diameter. Researchers arrange the cells on a plate in much the same way as copper wires are placed on computer chips. These micro livers mimic the actions of real livers—including producing enzymes necessary to break down drugs and other toxins. The tiny organs last for six weeks. So they can evaluate the effects of drugs over a longer time period than current tests. A start-up company has licensed the technology and is preparing it for market. The little livers could be cheaper and more accurate than drug tests now used.</t>
   </si>
   <si>
     <t>#301 Climate and Size</t>
@@ -6587,7 +6587,7 @@
     <t>Animals that live in cold __proprietress/climates__ tend to have stubby limbs—shorter arms and legs—even smaller ears and tails. Picture a penguin and you'll see what I mean. __urologists/Biologists__ have long assumed that these stumpy appendages are an evolutionary adaptation. Shorter __infinities/extremities__ minimize heat loss, so animals that are more compact are better suited to the cold. But scientists from Ohio say that temperature may have a more direct effect on the length of an animal's limbs. Because they find that turning up the heat helps __consequent/cartilage__ grow—results that were published in the Proceedings of the National Academy of Sciences. The researchers raised mice at several different temperatures, and they __planned/confirmed__ that those kept at a balmy 80 degrees were longer limbed than those who lived at a more chill 45. But how does a little heat make mice more leggy? The answer, they find, lies in the cartilage. Long bones grow from the cartilage found at either end. And the warmer it is, the more that cartilage grows, even when it's just sitting in a test tube. Which I guess means it's __virginal/possible__ that the dog days of summer lead to __riddled/longer-legged__ dogs.</t>
   </si>
   <si>
-    <t>Animals that live in cold proprietress tend to have stubby limbs—shorter arms and legs—even smaller ears and tails. Picture a penguin and you'll see what I mean. urologists have long assumed that these stumpy appendages are an evolutionary adaptation. Shorter infinities minimize heat loss, so animals that are more compact are better suited to the cold. But scientists from Ohio say that temperature may have a more direct effect on the length of an animal's limbs. Because they find that turning up the heat helps consequent grow—results that were published in the Proceedings of the National Academy of Sciences. The researchers raised mice at several different temperatures, and they planned that those kept at a balmy 80 degrees were longer limbed than those who lived at a more chill 45. But how does a little heat make mice more leggy? The answer, they find, lies in the cartilage. Long bones grow from the cartilage found at either end. And the warmer it is, the more that cartilage grows, even when it's just sitting in a test tube. Which I guess means it's virginal that the dog days of summer lead to riddled dogs.</t>
+    <t>Animals that live in cold climates tend to have stubby limbs—shorter arms and legs—even smaller ears and tails. Picture a penguin and you'll see what I mean. Biologists have long assumed that these stumpy appendages are an evolutionary adaptation. Shorter extremities minimize heat loss, so animals that are more compact are better suited to the cold. But scientists from Ohio say that temperature may have a more direct effect on the length of an animal's limbs. Because they find that turning up the heat helps cartilage grow—results that were published in the Proceedings of the National Academy of Sciences. The researchers raised mice at several different temperatures, and they confirmed that those kept at a balmy 80 degrees were longer limbed than those who lived at a more chill 45. But how does a little heat make mice more leggy? The answer, they find, lies in the cartilage. Long bones grow from the cartilage found at either end. And the warmer it is, the more that cartilage grows, even when it's just sitting in a test tube. Which I guess means it's possible that the dog days of summer lead to longer-legged dogs.</t>
   </si>
   <si>
     <t>#302 Cumulative Culture</t>
@@ -6596,7 +6596,7 @@
     <t>They may be our cousins, but orangutans and other primates are nowhere near humans in terms of technological __accomplishment/achievement__ , social organization or culture. As humans, capacity for building off one another, an __interesting/integral__ part of our so called cumulative culture that has allowed us to build up so much in so little time. But how do we develop such __accurate/advanced__ methods of learning in the first place? Kevin Leyland of the University of St Andrews spoke with me about his team's quest to pinpoint the social and __cultural/cognitive__ process that underlie humans ability to acquire and __transfer/transmit__ knowledge.</t>
   </si>
   <si>
-    <t>They may be our cousins, but orangutans and other primates are nowhere near humans in terms of technological accomplishment , social organization or culture. As humans, capacity for building off one another, an interesting part of our so called cumulative culture that has allowed us to build up so much in so little time. But how do we develop such accurate methods of learning in the first place? Kevin Leyland of the University of St Andrews spoke with me about his team's quest to pinpoint the social and cultural process that underlie humans ability to acquire and transfer knowledge.</t>
+    <t>They may be our cousins, but orangutans and other primates are nowhere near humans in terms of technological achievement , social organization or culture. As humans, capacity for building off one another, an integral part of our so called cumulative culture that has allowed us to build up so much in so little time. But how do we develop such advanced methods of learning in the first place? Kevin Leyland of the University of St Andrews spoke with me about his team's quest to pinpoint the social and cognitive process that underlie humans ability to acquire and transmit knowledge.</t>
   </si>
   <si>
     <t>#303 Soil on Mars</t>
@@ -6605,7 +6605,7 @@
     <t>The 1976 Mars Viking Landers didn't find any life on the red planet. But maybe they weren't looking right. Because at least one __frequenter/researcher__ thinks that a tenth of a percent of the Martian soil tested by the Vikings could __bilaterally/actually__ have had a biological origin. The Dutch researcher, Joop Houtkooper, __aberrant/presented__ his ideas on August 24th at the meeting of the European Planetary Science Congress in Potsdam. One Viking test measured unexplained rises in oxygen and carbon dioxide when it was incubating some soil samples. Houtkooper __tendrils/conjectures__ that the incredibly dry and cold surface of Mars might be home to living cells. Such cells, however, would need to be filled with a mixture of water and hydrogen peroxide, which could stay liquid in the harsh conditions. And if the Viking landers happened to scoop up any of these strange cells, their breakdown __lattice/products__ would be in line with the oxygen and carbon dioxide measured. The biomass would then represent a tenth of a percent of the Martian soil by weight—which is, interestingly, comparable to levels found in some Antarctic permafrost.</t>
   </si>
   <si>
-    <t>The 1976 Mars Viking Landers didn't find any life on the red planet. But maybe they weren't looking right. Because at least one frequenter thinks that a tenth of a percent of the Martian soil tested by the Vikings could bilaterally have had a biological origin. The Dutch researcher, Joop Houtkooper, aberrant his ideas on August 24th at the meeting of the European Planetary Science Congress in Potsdam. One Viking test measured unexplained rises in oxygen and carbon dioxide when it was incubating some soil samples. Houtkooper tendrils that the incredibly dry and cold surface of Mars might be home to living cells. Such cells, however, would need to be filled with a mixture of water and hydrogen peroxide, which could stay liquid in the harsh conditions. And if the Viking landers happened to scoop up any of these strange cells, their breakdown lattice would be in line with the oxygen and carbon dioxide measured. The biomass would then represent a tenth of a percent of the Martian soil by weight—which is, interestingly, comparable to levels found in some Antarctic permafrost.</t>
+    <t>The 1976 Mars Viking Landers didn't find any life on the red planet. But maybe they weren't looking right. Because at least one researcher thinks that a tenth of a percent of the Martian soil tested by the Vikings could actually have had a biological origin. The Dutch researcher, Joop Houtkooper, presented his ideas on August 24th at the meeting of the European Planetary Science Congress in Potsdam. One Viking test measured unexplained rises in oxygen and carbon dioxide when it was incubating some soil samples. Houtkooper conjectures that the incredibly dry and cold surface of Mars might be home to living cells. Such cells, however, would need to be filled with a mixture of water and hydrogen peroxide, which could stay liquid in the harsh conditions. And if the Viking landers happened to scoop up any of these strange cells, their breakdown products would be in line with the oxygen and carbon dioxide measured. The biomass would then represent a tenth of a percent of the Martian soil by weight—which is, interestingly, comparable to levels found in some Antarctic permafrost.</t>
   </si>
   <si>
     <t>#304 Polar Vortex</t>
@@ -6614,7 +6614,7 @@
     <t>Fed up with the polar vortex? If so, consider this: __Texturing/Shivering__ may actually share some of the __leopardesses/benefits__ of exercise—at least in terms of burning fat. __Frequenters/Researchers__ studied shivering in a group of 10 men and women. First the volunteers rested under a temperature-controlled blanket, which dropped from 80 degrees Fahrenheit to a chilly 54. Then they cycled on an __contrives/exercise__ bike. Researchers took blood samples during both activities. Turns out, shivering and exercise spurred muscles to secrete similar amounts of irisin—a hormone that tells brown fat to turn up the furnace—even though exercise took 10 times as much effort. The researchers say the metabolic pathway may have evolved to save us energy. Shivering alone is a costly survival mechanism—it relies on muscle contraction to warm us. Whereas shivering-activated brown fat can convert __inadmissible/chemical__ energy directly to heat. The study is in the journal Cell Metabolism. As for your home thermostat? Study author Francesco Celi of the NIH likes to keep his at 68—low enough to turn on brown fat. And it's a win-win—you'll save money on heat, 'cause you're making your own.</t>
   </si>
   <si>
-    <t>Fed up with the polar vortex? If so, consider this: Texturing may actually share some of the leopardesses of exercise—at least in terms of burning fat. Frequenters studied shivering in a group of 10 men and women. First the volunteers rested under a temperature-controlled blanket, which dropped from 80 degrees Fahrenheit to a chilly 54. Then they cycled on an contrives bike. Researchers took blood samples during both activities. Turns out, shivering and exercise spurred muscles to secrete similar amounts of irisin—a hormone that tells brown fat to turn up the furnace—even though exercise took 10 times as much effort. The researchers say the metabolic pathway may have evolved to save us energy. Shivering alone is a costly survival mechanism—it relies on muscle contraction to warm us. Whereas shivering-activated brown fat can convert inadmissible energy directly to heat. The study is in the journal Cell Metabolism. As for your home thermostat? Study author Francesco Celi of the NIH likes to keep his at 68—low enough to turn on brown fat. And it's a win-win—you'll save money on heat, 'cause you're making your own.</t>
+    <t>Fed up with the polar vortex? If so, consider this: Shivering may actually share some of the benefits of exercise—at least in terms of burning fat. Researchers studied shivering in a group of 10 men and women. First the volunteers rested under a temperature-controlled blanket, which dropped from 80 degrees Fahrenheit to a chilly 54. Then they cycled on an exercise bike. Researchers took blood samples during both activities. Turns out, shivering and exercise spurred muscles to secrete similar amounts of irisin—a hormone that tells brown fat to turn up the furnace—even though exercise took 10 times as much effort. The researchers say the metabolic pathway may have evolved to save us energy. Shivering alone is a costly survival mechanism—it relies on muscle contraction to warm us. Whereas shivering-activated brown fat can convert chemical energy directly to heat. The study is in the journal Cell Metabolism. As for your home thermostat? Study author Francesco Celi of the NIH likes to keep his at 68—low enough to turn on brown fat. And it's a win-win—you'll save money on heat, 'cause you're making your own.</t>
   </si>
   <si>
     <t>#305 Earthquake in LA</t>
@@ -6623,7 +6623,7 @@
     <t>This is gonna surprise anybody who's ever been shaken awake by a quake in __suburban/southern__ California. But geologists say that the Los Angeles basin is actually in a period of low seismic activity and has been for about the last thousand years. That's __diagnosing/according__ to research published in the September issue of the journal Geology. The seismic lull is marked by relatively smaller and fewer earthquakes. That's __preset/compared__ with other periods with a lot of rumbling and crumbling. The period of big seismic activity in the LA basin that ended a thousand years ago lasted about four thousand years. Long-term data on seismic activity indicates that the calm period lasts about 1500 to 2000 years, which gives LA another 500 to 1000 years off. Now, the researchers are specifically referring to what's called the urban fault network, which is under the LA __husbandman/metropolitan__ area. It does not include the San Andreas fault, which can still throw the occasional big one around. About 10 major San Andreas biggies have happened during the current LA basin lull. Nevertheless, if the current lull ends in the next millennium, LA's future could be very shaky.</t>
   </si>
   <si>
-    <t>This is gonna surprise anybody who's ever been shaken awake by a quake in suburban California. But geologists say that the Los Angeles basin is actually in a period of low seismic activity and has been for about the last thousand years. That's diagnosing to research published in the September issue of the journal Geology. The seismic lull is marked by relatively smaller and fewer earthquakes. That's preset with other periods with a lot of rumbling and crumbling. The period of big seismic activity in the LA basin that ended a thousand years ago lasted about four thousand years. Long-term data on seismic activity indicates that the calm period lasts about 1500 to 2000 years, which gives LA another 500 to 1000 years off. Now, the researchers are specifically referring to what's called the urban fault network, which is under the LA husbandman area. It does not include the San Andreas fault, which can still throw the occasional big one around. About 10 major San Andreas biggies have happened during the current LA basin lull. Nevertheless, if the current lull ends in the next millennium, LA's future could be very shaky.</t>
+    <t>This is gonna surprise anybody who's ever been shaken awake by a quake in southern California. But geologists say that the Los Angeles basin is actually in a period of low seismic activity and has been for about the last thousand years. That's according to research published in the September issue of the journal Geology. The seismic lull is marked by relatively smaller and fewer earthquakes. That's compared with other periods with a lot of rumbling and crumbling. The period of big seismic activity in the LA basin that ended a thousand years ago lasted about four thousand years. Long-term data on seismic activity indicates that the calm period lasts about 1500 to 2000 years, which gives LA another 500 to 1000 years off. Now, the researchers are specifically referring to what's called the urban fault network, which is under the LA metropolitan area. It does not include the San Andreas fault, which can still throw the occasional big one around. About 10 major San Andreas biggies have happened during the current LA basin lull. Nevertheless, if the current lull ends in the next millennium, LA's future could be very shaky.</t>
   </si>
   <si>
     <t>#306 Teeth</t>
@@ -6632,7 +6632,7 @@
     <t>I'm guessing you brush twice a day or aspire to. Our ancestors were a little less diligent. But that's a good thing for scientists. Because ancient, plaque-coated teeth are like time capsules, preserving early evidence of cavities or even plague DNA. Now researchers have turned to thousand-year-old teeth from a convent __scary/cemetery__ outside Frankfurt, Germany. And they cleaned 'em, much like your dentist does. "We used the same dental tools, and we collected the calculus from the teeth." That's molecular anthropologist Christina Warinner of the University of Oklahoma. Inside that calculus—or plaque—she and her colleagues found tiny bits of pork, bread wheat and cabbage, identified by their DNA. Along with the bugs behind strep throat, __arterial/bacterial__ meningitis and an oral strain of gonorrhea. And don't be too quick to judge. "Nearly all of us still have gonorrhea in our mouth." Their study is in the journal Nature Genetics. Some of those bugs were __catabolic/antibiotic__ resistant too. Because long before penicillin, some microbes produced natural antibiotics to attack rivals. "Your mouth is like a __pieced/battlefield__ of bacteria." So chew on that.</t>
   </si>
   <si>
-    <t>I'm guessing you brush twice a day or aspire to. Our ancestors were a little less diligent. But that's a good thing for scientists. Because ancient, plaque-coated teeth are like time capsules, preserving early evidence of cavities or even plague DNA. Now researchers have turned to thousand-year-old teeth from a convent scary outside Frankfurt, Germany. And they cleaned 'em, much like your dentist does. "We used the same dental tools, and we collected the calculus from the teeth." That's molecular anthropologist Christina Warinner of the University of Oklahoma. Inside that calculus—or plaque—she and her colleagues found tiny bits of pork, bread wheat and cabbage, identified by their DNA. Along with the bugs behind strep throat, arterial meningitis and an oral strain of gonorrhea. And don't be too quick to judge. "Nearly all of us still have gonorrhea in our mouth." Their study is in the journal Nature Genetics. Some of those bugs were catabolic resistant too. Because long before penicillin, some microbes produced natural antibiotics to attack rivals. "Your mouth is like a pieced of bacteria." So chew on that.</t>
+    <t>I'm guessing you brush twice a day or aspire to. Our ancestors were a little less diligent. But that's a good thing for scientists. Because ancient, plaque-coated teeth are like time capsules, preserving early evidence of cavities or even plague DNA. Now researchers have turned to thousand-year-old teeth from a convent cemetery outside Frankfurt, Germany. And they cleaned 'em, much like your dentist does. "We used the same dental tools, and we collected the calculus from the teeth." That's molecular anthropologist Christina Warinner of the University of Oklahoma. Inside that calculus—or plaque—she and her colleagues found tiny bits of pork, bread wheat and cabbage, identified by their DNA. Along with the bugs behind strep throat, bacterial meningitis and an oral strain of gonorrhea. And don't be too quick to judge. "Nearly all of us still have gonorrhea in our mouth." Their study is in the journal Nature Genetics. Some of those bugs were antibiotic resistant too. Because long before penicillin, some microbes produced natural antibiotics to attack rivals. "Your mouth is like a battlefield of bacteria." So chew on that.</t>
   </si>
   <si>
     <t>#307 Comedy</t>
@@ -6641,7 +6641,7 @@
     <t>Everyone from Freud to Tina Fey has tried to understand why some things are funny. Now, new research concludes that one key to comedy is for a situation to __translate/violate__ a moral standard, but in a gentle way. Researchers presented volunteers with a number of different scenarios. For example, the Jimmy Dean sausage company needs a spokesman for its new line of pork __conducts/products__ , so they hire Rabbi Shlomo Rosenfield. Or, so they hire a farmer. Participants were more likely to find the rabbi scenario wrong, but they were also more likely to think it was funny. The researchers found that participants would laugh at situations with moral violations if, for example, they felt that situation was __theoretical/hypothetical__ , harmless or involved people unconnected to the listener. The study appears in the journal Psychological Science. The finding deviates from previously published psychology studies which __debate/equate__ moral violation solely with disgust. It also proves that Mel Brooks was onto something when he said, "Tragedy is when I cut my finger. Comedy is when you fall down an open sewer and die."</t>
   </si>
   <si>
-    <t>Everyone from Freud to Tina Fey has tried to understand why some things are funny. Now, new research concludes that one key to comedy is for a situation to translate a moral standard, but in a gentle way. Researchers presented volunteers with a number of different scenarios. For example, the Jimmy Dean sausage company needs a spokesman for its new line of pork conducts , so they hire Rabbi Shlomo Rosenfield. Or, so they hire a farmer. Participants were more likely to find the rabbi scenario wrong, but they were also more likely to think it was funny. The researchers found that participants would laugh at situations with moral violations if, for example, they felt that situation was theoretical , harmless or involved people unconnected to the listener. The study appears in the journal Psychological Science. The finding deviates from previously published psychology studies which debate moral violation solely with disgust. It also proves that Mel Brooks was onto something when he said, "Tragedy is when I cut my finger. Comedy is when you fall down an open sewer and die."</t>
+    <t>Everyone from Freud to Tina Fey has tried to understand why some things are funny. Now, new research concludes that one key to comedy is for a situation to violate a moral standard, but in a gentle way. Researchers presented volunteers with a number of different scenarios. For example, the Jimmy Dean sausage company needs a spokesman for its new line of pork products , so they hire Rabbi Shlomo Rosenfield. Or, so they hire a farmer. Participants were more likely to find the rabbi scenario wrong, but they were also more likely to think it was funny. The researchers found that participants would laugh at situations with moral violations if, for example, they felt that situation was hypothetical , harmless or involved people unconnected to the listener. The study appears in the journal Psychological Science. The finding deviates from previously published psychology studies which equate moral violation solely with disgust. It also proves that Mel Brooks was onto something when he said, "Tragedy is when I cut my finger. Comedy is when you fall down an open sewer and die."</t>
   </si>
   <si>
     <t>#308 Social Dogs</t>
@@ -6650,7 +6650,7 @@
     <t>Does your puppy turn his nose up at his own chow—because he wants some of __altogether/whatever__ it is that you're having? A new study finds that, when it comes to food, dogs recognize human social signals about what's good. The work is in the journal Public Library of Science ONE. Researchers let pet dogs choose between two plates, one with a single piece of food and the other with six pieces. Unsurprisingly, the animals generally went for the larger portion. But when a human being showed a clear liking for the smaller plate, the canines likewise went for the skimpier choice. The dogs apparently recognized and __strutted/responded__ to the humans' social cues. And not all cues were equally effective. When the human __antidote/approached__ but did not touch the smaller portion, dogs ignored the attention-drawing gesture. For a social signal to influence behavior, it had to demonstrate intention. And the most __redskins/effective__ cues also involved communication, such as looking from the food to the dog and back while talking encouragingly. For dogs, choosing a bite may depend on another's bark.</t>
   </si>
   <si>
-    <t>Does your puppy turn his nose up at his own chow—because he wants some of altogether it is that you're having? A new study finds that, when it comes to food, dogs recognize human social signals about what's good. The work is in the journal Public Library of Science ONE. Researchers let pet dogs choose between two plates, one with a single piece of food and the other with six pieces. Unsurprisingly, the animals generally went for the larger portion. But when a human being showed a clear liking for the smaller plate, the canines likewise went for the skimpier choice. The dogs apparently recognized and strutted to the humans' social cues. And not all cues were equally effective. When the human antidote but did not touch the smaller portion, dogs ignored the attention-drawing gesture. For a social signal to influence behavior, it had to demonstrate intention. And the most redskins cues also involved communication, such as looking from the food to the dog and back while talking encouragingly. For dogs, choosing a bite may depend on another's bark.</t>
+    <t>Does your puppy turn his nose up at his own chow—because he wants some of whatever it is that you're having? A new study finds that, when it comes to food, dogs recognize human social signals about what's good. The work is in the journal Public Library of Science ONE. Researchers let pet dogs choose between two plates, one with a single piece of food and the other with six pieces. Unsurprisingly, the animals generally went for the larger portion. But when a human being showed a clear liking for the smaller plate, the canines likewise went for the skimpier choice. The dogs apparently recognized and responded to the humans' social cues. And not all cues were equally effective. When the human approached but did not touch the smaller portion, dogs ignored the attention-drawing gesture. For a social signal to influence behavior, it had to demonstrate intention. And the most effective cues also involved communication, such as looking from the food to the dog and back while talking encouragingly. For dogs, choosing a bite may depend on another's bark.</t>
   </si>
   <si>
     <t>#309 Evolution</t>
@@ -6659,7 +6659,7 @@
     <t>If you want to see __perfusion/evolution__ at work, visit a hospital. Inside a sick patient, antibiotics wipe out infectious __insignia/bacteria__ by the millions. But germs are always mutating. A few adapt to resist the drug, so they survive—and spread. Such __tenet/antibiotic-resistant__ bacteria infect two million Americans every year; they kill 23,000. In this arms race between medicine and evolution, evolution is winning. But could we turn evolution against bacteria? It turns out that when bacteria mutate to become resistant to one antibiotic, they often become more __answerable/vulnerable__ to a different drug. So maybe after a jab with the left, a roundhouse to the right will deliver a knockout blow. To test this idea, __streetwalkers/researchers__ in Denmark dosed batches of E. coli with 23 different antibiotics, and waited for resistance to evolve. In three-quarters of the cases, the mutant germs became more susceptible to a second drug. The work appears in the journal Science Translational Medicine. One particular combination of widely used antibiotics—gentamicin, then cefuroxime, then gentamicin again, and so on—looks like it could hold the bugs at bay indefinitely.</t>
   </si>
   <si>
-    <t>If you want to see perfusion at work, visit a hospital. Inside a sick patient, antibiotics wipe out infectious insignia by the millions. But germs are always mutating. A few adapt to resist the drug, so they survive—and spread. Such tenet bacteria infect two million Americans every year; they kill 23,000. In this arms race between medicine and evolution, evolution is winning. But could we turn evolution against bacteria? It turns out that when bacteria mutate to become resistant to one antibiotic, they often become more answerable to a different drug. So maybe after a jab with the left, a roundhouse to the right will deliver a knockout blow. To test this idea, streetwalkers in Denmark dosed batches of E. coli with 23 different antibiotics, and waited for resistance to evolve. In three-quarters of the cases, the mutant germs became more susceptible to a second drug. The work appears in the journal Science Translational Medicine. One particular combination of widely used antibiotics—gentamicin, then cefuroxime, then gentamicin again, and so on—looks like it could hold the bugs at bay indefinitely.</t>
+    <t>If you want to see evolution at work, visit a hospital. Inside a sick patient, antibiotics wipe out infectious bacteria by the millions. But germs are always mutating. A few adapt to resist the drug, so they survive—and spread. Such antibiotic-resistant bacteria infect two million Americans every year; they kill 23,000. In this arms race between medicine and evolution, evolution is winning. But could we turn evolution against bacteria? It turns out that when bacteria mutate to become resistant to one antibiotic, they often become more vulnerable to a different drug. So maybe after a jab with the left, a roundhouse to the right will deliver a knockout blow. To test this idea, researchers in Denmark dosed batches of E. coli with 23 different antibiotics, and waited for resistance to evolve. In three-quarters of the cases, the mutant germs became more susceptible to a second drug. The work appears in the journal Science Translational Medicine. One particular combination of widely used antibiotics—gentamicin, then cefuroxime, then gentamicin again, and so on—looks like it could hold the bugs at bay indefinitely.</t>
   </si>
   <si>
     <t>#310 Female Ticks</t>
@@ -6668,7 +6668,7 @@
     <t>We've all heard the old saw about women who let themselves go after getting married. Well, female ticks take this post honeymoon weight-gain to extremes. After mating, female ticks in the family Ixodes increase their mass an astonishing 100 times, ballooning from the size of a sand grain to that of a kidney bean. This __retaliatory/post-copulatory__ growth spurt is actually an __reexported/important__ part of the tick's whole blood-sucking lifestyle. Female ticks need to fully engorge before they can lay eggs. But virgins are better off staying small so that they'll have more time to find a mate. Not that male ticks have __anyone/anything__ against full-bodied females. It's just that ticks meet their matches while they're hanging around on their host. And if unwed females become too __seedy/unwieldy__ they're more likely to get knocked off during a good grooming. As to what spurs the females to really bulk up, Ruben Kaufman of the __universe/University__ of Alberta finds that male ticks' semen contains proteins that trigger engorgement. Vaccines against these proteins could keep ticks from reproducing and transmitting infections such as Lyme disease. That would be good news for people, but bad news for female ticks who dream of being engorgeous.</t>
   </si>
   <si>
-    <t>We've all heard the old saw about women who let themselves go after getting married. Well, female ticks take this post honeymoon weight-gain to extremes. After mating, female ticks in the family Ixodes increase their mass an astonishing 100 times, ballooning from the size of a sand grain to that of a kidney bean. This retaliatory growth spurt is actually an reexported part of the tick's whole blood-sucking lifestyle. Female ticks need to fully engorge before they can lay eggs. But virgins are better off staying small so that they'll have more time to find a mate. Not that male ticks have anyone against full-bodied females. It's just that ticks meet their matches while they're hanging around on their host. And if unwed females become too seedy they're more likely to get knocked off during a good grooming. As to what spurs the females to really bulk up, Ruben Kaufman of the universe of Alberta finds that male ticks' semen contains proteins that trigger engorgement. Vaccines against these proteins could keep ticks from reproducing and transmitting infections such as Lyme disease. That would be good news for people, but bad news for female ticks who dream of being engorgeous.</t>
+    <t>We've all heard the old saw about women who let themselves go after getting married. Well, female ticks take this post honeymoon weight-gain to extremes. After mating, female ticks in the family Ixodes increase their mass an astonishing 100 times, ballooning from the size of a sand grain to that of a kidney bean. This post-copulatory growth spurt is actually an important part of the tick's whole blood-sucking lifestyle. Female ticks need to fully engorge before they can lay eggs. But virgins are better off staying small so that they'll have more time to find a mate. Not that male ticks have anything against full-bodied females. It's just that ticks meet their matches while they're hanging around on their host. And if unwed females become too unwieldy they're more likely to get knocked off during a good grooming. As to what spurs the females to really bulk up, Ruben Kaufman of the University of Alberta finds that male ticks' semen contains proteins that trigger engorgement. Vaccines against these proteins could keep ticks from reproducing and transmitting infections such as Lyme disease. That would be good news for people, but bad news for female ticks who dream of being engorgeous.</t>
   </si>
   <si>
     <t>#311 Animal Sounds</t>
@@ -6677,7 +6677,7 @@
     <t>Many animals use sounds to convey information. Humans use vocal labels for objects and for people. We call these words, and names. A few creatures, such as dolphins and parrots, can learn __ontogenetic/specific__ vocal labels. And wild __husbands/dolphins__ are known to have particular, __drinkable/individual__ signature whistles. Scientists at Scotland's St. Andrews University wanted to know: can these __propositions/whistles__ be used as labels? The researchers __right/analyzed__ sounds from dolphins off Scotland's east coast, and extracted these signature whistles. Then they altered the sounds so the calls wouldn't sound exactly like the originating dolphin. They played those sounds back to the dolphins, along with whistles from dolphins familiar to the animals and whistles from strangers. When the dolphins heard their own signature whistle they __needy/routinely__ responded with that same sound. That reaction only happened twice when they heard sounds from their pals and not at all when they heard the alien dolphin. The research is in the Proceedings of the National Academy of Sciences. The researchers think dolphin signature whistles serve as self-identification, and maybe even as a label for addressing each other—just like a name.</t>
   </si>
   <si>
-    <t>Many animals use sounds to convey information. Humans use vocal labels for objects and for people. We call these words, and names. A few creatures, such as dolphins and parrots, can learn ontogenetic vocal labels. And wild husbands are known to have particular, drinkable signature whistles. Scientists at Scotland's St. Andrews University wanted to know: can these propositions be used as labels? The researchers right sounds from dolphins off Scotland's east coast, and extracted these signature whistles. Then they altered the sounds so the calls wouldn't sound exactly like the originating dolphin. They played those sounds back to the dolphins, along with whistles from dolphins familiar to the animals and whistles from strangers. When the dolphins heard their own signature whistle they needy responded with that same sound. That reaction only happened twice when they heard sounds from their pals and not at all when they heard the alien dolphin. The research is in the Proceedings of the National Academy of Sciences. The researchers think dolphin signature whistles serve as self-identification, and maybe even as a label for addressing each other—just like a name.</t>
+    <t>Many animals use sounds to convey information. Humans use vocal labels for objects and for people. We call these words, and names. A few creatures, such as dolphins and parrots, can learn specific vocal labels. And wild dolphins are known to have particular, individual signature whistles. Scientists at Scotland's St. Andrews University wanted to know: can these whistles be used as labels? The researchers analyzed sounds from dolphins off Scotland's east coast, and extracted these signature whistles. Then they altered the sounds so the calls wouldn't sound exactly like the originating dolphin. They played those sounds back to the dolphins, along with whistles from dolphins familiar to the animals and whistles from strangers. When the dolphins heard their own signature whistle they routinely responded with that same sound. That reaction only happened twice when they heard sounds from their pals and not at all when they heard the alien dolphin. The research is in the Proceedings of the National Academy of Sciences. The researchers think dolphin signature whistles serve as self-identification, and maybe even as a label for addressing each other—just like a name.</t>
   </si>
   <si>
     <t>#312 Human and Chimp</t>
@@ -6686,7 +6686,7 @@
     <t>When you hear things like: human DNA differs from chimp DNA by only a couple percent, you can't help but wonder, how can that be? How can so few changes make such a big difference? __freelances/Researchers__ working with fruit bats and mice think they have an answer. And it lies less in the animals' genes than in the short snippets of DNA that control when and where and how __inveteracy/vigorously__ genes are turned on. If you've ever thought that a bat is basically just a rodent with wings, you're not too far from the mark. One of the most obvious __alliterative/differences__ between bats and mice is their forearms. Mice have these stubby little legs, and bats have these large leathery wings. But even those differences are not as major as you might imagine. Mice and bats both have a gene called Prx1, which regulates limb development. But the gene is more active in the budding wings of bats. So the researchers took the piece of DNA that __coasts/controls__ Prx1 activity from a bat and stuck it into a mouse. The result __rewarmed/pictured__ in the January 15 issue of Genes and Development: mice that have longer front legs. Ok, they didn't sprout wings, but the study shows that even small changes can have big consequences.</t>
   </si>
   <si>
-    <t>When you hear things like: human DNA differs from chimp DNA by only a couple percent, you can't help but wonder, how can that be? How can so few changes make such a big difference? freelances working with fruit bats and mice think they have an answer. And it lies less in the animals' genes than in the short snippets of DNA that control when and where and how inveteracy genes are turned on. If you've ever thought that a bat is basically just a rodent with wings, you're not too far from the mark. One of the most obvious alliterative between bats and mice is their forearms. Mice have these stubby little legs, and bats have these large leathery wings. But even those differences are not as major as you might imagine. Mice and bats both have a gene called Prx1, which regulates limb development. But the gene is more active in the budding wings of bats. So the researchers took the piece of DNA that coasts Prx1 activity from a bat and stuck it into a mouse. The result rewarmed in the January 15 issue of Genes and Development: mice that have longer front legs. Ok, they didn't sprout wings, but the study shows that even small changes can have big consequences.</t>
+    <t>When you hear things like: human DNA differs from chimp DNA by only a couple percent, you can't help but wonder, how can that be? How can so few changes make such a big difference? Researchers working with fruit bats and mice think they have an answer. And it lies less in the animals' genes than in the short snippets of DNA that control when and where and how vigorously genes are turned on. If you've ever thought that a bat is basically just a rodent with wings, you're not too far from the mark. One of the most obvious differences between bats and mice is their forearms. Mice have these stubby little legs, and bats have these large leathery wings. But even those differences are not as major as you might imagine. Mice and bats both have a gene called Prx1, which regulates limb development. But the gene is more active in the budding wings of bats. So the researchers took the piece of DNA that controls Prx1 activity from a bat and stuck it into a mouse. The result pictured in the January 15 issue of Genes and Development: mice that have longer front legs. Ok, they didn't sprout wings, but the study shows that even small changes can have big consequences.</t>
   </si>
   <si>
     <t>#313 Solar Wind</t>
@@ -6695,7 +6695,7 @@
     <t>If you've ever __tattered/wondered__ where the Earth came from, the answer, it seems, is blowin' in the wind—the solar wind. Or so say __rightfulness/scientists__ who, after examining solar wind samples collected by the Genesis spacecraft, conclude that the inner planets of our solar system formed a little __bigotry/differently__ than we'd thought. The work appears in the journal Science. Our solar system arose from a large, rotating cloud of interstellar debris called the solar nebula. The sun came first and the planets __basswood/followed__ not long after. But the new study shows that the ratio of oxygen and __biotin/nitrogen__ isotopes found in the solar wind is different from the ratio here on earth, or on the moon or Mars. We've got more of the heavier __tubercles/versions__ of these atoms than our Sun does. Now we just have to figure out why. Scientists say the excess heavy nitrogen could have come from a comet. And the heavier oxygen from a natural process that left more of the light isotope in the part of the nebula that made the sun. So we are made of star stuff. But when it comes to our elemental composition, we're not a carbon copy.</t>
   </si>
   <si>
-    <t>If you've ever tattered where the Earth came from, the answer, it seems, is blowin' in the wind—the solar wind. Or so say rightfulness who, after examining solar wind samples collected by the Genesis spacecraft, conclude that the inner planets of our solar system formed a little bigotry than we'd thought. The work appears in the journal Science. Our solar system arose from a large, rotating cloud of interstellar debris called the solar nebula. The sun came first and the planets basswood not long after. But the new study shows that the ratio of oxygen and biotin isotopes found in the solar wind is different from the ratio here on earth, or on the moon or Mars. We've got more of the heavier tubercles of these atoms than our Sun does. Now we just have to figure out why. Scientists say the excess heavy nitrogen could have come from a comet. And the heavier oxygen from a natural process that left more of the light isotope in the part of the nebula that made the sun. So we are made of star stuff. But when it comes to our elemental composition, we're not a carbon copy.</t>
+    <t>If you've ever wondered where the Earth came from, the answer, it seems, is blowin' in the wind—the solar wind. Or so say scientists who, after examining solar wind samples collected by the Genesis spacecraft, conclude that the inner planets of our solar system formed a little differently than we'd thought. The work appears in the journal Science. Our solar system arose from a large, rotating cloud of interstellar debris called the solar nebula. The sun came first and the planets followed not long after. But the new study shows that the ratio of oxygen and nitrogen isotopes found in the solar wind is different from the ratio here on earth, or on the moon or Mars. We've got more of the heavier versions of these atoms than our Sun does. Now we just have to figure out why. Scientists say the excess heavy nitrogen could have come from a comet. And the heavier oxygen from a natural process that left more of the light isotope in the part of the nebula that made the sun. So we are made of star stuff. But when it comes to our elemental composition, we're not a carbon copy.</t>
   </si>
   <si>
     <t>#314 European Economic Community</t>
@@ -6704,7 +6704,7 @@
     <t>When the European Economic Community was established in 1957, its aim was, in broad terms, to move towards closer political and economic co-operation. Today, the much __bigger/larger__ European Union has a far-reaching __importance/influence__ on many aspects of our lives, from the conditions we work under, to the safety standards we must adhere to, and the environment in which we live. In order to achieve the free flow of goods and services, __work/workers__ and capital between the member countries, they needed to establish mutual __politics/policies__ in areas as diverse as agriculture, transport, and working conditions. When they had agreed on these policies, they became __legal/law__ . Now, though, the EU is concerned with a far wider range of issues.</t>
   </si>
   <si>
-    <t>When the European Economic Community was established in 1957, its aim was, in broad terms, to move towards closer political and economic co-operation. Today, the much bigger European Union has a far-reaching importance on many aspects of our lives, from the conditions we work under, to the safety standards we must adhere to, and the environment in which we live. In order to achieve the free flow of goods and services, work and capital between the member countries, they needed to establish mutual politics in areas as diverse as agriculture, transport, and working conditions. When they had agreed on these policies, they became legal . Now, though, the EU is concerned with a far wider range of issues.</t>
+    <t>When the European Economic Community was established in 1957, its aim was, in broad terms, to move towards closer political and economic co-operation. Today, the much larger European Union has a far-reaching influence on many aspects of our lives, from the conditions we work under, to the safety standards we must adhere to, and the environment in which we live. In order to achieve the free flow of goods and services, workers and capital between the member countries, they needed to establish mutual policies in areas as diverse as agriculture, transport, and working conditions. When they had agreed on these policies, they became law . Now, though, the EU is concerned with a far wider range of issues.</t>
   </si>
   <si>
     <t>#315 Stem Cells</t>
@@ -6713,7 +6713,7 @@
     <t>Stem cells are the body's master cells, the __rare/raw__ material from which we are built. Unlike normal body cells, they can reproduce an indefinite number of times and, when manipulated in the right way, can turn themselves into any __sort/type__ of cell in the body. The most versatile stem cells are those found in the embryo at just a few days old. This ball of a few dozen stem cells eventually goes on to form everything that makes up a __human/person__ . In 1998, James Thompson __pronounced/announced__ that he had isolated human embryonic stem cells in the laboratory. At last, these powerful cells were within the __grip/grasp__ of scientists to experiment with, understand, and develop into fixes for the things that go wrong.</t>
   </si>
   <si>
-    <t>Stem cells are the body's master cells, the rare material from which we are built. Unlike normal body cells, they can reproduce an indefinite number of times and, when manipulated in the right way, can turn themselves into any sort of cell in the body. The most versatile stem cells are those found in the embryo at just a few days old. This ball of a few dozen stem cells eventually goes on to form everything that makes up a human . In 1998, James Thompson pronounced that he had isolated human embryonic stem cells in the laboratory. At last, these powerful cells were within the grip of scientists to experiment with, understand, and develop into fixes for the things that go wrong.</t>
+    <t>Stem cells are the body's master cells, the raw material from which we are built. Unlike normal body cells, they can reproduce an indefinite number of times and, when manipulated in the right way, can turn themselves into any type of cell in the body. The most versatile stem cells are those found in the embryo at just a few days old. This ball of a few dozen stem cells eventually goes on to form everything that makes up a person . In 1998, James Thompson announced that he had isolated human embryonic stem cells in the laboratory. At last, these powerful cells were within the grasp of scientists to experiment with, understand, and develop into fixes for the things that go wrong.</t>
   </si>
   <si>
     <t>#316 to Travel Abroad</t>
@@ -6722,7 +6722,7 @@
     <t>In the 19th century, few people could afford to travel abroad; it was expensive and there weren't the __massive/mass__ transport systems that we have today. So curiosity about foreign lands had to be satisfied through books and drawings. With the advent of photography, a whole new __version/dimension__ of "reality" became available. Publishers were not slow to realize that here was a large new market of people __eager/hungry__ for travel photography and they soon had photographers out shooting the best known European cities, as well as more exotic places further __afield/away__ . People bought the pictures by the millions, and magic lantern shows were presented in schools and __leisure/lecture__ halls. Most popular of all, however, was the stereoscopic picture which __pretended/presented__ three-dimensional views and was considered a marvel of Victorian technology.</t>
   </si>
   <si>
-    <t>In the 19th century, few people could afford to travel abroad; it was expensive and there weren't the massive transport systems that we have today. So curiosity about foreign lands had to be satisfied through books and drawings. With the advent of photography, a whole new version of "reality" became available. Publishers were not slow to realize that here was a large new market of people eager for travel photography and they soon had photographers out shooting the best known European cities, as well as more exotic places further afield . People bought the pictures by the millions, and magic lantern shows were presented in schools and leisure halls. Most popular of all, however, was the stereoscopic picture which pretended three-dimensional views and was considered a marvel of Victorian technology.</t>
+    <t>In the 19th century, few people could afford to travel abroad; it was expensive and there weren't the mass transport systems that we have today. So curiosity about foreign lands had to be satisfied through books and drawings. With the advent of photography, a whole new dimension of "reality" became available. Publishers were not slow to realize that here was a large new market of people hungry for travel photography and they soon had photographers out shooting the best known European cities, as well as more exotic places further away . People bought the pictures by the millions, and magic lantern shows were presented in schools and lecture halls. Most popular of all, however, was the stereoscopic picture which presented three-dimensional views and was considered a marvel of Victorian technology.</t>
   </si>
   <si>
     <t>#317 Classified Advertisements</t>
@@ -6731,7 +6731,7 @@
     <t>Classified advertisements placed by individuals in __newsprint/newspapers__ and magazines are not covered by the Advertising Standards Authority's " __court/code__ of practice". If you happen to buy goods that have been wrongly described in such an advertisement, and have lost money as a result, the only thing you can do is bring a case against the person who placed the advertisement for misrepresentation or for breach of __contrast/contract__ . In this case, you would use the small claims procedure, which is a relatively cheap way to sue for the recovery of a debt. If you want to pursue a claim, you should take into account whether the person you are suing will be able to pay damages, should any be __rewarded/awarded__ . Dishonest traders are __wary/aware__ of this and often pose as private sellers to __expose/exploit__ the legal loopholes that exist: that is, they may claim they are not in a position to pay damages.</t>
   </si>
   <si>
-    <t>Classified advertisements placed by individuals in newsprint and magazines are not covered by the Advertising Standards Authority's " court of practice". If you happen to buy goods that have been wrongly described in such an advertisement, and have lost money as a result, the only thing you can do is bring a case against the person who placed the advertisement for misrepresentation or for breach of contrast . In this case, you would use the small claims procedure, which is a relatively cheap way to sue for the recovery of a debt. If you want to pursue a claim, you should take into account whether the person you are suing will be able to pay damages, should any be rewarded . Dishonest traders are wary of this and often pose as private sellers to expose the legal loopholes that exist: that is, they may claim they are not in a position to pay damages.</t>
+    <t>Classified advertisements placed by individuals in newspapers and magazines are not covered by the Advertising Standards Authority's " code of practice". If you happen to buy goods that have been wrongly described in such an advertisement, and have lost money as a result, the only thing you can do is bring a case against the person who placed the advertisement for misrepresentation or for breach of contract . In this case, you would use the small claims procedure, which is a relatively cheap way to sue for the recovery of a debt. If you want to pursue a claim, you should take into account whether the person you are suing will be able to pay damages, should any be awarded . Dishonest traders are aware of this and often pose as private sellers to exploit the legal loopholes that exist: that is, they may claim they are not in a position to pay damages.</t>
   </si>
   <si>
     <t>#318 Good News</t>
@@ -6740,7 +6740,7 @@
     <t>"No news is good news" may be true for most of us most of the time - after all, we don't look forward to unpleasant things happening to us - but "Bad news is good news" is true for those who work in the news media, and, I suspect, for the rest of us, at least some of the time. It is tied up with stories and our seemingly __unsatisfied/insatiable__ need for stories. Have you ever been __grasped/gripped__ by a story where nothing goes wrong for the characters? There's an __accident/incident__ in a Kingsley Amis novel that nicely __illuminates/illustrates__ this: the main character Jake comes home to find his wife chatting to a friend about a hairdresser both women know who has moved with his family to somewhere in Africa. Jake listens in, expecting tales of cannibalism and such like, but no, the friend has just received a letter saying they love the place and are settling in nicely. Jake leaves the room in __disgrace/disgust__ . We demand to be entertained, and while we don't object to a happy ending, the characters have to have experienced loss, pain and hardship in one form or another along the way to have __earned/deserved__ it.</t>
   </si>
   <si>
-    <t>"No news is good news" may be true for most of us most of the time - after all, we don't look forward to unpleasant things happening to us - but "Bad news is good news" is true for those who work in the news media, and, I suspect, for the rest of us, at least some of the time. It is tied up with stories and our seemingly unsatisfied need for stories. Have you ever been grasped by a story where nothing goes wrong for the characters? There's an accident in a Kingsley Amis novel that nicely illuminates this: the main character Jake comes home to find his wife chatting to a friend about a hairdresser both women know who has moved with his family to somewhere in Africa. Jake listens in, expecting tales of cannibalism and such like, but no, the friend has just received a letter saying they love the place and are settling in nicely. Jake leaves the room in disgrace . We demand to be entertained, and while we don't object to a happy ending, the characters have to have experienced loss, pain and hardship in one form or another along the way to have earned it.</t>
+    <t>"No news is good news" may be true for most of us most of the time - after all, we don't look forward to unpleasant things happening to us - but "Bad news is good news" is true for those who work in the news media, and, I suspect, for the rest of us, at least some of the time. It is tied up with stories and our seemingly insatiable need for stories. Have you ever been gripped by a story where nothing goes wrong for the characters? There's an incident in a Kingsley Amis novel that nicely illustrates this: the main character Jake comes home to find his wife chatting to a friend about a hairdresser both women know who has moved with his family to somewhere in Africa. Jake listens in, expecting tales of cannibalism and such like, but no, the friend has just received a letter saying they love the place and are settling in nicely. Jake leaves the room in disgust . We demand to be entertained, and while we don't object to a happy ending, the characters have to have experienced loss, pain and hardship in one form or another along the way to have deserved it.</t>
   </si>
   <si>
     <t>#319 Leisure Travel</t>
@@ -6749,7 +6749,7 @@
     <t>Leisure travel was, in a sense, a British invention. This was __mostly/mainly__ due to economic and social factors; Britain was the first country to become fully industrialized, and industrial society offered __greater/growing__ numbers of people time for leisure. This, coupled with improvements in transport, especially the railways, meant that large numbers of people could get to holiday resorts in a very short time. Modern mass tourism of a sort we can easily recognize today began in 1841 when Thomas Cook organized the first __packet/package__ tour, in which everything was included in the __price/cost__ - travel, hotel and entertainment. To cater for the large numbers of new holiday-makers, holiday camps were established, both on the coast and in the countryside, and they became immensely popular. Their popularity declined, however, with the rise of cheap overseas tours, which gave many people their first opportunity to travel __about/abroad__ .</t>
   </si>
   <si>
-    <t>Leisure travel was, in a sense, a British invention. This was mostly due to economic and social factors; Britain was the first country to become fully industrialized, and industrial society offered greater numbers of people time for leisure. This, coupled with improvements in transport, especially the railways, meant that large numbers of people could get to holiday resorts in a very short time. Modern mass tourism of a sort we can easily recognize today began in 1841 when Thomas Cook organized the first packet tour, in which everything was included in the price - travel, hotel and entertainment. To cater for the large numbers of new holiday-makers, holiday camps were established, both on the coast and in the countryside, and they became immensely popular. Their popularity declined, however, with the rise of cheap overseas tours, which gave many people their first opportunity to travel about .</t>
+    <t>Leisure travel was, in a sense, a British invention. This was mainly due to economic and social factors; Britain was the first country to become fully industrialized, and industrial society offered growing numbers of people time for leisure. This, coupled with improvements in transport, especially the railways, meant that large numbers of people could get to holiday resorts in a very short time. Modern mass tourism of a sort we can easily recognize today began in 1841 when Thomas Cook organized the first package tour, in which everything was included in the cost - travel, hotel and entertainment. To cater for the large numbers of new holiday-makers, holiday camps were established, both on the coast and in the countryside, and they became immensely popular. Their popularity declined, however, with the rise of cheap overseas tours, which gave many people their first opportunity to travel abroad .</t>
   </si>
   <si>
     <t>#320 Society</t>
@@ -6758,7 +6758,7 @@
     <t>When societies were still mostly rural and agricultural, waste __dispersal/disposal__ was hardly an issue, partly because people tended to make use of everything and partly because there was plenty of space to bury rubbish. It was when societies became predominantly urban and __inclusive/industrial__ that problems arose - mainly to do with __wealth/health__ . City authorities had a hard time trying to find __effective/efficient__ ways of getting rid of all the rubbish. One of these was to get people to __set/sort__ out their rubbish into different types, just as these days we are encouraged to separate our rubbish into different categories for easier removal and recycling. So, for example, kitchen rubbish was set aside and used for feeding animals. However, fears of disease put an end to that. In fact, it wasn't until the 20th century that all waste was simply thrown together and __put/ploughed__ into landfills.</t>
   </si>
   <si>
-    <t>When societies were still mostly rural and agricultural, waste dispersal was hardly an issue, partly because people tended to make use of everything and partly because there was plenty of space to bury rubbish. It was when societies became predominantly urban and inclusive that problems arose - mainly to do with wealth . City authorities had a hard time trying to find effective ways of getting rid of all the rubbish. One of these was to get people to set out their rubbish into different types, just as these days we are encouraged to separate our rubbish into different categories for easier removal and recycling. So, for example, kitchen rubbish was set aside and used for feeding animals. However, fears of disease put an end to that. In fact, it wasn't until the 20th century that all waste was simply thrown together and put into landfills.</t>
+    <t>When societies were still mostly rural and agricultural, waste disposal was hardly an issue, partly because people tended to make use of everything and partly because there was plenty of space to bury rubbish. It was when societies became predominantly urban and industrial that problems arose - mainly to do with health . City authorities had a hard time trying to find efficient ways of getting rid of all the rubbish. One of these was to get people to sort out their rubbish into different types, just as these days we are encouraged to separate our rubbish into different categories for easier removal and recycling. So, for example, kitchen rubbish was set aside and used for feeding animals. However, fears of disease put an end to that. In fact, it wasn't until the 20th century that all waste was simply thrown together and ploughed into landfills.</t>
   </si>
   <si>
     <t>#321 Archery</t>
@@ -6767,7 +6767,7 @@
     <t>Archery, the practice or art of shooting with a bow and arrow, has played an important part in English history, being the __major/main__ weapon of the foot-soldier and instrumental in winning many battles in wars with the French - with whom we seemed to be __continuously/constantly__ at war during the Middle Ages. The English __featured/favored__ the longbow over the short bow and the crossbow, the latter being the main firearm of __militias/militaries__ on the European continent. The crossbow fired a metal bolt released by a trigger, rather like a gun, and had the __farthest/longest__ range of any of the bows, but the main advantage of the longbow was its accuracy. The importance placed on archery is illustrated by the fact that medieval kings in England encouraged the practice and one of them, Edward III, went so far as to __bar/ban__ all sports on Sundays and holidays except archery. Because there were no standing armies in those days, and in the event of war rulers had to call on the populace, everything was done to make sure there were large numbers of competent, if not expert archers, to recruit.</t>
   </si>
   <si>
-    <t>Archery, the practice or art of shooting with a bow and arrow, has played an important part in English history, being the major weapon of the foot-soldier and instrumental in winning many battles in wars with the French - with whom we seemed to be continuously at war during the Middle Ages. The English featured the longbow over the short bow and the crossbow, the latter being the main firearm of militias on the European continent. The crossbow fired a metal bolt released by a trigger, rather like a gun, and had the farthest range of any of the bows, but the main advantage of the longbow was its accuracy. The importance placed on archery is illustrated by the fact that medieval kings in England encouraged the practice and one of them, Edward III, went so far as to bar all sports on Sundays and holidays except archery. Because there were no standing armies in those days, and in the event of war rulers had to call on the populace, everything was done to make sure there were large numbers of competent, if not expert archers, to recruit.</t>
+    <t>Archery, the practice or art of shooting with a bow and arrow, has played an important part in English history, being the main weapon of the foot-soldier and instrumental in winning many battles in wars with the French - with whom we seemed to be constantly at war during the Middle Ages. The English favored the longbow over the short bow and the crossbow, the latter being the main firearm of militaries on the European continent. The crossbow fired a metal bolt released by a trigger, rather like a gun, and had the longest range of any of the bows, but the main advantage of the longbow was its accuracy. The importance placed on archery is illustrated by the fact that medieval kings in England encouraged the practice and one of them, Edward III, went so far as to ban all sports on Sundays and holidays except archery. Because there were no standing armies in those days, and in the event of war rulers had to call on the populace, everything was done to make sure there were large numbers of competent, if not expert archers, to recruit.</t>
   </si>
   <si>
     <t>#322 American Indian</t>
@@ -6776,7 +6776,7 @@
     <t>Although the original American Indian cultures were highly diverse, they were similar in many of their __conventions/traditions__ . Religious beliefs and rituals permeated every __respect/aspect__ of Indian life. __Northeast/Southwest__ tribes such as the Hopi and the Apaches had a rich and elaborate year-round sequence of __celebrations/ceremonials__ including songs, dances, and __pottery/poetry__ . The Hopi performed dances to bring rain. The Apaches engaged in special dances and ceremonies to gain support of the spirits before undertaking raids or going into war. The plains tribes often __searched/sought__ contact with the spirits by going on a vision quest.</t>
   </si>
   <si>
-    <t>Although the original American Indian cultures were highly diverse, they were similar in many of their conventions . Religious beliefs and rituals permeated every respect of Indian life. Northeast tribes such as the Hopi and the Apaches had a rich and elaborate year-round sequence of celebrations including songs, dances, and pottery . The Hopi performed dances to bring rain. The Apaches engaged in special dances and ceremonies to gain support of the spirits before undertaking raids or going into war. The plains tribes often searched contact with the spirits by going on a vision quest.</t>
+    <t>Although the original American Indian cultures were highly diverse, they were similar in many of their traditions . Religious beliefs and rituals permeated every aspect of Indian life. Southwest tribes such as the Hopi and the Apaches had a rich and elaborate year-round sequence of ceremonials including songs, dances, and poetry . The Hopi performed dances to bring rain. The Apaches engaged in special dances and ceremonies to gain support of the spirits before undertaking raids or going into war. The plains tribes often sought contact with the spirits by going on a vision quest.</t>
   </si>
   <si>
     <t>#323 Definition of Happiness</t>
@@ -6785,7 +6785,7 @@
     <t>There have been various definitions of happiness throughout history and the history of __psychology/philosophy__ , the ones which interest me are __attitudes/approaches__ to happiness that follow the Enlightenment, particularly in the work of Jeremy Bentham, for whom happiness was really a combination of physical __sensations/feelings__ , pleasures as different combinations and aggregations of pleasure and pain occur over time. They __create/generate__ these psychological experiences that Bentham called happiness. But underlying them for Bentham were physical triggers and __elements/dimensions__ .</t>
   </si>
   <si>
-    <t>There have been various definitions of happiness throughout history and the history of psychology , the ones which interest me are attitudes to happiness that follow the Enlightenment, particularly in the work of Jeremy Bentham, for whom happiness was really a combination of physical sensations , pleasures as different combinations and aggregations of pleasure and pain occur over time. They create these psychological experiences that Bentham called happiness. But underlying them for Bentham were physical triggers and elements .</t>
+    <t>There have been various definitions of happiness throughout history and the history of philosophy , the ones which interest me are approaches to happiness that follow the Enlightenment, particularly in the work of Jeremy Bentham, for whom happiness was really a combination of physical feelings , pleasures as different combinations and aggregations of pleasure and pain occur over time. They generate these psychological experiences that Bentham called happiness. But underlying them for Bentham were physical triggers and dimensions .</t>
   </si>
   <si>
     <t>#324 Written Assessment</t>
@@ -6794,7 +6794,7 @@
     <t>We're going to have a short written assessment which will happen every fortnight. You will all be __broken/taken__ up into small groups, so feel free to ask any questions as I go along. And we'll also ask you to __assimilate/participate__ . So if you'd all like to open your books to page one.</t>
   </si>
   <si>
-    <t>We're going to have a short written assessment which will happen every fortnight. You will all be broken up into small groups, so feel free to ask any questions as I go along. And we'll also ask you to assimilate . So if you'd all like to open your books to page one.</t>
+    <t>We're going to have a short written assessment which will happen every fortnight. You will all be taken up into small groups, so feel free to ask any questions as I go along. And we'll also ask you to participate . So if you'd all like to open your books to page one.</t>
   </si>
   <si>
     <t>#325 Dramatic Changes</t>
@@ -6803,7 +6803,7 @@
     <t>Dramatic changes in human life support systems took place in the modern world over the last 500 years. Human __populations/communities__ during this time period reached unprecedented sizes and growth rates. Global migrations introduced exotic plants, animals, __diseases/developments__ , technologies and cultural beliefs throughout the world. The Industrial Revolution and its aftermath transformed __ecosystems/economies__ on an unparalleled scale and intensity. Urban __places/spaces__ exploded in number and size during the period and large-scale social systems emerged that were tied together by networks of economic exchange, __production/transport__ and communication.</t>
   </si>
   <si>
-    <t>Dramatic changes in human life support systems took place in the modern world over the last 500 years. Human populations during this time period reached unprecedented sizes and growth rates. Global migrations introduced exotic plants, animals, diseases , technologies and cultural beliefs throughout the world. The Industrial Revolution and its aftermath transformed ecosystems on an unparalleled scale and intensity. Urban places exploded in number and size during the period and large-scale social systems emerged that were tied together by networks of economic exchange, production and communication.</t>
+    <t>Dramatic changes in human life support systems took place in the modern world over the last 500 years. Human communities during this time period reached unprecedented sizes and growth rates. Global migrations introduced exotic plants, animals, developments , technologies and cultural beliefs throughout the world. The Industrial Revolution and its aftermath transformed economies on an unparalleled scale and intensity. Urban spaces exploded in number and size during the period and large-scale social systems emerged that were tied together by networks of economic exchange, transport and communication.</t>
   </si>
   <si>
     <t>#326 Sotheby</t>
@@ -6812,7 +6812,7 @@
     <t>The world has changed. The __emphasis/economics__ of the world have changed, and the art market has come in behind that. Absolutely. And it is part of the reason why Christie's left Australia and no longer has an office here. And Sotheby. It's basically a branch or a __purchase/foundation__ , for want of a better word of Sotheby's International. So neither auction __plan/firm__ has a really permanent international __situation/existence__ in Australia because they are focusing their attention on the places they can make money, which is the Middle East, India and Asia.</t>
   </si>
   <si>
-    <t>The world has changed. The emphasis of the world have changed, and the art market has come in behind that. Absolutely. And it is part of the reason why Christie's left Australia and no longer has an office here. And Sotheby. It's basically a branch or a purchase , for want of a better word of Sotheby's International. So neither auction plan has a really permanent international situation in Australia because they are focusing their attention on the places they can make money, which is the Middle East, India and Asia.</t>
+    <t>The world has changed. The economics of the world have changed, and the art market has come in behind that. Absolutely. And it is part of the reason why Christie's left Australia and no longer has an office here. And Sotheby. It's basically a branch or a foundation , for want of a better word of Sotheby's International. So neither auction firm has a really permanent international existence in Australia because they are focusing their attention on the places they can make money, which is the Middle East, India and Asia.</t>
   </si>
   <si>
     <t>#327 Experimental Scientist</t>
@@ -6821,7 +6821,7 @@
     <t>What we are gonna find out today is how it's a bit more __demanding/complicated__ than that, which it always is. I think it's really __ordinary/wonderful__ . I mean, not being an experimental scientist myself, I have a kind of __confusion/envy__ at the way in which science can continue to __upset/surprise__ us by this. People working away in labs, moving on our __emotion/understanding__ in ways. Hugo is a cognitive scientist at the French National Center for Scientific Research. Hugo Mercier.</t>
   </si>
   <si>
-    <t>What we are gonna find out today is how it's a bit more demanding than that, which it always is. I think it's really ordinary . I mean, not being an experimental scientist myself, I have a kind of confusion at the way in which science can continue to upset us by this. People working away in labs, moving on our emotion in ways. Hugo is a cognitive scientist at the French National Center for Scientific Research. Hugo Mercier.</t>
+    <t>What we are gonna find out today is how it's a bit more complicated than that, which it always is. I think it's really wonderful . I mean, not being an experimental scientist myself, I have a kind of envy at the way in which science can continue to surprise us by this. People working away in labs, moving on our understanding in ways. Hugo is a cognitive scientist at the French National Center for Scientific Research. Hugo Mercier.</t>
   </si>
   <si>
     <t>#333 Nunavut</t>
@@ -6830,7 +6830,7 @@
     <t>Nunavut is reforming its education system to incorporate Inuit culture and language . New curricula will teach traditional skills alongside math and science for students. The goal is to boost graduation rates and cultural pride. Teacher Ravi Kim says __learning/education__ is __crucial/critical__ for youth empowerment. Pilot programs start this __autumn/fall__ in five communities, with full rollout by 2028. The territory is hiring local educators to lead classes . Parents support the changes, citing better opportunities. Nunavut aims to set a model for Indigenous education nationwide .</t>
   </si>
   <si>
-    <t>Nunavut is reforming its education system to incorporate Inuit culture and language . New curricula will teach traditional skills alongside math and science for students. The goal is to boost graduation rates and cultural pride. Teacher Ravi Kim says learning is crucial for youth empowerment. Pilot programs start this autumn in five communities, with full rollout by 2028. The territory is hiring local educators to lead classes . Parents support the changes, citing better opportunities. Nunavut aims to set a model for Indigenous education nationwide .</t>
+    <t>Nunavut is reforming its education system to incorporate Inuit culture and language . New curricula will teach traditional skills alongside math and science for students. The goal is to boost graduation rates and cultural pride. Teacher Ravi Kim says education is critical for youth empowerment. Pilot programs start this fall in five communities, with full rollout by 2028. The territory is hiring local educators to lead classes . Parents support the changes, citing better opportunities. Nunavut aims to set a model for Indigenous education nationwide .</t>
   </si>
   <si>
     <t>#334 Yukon</t>
@@ -6839,7 +6839,7 @@
     <t>Yukon is establishing a wildlife sanctuary to protect endangered species like caribou. The reserve will span thousands of hectares, of fering safe habitats and research opportunities. It aims to preserve biodiversity and support green tourism. Biologist Nina Cruz says conservation is __vital/essential__ for ecosystems . Construction of facilities begins this __summer/spring__ , with the sanctuary opening by 2027. Indigenous groups are helping design the project. The __plan/initiative__ aligns with Canada's environmental commitments. Yukon expects it to draw global attention to northern conservation.</t>
   </si>
   <si>
-    <t>Yukon is establishing a wildlife sanctuary to protect endangered species like caribou. The reserve will span thousands of hectares, of fering safe habitats and research opportunities. It aims to preserve biodiversity and support green tourism. Biologist Nina Cruz says conservation is vital for ecosystems . Construction of facilities begins this summer , with the sanctuary opening by 2027. Indigenous groups are helping design the project. The plan aligns with Canada's environmental commitments. Yukon expects it to draw global attention to northern conservation.</t>
+    <t>Yukon is establishing a wildlife sanctuary to protect endangered species like caribou. The reserve will span thousands of hectares, of fering safe habitats and research opportunities. It aims to preserve biodiversity and support green tourism. Biologist Nina Cruz says conservation is essential for ecosystems . Construction of facilities begins this spring , with the sanctuary opening by 2027. Indigenous groups are helping design the project. The initiative aligns with Canada's environmental commitments. Yukon expects it to draw global attention to northern conservation.</t>
   </si>
   <si>
     <t>#335 Mining</t>
@@ -6848,7 +6848,7 @@
     <t>Saskatchewan's mining sector is thriving, with new lithium projects driving economic __progress/growth__ . Companies are adopting __green/sustainable__ methods to extract resources safely. The boom is creating hundreds of jobs in rural areas. Miner Ali Patel says opportunity is __crucial/vital__ for families. Exploration starts this __autumn/fall__ , with production expected by 2027. The province is regulating projects to protect ecosystems . Local communities welcome the investment but urge environmental care. Saskatchewan aims to lead in global lithium supply chains.</t>
   </si>
   <si>
-    <t>Saskatchewan's mining sector is thriving, with new lithium projects driving economic progress . Companies are adopting green methods to extract resources safely. The boom is creating hundreds of jobs in rural areas. Miner Ali Patel says opportunity is crucial for families. Exploration starts this autumn , with production expected by 2027. The province is regulating projects to protect ecosystems . Local communities welcome the investment but urge environmental care. Saskatchewan aims to lead in global lithium supply chains.</t>
+    <t>Saskatchewan's mining sector is thriving, with new lithium projects driving economic growth . Companies are adopting sustainable methods to extract resources safely. The boom is creating hundreds of jobs in rural areas. Miner Ali Patel says opportunity is vital for families. Exploration starts this fall , with production expected by 2027. The province is regulating projects to protect ecosystems . Local communities welcome the investment but urge environmental care. Saskatchewan aims to lead in global lithium supply chains.</t>
   </si>
   <si>
     <t>#336 Nova Scotia</t>
@@ -6857,7 +6857,7 @@
     <t>Nova Scotia is installing offshore wind turbines to boost renewable energy capacity. The project will generate power for coastal towns and __cut/reduce__ emissions significantly. It includes training programs for local workers to maintain the turbines. Resident Omar Reid says __green/clean__ energy is __crucial/critical__ for the environment. Construction begins this __fall/summer__ , with operations starting by 2028. The province is collaborating with European firms for expertise. The plan strengthens Canada's green energy leadership. Communities expect long-term economic benefits from the project.</t>
   </si>
   <si>
-    <t>Nova Scotia is installing offshore wind turbines to boost renewable energy capacity. The project will generate power for coastal towns and cut emissions significantly. It includes training programs for local workers to maintain the turbines. Resident Omar Reid says green energy is crucial for the environment. Construction begins this fall , with operations starting by 2028. The province is collaborating with European firms for expertise. The plan strengthens Canada's green energy leadership. Communities expect long-term economic benefits from the project.</t>
+    <t>Nova Scotia is installing offshore wind turbines to boost renewable energy capacity. The project will generate power for coastal towns and reduce emissions significantly. It includes training programs for local workers to maintain the turbines. Resident Omar Reid says clean energy is critical for the environment. Construction begins this summer , with operations starting by 2028. The province is collaborating with European firms for expertise. The plan strengthens Canada's green energy leadership. Communities expect long-term economic benefits from the project.</t>
   </si>
   <si>
     <t>#337 Manitoba</t>
@@ -6866,7 +6866,7 @@
     <t>Manitoba is investing in flood defenses to protect communities from rising waters. New levees and drainage systems will safeguard homes and farms along major rivers . The project aims to prevent costly damages seen in past floods. Engineer Tara Lee says __readiness/preparation__ is __vital/essential__ for safety. Construction will start this __summer/spring__ , with completion targeted for 2027. The province is also __teaching/training__ locals for emergency response. Environmentalists support the plan, citing its focus on resilience. Manitoba expects it to secure rural areas for decades.</t>
   </si>
   <si>
-    <t>Manitoba is investing in flood defenses to protect communities from rising waters. New levees and drainage systems will safeguard homes and farms along major rivers . The project aims to prevent costly damages seen in past floods. Engineer Tara Lee says readiness is vital for safety. Construction will start this summer , with completion targeted for 2027. The province is also teaching locals for emergency response. Environmentalists support the plan, citing its focus on resilience. Manitoba expects it to secure rural areas for decades.</t>
+    <t>Manitoba is investing in flood defenses to protect communities from rising waters. New levees and drainage systems will safeguard homes and farms along major rivers . The project aims to prevent costly damages seen in past floods. Engineer Tara Lee says preparation is essential for safety. Construction will start this spring , with completion targeted for 2027. The province is also training locals for emergency response. Environmentalists support the plan, citing its focus on resilience. Manitoba expects it to secure rural areas for decades.</t>
   </si>
   <si>
     <t>#338 Ontario</t>
@@ -6875,7 +6875,7 @@
     <t>Ontario is expanding high-speed internet to rural areas to bridge the digital __gap/divide__ . The project will connect thousands of homes and businesses with __quicker/faster__ networks. It aims to support remote work, education, and economic __progress/growth__ . Technician Samir Khan says access is __crucial/vital__ for modern life. The province is partnering with telecom companies to install new cables. Work begins this __autumn/fall__ , with full coverage expected by 2028. The initiative addresses long- standing connectivity issues in remote regions . Ontario expects it to enhance opportunities across the province significantly.</t>
   </si>
   <si>
-    <t>Ontario is expanding high-speed internet to rural areas to bridge the digital gap . The project will connect thousands of homes and businesses with quicker networks. It aims to support remote work, education, and economic progress . Technician Samir Khan says access is crucial for modern life. The province is partnering with telecom companies to install new cables. Work begins this autumn , with full coverage expected by 2028. The initiative addresses long- standing connectivity issues in remote regions . Ontario expects it to enhance opportunities across the province significantly.</t>
+    <t>Ontario is expanding high-speed internet to rural areas to bridge the digital divide . The project will connect thousands of homes and businesses with faster networks. It aims to support remote work, education, and economic growth . Technician Samir Khan says access is vital for modern life. The province is partnering with telecom companies to install new cables. Work begins this fall , with full coverage expected by 2028. The initiative addresses long- standing connectivity issues in remote regions . Ontario expects it to enhance opportunities across the province significantly.</t>
   </si>
   <si>
     <t>#339 British Columbia</t>
@@ -6884,7 +6884,7 @@
     <t>British Columbia is hosting a __big/major__ Indigenous art festival to celebrate First Nations culture. The event will feature carvings, paintings, and performances from artists across the province. Organizers aim to foster reconciliation and showcase traditional __wisdom/knowledge__ . Curator Maria Hill says art is __crucial/critical__ for cultural pride. The festival, set for next __fall/summer__ in Vancouver, will include workshops and markets. It's expected to draw thousands, boosting tourism and local economies. Funding comes from provincial and federal __subsidies/grants__ . The event strengthens ties between communities and highlights Canada's diverse heritage.</t>
   </si>
   <si>
-    <t>British Columbia is hosting a big Indigenous art festival to celebrate First Nations culture. The event will feature carvings, paintings, and performances from artists across the province. Organizers aim to foster reconciliation and showcase traditional wisdom . Curator Maria Hill says art is crucial for cultural pride. The festival, set for next fall in Vancouver, will include workshops and markets. It's expected to draw thousands, boosting tourism and local economies. Funding comes from provincial and federal subsidies . The event strengthens ties between communities and highlights Canada's diverse heritage.</t>
+    <t>British Columbia is hosting a major Indigenous art festival to celebrate First Nations culture. The event will feature carvings, paintings, and performances from artists across the province. Organizers aim to foster reconciliation and showcase traditional knowledge . Curator Maria Hill says art is critical for cultural pride. The festival, set for next summer in Vancouver, will include workshops and markets. It's expected to draw thousands, boosting tourism and local economies. Funding comes from provincial and federal grants . The event strengthens ties between communities and highlights Canada's diverse heritage.</t>
   </si>
   <si>
     <t>#340 Urban Farming Program</t>
@@ -6893,7 +6893,7 @@
     <t>Quebec is rolling out a __bold/ambitious__ urban farming program to boost food security in cities. The plan supports rooftop gardens and community plots to grow fresh produce locally. It aims to __cut/reduce__ grocery costs and promote __green/sustainable__ living among residents. Farmer Jean Dupont says local food is __vital/essential__ for healthy communities. The province is offering __funds/grants__ to municipalities and training for new farmers. Pilot projects will launch in Montreal and Quebec City this __summer/spring__ , with expansion planned by 2027. The initiative also tackles climate change by __cutting/reducing__ transport emissions. Officials expect it to inspire other Canadian cities.</t>
   </si>
   <si>
-    <t>Quebec is rolling out a bold urban farming program to boost food security in cities. The plan supports rooftop gardens and community plots to grow fresh produce locally. It aims to cut grocery costs and promote green living among residents. Farmer Jean Dupont says local food is vital for healthy communities. The province is offering funds to municipalities and training for new farmers. Pilot projects will launch in Montreal and Quebec City this summer , with expansion planned by 2027. The initiative also tackles climate change by cutting transport emissions. Officials expect it to inspire other Canadian cities.</t>
+    <t>Quebec is rolling out a ambitious urban farming program to boost food security in cities. The plan supports rooftop gardens and community plots to grow fresh produce locally. It aims to reduce grocery costs and promote sustainable living among residents. Farmer Jean Dupont says local food is essential for healthy communities. The province is offering grants to municipalities and training for new farmers. Pilot projects will launch in Montreal and Quebec City this spring , with expansion planned by 2027. The initiative also tackles climate change by reducing transport emissions. Officials expect it to inspire other Canadian cities.</t>
   </si>
   <si>
     <t>#341 Northwest Territories</t>
@@ -6902,7 +6902,7 @@
     <t>Northwest Territories is launching a cultural revival program to preserve Dene traditions. Elders will teach youth drumming, storytelling, and crafts in communities. The initiative aims to strengthen identity and pride among locals. Organizer Clara Reid says heritage is __crucial/critical__ for unity. Programs start this __summer/spring__ , expanding territory-wide by 2026. The territory is funding local artists to lead. Residents see it as a way to heal past trauma. NWT expects it to inspire cultural __wealth/pride__ nationwide.</t>
   </si>
   <si>
-    <t>Northwest Territories is launching a cultural revival program to preserve Dene traditions. Elders will teach youth drumming, storytelling, and crafts in communities. The initiative aims to strengthen identity and pride among locals. Organizer Clara Reid says heritage is crucial for unity. Programs start this summer , expanding territory-wide by 2026. The territory is funding local artists to lead. Residents see it as a way to heal past trauma. NWT expects it to inspire cultural wealth nationwide.</t>
+    <t>Northwest Territories is launching a cultural revival program to preserve Dene traditions. Elders will teach youth drumming, storytelling, and crafts in communities. The initiative aims to strengthen identity and pride among locals. Organizer Clara Reid says heritage is critical for unity. Programs start this spring , expanding territory-wide by 2026. The territory is funding local artists to lead. Residents see it as a way to heal past trauma. NWT expects it to inspire cultural pride nationwide.</t>
   </si>
   <si>
     <t>#342 Edmonton</t>
@@ -6911,7 +6911,7 @@
     <t>Edmonton is building new health clinics to improve access in growing suburbs. The facilities will offer urgent care, mental health, and family services. The goal is to __cut/reduce__ hospital wait times and support residents. Nurse Kai Wong says care is __vital/essential__ for communities. Construction starts this __autumn/fall__ , with openings by 2027. The city is hiring local staff for operations. Advocates praise the focus on equity. Edmonton expects it to enhance public health significantly.</t>
   </si>
   <si>
-    <t>Edmonton is building new health clinics to improve access in growing suburbs. The facilities will offer urgent care, mental health, and family services. The goal is to cut hospital wait times and support residents. Nurse Kai Wong says care is vital for communities. Construction starts this autumn , with openings by 2027. The city is hiring local staff for operations. Advocates praise the focus on equity. Edmonton expects it to enhance public health significantly.</t>
+    <t>Edmonton is building new health clinics to improve access in growing suburbs. The facilities will offer urgent care, mental health, and family services. The goal is to reduce hospital wait times and support residents. Nurse Kai Wong says care is essential for communities. Construction starts this fall , with openings by 2027. The city is hiring local staff for operations. Advocates praise the focus on equity. Edmonton expects it to enhance public health significantly.</t>
   </si>
   <si>
     <t>#343 Newfoundland</t>
@@ -6920,7 +6920,7 @@
     <t>Newfoundland is launching a coastal management plan to protect shores from __degradation/erosion__ . The initiative includes building seawalls and restoring wetlands for resilience. It aims to safeguard fishing villages and marine life long-term.Biologist Mark Lee says action is __crucial/vital__ for ecosystems. Work begins this fall, with {{3)) by 2027. The province is consuIting locals for input. Environmental groups support the focus on sustainability. Newfoundland expects it to preserve its coastal heritage for generations.</t>
   </si>
   <si>
-    <t>Newfoundland is launching a coastal management plan to protect shores from degradation . The initiative includes building seawalls and restoring wetlands for resilience. It aims to safeguard fishing villages and marine life long-term.Biologist Mark Lee says action is crucial for ecosystems. Work begins this fall, with {{3)) by 2027. The province is consuIting locals for input. Environmental groups support the focus on sustainability. Newfoundland expects it to preserve its coastal heritage for generations.</t>
+    <t>Newfoundland is launching a coastal management plan to protect shores from erosion . The initiative includes building seawalls and restoring wetlands for resilience. It aims to safeguard fishing villages and marine life long-term.Biologist Mark Lee says action is vital for ecosystems. Work begins this fall, with {{3)) by 2027. The province is consuIting locals for input. Environmental groups support the focus on sustainability. Newfoundland expects it to preserve its coastal heritage for generations.</t>
   </si>
   <si>
     <t>#344 Public Transit</t>
@@ -6929,7 +6929,7 @@
     <t>Montreal is upgrading its public transit with new electric buses and trams. The project aims to improve service __effect/reliability__ and cut emissions across the city. It includes better shelters and real-time tracking for riders. Driver Lena Kim says efficiency is crucial for commuters . Construction starts this autumn, with full __reforms/upgrades__ by 2028. The city is training staff for eco-friendly operations. Residents expect less traffic and cleaner air. Montreal aims to set a __sample/model__ for Canadian transit systems.</t>
   </si>
   <si>
-    <t>Montreal is upgrading its public transit with new electric buses and trams. The project aims to improve service effect and cut emissions across the city. It includes better shelters and real-time tracking for riders. Driver Lena Kim says efficiency is crucial for commuters . Construction starts this autumn, with full reforms by 2028. The city is training staff for eco-friendly operations. Residents expect less traffic and cleaner air. Montreal aims to set a sample for Canadian transit systems.</t>
+    <t>Montreal is upgrading its public transit with new electric buses and trams. The project aims to improve service reliability and cut emissions across the city. It includes better shelters and real-time tracking for riders. Driver Lena Kim says efficiency is crucial for commuters . Construction starts this autumn, with full upgrades by 2028. The city is training staff for eco-friendly operations. Residents expect less traffic and cleaner air. Montreal aims to set a model for Canadian transit systems.</t>
   </si>
   <si>
     <t>#345 Climate Risks</t>
@@ -6938,7 +6938,7 @@
     <t>Ottawa is funding climate research to study urban heat and flood risks. Labs will develop solutions like better __heating/drainage__ and cooling systems for cities. The goal is to protect residents and infrastructure long-term. Scientist Aisha Noor says __decision/data__ is vital for policy. Projects launch this summer, with findings expected by 2028. The city is involving schools for education. The plan strengthens Canada's __performance/resilience__ to climate change. Ottawa aims to lead in sustainable urban planning.</t>
   </si>
   <si>
-    <t>Ottawa is funding climate research to study urban heat and flood risks. Labs will develop solutions like better heating and cooling systems for cities. The goal is to protect residents and infrastructure long-term. Scientist Aisha Noor says decision is vital for policy. Projects launch this summer, with findings expected by 2028. The city is involving schools for education. The plan strengthens Canada's performance to climate change. Ottawa aims to lead in sustainable urban planning.</t>
+    <t>Ottawa is funding climate research to study urban heat and flood risks. Labs will develop solutions like better drainage and cooling systems for cities. The goal is to protect residents and infrastructure long-term. Scientist Aisha Noor says data is vital for policy. Projects launch this summer, with findings expected by 2028. The city is involving schools for education. The plan strengthens Canada's resilience to climate change. Ottawa aims to lead in sustainable urban planning.</t>
   </si>
   <si>
     <t>#346 Youth Programs</t>
@@ -6947,7 +6947,7 @@
     <t>Winnipeg is launching youth programs to teach skills like __painting/coding__ and music. The initiative targets underserved areas, offering free lessons to teens. It aims to boost confidence and career __profits/prospects__ for participants. Mentor Alex Reid says opportunity is crucial for growth. Programs start this autumn, expanding __countryside/citywide__ by 2026. The city is hiring local instructors for authenticity. Community leaders see it as a way to reduce inequality. Winnipeg expects it to inspire future leaders.</t>
   </si>
   <si>
-    <t>Winnipeg is launching youth programs to teach skills like painting and music. The initiative targets underserved areas, offering free lessons to teens. It aims to boost confidence and career profits for participants. Mentor Alex Reid says opportunity is crucial for growth. Programs start this autumn, expanding countryside by 2026. The city is hiring local instructors for authenticity. Community leaders see it as a way to reduce inequality. Winnipeg expects it to inspire future leaders.</t>
+    <t>Winnipeg is launching youth programs to teach skills like coding and music. The initiative targets underserved areas, offering free lessons to teens. It aims to boost confidence and career prospects for participants. Mentor Alex Reid says opportunity is crucial for growth. Programs start this autumn, expanding citywide by 2026. The city is hiring local instructors for authenticity. Community leaders see it as a way to reduce inequality. Winnipeg expects it to inspire future leaders.</t>
   </si>
   <si>
     <t>#347 Bike Network</t>
@@ -6956,7 +6956,7 @@
     <t>Vancouver is expanding its bike network to promote cycling as a __unique/primary__ transport mode. New lanes will connect suburbs to downtown,ensuring rider safety. The project aims to cut car use and improve __common/public__ health. Cyclist Mary Qamut says access is vital for commuters. Construction starts this fall, with completion by 2027. The city is adding bike-sharing __parts/stations__ too. Environmentalists praise the plan's focus on sustainability. Vancouver expects it to lower __levels/emissions__ significantly .</t>
   </si>
   <si>
-    <t>Vancouver is expanding its bike network to promote cycling as a unique transport mode. New lanes will connect suburbs to downtown,ensuring rider safety. The project aims to cut car use and improve common health. Cyclist Mary Qamut says access is vital for commuters. Construction starts this fall, with completion by 2027. The city is adding bike-sharing parts too. Environmentalists praise the plan's focus on sustainability. Vancouver expects it to lower levels significantly .</t>
+    <t>Vancouver is expanding its bike network to promote cycling as a primary transport mode. New lanes will connect suburbs to downtown,ensuring rider safety. The project aims to cut car use and improve public health. Cyclist Mary Qamut says access is vital for commuters. Construction starts this fall, with completion by 2027. The city is adding bike-sharing stations too. Environmentalists praise the plan's focus on sustainability. Vancouver expects it to lower emissions significantly .</t>
   </si>
   <si>
     <t>#349 Toronto Greenery</t>
@@ -6965,7 +6965,7 @@
     <t>Toronto is promoting green __covers/roofs__ to combat urban heat and improve air quality. The city offers funds for buildings to install plant-covered roofs widely. The initiative aims to cut energy __wastes/costs__ and support biodiversity. Architect Lara Evans says sustainability is crucial for cities. Installations begin this summer, with thousands expected by 2027. The plan includes public education on environmental benefits. Residents support the move, citing cooler summers. Toronto aims to set a global __target/standard__ for urban greenery.</t>
   </si>
   <si>
-    <t>Toronto is promoting green covers to combat urban heat and improve air quality. The city offers funds for buildings to install plant-covered roofs widely. The initiative aims to cut energy wastes and support biodiversity. Architect Lara Evans says sustainability is crucial for cities. Installations begin this summer, with thousands expected by 2027. The plan includes public education on environmental benefits. Residents support the move, citing cooler summers. Toronto aims to set a global target for urban greenery.</t>
+    <t>Toronto is promoting green roofs to combat urban heat and improve air quality. The city offers funds for buildings to install plant-covered roofs widely. The initiative aims to cut energy costs and support biodiversity. Architect Lara Evans says sustainability is crucial for cities. Installations begin this summer, with thousands expected by 2027. The plan includes public education on environmental benefits. Residents support the move, citing cooler summers. Toronto aims to set a global standard for urban greenery.</t>
   </si>
   <si>
     <t>#350 Rail System</t>
@@ -6974,7 +6974,7 @@
     <t>New Brunswick is upgrading its rail system to improve __product/freight__ and passenger services. New tracks and trains will connect rural towns to urban __nodes/hubs__ faster. The project aims to cut road congestion and emissions significantly. Worker Eli Ross says efficiency is vital for trade. Construction starts this autumn, with completion by 2028. The __proportion/province__ is investing in local labor for the work. Businesses expect smoother supply __groups/chains__ soon. New Brunswick hopes to lead in sustainable transport solutions.</t>
   </si>
   <si>
-    <t>New Brunswick is upgrading its rail system to improve product and passenger services. New tracks and trains will connect rural towns to urban nodes faster. The project aims to cut road congestion and emissions significantly. Worker Eli Ross says efficiency is vital for trade. Construction starts this autumn, with completion by 2028. The proportion is investing in local labor for the work. Businesses expect smoother supply groups soon. New Brunswick hopes to lead in sustainable transport solutions.</t>
+    <t>New Brunswick is upgrading its rail system to improve freight and passenger services. New tracks and trains will connect rural towns to urban hubs faster. The project aims to cut road congestion and emissions significantly. Worker Eli Ross says efficiency is vital for trade. Construction starts this autumn, with completion by 2028. The province is investing in local labor for the work. Businesses expect smoother supply chains soon. New Brunswick hopes to lead in sustainable transport solutions.</t>
   </si>
   <si>
     <t>#351 Tourism Campaign</t>
@@ -6983,7 +6983,7 @@
     <t>Prince Edward Island is launching a tourism campaign to highlight its __culture/beaches__ and history. The initiative promotes festivals, seafood, and hiking trails to attract visitors . It aims to boost local businesses and create __temporal/seasonal__ jobs. Guide Zara Wong says tourism is vital for the economy. Marketing begins this summer, with a __change/surge__ expected by 2026. The province is partnering with airlines for promotions. Residents welcome the plan, citing cultural pride . PEI expects to rival top Canadian destinations soon.</t>
   </si>
   <si>
-    <t>Prince Edward Island is launching a tourism campaign to highlight its culture and history. The initiative promotes festivals, seafood, and hiking trails to attract visitors . It aims to boost local businesses and create temporal jobs. Guide Zara Wong says tourism is vital for the economy. Marketing begins this summer, with a change expected by 2026. The province is partnering with airlines for promotions. Residents welcome the plan, citing cultural pride . PEI expects to rival top Canadian destinations soon.</t>
+    <t>Prince Edward Island is launching a tourism campaign to highlight its beaches and history. The initiative promotes festivals, seafood, and hiking trails to attract visitors . It aims to boost local businesses and create seasonal jobs. Guide Zara Wong says tourism is vital for the economy. Marketing begins this summer, with a surge expected by 2026. The province is partnering with airlines for promotions. Residents welcome the plan, citing cultural pride . PEI expects to rival top Canadian destinations soon.</t>
   </si>
   <si>
     <t>#352 Ward Division</t>
@@ -6992,7 +6992,7 @@
     <t>The idea is that we divide the ward - the patients if you like - and the nurses into three different teams, which we call __lively/primary__ nursing teams. And in those teams we then have the primary nurse which is myself, associate nurses which __might/generally__ tend to be D grade nurses, and health care __officials/assistant__ , and you're all in one team together. The idea is that you would hopefully work as a team in co-ordinating the care for the patients who come in under your care as in the red team. In our teams we have eight patients each. The idea would be that I would __always/normally__ prescribe the care or plan the care, for those patients. In reality, it doesn't always work like that and besides which the associate nurses that are in the teams have those skills anyway from their __upgrading/training__ .</t>
   </si>
   <si>
-    <t>The idea is that we divide the ward - the patients if you like - and the nurses into three different teams, which we call lively nursing teams. And in those teams we then have the primary nurse which is myself, associate nurses which might tend to be D grade nurses, and health care officials , and you're all in one team together. The idea is that you would hopefully work as a team in co-ordinating the care for the patients who come in under your care as in the red team. In our teams we have eight patients each. The idea would be that I would always prescribe the care or plan the care, for those patients. In reality, it doesn't always work like that and besides which the associate nurses that are in the teams have those skills anyway from their upgrading .</t>
+    <t>The idea is that we divide the ward - the patients if you like - and the nurses into three different teams, which we call primary nursing teams. And in those teams we then have the primary nurse which is myself, associate nurses which generally tend to be D grade nurses, and health care assistant , and you're all in one team together. The idea is that you would hopefully work as a team in co-ordinating the care for the patients who come in under your care as in the red team. In our teams we have eight patients each. The idea would be that I would normally prescribe the care or plan the care, for those patients. In reality, it doesn't always work like that and besides which the associate nurses that are in the teams have those skills anyway from their training .</t>
   </si>
   <si>
     <t>#353 Heritage</t>
@@ -7001,7 +7001,7 @@
     <t>Heritage is what the present chooses to make of the past. That means that heritage is dynamic. It's a __challenging/changing__ concept. And it also means that it tends to be __confined/defined__ in opposition to much that is going on in the present. It's endangered. Where there is heritage, there is often a sense of __identity/threat__ , you know, whether it's a building that's about to be bull-dozed, or a way of life that is dying out because of __prolific/economic__ change. The heritage that we speak about in this country in terms of conservation tends to be a term that becomes very central - or more central in new ways - as the state becomes __mired/involved__ in this field of administering conservation.</t>
   </si>
   <si>
-    <t>Heritage is what the present chooses to make of the past. That means that heritage is dynamic. It's a challenging concept. And it also means that it tends to be confined in opposition to much that is going on in the present. It's endangered. Where there is heritage, there is often a sense of identity , you know, whether it's a building that's about to be bull-dozed, or a way of life that is dying out because of prolific change. The heritage that we speak about in this country in terms of conservation tends to be a term that becomes very central - or more central in new ways - as the state becomes mired in this field of administering conservation.</t>
+    <t>Heritage is what the present chooses to make of the past. That means that heritage is dynamic. It's a changing concept. And it also means that it tends to be defined in opposition to much that is going on in the present. It's endangered. Where there is heritage, there is often a sense of threat , you know, whether it's a building that's about to be bull-dozed, or a way of life that is dying out because of economic change. The heritage that we speak about in this country in terms of conservation tends to be a term that becomes very central - or more central in new ways - as the state becomes involved in this field of administering conservation.</t>
   </si>
   <si>
     <t>#354 Joseph Heller</t>
@@ -7010,7 +7010,7 @@
     <t>By way of introduction, Joseph Heller, the author who introduced the phrase "Catch-22" into the English language, died on December 12th at the age of 76 in his home in East Hampton, New York. In 1961, Heller published his first novel, Catch-22, a __succinct/surreal__ anti-war story set in World War Il. Heller's protagonist, a fighter pilot, comes to understand that a man deemed insane by the military __administration/bureaucracy__ may be released from duty. The "Catch-22" of Heller's title is that when a man recognizes his __situation/condition__ , he is no longer insane, Heller spoke at numerous college campuses throughout the 60s, and Catch-22 seemed to __reflect/capture__ the anti-war sentiment of many protesters during the Vietnam War.</t>
   </si>
   <si>
-    <t>By way of introduction, Joseph Heller, the author who introduced the phrase "Catch-22" into the English language, died on December 12th at the age of 76 in his home in East Hampton, New York. In 1961, Heller published his first novel, Catch-22, a succinct anti-war story set in World War Il. Heller's protagonist, a fighter pilot, comes to understand that a man deemed insane by the military administration may be released from duty. The "Catch-22" of Heller's title is that when a man recognizes his situation , he is no longer insane, Heller spoke at numerous college campuses throughout the 60s, and Catch-22 seemed to reflect the anti-war sentiment of many protesters during the Vietnam War.</t>
+    <t>By way of introduction, Joseph Heller, the author who introduced the phrase "Catch-22" into the English language, died on December 12th at the age of 76 in his home in East Hampton, New York. In 1961, Heller published his first novel, Catch-22, a surreal anti-war story set in World War Il. Heller's protagonist, a fighter pilot, comes to understand that a man deemed insane by the military bureaucracy may be released from duty. The "Catch-22" of Heller's title is that when a man recognizes his condition , he is no longer insane, Heller spoke at numerous college campuses throughout the 60s, and Catch-22 seemed to capture the anti-war sentiment of many protesters during the Vietnam War.</t>
   </si>
   <si>
     <t>#355 French Language</t>
@@ -7019,7 +7019,7 @@
     <t>French, on the other hand, is a highly __gentrified/centralized__ language, with the Parisian accent setting the standard for the world. If other French-speaking political __abilities/entities__ had risen to rival France, the situation might be __dissident/different__ . If for instance, Quebec had remained a separate __monarchy/country__ , or if Haiti had been a larger country, then perhaps other French dialects might have become more accepted.</t>
   </si>
   <si>
-    <t>French, on the other hand, is a highly gentrified language, with the Parisian accent setting the standard for the world. If other French-speaking political abilities had risen to rival France, the situation might be dissident . If for instance, Quebec had remained a separate monarchy , or if Haiti had been a larger country, then perhaps other French dialects might have become more accepted.</t>
+    <t>French, on the other hand, is a highly centralized language, with the Parisian accent setting the standard for the world. If other French-speaking political entities had risen to rival France, the situation might be different . If for instance, Quebec had remained a separate country , or if Haiti had been a larger country, then perhaps other French dialects might have become more accepted.</t>
   </si>
   <si>
     <t>#356 UN Charter</t>
@@ -7028,7 +7028,7 @@
     <t>The UN Charter comprises a preamble and 19 chapters divided into 111 articles. The Charter sets __out/forth__ the purposes of the United Nations as: the maintenance of international peace and __civility/security__ , the development of friendly relations between states, and the achievement of cooperation in solving international __ecologic/economic__ , social, cultural, and humanitarian problems. It expresses a strong hope for the __ability/equality__ of all people and the expansion of basic freedoms. The principal organs of the United Nations, as specified in the Charter, are the General Assembly, the Security Council, the Economic and Social Council, the Trusteeship Council, the International Court of Justice, and the Secretariat.</t>
   </si>
   <si>
-    <t>The UN Charter comprises a preamble and 19 chapters divided into 111 articles. The Charter sets out the purposes of the United Nations as: the maintenance of international peace and civility , the development of friendly relations between states, and the achievement of cooperation in solving international ecologic , social, cultural, and humanitarian problems. It expresses a strong hope for the ability of all people and the expansion of basic freedoms. The principal organs of the United Nations, as specified in the Charter, are the General Assembly, the Security Council, the Economic and Social Council, the Trusteeship Council, the International Court of Justice, and the Secretariat.</t>
+    <t>The UN Charter comprises a preamble and 19 chapters divided into 111 articles. The Charter sets forth the purposes of the United Nations as: the maintenance of international peace and security , the development of friendly relations between states, and the achievement of cooperation in solving international economic , social, cultural, and humanitarian problems. It expresses a strong hope for the equality of all people and the expansion of basic freedoms. The principal organs of the United Nations, as specified in the Charter, are the General Assembly, the Security Council, the Economic and Social Council, the Trusteeship Council, the International Court of Justice, and the Secretariat.</t>
   </si>
   <si>
     <t>#357 Quantum Mechanics</t>
@@ -7037,7 +7037,7 @@
     <t>You know that the incredible thing about quantum mechanics were many incredible things, but one of them, at least to me, is that it really works. It is the __science/theory__ of the universe. It describes what's going on here on Earth, that it describes what happens in the universe that Andre's studies. And so when we think about how those building blocks that Leon was just __discussing/describing__ fit together to make the world around us are we use quantum mechanics to describe atoms, nuclei, molecules, light. It is the theory of the world. And so it's not surprising that we see it in many everyday __happenings/occurrences__ and many everyday applications. An example might be the lasers that you see in a compact disc __machine/player__ or the supermarket scanner.</t>
   </si>
   <si>
-    <t>You know that the incredible thing about quantum mechanics were many incredible things, but one of them, at least to me, is that it really works. It is the science of the universe. It describes what's going on here on Earth, that it describes what happens in the universe that Andre's studies. And so when we think about how those building blocks that Leon was just discussing fit together to make the world around us are we use quantum mechanics to describe atoms, nuclei, molecules, light. It is the theory of the world. And so it's not surprising that we see it in many everyday happenings and many everyday applications. An example might be the lasers that you see in a compact disc machine or the supermarket scanner.</t>
+    <t>You know that the incredible thing about quantum mechanics were many incredible things, but one of them, at least to me, is that it really works. It is the theory of the universe. It describes what's going on here on Earth, that it describes what happens in the universe that Andre's studies. And so when we think about how those building blocks that Leon was just describing fit together to make the world around us are we use quantum mechanics to describe atoms, nuclei, molecules, light. It is the theory of the world. And so it's not surprising that we see it in many everyday occurrences and many everyday applications. An example might be the lasers that you see in a compact disc player or the supermarket scanner.</t>
   </si>
   <si>
     <t>#358 Red Fruit</t>
@@ -7046,7 +7046,7 @@
     <t>There is something hard to resist about __fruits/cherries__ . The small red fruit is a popular seasonal food around the __globe/world__ . In northern areas, cherry trees are just beginning to produce flowers. The cherry is a member of the same family of plants as the rose. It is closely related to the plum. Like cherry trees, plum trees also flower in early spring. Cherries are thought to be native to __Eastern/Western__ Asia. There are two major kinds of cherries harvested in the world: sweet and sour. Sour cherries are not eaten fresh because they contain little sugar. Instead, they are processed to start prepared foods like jellies and pies and to __make/start__ alcoholic drinks. The United States is a major producer of sour cherries. Among the states, Michigan is the top producer.</t>
   </si>
   <si>
-    <t>There is something hard to resist about fruits . The small red fruit is a popular seasonal food around the globe . In northern areas, cherry trees are just beginning to produce flowers. The cherry is a member of the same family of plants as the rose. It is closely related to the plum. Like cherry trees, plum trees also flower in early spring. Cherries are thought to be native to Eastern Asia. There are two major kinds of cherries harvested in the world: sweet and sour. Sour cherries are not eaten fresh because they contain little sugar. Instead, they are processed to start prepared foods like jellies and pies and to make alcoholic drinks. The United States is a major producer of sour cherries. Among the states, Michigan is the top producer.</t>
+    <t>There is something hard to resist about cherries . The small red fruit is a popular seasonal food around the world . In northern areas, cherry trees are just beginning to produce flowers. The cherry is a member of the same family of plants as the rose. It is closely related to the plum. Like cherry trees, plum trees also flower in early spring. Cherries are thought to be native to Western Asia. There are two major kinds of cherries harvested in the world: sweet and sour. Sour cherries are not eaten fresh because they contain little sugar. Instead, they are processed to start prepared foods like jellies and pies and to start alcoholic drinks. The United States is a major producer of sour cherries. Among the states, Michigan is the top producer.</t>
   </si>
   <si>
     <t>#359 Clock</t>
@@ -7055,7 +7055,7 @@
     <t>If you can read a clock, you can know the time of __night/day__ . But no one knows what time itself is. We cannot see it. We cannot __feel/touch__ it. We cannot hear it. We know it only by the way we mark its passing. For all our success in measuring the smallest parts of time, time remains one of the great __invention/mysteries__ of the universe. One way to think about time is to imagine a world without time. There could be no __wave/movement__ because time and movement cannot be __divided/separated__ . A world without time could exist only as long as there were no changes. For time and change are linked. We know that time has passed when something changes.</t>
   </si>
   <si>
-    <t>If you can read a clock, you can know the time of night . But no one knows what time itself is. We cannot see it. We cannot feel it. We cannot hear it. We know it only by the way we mark its passing. For all our success in measuring the smallest parts of time, time remains one of the great invention of the universe. One way to think about time is to imagine a world without time. There could be no wave because time and movement cannot be divided . A world without time could exist only as long as there were no changes. For time and change are linked. We know that time has passed when something changes.</t>
+    <t>If you can read a clock, you can know the time of day . But no one knows what time itself is. We cannot see it. We cannot touch it. We cannot hear it. We know it only by the way we mark its passing. For all our success in measuring the smallest parts of time, time remains one of the great mysteries of the universe. One way to think about time is to imagine a world without time. There could be no movement because time and movement cannot be separated . A world without time could exist only as long as there were no changes. For time and change are linked. We know that time has passed when something changes.</t>
   </si>
   <si>
     <t>#360 Winter</t>
@@ -7064,7 +7064,7 @@
     <t>Winter has returned to the northern parts of the world. In the __southern/northern__ United States, winter can mean the return of snow. Large amounts of snow fell in some American cities __first/last__ month. One storm hit the East Coast, causing flight cancellations and temporarily stopping traffic in __all/some__ areas. Snow is a subject of great interest to weather experts. They sometimes have difficulty estimating where, when, or how much __water/snow__ will fall. One reason is that heavy amounts of snow fall in surprisingly small areas. Another reason is that a small __chance/change__ in temperature can mean the difference between snow and rain.</t>
   </si>
   <si>
-    <t>Winter has returned to the northern parts of the world. In the southern United States, winter can mean the return of snow. Large amounts of snow fell in some American cities first month. One storm hit the East Coast, causing flight cancellations and temporarily stopping traffic in all areas. Snow is a subject of great interest to weather experts. They sometimes have difficulty estimating where, when, or how much water will fall. One reason is that heavy amounts of snow fall in surprisingly small areas. Another reason is that a small chance in temperature can mean the difference between snow and rain.</t>
+    <t>Winter has returned to the northern parts of the world. In the northern United States, winter can mean the return of snow. Large amounts of snow fell in some American cities last month. One storm hit the East Coast, causing flight cancellations and temporarily stopping traffic in some areas. Snow is a subject of great interest to weather experts. They sometimes have difficulty estimating where, when, or how much snow will fall. One reason is that heavy amounts of snow fall in surprisingly small areas. Another reason is that a small change in temperature can mean the difference between snow and rain.</t>
   </si>
   <si>
     <t>#361 Allergy</t>
@@ -7073,7 +7073,7 @@
     <t>An allergy is an __often/usually__ strong reaction to a substance. Many things can cause allergies. The most common cause is pollen. Trees usually produce pollen in the spring, grasses in the summer, and weeds in the __winter/fall__ as part of their reproductive process. Other causes include organisms such as dust mites and molds. Chemicals, plants and __bad/dead__ skin particles from dogs and cats can also cause allergic reactions. So can insect stings and some foods. The most common kind of allergic reaction is itchy, watery __mouth/eyes__ , and a blocked or watery nose. Allergies can also __issue/cause__ red, itchy skin. Some reactions can be life-threatening—for example, when breathing passages become blocked.</t>
   </si>
   <si>
-    <t>An allergy is an often strong reaction to a substance. Many things can cause allergies. The most common cause is pollen. Trees usually produce pollen in the spring, grasses in the summer, and weeds in the winter as part of their reproductive process. Other causes include organisms such as dust mites and molds. Chemicals, plants and bad skin particles from dogs and cats can also cause allergic reactions. So can insect stings and some foods. The most common kind of allergic reaction is itchy, watery mouth , and a blocked or watery nose. Allergies can also issue red, itchy skin. Some reactions can be life-threatening—for example, when breathing passages become blocked.</t>
+    <t>An allergy is an usually strong reaction to a substance. Many things can cause allergies. The most common cause is pollen. Trees usually produce pollen in the spring, grasses in the summer, and weeds in the fall as part of their reproductive process. Other causes include organisms such as dust mites and molds. Chemicals, plants and dead skin particles from dogs and cats can also cause allergic reactions. So can insect stings and some foods. The most common kind of allergic reaction is itchy, watery eyes , and a blocked or watery nose. Allergies can also cause red, itchy skin. Some reactions can be life-threatening—for example, when breathing passages become blocked.</t>
   </si>
   <si>
     <t>#362 Cats</t>
@@ -7082,7 +7082,7 @@
     <t>Cats are the __must/most__ popular pets among Americans. So it is not surprising that there are many expressions about cats. Some cats like to __fly/catch__ small birds, like canaries. If someone looks very proud or satisfied with himself, we say he looks like the cat that ate the canary. Sometimes, a cat likes to __hold/play__ with a small animal it catches. So if you play cat and mouse with someone, you change between different kinds of behavior when dealing with another person. For example, a child might offer something sweet to her little brother and then take it away when he reaches for it. A cat will often catch a small animal and present it to its owner. The saying that looks like something the cat dragged in __draws/describes__ something in bad condition.</t>
   </si>
   <si>
-    <t>Cats are the must popular pets among Americans. So it is not surprising that there are many expressions about cats. Some cats like to fly small birds, like canaries. If someone looks very proud or satisfied with himself, we say he looks like the cat that ate the canary. Sometimes, a cat likes to hold with a small animal it catches. So if you play cat and mouse with someone, you change between different kinds of behavior when dealing with another person. For example, a child might offer something sweet to her little brother and then take it away when he reaches for it. A cat will often catch a small animal and present it to its owner. The saying that looks like something the cat dragged in draws something in bad condition.</t>
+    <t>Cats are the most popular pets among Americans. So it is not surprising that there are many expressions about cats. Some cats like to catch small birds, like canaries. If someone looks very proud or satisfied with himself, we say he looks like the cat that ate the canary. Sometimes, a cat likes to play with a small animal it catches. So if you play cat and mouse with someone, you change between different kinds of behavior when dealing with another person. For example, a child might offer something sweet to her little brother and then take it away when he reaches for it. A cat will often catch a small animal and present it to its owner. The saying that looks like something the cat dragged in describes something in bad condition.</t>
   </si>
   <si>
     <t>#363 Vocation</t>
@@ -7091,7 +7091,7 @@
     <t>Now, a professor is also a member of a profession, presumably one that regards its __discretion/discipline__ as a vocation in the full sense of the word — from vocare, 'to call'. Despite some modern uses that reduce it to the mere practicalities of __motivation/employment__ — practice rather than theory, the product of training rather than education — vocation is more than this. A calling is both active and passive. It implies a sense of __intention/purpose__ . It carries with it a __guilty/duty__ to be vocal.</t>
   </si>
   <si>
-    <t>Now, a professor is also a member of a profession, presumably one that regards its discretion as a vocation in the full sense of the word — from vocare, 'to call'. Despite some modern uses that reduce it to the mere practicalities of motivation — practice rather than theory, the product of training rather than education — vocation is more than this. A calling is both active and passive. It implies a sense of intention . It carries with it a guilty to be vocal.</t>
+    <t>Now, a professor is also a member of a profession, presumably one that regards its discipline as a vocation in the full sense of the word — from vocare, 'to call'. Despite some modern uses that reduce it to the mere practicalities of employment — practice rather than theory, the product of training rather than education — vocation is more than this. A calling is both active and passive. It implies a sense of purpose . It carries with it a duty to be vocal.</t>
   </si>
 </sst>
 </file>

</xml_diff>